<commit_message>
Update Clan Capital data - 2026-03-01
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3547,7 +3547,7 @@
         <v>6</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -3825,7 +3825,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -3947,7 +3947,7 @@
         <v>6</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4383,7 +4383,7 @@
         <v>6</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -4505,7 +4505,7 @@
         <v>6</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -4686,7 +4686,7 @@
         <v>6</v>
       </c>
       <c r="R28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -4747,7 +4747,7 @@
         <v>6</v>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -4869,7 +4869,7 @@
         <v>6</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -5156,7 +5156,7 @@
         <v>6</v>
       </c>
       <c r="R37" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -5217,7 +5217,7 @@
         <v>6</v>
       </c>
       <c r="R39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-02
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3129,7 +3129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH48"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3608,7 +3608,7 @@
         <v>6</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -3825,7 +3825,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -4140,7 +4140,7 @@
         <v>6</v>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4331,7 +4331,7 @@
         <v>6</v>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -4383,7 +4383,7 @@
         <v>6</v>
       </c>
       <c r="R22" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -4557,7 +4557,7 @@
         <v>6</v>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -4609,7 +4609,7 @@
         <v>6</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -4747,13 +4747,13 @@
         <v>6</v>
       </c>
       <c r="R29" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Roberta</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
@@ -4766,26 +4766,26 @@
         <v/>
       </c>
       <c r="D30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J30" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="E30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H30" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K30" s="10" t="n">
         <v>6</v>
       </c>
@@ -4808,13 +4808,13 @@
         <v>6</v>
       </c>
       <c r="R30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
@@ -4827,7 +4827,7 @@
         <v/>
       </c>
       <c r="D31" s="14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E31" s="9" t="n">
         <v>6</v>
@@ -4845,7 +4845,7 @@
         <v>6</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K31" s="10" t="n">
         <v>6</v>
@@ -4875,7 +4875,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
@@ -4887,27 +4887,7 @@
         <f>ROUND(AVERAGE(D32:AH32), 0)</f>
         <v/>
       </c>
-      <c r="D32" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="J32" s="10" t="n"/>
       <c r="K32" s="10" t="n">
         <v>6</v>
       </c>
@@ -4936,7 +4916,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>th4nos</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
@@ -4948,12 +4928,32 @@
         <f>ROUND(AVERAGE(D33:AH33), 0)</f>
         <v/>
       </c>
-      <c r="J33" s="10" t="n"/>
+      <c r="D33" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K33" s="10" t="n">
         <v>6</v>
       </c>
       <c r="L33" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M33" s="9" t="n">
         <v>6</v>
@@ -4977,7 +4977,7 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>th4nos</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
@@ -4989,15 +4989,6 @@
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
-      <c r="D34" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F34" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G34" s="9" t="n">
         <v>6</v>
       </c>
@@ -5014,54 +5005,42 @@
         <v>6</v>
       </c>
       <c r="L34" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M34" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N34" s="33" t="n">
+      <c r="N34" s="10" t="n">
         <v>6</v>
       </c>
       <c r="O34" t="n">
         <v>6</v>
       </c>
       <c r="P34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q34" t="n">
         <v>6</v>
       </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
         <f>ROUND(AVERAGE(D35:AH35), 0)</f>
         <v/>
       </c>
-      <c r="G35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J35" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K35" s="10" t="n">
         <v>6</v>
       </c>
@@ -5069,16 +5048,16 @@
         <v>6</v>
       </c>
       <c r="M35" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N35" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O35" t="n">
         <v>6</v>
       </c>
       <c r="P35" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q35" t="n">
         <v>6</v>
@@ -5090,32 +5069,24 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C36" s="13">
         <f>ROUND(AVERAGE(D36:AH36), 0)</f>
         <v/>
       </c>
-      <c r="K36" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L36" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K36" s="10" t="n"/>
+      <c r="L36" s="10" t="n"/>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="10" t="n"/>
       <c r="O36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P36" t="n">
         <v>6</v>
@@ -5124,13 +5095,13 @@
         <v>6</v>
       </c>
       <c r="R36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
@@ -5147,13 +5118,13 @@
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="10" t="n"/>
       <c r="O37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>6</v>
@@ -5162,12 +5133,12 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
@@ -5178,14 +5149,11 @@
       <c r="L38" s="10" t="n"/>
       <c r="M38" s="9" t="n"/>
       <c r="N38" s="10" t="n"/>
-      <c r="O38" t="n">
-        <v>6</v>
-      </c>
       <c r="P38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R38" t="n">
         <v>6</v>
@@ -5194,7 +5162,7 @@
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>terracrom</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
@@ -5211,24 +5179,24 @@
       <c r="M39" s="9" t="n"/>
       <c r="N39" s="10" t="n"/>
       <c r="P39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>fede61mito</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5252,7 +5220,7 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
@@ -5269,24 +5237,24 @@
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="10" t="n"/>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R41" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Xx_Herman_xX</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5297,25 +5265,22 @@
       <c r="L42" s="10" t="n"/>
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="10" t="n"/>
-      <c r="P42" t="n">
-        <v>1</v>
-      </c>
       <c r="Q42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R42" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Xx_Herman_xX</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -5326,22 +5291,19 @@
       <c r="L43" s="10" t="n"/>
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="10" t="n"/>
-      <c r="Q43" t="n">
-        <v>0</v>
-      </c>
       <c r="R43" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>dibba10</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5352,17 +5314,14 @@
       <c r="L44" s="10" t="n"/>
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="10" t="n"/>
-      <c r="Q44" t="n">
-        <v>2</v>
-      </c>
       <c r="R44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
@@ -5379,18 +5338,18 @@
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="10" t="n"/>
       <c r="R45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>thommyspine</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5402,18 +5361,18 @@
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="10" t="n"/>
       <c r="R46" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>eltishqipe</t>
+          <t>I puma</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C47" s="13">
@@ -5425,18 +5384,18 @@
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="10" t="n"/>
       <c r="R47" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5451,7 +5410,52 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>BigGiurz08</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>02/03/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="13">
+        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
+        <v/>
+      </c>
+      <c r="K49" s="10" t="n"/>
+      <c r="L49" s="10" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="10" t="n"/>
+      <c r="R49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>StepanYT Ita Uk</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>02/03/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="13">
+        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="10" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="10" t="n"/>
+      <c r="R50" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AH50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-07
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3238,7 +3238,7 @@
       </c>
       <c r="S1" s="7" t="inlineStr">
         <is>
-          <t>Colonna17</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="T1" s="7" t="inlineStr">
@@ -3359,6 +3359,9 @@
       <c r="R2" t="n">
         <v>6</v>
       </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -3399,6 +3402,9 @@
       <c r="R3" t="n">
         <v>0</v>
       </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -3460,6 +3466,9 @@
       <c r="R4" t="n">
         <v>6</v>
       </c>
+      <c r="S4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -3497,6 +3506,9 @@
       <c r="R5" t="n">
         <v>6</v>
       </c>
+      <c r="S5" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -3549,6 +3561,9 @@
       <c r="R6" t="n">
         <v>6</v>
       </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -3610,6 +3625,9 @@
       <c r="R7" t="n">
         <v>6</v>
       </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -3671,6 +3689,9 @@
       <c r="R8" t="n">
         <v>0</v>
       </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -3723,6 +3744,9 @@
       <c r="R9" t="n">
         <v>0</v>
       </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -3775,6 +3799,9 @@
       <c r="R10" t="n">
         <v>6</v>
       </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -3827,6 +3854,9 @@
       <c r="R11" t="n">
         <v>6</v>
       </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -3888,6 +3918,9 @@
       <c r="R12" t="n">
         <v>6</v>
       </c>
+      <c r="S12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -3949,6 +3982,9 @@
       <c r="R13" t="n">
         <v>6</v>
       </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -3995,6 +4031,9 @@
       <c r="R14" t="n">
         <v>6</v>
       </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -4044,6 +4083,9 @@
       <c r="R15" t="n">
         <v>6</v>
       </c>
+      <c r="S15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -4081,6 +4123,9 @@
       <c r="R16" t="n">
         <v>6</v>
       </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -4142,6 +4187,9 @@
       <c r="R17" t="n">
         <v>6</v>
       </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -4198,6 +4246,9 @@
         <v>6</v>
       </c>
       <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4236,6 +4287,9 @@
       <c r="R19" t="n">
         <v>6</v>
       </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -4295,6 +4349,9 @@
         <v>6</v>
       </c>
       <c r="R20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S20" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4333,6 +4390,9 @@
       <c r="R21" t="n">
         <v>6</v>
       </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -4385,11 +4445,14 @@
       <c r="R22" t="n">
         <v>6</v>
       </c>
+      <c r="S22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Luxor</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -4414,16 +4477,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I23" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L23" s="10" t="n">
         <v>0</v>
@@ -4435,22 +4498,25 @@
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="S23" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
@@ -4462,20 +4528,11 @@
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
-      <c r="D24" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G24" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I24" s="9" t="n">
         <v>6</v>
@@ -4484,16 +4541,16 @@
         <v>6</v>
       </c>
       <c r="K24" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L24" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M24" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N24" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O24" t="n">
         <v>6</v>
@@ -4505,13 +4562,16 @@
         <v>6</v>
       </c>
       <c r="R24" t="n">
+        <v>6</v>
+      </c>
+      <c r="S24" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
@@ -4524,7 +4584,7 @@
         <v/>
       </c>
       <c r="G25" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H25" s="9" t="n">
         <v>6</v>
@@ -4558,38 +4618,26 @@
       </c>
       <c r="R25" t="n">
         <v>6</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C26" s="13">
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
-      <c r="G26" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J26" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K26" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L26" s="10" t="n">
         <v>6</v>
       </c>
@@ -4609,24 +4657,30 @@
         <v>6</v>
       </c>
       <c r="R26" t="n">
+        <v>6</v>
+      </c>
+      <c r="S26" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C27" s="13">
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
+      <c r="K27" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L27" s="10" t="n">
         <v>6</v>
       </c>
@@ -4646,24 +4700,48 @@
         <v>6</v>
       </c>
       <c r="R27" t="n">
+        <v>6</v>
+      </c>
+      <c r="S27" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C28" s="13">
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
+      <c r="D28" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K28" s="10" t="n">
         <v>6</v>
       </c>
@@ -4687,12 +4765,15 @@
       </c>
       <c r="R28" t="n">
         <v>6</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -4705,7 +4786,7 @@
         <v/>
       </c>
       <c r="D29" s="14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E29" s="9" t="n">
         <v>6</v>
@@ -4723,7 +4804,7 @@
         <v>6</v>
       </c>
       <c r="J29" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K29" s="10" t="n">
         <v>6</v>
@@ -4748,12 +4829,15 @@
       </c>
       <c r="R29" t="n">
         <v>6</v>
+      </c>
+      <c r="S29" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
@@ -4766,7 +4850,7 @@
         <v/>
       </c>
       <c r="D30" s="14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>6</v>
@@ -4784,7 +4868,7 @@
         <v>6</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K30" s="10" t="n">
         <v>6</v>
@@ -4809,12 +4893,15 @@
       </c>
       <c r="R30" t="n">
         <v>6</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
@@ -4826,27 +4913,7 @@
         <f>ROUND(AVERAGE(D31:AH31), 0)</f>
         <v/>
       </c>
-      <c r="D31" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J31" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="J31" s="10" t="n"/>
       <c r="K31" s="10" t="n">
         <v>6</v>
       </c>
@@ -4870,12 +4937,15 @@
       </c>
       <c r="R31" t="n">
         <v>6</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>th4nos</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
@@ -4887,12 +4957,32 @@
         <f>ROUND(AVERAGE(D32:AH32), 0)</f>
         <v/>
       </c>
-      <c r="J32" s="10" t="n"/>
+      <c r="D32" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K32" s="10" t="n">
         <v>6</v>
       </c>
       <c r="L32" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M32" s="9" t="n">
         <v>6</v>
@@ -4910,13 +5000,16 @@
         <v>6</v>
       </c>
       <c r="R32" t="n">
+        <v>6</v>
+      </c>
+      <c r="S32" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>th4nos</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
@@ -4928,15 +5021,6 @@
         <f>ROUND(AVERAGE(D33:AH33), 0)</f>
         <v/>
       </c>
-      <c r="D33" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E33" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F33" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G33" s="9" t="n">
         <v>6</v>
       </c>
@@ -4953,54 +5037,45 @@
         <v>6</v>
       </c>
       <c r="L33" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M33" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N33" s="33" t="n">
+      <c r="N33" s="10" t="n">
         <v>6</v>
       </c>
       <c r="O33" t="n">
         <v>6</v>
       </c>
       <c r="P33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q33" t="n">
         <v>6</v>
       </c>
       <c r="R33" t="n">
+        <v>6</v>
+      </c>
+      <c r="S33" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C34" s="13">
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
-      <c r="G34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J34" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K34" s="10" t="n">
         <v>6</v>
       </c>
@@ -5008,53 +5083,48 @@
         <v>6</v>
       </c>
       <c r="M34" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N34" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
         <v>6</v>
       </c>
       <c r="P34" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q34" t="n">
         <v>6</v>
       </c>
       <c r="R34" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
         <f>ROUND(AVERAGE(D35:AH35), 0)</f>
         <v/>
       </c>
-      <c r="K35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K35" s="10" t="n"/>
+      <c r="L35" s="10" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="10" t="n"/>
       <c r="O35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P35" t="n">
         <v>6</v>
@@ -5063,13 +5133,16 @@
         <v>6</v>
       </c>
       <c r="R35" t="n">
+        <v>6</v>
+      </c>
+      <c r="S35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
@@ -5086,27 +5159,30 @@
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="10" t="n"/>
       <c r="O36" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R36" t="n">
         <v>6</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
@@ -5117,23 +5193,23 @@
       <c r="L37" s="10" t="n"/>
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="10" t="n"/>
-      <c r="O37" t="n">
-        <v>6</v>
-      </c>
       <c r="P37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R37" t="n">
+        <v>6</v>
+      </c>
+      <c r="S37" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>terracrom</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
@@ -5150,24 +5226,27 @@
       <c r="M38" s="9" t="n"/>
       <c r="N38" s="10" t="n"/>
       <c r="P38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R38" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>fede61mito</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5187,11 +5266,14 @@
       <c r="R39" t="n">
         <v>0</v>
       </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
@@ -5208,24 +5290,27 @@
       <c r="M40" s="9" t="n"/>
       <c r="N40" s="10" t="n"/>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R40" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="S40" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5236,25 +5321,22 @@
       <c r="L41" s="10" t="n"/>
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="10" t="n"/>
-      <c r="P41" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>2</v>
-      </c>
       <c r="R41" t="n">
+        <v>6</v>
+      </c>
+      <c r="S41" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>Xx_Herman_xX</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5265,17 +5347,17 @@
       <c r="L42" s="10" t="n"/>
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="10" t="n"/>
-      <c r="Q42" t="n">
-        <v>0</v>
-      </c>
       <c r="R42" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="S42" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
@@ -5292,18 +5374,21 @@
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="10" t="n"/>
       <c r="R43" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>thommyspine</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5315,18 +5400,21 @@
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="10" t="n"/>
       <c r="R44" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5340,11 +5428,14 @@
       <c r="R45" t="n">
         <v>0</v>
       </c>
+      <c r="S45" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>thommyspine</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
@@ -5363,11 +5454,14 @@
       <c r="R46" t="n">
         <v>0</v>
       </c>
+      <c r="S46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>I puma</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
@@ -5384,18 +5478,21 @@
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="10" t="n"/>
       <c r="R47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5406,19 +5503,19 @@
       <c r="L48" s="10" t="n"/>
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="10" t="n"/>
-      <c r="R48" t="n">
+      <c r="S48" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5429,19 +5526,19 @@
       <c r="L49" s="10" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="10" t="n"/>
-      <c r="R49" t="n">
+      <c r="S49" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>metracros</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5452,7 +5549,7 @@
       <c r="L50" s="10" t="n"/>
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="10" t="n"/>
-      <c r="R50" t="n">
+      <c r="S50" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-08
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3129,7 +3129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3690,7 +3690,7 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -4288,7 +4288,7 @@
         <v>6</v>
       </c>
       <c r="S19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -4391,7 +4391,7 @@
         <v>6</v>
       </c>
       <c r="S21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -4620,7 +4620,7 @@
         <v>6</v>
       </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -4831,7 +4831,7 @@
         <v>6</v>
       </c>
       <c r="S29" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -4895,7 +4895,7 @@
         <v>6</v>
       </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
@@ -5136,7 +5136,7 @@
         <v>6</v>
       </c>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -5299,7 +5299,7 @@
         <v>6</v>
       </c>
       <c r="S40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -5504,7 +5504,7 @@
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="10" t="n"/>
       <c r="S48" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49">
@@ -5551,6 +5551,29 @@
       <c r="N50" s="10" t="n"/>
       <c r="S50" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>Alessio9797</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="13">
+        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="10" t="n"/>
+      <c r="L51" s="10" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="10" t="n"/>
+      <c r="S51" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-09
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3562,7 +3562,7 @@
         <v>6</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -3626,7 +3626,7 @@
         <v>6</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -3983,7 +3983,7 @@
         <v>6</v>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4032,7 +4032,7 @@
         <v>6</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -4188,7 +4188,7 @@
         <v>6</v>
       </c>
       <c r="S17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4249,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -4391,7 +4391,7 @@
         <v>6</v>
       </c>
       <c r="S21" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -4767,7 +4767,7 @@
         <v>6</v>
       </c>
       <c r="S28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -4939,7 +4939,7 @@
         <v>6</v>
       </c>
       <c r="S31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -5171,7 +5171,7 @@
         <v>6</v>
       </c>
       <c r="S36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-14
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3243,7 +3243,7 @@
       </c>
       <c r="T1" s="7" t="inlineStr">
         <is>
-          <t>Colonna18</t>
+          <t>13/03/2026</t>
         </is>
       </c>
       <c r="U1" s="7" t="inlineStr">
@@ -3362,6 +3362,9 @@
       <c r="S2" t="n">
         <v>0</v>
       </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -3405,54 +3408,33 @@
       <c r="S3" t="n">
         <v>0</v>
       </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>ajejebrazorf</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C4" s="13">
         <f>ROUND(AVERAGE(D4:AH4), 0)</f>
         <v/>
       </c>
-      <c r="D4" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F4" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K4" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L4" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M4" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N4" s="33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
         <v>6</v>
@@ -3468,31 +3450,49 @@
       </c>
       <c r="S4" t="n">
         <v>6</v>
+      </c>
+      <c r="T4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C5" s="13">
         <f>ROUND(AVERAGE(D5:AH5), 0)</f>
         <v/>
       </c>
+      <c r="G5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L5" s="10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M5" s="9" t="n">
         <v>0</v>
       </c>
       <c r="N5" s="33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O5" t="n">
         <v>6</v>
@@ -3508,12 +3508,15 @@
       </c>
       <c r="S5" t="n">
         <v>6</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -3525,11 +3528,20 @@
         <f>ROUND(AVERAGE(D6:AH6), 0)</f>
         <v/>
       </c>
+      <c r="D6" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G6" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>6</v>
@@ -3541,13 +3553,13 @@
         <v>6</v>
       </c>
       <c r="L6" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N6" s="33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O6" t="n">
         <v>6</v>
@@ -3563,12 +3575,15 @@
       </c>
       <c r="S6" t="n">
         <v>6</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -3596,43 +3611,46 @@
         <v>0</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N7" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>6</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
@@ -3644,59 +3662,53 @@
         <f>ROUND(AVERAGE(D8:AH8), 0)</f>
         <v/>
       </c>
-      <c r="D8" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G8" s="9" t="n">
         <v>6</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K8" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L8" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N8" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -3709,16 +3721,16 @@
         <v/>
       </c>
       <c r="G9" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H9" s="9" t="n">
         <v>6</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K9" s="10" t="n">
         <v>6</v>
@@ -3727,31 +3739,34 @@
         <v>6</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="P9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>ER DANDI 1927</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -3764,49 +3779,52 @@
         <v/>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>6</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K10" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L10" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N10" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>6</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -3818,50 +3836,62 @@
         <f>ROUND(AVERAGE(D11:AH11), 0)</f>
         <v/>
       </c>
+      <c r="D11" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G11" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" t="n">
+        <v>6</v>
+      </c>
+      <c r="P11" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q11" t="n">
         <v>5</v>
       </c>
-      <c r="I11" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
       <c r="R11" t="n">
         <v>6</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="T11" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -3883,7 +3913,7 @@
         <v>6</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>6</v>
@@ -3913,45 +3943,33 @@
         <v>6</v>
       </c>
       <c r="Q12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R12" t="n">
         <v>6</v>
       </c>
       <c r="S12" t="n">
         <v>6</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>Giorgio</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/12/2025</t>
         </is>
       </c>
       <c r="C13" s="13">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
-      <c r="D13" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="I13" s="9" t="n">
         <v>6</v>
       </c>
@@ -3962,7 +3980,7 @@
         <v>6</v>
       </c>
       <c r="L13" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M13" s="9" t="n">
         <v>6</v>
@@ -3984,23 +4002,29 @@
       </c>
       <c r="S13" t="n">
         <v>6</v>
+      </c>
+      <c r="T13" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Giorgio</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>29/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C14" s="13">
         <f>ROUND(AVERAGE(D14:AH14), 0)</f>
         <v/>
       </c>
+      <c r="H14" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="I14" s="9" t="n">
         <v>6</v>
       </c>
@@ -4011,7 +4035,7 @@
         <v>6</v>
       </c>
       <c r="L14" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M14" s="9" t="n">
         <v>6</v>
@@ -4032,24 +4056,39 @@
         <v>6</v>
       </c>
       <c r="S14" t="n">
+        <v>6</v>
+      </c>
+      <c r="T14" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C15" s="13">
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
+      <c r="D15" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="H15" s="9" t="n">
         <v>6</v>
       </c>
@@ -4085,95 +4124,97 @@
       </c>
       <c r="S15" t="n">
         <v>6</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>GioStyle</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="13">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
+      <c r="D16" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="L16" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M16" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N16" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
+        <v>3</v>
+      </c>
+      <c r="T16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C17" s="13">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="D17" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L17" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="10" t="n"/>
       <c r="M17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
         <v>6</v>
@@ -4189,12 +4230,15 @@
       </c>
       <c r="S17" t="n">
         <v>6</v>
+      </c>
+      <c r="T17" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -4216,46 +4260,52 @@
         <v>6</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K18" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L18" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N18" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q18" t="n">
         <v>6</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S18" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -4273,7 +4323,7 @@
         <v>6</v>
       </c>
       <c r="N19" s="33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
         <v>6</v>
@@ -4289,12 +4339,15 @@
       </c>
       <c r="S19" t="n">
         <v>6</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -4306,17 +4359,8 @@
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="D20" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G20" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H20" s="9" t="n">
         <v>6</v>
@@ -4353,27 +4397,55 @@
       </c>
       <c r="S20" t="n">
         <v>6</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C21" s="13">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="K21" s="10" t="n"/>
-      <c r="L21" s="10" t="n"/>
+      <c r="D21" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M21" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N21" s="33" t="n">
         <v>0</v>
@@ -4392,12 +4464,15 @@
       </c>
       <c r="S21" t="n">
         <v>6</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
@@ -4410,7 +4485,7 @@
         <v/>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H22" s="9" t="n">
         <v>6</v>
@@ -4446,13 +4521,16 @@
         <v>6</v>
       </c>
       <c r="S22" t="n">
+        <v>6</v>
+      </c>
+      <c r="T22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -4464,20 +4542,11 @@
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
-      <c r="D23" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G23" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>6</v>
@@ -4486,16 +4555,16 @@
         <v>6</v>
       </c>
       <c r="K23" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L23" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M23" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N23" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O23" t="n">
         <v>6</v>
@@ -4511,38 +4580,26 @@
       </c>
       <c r="S23" t="n">
         <v>6</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C24" s="13">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
-      <c r="G24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K24" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L24" s="10" t="n">
         <v>6</v>
       </c>
@@ -4566,35 +4623,26 @@
       </c>
       <c r="S24" t="n">
         <v>6</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C25" s="13">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
-      <c r="G25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J25" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K25" s="10" t="n">
         <v>6</v>
       </c>
@@ -4620,24 +4668,51 @@
         <v>6</v>
       </c>
       <c r="S25" t="n">
+        <v>6</v>
+      </c>
+      <c r="T25" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C26" s="13">
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
+      <c r="D26" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J26" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K26" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L26" s="10" t="n">
         <v>6</v>
       </c>
@@ -4661,23 +4736,47 @@
       </c>
       <c r="S26" t="n">
         <v>6</v>
+      </c>
+      <c r="T26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C27" s="13">
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
+      <c r="D27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>5</v>
+      </c>
       <c r="K27" s="10" t="n">
         <v>6</v>
       </c>
@@ -4704,12 +4803,15 @@
       </c>
       <c r="S27" t="n">
         <v>6</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
@@ -4769,11 +4871,14 @@
       <c r="S28" t="n">
         <v>6</v>
       </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -4785,27 +4890,7 @@
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="D29" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>5</v>
-      </c>
+      <c r="J29" s="10" t="n"/>
       <c r="K29" s="10" t="n">
         <v>6</v>
       </c>
@@ -4831,13 +4916,16 @@
         <v>6</v>
       </c>
       <c r="S29" t="n">
+        <v>6</v>
+      </c>
+      <c r="T29" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
@@ -4849,15 +4937,6 @@
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
-      <c r="D30" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G30" s="9" t="n">
         <v>6</v>
       </c>
@@ -4879,14 +4958,14 @@
       <c r="M30" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N30" s="33" t="n">
+      <c r="N30" s="10" t="n">
         <v>6</v>
       </c>
       <c r="O30" t="n">
         <v>6</v>
       </c>
       <c r="P30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="n">
         <v>6</v>
@@ -4895,25 +4974,27 @@
         <v>6</v>
       </c>
       <c r="S30" t="n">
+        <v>6</v>
+      </c>
+      <c r="T30" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C31" s="13">
         <f>ROUND(AVERAGE(D31:AH31), 0)</f>
         <v/>
       </c>
-      <c r="J31" s="10" t="n"/>
       <c r="K31" s="10" t="n">
         <v>6</v>
       </c>
@@ -4921,10 +5002,10 @@
         <v>6</v>
       </c>
       <c r="M31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N31" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="N31" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="O31" t="n">
         <v>6</v>
@@ -4936,63 +5017,37 @@
         <v>6</v>
       </c>
       <c r="R31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>th4nos</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C32" s="13">
         <f>ROUND(AVERAGE(D32:AH32), 0)</f>
         <v/>
       </c>
-      <c r="D32" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K32" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L32" s="10" t="n">
+      <c r="K32" s="10" t="n"/>
+      <c r="L32" s="10" t="n"/>
+      <c r="M32" s="9" t="n"/>
+      <c r="N32" s="10" t="n"/>
+      <c r="O32" t="n">
         <v>5</v>
       </c>
-      <c r="M32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N32" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="O32" t="n">
-        <v>6</v>
-      </c>
       <c r="P32" t="n">
         <v>6</v>
       </c>
@@ -5004,93 +5059,68 @@
       </c>
       <c r="S32" t="n">
         <v>6</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C33" s="13">
         <f>ROUND(AVERAGE(D33:AH33), 0)</f>
         <v/>
       </c>
-      <c r="G33" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H33" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I33" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J33" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K33" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L33" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M33" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N33" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="K33" s="10" t="n"/>
+      <c r="L33" s="10" t="n"/>
+      <c r="M33" s="9" t="n"/>
+      <c r="N33" s="10" t="n"/>
       <c r="O33" t="n">
         <v>6</v>
       </c>
       <c r="P33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R33" t="n">
         <v>6</v>
       </c>
       <c r="S33" t="n">
         <v>6</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C34" s="13">
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
-      <c r="K34" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L34" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M34" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" t="n">
-        <v>6</v>
-      </c>
+      <c r="K34" s="10" t="n"/>
+      <c r="L34" s="10" t="n"/>
+      <c r="M34" s="9" t="n"/>
+      <c r="N34" s="10" t="n"/>
       <c r="P34" t="n">
         <v>6</v>
       </c>
@@ -5098,21 +5128,24 @@
         <v>6</v>
       </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S34" t="n">
+        <v>6</v>
+      </c>
+      <c r="T34" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>terracrom</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
@@ -5123,31 +5156,31 @@
       <c r="L35" s="10" t="n"/>
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="10" t="n"/>
-      <c r="O35" t="n">
-        <v>5</v>
-      </c>
       <c r="P35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>fede61mito</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="C36" s="13">
@@ -5158,9 +5191,6 @@
       <c r="L36" s="10" t="n"/>
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="10" t="n"/>
-      <c r="O36" t="n">
-        <v>6</v>
-      </c>
       <c r="P36" t="n">
         <v>0</v>
       </c>
@@ -5168,21 +5198,24 @@
         <v>0</v>
       </c>
       <c r="R36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
@@ -5194,27 +5227,30 @@
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="10" t="n"/>
       <c r="P37" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R37" t="n">
         <v>6</v>
       </c>
       <c r="S37" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
@@ -5225,28 +5261,25 @@
       <c r="L38" s="10" t="n"/>
       <c r="M38" s="9" t="n"/>
       <c r="N38" s="10" t="n"/>
-      <c r="P38" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>0</v>
-      </c>
       <c r="R38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S38" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="T38" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5257,28 +5290,25 @@
       <c r="L39" s="10" t="n"/>
       <c r="M39" s="9" t="n"/>
       <c r="N39" s="10" t="n"/>
-      <c r="P39" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>0</v>
-      </c>
       <c r="R39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S39" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="T39" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5289,28 +5319,25 @@
       <c r="L40" s="10" t="n"/>
       <c r="M40" s="9" t="n"/>
       <c r="N40" s="10" t="n"/>
-      <c r="P40" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>2</v>
-      </c>
       <c r="R40" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>thommyspine</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5322,21 +5349,24 @@
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="10" t="n"/>
       <c r="R41" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="T41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5348,21 +5378,24 @@
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="10" t="n"/>
       <c r="R42" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S42" t="n">
+        <v>6</v>
+      </c>
+      <c r="T42" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -5379,11 +5412,14 @@
       <c r="S43" t="n">
         <v>0</v>
       </c>
+      <c r="T43" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>thommyspine</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
@@ -5403,18 +5439,21 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="T44" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5425,22 +5464,22 @@
       <c r="L45" s="10" t="n"/>
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="10" t="n"/>
-      <c r="R45" t="n">
-        <v>0</v>
-      </c>
       <c r="S45" t="n">
+        <v>6</v>
+      </c>
+      <c r="T45" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5451,22 +5490,22 @@
       <c r="L46" s="10" t="n"/>
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="10" t="n"/>
-      <c r="R46" t="n">
-        <v>0</v>
-      </c>
       <c r="S46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="C47" s="13">
@@ -5477,22 +5516,22 @@
       <c r="L47" s="10" t="n"/>
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="10" t="n"/>
-      <c r="R47" t="n">
-        <v>0</v>
-      </c>
       <c r="S47" t="n">
         <v>6</v>
+      </c>
+      <c r="T47" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5503,19 +5542,19 @@
       <c r="L48" s="10" t="n"/>
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="10" t="n"/>
-      <c r="S48" t="n">
-        <v>6</v>
+      <c r="T48" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5526,19 +5565,19 @@
       <c r="L49" s="10" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="10" t="n"/>
-      <c r="S49" t="n">
-        <v>0</v>
+      <c r="T49" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>metracros</t>
+          <t>Samu-Nighix</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5549,19 +5588,19 @@
       <c r="L50" s="10" t="n"/>
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="10" t="n"/>
-      <c r="S50" t="n">
-        <v>0</v>
+      <c r="T50" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>Marchi™</t>
         </is>
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C51" s="13">
@@ -5572,8 +5611,8 @@
       <c r="L51" s="10" t="n"/>
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="10" t="n"/>
-      <c r="S51" t="n">
-        <v>6</v>
+      <c r="T51" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-15
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3129,7 +3129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3818,7 +3818,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -3952,7 +3952,7 @@
         <v>6</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -4004,7 +4004,7 @@
         <v>6</v>
       </c>
       <c r="T13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4126,7 +4126,7 @@
         <v>6</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -4190,7 +4190,7 @@
         <v>3</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -4232,7 +4232,7 @@
         <v>6</v>
       </c>
       <c r="T17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4299,7 +4299,7 @@
         <v>6</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -4399,7 +4399,7 @@
         <v>6</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -4466,7 +4466,7 @@
         <v>6</v>
       </c>
       <c r="T21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -4582,7 +4582,7 @@
         <v>6</v>
       </c>
       <c r="T23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -4625,7 +4625,7 @@
         <v>6</v>
       </c>
       <c r="T24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -4805,7 +4805,7 @@
         <v>6</v>
       </c>
       <c r="T27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -4872,7 +4872,7 @@
         <v>6</v>
       </c>
       <c r="T28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -5061,7 +5061,7 @@
         <v>6</v>
       </c>
       <c r="T32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -5134,7 +5134,7 @@
         <v>6</v>
       </c>
       <c r="T34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
@@ -5175,7 +5175,7 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
@@ -5192,16 +5192,16 @@
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="10" t="n"/>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T36" t="n">
         <v>0</v>
@@ -5210,12 +5210,12 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
@@ -5226,26 +5226,20 @@
       <c r="L37" s="10" t="n"/>
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="10" t="n"/>
-      <c r="P37" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>2</v>
-      </c>
       <c r="R37" t="n">
         <v>6</v>
       </c>
       <c r="S37" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
@@ -5274,7 +5268,7 @@
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
@@ -5291,24 +5285,24 @@
       <c r="M39" s="9" t="n"/>
       <c r="N39" s="10" t="n"/>
       <c r="R39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5323,16 +5317,16 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>thommyspine</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
@@ -5355,13 +5349,13 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
@@ -5390,12 +5384,12 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -5406,25 +5400,22 @@
       <c r="L43" s="10" t="n"/>
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="10" t="n"/>
-      <c r="R43" t="n">
-        <v>0</v>
-      </c>
       <c r="S43" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T43" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5435,25 +5426,22 @@
       <c r="L44" s="10" t="n"/>
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="10" t="n"/>
-      <c r="R44" t="n">
-        <v>0</v>
-      </c>
       <c r="S44" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5468,18 +5456,18 @@
         <v>6</v>
       </c>
       <c r="T45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5490,9 +5478,6 @@
       <c r="L46" s="10" t="n"/>
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="10" t="n"/>
-      <c r="S46" t="n">
-        <v>0</v>
-      </c>
       <c r="T46" t="n">
         <v>0</v>
       </c>
@@ -5500,12 +5485,12 @@
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C47" s="13">
@@ -5516,17 +5501,14 @@
       <c r="L47" s="10" t="n"/>
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="10" t="n"/>
-      <c r="S47" t="n">
-        <v>6</v>
-      </c>
       <c r="T47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>jacopo</t>
+          <t>Samu-Nighix</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
@@ -5543,13 +5525,13 @@
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="10" t="n"/>
       <c r="T48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>Marchi™</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
@@ -5566,18 +5548,18 @@
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="10" t="n"/>
       <c r="T49" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Samu-Nighix</t>
+          <t>Ernis</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5589,29 +5571,6 @@
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="10" t="n"/>
       <c r="T50" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>Marchi™</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>14/03/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="T51" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-16
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3129,7 +3129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3577,7 +3577,7 @@
         <v>6</v>
       </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -3644,7 +3644,7 @@
         <v>6</v>
       </c>
       <c r="T7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -3760,7 +3760,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -3958,18 +3958,21 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Giorgio</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>29/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C13" s="13">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
+      <c r="H13" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="I13" s="9" t="n">
         <v>6</v>
       </c>
@@ -3980,7 +3983,7 @@
         <v>6</v>
       </c>
       <c r="L13" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M13" s="9" t="n">
         <v>6</v>
@@ -4010,18 +4013,30 @@
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C14" s="13">
         <f>ROUND(AVERAGE(D14:AH14), 0)</f>
         <v/>
       </c>
+      <c r="D14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="H14" s="9" t="n">
         <v>6</v>
       </c>
@@ -4065,7 +4080,7 @@
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -4087,43 +4102,40 @@
         <v>6</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K15" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L15" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M15" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N15" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="n">
         <v>6</v>
       </c>
       <c r="R15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T15" t="n">
         <v>6</v>
@@ -4132,89 +4144,92 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C16" s="13">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="D16" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K16" s="10" t="n"/>
+      <c r="L16" s="10" t="n"/>
       <c r="M16" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N16" s="33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q16" t="n">
         <v>6</v>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C17" s="13">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="n"/>
+      <c r="D17" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O17" t="n">
         <v>6</v>
@@ -4238,50 +4253,25 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C18" s="13">
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
-      <c r="D18" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J18" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K18" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L18" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="K18" s="10" t="n"/>
+      <c r="L18" s="10" t="n"/>
       <c r="M18" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N18" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
         <v>6</v>
@@ -4305,25 +4295,41 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C19" s="13">
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
-      <c r="K19" s="10" t="n"/>
-      <c r="L19" s="10" t="n"/>
+      <c r="G19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L19" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M19" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N19" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O19" t="n">
         <v>6</v>
@@ -4341,13 +4347,13 @@
         <v>6</v>
       </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -4359,11 +4365,20 @@
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
+      <c r="D20" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I20" s="9" t="n">
         <v>6</v>
@@ -4372,16 +4387,16 @@
         <v>6</v>
       </c>
       <c r="K20" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L20" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N20" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
         <v>6</v>
@@ -4405,7 +4420,7 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
@@ -4417,20 +4432,11 @@
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="D21" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G21" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I21" s="9" t="n">
         <v>6</v>
@@ -4439,16 +4445,16 @@
         <v>6</v>
       </c>
       <c r="K21" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L21" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M21" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N21" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O21" t="n">
         <v>6</v>
@@ -4472,7 +4478,7 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
@@ -4485,7 +4491,7 @@
         <v/>
       </c>
       <c r="G22" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H22" s="9" t="n">
         <v>6</v>
@@ -4530,33 +4536,18 @@
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C23" s="13">
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
-      <c r="G23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J23" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K23" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L23" s="10" t="n">
         <v>6</v>
       </c>
@@ -4588,18 +4579,21 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C24" s="13">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
+      <c r="K24" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L24" s="10" t="n">
         <v>6</v>
       </c>
@@ -4631,18 +4625,39 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C25" s="13">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
+      <c r="D25" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K25" s="10" t="n">
         <v>6</v>
       </c>
@@ -4671,13 +4686,13 @@
         <v>6</v>
       </c>
       <c r="T25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
@@ -4690,7 +4705,7 @@
         <v/>
       </c>
       <c r="D26" s="14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E26" s="9" t="n">
         <v>6</v>
@@ -4708,7 +4723,7 @@
         <v>6</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K26" s="10" t="n">
         <v>6</v>
@@ -4738,13 +4753,13 @@
         <v>6</v>
       </c>
       <c r="T26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
@@ -4757,7 +4772,7 @@
         <v/>
       </c>
       <c r="D27" s="14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E27" s="9" t="n">
         <v>6</v>
@@ -4775,7 +4790,7 @@
         <v>6</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K27" s="10" t="n">
         <v>6</v>
@@ -4811,7 +4826,7 @@
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
@@ -4823,27 +4838,7 @@
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
-      <c r="D28" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J28" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="J28" s="10" t="n"/>
       <c r="K28" s="10" t="n">
         <v>6</v>
       </c>
@@ -4878,7 +4873,7 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -4890,7 +4885,18 @@
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="J29" s="10" t="n"/>
+      <c r="G29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K29" s="10" t="n">
         <v>6</v>
       </c>
@@ -4900,14 +4906,14 @@
       <c r="M29" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N29" s="33" t="n">
+      <c r="N29" s="10" t="n">
         <v>6</v>
       </c>
       <c r="O29" t="n">
         <v>6</v>
       </c>
       <c r="P29" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q29" t="n">
         <v>6</v>
@@ -4925,30 +4931,18 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C30" s="13">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
-      <c r="G30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K30" s="10" t="n">
         <v>6</v>
       </c>
@@ -4956,59 +4950,51 @@
         <v>6</v>
       </c>
       <c r="M30" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N30" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O30" t="n">
         <v>6</v>
       </c>
       <c r="P30" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q30" t="n">
         <v>6</v>
       </c>
       <c r="R30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C31" s="13">
         <f>ROUND(AVERAGE(D31:AH31), 0)</f>
         <v/>
       </c>
-      <c r="K31" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L31" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K31" s="10" t="n"/>
+      <c r="L31" s="10" t="n"/>
+      <c r="M31" s="9" t="n"/>
+      <c r="N31" s="10" t="n"/>
       <c r="O31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P31" t="n">
         <v>6</v>
@@ -5017,19 +5003,19 @@
         <v>6</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
@@ -5046,13 +5032,13 @@
       <c r="M32" s="9" t="n"/>
       <c r="N32" s="10" t="n"/>
       <c r="O32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R32" t="n">
         <v>6</v>
@@ -5067,12 +5053,12 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C33" s="13">
@@ -5083,14 +5069,11 @@
       <c r="L33" s="10" t="n"/>
       <c r="M33" s="9" t="n"/>
       <c r="N33" s="10" t="n"/>
-      <c r="O33" t="n">
-        <v>6</v>
-      </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R33" t="n">
         <v>6</v>
@@ -5099,13 +5082,13 @@
         <v>6</v>
       </c>
       <c r="T33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>terracrom</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
@@ -5122,30 +5105,30 @@
       <c r="M34" s="9" t="n"/>
       <c r="N34" s="10" t="n"/>
       <c r="P34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
@@ -5157,16 +5140,16 @@
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="10" t="n"/>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T35" t="n">
         <v>0</v>
@@ -5175,12 +5158,12 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C36" s="13">
@@ -5191,26 +5174,20 @@
       <c r="L36" s="10" t="n"/>
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="10" t="n"/>
-      <c r="P36" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>2</v>
-      </c>
       <c r="R36" t="n">
         <v>6</v>
       </c>
       <c r="S36" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
@@ -5239,7 +5216,7 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
@@ -5256,24 +5233,24 @@
       <c r="M38" s="9" t="n"/>
       <c r="N38" s="10" t="n"/>
       <c r="R38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5288,16 +5265,16 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
@@ -5317,16 +5294,16 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
@@ -5346,21 +5323,21 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5371,9 +5348,6 @@
       <c r="L42" s="10" t="n"/>
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="10" t="n"/>
-      <c r="R42" t="n">
-        <v>0</v>
-      </c>
       <c r="S42" t="n">
         <v>6</v>
       </c>
@@ -5384,7 +5358,7 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
@@ -5401,21 +5375,21 @@
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="10" t="n"/>
       <c r="S43" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5427,21 +5401,21 @@
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="10" t="n"/>
       <c r="S44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T44" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5452,17 +5426,14 @@
       <c r="L45" s="10" t="n"/>
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="10" t="n"/>
-      <c r="S45" t="n">
-        <v>6</v>
-      </c>
       <c r="T45" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>jacopo</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
@@ -5479,13 +5450,13 @@
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="10" t="n"/>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>Samu-Nighix</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
@@ -5502,13 +5473,13 @@
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="10" t="n"/>
       <c r="T47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Samu-Nighix</t>
+          <t>Marchi™</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
@@ -5525,18 +5496,18 @@
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="10" t="n"/>
       <c r="T48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>Marchi™</t>
+          <t>Ernis</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5554,12 +5525,12 @@
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Ernis</t>
+          <t>Spiderman</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5571,6 +5542,29 @@
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="10" t="n"/>
       <c r="T50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>king</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="13">
+        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="10" t="n"/>
+      <c r="L51" s="10" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="10" t="n"/>
+      <c r="T51" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-03-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -763,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA48"/>
+  <dimension ref="A1:AA51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="25" min="1" max="1"/>
@@ -919,58 +919,54 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>¥CATA¥</t>
-        </is>
-      </c>
-      <c r="B2" s="26" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>655321</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
       </c>
-      <c r="C2" s="16">
+      <c r="C2" s="19">
         <f>ROUND(AVERAGE(F2:AB2), 0)</f>
         <v/>
       </c>
-      <c r="D2" s="29">
+      <c r="D2" s="1">
         <f>SUM(F2:AB2)</f>
         <v/>
       </c>
-      <c r="E2" s="23" t="n">
-        <v>32505</v>
-      </c>
-      <c r="F2" s="17" t="n"/>
-      <c r="G2" s="17" t="n"/>
-      <c r="H2" s="17" t="n"/>
-      <c r="I2" s="17" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J2" s="17" t="n">
-        <v>2950</v>
-      </c>
-      <c r="K2" s="17" t="n"/>
-      <c r="L2" s="17" t="n"/>
-      <c r="M2" s="17" t="n"/>
-      <c r="N2" s="17" t="n"/>
-      <c r="O2" s="17" t="n"/>
-      <c r="P2" s="17" t="n"/>
-      <c r="Q2" s="17" t="n"/>
-      <c r="R2" s="17" t="n"/>
-      <c r="S2" s="17" t="n"/>
-      <c r="T2" s="17" t="n"/>
-      <c r="U2" s="17" t="n"/>
-      <c r="V2" s="17" t="n"/>
-      <c r="W2" s="17" t="n"/>
-      <c r="X2" s="18" t="n"/>
-      <c r="Y2" s="18" t="n"/>
-      <c r="Z2" s="18" t="n"/>
-      <c r="AA2" s="18" t="n"/>
+      <c r="E2" s="24" t="n">
+        <v>6800</v>
+      </c>
+      <c r="F2" s="33" t="n"/>
+      <c r="G2" s="33" t="n"/>
+      <c r="H2" s="33" t="n"/>
+      <c r="I2" s="33" t="n">
+        <v>4150</v>
+      </c>
+      <c r="J2" s="33" t="n">
+        <v>2650</v>
+      </c>
+      <c r="K2" s="33" t="n"/>
+      <c r="L2" s="33" t="n"/>
+      <c r="M2" s="33" t="n"/>
+      <c r="N2" s="33" t="n"/>
+      <c r="O2" s="33" t="n"/>
+      <c r="P2" s="33" t="n"/>
+      <c r="Q2" s="33" t="n"/>
+      <c r="R2" s="33" t="n"/>
+      <c r="S2" s="33" t="n"/>
+      <c r="T2" s="33" t="n"/>
+      <c r="U2" s="33" t="n"/>
+      <c r="V2" s="33" t="n"/>
+      <c r="W2" s="33" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B3" s="27" t="inlineStr">
@@ -987,16 +983,16 @@
         <v/>
       </c>
       <c r="E3" s="24" t="n">
-        <v>6800</v>
+        <v>28225</v>
       </c>
       <c r="F3" s="33" t="n"/>
       <c r="G3" s="33" t="n"/>
       <c r="H3" s="33" t="n"/>
       <c r="I3" s="33" t="n">
-        <v>4150</v>
+        <v>2000</v>
       </c>
       <c r="J3" s="33" t="n">
-        <v>2650</v>
+        <v>8000</v>
       </c>
       <c r="K3" s="33" t="n"/>
       <c r="L3" s="33" t="n"/>
@@ -1015,7 +1011,7 @@
     <row r="4">
       <c r="A4" s="24" t="inlineStr">
         <is>
-          <t>ajejebrazorf</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B4" s="27" t="inlineStr">
@@ -1032,20 +1028,18 @@
         <v/>
       </c>
       <c r="E4" s="24" t="n">
-        <v>16500</v>
+        <v>15150</v>
       </c>
       <c r="F4" s="33" t="n"/>
-      <c r="G4" s="33" t="n">
-        <v>4000</v>
-      </c>
+      <c r="G4" s="33" t="n"/>
       <c r="H4" s="33" t="n">
-        <v>3400</v>
+        <v>500</v>
       </c>
       <c r="I4" s="33" t="n">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="J4" s="33" t="n">
-        <v>4050</v>
+        <v>0</v>
       </c>
       <c r="K4" s="33" t="n"/>
       <c r="L4" s="33" t="n"/>
@@ -1064,12 +1058,12 @@
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C5" s="19">
@@ -1081,16 +1075,22 @@
         <v/>
       </c>
       <c r="E5" s="24" t="n">
-        <v>28225</v>
-      </c>
-      <c r="F5" s="33" t="n"/>
-      <c r="G5" s="33" t="n"/>
-      <c r="H5" s="33" t="n"/>
+        <v>32200</v>
+      </c>
+      <c r="F5" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G5" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H5" s="33" t="n">
+        <v>4100</v>
+      </c>
       <c r="I5" s="33" t="n">
-        <v>2000</v>
+        <v>4400</v>
       </c>
       <c r="J5" s="33" t="n">
-        <v>8000</v>
+        <v>4700</v>
       </c>
       <c r="K5" s="33" t="n"/>
       <c r="L5" s="33" t="n"/>
@@ -1109,7 +1109,7 @@
     <row r="6">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B6" s="27" t="inlineStr">
@@ -1126,15 +1126,17 @@
         <v/>
       </c>
       <c r="E6" s="24" t="n">
-        <v>15150</v>
+        <v>12250</v>
       </c>
       <c r="F6" s="33" t="n"/>
-      <c r="G6" s="33" t="n"/>
+      <c r="G6" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="H6" s="33" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="I6" s="33" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="J6" s="33" t="n">
         <v>0</v>
@@ -1156,7 +1158,7 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
@@ -1173,22 +1175,18 @@
         <v/>
       </c>
       <c r="E7" s="24" t="n">
-        <v>32200</v>
-      </c>
-      <c r="F7" s="33" t="n">
+        <v>41000</v>
+      </c>
+      <c r="F7" s="33" t="n"/>
+      <c r="G7" s="33" t="n"/>
+      <c r="H7" s="33" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I7" s="33" t="n">
         <v>4000</v>
       </c>
-      <c r="G7" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H7" s="33" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I7" s="33" t="n">
-        <v>4400</v>
-      </c>
       <c r="J7" s="33" t="n">
-        <v>4700</v>
+        <v>150</v>
       </c>
       <c r="K7" s="33" t="n"/>
       <c r="L7" s="33" t="n"/>
@@ -1207,7 +1205,7 @@
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B8" s="27" t="inlineStr">
@@ -1224,20 +1222,18 @@
         <v/>
       </c>
       <c r="E8" s="24" t="n">
-        <v>12250</v>
+        <v>29350</v>
       </c>
       <c r="F8" s="33" t="n"/>
-      <c r="G8" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="G8" s="33" t="n"/>
       <c r="H8" s="33" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="33" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="J8" s="33" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="K8" s="33" t="n"/>
       <c r="L8" s="33" t="n"/>
@@ -1256,7 +1252,7 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>ER DANDI 1927</t>
         </is>
       </c>
       <c r="B9" s="27" t="inlineStr">
@@ -1273,18 +1269,18 @@
         <v/>
       </c>
       <c r="E9" s="24" t="n">
-        <v>41000</v>
+        <v>73250</v>
       </c>
       <c r="F9" s="33" t="n"/>
       <c r="G9" s="33" t="n"/>
       <c r="H9" s="33" t="n">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="I9" s="33" t="n">
         <v>4000</v>
       </c>
       <c r="J9" s="33" t="n">
-        <v>150</v>
+        <v>3000</v>
       </c>
       <c r="K9" s="33" t="n"/>
       <c r="L9" s="33" t="n"/>
@@ -1303,7 +1299,7 @@
     <row r="10">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B10" s="27" t="inlineStr">
@@ -1320,15 +1316,19 @@
         <v/>
       </c>
       <c r="E10" s="24" t="n">
-        <v>29350</v>
-      </c>
-      <c r="F10" s="33" t="n"/>
-      <c r="G10" s="33" t="n"/>
+        <v>33700</v>
+      </c>
+      <c r="F10" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G10" s="33" t="n">
+        <v>4000</v>
+      </c>
       <c r="H10" s="33" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I10" s="33" t="n">
-        <v>3500</v>
+        <v>2450</v>
       </c>
       <c r="J10" s="33" t="n">
         <v>4050</v>
@@ -1350,7 +1350,7 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B11" s="27" t="inlineStr">
@@ -1367,18 +1367,20 @@
         <v/>
       </c>
       <c r="E11" s="24" t="n">
-        <v>73250</v>
+        <v>22000</v>
       </c>
       <c r="F11" s="33" t="n"/>
-      <c r="G11" s="33" t="n"/>
+      <c r="G11" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="H11" s="33" t="n">
-        <v>1300</v>
+        <v>6050</v>
       </c>
       <c r="I11" s="33" t="n">
-        <v>4000</v>
+        <v>8300</v>
       </c>
       <c r="J11" s="33" t="n">
-        <v>3000</v>
+        <v>5950</v>
       </c>
       <c r="K11" s="33" t="n"/>
       <c r="L11" s="33" t="n"/>
@@ -1397,12 +1399,12 @@
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C12" s="19">
@@ -1414,22 +1416,18 @@
         <v/>
       </c>
       <c r="E12" s="24" t="n">
-        <v>33700</v>
-      </c>
-      <c r="F12" s="33" t="n">
+        <v>123800</v>
+      </c>
+      <c r="F12" s="33" t="n"/>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="33" t="n">
+        <v>4050</v>
+      </c>
+      <c r="I12" s="33" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J12" s="33" t="n">
         <v>4000</v>
-      </c>
-      <c r="G12" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H12" s="33" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I12" s="33" t="n">
-        <v>2450</v>
-      </c>
-      <c r="J12" s="33" t="n">
-        <v>4050</v>
       </c>
       <c r="K12" s="33" t="n"/>
       <c r="L12" s="33" t="n"/>
@@ -1448,7 +1446,7 @@
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B13" s="27" t="inlineStr">
@@ -1465,20 +1463,22 @@
         <v/>
       </c>
       <c r="E13" s="24" t="n">
-        <v>22000</v>
-      </c>
-      <c r="F13" s="33" t="n"/>
+        <v>47650</v>
+      </c>
+      <c r="F13" s="33" t="n">
+        <v>4000</v>
+      </c>
       <c r="G13" s="33" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>6050</v>
+        <v>10000</v>
       </c>
       <c r="I13" s="33" t="n">
-        <v>8300</v>
+        <v>10000</v>
       </c>
       <c r="J13" s="33" t="n">
-        <v>5950</v>
+        <v>10000</v>
       </c>
       <c r="K13" s="33" t="n"/>
       <c r="L13" s="33" t="n"/>
@@ -1497,12 +1497,12 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>Giorgio</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>26/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C14" s="19">
@@ -1514,18 +1514,20 @@
         <v/>
       </c>
       <c r="E14" s="24" t="n">
-        <v>27050</v>
+        <v>33550</v>
       </c>
       <c r="F14" s="33" t="n"/>
-      <c r="G14" s="33" t="n"/>
+      <c r="G14" s="33" t="n">
+        <v>4000</v>
+      </c>
       <c r="H14" s="33" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I14" s="33" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="J14" s="33" t="n">
-        <v>5100</v>
+        <v>5050</v>
       </c>
       <c r="K14" s="33" t="n"/>
       <c r="L14" s="33" t="n"/>
@@ -1544,12 +1546,12 @@
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C15" s="19">
@@ -1561,18 +1563,16 @@
         <v/>
       </c>
       <c r="E15" s="24" t="n">
-        <v>123800</v>
+        <v>75000</v>
       </c>
       <c r="F15" s="33" t="n"/>
       <c r="G15" s="33" t="n"/>
-      <c r="H15" s="33" t="n">
-        <v>4050</v>
-      </c>
+      <c r="H15" s="33" t="n"/>
       <c r="I15" s="33" t="n">
-        <v>4100</v>
+        <v>0</v>
       </c>
       <c r="J15" s="33" t="n">
-        <v>4000</v>
+        <v>950</v>
       </c>
       <c r="K15" s="33" t="n"/>
       <c r="L15" s="33" t="n"/>
@@ -1591,12 +1591,12 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>GioStyle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="19">
@@ -1608,16 +1608,20 @@
         <v/>
       </c>
       <c r="E16" s="24" t="n">
-        <v>65520</v>
+        <v>55400</v>
       </c>
       <c r="F16" s="33" t="n"/>
-      <c r="G16" s="33" t="n"/>
-      <c r="H16" s="33" t="n"/>
+      <c r="G16" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H16" s="33" t="n">
+        <v>10000</v>
+      </c>
       <c r="I16" s="33" t="n">
-        <v>6350</v>
+        <v>10000</v>
       </c>
       <c r="J16" s="33" t="n">
-        <v>4500</v>
+        <v>10000</v>
       </c>
       <c r="K16" s="33" t="n"/>
       <c r="L16" s="33" t="n"/>
@@ -1636,12 +1640,12 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C17" s="19">
@@ -1653,22 +1657,16 @@
         <v/>
       </c>
       <c r="E17" s="24" t="n">
-        <v>47650</v>
-      </c>
-      <c r="F17" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G17" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H17" s="33" t="n">
-        <v>10000</v>
-      </c>
+        <v>65375</v>
+      </c>
+      <c r="F17" s="33" t="n"/>
+      <c r="G17" s="33" t="n"/>
+      <c r="H17" s="33" t="n"/>
       <c r="I17" s="33" t="n">
-        <v>10000</v>
+        <v>6250</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>10000</v>
+        <v>3250</v>
       </c>
       <c r="K17" s="33" t="n"/>
       <c r="L17" s="33" t="n"/>
@@ -1687,7 +1685,7 @@
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -1704,23 +1702,21 @@
         <v/>
       </c>
       <c r="E18" s="24" t="n">
-        <v>33550</v>
+        <v>56300</v>
       </c>
       <c r="F18" s="33" t="n"/>
-      <c r="G18" s="33" t="n">
-        <v>4000</v>
-      </c>
+      <c r="G18" s="33" t="n"/>
       <c r="H18" s="33" t="n">
         <v>10000</v>
       </c>
       <c r="I18" s="33" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="J18" s="33" t="n">
-        <v>5050</v>
+        <v>10000</v>
       </c>
       <c r="K18" s="33" t="n"/>
-      <c r="L18" s="33" t="n"/>
+      <c r="L18" s="21" t="n"/>
       <c r="M18" s="33" t="n"/>
       <c r="N18" s="33" t="n"/>
       <c r="O18" s="33" t="n"/>
@@ -1736,12 +1732,12 @@
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C19" s="19">
@@ -1753,16 +1749,22 @@
         <v/>
       </c>
       <c r="E19" s="24" t="n">
-        <v>75000</v>
-      </c>
-      <c r="F19" s="33" t="n"/>
-      <c r="G19" s="33" t="n"/>
-      <c r="H19" s="33" t="n"/>
+        <v>33050</v>
+      </c>
+      <c r="F19" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G19" s="33" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H19" s="33" t="n">
+        <v>5800</v>
+      </c>
       <c r="I19" s="33" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="J19" s="33" t="n">
-        <v>950</v>
+        <v>4350</v>
       </c>
       <c r="K19" s="33" t="n"/>
       <c r="L19" s="33" t="n"/>
@@ -1781,7 +1783,7 @@
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
@@ -1798,12 +1800,10 @@
         <v/>
       </c>
       <c r="E20" s="24" t="n">
-        <v>55400</v>
+        <v>58700</v>
       </c>
       <c r="F20" s="33" t="n"/>
-      <c r="G20" s="33" t="n">
-        <v>4000</v>
-      </c>
+      <c r="G20" s="33" t="n"/>
       <c r="H20" s="33" t="n">
         <v>10000</v>
       </c>
@@ -1830,12 +1830,12 @@
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C21" s="19">
@@ -1847,16 +1847,18 @@
         <v/>
       </c>
       <c r="E21" s="24" t="n">
-        <v>65375</v>
+        <v>51200</v>
       </c>
       <c r="F21" s="33" t="n"/>
       <c r="G21" s="33" t="n"/>
-      <c r="H21" s="33" t="n"/>
+      <c r="H21" s="33" t="n">
+        <v>10000</v>
+      </c>
       <c r="I21" s="33" t="n">
-        <v>6250</v>
+        <v>10000</v>
       </c>
       <c r="J21" s="33" t="n">
-        <v>3250</v>
+        <v>10000</v>
       </c>
       <c r="K21" s="33" t="n"/>
       <c r="L21" s="33" t="n"/>
@@ -1875,12 +1877,12 @@
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C22" s="19">
@@ -1892,13 +1894,11 @@
         <v/>
       </c>
       <c r="E22" s="24" t="n">
-        <v>56300</v>
+        <v>106725</v>
       </c>
       <c r="F22" s="33" t="n"/>
       <c r="G22" s="33" t="n"/>
-      <c r="H22" s="33" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H22" s="33" t="n"/>
       <c r="I22" s="33" t="n">
         <v>10000</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>10000</v>
       </c>
       <c r="K22" s="33" t="n"/>
-      <c r="L22" s="21" t="n"/>
+      <c r="L22" s="33" t="n"/>
       <c r="M22" s="33" t="n"/>
       <c r="N22" s="33" t="n"/>
       <c r="O22" s="33" t="n"/>
@@ -1922,12 +1922,12 @@
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>Luxor</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C23" s="19">
@@ -1939,22 +1939,16 @@
         <v/>
       </c>
       <c r="E23" s="24" t="n">
-        <v>6175</v>
-      </c>
-      <c r="F23" s="33" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G23" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="33" t="n">
-        <v>0</v>
-      </c>
+        <v>44550</v>
+      </c>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="33" t="n"/>
       <c r="I23" s="33" t="n">
-        <v>1150</v>
+        <v>4300</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>0</v>
+        <v>4100</v>
       </c>
       <c r="K23" s="33" t="n"/>
       <c r="L23" s="33" t="n"/>
@@ -1973,7 +1967,7 @@
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B24" s="27" t="inlineStr">
@@ -1990,22 +1984,22 @@
         <v/>
       </c>
       <c r="E24" s="24" t="n">
-        <v>33050</v>
+        <v>39900</v>
       </c>
       <c r="F24" s="33" t="n">
         <v>4000</v>
       </c>
       <c r="G24" s="33" t="n">
-        <v>2100</v>
+        <v>4000</v>
       </c>
       <c r="H24" s="33" t="n">
-        <v>5800</v>
+        <v>4050</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>4050</v>
+        <v>5600</v>
       </c>
       <c r="J24" s="33" t="n">
-        <v>4350</v>
+        <v>1300</v>
       </c>
       <c r="K24" s="33" t="n"/>
       <c r="L24" s="33" t="n"/>
@@ -2024,7 +2018,7 @@
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B25" s="27" t="inlineStr">
@@ -2041,18 +2035,20 @@
         <v/>
       </c>
       <c r="E25" s="24" t="n">
-        <v>58700</v>
+        <v>27500</v>
       </c>
       <c r="F25" s="33" t="n"/>
-      <c r="G25" s="33" t="n"/>
+      <c r="G25" s="33" t="n">
+        <v>4000</v>
+      </c>
       <c r="H25" s="33" t="n">
         <v>10000</v>
       </c>
       <c r="I25" s="33" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="J25" s="33" t="n">
-        <v>10000</v>
+        <v>4300</v>
       </c>
       <c r="K25" s="33" t="n"/>
       <c r="L25" s="33" t="n"/>
@@ -2071,7 +2067,7 @@
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B26" s="27" t="inlineStr">
@@ -2088,18 +2084,22 @@
         <v/>
       </c>
       <c r="E26" s="24" t="n">
-        <v>51200</v>
-      </c>
-      <c r="F26" s="33" t="n"/>
-      <c r="G26" s="33" t="n"/>
+        <v>33025</v>
+      </c>
+      <c r="F26" s="33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G26" s="33" t="n">
+        <v>4000</v>
+      </c>
       <c r="H26" s="33" t="n">
-        <v>10000</v>
+        <v>4050</v>
       </c>
       <c r="I26" s="33" t="n">
-        <v>10000</v>
+        <v>4850</v>
       </c>
       <c r="J26" s="33" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="K26" s="33" t="n"/>
       <c r="L26" s="33" t="n"/>
@@ -2118,12 +2118,12 @@
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B27" s="27" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C27" s="19">
@@ -2135,16 +2135,18 @@
         <v/>
       </c>
       <c r="E27" s="24" t="n">
-        <v>106725</v>
+        <v>31825</v>
       </c>
       <c r="F27" s="33" t="n"/>
       <c r="G27" s="33" t="n"/>
-      <c r="H27" s="33" t="n"/>
+      <c r="H27" s="33" t="n">
+        <v>3650</v>
+      </c>
       <c r="I27" s="33" t="n">
-        <v>10000</v>
+        <v>7600</v>
       </c>
       <c r="J27" s="33" t="n">
-        <v>10000</v>
+        <v>3150</v>
       </c>
       <c r="K27" s="33" t="n"/>
       <c r="L27" s="33" t="n"/>
@@ -2163,12 +2165,12 @@
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C28" s="19">
@@ -2180,16 +2182,18 @@
         <v/>
       </c>
       <c r="E28" s="24" t="n">
-        <v>44550</v>
+        <v>109220</v>
       </c>
       <c r="F28" s="33" t="n"/>
       <c r="G28" s="33" t="n"/>
-      <c r="H28" s="33" t="n"/>
+      <c r="H28" s="33" t="n">
+        <v>3850</v>
+      </c>
       <c r="I28" s="33" t="n">
-        <v>4300</v>
+        <v>10000</v>
       </c>
       <c r="J28" s="33" t="n">
-        <v>4100</v>
+        <v>0</v>
       </c>
       <c r="K28" s="33" t="n"/>
       <c r="L28" s="33" t="n"/>
@@ -2208,12 +2212,12 @@
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C29" s="19">
@@ -2225,22 +2229,16 @@
         <v/>
       </c>
       <c r="E29" s="24" t="n">
-        <v>39900</v>
-      </c>
-      <c r="F29" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G29" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H29" s="33" t="n">
-        <v>4050</v>
-      </c>
+        <v>69000</v>
+      </c>
+      <c r="F29" s="33" t="n"/>
+      <c r="G29" s="33" t="n"/>
+      <c r="H29" s="33" t="n"/>
       <c r="I29" s="33" t="n">
-        <v>5600</v>
+        <v>10000</v>
       </c>
       <c r="J29" s="33" t="n">
-        <v>1300</v>
+        <v>10000</v>
       </c>
       <c r="K29" s="33" t="n"/>
       <c r="L29" s="33" t="n"/>
@@ -2259,12 +2257,12 @@
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>Roberta</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C30" s="19">
@@ -2276,20 +2274,14 @@
         <v/>
       </c>
       <c r="E30" s="24" t="n">
-        <v>19530</v>
+        <v>76700</v>
       </c>
       <c r="F30" s="33" t="n"/>
-      <c r="G30" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H30" s="33" t="n">
-        <v>5150</v>
-      </c>
-      <c r="I30" s="33" t="n">
-        <v>2500</v>
-      </c>
+      <c r="G30" s="33" t="n"/>
+      <c r="H30" s="33" t="n"/>
+      <c r="I30" s="33" t="n"/>
       <c r="J30" s="33" t="n">
-        <v>1600</v>
+        <v>5000</v>
       </c>
       <c r="K30" s="33" t="n"/>
       <c r="L30" s="33" t="n"/>
@@ -2308,12 +2300,12 @@
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B31" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C31" s="19">
@@ -2325,20 +2317,14 @@
         <v/>
       </c>
       <c r="E31" s="24" t="n">
-        <v>27500</v>
+        <v>27155</v>
       </c>
       <c r="F31" s="33" t="n"/>
-      <c r="G31" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H31" s="33" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I31" s="33" t="n">
-        <v>4500</v>
-      </c>
+      <c r="G31" s="33" t="n"/>
+      <c r="H31" s="33" t="n"/>
+      <c r="I31" s="33" t="n"/>
       <c r="J31" s="33" t="n">
-        <v>4300</v>
+        <v>4250</v>
       </c>
       <c r="K31" s="33" t="n"/>
       <c r="L31" s="33" t="n"/>
@@ -2357,12 +2343,12 @@
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C32" s="19">
@@ -2374,22 +2360,14 @@
         <v/>
       </c>
       <c r="E32" s="24" t="n">
-        <v>33025</v>
-      </c>
-      <c r="F32" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G32" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H32" s="33" t="n">
-        <v>4050</v>
-      </c>
-      <c r="I32" s="33" t="n">
-        <v>4850</v>
-      </c>
+        <v>31350</v>
+      </c>
+      <c r="F32" s="33" t="n"/>
+      <c r="G32" s="33" t="n"/>
+      <c r="H32" s="33" t="n"/>
+      <c r="I32" s="33" t="n"/>
       <c r="J32" s="33" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
       <c r="K32" s="33" t="n"/>
       <c r="L32" s="33" t="n"/>
@@ -2408,12 +2386,12 @@
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B33" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C33" s="19">
@@ -2425,18 +2403,14 @@
         <v/>
       </c>
       <c r="E33" s="24" t="n">
-        <v>31825</v>
+        <v>23750</v>
       </c>
       <c r="F33" s="33" t="n"/>
       <c r="G33" s="33" t="n"/>
-      <c r="H33" s="33" t="n">
-        <v>3650</v>
-      </c>
-      <c r="I33" s="33" t="n">
-        <v>7600</v>
-      </c>
+      <c r="H33" s="33" t="n"/>
+      <c r="I33" s="33" t="n"/>
       <c r="J33" s="33" t="n">
-        <v>3150</v>
+        <v>4300</v>
       </c>
       <c r="K33" s="33" t="n"/>
       <c r="L33" s="33" t="n"/>
@@ -2455,12 +2429,12 @@
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>th4nos</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="C34" s="19">
@@ -2472,22 +2446,14 @@
         <v/>
       </c>
       <c r="E34" s="24" t="n">
-        <v>35900</v>
-      </c>
-      <c r="F34" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G34" s="33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H34" s="33" t="n">
-        <v>5750</v>
-      </c>
-      <c r="I34" s="33" t="n">
-        <v>4500</v>
-      </c>
+        <v>11775</v>
+      </c>
+      <c r="F34" s="33" t="n"/>
+      <c r="G34" s="33" t="n"/>
+      <c r="H34" s="33" t="n"/>
+      <c r="I34" s="33" t="n"/>
       <c r="J34" s="33" t="n">
-        <v>6450</v>
+        <v>0</v>
       </c>
       <c r="K34" s="33" t="n"/>
       <c r="L34" s="33" t="n"/>
@@ -2506,12 +2472,12 @@
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B35" s="27" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="C35" s="19">
@@ -2523,16 +2489,12 @@
         <v/>
       </c>
       <c r="E35" s="24" t="n">
-        <v>109220</v>
+        <v>21145</v>
       </c>
       <c r="F35" s="33" t="n"/>
       <c r="G35" s="33" t="n"/>
-      <c r="H35" s="33" t="n">
-        <v>3850</v>
-      </c>
-      <c r="I35" s="33" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H35" s="33" t="n"/>
+      <c r="I35" s="33" t="n"/>
       <c r="J35" s="33" t="n">
         <v>0</v>
       </c>
@@ -2553,12 +2515,12 @@
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="C36" s="19">
@@ -2570,16 +2532,14 @@
         <v/>
       </c>
       <c r="E36" s="24" t="n">
-        <v>69000</v>
+        <v>2150</v>
       </c>
       <c r="F36" s="33" t="n"/>
       <c r="G36" s="33" t="n"/>
       <c r="H36" s="33" t="n"/>
-      <c r="I36" s="33" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I36" s="33" t="n"/>
       <c r="J36" s="33" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K36" s="33" t="n"/>
       <c r="L36" s="33" t="n"/>
@@ -2598,12 +2558,12 @@
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>antony</t>
         </is>
       </c>
       <c r="B37" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C37" s="19">
@@ -2615,15 +2575,13 @@
         <v/>
       </c>
       <c r="E37" s="24" t="n">
-        <v>76700</v>
+        <v>22300</v>
       </c>
       <c r="F37" s="33" t="n"/>
       <c r="G37" s="33" t="n"/>
       <c r="H37" s="33" t="n"/>
       <c r="I37" s="33" t="n"/>
-      <c r="J37" s="33" t="n">
-        <v>5000</v>
-      </c>
+      <c r="J37" s="33" t="n"/>
       <c r="K37" s="33" t="n"/>
       <c r="L37" s="33" t="n"/>
       <c r="M37" s="33" t="n"/>
@@ -2641,12 +2599,12 @@
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B38" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C38" s="19">
@@ -2658,15 +2616,13 @@
         <v/>
       </c>
       <c r="E38" s="24" t="n">
-        <v>22075</v>
+        <v>26050</v>
       </c>
       <c r="F38" s="33" t="n"/>
       <c r="G38" s="33" t="n"/>
       <c r="H38" s="33" t="n"/>
       <c r="I38" s="33" t="n"/>
-      <c r="J38" s="33" t="n">
-        <v>1200</v>
-      </c>
+      <c r="J38" s="33" t="n"/>
       <c r="K38" s="33" t="n"/>
       <c r="L38" s="33" t="n"/>
       <c r="M38" s="33" t="n"/>
@@ -2684,12 +2640,12 @@
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B39" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C39" s="19">
@@ -2701,15 +2657,13 @@
         <v/>
       </c>
       <c r="E39" s="24" t="n">
-        <v>27155</v>
+        <v>1825</v>
       </c>
       <c r="F39" s="33" t="n"/>
       <c r="G39" s="33" t="n"/>
       <c r="H39" s="33" t="n"/>
       <c r="I39" s="33" t="n"/>
-      <c r="J39" s="33" t="n">
-        <v>4250</v>
-      </c>
+      <c r="J39" s="33" t="n"/>
       <c r="K39" s="33" t="n"/>
       <c r="L39" s="33" t="n"/>
       <c r="M39" s="33" t="n"/>
@@ -2727,12 +2681,12 @@
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>dibba10</t>
+          <t>TaifTuff</t>
         </is>
       </c>
       <c r="B40" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C40" s="19">
@@ -2744,15 +2698,13 @@
         <v/>
       </c>
       <c r="E40" s="24" t="n">
-        <v>13360</v>
+        <v>49005</v>
       </c>
       <c r="F40" s="33" t="n"/>
       <c r="G40" s="33" t="n"/>
       <c r="H40" s="33" t="n"/>
       <c r="I40" s="33" t="n"/>
-      <c r="J40" s="33" t="n">
-        <v>900</v>
-      </c>
+      <c r="J40" s="33" t="n"/>
       <c r="K40" s="33" t="n"/>
       <c r="L40" s="33" t="n"/>
       <c r="M40" s="33" t="n"/>
@@ -2770,12 +2722,12 @@
     <row r="41">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B41" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C41" s="19">
@@ -2787,15 +2739,13 @@
         <v/>
       </c>
       <c r="E41" s="24" t="n">
-        <v>31350</v>
+        <v>3550</v>
       </c>
       <c r="F41" s="33" t="n"/>
       <c r="G41" s="33" t="n"/>
       <c r="H41" s="33" t="n"/>
       <c r="I41" s="33" t="n"/>
-      <c r="J41" s="33" t="n">
-        <v>10000</v>
-      </c>
+      <c r="J41" s="33" t="n"/>
       <c r="K41" s="33" t="n"/>
       <c r="L41" s="33" t="n"/>
       <c r="M41" s="33" t="n"/>
@@ -2813,12 +2763,12 @@
     <row r="42">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>Spiderman</t>
         </is>
       </c>
       <c r="B42" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C42" s="19">
@@ -2830,15 +2780,13 @@
         <v/>
       </c>
       <c r="E42" s="24" t="n">
-        <v>400</v>
+        <v>23625</v>
       </c>
       <c r="F42" s="33" t="n"/>
       <c r="G42" s="33" t="n"/>
       <c r="H42" s="33" t="n"/>
       <c r="I42" s="33" t="n"/>
-      <c r="J42" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J42" s="33" t="n"/>
       <c r="K42" s="33" t="n"/>
       <c r="L42" s="33" t="n"/>
       <c r="M42" s="33" t="n"/>
@@ -2856,12 +2804,12 @@
     <row r="43">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>micky</t>
         </is>
       </c>
       <c r="B43" s="27" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C43" s="19">
@@ -2873,15 +2821,13 @@
         <v/>
       </c>
       <c r="E43" s="24" t="n">
-        <v>23750</v>
+        <v>16600</v>
       </c>
       <c r="F43" s="33" t="n"/>
       <c r="G43" s="33" t="n"/>
       <c r="H43" s="33" t="n"/>
       <c r="I43" s="33" t="n"/>
-      <c r="J43" s="33" t="n">
-        <v>4300</v>
-      </c>
+      <c r="J43" s="33" t="n"/>
       <c r="K43" s="33" t="n"/>
       <c r="L43" s="33" t="n"/>
       <c r="M43" s="33" t="n"/>
@@ -2899,12 +2845,12 @@
     <row r="44">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B44" s="27" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C44" s="19">
@@ -2916,15 +2862,13 @@
         <v/>
       </c>
       <c r="E44" s="24" t="n">
-        <v>11775</v>
+        <v>6550</v>
       </c>
       <c r="F44" s="33" t="n"/>
       <c r="G44" s="33" t="n"/>
       <c r="H44" s="33" t="n"/>
       <c r="I44" s="33" t="n"/>
-      <c r="J44" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J44" s="33" t="n"/>
       <c r="K44" s="33" t="n"/>
       <c r="L44" s="33" t="n"/>
       <c r="M44" s="33" t="n"/>
@@ -2942,12 +2886,12 @@
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B45" s="27" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C45" s="19">
@@ -2959,15 +2903,13 @@
         <v/>
       </c>
       <c r="E45" s="24" t="n">
-        <v>21145</v>
+        <v>0</v>
       </c>
       <c r="F45" s="33" t="n"/>
       <c r="G45" s="33" t="n"/>
       <c r="H45" s="33" t="n"/>
       <c r="I45" s="33" t="n"/>
-      <c r="J45" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J45" s="33" t="n"/>
       <c r="K45" s="33" t="n"/>
       <c r="L45" s="33" t="n"/>
       <c r="M45" s="33" t="n"/>
@@ -2985,12 +2927,12 @@
     <row r="46">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B46" s="27" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C46" s="19">
@@ -3002,15 +2944,13 @@
         <v/>
       </c>
       <c r="E46" s="24" t="n">
-        <v>2150</v>
+        <v>1800</v>
       </c>
       <c r="F46" s="33" t="n"/>
       <c r="G46" s="33" t="n"/>
       <c r="H46" s="33" t="n"/>
       <c r="I46" s="33" t="n"/>
-      <c r="J46" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J46" s="33" t="n"/>
       <c r="K46" s="33" t="n"/>
       <c r="L46" s="33" t="n"/>
       <c r="M46" s="33" t="n"/>
@@ -3028,12 +2968,12 @@
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>eltishqipe</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B47" s="27" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C47" s="19">
@@ -3045,15 +2985,13 @@
         <v/>
       </c>
       <c r="E47" s="24" t="n">
-        <v>20225</v>
+        <v>5500</v>
       </c>
       <c r="F47" s="33" t="n"/>
       <c r="G47" s="33" t="n"/>
       <c r="H47" s="33" t="n"/>
       <c r="I47" s="33" t="n"/>
-      <c r="J47" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J47" s="33" t="n"/>
       <c r="K47" s="33" t="n"/>
       <c r="L47" s="33" t="n"/>
       <c r="M47" s="33" t="n"/>
@@ -3071,12 +3009,12 @@
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>Xx_Herman_xX</t>
+          <t>Fra</t>
         </is>
       </c>
       <c r="B48" s="27" t="inlineStr">
         <is>
-          <t>27/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C48" s="19">
@@ -3088,15 +3026,13 @@
         <v/>
       </c>
       <c r="E48" s="24" t="n">
-        <v>11735</v>
+        <v>0</v>
       </c>
       <c r="F48" s="33" t="n"/>
       <c r="G48" s="33" t="n"/>
       <c r="H48" s="33" t="n"/>
       <c r="I48" s="33" t="n"/>
-      <c r="J48" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="J48" s="33" t="n"/>
       <c r="K48" s="33" t="n"/>
       <c r="L48" s="33" t="n"/>
       <c r="M48" s="33" t="n"/>
@@ -3111,7 +3047,129 @@
       <c r="V48" s="33" t="n"/>
       <c r="W48" s="33" t="n"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1" thickBot="1"/>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>EMANUELE</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="19">
+        <f>ROUND(AVERAGE(F49:AB49), 0)</f>
+        <v/>
+      </c>
+      <c r="D49" s="1">
+        <f>SUM(F49:AB49)</f>
+        <v/>
+      </c>
+      <c r="E49" s="24" t="n">
+        <v>150</v>
+      </c>
+      <c r="F49" s="33" t="n"/>
+      <c r="G49" s="33" t="n"/>
+      <c r="H49" s="33" t="n"/>
+      <c r="I49" s="33" t="n"/>
+      <c r="J49" s="33" t="n"/>
+      <c r="K49" s="33" t="n"/>
+      <c r="L49" s="33" t="n"/>
+      <c r="M49" s="33" t="n"/>
+      <c r="N49" s="33" t="n"/>
+      <c r="O49" s="33" t="n"/>
+      <c r="P49" s="33" t="n"/>
+      <c r="Q49" s="33" t="n"/>
+      <c r="R49" s="33" t="n"/>
+      <c r="S49" s="33" t="n"/>
+      <c r="T49" s="33" t="n"/>
+      <c r="U49" s="33" t="n"/>
+      <c r="V49" s="33" t="n"/>
+      <c r="W49" s="33" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>omar</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="19">
+        <f>ROUND(AVERAGE(F50:AB50), 0)</f>
+        <v/>
+      </c>
+      <c r="D50" s="1">
+        <f>SUM(F50:AB50)</f>
+        <v/>
+      </c>
+      <c r="E50" s="24" t="n">
+        <v>5350</v>
+      </c>
+      <c r="F50" s="33" t="n"/>
+      <c r="G50" s="33" t="n"/>
+      <c r="H50" s="33" t="n"/>
+      <c r="I50" s="33" t="n"/>
+      <c r="J50" s="33" t="n"/>
+      <c r="K50" s="33" t="n"/>
+      <c r="L50" s="33" t="n"/>
+      <c r="M50" s="33" t="n"/>
+      <c r="N50" s="33" t="n"/>
+      <c r="O50" s="33" t="n"/>
+      <c r="P50" s="33" t="n"/>
+      <c r="Q50" s="33" t="n"/>
+      <c r="R50" s="33" t="n"/>
+      <c r="S50" s="33" t="n"/>
+      <c r="T50" s="33" t="n"/>
+      <c r="U50" s="33" t="n"/>
+      <c r="V50" s="33" t="n"/>
+      <c r="W50" s="33" t="n"/>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>perte</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="19">
+        <f>ROUND(AVERAGE(F51:AB51), 0)</f>
+        <v/>
+      </c>
+      <c r="D51" s="1">
+        <f>SUM(F51:AB51)</f>
+        <v/>
+      </c>
+      <c r="E51" s="24" t="n">
+        <v>8060</v>
+      </c>
+      <c r="F51" s="33" t="n"/>
+      <c r="G51" s="33" t="n"/>
+      <c r="H51" s="33" t="n"/>
+      <c r="I51" s="33" t="n"/>
+      <c r="J51" s="33" t="n"/>
+      <c r="K51" s="33" t="n"/>
+      <c r="L51" s="33" t="n"/>
+      <c r="M51" s="33" t="n"/>
+      <c r="N51" s="33" t="n"/>
+      <c r="O51" s="33" t="n"/>
+      <c r="P51" s="33" t="n"/>
+      <c r="Q51" s="33" t="n"/>
+      <c r="R51" s="33" t="n"/>
+      <c r="S51" s="33" t="n"/>
+      <c r="T51" s="33" t="n"/>
+      <c r="U51" s="33" t="n"/>
+      <c r="V51" s="33" t="n"/>
+      <c r="W51" s="33" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AA1">
     <sortState ref="A2:AA51">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3306,7 +3306,7 @@
       </c>
       <c r="U1" s="7" t="inlineStr">
         <is>
-          <t>Colonna19</t>
+          <t>20/03/2026</t>
         </is>
       </c>
       <c r="V1" s="7" t="inlineStr">
@@ -3378,32 +3378,29 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>¥CATA¥</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>03/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C2" s="13">
         <f>ROUND(AVERAGE(D2:AH2), 0)</f>
         <v/>
       </c>
-      <c r="J2" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K2" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L2" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M2" s="9" t="n">
         <v>0</v>
       </c>
       <c r="N2" s="33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
         <v>6</v>
@@ -3415,33 +3412,33 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
       </c>
       <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C3" s="13">
         <f>ROUND(AVERAGE(D3:AH3), 0)</f>
         <v/>
       </c>
-      <c r="K3" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="L3" s="10" t="n">
         <v>0</v>
       </c>
@@ -3449,50 +3446,68 @@
         <v>0</v>
       </c>
       <c r="N3" s="33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O3" t="n">
         <v>6</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="U3" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C4" s="13">
         <f>ROUND(AVERAGE(D4:AH4), 0)</f>
         <v/>
       </c>
+      <c r="G4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L4" s="10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M4" s="9" t="n">
         <v>0</v>
       </c>
       <c r="N4" s="33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O4" t="n">
         <v>6</v>
@@ -3510,13 +3525,16 @@
         <v>6</v>
       </c>
       <c r="T4" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -3528,11 +3546,20 @@
         <f>ROUND(AVERAGE(D5:AH5), 0)</f>
         <v/>
       </c>
+      <c r="D5" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G5" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I5" s="9" t="n">
         <v>6</v>
@@ -3544,13 +3571,13 @@
         <v>6</v>
       </c>
       <c r="L5" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M5" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N5" s="33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O5" t="n">
         <v>6</v>
@@ -3568,13 +3595,16 @@
         <v>6</v>
       </c>
       <c r="T5" t="n">
+        <v>6</v>
+      </c>
+      <c r="U5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -3602,46 +3632,49 @@
         <v>0</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K6" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L6" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N6" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>6</v>
       </c>
       <c r="T6" t="n">
         <v>6</v>
+      </c>
+      <c r="U6" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -3653,62 +3686,56 @@
         <f>ROUND(AVERAGE(D7:AH7), 0)</f>
         <v/>
       </c>
-      <c r="D7" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G7" s="9" t="n">
         <v>6</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N7" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
@@ -3721,16 +3748,16 @@
         <v/>
       </c>
       <c r="G8" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H8" s="9" t="n">
         <v>6</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K8" s="10" t="n">
         <v>6</v>
@@ -3739,34 +3766,37 @@
         <v>6</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N8" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="P8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="U8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>ER DANDI 1927</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -3779,37 +3809,37 @@
         <v/>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I9" s="9" t="n">
         <v>6</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N9" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>6</v>
@@ -3819,12 +3849,15 @@
       </c>
       <c r="T9" t="n">
         <v>6</v>
+      </c>
+      <c r="U9" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -3836,53 +3869,65 @@
         <f>ROUND(AVERAGE(D10:AH10), 0)</f>
         <v/>
       </c>
+      <c r="D10" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G10" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="O10" t="n">
+        <v>6</v>
+      </c>
+      <c r="P10" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q10" t="n">
         <v>5</v>
       </c>
-      <c r="I10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L10" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
       <c r="R10" t="n">
         <v>6</v>
       </c>
       <c r="S10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T10" t="n">
+        <v>6</v>
+      </c>
+      <c r="U10" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -3904,7 +3949,7 @@
         <v>6</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11" s="9" t="n">
         <v>6</v>
@@ -3934,7 +3979,7 @@
         <v>6</v>
       </c>
       <c r="Q11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R11" t="n">
         <v>6</v>
@@ -3944,35 +3989,26 @@
       </c>
       <c r="T11" t="n">
         <v>6</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C12" s="13">
         <f>ROUND(AVERAGE(D12:AH12), 0)</f>
         <v/>
       </c>
-      <c r="D12" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="H12" s="9" t="n">
         <v>6</v>
       </c>
@@ -4010,24 +4046,39 @@
         <v>6</v>
       </c>
       <c r="T12" t="n">
+        <v>6</v>
+      </c>
+      <c r="U12" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C13" s="13">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
+      <c r="D13" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="H13" s="9" t="n">
         <v>6</v>
       </c>
@@ -4066,12 +4117,15 @@
       </c>
       <c r="T13" t="n">
         <v>6</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -4093,134 +4147,140 @@
         <v>6</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I14" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L14" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N14" s="33" t="n">
         <v>6</v>
       </c>
       <c r="O14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q14" t="n">
         <v>6</v>
       </c>
       <c r="R14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T14" t="n">
         <v>6</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C15" s="13">
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
-      <c r="D15" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K15" s="10" t="n"/>
+      <c r="L15" s="10" t="n"/>
       <c r="M15" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N15" s="33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q15" t="n">
         <v>6</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T15" t="n">
         <v>6</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="13">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="n"/>
+      <c r="D16" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M16" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N16" s="33" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O16" t="n">
         <v>6</v>
@@ -4239,55 +4299,33 @@
       </c>
       <c r="T16" t="n">
         <v>6</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C17" s="13">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="D17" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L17" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="10" t="n"/>
       <c r="M17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N17" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
         <v>6</v>
@@ -4306,30 +4344,49 @@
       </c>
       <c r="T17" t="n">
         <v>6</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C18" s="13">
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
-      <c r="K18" s="10" t="n"/>
-      <c r="L18" s="10" t="n"/>
+      <c r="G18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L18" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M18" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N18" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O18" t="n">
         <v>6</v>
@@ -4347,13 +4404,16 @@
         <v>6</v>
       </c>
       <c r="T18" t="n">
+        <v>6</v>
+      </c>
+      <c r="U18" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -4365,11 +4425,20 @@
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
+      <c r="D19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I19" s="9" t="n">
         <v>6</v>
@@ -4378,16 +4447,16 @@
         <v>6</v>
       </c>
       <c r="K19" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L19" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N19" s="33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
         <v>6</v>
@@ -4406,12 +4475,15 @@
       </c>
       <c r="T19" t="n">
         <v>6</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -4423,20 +4495,11 @@
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="D20" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G20" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20" s="9" t="n">
         <v>6</v>
@@ -4445,16 +4508,16 @@
         <v>6</v>
       </c>
       <c r="K20" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L20" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N20" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O20" t="n">
         <v>6</v>
@@ -4473,12 +4536,15 @@
       </c>
       <c r="T20" t="n">
         <v>6</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
@@ -4491,7 +4557,7 @@
         <v/>
       </c>
       <c r="G21" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H21" s="9" t="n">
         <v>6</v>
@@ -4531,38 +4597,26 @@
       </c>
       <c r="T21" t="n">
         <v>6</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C22" s="13">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
-      <c r="G22" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K22" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L22" s="10" t="n">
         <v>6</v>
       </c>
@@ -4589,23 +4643,29 @@
       </c>
       <c r="T22" t="n">
         <v>6</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C23" s="13">
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
+      <c r="K23" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L23" s="10" t="n">
         <v>6</v>
       </c>
@@ -4632,23 +4692,47 @@
       </c>
       <c r="T23" t="n">
         <v>6</v>
+      </c>
+      <c r="U23" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C24" s="13">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
+      <c r="D24" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J24" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K24" s="10" t="n">
         <v>6</v>
       </c>
@@ -4677,13 +4761,16 @@
         <v>6</v>
       </c>
       <c r="T24" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
@@ -4696,7 +4783,7 @@
         <v/>
       </c>
       <c r="D25" s="14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E25" s="9" t="n">
         <v>6</v>
@@ -4714,7 +4801,7 @@
         <v>6</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K25" s="10" t="n">
         <v>6</v>
@@ -4744,13 +4831,16 @@
         <v>6</v>
       </c>
       <c r="T25" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
@@ -4763,7 +4853,7 @@
         <v/>
       </c>
       <c r="D26" s="14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E26" s="9" t="n">
         <v>6</v>
@@ -4781,7 +4871,7 @@
         <v>6</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K26" s="10" t="n">
         <v>6</v>
@@ -4811,13 +4901,16 @@
         <v>6</v>
       </c>
       <c r="T26" t="n">
+        <v>6</v>
+      </c>
+      <c r="U26" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
@@ -4829,27 +4922,7 @@
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
-      <c r="D27" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J27" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="J27" s="10" t="n"/>
       <c r="K27" s="10" t="n">
         <v>6</v>
       </c>
@@ -4879,12 +4952,15 @@
       </c>
       <c r="T27" t="n">
         <v>6</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
@@ -4896,7 +4972,18 @@
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
-      <c r="J28" s="10" t="n"/>
+      <c r="G28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K28" s="10" t="n">
         <v>6</v>
       </c>
@@ -4906,14 +4993,14 @@
       <c r="M28" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N28" s="33" t="n">
+      <c r="N28" s="10" t="n">
         <v>6</v>
       </c>
       <c r="O28" t="n">
         <v>6</v>
       </c>
       <c r="P28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="n">
         <v>6</v>
@@ -4926,35 +5013,26 @@
       </c>
       <c r="T28" t="n">
         <v>6</v>
+      </c>
+      <c r="U28" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C29" s="13">
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="G29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K29" s="10" t="n">
         <v>6</v>
       </c>
@@ -4962,59 +5040,54 @@
         <v>6</v>
       </c>
       <c r="M29" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N29" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
         <v>6</v>
       </c>
       <c r="P29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q29" t="n">
         <v>6</v>
       </c>
       <c r="R29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C30" s="13">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
-      <c r="K30" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L30" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M30" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K30" s="10" t="n"/>
+      <c r="L30" s="10" t="n"/>
+      <c r="M30" s="9" t="n"/>
+      <c r="N30" s="10" t="n"/>
       <c r="O30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P30" t="n">
         <v>6</v>
@@ -5023,19 +5096,22 @@
         <v>6</v>
       </c>
       <c r="R30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T30" t="n">
+        <v>6</v>
+      </c>
+      <c r="U30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
@@ -5052,13 +5128,13 @@
       <c r="M31" s="9" t="n"/>
       <c r="N31" s="10" t="n"/>
       <c r="O31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R31" t="n">
         <v>6</v>
@@ -5068,17 +5144,20 @@
       </c>
       <c r="T31" t="n">
         <v>6</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C32" s="13">
@@ -5089,14 +5168,11 @@
       <c r="L32" s="10" t="n"/>
       <c r="M32" s="9" t="n"/>
       <c r="N32" s="10" t="n"/>
-      <c r="O32" t="n">
-        <v>6</v>
-      </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R32" t="n">
         <v>6</v>
@@ -5106,17 +5182,20 @@
       </c>
       <c r="T32" t="n">
         <v>6</v>
+      </c>
+      <c r="U32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="C33" s="13">
@@ -5128,30 +5207,33 @@
       <c r="M33" s="9" t="n"/>
       <c r="N33" s="10" t="n"/>
       <c r="P33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R33" t="n">
         <v>6</v>
       </c>
       <c r="S33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T33" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C34" s="13">
@@ -5162,31 +5244,28 @@
       <c r="L34" s="10" t="n"/>
       <c r="M34" s="9" t="n"/>
       <c r="N34" s="10" t="n"/>
-      <c r="P34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>0</v>
-      </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T34" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="U34" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
@@ -5197,26 +5276,23 @@
       <c r="L35" s="10" t="n"/>
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="10" t="n"/>
-      <c r="P35" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>2</v>
-      </c>
       <c r="R35" t="n">
         <v>6</v>
       </c>
       <c r="S35" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T35" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="U35" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
@@ -5233,24 +5309,27 @@
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="10" t="n"/>
       <c r="R36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
@@ -5262,24 +5341,27 @@
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="10" t="n"/>
       <c r="R37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S37" t="n">
         <v>6</v>
       </c>
       <c r="T37" t="n">
+        <v>6</v>
+      </c>
+      <c r="U37" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
@@ -5297,13 +5379,16 @@
         <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="U38" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
@@ -5328,16 +5413,19 @@
       <c r="T39" t="n">
         <v>6</v>
       </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5348,25 +5436,25 @@
       <c r="L40" s="10" t="n"/>
       <c r="M40" s="9" t="n"/>
       <c r="N40" s="10" t="n"/>
-      <c r="R40" t="n">
-        <v>0</v>
-      </c>
       <c r="S40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T40" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="U40" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5377,25 +5465,25 @@
       <c r="L41" s="10" t="n"/>
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="10" t="n"/>
-      <c r="R41" t="n">
-        <v>0</v>
-      </c>
       <c r="S41" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5410,18 +5498,21 @@
         <v>6</v>
       </c>
       <c r="T42" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -5432,22 +5523,22 @@
       <c r="L43" s="10" t="n"/>
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="10" t="n"/>
-      <c r="S43" t="n">
-        <v>0</v>
-      </c>
       <c r="T43" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5458,22 +5549,22 @@
       <c r="L44" s="10" t="n"/>
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="10" t="n"/>
-      <c r="S44" t="n">
-        <v>6</v>
-      </c>
       <c r="T44" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="U44" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>jacopo</t>
+          <t>Spiderman</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5487,16 +5578,19 @@
       <c r="T45" t="n">
         <v>0</v>
       </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>antony</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5507,19 +5601,19 @@
       <c r="L46" s="10" t="n"/>
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="10" t="n"/>
-      <c r="T46" t="n">
+      <c r="U46" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>Samu-Nighix</t>
+          <t>micky</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C47" s="13">
@@ -5530,19 +5624,19 @@
       <c r="L47" s="10" t="n"/>
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="10" t="n"/>
-      <c r="T47" t="n">
-        <v>1</v>
+      <c r="U47" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Marchi™</t>
+          <t>perte</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5553,19 +5647,19 @@
       <c r="L48" s="10" t="n"/>
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="10" t="n"/>
-      <c r="T48" t="n">
+      <c r="U48" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>Ernis</t>
+          <t>EMANUELE</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5576,19 +5670,19 @@
       <c r="L49" s="10" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="10" t="n"/>
-      <c r="T49" t="n">
+      <c r="U49" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Spiderman</t>
+          <t>TaifTuff</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5599,19 +5693,19 @@
       <c r="L50" s="10" t="n"/>
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="10" t="n"/>
-      <c r="T50" t="n">
+      <c r="U50" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>king</t>
+          <t>Fra</t>
         </is>
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C51" s="13">
@@ -5622,7 +5716,7 @@
       <c r="L51" s="10" t="n"/>
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="10" t="n"/>
-      <c r="T51" t="n">
+      <c r="U51" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-03-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -949,7 +949,9 @@
       <c r="J2" s="33" t="n">
         <v>2650</v>
       </c>
-      <c r="K2" s="33" t="n"/>
+      <c r="K2" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L2" s="33" t="n"/>
       <c r="M2" s="33" t="n"/>
       <c r="N2" s="33" t="n"/>
@@ -994,7 +996,9 @@
       <c r="J3" s="33" t="n">
         <v>8000</v>
       </c>
-      <c r="K3" s="33" t="n"/>
+      <c r="K3" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L3" s="33" t="n"/>
       <c r="M3" s="33" t="n"/>
       <c r="N3" s="33" t="n"/>
@@ -1041,7 +1045,9 @@
       <c r="J4" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="33" t="n"/>
+      <c r="K4" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L4" s="33" t="n"/>
       <c r="M4" s="33" t="n"/>
       <c r="N4" s="33" t="n"/>
@@ -1092,7 +1098,9 @@
       <c r="J5" s="33" t="n">
         <v>4700</v>
       </c>
-      <c r="K5" s="33" t="n"/>
+      <c r="K5" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L5" s="33" t="n"/>
       <c r="M5" s="33" t="n"/>
       <c r="N5" s="33" t="n"/>
@@ -1141,7 +1149,9 @@
       <c r="J6" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="33" t="n"/>
+      <c r="K6" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L6" s="33" t="n"/>
       <c r="M6" s="33" t="n"/>
       <c r="N6" s="33" t="n"/>
@@ -1188,7 +1198,9 @@
       <c r="J7" s="33" t="n">
         <v>150</v>
       </c>
-      <c r="K7" s="33" t="n"/>
+      <c r="K7" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L7" s="33" t="n"/>
       <c r="M7" s="33" t="n"/>
       <c r="N7" s="33" t="n"/>
@@ -1235,7 +1247,9 @@
       <c r="J8" s="33" t="n">
         <v>4050</v>
       </c>
-      <c r="K8" s="33" t="n"/>
+      <c r="K8" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L8" s="33" t="n"/>
       <c r="M8" s="33" t="n"/>
       <c r="N8" s="33" t="n"/>
@@ -1282,7 +1296,9 @@
       <c r="J9" s="33" t="n">
         <v>3000</v>
       </c>
-      <c r="K9" s="33" t="n"/>
+      <c r="K9" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L9" s="33" t="n"/>
       <c r="M9" s="33" t="n"/>
       <c r="N9" s="33" t="n"/>
@@ -1333,7 +1349,9 @@
       <c r="J10" s="33" t="n">
         <v>4050</v>
       </c>
-      <c r="K10" s="33" t="n"/>
+      <c r="K10" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="33" t="n"/>
       <c r="M10" s="33" t="n"/>
       <c r="N10" s="33" t="n"/>
@@ -1382,7 +1400,9 @@
       <c r="J11" s="33" t="n">
         <v>5950</v>
       </c>
-      <c r="K11" s="33" t="n"/>
+      <c r="K11" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L11" s="33" t="n"/>
       <c r="M11" s="33" t="n"/>
       <c r="N11" s="33" t="n"/>
@@ -1429,7 +1449,9 @@
       <c r="J12" s="33" t="n">
         <v>4000</v>
       </c>
-      <c r="K12" s="33" t="n"/>
+      <c r="K12" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="33" t="n"/>
       <c r="M12" s="33" t="n"/>
       <c r="N12" s="33" t="n"/>
@@ -1480,7 +1502,9 @@
       <c r="J13" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K13" s="33" t="n"/>
+      <c r="K13" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L13" s="33" t="n"/>
       <c r="M13" s="33" t="n"/>
       <c r="N13" s="33" t="n"/>
@@ -1529,7 +1553,9 @@
       <c r="J14" s="33" t="n">
         <v>5050</v>
       </c>
-      <c r="K14" s="33" t="n"/>
+      <c r="K14" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L14" s="33" t="n"/>
       <c r="M14" s="33" t="n"/>
       <c r="N14" s="33" t="n"/>
@@ -1574,7 +1600,9 @@
       <c r="J15" s="33" t="n">
         <v>950</v>
       </c>
-      <c r="K15" s="33" t="n"/>
+      <c r="K15" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L15" s="33" t="n"/>
       <c r="M15" s="33" t="n"/>
       <c r="N15" s="33" t="n"/>
@@ -1623,7 +1651,9 @@
       <c r="J16" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K16" s="33" t="n"/>
+      <c r="K16" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L16" s="33" t="n"/>
       <c r="M16" s="33" t="n"/>
       <c r="N16" s="33" t="n"/>
@@ -1668,7 +1698,9 @@
       <c r="J17" s="33" t="n">
         <v>3250</v>
       </c>
-      <c r="K17" s="33" t="n"/>
+      <c r="K17" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L17" s="33" t="n"/>
       <c r="M17" s="33" t="n"/>
       <c r="N17" s="33" t="n"/>
@@ -1715,7 +1747,9 @@
       <c r="J18" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K18" s="33" t="n"/>
+      <c r="K18" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L18" s="21" t="n"/>
       <c r="M18" s="33" t="n"/>
       <c r="N18" s="33" t="n"/>
@@ -1766,7 +1800,9 @@
       <c r="J19" s="33" t="n">
         <v>4350</v>
       </c>
-      <c r="K19" s="33" t="n"/>
+      <c r="K19" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L19" s="33" t="n"/>
       <c r="M19" s="33" t="n"/>
       <c r="N19" s="33" t="n"/>
@@ -1813,7 +1849,9 @@
       <c r="J20" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K20" s="33" t="n"/>
+      <c r="K20" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L20" s="33" t="n"/>
       <c r="M20" s="33" t="n"/>
       <c r="N20" s="33" t="n"/>
@@ -1860,7 +1898,9 @@
       <c r="J21" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K21" s="33" t="n"/>
+      <c r="K21" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L21" s="33" t="n"/>
       <c r="M21" s="33" t="n"/>
       <c r="N21" s="33" t="n"/>
@@ -1905,7 +1945,9 @@
       <c r="J22" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K22" s="33" t="n"/>
+      <c r="K22" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L22" s="33" t="n"/>
       <c r="M22" s="33" t="n"/>
       <c r="N22" s="33" t="n"/>
@@ -1950,7 +1992,9 @@
       <c r="J23" s="33" t="n">
         <v>4100</v>
       </c>
-      <c r="K23" s="33" t="n"/>
+      <c r="K23" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L23" s="33" t="n"/>
       <c r="M23" s="33" t="n"/>
       <c r="N23" s="33" t="n"/>
@@ -2001,7 +2045,9 @@
       <c r="J24" s="33" t="n">
         <v>1300</v>
       </c>
-      <c r="K24" s="33" t="n"/>
+      <c r="K24" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L24" s="33" t="n"/>
       <c r="M24" s="33" t="n"/>
       <c r="N24" s="33" t="n"/>
@@ -2050,7 +2096,9 @@
       <c r="J25" s="33" t="n">
         <v>4300</v>
       </c>
-      <c r="K25" s="33" t="n"/>
+      <c r="K25" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L25" s="33" t="n"/>
       <c r="M25" s="33" t="n"/>
       <c r="N25" s="33" t="n"/>
@@ -2101,7 +2149,9 @@
       <c r="J26" s="33" t="n">
         <v>4000</v>
       </c>
-      <c r="K26" s="33" t="n"/>
+      <c r="K26" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L26" s="33" t="n"/>
       <c r="M26" s="33" t="n"/>
       <c r="N26" s="33" t="n"/>
@@ -2148,7 +2198,9 @@
       <c r="J27" s="33" t="n">
         <v>3150</v>
       </c>
-      <c r="K27" s="33" t="n"/>
+      <c r="K27" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L27" s="33" t="n"/>
       <c r="M27" s="33" t="n"/>
       <c r="N27" s="33" t="n"/>
@@ -2195,7 +2247,9 @@
       <c r="J28" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="33" t="n"/>
+      <c r="K28" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L28" s="33" t="n"/>
       <c r="M28" s="33" t="n"/>
       <c r="N28" s="33" t="n"/>
@@ -2240,7 +2294,9 @@
       <c r="J29" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K29" s="33" t="n"/>
+      <c r="K29" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L29" s="33" t="n"/>
       <c r="M29" s="33" t="n"/>
       <c r="N29" s="33" t="n"/>
@@ -2283,7 +2339,9 @@
       <c r="J30" s="33" t="n">
         <v>5000</v>
       </c>
-      <c r="K30" s="33" t="n"/>
+      <c r="K30" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L30" s="33" t="n"/>
       <c r="M30" s="33" t="n"/>
       <c r="N30" s="33" t="n"/>
@@ -2326,7 +2384,9 @@
       <c r="J31" s="33" t="n">
         <v>4250</v>
       </c>
-      <c r="K31" s="33" t="n"/>
+      <c r="K31" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L31" s="33" t="n"/>
       <c r="M31" s="33" t="n"/>
       <c r="N31" s="33" t="n"/>
@@ -2369,7 +2429,9 @@
       <c r="J32" s="33" t="n">
         <v>10000</v>
       </c>
-      <c r="K32" s="33" t="n"/>
+      <c r="K32" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L32" s="33" t="n"/>
       <c r="M32" s="33" t="n"/>
       <c r="N32" s="33" t="n"/>
@@ -2412,7 +2474,9 @@
       <c r="J33" s="33" t="n">
         <v>4300</v>
       </c>
-      <c r="K33" s="33" t="n"/>
+      <c r="K33" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L33" s="33" t="n"/>
       <c r="M33" s="33" t="n"/>
       <c r="N33" s="33" t="n"/>
@@ -2455,7 +2519,9 @@
       <c r="J34" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K34" s="33" t="n"/>
+      <c r="K34" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L34" s="33" t="n"/>
       <c r="M34" s="33" t="n"/>
       <c r="N34" s="33" t="n"/>
@@ -2498,7 +2564,9 @@
       <c r="J35" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K35" s="33" t="n"/>
+      <c r="K35" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L35" s="33" t="n"/>
       <c r="M35" s="33" t="n"/>
       <c r="N35" s="33" t="n"/>
@@ -2541,7 +2609,9 @@
       <c r="J36" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="K36" s="33" t="n"/>
+      <c r="K36" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L36" s="33" t="n"/>
       <c r="M36" s="33" t="n"/>
       <c r="N36" s="33" t="n"/>
@@ -2582,7 +2652,9 @@
       <c r="H37" s="33" t="n"/>
       <c r="I37" s="33" t="n"/>
       <c r="J37" s="33" t="n"/>
-      <c r="K37" s="33" t="n"/>
+      <c r="K37" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L37" s="33" t="n"/>
       <c r="M37" s="33" t="n"/>
       <c r="N37" s="33" t="n"/>
@@ -2623,7 +2695,9 @@
       <c r="H38" s="33" t="n"/>
       <c r="I38" s="33" t="n"/>
       <c r="J38" s="33" t="n"/>
-      <c r="K38" s="33" t="n"/>
+      <c r="K38" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L38" s="33" t="n"/>
       <c r="M38" s="33" t="n"/>
       <c r="N38" s="33" t="n"/>
@@ -2664,7 +2738,9 @@
       <c r="H39" s="33" t="n"/>
       <c r="I39" s="33" t="n"/>
       <c r="J39" s="33" t="n"/>
-      <c r="K39" s="33" t="n"/>
+      <c r="K39" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L39" s="33" t="n"/>
       <c r="M39" s="33" t="n"/>
       <c r="N39" s="33" t="n"/>
@@ -2705,7 +2781,9 @@
       <c r="H40" s="33" t="n"/>
       <c r="I40" s="33" t="n"/>
       <c r="J40" s="33" t="n"/>
-      <c r="K40" s="33" t="n"/>
+      <c r="K40" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L40" s="33" t="n"/>
       <c r="M40" s="33" t="n"/>
       <c r="N40" s="33" t="n"/>
@@ -2746,7 +2824,9 @@
       <c r="H41" s="33" t="n"/>
       <c r="I41" s="33" t="n"/>
       <c r="J41" s="33" t="n"/>
-      <c r="K41" s="33" t="n"/>
+      <c r="K41" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L41" s="33" t="n"/>
       <c r="M41" s="33" t="n"/>
       <c r="N41" s="33" t="n"/>
@@ -2787,7 +2867,9 @@
       <c r="H42" s="33" t="n"/>
       <c r="I42" s="33" t="n"/>
       <c r="J42" s="33" t="n"/>
-      <c r="K42" s="33" t="n"/>
+      <c r="K42" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L42" s="33" t="n"/>
       <c r="M42" s="33" t="n"/>
       <c r="N42" s="33" t="n"/>
@@ -2828,7 +2910,9 @@
       <c r="H43" s="33" t="n"/>
       <c r="I43" s="33" t="n"/>
       <c r="J43" s="33" t="n"/>
-      <c r="K43" s="33" t="n"/>
+      <c r="K43" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L43" s="33" t="n"/>
       <c r="M43" s="33" t="n"/>
       <c r="N43" s="33" t="n"/>
@@ -2869,7 +2953,9 @@
       <c r="H44" s="33" t="n"/>
       <c r="I44" s="33" t="n"/>
       <c r="J44" s="33" t="n"/>
-      <c r="K44" s="33" t="n"/>
+      <c r="K44" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L44" s="33" t="n"/>
       <c r="M44" s="33" t="n"/>
       <c r="N44" s="33" t="n"/>
@@ -2910,7 +2996,9 @@
       <c r="H45" s="33" t="n"/>
       <c r="I45" s="33" t="n"/>
       <c r="J45" s="33" t="n"/>
-      <c r="K45" s="33" t="n"/>
+      <c r="K45" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L45" s="33" t="n"/>
       <c r="M45" s="33" t="n"/>
       <c r="N45" s="33" t="n"/>
@@ -2951,7 +3039,9 @@
       <c r="H46" s="33" t="n"/>
       <c r="I46" s="33" t="n"/>
       <c r="J46" s="33" t="n"/>
-      <c r="K46" s="33" t="n"/>
+      <c r="K46" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L46" s="33" t="n"/>
       <c r="M46" s="33" t="n"/>
       <c r="N46" s="33" t="n"/>
@@ -2992,7 +3082,9 @@
       <c r="H47" s="33" t="n"/>
       <c r="I47" s="33" t="n"/>
       <c r="J47" s="33" t="n"/>
-      <c r="K47" s="33" t="n"/>
+      <c r="K47" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L47" s="33" t="n"/>
       <c r="M47" s="33" t="n"/>
       <c r="N47" s="33" t="n"/>
@@ -3033,7 +3125,9 @@
       <c r="H48" s="33" t="n"/>
       <c r="I48" s="33" t="n"/>
       <c r="J48" s="33" t="n"/>
-      <c r="K48" s="33" t="n"/>
+      <c r="K48" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L48" s="33" t="n"/>
       <c r="M48" s="33" t="n"/>
       <c r="N48" s="33" t="n"/>
@@ -3074,7 +3168,9 @@
       <c r="H49" s="33" t="n"/>
       <c r="I49" s="33" t="n"/>
       <c r="J49" s="33" t="n"/>
-      <c r="K49" s="33" t="n"/>
+      <c r="K49" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L49" s="33" t="n"/>
       <c r="M49" s="33" t="n"/>
       <c r="N49" s="33" t="n"/>
@@ -3115,7 +3211,9 @@
       <c r="H50" s="33" t="n"/>
       <c r="I50" s="33" t="n"/>
       <c r="J50" s="33" t="n"/>
-      <c r="K50" s="33" t="n"/>
+      <c r="K50" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L50" s="33" t="n"/>
       <c r="M50" s="33" t="n"/>
       <c r="N50" s="33" t="n"/>
@@ -3156,7 +3254,9 @@
       <c r="H51" s="33" t="n"/>
       <c r="I51" s="33" t="n"/>
       <c r="J51" s="33" t="n"/>
-      <c r="K51" s="33" t="n"/>
+      <c r="K51" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="L51" s="33" t="n"/>
       <c r="M51" s="33" t="n"/>
       <c r="N51" s="33" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3951,7 +3951,7 @@
         <v>6</v>
       </c>
       <c r="U9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -4219,7 +4219,7 @@
         <v>6</v>
       </c>
       <c r="U13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4401,7 +4401,7 @@
         <v>6</v>
       </c>
       <c r="U16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -4745,7 +4745,7 @@
         <v>6</v>
       </c>
       <c r="U22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -4794,7 +4794,7 @@
         <v>6</v>
       </c>
       <c r="U23" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -4934,7 +4934,7 @@
         <v>6</v>
       </c>
       <c r="U25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -5115,7 +5115,7 @@
         <v>6</v>
       </c>
       <c r="U28" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -5205,7 +5205,7 @@
         <v>6</v>
       </c>
       <c r="U30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
@@ -5246,7 +5246,7 @@
         <v>6</v>
       </c>
       <c r="U31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -5284,7 +5284,7 @@
         <v>6</v>
       </c>
       <c r="U32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -5514,7 +5514,7 @@
         <v>6</v>
       </c>
       <c r="U39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -5601,7 +5601,7 @@
         <v>5</v>
       </c>
       <c r="U42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
@@ -5653,7 +5653,7 @@
         <v>6</v>
       </c>
       <c r="U44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -5679,7 +5679,7 @@
         <v>0</v>
       </c>
       <c r="U45" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -5817,7 +5817,7 @@
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="10" t="n"/>
       <c r="U51" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3694,7 +3694,7 @@
         <v>6</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3764,7 +3764,7 @@
         <v>6</v>
       </c>
       <c r="U6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4087,7 +4087,7 @@
         <v>6</v>
       </c>
       <c r="U11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -4282,7 +4282,7 @@
         <v>6</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -4442,7 +4442,7 @@
         <v>6</v>
       </c>
       <c r="U17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4634,7 +4634,7 @@
         <v>6</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -4695,7 +4695,7 @@
         <v>6</v>
       </c>
       <c r="U21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -5050,7 +5050,7 @@
         <v>6</v>
       </c>
       <c r="U27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -5727,7 +5727,7 @@
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>perte</t>
+          <t>EMANUELE</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
@@ -5750,7 +5750,7 @@
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>EMANUELE</t>
+          <t>Fra</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
@@ -5767,18 +5767,18 @@
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="10" t="n"/>
       <c r="U49" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>TaifTuff</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5796,12 +5796,12 @@
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>Fra</t>
+          <t>salvo24</t>
         </is>
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C51" s="13">
@@ -5813,7 +5813,7 @@
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="10" t="n"/>
       <c r="U51" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-03-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -763,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA51"/>
+  <dimension ref="A1:AA48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="25" min="1" max="1"/>
@@ -3058,7 +3058,7 @@
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>Fra</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B47" s="27" t="inlineStr">
@@ -3075,7 +3075,7 @@
         <v/>
       </c>
       <c r="E47" s="24" t="n">
-        <v>0</v>
+        <v>5350</v>
       </c>
       <c r="F47" s="33" t="n"/>
       <c r="G47" s="33" t="n"/>
@@ -3101,12 +3101,12 @@
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>EMANUELE</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B48" s="27" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C48" s="19">
@@ -3118,16 +3118,14 @@
         <v/>
       </c>
       <c r="E48" s="24" t="n">
-        <v>150</v>
+        <v>18000</v>
       </c>
       <c r="F48" s="33" t="n"/>
       <c r="G48" s="33" t="n"/>
       <c r="H48" s="33" t="n"/>
       <c r="I48" s="33" t="n"/>
       <c r="J48" s="33" t="n"/>
-      <c r="K48" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="K48" s="33" t="n"/>
       <c r="L48" s="33" t="n"/>
       <c r="M48" s="33" t="n"/>
       <c r="N48" s="33" t="n"/>
@@ -3141,131 +3139,7 @@
       <c r="V48" s="33" t="n"/>
       <c r="W48" s="33" t="n"/>
     </row>
-    <row r="49">
-      <c r="A49" s="24" t="inlineStr">
-        <is>
-          <t>omar</t>
-        </is>
-      </c>
-      <c r="B49" s="27" t="inlineStr">
-        <is>
-          <t>21/03/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="19">
-        <f>ROUND(AVERAGE(F49:AB49), 0)</f>
-        <v/>
-      </c>
-      <c r="D49" s="1">
-        <f>SUM(F49:AB49)</f>
-        <v/>
-      </c>
-      <c r="E49" s="24" t="n">
-        <v>5350</v>
-      </c>
-      <c r="F49" s="33" t="n"/>
-      <c r="G49" s="33" t="n"/>
-      <c r="H49" s="33" t="n"/>
-      <c r="I49" s="33" t="n"/>
-      <c r="J49" s="33" t="n"/>
-      <c r="K49" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" s="33" t="n"/>
-      <c r="M49" s="33" t="n"/>
-      <c r="N49" s="33" t="n"/>
-      <c r="O49" s="33" t="n"/>
-      <c r="P49" s="33" t="n"/>
-      <c r="Q49" s="33" t="n"/>
-      <c r="R49" s="33" t="n"/>
-      <c r="S49" s="33" t="n"/>
-      <c r="T49" s="33" t="n"/>
-      <c r="U49" s="33" t="n"/>
-      <c r="V49" s="33" t="n"/>
-      <c r="W49" s="33" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="24" t="inlineStr">
-        <is>
-          <t>Edoardo9</t>
-        </is>
-      </c>
-      <c r="B50" s="27" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="19">
-        <f>ROUND(AVERAGE(F50:AB50), 0)</f>
-        <v/>
-      </c>
-      <c r="D50" s="1">
-        <f>SUM(F50:AB50)</f>
-        <v/>
-      </c>
-      <c r="E50" s="24" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F50" s="33" t="n"/>
-      <c r="G50" s="33" t="n"/>
-      <c r="H50" s="33" t="n"/>
-      <c r="I50" s="33" t="n"/>
-      <c r="J50" s="33" t="n"/>
-      <c r="K50" s="33" t="n"/>
-      <c r="L50" s="33" t="n"/>
-      <c r="M50" s="33" t="n"/>
-      <c r="N50" s="33" t="n"/>
-      <c r="O50" s="33" t="n"/>
-      <c r="P50" s="33" t="n"/>
-      <c r="Q50" s="33" t="n"/>
-      <c r="R50" s="33" t="n"/>
-      <c r="S50" s="33" t="n"/>
-      <c r="T50" s="33" t="n"/>
-      <c r="U50" s="33" t="n"/>
-      <c r="V50" s="33" t="n"/>
-      <c r="W50" s="33" t="n"/>
-    </row>
-    <row r="51" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A51" s="24" t="inlineStr">
-        <is>
-          <t>salvo24</t>
-        </is>
-      </c>
-      <c r="B51" s="27" t="inlineStr">
-        <is>
-          <t>22/03/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="19">
-        <f>ROUND(AVERAGE(F51:AB51), 0)</f>
-        <v/>
-      </c>
-      <c r="D51" s="1">
-        <f>SUM(F51:AB51)</f>
-        <v/>
-      </c>
-      <c r="E51" s="24" t="n">
-        <v>64980</v>
-      </c>
-      <c r="F51" s="33" t="n"/>
-      <c r="G51" s="33" t="n"/>
-      <c r="H51" s="33" t="n"/>
-      <c r="I51" s="33" t="n"/>
-      <c r="J51" s="33" t="n"/>
-      <c r="K51" s="33" t="n"/>
-      <c r="L51" s="33" t="n"/>
-      <c r="M51" s="33" t="n"/>
-      <c r="N51" s="33" t="n"/>
-      <c r="O51" s="33" t="n"/>
-      <c r="P51" s="33" t="n"/>
-      <c r="Q51" s="33" t="n"/>
-      <c r="R51" s="33" t="n"/>
-      <c r="S51" s="33" t="n"/>
-      <c r="T51" s="33" t="n"/>
-      <c r="U51" s="33" t="n"/>
-      <c r="V51" s="33" t="n"/>
-      <c r="W51" s="33" t="n"/>
-    </row>
+    <row r="51" ht="15.75" customHeight="1" thickBot="1"/>
   </sheetData>
   <autoFilter ref="A1:AA1">
     <sortState ref="A2:AA51">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-03-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3239,7 +3239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="V1" s="7" t="inlineStr">
         <is>
-          <t>Colonna20</t>
+          <t>27/03/2026</t>
         </is>
       </c>
       <c r="W1" s="7" t="inlineStr">
@@ -3475,6 +3475,9 @@
       <c r="U2" t="n">
         <v>0</v>
       </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -3521,6 +3524,9 @@
       <c r="U3" t="n">
         <v>6</v>
       </c>
+      <c r="V3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -3582,6 +3588,9 @@
       <c r="U4" t="n">
         <v>6</v>
       </c>
+      <c r="V4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
@@ -3652,6 +3661,9 @@
       <c r="U5" t="n">
         <v>6</v>
       </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -3722,6 +3734,9 @@
       <c r="U6" t="n">
         <v>6</v>
       </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -3783,6 +3798,9 @@
       <c r="U7" t="n">
         <v>0</v>
       </c>
+      <c r="V7" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -3844,6 +3862,9 @@
       <c r="U8" t="n">
         <v>6</v>
       </c>
+      <c r="V8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -3905,6 +3926,9 @@
       <c r="U9" t="n">
         <v>6</v>
       </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -3975,6 +3999,9 @@
       <c r="U10" t="n">
         <v>6</v>
       </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -4045,6 +4072,9 @@
       <c r="U11" t="n">
         <v>6</v>
       </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -4103,6 +4133,9 @@
       <c r="U12" t="n">
         <v>6</v>
       </c>
+      <c r="V12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -4173,6 +4206,9 @@
       <c r="U13" t="n">
         <v>6</v>
       </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -4239,6 +4275,9 @@
       </c>
       <c r="U14" t="n">
         <v>4</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -4285,6 +4324,9 @@
       <c r="U15" t="n">
         <v>0</v>
       </c>
+      <c r="V15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -4353,6 +4395,9 @@
         <v>6</v>
       </c>
       <c r="U16" t="n">
+        <v>6</v>
+      </c>
+      <c r="V16" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4400,6 +4445,9 @@
       <c r="U17" t="n">
         <v>6</v>
       </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -4461,6 +4509,9 @@
       <c r="U18" t="n">
         <v>6</v>
       </c>
+      <c r="V18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -4531,6 +4582,9 @@
       <c r="U19" t="n">
         <v>0</v>
       </c>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -4592,6 +4646,9 @@
       <c r="U20" t="n">
         <v>6</v>
       </c>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -4653,6 +4710,9 @@
       <c r="U21" t="n">
         <v>6</v>
       </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -4699,6 +4759,9 @@
       <c r="U22" t="n">
         <v>6</v>
       </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -4748,6 +4811,9 @@
       <c r="U23" t="n">
         <v>6</v>
       </c>
+      <c r="V23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
@@ -4818,6 +4884,9 @@
       <c r="U24" t="n">
         <v>0</v>
       </c>
+      <c r="V24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
@@ -4888,6 +4957,9 @@
       <c r="U25" t="n">
         <v>6</v>
       </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
@@ -4958,6 +5030,9 @@
       <c r="U26" t="n">
         <v>6</v>
       </c>
+      <c r="V26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -5008,6 +5083,9 @@
       <c r="U27" t="n">
         <v>6</v>
       </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
@@ -5069,6 +5147,9 @@
       <c r="U28" t="n">
         <v>6</v>
       </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -5116,6 +5197,9 @@
         <v>0</v>
       </c>
       <c r="U29" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5159,6 +5243,9 @@
       <c r="U30" t="n">
         <v>6</v>
       </c>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
@@ -5200,6 +5287,9 @@
       <c r="U31" t="n">
         <v>6</v>
       </c>
+      <c r="V31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -5237,6 +5327,9 @@
       </c>
       <c r="U32" t="n">
         <v>6</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -5276,6 +5369,9 @@
       <c r="U33" t="n">
         <v>0</v>
       </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -5308,6 +5404,9 @@
       <c r="U34" t="n">
         <v>6</v>
       </c>
+      <c r="V34" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
@@ -5340,6 +5439,9 @@
       <c r="U35" t="n">
         <v>6</v>
       </c>
+      <c r="V35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
@@ -5372,6 +5474,9 @@
       <c r="U36" t="n">
         <v>0</v>
       </c>
+      <c r="V36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
@@ -5404,6 +5509,9 @@
       <c r="U37" t="n">
         <v>6</v>
       </c>
+      <c r="V37" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
@@ -5436,6 +5544,9 @@
       <c r="U38" t="n">
         <v>6</v>
       </c>
+      <c r="V38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
@@ -5468,6 +5579,9 @@
       <c r="U39" t="n">
         <v>6</v>
       </c>
+      <c r="V39" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
@@ -5497,6 +5611,9 @@
       <c r="U40" t="n">
         <v>6</v>
       </c>
+      <c r="V40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
@@ -5526,6 +5643,9 @@
       <c r="U41" t="n">
         <v>0</v>
       </c>
+      <c r="V41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
@@ -5555,6 +5675,9 @@
       <c r="U42" t="n">
         <v>6</v>
       </c>
+      <c r="V42" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
@@ -5581,6 +5704,9 @@
       <c r="U43" t="n">
         <v>0</v>
       </c>
+      <c r="V43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
@@ -5607,6 +5733,9 @@
       <c r="U44" t="n">
         <v>6</v>
       </c>
+      <c r="V44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
@@ -5633,6 +5762,9 @@
       <c r="U45" t="n">
         <v>6</v>
       </c>
+      <c r="V45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
@@ -5656,6 +5788,9 @@
       <c r="U46" t="n">
         <v>6</v>
       </c>
+      <c r="V46" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
@@ -5679,16 +5814,19 @@
       <c r="U47" t="n">
         <v>0</v>
       </c>
+      <c r="V47" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>EMANUELE</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5702,16 +5840,19 @@
       <c r="U48" t="n">
         <v>0</v>
       </c>
+      <c r="V48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>Fra</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5722,19 +5863,19 @@
       <c r="L49" s="10" t="n"/>
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="10" t="n"/>
-      <c r="U49" t="n">
-        <v>6</v>
+      <c r="V49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>Er Caciotta</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5745,30 +5886,7 @@
       <c r="L50" s="10" t="n"/>
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="10" t="n"/>
-      <c r="U50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>salvo24</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>23/03/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="U51" t="n">
+      <c r="V50" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-03-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -763,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA50"/>
+  <dimension ref="A1:AA49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="25" min="1" max="1"/>
@@ -2843,7 +2843,7 @@
     <row r="42">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>micky</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B42" s="27" t="inlineStr">
@@ -2860,7 +2860,7 @@
         <v/>
       </c>
       <c r="E42" s="24" t="n">
-        <v>16600</v>
+        <v>6550</v>
       </c>
       <c r="F42" s="33" t="n"/>
       <c r="G42" s="33" t="n"/>
@@ -2886,7 +2886,7 @@
     <row r="43">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B43" s="27" t="inlineStr">
@@ -2903,7 +2903,7 @@
         <v/>
       </c>
       <c r="E43" s="24" t="n">
-        <v>6550</v>
+        <v>0</v>
       </c>
       <c r="F43" s="33" t="n"/>
       <c r="G43" s="33" t="n"/>
@@ -2929,7 +2929,7 @@
     <row r="44">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B44" s="27" t="inlineStr">
@@ -2946,7 +2946,7 @@
         <v/>
       </c>
       <c r="E44" s="24" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="F44" s="33" t="n"/>
       <c r="G44" s="33" t="n"/>
@@ -2972,7 +2972,7 @@
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B45" s="27" t="inlineStr">
@@ -2989,7 +2989,7 @@
         <v/>
       </c>
       <c r="E45" s="24" t="n">
-        <v>1800</v>
+        <v>5500</v>
       </c>
       <c r="F45" s="33" t="n"/>
       <c r="G45" s="33" t="n"/>
@@ -3015,7 +3015,7 @@
     <row r="46">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B46" s="27" t="inlineStr">
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
       <c r="E46" s="24" t="n">
-        <v>5500</v>
+        <v>5350</v>
       </c>
       <c r="F46" s="33" t="n"/>
       <c r="G46" s="33" t="n"/>
@@ -3058,12 +3058,12 @@
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B47" s="27" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C47" s="19">
@@ -3075,16 +3075,14 @@
         <v/>
       </c>
       <c r="E47" s="24" t="n">
-        <v>5350</v>
+        <v>18000</v>
       </c>
       <c r="F47" s="33" t="n"/>
       <c r="G47" s="33" t="n"/>
       <c r="H47" s="33" t="n"/>
       <c r="I47" s="33" t="n"/>
       <c r="J47" s="33" t="n"/>
-      <c r="K47" s="33" t="n">
-        <v>0</v>
-      </c>
+      <c r="K47" s="33" t="n"/>
       <c r="L47" s="33" t="n"/>
       <c r="M47" s="33" t="n"/>
       <c r="N47" s="33" t="n"/>
@@ -3101,12 +3099,12 @@
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>Er Caciotta</t>
         </is>
       </c>
       <c r="B48" s="27" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>27/03/2026</t>
         </is>
       </c>
       <c r="C48" s="19">
@@ -3118,7 +3116,7 @@
         <v/>
       </c>
       <c r="E48" s="24" t="n">
-        <v>18000</v>
+        <v>10025</v>
       </c>
       <c r="F48" s="33" t="n"/>
       <c r="G48" s="33" t="n"/>
@@ -3142,7 +3140,7 @@
     <row r="49">
       <c r="A49" s="24" t="inlineStr">
         <is>
-          <t>Er Caciotta</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B49" s="27" t="inlineStr">
@@ -3159,7 +3157,7 @@
         <v/>
       </c>
       <c r="E49" s="24" t="n">
-        <v>10025</v>
+        <v>250</v>
       </c>
       <c r="F49" s="33" t="n"/>
       <c r="G49" s="33" t="n"/>
@@ -3179,47 +3177,6 @@
       <c r="U49" s="33" t="n"/>
       <c r="V49" s="33" t="n"/>
       <c r="W49" s="33" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="24" t="inlineStr">
-        <is>
-          <t>falcuns</t>
-        </is>
-      </c>
-      <c r="B50" s="27" t="inlineStr">
-        <is>
-          <t>27/03/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="19">
-        <f>ROUND(AVERAGE(F50:AB50), 0)</f>
-        <v/>
-      </c>
-      <c r="D50" s="1">
-        <f>SUM(F50:AB50)</f>
-        <v/>
-      </c>
-      <c r="E50" s="24" t="n">
-        <v>250</v>
-      </c>
-      <c r="F50" s="33" t="n"/>
-      <c r="G50" s="33" t="n"/>
-      <c r="H50" s="33" t="n"/>
-      <c r="I50" s="33" t="n"/>
-      <c r="J50" s="33" t="n"/>
-      <c r="K50" s="33" t="n"/>
-      <c r="L50" s="33" t="n"/>
-      <c r="M50" s="33" t="n"/>
-      <c r="N50" s="33" t="n"/>
-      <c r="O50" s="33" t="n"/>
-      <c r="P50" s="33" t="n"/>
-      <c r="Q50" s="33" t="n"/>
-      <c r="R50" s="33" t="n"/>
-      <c r="S50" s="33" t="n"/>
-      <c r="T50" s="33" t="n"/>
-      <c r="U50" s="33" t="n"/>
-      <c r="V50" s="33" t="n"/>
-      <c r="W50" s="33" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" thickBot="1"/>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-04
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="W1" s="7" t="inlineStr">
         <is>
-          <t>Colonna21</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="X1" s="7" t="inlineStr">
@@ -3421,6 +3421,9 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3458,6 +3461,9 @@
       <c r="V3" t="n">
         <v>6</v>
       </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -3505,6 +3511,9 @@
         <v>6</v>
       </c>
       <c r="V4" t="n">
+        <v>6</v>
+      </c>
+      <c r="W4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3547,6 +3556,9 @@
       </c>
       <c r="V5" t="n">
         <v>6</v>
+      </c>
+      <c r="W5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -3579,6 +3591,9 @@
       <c r="V6" t="n">
         <v>6</v>
       </c>
+      <c r="W6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -3616,6 +3631,9 @@
       <c r="V7" t="n">
         <v>1</v>
       </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -3680,6 +3698,9 @@
       <c r="V8" t="n">
         <v>6</v>
       </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -3753,6 +3774,9 @@
       <c r="V9" t="n">
         <v>0</v>
       </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -3824,6 +3848,9 @@
         <v>6</v>
       </c>
       <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3869,6 +3896,9 @@
       <c r="V11" t="n">
         <v>5</v>
       </c>
+      <c r="W11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -3932,6 +3962,9 @@
       </c>
       <c r="V12" t="n">
         <v>6</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -3972,6 +4005,9 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4005,6 +4041,9 @@
       <c r="V14" t="n">
         <v>0</v>
       </c>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -4069,186 +4108,206 @@
       <c r="V15" t="n">
         <v>6</v>
       </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Er Caciotta</t>
+          <t>ER DANDI 1927</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>28/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="13">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="n"/>
-      <c r="N16" s="26" t="n"/>
-      <c r="O16" s="27" t="n"/>
-      <c r="P16" s="27" t="n"/>
-      <c r="Q16" s="27" t="n"/>
-      <c r="R16" s="27" t="n"/>
-      <c r="S16" s="27" t="n"/>
-      <c r="T16" s="27" t="n"/>
-      <c r="U16" s="27" t="n"/>
+      <c r="G16" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="L16" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>6</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>6</v>
+      </c>
+      <c r="U16" t="n">
+        <v>6</v>
+      </c>
       <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="C17" s="13">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="G17" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K17" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L17" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>6</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" t="n">
-        <v>6</v>
-      </c>
-      <c r="U17" t="n">
-        <v>6</v>
-      </c>
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="10" t="n"/>
+      <c r="N17" s="26" t="n"/>
+      <c r="O17" s="27" t="n"/>
+      <c r="P17" s="27" t="n"/>
+      <c r="Q17" s="27" t="n"/>
+      <c r="R17" s="27" t="n"/>
+      <c r="S17" s="27" t="n"/>
+      <c r="T17" s="27" t="n"/>
+      <c r="U17" s="27" t="n"/>
       <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>falcuns</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>28/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C18" s="13">
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
-      <c r="K18" s="10" t="n"/>
-      <c r="L18" s="10" t="n"/>
-      <c r="N18" s="26" t="n"/>
-      <c r="O18" s="27" t="n"/>
-      <c r="P18" s="27" t="n"/>
-      <c r="Q18" s="27" t="n"/>
-      <c r="R18" s="27" t="n"/>
-      <c r="S18" s="27" t="n"/>
-      <c r="T18" s="27" t="n"/>
-      <c r="U18" s="27" t="n"/>
+      <c r="D18" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L18" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N18" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O18" t="n">
+        <v>6</v>
+      </c>
+      <c r="P18" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>5</v>
+      </c>
+      <c r="R18" t="n">
+        <v>6</v>
+      </c>
+      <c r="S18" t="n">
+        <v>6</v>
+      </c>
+      <c r="T18" t="n">
+        <v>6</v>
+      </c>
+      <c r="U18" t="n">
+        <v>6</v>
+      </c>
       <c r="V18" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="W18" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C19" s="13">
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
-      <c r="D19" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K19" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L19" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N19" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O19" t="n">
-        <v>6</v>
-      </c>
-      <c r="P19" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>5</v>
-      </c>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="n"/>
+      <c r="N19" s="26" t="n"/>
+      <c r="O19" s="27" t="n"/>
+      <c r="P19" s="27" t="n"/>
+      <c r="Q19" s="27" t="n"/>
       <c r="R19" t="n">
         <v>6</v>
       </c>
@@ -4263,29 +4322,68 @@
       </c>
       <c r="V19" t="n">
         <v>6</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C20" s="13">
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="K20" s="10" t="n"/>
-      <c r="L20" s="10" t="n"/>
-      <c r="N20" s="26" t="n"/>
-      <c r="O20" s="27" t="n"/>
-      <c r="P20" s="27" t="n"/>
-      <c r="Q20" s="27" t="n"/>
+      <c r="D20" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L20" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>6</v>
+      </c>
       <c r="R20" t="n">
         <v>6</v>
       </c>
@@ -4300,35 +4398,26 @@
       </c>
       <c r="V20" t="n">
         <v>6</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C21" s="13">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="D21" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="H21" s="9" t="n">
         <v>6</v>
       </c>
@@ -4372,24 +4461,39 @@
         <v>6</v>
       </c>
       <c r="V21" t="n">
+        <v>6</v>
+      </c>
+      <c r="W21" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C22" s="13">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
+      <c r="D22" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="H22" s="9" t="n">
         <v>6</v>
       </c>
@@ -4433,13 +4537,16 @@
         <v>6</v>
       </c>
       <c r="V22" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -4461,146 +4568,152 @@
         <v>6</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M23" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N23" s="26" t="n">
         <v>6</v>
       </c>
       <c r="O23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q23" t="n">
         <v>6</v>
       </c>
       <c r="R23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T23" t="n">
         <v>6</v>
       </c>
       <c r="U23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V23" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C24" s="13">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
-      <c r="D24" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="10" t="n"/>
       <c r="M24" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N24" s="26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q24" t="n">
         <v>6</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T24" t="n">
         <v>6</v>
       </c>
       <c r="U24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="W24" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C25" s="13">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
-      <c r="K25" s="10" t="n"/>
-      <c r="L25" s="10" t="n"/>
+      <c r="D25" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L25" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M25" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N25" s="26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O25" t="n">
         <v>6</v>
@@ -4621,71 +4734,38 @@
         <v>6</v>
       </c>
       <c r="U25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V25" t="n">
         <v>6</v>
+      </c>
+      <c r="W25" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C26" s="13">
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
-      <c r="D26" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J26" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K26" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L26" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N26" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O26" t="n">
-        <v>6</v>
-      </c>
-      <c r="P26" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>6</v>
-      </c>
+      <c r="K26" s="10" t="n"/>
+      <c r="L26" s="10" t="n"/>
+      <c r="N26" s="10" t="n"/>
+      <c r="O26" s="27" t="n"/>
+      <c r="P26" s="27" t="n"/>
+      <c r="Q26" s="27" t="n"/>
       <c r="R26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
         <v>6</v>
@@ -4697,18 +4777,21 @@
         <v>6</v>
       </c>
       <c r="V26" t="n">
+        <v>6</v>
+      </c>
+      <c r="W26" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C27" s="13">
@@ -4717,12 +4800,23 @@
       </c>
       <c r="K27" s="10" t="n"/>
       <c r="L27" s="10" t="n"/>
-      <c r="N27" s="10" t="n"/>
-      <c r="O27" s="27" t="n"/>
-      <c r="P27" s="27" t="n"/>
-      <c r="Q27" s="27" t="n"/>
+      <c r="M27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>6</v>
+      </c>
+      <c r="P27" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>6</v>
+      </c>
       <c r="R27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S27" t="n">
         <v>6</v>
@@ -4734,31 +4828,50 @@
         <v>6</v>
       </c>
       <c r="V27" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C28" s="13">
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
-      <c r="K28" s="10" t="n"/>
-      <c r="L28" s="10" t="n"/>
+      <c r="G28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K28" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L28" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M28" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N28" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O28" t="n">
         <v>6</v>
@@ -4782,13 +4895,16 @@
         <v>6</v>
       </c>
       <c r="V28" t="n">
+        <v>6</v>
+      </c>
+      <c r="W28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -4800,11 +4916,20 @@
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
+      <c r="D29" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I29" s="9" t="n">
         <v>6</v>
@@ -4813,16 +4938,16 @@
         <v>6</v>
       </c>
       <c r="K29" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L29" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M29" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N29" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
         <v>6</v>
@@ -4843,94 +4968,61 @@
         <v>6</v>
       </c>
       <c r="U29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V29" t="n">
+        <v>5</v>
+      </c>
+      <c r="W29" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C30" s="13">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
-      <c r="D30" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" t="n">
-        <v>6</v>
-      </c>
-      <c r="P30" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>6</v>
-      </c>
-      <c r="R30" t="n">
-        <v>6</v>
-      </c>
+      <c r="K30" s="10" t="n"/>
+      <c r="L30" s="10" t="n"/>
+      <c r="N30" s="10" t="n"/>
+      <c r="P30" s="27" t="n"/>
+      <c r="Q30" s="27" t="n"/>
+      <c r="R30" s="27" t="n"/>
       <c r="S30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
       </c>
       <c r="V30" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C31" s="13">
@@ -4940,31 +5032,43 @@
       <c r="K31" s="10" t="n"/>
       <c r="L31" s="10" t="n"/>
       <c r="N31" s="10" t="n"/>
-      <c r="P31" s="27" t="n"/>
-      <c r="Q31" s="27" t="n"/>
-      <c r="R31" s="27" t="n"/>
+      <c r="O31" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="P31" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q31" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R31" t="n">
+        <v>6</v>
+      </c>
       <c r="S31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C32" s="13">
@@ -4974,40 +5078,30 @@
       <c r="K32" s="10" t="n"/>
       <c r="L32" s="10" t="n"/>
       <c r="N32" s="10" t="n"/>
-      <c r="O32" s="28" t="n">
+      <c r="R32" s="27" t="n"/>
+      <c r="S32" s="27" t="n"/>
+      <c r="T32" t="n">
+        <v>6</v>
+      </c>
+      <c r="U32" t="n">
+        <v>6</v>
+      </c>
+      <c r="V32" t="n">
         <v>5</v>
       </c>
-      <c r="P32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R32" t="n">
-        <v>6</v>
-      </c>
-      <c r="S32" t="n">
-        <v>6</v>
-      </c>
-      <c r="T32" t="n">
-        <v>6</v>
-      </c>
-      <c r="U32" t="n">
-        <v>6</v>
-      </c>
-      <c r="V32" t="n">
+      <c r="W32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C33" s="13">
@@ -5018,7 +5112,9 @@
       <c r="L33" s="10" t="n"/>
       <c r="N33" s="10" t="n"/>
       <c r="R33" s="27" t="n"/>
-      <c r="S33" s="27" t="n"/>
+      <c r="S33" t="n">
+        <v>6</v>
+      </c>
       <c r="T33" t="n">
         <v>6</v>
       </c>
@@ -5026,28 +5122,63 @@
         <v>6</v>
       </c>
       <c r="V33" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C34" s="13">
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
-      <c r="K34" s="10" t="n"/>
-      <c r="L34" s="10" t="n"/>
-      <c r="N34" s="10" t="n"/>
-      <c r="R34" s="27" t="n"/>
+      <c r="G34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L34" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N34" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O34" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P34" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q34" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R34" t="n">
+        <v>6</v>
+      </c>
       <c r="S34" t="n">
         <v>6</v>
       </c>
@@ -5059,26 +5190,59 @@
       </c>
       <c r="V34" t="n">
         <v>6</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C35" s="13">
         <f>ROUND(AVERAGE(D35:AH35), 0)</f>
         <v/>
       </c>
-      <c r="K35" s="10" t="n"/>
-      <c r="L35" s="10" t="n"/>
-      <c r="N35" s="10" t="n"/>
+      <c r="G35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O35" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P35" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q35" s="28" t="n">
+        <v>6</v>
+      </c>
       <c r="R35" t="n">
         <v>6</v>
       </c>
@@ -5093,38 +5257,26 @@
       </c>
       <c r="V35" t="n">
         <v>6</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C36" s="13">
         <f>ROUND(AVERAGE(D36:AH36), 0)</f>
         <v/>
       </c>
-      <c r="G36" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H36" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I36" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J36" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K36" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L36" s="10" t="n">
         <v>6</v>
       </c>
@@ -5143,7 +5295,7 @@
       <c r="Q36" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R36" t="n">
+      <c r="R36" s="28" t="n">
         <v>6</v>
       </c>
       <c r="S36" t="n">
@@ -5157,35 +5309,26 @@
       </c>
       <c r="V36" t="n">
         <v>6</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
         <f>ROUND(AVERAGE(D37:AH37), 0)</f>
         <v/>
       </c>
-      <c r="G37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J37" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K37" s="10" t="n">
         <v>6</v>
       </c>
@@ -5207,7 +5350,7 @@
       <c r="Q37" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R37" t="n">
+      <c r="R37" s="28" t="n">
         <v>6</v>
       </c>
       <c r="S37" t="n">
@@ -5221,23 +5364,50 @@
       </c>
       <c r="V37" t="n">
         <v>6</v>
+      </c>
+      <c r="W37" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C38" s="13">
         <f>ROUND(AVERAGE(D38:AH38), 0)</f>
         <v/>
       </c>
+      <c r="D38" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I38" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J38" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K38" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L38" s="10" t="n">
         <v>6</v>
       </c>
@@ -5263,30 +5433,54 @@
         <v>6</v>
       </c>
       <c r="T38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V38" t="n">
         <v>6</v>
+      </c>
+      <c r="W38" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C39" s="13">
         <f>ROUND(AVERAGE(D39:AH39), 0)</f>
         <v/>
       </c>
+      <c r="D39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>5</v>
+      </c>
       <c r="K39" s="10" t="n">
         <v>6</v>
       </c>
@@ -5311,7 +5505,7 @@
       <c r="R39" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S39" t="n">
+      <c r="S39" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T39" t="n">
@@ -5321,13 +5515,16 @@
         <v>6</v>
       </c>
       <c r="V39" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
@@ -5384,96 +5581,63 @@
       <c r="R40" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S40" t="n">
+      <c r="S40" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T40" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V40" t="n">
+        <v>6</v>
+      </c>
+      <c r="W40" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
         <f>ROUND(AVERAGE(D41:AH41), 0)</f>
         <v/>
       </c>
-      <c r="D41" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J41" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K41" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L41" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N41" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O41" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P41" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q41" s="28" t="n">
-        <v>6</v>
-      </c>
+      <c r="K41" s="10" t="n"/>
+      <c r="L41" s="10" t="n"/>
+      <c r="N41" s="10" t="n"/>
       <c r="R41" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S41" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="T41" t="n">
+      <c r="T41" s="28" t="n">
         <v>6</v>
       </c>
       <c r="U41" t="n">
         <v>6</v>
       </c>
       <c r="V41" t="n">
+        <v>6</v>
+      </c>
+      <c r="W41" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
@@ -5485,27 +5649,7 @@
         <f>ROUND(AVERAGE(D42:AH42), 0)</f>
         <v/>
       </c>
-      <c r="D42" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E42" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F42" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G42" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H42" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I42" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J42" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="J42" s="10" t="n"/>
       <c r="K42" s="10" t="n">
         <v>6</v>
       </c>
@@ -5533,36 +5677,69 @@
       <c r="S42" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="T42" t="n">
+      <c r="T42" s="28" t="n">
         <v>6</v>
       </c>
       <c r="U42" t="n">
         <v>6</v>
       </c>
       <c r="V42" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C43" s="13">
         <f>ROUND(AVERAGE(D43:AH43), 0)</f>
         <v/>
       </c>
-      <c r="K43" s="10" t="n"/>
-      <c r="L43" s="10" t="n"/>
-      <c r="N43" s="10" t="n"/>
+      <c r="G43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J43" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K43" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L43" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N43" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O43" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P43" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" s="28" t="n">
+        <v>6</v>
+      </c>
       <c r="R43" s="28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S43" s="28" t="n">
         <v>6</v>
@@ -5570,29 +5747,31 @@
       <c r="T43" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="U43" t="n">
+      <c r="U43" s="28" t="n">
         <v>6</v>
       </c>
       <c r="V43" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="W43" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
         <f>ROUND(AVERAGE(D44:AH44), 0)</f>
         <v/>
       </c>
-      <c r="J44" s="10" t="n"/>
       <c r="K44" s="10" t="n">
         <v>6</v>
       </c>
@@ -5600,10 +5779,10 @@
         <v>6</v>
       </c>
       <c r="M44" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N44" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O44" s="28" t="n">
         <v>6</v>
@@ -5615,141 +5794,94 @@
         <v>6</v>
       </c>
       <c r="R44" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S44" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T44" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U44" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U44" s="28" t="n">
+        <v>0</v>
       </c>
       <c r="V44" t="n">
+        <v>0</v>
+      </c>
+      <c r="W44" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>krigohard</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
         <f>ROUND(AVERAGE(D45:AH45), 0)</f>
         <v/>
       </c>
-      <c r="G45" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H45" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I45" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J45" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K45" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L45" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M45" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N45" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O45" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P45" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q45" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R45" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S45" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T45" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U45" s="28" t="n">
-        <v>6</v>
-      </c>
+      <c r="K45" s="10" t="n"/>
+      <c r="L45" s="10" t="n"/>
+      <c r="M45" s="9" t="n"/>
+      <c r="N45" s="10" t="n"/>
+      <c r="O45" s="28" t="n"/>
+      <c r="P45" s="28" t="n"/>
+      <c r="Q45" s="28" t="n"/>
+      <c r="R45" s="28" t="n"/>
+      <c r="S45" s="28" t="n"/>
+      <c r="T45" s="28" t="n"/>
+      <c r="U45" s="28" t="n"/>
       <c r="V45" t="n">
+        <v>0</v>
+      </c>
+      <c r="W45" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
         <f>ROUND(AVERAGE(D46:AH46), 0)</f>
         <v/>
       </c>
-      <c r="K46" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L46" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M46" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P46" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q46" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R46" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S46" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T46" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="U46" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="K46" s="10" t="n"/>
+      <c r="L46" s="10" t="n"/>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="10" t="n"/>
+      <c r="O46" s="28" t="n"/>
+      <c r="P46" s="28" t="n"/>
+      <c r="Q46" s="28" t="n"/>
+      <c r="R46" s="28" t="n"/>
+      <c r="S46" s="28" t="n"/>
+      <c r="T46" s="28" t="n"/>
+      <c r="U46" s="28" t="n"/>
       <c r="V46" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>krigohard</t>
+          <t>er samu</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
@@ -5773,18 +5905,21 @@
       <c r="T47" s="28" t="n"/>
       <c r="U47" s="28" t="n"/>
       <c r="V47" t="n">
+        <v>1</v>
+      </c>
+      <c r="W47" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5802,19 +5937,19 @@
       <c r="S48" s="28" t="n"/>
       <c r="T48" s="28" t="n"/>
       <c r="U48" s="28" t="n"/>
-      <c r="V48" t="n">
-        <v>0</v>
+      <c r="W48" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>salvuz11</t>
+          <t>l0ki</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5832,19 +5967,19 @@
       <c r="S49" s="28" t="n"/>
       <c r="T49" s="28" t="n"/>
       <c r="U49" s="28" t="n"/>
-      <c r="V49" t="n">
-        <v>6</v>
+      <c r="W49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="29">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>er samu</t>
+          <t>Steninja:)</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -5862,38 +5997,8 @@
       <c r="S50" s="28" t="n"/>
       <c r="T50" s="28" t="n"/>
       <c r="U50" s="28" t="n"/>
-      <c r="V50" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>_loris_yt</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>29/03/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="O51" s="28" t="n"/>
-      <c r="P51" s="28" t="n"/>
-      <c r="Q51" s="28" t="n"/>
-      <c r="R51" s="28" t="n"/>
-      <c r="S51" s="28" t="n"/>
-      <c r="T51" s="28" t="n"/>
-      <c r="U51" s="28" t="n"/>
-      <c r="V51" t="n">
-        <v>6</v>
+      <c r="W50" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-05
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3558,7 +3558,7 @@
         <v>6</v>
       </c>
       <c r="W5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3699,7 +3699,7 @@
         <v>6</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -3851,7 +3851,7 @@
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4284,7 +4284,7 @@
         <v>6</v>
       </c>
       <c r="W18" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -4740,7 +4740,7 @@
         <v>6</v>
       </c>
       <c r="W25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -5090,7 +5090,7 @@
         <v>5</v>
       </c>
       <c r="W32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -5366,7 +5366,7 @@
         <v>6</v>
       </c>
       <c r="W37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
@@ -5687,7 +5687,7 @@
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -5754,7 +5754,7 @@
         <v>0</v>
       </c>
       <c r="W43" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -5908,7 +5908,7 @@
         <v>1</v>
       </c>
       <c r="W47" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-11
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3318,7 +3318,7 @@
       </c>
       <c r="X1" s="7" t="inlineStr">
         <is>
-          <t>Colonna22</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="Y1" s="7" t="inlineStr">
@@ -3424,6 +3424,9 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3464,6 +3467,9 @@
       <c r="W3" t="n">
         <v>0</v>
       </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -3515,6 +3521,9 @@
       </c>
       <c r="W4" t="n">
         <v>6</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3559,6 +3568,9 @@
       </c>
       <c r="W5" t="n">
         <v>6</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3594,51 +3606,84 @@
       <c r="W6" t="n">
         <v>6</v>
       </c>
+      <c r="X6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C7" s="13">
         <f>ROUND(AVERAGE(D7:AH7), 0)</f>
         <v/>
       </c>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="10" t="n"/>
-      <c r="N7" s="26" t="n"/>
-      <c r="O7" s="27" t="n"/>
-      <c r="P7" s="27" t="n"/>
-      <c r="Q7" s="27" t="n"/>
+      <c r="G7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>6</v>
+      </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
         <v>6</v>
       </c>
       <c r="V7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W7" t="n">
+        <v>6</v>
+      </c>
+      <c r="X7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
@@ -3650,11 +3695,20 @@
         <f>ROUND(AVERAGE(D8:AH8), 0)</f>
         <v/>
       </c>
+      <c r="D8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G8" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>6</v>
@@ -3666,13 +3720,13 @@
         <v>6</v>
       </c>
       <c r="L8" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N8" s="26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O8" t="n">
         <v>6</v>
@@ -3690,22 +3744,25 @@
         <v>6</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U8" t="n">
         <v>6</v>
       </c>
       <c r="V8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -3733,34 +3790,34 @@
         <v>0</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N9" s="26" t="n">
         <v>6</v>
       </c>
       <c r="O9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>6</v>
@@ -3775,68 +3832,41 @@
         <v>0</v>
       </c>
       <c r="W9" t="n">
+        <v>6</v>
+      </c>
+      <c r="X9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C10" s="13">
         <f>ROUND(AVERAGE(D10:AH10), 0)</f>
         <v/>
       </c>
-      <c r="D10" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="M10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="26" t="n">
-        <v>6</v>
-      </c>
+      <c r="K10" s="10" t="n"/>
+      <c r="L10" s="10" t="n"/>
+      <c r="N10" s="26" t="n"/>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S10" t="n">
         <v>6</v>
@@ -3848,178 +3878,201 @@
         <v>6</v>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W10" t="n">
+        <v>6</v>
+      </c>
+      <c r="X10" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C11" s="13">
         <f>ROUND(AVERAGE(D11:AH11), 0)</f>
         <v/>
       </c>
-      <c r="K11" s="10" t="n"/>
-      <c r="L11" s="10" t="n"/>
-      <c r="N11" s="26" t="n"/>
+      <c r="G11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="O11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W11" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C12" s="13">
         <f>ROUND(AVERAGE(D12:AH12), 0)</f>
         <v/>
       </c>
-      <c r="G12" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K12" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L12" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M12" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="N12" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O12" t="n">
-        <v>1</v>
-      </c>
-      <c r="P12" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>4</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="N12" s="26" t="n"/>
+      <c r="O12" s="27" t="n"/>
+      <c r="P12" s="27" t="n"/>
+      <c r="Q12" s="27" t="n"/>
+      <c r="R12" s="27" t="n"/>
+      <c r="S12" s="27" t="n"/>
+      <c r="T12" s="27" t="n"/>
       <c r="U12" t="n">
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C13" s="13">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
-      <c r="K13" s="10" t="n"/>
-      <c r="L13" s="10" t="n"/>
-      <c r="N13" s="26" t="n"/>
-      <c r="O13" s="27" t="n"/>
+      <c r="G13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N13" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O13" t="n">
+        <v>6</v>
+      </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R13" t="n">
         <v>6</v>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="C14" s="13">
@@ -4035,20 +4088,21 @@
       <c r="R14" s="27" t="n"/>
       <c r="S14" s="27" t="n"/>
       <c r="T14" s="27" t="n"/>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
+      <c r="U14" s="27" t="n"/>
       <c r="V14" t="n">
         <v>0</v>
       </c>
       <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -4060,8 +4114,17 @@
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
+      <c r="D15" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G15" s="9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>6</v>
@@ -4070,7 +4133,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K15" s="10" t="n">
         <v>6</v>
@@ -4091,13 +4154,13 @@
         <v>6</v>
       </c>
       <c r="Q15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R15" t="n">
         <v>6</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T15" t="n">
         <v>6</v>
@@ -4109,62 +4172,38 @@
         <v>6</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="X15" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C16" s="13">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="G16" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J16" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L16" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
+      <c r="K16" s="10" t="n"/>
+      <c r="L16" s="10" t="n"/>
+      <c r="N16" s="26" t="n"/>
+      <c r="O16" s="27" t="n"/>
+      <c r="P16" s="27" t="n"/>
+      <c r="Q16" s="27" t="n"/>
       <c r="R16" t="n">
         <v>6</v>
       </c>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T16" t="n">
         <v>6</v>
@@ -4173,71 +4212,109 @@
         <v>6</v>
       </c>
       <c r="V16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>falcuns</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>28/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C17" s="13">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="n"/>
-      <c r="N17" s="26" t="n"/>
-      <c r="O17" s="27" t="n"/>
-      <c r="P17" s="27" t="n"/>
-      <c r="Q17" s="27" t="n"/>
-      <c r="R17" s="27" t="n"/>
-      <c r="S17" s="27" t="n"/>
-      <c r="T17" s="27" t="n"/>
-      <c r="U17" s="27" t="n"/>
+      <c r="D17" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" t="n">
+        <v>6</v>
+      </c>
+      <c r="P17" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>6</v>
+      </c>
+      <c r="R17" t="n">
+        <v>6</v>
+      </c>
+      <c r="S17" t="n">
+        <v>6</v>
+      </c>
+      <c r="T17" t="n">
+        <v>6</v>
+      </c>
+      <c r="U17" t="n">
+        <v>6</v>
+      </c>
       <c r="V17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C18" s="13">
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
-      <c r="D18" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>5</v>
-      </c>
       <c r="H18" s="9" t="n">
         <v>6</v>
       </c>
@@ -4266,7 +4343,7 @@
         <v>6</v>
       </c>
       <c r="Q18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R18" t="n">
         <v>6</v>
@@ -4284,30 +4361,69 @@
         <v>6</v>
       </c>
       <c r="W18" t="n">
+        <v>6</v>
+      </c>
+      <c r="X18" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C19" s="13">
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
-      <c r="K19" s="10" t="n"/>
-      <c r="L19" s="10" t="n"/>
-      <c r="N19" s="26" t="n"/>
-      <c r="O19" s="27" t="n"/>
-      <c r="P19" s="27" t="n"/>
-      <c r="Q19" s="27" t="n"/>
+      <c r="D19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N19" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O19" t="n">
+        <v>6</v>
+      </c>
+      <c r="P19" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>6</v>
+      </c>
       <c r="R19" t="n">
         <v>6</v>
       </c>
@@ -4321,16 +4437,19 @@
         <v>6</v>
       </c>
       <c r="V19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W19" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -4352,92 +4471,79 @@
         <v>6</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I20" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K20" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L20" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N20" s="26" t="n">
         <v>6</v>
       </c>
       <c r="O20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q20" t="n">
         <v>6</v>
       </c>
       <c r="R20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T20" t="n">
         <v>6</v>
       </c>
       <c r="U20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W20" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C21" s="13">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="H21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K21" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L21" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="10" t="n"/>
       <c r="M21" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N21" s="26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O21" t="n">
         <v>6</v>
@@ -4458,19 +4564,22 @@
         <v>6</v>
       </c>
       <c r="U21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V21" t="n">
         <v>6</v>
       </c>
       <c r="W21" t="n">
+        <v>6</v>
+      </c>
+      <c r="X21" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
@@ -4537,107 +4646,96 @@
         <v>6</v>
       </c>
       <c r="V22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W22" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="X22" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C23" s="13">
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
-      <c r="D23" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O23" t="n">
-        <v>4</v>
-      </c>
-      <c r="P23" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>6</v>
-      </c>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="10" t="n"/>
+      <c r="N23" s="10" t="n"/>
+      <c r="O23" s="27" t="n"/>
+      <c r="P23" s="27" t="n"/>
+      <c r="Q23" s="27" t="n"/>
       <c r="R23" t="n">
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T23" t="n">
         <v>6</v>
       </c>
       <c r="U23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W23" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="X23" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C24" s="13">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
-      <c r="K24" s="10" t="n"/>
-      <c r="L24" s="10" t="n"/>
+      <c r="G24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J24" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M24" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N24" s="26" t="n">
-        <v>1</v>
+      <c r="N24" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="O24" t="n">
         <v>6</v>
@@ -4658,19 +4756,22 @@
         <v>6</v>
       </c>
       <c r="U24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V24" t="n">
         <v>6</v>
       </c>
       <c r="W24" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
@@ -4686,16 +4787,16 @@
         <v>6</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>6</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I25" s="9" t="n">
         <v>6</v>
@@ -4704,16 +4805,16 @@
         <v>6</v>
       </c>
       <c r="K25" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M25" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N25" s="26" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="N25" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="O25" t="n">
         <v>6</v>
@@ -4734,24 +4835,27 @@
         <v>6</v>
       </c>
       <c r="U25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W25" t="n">
+        <v>6</v>
+      </c>
+      <c r="X25" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C26" s="13">
@@ -4761,37 +4865,37 @@
       <c r="K26" s="10" t="n"/>
       <c r="L26" s="10" t="n"/>
       <c r="N26" s="10" t="n"/>
-      <c r="O26" s="27" t="n"/>
       <c r="P26" s="27" t="n"/>
       <c r="Q26" s="27" t="n"/>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
+      <c r="R26" s="27" t="n"/>
       <c r="S26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C27" s="13">
@@ -4800,19 +4904,14 @@
       </c>
       <c r="K27" s="10" t="n"/>
       <c r="L27" s="10" t="n"/>
-      <c r="M27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N27" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>6</v>
-      </c>
-      <c r="P27" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q27" t="n">
+      <c r="N27" s="10" t="n"/>
+      <c r="O27" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="P27" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q27" s="28" t="n">
         <v>6</v>
       </c>
       <c r="R27" t="n">
@@ -4832,12 +4931,15 @@
       </c>
       <c r="W27" t="n">
         <v>0</v>
+      </c>
+      <c r="X27" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
@@ -4850,7 +4952,7 @@
         <v/>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H28" s="9" t="n">
         <v>6</v>
@@ -4873,13 +4975,13 @@
       <c r="N28" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="O28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q28" t="n">
+      <c r="O28" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P28" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q28" s="28" t="n">
         <v>6</v>
       </c>
       <c r="R28" t="n">
@@ -4898,13 +5000,16 @@
         <v>6</v>
       </c>
       <c r="W28" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -4916,20 +5021,11 @@
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="D29" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I29" s="9" t="n">
         <v>6</v>
@@ -4938,24 +5034,24 @@
         <v>6</v>
       </c>
       <c r="K29" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L29" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M29" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N29" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>6</v>
-      </c>
-      <c r="P29" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q29" t="n">
+        <v>6</v>
+      </c>
+      <c r="O29" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P29" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q29" s="28" t="n">
         <v>6</v>
       </c>
       <c r="R29" t="n">
@@ -4968,72 +5064,102 @@
         <v>6</v>
       </c>
       <c r="U29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W29" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="X29" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C30" s="13">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
-      <c r="K30" s="10" t="n"/>
-      <c r="L30" s="10" t="n"/>
-      <c r="N30" s="10" t="n"/>
-      <c r="P30" s="27" t="n"/>
-      <c r="Q30" s="27" t="n"/>
-      <c r="R30" s="27" t="n"/>
+      <c r="L30" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N30" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O30" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P30" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q30" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R30" s="28" t="n">
+        <v>6</v>
+      </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W30" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C31" s="13">
         <f>ROUND(AVERAGE(D31:AH31), 0)</f>
         <v/>
       </c>
-      <c r="K31" s="10" t="n"/>
-      <c r="L31" s="10" t="n"/>
-      <c r="N31" s="10" t="n"/>
+      <c r="K31" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L31" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N31" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="O31" s="28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P31" s="28" t="n">
         <v>6</v>
@@ -5041,7 +5167,7 @@
       <c r="Q31" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R31" t="n">
+      <c r="R31" s="28" t="n">
         <v>6</v>
       </c>
       <c r="S31" t="n">
@@ -5054,65 +5180,155 @@
         <v>6</v>
       </c>
       <c r="V31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W31" t="n">
+        <v>4</v>
+      </c>
+      <c r="X31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C32" s="13">
         <f>ROUND(AVERAGE(D32:AH32), 0)</f>
         <v/>
       </c>
-      <c r="K32" s="10" t="n"/>
-      <c r="L32" s="10" t="n"/>
-      <c r="N32" s="10" t="n"/>
-      <c r="R32" s="27" t="n"/>
-      <c r="S32" s="27" t="n"/>
+      <c r="D32" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="S32" t="n">
+        <v>6</v>
+      </c>
       <c r="T32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W32" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="X32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C33" s="13">
         <f>ROUND(AVERAGE(D33:AH33), 0)</f>
         <v/>
       </c>
-      <c r="K33" s="10" t="n"/>
-      <c r="L33" s="10" t="n"/>
-      <c r="N33" s="10" t="n"/>
-      <c r="R33" s="27" t="n"/>
-      <c r="S33" t="n">
+      <c r="D33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L33" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N33" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O33" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P33" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q33" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R33" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="S33" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T33" t="n">
@@ -5122,16 +5338,19 @@
         <v>6</v>
       </c>
       <c r="V33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
@@ -5143,6 +5362,15 @@
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
+      <c r="D34" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G34" s="9" t="n">
         <v>6</v>
       </c>
@@ -5176,10 +5404,10 @@
       <c r="Q34" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R34" t="n">
-        <v>6</v>
-      </c>
-      <c r="S34" t="n">
+      <c r="R34" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="S34" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T34" t="n">
@@ -5192,64 +5420,37 @@
         <v>6</v>
       </c>
       <c r="W34" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="X34" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
         <f>ROUND(AVERAGE(D35:AH35), 0)</f>
         <v/>
       </c>
-      <c r="G35" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R35" t="n">
-        <v>6</v>
-      </c>
-      <c r="S35" t="n">
-        <v>6</v>
-      </c>
-      <c r="T35" t="n">
+      <c r="K35" s="10" t="n"/>
+      <c r="L35" s="10" t="n"/>
+      <c r="N35" s="10" t="n"/>
+      <c r="R35" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="T35" s="28" t="n">
         <v>6</v>
       </c>
       <c r="U35" t="n">
@@ -5259,24 +5460,31 @@
         <v>6</v>
       </c>
       <c r="W35" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C36" s="13">
         <f>ROUND(AVERAGE(D36:AH36), 0)</f>
         <v/>
       </c>
+      <c r="J36" s="10" t="n"/>
+      <c r="K36" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L36" s="10" t="n">
         <v>6</v>
       </c>
@@ -5298,37 +5506,52 @@
       <c r="R36" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S36" t="n">
-        <v>6</v>
-      </c>
-      <c r="T36" t="n">
+      <c r="S36" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="T36" s="28" t="n">
         <v>6</v>
       </c>
       <c r="U36" t="n">
         <v>6</v>
       </c>
       <c r="V36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W36" t="n">
+        <v>5</v>
+      </c>
+      <c r="X36" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C37" s="13">
         <f>ROUND(AVERAGE(D37:AH37), 0)</f>
         <v/>
       </c>
+      <c r="G37" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I37" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J37" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K37" s="10" t="n">
         <v>6</v>
       </c>
@@ -5345,7 +5568,7 @@
         <v>6</v>
       </c>
       <c r="P37" s="28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q37" s="28" t="n">
         <v>6</v>
@@ -5353,58 +5576,40 @@
       <c r="R37" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S37" t="n">
-        <v>6</v>
-      </c>
-      <c r="T37" t="n">
-        <v>6</v>
-      </c>
-      <c r="U37" t="n">
+      <c r="S37" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="T37" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="U37" s="28" t="n">
         <v>6</v>
       </c>
       <c r="V37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="X37" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
         <f>ROUND(AVERAGE(D38:AH38), 0)</f>
         <v/>
       </c>
-      <c r="D38" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E38" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H38" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I38" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J38" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K38" s="10" t="n">
         <v>6</v>
       </c>
@@ -5412,10 +5617,10 @@
         <v>6</v>
       </c>
       <c r="M38" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N38" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O38" s="28" t="n">
         <v>6</v>
@@ -5427,185 +5632,108 @@
         <v>6</v>
       </c>
       <c r="R38" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S38" t="n">
-        <v>6</v>
-      </c>
-      <c r="T38" t="n">
-        <v>4</v>
-      </c>
-      <c r="U38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" s="28" t="n">
         <v>0</v>
       </c>
       <c r="V38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="X38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>krigohard</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
         <f>ROUND(AVERAGE(D39:AH39), 0)</f>
         <v/>
       </c>
-      <c r="D39" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J39" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K39" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L39" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N39" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O39" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P39" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q39" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R39" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S39" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T39" t="n">
-        <v>6</v>
-      </c>
-      <c r="U39" t="n">
-        <v>6</v>
-      </c>
+      <c r="K39" s="10" t="n"/>
+      <c r="L39" s="10" t="n"/>
+      <c r="M39" s="9" t="n"/>
+      <c r="N39" s="10" t="n"/>
+      <c r="O39" s="28" t="n"/>
+      <c r="P39" s="28" t="n"/>
+      <c r="Q39" s="28" t="n"/>
+      <c r="R39" s="28" t="n"/>
+      <c r="S39" s="28" t="n"/>
+      <c r="T39" s="28" t="n"/>
+      <c r="U39" s="28" t="n"/>
       <c r="V39" t="n">
         <v>0</v>
       </c>
       <c r="W39" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
         <f>ROUND(AVERAGE(D40:AH40), 0)</f>
         <v/>
       </c>
-      <c r="D40" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E40" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F40" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H40" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I40" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J40" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K40" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L40" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M40" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N40" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O40" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P40" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q40" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R40" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S40" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T40" t="n">
-        <v>6</v>
-      </c>
-      <c r="U40" t="n">
-        <v>6</v>
-      </c>
+      <c r="K40" s="10" t="n"/>
+      <c r="L40" s="10" t="n"/>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="10" t="n"/>
+      <c r="O40" s="28" t="n"/>
+      <c r="P40" s="28" t="n"/>
+      <c r="Q40" s="28" t="n"/>
+      <c r="R40" s="28" t="n"/>
+      <c r="S40" s="28" t="n"/>
+      <c r="T40" s="28" t="n"/>
+      <c r="U40" s="28" t="n"/>
       <c r="V40" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W40" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5614,393 +5742,116 @@
       </c>
       <c r="K41" s="10" t="n"/>
       <c r="L41" s="10" t="n"/>
+      <c r="M41" s="9" t="n"/>
       <c r="N41" s="10" t="n"/>
-      <c r="R41" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S41" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T41" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U41" t="n">
-        <v>6</v>
-      </c>
-      <c r="V41" t="n">
-        <v>6</v>
-      </c>
+      <c r="O41" s="28" t="n"/>
+      <c r="P41" s="28" t="n"/>
+      <c r="Q41" s="28" t="n"/>
+      <c r="R41" s="28" t="n"/>
+      <c r="S41" s="28" t="n"/>
+      <c r="T41" s="28" t="n"/>
+      <c r="U41" s="28" t="n"/>
       <c r="W41" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="X41" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Steninja:)</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
         <f>ROUND(AVERAGE(D42:AH42), 0)</f>
         <v/>
       </c>
-      <c r="J42" s="10" t="n"/>
-      <c r="K42" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L42" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M42" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N42" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O42" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P42" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q42" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R42" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S42" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T42" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U42" t="n">
-        <v>6</v>
-      </c>
-      <c r="V42" t="n">
-        <v>0</v>
-      </c>
+      <c r="K42" s="10" t="n"/>
+      <c r="L42" s="10" t="n"/>
+      <c r="M42" s="9" t="n"/>
+      <c r="N42" s="10" t="n"/>
+      <c r="O42" s="28" t="n"/>
+      <c r="P42" s="28" t="n"/>
+      <c r="Q42" s="28" t="n"/>
+      <c r="R42" s="28" t="n"/>
+      <c r="S42" s="28" t="n"/>
+      <c r="T42" s="28" t="n"/>
+      <c r="U42" s="28" t="n"/>
       <c r="W42" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="X42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Splaticon</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
         <f>ROUND(AVERAGE(D43:AH43), 0)</f>
         <v/>
       </c>
-      <c r="G43" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H43" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I43" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J43" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K43" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L43" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M43" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N43" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O43" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P43" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q43" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R43" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S43" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T43" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U43" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="V43" t="n">
-        <v>0</v>
-      </c>
-      <c r="W43" t="n">
-        <v>6</v>
+      <c r="K43" s="10" t="n"/>
+      <c r="L43" s="10" t="n"/>
+      <c r="M43" s="9" t="n"/>
+      <c r="N43" s="10" t="n"/>
+      <c r="O43" s="28" t="n"/>
+      <c r="P43" s="28" t="n"/>
+      <c r="Q43" s="28" t="n"/>
+      <c r="R43" s="28" t="n"/>
+      <c r="S43" s="28" t="n"/>
+      <c r="T43" s="28" t="n"/>
+      <c r="U43" s="28" t="n"/>
+      <c r="X43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>~¥AKAZA¥~</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
         <f>ROUND(AVERAGE(D44:AH44), 0)</f>
         <v/>
       </c>
-      <c r="K44" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L44" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M44" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P44" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q44" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R44" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S44" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T44" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="U44" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="V44" t="n">
-        <v>0</v>
-      </c>
-      <c r="W44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>krigohard</t>
-        </is>
-      </c>
-      <c r="B45" s="15" t="inlineStr">
-        <is>
-          <t>29/03/2026</t>
-        </is>
-      </c>
-      <c r="C45" s="13">
-        <f>ROUND(AVERAGE(D45:AH45), 0)</f>
-        <v/>
-      </c>
-      <c r="K45" s="10" t="n"/>
-      <c r="L45" s="10" t="n"/>
-      <c r="M45" s="9" t="n"/>
-      <c r="N45" s="10" t="n"/>
-      <c r="O45" s="28" t="n"/>
-      <c r="P45" s="28" t="n"/>
-      <c r="Q45" s="28" t="n"/>
-      <c r="R45" s="28" t="n"/>
-      <c r="S45" s="28" t="n"/>
-      <c r="T45" s="28" t="n"/>
-      <c r="U45" s="28" t="n"/>
-      <c r="V45" t="n">
-        <v>0</v>
-      </c>
-      <c r="W45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>Juri</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="inlineStr">
-        <is>
-          <t>29/03/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="13">
-        <f>ROUND(AVERAGE(D46:AH46), 0)</f>
-        <v/>
-      </c>
-      <c r="K46" s="10" t="n"/>
-      <c r="L46" s="10" t="n"/>
-      <c r="M46" s="9" t="n"/>
-      <c r="N46" s="10" t="n"/>
-      <c r="O46" s="28" t="n"/>
-      <c r="P46" s="28" t="n"/>
-      <c r="Q46" s="28" t="n"/>
-      <c r="R46" s="28" t="n"/>
-      <c r="S46" s="28" t="n"/>
-      <c r="T46" s="28" t="n"/>
-      <c r="U46" s="28" t="n"/>
-      <c r="V46" t="n">
-        <v>0</v>
-      </c>
-      <c r="W46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>er samu</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="inlineStr">
-        <is>
-          <t>29/03/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="13">
-        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
-        <v/>
-      </c>
-      <c r="K47" s="10" t="n"/>
-      <c r="L47" s="10" t="n"/>
-      <c r="M47" s="9" t="n"/>
-      <c r="N47" s="10" t="n"/>
-      <c r="O47" s="28" t="n"/>
-      <c r="P47" s="28" t="n"/>
-      <c r="Q47" s="28" t="n"/>
-      <c r="R47" s="28" t="n"/>
-      <c r="S47" s="28" t="n"/>
-      <c r="T47" s="28" t="n"/>
-      <c r="U47" s="28" t="n"/>
-      <c r="V47" t="n">
-        <v>1</v>
-      </c>
-      <c r="W47" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>TinoGiusa</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="13">
-        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
-        <v/>
-      </c>
-      <c r="K48" s="10" t="n"/>
-      <c r="L48" s="10" t="n"/>
-      <c r="M48" s="9" t="n"/>
-      <c r="N48" s="10" t="n"/>
-      <c r="O48" s="28" t="n"/>
-      <c r="P48" s="28" t="n"/>
-      <c r="Q48" s="28" t="n"/>
-      <c r="R48" s="28" t="n"/>
-      <c r="S48" s="28" t="n"/>
-      <c r="T48" s="28" t="n"/>
-      <c r="U48" s="28" t="n"/>
-      <c r="W48" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>l0ki</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="13">
-        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
-        <v/>
-      </c>
-      <c r="K49" s="10" t="n"/>
-      <c r="L49" s="10" t="n"/>
-      <c r="M49" s="9" t="n"/>
-      <c r="N49" s="10" t="n"/>
-      <c r="O49" s="28" t="n"/>
-      <c r="P49" s="28" t="n"/>
-      <c r="Q49" s="28" t="n"/>
-      <c r="R49" s="28" t="n"/>
-      <c r="S49" s="28" t="n"/>
-      <c r="T49" s="28" t="n"/>
-      <c r="U49" s="28" t="n"/>
-      <c r="W49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="29">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>Steninja:)</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="13">
-        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="10" t="n"/>
-      <c r="L50" s="10" t="n"/>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="10" t="n"/>
-      <c r="O50" s="28" t="n"/>
-      <c r="P50" s="28" t="n"/>
-      <c r="Q50" s="28" t="n"/>
-      <c r="R50" s="28" t="n"/>
-      <c r="S50" s="28" t="n"/>
-      <c r="T50" s="28" t="n"/>
-      <c r="U50" s="28" t="n"/>
-      <c r="W50" t="n">
-        <v>0</v>
-      </c>
-    </row>
+      <c r="K44" s="10" t="n"/>
+      <c r="L44" s="10" t="n"/>
+      <c r="M44" s="9" t="n"/>
+      <c r="N44" s="10" t="n"/>
+      <c r="O44" s="28" t="n"/>
+      <c r="P44" s="28" t="n"/>
+      <c r="Q44" s="28" t="n"/>
+      <c r="R44" s="28" t="n"/>
+      <c r="S44" s="28" t="n"/>
+      <c r="T44" s="28" t="n"/>
+      <c r="U44" s="28" t="n"/>
+      <c r="X44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="29"/>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-12
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH44"/>
+  <dimension ref="A1:AH47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3570,7 +3570,7 @@
         <v>6</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3756,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -3954,7 +3954,7 @@
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -3991,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -5186,7 +5186,7 @@
         <v>4</v>
       </c>
       <c r="X31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -5265,7 +5265,7 @@
         <v>3</v>
       </c>
       <c r="X32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
@@ -5423,7 +5423,7 @@
         <v>6</v>
       </c>
       <c r="X34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -5522,7 +5522,7 @@
         <v>5</v>
       </c>
       <c r="X36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
@@ -5848,6 +5848,96 @@
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
       <c r="X44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>ggvitotmm</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="13">
+        <f>ROUND(AVERAGE(D45:AH45), 0)</f>
+        <v/>
+      </c>
+      <c r="K45" s="10" t="n"/>
+      <c r="L45" s="10" t="n"/>
+      <c r="M45" s="9" t="n"/>
+      <c r="N45" s="10" t="n"/>
+      <c r="O45" s="28" t="n"/>
+      <c r="P45" s="28" t="n"/>
+      <c r="Q45" s="28" t="n"/>
+      <c r="R45" s="28" t="n"/>
+      <c r="S45" s="28" t="n"/>
+      <c r="T45" s="28" t="n"/>
+      <c r="U45" s="28" t="n"/>
+      <c r="X45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>toxic</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="13">
+        <f>ROUND(AVERAGE(D46:AH46), 0)</f>
+        <v/>
+      </c>
+      <c r="K46" s="10" t="n"/>
+      <c r="L46" s="10" t="n"/>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="10" t="n"/>
+      <c r="O46" s="28" t="n"/>
+      <c r="P46" s="28" t="n"/>
+      <c r="Q46" s="28" t="n"/>
+      <c r="R46" s="28" t="n"/>
+      <c r="S46" s="28" t="n"/>
+      <c r="T46" s="28" t="n"/>
+      <c r="U46" s="28" t="n"/>
+      <c r="X46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>color052</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="13">
+        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
+        <v/>
+      </c>
+      <c r="K47" s="10" t="n"/>
+      <c r="L47" s="10" t="n"/>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="10" t="n"/>
+      <c r="O47" s="28" t="n"/>
+      <c r="P47" s="28" t="n"/>
+      <c r="Q47" s="28" t="n"/>
+      <c r="R47" s="28" t="n"/>
+      <c r="S47" s="28" t="n"/>
+      <c r="T47" s="28" t="n"/>
+      <c r="U47" s="28" t="n"/>
+      <c r="X47" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-13
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH47"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -5941,7 +5941,114 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1" s="29"/>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>Dasters79</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="13">
+        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
+        <v/>
+      </c>
+      <c r="K48" s="10" t="n"/>
+      <c r="L48" s="10" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="10" t="n"/>
+      <c r="O48" s="28" t="n"/>
+      <c r="P48" s="28" t="n"/>
+      <c r="Q48" s="28" t="n"/>
+      <c r="R48" s="28" t="n"/>
+      <c r="S48" s="28" t="n"/>
+      <c r="T48" s="28" t="n"/>
+      <c r="U48" s="28" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>samuel</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="13">
+        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
+        <v/>
+      </c>
+      <c r="K49" s="10" t="n"/>
+      <c r="L49" s="10" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="10" t="n"/>
+      <c r="O49" s="28" t="n"/>
+      <c r="P49" s="28" t="n"/>
+      <c r="Q49" s="28" t="n"/>
+      <c r="R49" s="28" t="n"/>
+      <c r="S49" s="28" t="n"/>
+      <c r="T49" s="28" t="n"/>
+      <c r="U49" s="28" t="n"/>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="29">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="13">
+        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="10" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="10" t="n"/>
+      <c r="O50" s="28" t="n"/>
+      <c r="P50" s="28" t="n"/>
+      <c r="Q50" s="28" t="n"/>
+      <c r="R50" s="28" t="n"/>
+      <c r="S50" s="28" t="n"/>
+      <c r="T50" s="28" t="n"/>
+      <c r="U50" s="28" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>matteo</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="13">
+        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="10" t="n"/>
+      <c r="L51" s="10" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="10" t="n"/>
+      <c r="O51" s="28" t="n"/>
+      <c r="P51" s="28" t="n"/>
+      <c r="Q51" s="28" t="n"/>
+      <c r="R51" s="28" t="n"/>
+      <c r="S51" s="28" t="n"/>
+      <c r="T51" s="28" t="n"/>
+      <c r="U51" s="28" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-18
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="Y1" s="7" t="inlineStr">
         <is>
-          <t>Colonna23</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="Z1" s="7" t="inlineStr">
@@ -3429,29 +3429,46 @@
       <c r="X2" t="n">
         <v>0</v>
       </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C3" s="13">
         <f>ROUND(AVERAGE(D3:AH3), 0)</f>
         <v/>
       </c>
-      <c r="K3" s="10" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="N3" s="26" t="n"/>
-      <c r="O3" s="27" t="n"/>
-      <c r="P3" s="27" t="n"/>
-      <c r="Q3" s="27" t="n"/>
-      <c r="R3" s="27" t="n"/>
+      <c r="L3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>6</v>
+      </c>
+      <c r="P3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R3" t="n">
+        <v>6</v>
+      </c>
       <c r="S3" t="n">
         <v>6</v>
       </c>
@@ -3465,39 +3482,34 @@
         <v>6</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C4" s="13">
         <f>ROUND(AVERAGE(D4:AH4), 0)</f>
         <v/>
       </c>
-      <c r="L4" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="O4" t="n">
-        <v>6</v>
-      </c>
+      <c r="K4" s="10" t="n"/>
+      <c r="L4" s="10" t="n"/>
+      <c r="N4" s="26" t="n"/>
+      <c r="O4" s="27" t="n"/>
       <c r="P4" t="n">
         <v>6</v>
       </c>
@@ -3511,7 +3523,7 @@
         <v>6</v>
       </c>
       <c r="T4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U4" t="n">
         <v>6</v>
@@ -3523,18 +3535,21 @@
         <v>6</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>antony</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C5" s="13">
@@ -3545,21 +3560,11 @@
       <c r="L5" s="10" t="n"/>
       <c r="N5" s="26" t="n"/>
       <c r="O5" s="27" t="n"/>
-      <c r="P5" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>6</v>
-      </c>
-      <c r="R5" t="n">
-        <v>6</v>
-      </c>
-      <c r="S5" t="n">
-        <v>6</v>
-      </c>
-      <c r="T5" t="n">
-        <v>6</v>
-      </c>
+      <c r="P5" s="27" t="n"/>
+      <c r="Q5" s="27" t="n"/>
+      <c r="R5" s="27" t="n"/>
+      <c r="S5" s="27" t="n"/>
+      <c r="T5" s="27" t="n"/>
       <c r="U5" t="n">
         <v>6</v>
       </c>
@@ -3571,32 +3576,68 @@
       </c>
       <c r="X5" t="n">
         <v>6</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>antony</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C6" s="13">
         <f>ROUND(AVERAGE(D6:AH6), 0)</f>
         <v/>
       </c>
-      <c r="K6" s="10" t="n"/>
-      <c r="L6" s="10" t="n"/>
-      <c r="N6" s="26" t="n"/>
-      <c r="O6" s="27" t="n"/>
-      <c r="P6" s="27" t="n"/>
-      <c r="Q6" s="27" t="n"/>
-      <c r="R6" s="27" t="n"/>
-      <c r="S6" s="27" t="n"/>
-      <c r="T6" s="27" t="n"/>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="O6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
       <c r="U6" t="n">
         <v>6</v>
       </c>
@@ -3607,13 +3648,16 @@
         <v>6</v>
       </c>
       <c r="X6" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -3625,11 +3669,20 @@
         <f>ROUND(AVERAGE(D7:AH7), 0)</f>
         <v/>
       </c>
+      <c r="D7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G7" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I7" s="9" t="n">
         <v>6</v>
@@ -3641,13 +3694,13 @@
         <v>6</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N7" s="26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O7" t="n">
         <v>6</v>
@@ -3665,25 +3718,28 @@
         <v>6</v>
       </c>
       <c r="T7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U7" t="n">
         <v>6</v>
       </c>
       <c r="V7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
@@ -3711,34 +3767,34 @@
         <v>0</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K8" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L8" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N8" s="26" t="n">
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
         <v>6</v>
@@ -3753,71 +3809,44 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X8" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C9" s="13">
         <f>ROUND(AVERAGE(D9:AH9), 0)</f>
         <v/>
       </c>
-      <c r="D9" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="M9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="26" t="n">
-        <v>6</v>
-      </c>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="10" t="n"/>
+      <c r="N9" s="26" t="n"/>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S9" t="n">
         <v>6</v>
@@ -3829,333 +3858,345 @@
         <v>6</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W9" t="n">
         <v>6</v>
       </c>
       <c r="X9" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C10" s="13">
         <f>ROUND(AVERAGE(D10:AH10), 0)</f>
         <v/>
       </c>
-      <c r="K10" s="10" t="n"/>
-      <c r="L10" s="10" t="n"/>
-      <c r="N10" s="26" t="n"/>
+      <c r="G10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="O10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
         <v>6</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C11" s="13">
         <f>ROUND(AVERAGE(D11:AH11), 0)</f>
         <v/>
       </c>
-      <c r="G11" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H11" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I11" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M11" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O11" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>4</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0</v>
-      </c>
+      <c r="K11" s="10" t="n"/>
+      <c r="L11" s="10" t="n"/>
+      <c r="N11" s="26" t="n"/>
+      <c r="O11" s="27" t="n"/>
+      <c r="P11" s="27" t="n"/>
+      <c r="Q11" s="27" t="n"/>
+      <c r="R11" s="27" t="n"/>
+      <c r="S11" s="27" t="n"/>
+      <c r="T11" s="27" t="n"/>
       <c r="U11" t="n">
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C12" s="13">
         <f>ROUND(AVERAGE(D12:AH12), 0)</f>
         <v/>
       </c>
-      <c r="K12" s="10" t="n"/>
-      <c r="L12" s="10" t="n"/>
-      <c r="N12" s="26" t="n"/>
-      <c r="O12" s="27" t="n"/>
-      <c r="P12" s="27" t="n"/>
-      <c r="Q12" s="27" t="n"/>
-      <c r="R12" s="27" t="n"/>
-      <c r="S12" s="27" t="n"/>
-      <c r="T12" s="27" t="n"/>
+      <c r="G12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N12" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O12" t="n">
+        <v>6</v>
+      </c>
+      <c r="P12" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>6</v>
+      </c>
+      <c r="R12" t="n">
+        <v>6</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>6</v>
+      </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="C13" s="13">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
-      <c r="G13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L13" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N13" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O13" t="n">
-        <v>6</v>
-      </c>
-      <c r="P13" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>6</v>
-      </c>
-      <c r="R13" t="n">
-        <v>6</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="n">
-        <v>6</v>
-      </c>
-      <c r="U13" t="n">
-        <v>6</v>
-      </c>
+      <c r="K13" s="10" t="n"/>
+      <c r="L13" s="10" t="n"/>
+      <c r="N13" s="26" t="n"/>
+      <c r="O13" s="27" t="n"/>
+      <c r="P13" s="27" t="n"/>
+      <c r="Q13" s="27" t="n"/>
+      <c r="R13" s="27" t="n"/>
+      <c r="S13" s="27" t="n"/>
+      <c r="T13" s="27" t="n"/>
+      <c r="U13" s="27" t="n"/>
       <c r="V13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>falcuns</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>28/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C14" s="13">
         <f>ROUND(AVERAGE(D14:AH14), 0)</f>
         <v/>
       </c>
-      <c r="K14" s="10" t="n"/>
-      <c r="L14" s="10" t="n"/>
-      <c r="N14" s="26" t="n"/>
-      <c r="O14" s="27" t="n"/>
-      <c r="P14" s="27" t="n"/>
-      <c r="Q14" s="27" t="n"/>
-      <c r="R14" s="27" t="n"/>
-      <c r="S14" s="27" t="n"/>
-      <c r="T14" s="27" t="n"/>
-      <c r="U14" s="27" t="n"/>
+      <c r="D14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O14" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>5</v>
+      </c>
+      <c r="R14" t="n">
+        <v>6</v>
+      </c>
+      <c r="S14" t="n">
+        <v>6</v>
+      </c>
+      <c r="T14" t="n">
+        <v>6</v>
+      </c>
+      <c r="U14" t="n">
+        <v>6</v>
+      </c>
       <c r="V14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C15" s="13">
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
-      <c r="D15" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M15" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N15" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O15" t="n">
-        <v>6</v>
-      </c>
-      <c r="P15" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>5</v>
-      </c>
+      <c r="K15" s="10" t="n"/>
+      <c r="L15" s="10" t="n"/>
+      <c r="N15" s="26" t="n"/>
+      <c r="O15" s="27" t="n"/>
+      <c r="P15" s="27" t="n"/>
+      <c r="Q15" s="27" t="n"/>
       <c r="R15" t="n">
         <v>6</v>
       </c>
@@ -4172,33 +4213,72 @@
         <v>6</v>
       </c>
       <c r="W15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="13">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="n"/>
-      <c r="N16" s="26" t="n"/>
-      <c r="O16" s="27" t="n"/>
-      <c r="P16" s="27" t="n"/>
-      <c r="Q16" s="27" t="n"/>
+      <c r="D16" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="O16" t="n">
+        <v>6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>6</v>
+      </c>
       <c r="R16" t="n">
         <v>6</v>
       </c>
@@ -4218,36 +4298,27 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C17" s="13">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="D17" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="H17" s="9" t="n">
         <v>6</v>
       </c>
@@ -4294,27 +4365,42 @@
         <v>6</v>
       </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C18" s="13">
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
+      <c r="D18" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="H18" s="9" t="n">
         <v>6</v>
       </c>
@@ -4358,19 +4444,22 @@
         <v>6</v>
       </c>
       <c r="V18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -4392,49 +4481,46 @@
         <v>6</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>6</v>
       </c>
       <c r="K19" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L19" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N19" s="26" t="n">
         <v>6</v>
       </c>
       <c r="O19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q19" t="n">
         <v>6</v>
       </c>
       <c r="R19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T19" t="n">
         <v>6</v>
       </c>
       <c r="U19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V19" t="n">
         <v>0</v>
@@ -4443,107 +4529,116 @@
         <v>0</v>
       </c>
       <c r="X19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C20" s="13">
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="D20" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="10" t="n"/>
       <c r="M20" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N20" s="26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>6</v>
+      </c>
+      <c r="W20" t="n">
+        <v>6</v>
+      </c>
+      <c r="X20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y20" t="n">
         <v>4</v>
-      </c>
-      <c r="P20" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" t="n">
-        <v>3</v>
-      </c>
-      <c r="T20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U20" t="n">
-        <v>4</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C21" s="13">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="K21" s="10" t="n"/>
-      <c r="L21" s="10" t="n"/>
+      <c r="D21" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L21" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M21" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N21" s="26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O21" t="n">
         <v>6</v>
@@ -4564,7 +4659,7 @@
         <v>6</v>
       </c>
       <c r="U21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V21" t="n">
         <v>6</v>
@@ -4574,67 +4669,34 @@
       </c>
       <c r="X21" t="n">
         <v>6</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C22" s="13">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
-      <c r="D22" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K22" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M22" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N22" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O22" t="n">
-        <v>6</v>
-      </c>
-      <c r="P22" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>6</v>
-      </c>
+      <c r="K22" s="10" t="n"/>
+      <c r="L22" s="10" t="n"/>
+      <c r="N22" s="10" t="n"/>
+      <c r="O22" s="27" t="n"/>
+      <c r="P22" s="27" t="n"/>
+      <c r="Q22" s="27" t="n"/>
       <c r="R22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S22" t="n">
         <v>6</v>
@@ -4652,32 +4714,62 @@
         <v>6</v>
       </c>
       <c r="X22" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C23" s="13">
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
-      <c r="K23" s="10" t="n"/>
-      <c r="L23" s="10" t="n"/>
-      <c r="N23" s="10" t="n"/>
-      <c r="O23" s="27" t="n"/>
-      <c r="P23" s="27" t="n"/>
-      <c r="Q23" s="27" t="n"/>
+      <c r="G23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M23" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N23" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O23" t="n">
+        <v>6</v>
+      </c>
+      <c r="P23" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>6</v>
+      </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S23" t="n">
         <v>6</v>
@@ -4692,16 +4784,19 @@
         <v>6</v>
       </c>
       <c r="W23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
@@ -4713,11 +4808,20 @@
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
+      <c r="D24" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I24" s="9" t="n">
         <v>6</v>
@@ -4726,16 +4830,16 @@
         <v>6</v>
       </c>
       <c r="K24" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L24" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M24" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N24" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
         <v>6</v>
@@ -4756,106 +4860,73 @@
         <v>6</v>
       </c>
       <c r="U24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X24" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y24" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C25" s="13">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
-      <c r="D25" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J25" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K25" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>6</v>
-      </c>
-      <c r="P25" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>6</v>
-      </c>
-      <c r="R25" t="n">
-        <v>6</v>
-      </c>
+      <c r="K25" s="10" t="n"/>
+      <c r="L25" s="10" t="n"/>
+      <c r="N25" s="10" t="n"/>
+      <c r="P25" s="27" t="n"/>
+      <c r="Q25" s="27" t="n"/>
+      <c r="R25" s="27" t="n"/>
       <c r="S25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C26" s="13">
@@ -4865,17 +4936,26 @@
       <c r="K26" s="10" t="n"/>
       <c r="L26" s="10" t="n"/>
       <c r="N26" s="10" t="n"/>
-      <c r="P26" s="27" t="n"/>
-      <c r="Q26" s="27" t="n"/>
-      <c r="R26" s="27" t="n"/>
+      <c r="O26" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="P26" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q26" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R26" t="n">
+        <v>6</v>
+      </c>
       <c r="S26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V26" t="n">
         <v>0</v>
@@ -4884,29 +4964,53 @@
         <v>0</v>
       </c>
       <c r="X26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C27" s="13">
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
-      <c r="K27" s="10" t="n"/>
-      <c r="L27" s="10" t="n"/>
-      <c r="N27" s="10" t="n"/>
+      <c r="G27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L27" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N27" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="O27" s="28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P27" s="28" t="n">
         <v>6</v>
@@ -4927,19 +5031,22 @@
         <v>6</v>
       </c>
       <c r="V27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W27" t="n">
         <v>0</v>
       </c>
       <c r="X27" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
@@ -4952,7 +5059,7 @@
         <v/>
       </c>
       <c r="G28" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H28" s="9" t="n">
         <v>6</v>
@@ -5003,39 +5110,27 @@
         <v>0</v>
       </c>
       <c r="X28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C29" s="13">
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="G29" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K29" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L29" s="10" t="n">
         <v>6</v>
       </c>
@@ -5054,7 +5149,7 @@
       <c r="Q29" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R29" t="n">
+      <c r="R29" s="28" t="n">
         <v>6</v>
       </c>
       <c r="S29" t="n">
@@ -5073,24 +5168,30 @@
         <v>0</v>
       </c>
       <c r="X29" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C30" s="13">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
+      <c r="K30" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L30" s="10" t="n">
         <v>6</v>
       </c>
@@ -5125,27 +5226,51 @@
         <v>6</v>
       </c>
       <c r="W30" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X30" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C31" s="13">
         <f>ROUND(AVERAGE(D31:AH31), 0)</f>
         <v/>
       </c>
+      <c r="D31" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="K31" s="10" t="n">
         <v>6</v>
       </c>
@@ -5174,25 +5299,28 @@
         <v>6</v>
       </c>
       <c r="T31" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V31" t="n">
         <v>6</v>
       </c>
       <c r="W31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X31" t="n">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
@@ -5205,7 +5333,7 @@
         <v/>
       </c>
       <c r="D32" s="14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E32" s="9" t="n">
         <v>6</v>
@@ -5223,7 +5351,7 @@
         <v>6</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K32" s="10" t="n">
         <v>6</v>
@@ -5249,29 +5377,32 @@
       <c r="R32" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S32" t="n">
+      <c r="S32" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T32" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X32" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
@@ -5284,7 +5415,7 @@
         <v/>
       </c>
       <c r="D33" s="14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E33" s="9" t="n">
         <v>6</v>
@@ -5302,7 +5433,7 @@
         <v>6</v>
       </c>
       <c r="J33" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K33" s="10" t="n">
         <v>6</v>
@@ -5338,19 +5469,22 @@
         <v>6</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X33" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
@@ -5362,27 +5496,7 @@
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
-      <c r="D34" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I34" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J34" s="10" t="n">
-        <v>6</v>
-      </c>
+      <c r="J34" s="10" t="n"/>
       <c r="K34" s="10" t="n">
         <v>6</v>
       </c>
@@ -5410,42 +5524,75 @@
       <c r="S34" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="T34" t="n">
+      <c r="T34" s="28" t="n">
         <v>6</v>
       </c>
       <c r="U34" t="n">
         <v>6</v>
       </c>
       <c r="V34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X34" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C35" s="13">
         <f>ROUND(AVERAGE(D35:AH35), 0)</f>
         <v/>
       </c>
-      <c r="K35" s="10" t="n"/>
-      <c r="L35" s="10" t="n"/>
-      <c r="N35" s="10" t="n"/>
+      <c r="G35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O35" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P35" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="28" t="n">
+        <v>6</v>
+      </c>
       <c r="R35" s="28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S35" s="28" t="n">
         <v>6</v>
@@ -5453,35 +5600,37 @@
       <c r="T35" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="U35" t="n">
+      <c r="U35" s="28" t="n">
         <v>6</v>
       </c>
       <c r="V35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X35" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C36" s="13">
         <f>ROUND(AVERAGE(D36:AH36), 0)</f>
         <v/>
       </c>
-      <c r="J36" s="10" t="n"/>
       <c r="K36" s="10" t="n">
         <v>6</v>
       </c>
@@ -5489,10 +5638,10 @@
         <v>6</v>
       </c>
       <c r="M36" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N36" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O36" s="28" t="n">
         <v>6</v>
@@ -5504,145 +5653,95 @@
         <v>6</v>
       </c>
       <c r="R36" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S36" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T36" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U36" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U36" s="28" t="n">
+        <v>0</v>
       </c>
       <c r="V36" t="n">
         <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X36" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>krigohard</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
         <f>ROUND(AVERAGE(D37:AH37), 0)</f>
         <v/>
       </c>
-      <c r="G37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J37" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K37" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L37" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N37" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O37" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P37" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q37" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R37" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S37" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T37" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U37" s="28" t="n">
-        <v>6</v>
-      </c>
+      <c r="K37" s="10" t="n"/>
+      <c r="L37" s="10" t="n"/>
+      <c r="M37" s="9" t="n"/>
+      <c r="N37" s="10" t="n"/>
+      <c r="O37" s="28" t="n"/>
+      <c r="P37" s="28" t="n"/>
+      <c r="Q37" s="28" t="n"/>
+      <c r="R37" s="28" t="n"/>
+      <c r="S37" s="28" t="n"/>
+      <c r="T37" s="28" t="n"/>
+      <c r="U37" s="28" t="n"/>
       <c r="V37" t="n">
         <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X37" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
         <f>ROUND(AVERAGE(D38:AH38), 0)</f>
         <v/>
       </c>
-      <c r="K38" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L38" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M38" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P38" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q38" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R38" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T38" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="U38" s="28" t="n">
-        <v>0</v>
-      </c>
+      <c r="K38" s="10" t="n"/>
+      <c r="L38" s="10" t="n"/>
+      <c r="M38" s="9" t="n"/>
+      <c r="N38" s="10" t="n"/>
+      <c r="O38" s="28" t="n"/>
+      <c r="P38" s="28" t="n"/>
+      <c r="Q38" s="28" t="n"/>
+      <c r="R38" s="28" t="n"/>
+      <c r="S38" s="28" t="n"/>
+      <c r="T38" s="28" t="n"/>
+      <c r="U38" s="28" t="n"/>
       <c r="V38" t="n">
         <v>0</v>
       </c>
@@ -5650,18 +5749,21 @@
         <v>0</v>
       </c>
       <c r="X38" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>krigohard</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5679,25 +5781,25 @@
       <c r="S39" s="28" t="n"/>
       <c r="T39" s="28" t="n"/>
       <c r="U39" s="28" t="n"/>
-      <c r="V39" t="n">
-        <v>0</v>
-      </c>
       <c r="W39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X39" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>Steninja:)</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5715,25 +5817,25 @@
       <c r="S40" s="28" t="n"/>
       <c r="T40" s="28" t="n"/>
       <c r="U40" s="28" t="n"/>
-      <c r="V40" t="n">
-        <v>0</v>
-      </c>
       <c r="W40" t="n">
         <v>0</v>
       </c>
       <c r="X40" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>ggvitotmm</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5751,22 +5853,22 @@
       <c r="S41" s="28" t="n"/>
       <c r="T41" s="28" t="n"/>
       <c r="U41" s="28" t="n"/>
-      <c r="W41" t="n">
-        <v>6</v>
-      </c>
       <c r="X41" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>Steninja:)</t>
+          <t>toxic</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5784,22 +5886,22 @@
       <c r="S42" s="28" t="n"/>
       <c r="T42" s="28" t="n"/>
       <c r="U42" s="28" t="n"/>
-      <c r="W42" t="n">
-        <v>0</v>
-      </c>
       <c r="X42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Splaticon</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -5817,19 +5919,19 @@
       <c r="S43" s="28" t="n"/>
       <c r="T43" s="28" t="n"/>
       <c r="U43" s="28" t="n"/>
-      <c r="X43" t="n">
+      <c r="Y43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>~¥AKAZA¥~</t>
+          <t>samuel</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5847,19 +5949,19 @@
       <c r="S44" s="28" t="n"/>
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
-      <c r="X44" t="n">
+      <c r="Y44" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>ggvitotmm</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5877,19 +5979,19 @@
       <c r="S45" s="28" t="n"/>
       <c r="T45" s="28" t="n"/>
       <c r="U45" s="28" t="n"/>
-      <c r="X45" t="n">
-        <v>0</v>
+      <c r="Y45" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>toxic</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5907,19 +6009,19 @@
       <c r="S46" s="28" t="n"/>
       <c r="T46" s="28" t="n"/>
       <c r="U46" s="28" t="n"/>
-      <c r="X46" t="n">
-        <v>0</v>
+      <c r="Y46" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>color052</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C47" s="13">
@@ -5937,19 +6039,19 @@
       <c r="S47" s="28" t="n"/>
       <c r="T47" s="28" t="n"/>
       <c r="U47" s="28" t="n"/>
-      <c r="X47" t="n">
+      <c r="Y47" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -5967,16 +6069,19 @@
       <c r="S48" s="28" t="n"/>
       <c r="T48" s="28" t="n"/>
       <c r="U48" s="28" t="n"/>
+      <c r="Y48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>samuel</t>
+          <t>piter</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -5994,16 +6099,19 @@
       <c r="S49" s="28" t="n"/>
       <c r="T49" s="28" t="n"/>
       <c r="U49" s="28" t="n"/>
+      <c r="Y49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="29">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>andrea</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C50" s="13">
@@ -6021,33 +6129,9 @@
       <c r="S50" s="28" t="n"/>
       <c r="T50" s="28" t="n"/>
       <c r="U50" s="28" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>matteo</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>13/04/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="O51" s="28" t="n"/>
-      <c r="P51" s="28" t="n"/>
-      <c r="Q51" s="28" t="n"/>
-      <c r="R51" s="28" t="n"/>
-      <c r="S51" s="28" t="n"/>
-      <c r="T51" s="28" t="n"/>
-      <c r="U51" s="28" t="n"/>
+      <c r="Y50" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AT1">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-19
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3651,7 +3651,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -3733,7 +3733,7 @@
         <v>6</v>
       </c>
       <c r="Y7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -3815,7 +3815,7 @@
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -3867,7 +3867,7 @@
         <v>6</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -4173,7 +4173,7 @@
         <v>6</v>
       </c>
       <c r="Y14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -4589,7 +4589,7 @@
         <v>6</v>
       </c>
       <c r="Y20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -4790,7 +4790,7 @@
         <v>6</v>
       </c>
       <c r="Y23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -5232,7 +5232,7 @@
         <v>2</v>
       </c>
       <c r="Y30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
@@ -5540,7 +5540,7 @@
         <v>6</v>
       </c>
       <c r="Y34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
@@ -5926,12 +5926,12 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>samuel</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5950,13 +5950,13 @@
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
       <c r="Y44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
@@ -5980,13 +5980,13 @@
       <c r="T45" s="28" t="n"/>
       <c r="U45" s="28" t="n"/>
       <c r="Y45" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
@@ -6010,13 +6010,13 @@
       <c r="T46" s="28" t="n"/>
       <c r="U46" s="28" t="n"/>
       <c r="Y46" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
@@ -6046,7 +6046,7 @@
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>piter</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
@@ -6076,7 +6076,7 @@
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>piter</t>
+          <t>andrea</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
@@ -6103,36 +6103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1" s="29">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>andrea</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>18/04/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="13">
-        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="10" t="n"/>
-      <c r="L50" s="10" t="n"/>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="10" t="n"/>
-      <c r="O50" s="28" t="n"/>
-      <c r="P50" s="28" t="n"/>
-      <c r="Q50" s="28" t="n"/>
-      <c r="R50" s="28" t="n"/>
-      <c r="S50" s="28" t="n"/>
-      <c r="T50" s="28" t="n"/>
-      <c r="U50" s="28" t="n"/>
-      <c r="Y50" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="50" ht="15.75" customHeight="1" s="29"/>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-20
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3184,7 +3184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH49"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -6103,7 +6103,60 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1" s="29"/>
+    <row r="50" ht="15.75" customHeight="1" s="29">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>Ema alba003</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="13">
+        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="10" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="10" t="n"/>
+      <c r="O50" s="28" t="n"/>
+      <c r="P50" s="28" t="n"/>
+      <c r="Q50" s="28" t="n"/>
+      <c r="R50" s="28" t="n"/>
+      <c r="S50" s="28" t="n"/>
+      <c r="T50" s="28" t="n"/>
+      <c r="U50" s="28" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>satana03</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="13">
+        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="10" t="n"/>
+      <c r="L51" s="10" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="10" t="n"/>
+      <c r="O51" s="28" t="n"/>
+      <c r="P51" s="28" t="n"/>
+      <c r="Q51" s="28" t="n"/>
+      <c r="R51" s="28" t="n"/>
+      <c r="S51" s="28" t="n"/>
+      <c r="T51" s="28" t="n"/>
+      <c r="U51" s="28" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Games data - 2026-04-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA49"/>
+  <dimension ref="A1:AA47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="21" min="1" max="1"/>
@@ -1832,12 +1832,12 @@
     <row r="21">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C21" s="16">
@@ -1849,15 +1849,17 @@
         <v/>
       </c>
       <c r="E21" s="20" t="n">
-        <v>6550</v>
+        <v>23750</v>
       </c>
       <c r="F21" s="26" t="n"/>
       <c r="G21" s="26" t="n"/>
       <c r="H21" s="26" t="n"/>
       <c r="I21" s="26" t="n"/>
-      <c r="J21" s="26" t="n"/>
+      <c r="J21" s="26" t="n">
+        <v>4300</v>
+      </c>
       <c r="K21" s="26" t="n">
-        <v>4600</v>
+        <v>4200</v>
       </c>
       <c r="L21" s="26" t="n"/>
       <c r="M21" s="26" t="n"/>
@@ -1875,12 +1877,12 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C22" s="16">
@@ -1892,14 +1894,16 @@
         <v/>
       </c>
       <c r="E22" s="20" t="n">
-        <v>23750</v>
+        <v>44550</v>
       </c>
       <c r="F22" s="26" t="n"/>
       <c r="G22" s="26" t="n"/>
       <c r="H22" s="26" t="n"/>
-      <c r="I22" s="26" t="n"/>
+      <c r="I22" s="26" t="n">
+        <v>4300</v>
+      </c>
       <c r="J22" s="26" t="n">
-        <v>4300</v>
+        <v>4100</v>
       </c>
       <c r="K22" s="26" t="n">
         <v>4200</v>
@@ -1920,12 +1924,12 @@
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C23" s="16">
@@ -1937,19 +1941,25 @@
         <v/>
       </c>
       <c r="E23" s="20" t="n">
-        <v>44550</v>
-      </c>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="26" t="n"/>
-      <c r="H23" s="26" t="n"/>
+        <v>32200</v>
+      </c>
+      <c r="F23" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G23" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H23" s="26" t="n">
+        <v>4100</v>
+      </c>
       <c r="I23" s="26" t="n">
-        <v>4300</v>
+        <v>4400</v>
       </c>
       <c r="J23" s="26" t="n">
-        <v>4100</v>
+        <v>4700</v>
       </c>
       <c r="K23" s="26" t="n">
-        <v>4200</v>
+        <v>4150</v>
       </c>
       <c r="L23" s="26" t="n"/>
       <c r="M23" s="26" t="n"/>
@@ -1967,7 +1977,7 @@
     <row r="24">
       <c r="A24" s="20" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B24" s="22" t="inlineStr">
@@ -1984,22 +1994,20 @@
         <v/>
       </c>
       <c r="E24" s="20" t="n">
-        <v>32200</v>
-      </c>
-      <c r="F24" s="26" t="n">
-        <v>4000</v>
-      </c>
+        <v>33550</v>
+      </c>
+      <c r="F24" s="26" t="n"/>
       <c r="G24" s="26" t="n">
         <v>4000</v>
       </c>
       <c r="H24" s="26" t="n">
-        <v>4100</v>
+        <v>10000</v>
       </c>
       <c r="I24" s="26" t="n">
-        <v>4400</v>
+        <v>5000</v>
       </c>
       <c r="J24" s="26" t="n">
-        <v>4700</v>
+        <v>5050</v>
       </c>
       <c r="K24" s="26" t="n">
         <v>4150</v>
@@ -2020,12 +2028,12 @@
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C25" s="16">
@@ -2037,23 +2045,21 @@
         <v/>
       </c>
       <c r="E25" s="20" t="n">
-        <v>33550</v>
+        <v>123800</v>
       </c>
       <c r="F25" s="26" t="n"/>
-      <c r="G25" s="26" t="n">
+      <c r="G25" s="26" t="n"/>
+      <c r="H25" s="26" t="n">
+        <v>4050</v>
+      </c>
+      <c r="I25" s="26" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J25" s="26" t="n">
         <v>4000</v>
       </c>
-      <c r="H25" s="26" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I25" s="26" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J25" s="26" t="n">
-        <v>5050</v>
-      </c>
       <c r="K25" s="26" t="n">
-        <v>4150</v>
+        <v>4100</v>
       </c>
       <c r="L25" s="26" t="n"/>
       <c r="M25" s="26" t="n"/>
@@ -2071,12 +2077,12 @@
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C26" s="16">
@@ -2088,21 +2094,21 @@
         <v/>
       </c>
       <c r="E26" s="20" t="n">
-        <v>123800</v>
+        <v>41000</v>
       </c>
       <c r="F26" s="26" t="n"/>
       <c r="G26" s="26" t="n"/>
       <c r="H26" s="26" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I26" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J26" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="K26" s="26" t="n">
         <v>4050</v>
-      </c>
-      <c r="I26" s="26" t="n">
-        <v>4100</v>
-      </c>
-      <c r="J26" s="26" t="n">
-        <v>4000</v>
-      </c>
-      <c r="K26" s="26" t="n">
-        <v>4100</v>
       </c>
       <c r="L26" s="26" t="n"/>
       <c r="M26" s="26" t="n"/>
@@ -2120,12 +2126,12 @@
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C27" s="16">
@@ -2137,18 +2143,14 @@
         <v/>
       </c>
       <c r="E27" s="20" t="n">
-        <v>41000</v>
+        <v>27155</v>
       </c>
       <c r="F27" s="26" t="n"/>
       <c r="G27" s="26" t="n"/>
-      <c r="H27" s="26" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I27" s="26" t="n">
-        <v>4000</v>
-      </c>
+      <c r="H27" s="26" t="n"/>
+      <c r="I27" s="26" t="n"/>
       <c r="J27" s="26" t="n">
-        <v>150</v>
+        <v>4250</v>
       </c>
       <c r="K27" s="26" t="n">
         <v>4050</v>
@@ -2169,12 +2171,12 @@
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C28" s="16">
@@ -2186,17 +2188,21 @@
         <v/>
       </c>
       <c r="E28" s="20" t="n">
-        <v>27155</v>
+        <v>29350</v>
       </c>
       <c r="F28" s="26" t="n"/>
       <c r="G28" s="26" t="n"/>
-      <c r="H28" s="26" t="n"/>
-      <c r="I28" s="26" t="n"/>
+      <c r="H28" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="26" t="n">
+        <v>3500</v>
+      </c>
       <c r="J28" s="26" t="n">
-        <v>4250</v>
+        <v>4050</v>
       </c>
       <c r="K28" s="26" t="n">
-        <v>4050</v>
+        <v>4000</v>
       </c>
       <c r="L28" s="26" t="n"/>
       <c r="M28" s="26" t="n"/>
@@ -2214,12 +2220,12 @@
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C29" s="16">
@@ -2231,19 +2237,25 @@
         <v/>
       </c>
       <c r="E29" s="20" t="n">
-        <v>65375</v>
-      </c>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="26" t="n"/>
-      <c r="H29" s="26" t="n"/>
+        <v>39900</v>
+      </c>
+      <c r="F29" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G29" s="26" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H29" s="26" t="n">
+        <v>4050</v>
+      </c>
       <c r="I29" s="26" t="n">
-        <v>6250</v>
+        <v>5600</v>
       </c>
       <c r="J29" s="26" t="n">
-        <v>3250</v>
+        <v>1300</v>
       </c>
       <c r="K29" s="26" t="n">
-        <v>4050</v>
+        <v>3100</v>
       </c>
       <c r="L29" s="26" t="n"/>
       <c r="M29" s="26" t="n"/>
@@ -2261,7 +2273,7 @@
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B30" s="22" t="inlineStr">
@@ -2278,21 +2290,21 @@
         <v/>
       </c>
       <c r="E30" s="20" t="n">
-        <v>29350</v>
+        <v>31825</v>
       </c>
       <c r="F30" s="26" t="n"/>
       <c r="G30" s="26" t="n"/>
       <c r="H30" s="26" t="n">
-        <v>0</v>
+        <v>3650</v>
       </c>
       <c r="I30" s="26" t="n">
-        <v>3500</v>
+        <v>7600</v>
       </c>
       <c r="J30" s="26" t="n">
-        <v>4050</v>
+        <v>3150</v>
       </c>
       <c r="K30" s="26" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="L30" s="26" t="n"/>
       <c r="M30" s="26" t="n"/>
@@ -2310,12 +2322,12 @@
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="C31" s="16">
@@ -2327,25 +2339,17 @@
         <v/>
       </c>
       <c r="E31" s="20" t="n">
-        <v>39900</v>
-      </c>
-      <c r="F31" s="26" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G31" s="26" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H31" s="26" t="n">
-        <v>4050</v>
-      </c>
-      <c r="I31" s="26" t="n">
-        <v>5600</v>
-      </c>
+        <v>2150</v>
+      </c>
+      <c r="F31" s="26" t="n"/>
+      <c r="G31" s="26" t="n"/>
+      <c r="H31" s="26" t="n"/>
+      <c r="I31" s="26" t="n"/>
       <c r="J31" s="26" t="n">
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="K31" s="26" t="n">
-        <v>3100</v>
+        <v>1750</v>
       </c>
       <c r="L31" s="26" t="n"/>
       <c r="M31" s="26" t="n"/>
@@ -2363,12 +2367,12 @@
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C32" s="16">
@@ -2380,21 +2384,19 @@
         <v/>
       </c>
       <c r="E32" s="20" t="n">
-        <v>31825</v>
+        <v>75000</v>
       </c>
       <c r="F32" s="26" t="n"/>
       <c r="G32" s="26" t="n"/>
-      <c r="H32" s="26" t="n">
-        <v>3650</v>
-      </c>
+      <c r="H32" s="26" t="n"/>
       <c r="I32" s="26" t="n">
-        <v>7600</v>
+        <v>0</v>
       </c>
       <c r="J32" s="26" t="n">
-        <v>3150</v>
+        <v>950</v>
       </c>
       <c r="K32" s="26" t="n">
-        <v>3000</v>
+        <v>1400</v>
       </c>
       <c r="L32" s="26" t="n"/>
       <c r="M32" s="26" t="n"/>
@@ -2412,12 +2414,12 @@
     <row r="33">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C33" s="16">
@@ -2429,17 +2431,19 @@
         <v/>
       </c>
       <c r="E33" s="20" t="n">
-        <v>2150</v>
+        <v>6800</v>
       </c>
       <c r="F33" s="26" t="n"/>
       <c r="G33" s="26" t="n"/>
       <c r="H33" s="26" t="n"/>
-      <c r="I33" s="26" t="n"/>
+      <c r="I33" s="26" t="n">
+        <v>4150</v>
+      </c>
       <c r="J33" s="26" t="n">
-        <v>0</v>
+        <v>2650</v>
       </c>
       <c r="K33" s="26" t="n">
-        <v>1750</v>
+        <v>1050</v>
       </c>
       <c r="L33" s="26" t="n"/>
       <c r="M33" s="26" t="n"/>
@@ -2457,12 +2461,12 @@
     <row r="34">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C34" s="16">
@@ -2474,21 +2478,15 @@
         <v/>
       </c>
       <c r="E34" s="20" t="n">
-        <v>73250</v>
+        <v>18000</v>
       </c>
       <c r="F34" s="26" t="n"/>
       <c r="G34" s="26" t="n"/>
-      <c r="H34" s="26" t="n">
-        <v>1300</v>
-      </c>
-      <c r="I34" s="26" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J34" s="26" t="n">
-        <v>3000</v>
-      </c>
+      <c r="H34" s="26" t="n"/>
+      <c r="I34" s="26" t="n"/>
+      <c r="J34" s="26" t="n"/>
       <c r="K34" s="26" t="n">
-        <v>1600</v>
+        <v>600</v>
       </c>
       <c r="L34" s="26" t="n"/>
       <c r="M34" s="26" t="n"/>
@@ -2506,12 +2504,12 @@
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C35" s="16">
@@ -2523,19 +2521,21 @@
         <v/>
       </c>
       <c r="E35" s="20" t="n">
-        <v>75000</v>
+        <v>15150</v>
       </c>
       <c r="F35" s="26" t="n"/>
       <c r="G35" s="26" t="n"/>
-      <c r="H35" s="26" t="n"/>
+      <c r="H35" s="26" t="n">
+        <v>500</v>
+      </c>
       <c r="I35" s="26" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="J35" s="26" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="K35" s="26" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="L35" s="26" t="n"/>
       <c r="M35" s="26" t="n"/>
@@ -2553,7 +2553,7 @@
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B36" s="22" t="inlineStr">
@@ -2570,19 +2570,19 @@
         <v/>
       </c>
       <c r="E36" s="20" t="n">
-        <v>6800</v>
+        <v>69000</v>
       </c>
       <c r="F36" s="26" t="n"/>
       <c r="G36" s="26" t="n"/>
       <c r="H36" s="26" t="n"/>
       <c r="I36" s="26" t="n">
-        <v>4150</v>
+        <v>10000</v>
       </c>
       <c r="J36" s="26" t="n">
-        <v>2650</v>
+        <v>10000</v>
       </c>
       <c r="K36" s="26" t="n">
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="L36" s="26" t="n"/>
       <c r="M36" s="26" t="n"/>
@@ -2600,12 +2600,12 @@
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B37" s="22" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>27/03/2026</t>
         </is>
       </c>
       <c r="C37" s="16">
@@ -2617,16 +2617,14 @@
         <v/>
       </c>
       <c r="E37" s="20" t="n">
-        <v>18000</v>
+        <v>250</v>
       </c>
       <c r="F37" s="26" t="n"/>
       <c r="G37" s="26" t="n"/>
       <c r="H37" s="26" t="n"/>
       <c r="I37" s="26" t="n"/>
       <c r="J37" s="26" t="n"/>
-      <c r="K37" s="26" t="n">
-        <v>600</v>
-      </c>
+      <c r="K37" s="26" t="n"/>
       <c r="L37" s="26" t="n"/>
       <c r="M37" s="26" t="n"/>
       <c r="N37" s="26" t="n"/>
@@ -2643,12 +2641,12 @@
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>jacopo</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C38" s="16">
@@ -2660,16 +2658,14 @@
         <v/>
       </c>
       <c r="E38" s="20" t="n">
-        <v>3550</v>
+        <v>43650</v>
       </c>
       <c r="F38" s="26" t="n"/>
       <c r="G38" s="26" t="n"/>
       <c r="H38" s="26" t="n"/>
       <c r="I38" s="26" t="n"/>
       <c r="J38" s="26" t="n"/>
-      <c r="K38" s="26" t="n">
-        <v>400</v>
-      </c>
+      <c r="K38" s="26" t="n"/>
       <c r="L38" s="26" t="n"/>
       <c r="M38" s="26" t="n"/>
       <c r="N38" s="26" t="n"/>
@@ -2686,12 +2682,12 @@
     <row r="39">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B39" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C39" s="16">
@@ -2703,16 +2699,14 @@
         <v/>
       </c>
       <c r="E39" s="20" t="n">
-        <v>5350</v>
+        <v>21200</v>
       </c>
       <c r="F39" s="26" t="n"/>
       <c r="G39" s="26" t="n"/>
       <c r="H39" s="26" t="n"/>
       <c r="I39" s="26" t="n"/>
       <c r="J39" s="26" t="n"/>
-      <c r="K39" s="26" t="n">
-        <v>300</v>
-      </c>
+      <c r="K39" s="26" t="n"/>
       <c r="L39" s="26" t="n"/>
       <c r="M39" s="26" t="n"/>
       <c r="N39" s="26" t="n"/>
@@ -2729,12 +2723,12 @@
     <row r="40">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C40" s="16">
@@ -2746,18 +2740,14 @@
         <v/>
       </c>
       <c r="E40" s="20" t="n">
-        <v>11775</v>
+        <v>13125</v>
       </c>
       <c r="F40" s="26" t="n"/>
       <c r="G40" s="26" t="n"/>
       <c r="H40" s="26" t="n"/>
       <c r="I40" s="26" t="n"/>
-      <c r="J40" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" s="26" t="n">
-        <v>300</v>
-      </c>
+      <c r="J40" s="26" t="n"/>
+      <c r="K40" s="26" t="n"/>
       <c r="L40" s="26" t="n"/>
       <c r="M40" s="26" t="n"/>
       <c r="N40" s="26" t="n"/>
@@ -2774,12 +2764,12 @@
     <row r="41">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C41" s="16">
@@ -2791,16 +2781,14 @@
         <v/>
       </c>
       <c r="E41" s="20" t="n">
-        <v>1800</v>
+        <v>250</v>
       </c>
       <c r="F41" s="26" t="n"/>
       <c r="G41" s="26" t="n"/>
       <c r="H41" s="26" t="n"/>
       <c r="I41" s="26" t="n"/>
       <c r="J41" s="26" t="n"/>
-      <c r="K41" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="K41" s="26" t="n"/>
       <c r="L41" s="26" t="n"/>
       <c r="M41" s="26" t="n"/>
       <c r="N41" s="26" t="n"/>
@@ -2817,12 +2805,12 @@
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C42" s="16">
@@ -2834,16 +2822,14 @@
         <v/>
       </c>
       <c r="E42" s="20" t="n">
-        <v>1825</v>
+        <v>0</v>
       </c>
       <c r="F42" s="26" t="n"/>
       <c r="G42" s="26" t="n"/>
       <c r="H42" s="26" t="n"/>
       <c r="I42" s="26" t="n"/>
       <c r="J42" s="26" t="n"/>
-      <c r="K42" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="K42" s="26" t="n"/>
       <c r="L42" s="26" t="n"/>
       <c r="M42" s="26" t="n"/>
       <c r="N42" s="26" t="n"/>
@@ -2860,12 +2846,12 @@
     <row r="43">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C43" s="16">
@@ -2877,22 +2863,14 @@
         <v/>
       </c>
       <c r="E43" s="20" t="n">
-        <v>15150</v>
+        <v>36750</v>
       </c>
       <c r="F43" s="26" t="n"/>
       <c r="G43" s="26" t="n"/>
-      <c r="H43" s="26" t="n">
-        <v>500</v>
-      </c>
-      <c r="I43" s="26" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J43" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="H43" s="26" t="n"/>
+      <c r="I43" s="26" t="n"/>
+      <c r="J43" s="26" t="n"/>
+      <c r="K43" s="26" t="n"/>
       <c r="L43" s="26" t="n"/>
       <c r="M43" s="26" t="n"/>
       <c r="N43" s="26" t="n"/>
@@ -2909,12 +2887,12 @@
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C44" s="16">
@@ -2926,16 +2904,14 @@
         <v/>
       </c>
       <c r="E44" s="20" t="n">
-        <v>0</v>
+        <v>11250</v>
       </c>
       <c r="F44" s="26" t="n"/>
       <c r="G44" s="26" t="n"/>
       <c r="H44" s="26" t="n"/>
       <c r="I44" s="26" t="n"/>
       <c r="J44" s="26" t="n"/>
-      <c r="K44" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="K44" s="26" t="n"/>
       <c r="L44" s="26" t="n"/>
       <c r="M44" s="26" t="n"/>
       <c r="N44" s="26" t="n"/>
@@ -2952,12 +2928,12 @@
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>Spiderman</t>
+          <t>Steninja:)</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C45" s="16">
@@ -2969,16 +2945,14 @@
         <v/>
       </c>
       <c r="E45" s="20" t="n">
-        <v>23625</v>
+        <v>700</v>
       </c>
       <c r="F45" s="26" t="n"/>
       <c r="G45" s="26" t="n"/>
       <c r="H45" s="26" t="n"/>
       <c r="I45" s="26" t="n"/>
       <c r="J45" s="26" t="n"/>
-      <c r="K45" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="K45" s="26" t="n"/>
       <c r="L45" s="26" t="n"/>
       <c r="M45" s="26" t="n"/>
       <c r="N45" s="26" t="n"/>
@@ -2995,12 +2969,12 @@
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C46" s="16">
@@ -3012,18 +2986,14 @@
         <v/>
       </c>
       <c r="E46" s="20" t="n">
-        <v>21145</v>
+        <v>40640</v>
       </c>
       <c r="F46" s="26" t="n"/>
       <c r="G46" s="26" t="n"/>
       <c r="H46" s="26" t="n"/>
       <c r="I46" s="26" t="n"/>
-      <c r="J46" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="J46" s="26" t="n"/>
+      <c r="K46" s="26" t="n"/>
       <c r="L46" s="26" t="n"/>
       <c r="M46" s="26" t="n"/>
       <c r="N46" s="26" t="n"/>
@@ -3040,12 +3010,12 @@
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>satana03</t>
         </is>
       </c>
       <c r="B47" s="22" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C47" s="16">
@@ -3057,20 +3027,14 @@
         <v/>
       </c>
       <c r="E47" s="20" t="n">
-        <v>69000</v>
+        <v>800</v>
       </c>
       <c r="F47" s="26" t="n"/>
       <c r="G47" s="26" t="n"/>
       <c r="H47" s="26" t="n"/>
-      <c r="I47" s="26" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J47" s="26" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K47" s="26" t="n">
-        <v>0</v>
-      </c>
+      <c r="I47" s="26" t="n"/>
+      <c r="J47" s="26" t="n"/>
+      <c r="K47" s="26" t="n"/>
       <c r="L47" s="26" t="n"/>
       <c r="M47" s="26" t="n"/>
       <c r="N47" s="26" t="n"/>
@@ -3083,88 +3047,6 @@
       <c r="U47" s="26" t="n"/>
       <c r="V47" s="26" t="n"/>
       <c r="W47" s="26" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>Er Caciotta</t>
-        </is>
-      </c>
-      <c r="B48" s="22" t="inlineStr">
-        <is>
-          <t>27/03/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="16">
-        <f>ROUND(AVERAGE(F48:AB48), 0)</f>
-        <v/>
-      </c>
-      <c r="D48" s="1">
-        <f>SUM(F48:AB48)</f>
-        <v/>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>10025</v>
-      </c>
-      <c r="F48" s="26" t="n"/>
-      <c r="G48" s="26" t="n"/>
-      <c r="H48" s="26" t="n"/>
-      <c r="I48" s="26" t="n"/>
-      <c r="J48" s="26" t="n"/>
-      <c r="K48" s="26" t="n"/>
-      <c r="L48" s="26" t="n"/>
-      <c r="M48" s="26" t="n"/>
-      <c r="N48" s="26" t="n"/>
-      <c r="O48" s="26" t="n"/>
-      <c r="P48" s="26" t="n"/>
-      <c r="Q48" s="26" t="n"/>
-      <c r="R48" s="26" t="n"/>
-      <c r="S48" s="26" t="n"/>
-      <c r="T48" s="26" t="n"/>
-      <c r="U48" s="26" t="n"/>
-      <c r="V48" s="26" t="n"/>
-      <c r="W48" s="26" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>falcuns</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>27/03/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="16">
-        <f>ROUND(AVERAGE(F49:AB49), 0)</f>
-        <v/>
-      </c>
-      <c r="D49" s="1">
-        <f>SUM(F49:AB49)</f>
-        <v/>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>250</v>
-      </c>
-      <c r="F49" s="26" t="n"/>
-      <c r="G49" s="26" t="n"/>
-      <c r="H49" s="26" t="n"/>
-      <c r="I49" s="26" t="n"/>
-      <c r="J49" s="26" t="n"/>
-      <c r="K49" s="26" t="n"/>
-      <c r="L49" s="26" t="n"/>
-      <c r="M49" s="26" t="n"/>
-      <c r="N49" s="26" t="n"/>
-      <c r="O49" s="26" t="n"/>
-      <c r="P49" s="26" t="n"/>
-      <c r="Q49" s="26" t="n"/>
-      <c r="R49" s="26" t="n"/>
-      <c r="S49" s="26" t="n"/>
-      <c r="T49" s="26" t="n"/>
-      <c r="U49" s="26" t="n"/>
-      <c r="V49" s="26" t="n"/>
-      <c r="W49" s="26" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="29" thickBot="1"/>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3148,7 +3148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="Z1" s="7" t="inlineStr">
         <is>
-          <t>Colonna24</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="AA1" s="7" t="inlineStr">
@@ -3396,6 +3396,9 @@
       <c r="Y2" t="n">
         <v>0</v>
       </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -3452,6 +3455,9 @@
         <v>0</v>
       </c>
       <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3502,6 +3508,9 @@
         <v>6</v>
       </c>
       <c r="Y4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3544,6 +3553,9 @@
       <c r="Y5" t="n">
         <v>0</v>
       </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -3617,6 +3629,9 @@
       <c r="Y6" t="n">
         <v>6</v>
       </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -3699,6 +3714,9 @@
       <c r="Y7" t="n">
         <v>6</v>
       </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -3779,6 +3797,9 @@
         <v>0</v>
       </c>
       <c r="Y8" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z8" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3833,6 +3854,9 @@
       <c r="Y9" t="n">
         <v>6</v>
       </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -3904,6 +3928,9 @@
         <v>6</v>
       </c>
       <c r="Y10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3946,6 +3973,9 @@
       <c r="Y11" t="n">
         <v>0</v>
       </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -4017,6 +4047,9 @@
         <v>0</v>
       </c>
       <c r="Y12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4057,6 +4090,9 @@
       <c r="Y13" t="n">
         <v>0</v>
       </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -4137,6 +4173,9 @@
         <v>6</v>
       </c>
       <c r="Y14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z14" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4185,6 +4224,9 @@
       <c r="Y15" t="n">
         <v>0</v>
       </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -4267,6 +4309,9 @@
       <c r="Y16" t="n">
         <v>0</v>
       </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -4337,6 +4382,9 @@
       <c r="Y17" t="n">
         <v>6</v>
       </c>
+      <c r="Z17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -4419,6 +4467,9 @@
       <c r="Y18" t="n">
         <v>0</v>
       </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -4496,6 +4547,9 @@
         <v>0</v>
       </c>
       <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4555,6 +4609,9 @@
       <c r="Y20" t="n">
         <v>6</v>
       </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -4635,6 +4692,9 @@
         <v>6</v>
       </c>
       <c r="Y21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4683,6 +4743,9 @@
       <c r="Y22" t="n">
         <v>6</v>
       </c>
+      <c r="Z22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -4756,6 +4819,9 @@
       <c r="Y23" t="n">
         <v>2</v>
       </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
@@ -4836,6 +4902,9 @@
         <v>6</v>
       </c>
       <c r="Y24" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4881,6 +4950,9 @@
       <c r="Y25" t="n">
         <v>0</v>
       </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
@@ -4933,6 +5005,9 @@
       <c r="Y26" t="n">
         <v>0</v>
       </c>
+      <c r="Z26" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -5006,6 +5081,9 @@
       <c r="Y27" t="n">
         <v>0</v>
       </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
@@ -5079,6 +5157,9 @@
       <c r="Y28" t="n">
         <v>0</v>
       </c>
+      <c r="Z28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -5137,6 +5218,9 @@
       <c r="Y29" t="n">
         <v>6</v>
       </c>
+      <c r="Z29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
@@ -5198,6 +5282,9 @@
       <c r="Y30" t="n">
         <v>6</v>
       </c>
+      <c r="Z30" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
@@ -5280,6 +5367,9 @@
       <c r="Y31" t="n">
         <v>0</v>
       </c>
+      <c r="Z31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -5362,6 +5452,9 @@
       <c r="Y32" t="n">
         <v>0</v>
       </c>
+      <c r="Z32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
@@ -5444,6 +5537,9 @@
       <c r="Y33" t="n">
         <v>3</v>
       </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -5506,6 +5602,9 @@
       <c r="Y34" t="n">
         <v>6</v>
       </c>
+      <c r="Z34" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
@@ -5579,6 +5678,9 @@
       <c r="Y35" t="n">
         <v>0</v>
       </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
@@ -5640,11 +5742,14 @@
       <c r="Y36" t="n">
         <v>0</v>
       </c>
+      <c r="Z36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>krigohard</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
@@ -5674,21 +5779,24 @@
         <v>0</v>
       </c>
       <c r="X37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
@@ -5706,23 +5814,23 @@
       <c r="S38" s="28" t="n"/>
       <c r="T38" s="28" t="n"/>
       <c r="U38" s="28" t="n"/>
-      <c r="V38" t="n">
-        <v>0</v>
-      </c>
       <c r="W38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X38" t="n">
         <v>6</v>
       </c>
       <c r="Y38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Steninja:)</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
@@ -5746,24 +5854,27 @@
       <c r="T39" s="28" t="n"/>
       <c r="U39" s="28" t="n"/>
       <c r="W39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Steninja:)</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5781,25 +5892,22 @@
       <c r="S40" s="28" t="n"/>
       <c r="T40" s="28" t="n"/>
       <c r="U40" s="28" t="n"/>
-      <c r="W40" t="n">
-        <v>0</v>
-      </c>
-      <c r="X40" t="n">
-        <v>0</v>
-      </c>
       <c r="Y40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>ggvitotmm</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5817,22 +5925,22 @@
       <c r="S41" s="28" t="n"/>
       <c r="T41" s="28" t="n"/>
       <c r="U41" s="28" t="n"/>
-      <c r="X41" t="n">
-        <v>0</v>
-      </c>
       <c r="Y41" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>toxic</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5850,22 +5958,22 @@
       <c r="S42" s="28" t="n"/>
       <c r="T42" s="28" t="n"/>
       <c r="U42" s="28" t="n"/>
-      <c r="X42" t="n">
-        <v>0</v>
-      </c>
       <c r="Y42" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -5884,13 +5992,16 @@
       <c r="T43" s="28" t="n"/>
       <c r="U43" s="28" t="n"/>
       <c r="Y43" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
@@ -5914,18 +6025,21 @@
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
       <c r="Y44" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5943,19 +6057,19 @@
       <c r="S45" s="28" t="n"/>
       <c r="T45" s="28" t="n"/>
       <c r="U45" s="28" t="n"/>
-      <c r="Y45" t="n">
-        <v>6</v>
+      <c r="Z45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>satana03</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5973,19 +6087,19 @@
       <c r="S46" s="28" t="n"/>
       <c r="T46" s="28" t="n"/>
       <c r="U46" s="28" t="n"/>
-      <c r="Y46" t="n">
-        <v>4</v>
+      <c r="Z46" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C47" s="13">
@@ -6003,19 +6117,19 @@
       <c r="S47" s="28" t="n"/>
       <c r="T47" s="28" t="n"/>
       <c r="U47" s="28" t="n"/>
-      <c r="Y47" t="n">
-        <v>0</v>
+      <c r="Z47" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>piter</t>
+          <t>Diego229</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C48" s="13">
@@ -6033,19 +6147,19 @@
       <c r="S48" s="28" t="n"/>
       <c r="T48" s="28" t="n"/>
       <c r="U48" s="28" t="n"/>
-      <c r="Y48" t="n">
+      <c r="Z48" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>andrea</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C49" s="13">
@@ -6063,64 +6177,11 @@
       <c r="S49" s="28" t="n"/>
       <c r="T49" s="28" t="n"/>
       <c r="U49" s="28" t="n"/>
-      <c r="Y49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="29">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>Ema alba003</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>20/04/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="13">
-        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="10" t="n"/>
-      <c r="L50" s="10" t="n"/>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="10" t="n"/>
-      <c r="O50" s="28" t="n"/>
-      <c r="P50" s="28" t="n"/>
-      <c r="Q50" s="28" t="n"/>
-      <c r="R50" s="28" t="n"/>
-      <c r="S50" s="28" t="n"/>
-      <c r="T50" s="28" t="n"/>
-      <c r="U50" s="28" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>satana03</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>20/04/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="O51" s="28" t="n"/>
-      <c r="P51" s="28" t="n"/>
-      <c r="Q51" s="28" t="n"/>
-      <c r="R51" s="28" t="n"/>
-      <c r="S51" s="28" t="n"/>
-      <c r="T51" s="28" t="n"/>
-      <c r="U51" s="28" t="n"/>
-    </row>
+      <c r="Z49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="29"/>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-26
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3855,7 +3855,7 @@
         <v>6</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -3931,7 +3931,7 @@
         <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -4820,7 +4820,7 @@
         <v>2</v>
       </c>
       <c r="Z23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -5219,7 +5219,7 @@
         <v>6</v>
       </c>
       <c r="Z29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -5679,7 +5679,7 @@
         <v>0</v>
       </c>
       <c r="Z35" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -5785,7 +5785,7 @@
         <v>0</v>
       </c>
       <c r="Z37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
Update Clan Games data - 2026-04-26
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA49"/>
+  <dimension ref="A1:AA46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="21" min="1" max="1"/>
@@ -2928,7 +2928,7 @@
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>Steninja:)</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
@@ -2945,7 +2945,7 @@
         <v/>
       </c>
       <c r="E45" s="20" t="n">
-        <v>700</v>
+        <v>40640</v>
       </c>
       <c r="F45" s="26" t="n"/>
       <c r="G45" s="26" t="n"/>
@@ -2969,7 +2969,7 @@
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
       <c r="E46" s="20" t="n">
-        <v>40640</v>
+        <v>12375</v>
       </c>
       <c r="F46" s="26" t="n"/>
       <c r="G46" s="26" t="n"/>
@@ -3006,129 +3006,6 @@
       <c r="U46" s="26" t="n"/>
       <c r="V46" s="26" t="n"/>
       <c r="W46" s="26" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>satana03</t>
-        </is>
-      </c>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="16">
-        <f>ROUND(AVERAGE(F47:AB47), 0)</f>
-        <v/>
-      </c>
-      <c r="D47" s="1">
-        <f>SUM(F47:AB47)</f>
-        <v/>
-      </c>
-      <c r="E47" s="20" t="n">
-        <v>800</v>
-      </c>
-      <c r="F47" s="26" t="n"/>
-      <c r="G47" s="26" t="n"/>
-      <c r="H47" s="26" t="n"/>
-      <c r="I47" s="26" t="n"/>
-      <c r="J47" s="26" t="n"/>
-      <c r="K47" s="26" t="n"/>
-      <c r="L47" s="26" t="n"/>
-      <c r="M47" s="26" t="n"/>
-      <c r="N47" s="26" t="n"/>
-      <c r="O47" s="26" t="n"/>
-      <c r="P47" s="26" t="n"/>
-      <c r="Q47" s="26" t="n"/>
-      <c r="R47" s="26" t="n"/>
-      <c r="S47" s="26" t="n"/>
-      <c r="T47" s="26" t="n"/>
-      <c r="U47" s="26" t="n"/>
-      <c r="V47" s="26" t="n"/>
-      <c r="W47" s="26" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="20" t="inlineStr">
-        <is>
-          <t>Diego229</t>
-        </is>
-      </c>
-      <c r="B48" s="22" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="16">
-        <f>ROUND(AVERAGE(F48:AB48), 0)</f>
-        <v/>
-      </c>
-      <c r="D48" s="1">
-        <f>SUM(F48:AB48)</f>
-        <v/>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>5775</v>
-      </c>
-      <c r="F48" s="26" t="n"/>
-      <c r="G48" s="26" t="n"/>
-      <c r="H48" s="26" t="n"/>
-      <c r="I48" s="26" t="n"/>
-      <c r="J48" s="26" t="n"/>
-      <c r="K48" s="26" t="n"/>
-      <c r="L48" s="26" t="n"/>
-      <c r="M48" s="26" t="n"/>
-      <c r="N48" s="26" t="n"/>
-      <c r="O48" s="26" t="n"/>
-      <c r="P48" s="26" t="n"/>
-      <c r="Q48" s="26" t="n"/>
-      <c r="R48" s="26" t="n"/>
-      <c r="S48" s="26" t="n"/>
-      <c r="T48" s="26" t="n"/>
-      <c r="U48" s="26" t="n"/>
-      <c r="V48" s="26" t="n"/>
-      <c r="W48" s="26" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>re deo</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="16">
-        <f>ROUND(AVERAGE(F49:AB49), 0)</f>
-        <v/>
-      </c>
-      <c r="D49" s="1">
-        <f>SUM(F49:AB49)</f>
-        <v/>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>12375</v>
-      </c>
-      <c r="F49" s="26" t="n"/>
-      <c r="G49" s="26" t="n"/>
-      <c r="H49" s="26" t="n"/>
-      <c r="I49" s="26" t="n"/>
-      <c r="J49" s="26" t="n"/>
-      <c r="K49" s="26" t="n"/>
-      <c r="L49" s="26" t="n"/>
-      <c r="M49" s="26" t="n"/>
-      <c r="N49" s="26" t="n"/>
-      <c r="O49" s="26" t="n"/>
-      <c r="P49" s="26" t="n"/>
-      <c r="Q49" s="26" t="n"/>
-      <c r="R49" s="26" t="n"/>
-      <c r="S49" s="26" t="n"/>
-      <c r="T49" s="26" t="n"/>
-      <c r="U49" s="26" t="n"/>
-      <c r="V49" s="26" t="n"/>
-      <c r="W49" s="26" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="29" thickBot="1"/>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-04-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3025,7 +3025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH49"/>
+  <dimension ref="A1:AH46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -5707,12 +5707,12 @@
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Steninja:)</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5730,12 +5730,6 @@
       <c r="S39" s="28" t="n"/>
       <c r="T39" s="28" t="n"/>
       <c r="U39" s="28" t="n"/>
-      <c r="W39" t="n">
-        <v>0</v>
-      </c>
-      <c r="X39" t="n">
-        <v>0</v>
-      </c>
       <c r="Y39" t="n">
         <v>0</v>
       </c>
@@ -5746,12 +5740,12 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5770,16 +5764,16 @@
       <c r="T40" s="28" t="n"/>
       <c r="U40" s="28" t="n"/>
       <c r="Y40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
@@ -5806,13 +5800,13 @@
         <v>6</v>
       </c>
       <c r="Z41" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
@@ -5836,16 +5830,16 @@
       <c r="T42" s="28" t="n"/>
       <c r="U42" s="28" t="n"/>
       <c r="Y42" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Z42" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
@@ -5869,7 +5863,7 @@
       <c r="T43" s="28" t="n"/>
       <c r="U43" s="28" t="n"/>
       <c r="Y43" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z43" t="n">
         <v>0</v>
@@ -5878,12 +5872,12 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -5901,9 +5895,6 @@
       <c r="S44" s="28" t="n"/>
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
-      <c r="Y44" t="n">
-        <v>0</v>
-      </c>
       <c r="Z44" t="n">
         <v>0</v>
       </c>
@@ -5911,12 +5902,12 @@
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -5935,18 +5926,18 @@
       <c r="T45" s="28" t="n"/>
       <c r="U45" s="28" t="n"/>
       <c r="Z45" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>satana03</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -5965,96 +5956,6 @@
       <c r="T46" s="28" t="n"/>
       <c r="U46" s="28" t="n"/>
       <c r="Z46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>re deo</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="inlineStr">
-        <is>
-          <t>25/04/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="13">
-        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
-        <v/>
-      </c>
-      <c r="K47" s="10" t="n"/>
-      <c r="L47" s="10" t="n"/>
-      <c r="M47" s="9" t="n"/>
-      <c r="N47" s="10" t="n"/>
-      <c r="O47" s="28" t="n"/>
-      <c r="P47" s="28" t="n"/>
-      <c r="Q47" s="28" t="n"/>
-      <c r="R47" s="28" t="n"/>
-      <c r="S47" s="28" t="n"/>
-      <c r="T47" s="28" t="n"/>
-      <c r="U47" s="28" t="n"/>
-      <c r="Z47" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>Diego229</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="inlineStr">
-        <is>
-          <t>25/04/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="13">
-        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
-        <v/>
-      </c>
-      <c r="K48" s="10" t="n"/>
-      <c r="L48" s="10" t="n"/>
-      <c r="M48" s="9" t="n"/>
-      <c r="N48" s="10" t="n"/>
-      <c r="O48" s="28" t="n"/>
-      <c r="P48" s="28" t="n"/>
-      <c r="Q48" s="28" t="n"/>
-      <c r="R48" s="28" t="n"/>
-      <c r="S48" s="28" t="n"/>
-      <c r="T48" s="28" t="n"/>
-      <c r="U48" s="28" t="n"/>
-      <c r="Z48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>ajaz064</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="inlineStr">
-        <is>
-          <t>25/04/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="13">
-        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
-        <v/>
-      </c>
-      <c r="K49" s="10" t="n"/>
-      <c r="L49" s="10" t="n"/>
-      <c r="M49" s="9" t="n"/>
-      <c r="N49" s="10" t="n"/>
-      <c r="O49" s="28" t="n"/>
-      <c r="P49" s="28" t="n"/>
-      <c r="Q49" s="28" t="n"/>
-      <c r="R49" s="28" t="n"/>
-      <c r="S49" s="28" t="n"/>
-      <c r="T49" s="28" t="n"/>
-      <c r="U49" s="28" t="n"/>
-      <c r="Z49" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-04-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA46"/>
+  <dimension ref="A1:AA45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="21" min="1" max="1"/>
@@ -2682,7 +2682,7 @@
     <row r="39">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B39" s="22" t="inlineStr">
@@ -2699,7 +2699,7 @@
         <v/>
       </c>
       <c r="E39" s="20" t="n">
-        <v>21200</v>
+        <v>13125</v>
       </c>
       <c r="F39" s="26" t="n"/>
       <c r="G39" s="26" t="n"/>
@@ -2723,7 +2723,7 @@
     <row r="40">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
@@ -2740,7 +2740,7 @@
         <v/>
       </c>
       <c r="E40" s="20" t="n">
-        <v>13125</v>
+        <v>250</v>
       </c>
       <c r="F40" s="26" t="n"/>
       <c r="G40" s="26" t="n"/>
@@ -2764,7 +2764,7 @@
     <row r="41">
       <c r="A41" s="20" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
@@ -2781,7 +2781,7 @@
         <v/>
       </c>
       <c r="E41" s="20" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="F41" s="26" t="n"/>
       <c r="G41" s="26" t="n"/>
@@ -2805,7 +2805,7 @@
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
@@ -2822,7 +2822,7 @@
         <v/>
       </c>
       <c r="E42" s="20" t="n">
-        <v>0</v>
+        <v>36750</v>
       </c>
       <c r="F42" s="26" t="n"/>
       <c r="G42" s="26" t="n"/>
@@ -2846,7 +2846,7 @@
     <row r="43">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
@@ -2863,7 +2863,7 @@
         <v/>
       </c>
       <c r="E43" s="20" t="n">
-        <v>36750</v>
+        <v>11250</v>
       </c>
       <c r="F43" s="26" t="n"/>
       <c r="G43" s="26" t="n"/>
@@ -2887,7 +2887,7 @@
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
@@ -2904,7 +2904,7 @@
         <v/>
       </c>
       <c r="E44" s="20" t="n">
-        <v>11250</v>
+        <v>40640</v>
       </c>
       <c r="F44" s="26" t="n"/>
       <c r="G44" s="26" t="n"/>
@@ -2928,7 +2928,7 @@
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
@@ -2945,7 +2945,7 @@
         <v/>
       </c>
       <c r="E45" s="20" t="n">
-        <v>40640</v>
+        <v>12375</v>
       </c>
       <c r="F45" s="26" t="n"/>
       <c r="G45" s="26" t="n"/>
@@ -2965,47 +2965,6 @@
       <c r="U45" s="26" t="n"/>
       <c r="V45" s="26" t="n"/>
       <c r="W45" s="26" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t>re deo</t>
-        </is>
-      </c>
-      <c r="B46" s="22" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="16">
-        <f>ROUND(AVERAGE(F46:AB46), 0)</f>
-        <v/>
-      </c>
-      <c r="D46" s="1">
-        <f>SUM(F46:AB46)</f>
-        <v/>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>12375</v>
-      </c>
-      <c r="F46" s="26" t="n"/>
-      <c r="G46" s="26" t="n"/>
-      <c r="H46" s="26" t="n"/>
-      <c r="I46" s="26" t="n"/>
-      <c r="J46" s="26" t="n"/>
-      <c r="K46" s="26" t="n"/>
-      <c r="L46" s="26" t="n"/>
-      <c r="M46" s="26" t="n"/>
-      <c r="N46" s="26" t="n"/>
-      <c r="O46" s="26" t="n"/>
-      <c r="P46" s="26" t="n"/>
-      <c r="Q46" s="26" t="n"/>
-      <c r="R46" s="26" t="n"/>
-      <c r="S46" s="26" t="n"/>
-      <c r="T46" s="26" t="n"/>
-      <c r="U46" s="26" t="n"/>
-      <c r="V46" s="26" t="n"/>
-      <c r="W46" s="26" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="29" thickBot="1"/>
   </sheetData>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-04-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2805,7 +2805,7 @@
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
@@ -2822,7 +2822,7 @@
         <v/>
       </c>
       <c r="E42" s="20" t="n">
-        <v>36750</v>
+        <v>11250</v>
       </c>
       <c r="F42" s="26" t="n"/>
       <c r="G42" s="26" t="n"/>
@@ -2846,7 +2846,7 @@
     <row r="43">
       <c r="A43" s="20" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
@@ -2863,7 +2863,7 @@
         <v/>
       </c>
       <c r="E43" s="20" t="n">
-        <v>11250</v>
+        <v>40640</v>
       </c>
       <c r="F43" s="26" t="n"/>
       <c r="G43" s="26" t="n"/>
@@ -2887,7 +2887,7 @@
     <row r="44">
       <c r="A44" s="20" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
@@ -2904,7 +2904,7 @@
         <v/>
       </c>
       <c r="E44" s="20" t="n">
-        <v>40640</v>
+        <v>12375</v>
       </c>
       <c r="F44" s="26" t="n"/>
       <c r="G44" s="26" t="n"/>
@@ -2928,12 +2928,12 @@
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
         <is>
-          <t>re deo</t>
+          <t>Dade_Aca_03</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C45" s="16">
@@ -2945,7 +2945,7 @@
         <v/>
       </c>
       <c r="E45" s="20" t="n">
-        <v>12375</v>
+        <v>26325</v>
       </c>
       <c r="F45" s="26" t="n"/>
       <c r="G45" s="26" t="n"/>
@@ -2969,7 +2969,7 @@
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Dade_Aca_03</t>
+          <t>-_HORROR_-</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
       <c r="E46" s="20" t="n">
-        <v>26325</v>
+        <v>0</v>
       </c>
       <c r="F46" s="26" t="n"/>
       <c r="G46" s="26" t="n"/>
@@ -3010,7 +3010,7 @@
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>-_HORROR_-</t>
+          <t>-WOLF-</t>
         </is>
       </c>
       <c r="B47" s="22" t="inlineStr">
@@ -3027,7 +3027,7 @@
         <v/>
       </c>
       <c r="E47" s="20" t="n">
-        <v>0</v>
+        <v>17500</v>
       </c>
       <c r="F47" s="26" t="n"/>
       <c r="G47" s="26" t="n"/>
@@ -3051,7 +3051,7 @@
     <row r="48">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>-WOLF-</t>
+          <t>AnT0x</t>
         </is>
       </c>
       <c r="B48" s="22" t="inlineStr">
@@ -3068,7 +3068,7 @@
         <v/>
       </c>
       <c r="E48" s="20" t="n">
-        <v>17500</v>
+        <v>30095</v>
       </c>
       <c r="F48" s="26" t="n"/>
       <c r="G48" s="26" t="n"/>
@@ -3092,7 +3092,7 @@
     <row r="49">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>AnT0x</t>
+          <t>Tropical</t>
         </is>
       </c>
       <c r="B49" s="22" t="inlineStr">
@@ -3109,7 +3109,7 @@
         <v/>
       </c>
       <c r="E49" s="20" t="n">
-        <v>30095</v>
+        <v>8350</v>
       </c>
       <c r="F49" s="26" t="n"/>
       <c r="G49" s="26" t="n"/>
@@ -3133,12 +3133,12 @@
     <row r="50">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>Tropical</t>
+          <t>ldl</t>
         </is>
       </c>
       <c r="B50" s="22" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C50" s="16">
@@ -3150,7 +3150,7 @@
         <v/>
       </c>
       <c r="E50" s="20" t="n">
-        <v>8350</v>
+        <v>100</v>
       </c>
       <c r="F50" s="26" t="n"/>
       <c r="G50" s="26" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-02
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3189,7 +3189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH46"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="AA1" s="7" t="inlineStr">
         <is>
-          <t>Colonna25</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="AB1" s="7" t="inlineStr">
@@ -3440,6 +3440,9 @@
       <c r="Z2" t="n">
         <v>0</v>
       </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -3499,6 +3502,9 @@
         <v>0</v>
       </c>
       <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3552,6 +3558,9 @@
         <v>6</v>
       </c>
       <c r="Z4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3597,6 +3606,9 @@
       <c r="Z5" t="n">
         <v>0</v>
       </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -3673,6 +3685,9 @@
       <c r="Z6" t="n">
         <v>0</v>
       </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -3758,6 +3773,9 @@
       <c r="Z7" t="n">
         <v>0</v>
       </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -3841,6 +3859,9 @@
         <v>6</v>
       </c>
       <c r="Z8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA8" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3898,6 +3919,9 @@
       <c r="Z9" t="n">
         <v>6</v>
       </c>
+      <c r="AA9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -3973,6 +3997,9 @@
       </c>
       <c r="Z10" t="n">
         <v>2</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4017,6 +4044,9 @@
       <c r="Z11" t="n">
         <v>0</v>
       </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -4091,6 +4121,9 @@
         <v>0</v>
       </c>
       <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4134,6 +4167,9 @@
       <c r="Z13" t="n">
         <v>0</v>
       </c>
+      <c r="AA13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -4217,6 +4253,9 @@
         <v>6</v>
       </c>
       <c r="Z14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA14" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4268,6 +4307,9 @@
       <c r="Z15" t="n">
         <v>0</v>
       </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -4353,6 +4395,9 @@
       <c r="Z16" t="n">
         <v>0</v>
       </c>
+      <c r="AA16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -4426,6 +4471,9 @@
       <c r="Z17" t="n">
         <v>6</v>
       </c>
+      <c r="AA17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -4511,111 +4559,120 @@
       <c r="Z18" t="n">
         <v>0</v>
       </c>
+      <c r="AA18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C19" s="13">
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
-      <c r="D19" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="n"/>
       <c r="M19" s="9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N19" s="26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q19" t="n">
         <v>6</v>
       </c>
       <c r="R19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T19" t="n">
         <v>6</v>
       </c>
       <c r="U19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C20" s="13">
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="K20" s="10" t="n"/>
-      <c r="L20" s="10" t="n"/>
+      <c r="D20" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L20" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="M20" s="9" t="n">
         <v>6</v>
       </c>
       <c r="N20" s="26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O20" t="n">
         <v>6</v>
@@ -4636,7 +4693,7 @@
         <v>6</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V20" t="n">
         <v>6</v>
@@ -4648,71 +4705,38 @@
         <v>6</v>
       </c>
       <c r="Y20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z20" t="n">
         <v>0</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C21" s="13">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="D21" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K21" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L21" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M21" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N21" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="O21" t="n">
-        <v>6</v>
-      </c>
-      <c r="P21" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>6</v>
-      </c>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="10" t="n"/>
+      <c r="N21" s="10" t="n"/>
+      <c r="O21" s="27" t="n"/>
+      <c r="P21" s="27" t="n"/>
+      <c r="Q21" s="27" t="n"/>
       <c r="R21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S21" t="n">
         <v>6</v>
@@ -4730,38 +4754,68 @@
         <v>6</v>
       </c>
       <c r="X21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z21" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C22" s="13">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
-      <c r="K22" s="10" t="n"/>
-      <c r="L22" s="10" t="n"/>
-      <c r="N22" s="10" t="n"/>
-      <c r="O22" s="27" t="n"/>
-      <c r="P22" s="27" t="n"/>
-      <c r="Q22" s="27" t="n"/>
+      <c r="G22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K22" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N22" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O22" t="n">
+        <v>6</v>
+      </c>
+      <c r="P22" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>6</v>
+      </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S22" t="n">
         <v>6</v>
@@ -4776,22 +4830,25 @@
         <v>6</v>
       </c>
       <c r="W22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y22" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z22" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -4803,11 +4860,20 @@
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
+      <c r="D23" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>6</v>
+      </c>
       <c r="G23" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>6</v>
@@ -4816,16 +4882,16 @@
         <v>6</v>
       </c>
       <c r="K23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M23" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O23" t="n">
         <v>6</v>
@@ -4846,79 +4912,52 @@
         <v>6</v>
       </c>
       <c r="U23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X23" t="n">
         <v>6</v>
       </c>
       <c r="Y23" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z23" t="n">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C24" s="13">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
-      <c r="D24" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="9" t="n">
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="10" t="n"/>
+      <c r="N24" s="10" t="n"/>
+      <c r="O24" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="I24" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>6</v>
-      </c>
-      <c r="P24" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q24" t="n">
+      <c r="P24" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q24" s="28" t="n">
         <v>6</v>
       </c>
       <c r="R24" t="n">
@@ -4931,56 +4970,89 @@
         <v>6</v>
       </c>
       <c r="U24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Y24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z24" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C25" s="13">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
-      <c r="K25" s="10" t="n"/>
-      <c r="L25" s="10" t="n"/>
-      <c r="N25" s="10" t="n"/>
-      <c r="P25" s="27" t="n"/>
-      <c r="Q25" s="27" t="n"/>
-      <c r="R25" s="27" t="n"/>
+      <c r="G25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O25" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P25" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q25" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>6</v>
+      </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W25" t="n">
         <v>0</v>
@@ -4992,29 +5064,53 @@
         <v>0</v>
       </c>
       <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C26" s="13">
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
-      <c r="K26" s="10" t="n"/>
-      <c r="L26" s="10" t="n"/>
-      <c r="N26" s="10" t="n"/>
+      <c r="G26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J26" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K26" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L26" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N26" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="O26" s="28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P26" s="28" t="n">
         <v>6</v>
@@ -5035,51 +5131,39 @@
         <v>6</v>
       </c>
       <c r="V26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W26" t="n">
         <v>0</v>
       </c>
       <c r="X26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y26" t="n">
         <v>0</v>
       </c>
       <c r="Z26" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C27" s="13">
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
-      <c r="G27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J27" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K27" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="L27" s="10" t="n">
         <v>6</v>
       </c>
@@ -5098,7 +5182,7 @@
       <c r="Q27" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R27" t="n">
+      <c r="R27" s="28" t="n">
         <v>6</v>
       </c>
       <c r="S27" t="n">
@@ -5120,39 +5204,30 @@
         <v>0</v>
       </c>
       <c r="Y27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C28" s="13">
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
-      <c r="G28" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J28" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="K28" s="10" t="n">
         <v>6</v>
       </c>
@@ -5174,7 +5249,7 @@
       <c r="Q28" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R28" t="n">
+      <c r="R28" s="28" t="n">
         <v>6</v>
       </c>
       <c r="S28" t="n">
@@ -5190,33 +5265,60 @@
         <v>6</v>
       </c>
       <c r="W28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z28" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C29" s="13">
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
+      <c r="D29" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K29" s="10" t="n">
+        <v>6</v>
+      </c>
       <c r="L29" s="10" t="n">
         <v>6</v>
       </c>
@@ -5242,42 +5344,66 @@
         <v>6</v>
       </c>
       <c r="T29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V29" t="n">
         <v>6</v>
       </c>
       <c r="W29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C30" s="13">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
+      <c r="D30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>5</v>
+      </c>
       <c r="K30" s="10" t="n">
         <v>6</v>
       </c>
@@ -5302,7 +5428,7 @@
       <c r="R30" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S30" t="n">
+      <c r="S30" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T30" t="n">
@@ -5312,25 +5438,28 @@
         <v>6</v>
       </c>
       <c r="V30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z30" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
@@ -5387,35 +5516,38 @@
       <c r="R31" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="S31" t="n">
+      <c r="S31" s="28" t="n">
         <v>6</v>
       </c>
       <c r="T31" t="n">
+        <v>6</v>
+      </c>
+      <c r="U31" t="n">
+        <v>6</v>
+      </c>
+      <c r="V31" t="n">
+        <v>6</v>
+      </c>
+      <c r="W31" t="n">
+        <v>6</v>
+      </c>
+      <c r="X31" t="n">
         <v>4</v>
       </c>
-      <c r="U31" t="n">
-        <v>0</v>
-      </c>
-      <c r="V31" t="n">
-        <v>6</v>
-      </c>
-      <c r="W31" t="n">
+      <c r="Y31" t="n">
         <v>3</v>
       </c>
-      <c r="X31" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>0</v>
-      </c>
       <c r="Z31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
@@ -5427,80 +5559,63 @@
         <f>ROUND(AVERAGE(D32:AH32), 0)</f>
         <v/>
       </c>
-      <c r="D32" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J32" s="10" t="n">
+      <c r="J32" s="10" t="n"/>
+      <c r="K32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="O32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="P32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="S32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="T32" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="U32" t="n">
+        <v>6</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="n">
         <v>5</v>
       </c>
-      <c r="K32" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L32" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M32" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N32" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S32" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T32" t="n">
-        <v>6</v>
-      </c>
-      <c r="U32" t="n">
-        <v>6</v>
-      </c>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" t="n">
-        <v>0</v>
-      </c>
       <c r="X32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z32" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
@@ -5512,15 +5627,6 @@
         <f>ROUND(AVERAGE(D33:AH33), 0)</f>
         <v/>
       </c>
-      <c r="D33" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E33" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F33" s="9" t="n">
-        <v>6</v>
-      </c>
       <c r="G33" s="9" t="n">
         <v>6</v>
       </c>
@@ -5549,7 +5655,7 @@
         <v>6</v>
       </c>
       <c r="P33" s="28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q33" s="28" t="n">
         <v>6</v>
@@ -5560,44 +5666,46 @@
       <c r="S33" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="T33" t="n">
-        <v>6</v>
-      </c>
-      <c r="U33" t="n">
+      <c r="T33" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="U33" s="28" t="n">
         <v>6</v>
       </c>
       <c r="V33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W33" t="n">
         <v>6</v>
       </c>
       <c r="X33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z33" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C34" s="13">
         <f>ROUND(AVERAGE(D34:AH34), 0)</f>
         <v/>
       </c>
-      <c r="J34" s="10" t="n"/>
       <c r="K34" s="10" t="n">
         <v>6</v>
       </c>
@@ -5605,10 +5713,10 @@
         <v>6</v>
       </c>
       <c r="M34" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N34" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O34" s="28" t="n">
         <v>6</v>
@@ -5620,182 +5728,132 @@
         <v>6</v>
       </c>
       <c r="R34" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S34" s="28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T34" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U34" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U34" s="28" t="n">
+        <v>0</v>
       </c>
       <c r="V34" t="n">
         <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z34" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C35" s="13">
         <f>ROUND(AVERAGE(D35:AH35), 0)</f>
         <v/>
       </c>
-      <c r="G35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="K35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N35" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="O35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P35" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="S35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="T35" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U35" s="28" t="n">
-        <v>6</v>
-      </c>
+      <c r="K35" s="10" t="n"/>
+      <c r="L35" s="10" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="10" t="n"/>
+      <c r="O35" s="28" t="n"/>
+      <c r="P35" s="28" t="n"/>
+      <c r="Q35" s="28" t="n"/>
+      <c r="R35" s="28" t="n"/>
+      <c r="S35" s="28" t="n"/>
+      <c r="T35" s="28" t="n"/>
+      <c r="U35" s="28" t="n"/>
       <c r="V35" t="n">
         <v>0</v>
       </c>
       <c r="W35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X35" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y35" t="n">
         <v>0</v>
       </c>
       <c r="Z35" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C36" s="13">
         <f>ROUND(AVERAGE(D36:AH36), 0)</f>
         <v/>
       </c>
-      <c r="K36" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="L36" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="P36" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q36" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="R36" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T36" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="U36" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="V36" t="n">
-        <v>0</v>
-      </c>
+      <c r="K36" s="10" t="n"/>
+      <c r="L36" s="10" t="n"/>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="10" t="n"/>
+      <c r="O36" s="28" t="n"/>
+      <c r="P36" s="28" t="n"/>
+      <c r="Q36" s="28" t="n"/>
+      <c r="R36" s="28" t="n"/>
+      <c r="S36" s="28" t="n"/>
+      <c r="T36" s="28" t="n"/>
+      <c r="U36" s="28" t="n"/>
       <c r="W36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y36" t="n">
         <v>0</v>
       </c>
       <c r="Z36" t="n">
         <v>0</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
@@ -5813,31 +5871,25 @@
       <c r="S37" s="28" t="n"/>
       <c r="T37" s="28" t="n"/>
       <c r="U37" s="28" t="n"/>
-      <c r="V37" t="n">
-        <v>0</v>
-      </c>
-      <c r="W37" t="n">
-        <v>0</v>
-      </c>
-      <c r="X37" t="n">
-        <v>6</v>
-      </c>
       <c r="Y37" t="n">
         <v>0</v>
       </c>
       <c r="Z37" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C38" s="13">
@@ -5855,28 +5907,25 @@
       <c r="S38" s="28" t="n"/>
       <c r="T38" s="28" t="n"/>
       <c r="U38" s="28" t="n"/>
-      <c r="W38" t="n">
-        <v>6</v>
-      </c>
-      <c r="X38" t="n">
-        <v>6</v>
-      </c>
       <c r="Y38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z38" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5900,16 +5949,19 @@
       <c r="Z39" t="n">
         <v>0</v>
       </c>
+      <c r="AA39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5927,22 +5979,22 @@
       <c r="S40" s="28" t="n"/>
       <c r="T40" s="28" t="n"/>
       <c r="U40" s="28" t="n"/>
-      <c r="Y40" t="n">
-        <v>6</v>
-      </c>
       <c r="Z40" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C41" s="13">
@@ -5960,22 +6012,22 @@
       <c r="S41" s="28" t="n"/>
       <c r="T41" s="28" t="n"/>
       <c r="U41" s="28" t="n"/>
-      <c r="Y41" t="n">
-        <v>6</v>
-      </c>
       <c r="Z41" t="n">
         <v>6</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -5993,22 +6045,22 @@
       <c r="S42" s="28" t="n"/>
       <c r="T42" s="28" t="n"/>
       <c r="U42" s="28" t="n"/>
-      <c r="Y42" t="n">
-        <v>4</v>
-      </c>
       <c r="Z42" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA42" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C43" s="13">
@@ -6026,22 +6078,19 @@
       <c r="S43" s="28" t="n"/>
       <c r="T43" s="28" t="n"/>
       <c r="U43" s="28" t="n"/>
-      <c r="Y43" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z43" t="n">
+      <c r="AA43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C44" s="13">
@@ -6059,19 +6108,19 @@
       <c r="S44" s="28" t="n"/>
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
-      <c r="Z44" t="n">
+      <c r="AA44" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>re deo</t>
+          <t>AnT0x</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C45" s="13">
@@ -6089,19 +6138,19 @@
       <c r="S45" s="28" t="n"/>
       <c r="T45" s="28" t="n"/>
       <c r="U45" s="28" t="n"/>
-      <c r="Z45" t="n">
-        <v>6</v>
+      <c r="AA45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Dade_Aca_03</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C46" s="13">
@@ -6119,11 +6168,160 @@
       <c r="S46" s="28" t="n"/>
       <c r="T46" s="28" t="n"/>
       <c r="U46" s="28" t="n"/>
-      <c r="Z46" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="29"/>
+      <c r="AA46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>⁰LÜKÄ⁰</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="13">
+        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
+        <v/>
+      </c>
+      <c r="K47" s="10" t="n"/>
+      <c r="L47" s="10" t="n"/>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="10" t="n"/>
+      <c r="O47" s="28" t="n"/>
+      <c r="P47" s="28" t="n"/>
+      <c r="Q47" s="28" t="n"/>
+      <c r="R47" s="28" t="n"/>
+      <c r="S47" s="28" t="n"/>
+      <c r="T47" s="28" t="n"/>
+      <c r="U47" s="28" t="n"/>
+      <c r="AA47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>El sushino</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="13">
+        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
+        <v/>
+      </c>
+      <c r="K48" s="10" t="n"/>
+      <c r="L48" s="10" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="10" t="n"/>
+      <c r="O48" s="28" t="n"/>
+      <c r="P48" s="28" t="n"/>
+      <c r="Q48" s="28" t="n"/>
+      <c r="R48" s="28" t="n"/>
+      <c r="S48" s="28" t="n"/>
+      <c r="T48" s="28" t="n"/>
+      <c r="U48" s="28" t="n"/>
+      <c r="AA48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>ldl</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="13">
+        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
+        <v/>
+      </c>
+      <c r="K49" s="10" t="n"/>
+      <c r="L49" s="10" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="10" t="n"/>
+      <c r="O49" s="28" t="n"/>
+      <c r="P49" s="28" t="n"/>
+      <c r="Q49" s="28" t="n"/>
+      <c r="R49" s="28" t="n"/>
+      <c r="S49" s="28" t="n"/>
+      <c r="T49" s="28" t="n"/>
+      <c r="U49" s="28" t="n"/>
+      <c r="AA49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="29">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>Tropical</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="13">
+        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="10" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="10" t="n"/>
+      <c r="O50" s="28" t="n"/>
+      <c r="P50" s="28" t="n"/>
+      <c r="Q50" s="28" t="n"/>
+      <c r="R50" s="28" t="n"/>
+      <c r="S50" s="28" t="n"/>
+      <c r="T50" s="28" t="n"/>
+      <c r="U50" s="28" t="n"/>
+      <c r="AA50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>-WOLF-</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="13">
+        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="10" t="n"/>
+      <c r="L51" s="10" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="10" t="n"/>
+      <c r="O51" s="28" t="n"/>
+      <c r="P51" s="28" t="n"/>
+      <c r="Q51" s="28" t="n"/>
+      <c r="R51" s="28" t="n"/>
+      <c r="S51" s="28" t="n"/>
+      <c r="T51" s="28" t="n"/>
+      <c r="U51" s="28" t="n"/>
+      <c r="AA51" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-03
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -4045,7 +4045,7 @@
         <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -4124,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="AA12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -5365,7 +5365,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -5609,7 +5609,7 @@
         <v>6</v>
       </c>
       <c r="AA32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -5914,7 +5914,7 @@
         <v>3</v>
       </c>
       <c r="AA38" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -6049,7 +6049,7 @@
         <v>6</v>
       </c>
       <c r="AA42" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -6109,7 +6109,7 @@
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
       <c r="AA44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-04
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3189,7 +3189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="13" min="1" max="1"/>
@@ -5848,12 +5848,12 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C37" s="13">
@@ -5872,19 +5872,19 @@
       <c r="T37" s="28" t="n"/>
       <c r="U37" s="28" t="n"/>
       <c r="Y37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
@@ -5908,24 +5908,24 @@
       <c r="T38" s="28" t="n"/>
       <c r="U38" s="28" t="n"/>
       <c r="Y38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z38" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C39" s="13">
@@ -5943,9 +5943,6 @@
       <c r="S39" s="28" t="n"/>
       <c r="T39" s="28" t="n"/>
       <c r="U39" s="28" t="n"/>
-      <c r="Y39" t="n">
-        <v>0</v>
-      </c>
       <c r="Z39" t="n">
         <v>0</v>
       </c>
@@ -5956,12 +5953,12 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C40" s="13">
@@ -5980,7 +5977,7 @@
       <c r="T40" s="28" t="n"/>
       <c r="U40" s="28" t="n"/>
       <c r="Z40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA40" t="n">
         <v>0</v>
@@ -5989,7 +5986,7 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>re deo</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
@@ -6016,18 +6013,18 @@
         <v>6</v>
       </c>
       <c r="AA41" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C42" s="13">
@@ -6045,17 +6042,14 @@
       <c r="S42" s="28" t="n"/>
       <c r="T42" s="28" t="n"/>
       <c r="U42" s="28" t="n"/>
-      <c r="Z42" t="n">
-        <v>6</v>
-      </c>
       <c r="AA42" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
@@ -6079,13 +6073,13 @@
       <c r="T43" s="28" t="n"/>
       <c r="U43" s="28" t="n"/>
       <c r="AA43" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>⁰LÜKÄ⁰</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
@@ -6109,13 +6103,13 @@
       <c r="T44" s="28" t="n"/>
       <c r="U44" s="28" t="n"/>
       <c r="AA44" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>AnT0x</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
@@ -6145,7 +6139,7 @@
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>Dade_Aca_03</t>
+          <t>-WOLF-</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
@@ -6172,156 +6166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>⁰LÜKÄ⁰</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="13">
-        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
-        <v/>
-      </c>
-      <c r="K47" s="10" t="n"/>
-      <c r="L47" s="10" t="n"/>
-      <c r="M47" s="9" t="n"/>
-      <c r="N47" s="10" t="n"/>
-      <c r="O47" s="28" t="n"/>
-      <c r="P47" s="28" t="n"/>
-      <c r="Q47" s="28" t="n"/>
-      <c r="R47" s="28" t="n"/>
-      <c r="S47" s="28" t="n"/>
-      <c r="T47" s="28" t="n"/>
-      <c r="U47" s="28" t="n"/>
-      <c r="AA47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>El sushino</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="13">
-        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
-        <v/>
-      </c>
-      <c r="K48" s="10" t="n"/>
-      <c r="L48" s="10" t="n"/>
-      <c r="M48" s="9" t="n"/>
-      <c r="N48" s="10" t="n"/>
-      <c r="O48" s="28" t="n"/>
-      <c r="P48" s="28" t="n"/>
-      <c r="Q48" s="28" t="n"/>
-      <c r="R48" s="28" t="n"/>
-      <c r="S48" s="28" t="n"/>
-      <c r="T48" s="28" t="n"/>
-      <c r="U48" s="28" t="n"/>
-      <c r="AA48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>ldl</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="13">
-        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
-        <v/>
-      </c>
-      <c r="K49" s="10" t="n"/>
-      <c r="L49" s="10" t="n"/>
-      <c r="M49" s="9" t="n"/>
-      <c r="N49" s="10" t="n"/>
-      <c r="O49" s="28" t="n"/>
-      <c r="P49" s="28" t="n"/>
-      <c r="Q49" s="28" t="n"/>
-      <c r="R49" s="28" t="n"/>
-      <c r="S49" s="28" t="n"/>
-      <c r="T49" s="28" t="n"/>
-      <c r="U49" s="28" t="n"/>
-      <c r="AA49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="29">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>Tropical</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="13">
-        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="10" t="n"/>
-      <c r="L50" s="10" t="n"/>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="10" t="n"/>
-      <c r="O50" s="28" t="n"/>
-      <c r="P50" s="28" t="n"/>
-      <c r="Q50" s="28" t="n"/>
-      <c r="R50" s="28" t="n"/>
-      <c r="S50" s="28" t="n"/>
-      <c r="T50" s="28" t="n"/>
-      <c r="U50" s="28" t="n"/>
-      <c r="AA50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>-WOLF-</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="13">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="9" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="O51" s="28" t="n"/>
-      <c r="P51" s="28" t="n"/>
-      <c r="Q51" s="28" t="n"/>
-      <c r="R51" s="28" t="n"/>
-      <c r="S51" s="28" t="n"/>
-      <c r="T51" s="28" t="n"/>
-      <c r="U51" s="28" t="n"/>
-      <c r="AA51" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="50" ht="15.75" customHeight="1" s="29"/>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-09
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN50"/>
+  <dimension ref="A1:AN44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -942,83 +942,91 @@
     <row r="2" ht="16.5" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>antony</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C2" s="12">
-        <f>ROUND(AVERAGE(F2:AA2), 0)</f>
+        <f>ROUND(AVERAGE(F2:AO2), 0)</f>
         <v/>
       </c>
       <c r="D2" s="1">
-        <f>SUM(F2:AA2)</f>
+        <f>SUM(F2:AO2)</f>
         <v/>
       </c>
       <c r="E2" s="14" t="n">
-        <v>22300</v>
+        <v>31350</v>
       </c>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
       <c r="H2" s="13" t="n"/>
       <c r="I2" s="13" t="n"/>
-      <c r="J2" s="13" t="n"/>
+      <c r="J2" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="K2" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="L2" s="13" t="n"/>
-      <c r="M2" s="13" t="n"/>
-      <c r="N2" s="13" t="n"/>
-      <c r="O2" s="13" t="n"/>
-      <c r="P2" s="13" t="n"/>
-      <c r="Q2" s="13" t="n"/>
-      <c r="R2" s="13" t="n"/>
-      <c r="S2" s="13" t="n"/>
-      <c r="T2" s="13" t="n"/>
-      <c r="U2" s="13" t="n"/>
-      <c r="V2" s="13" t="n"/>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C3" s="12">
-        <f>ROUND(AVERAGE(F3:AA3), 0)</f>
+        <f>ROUND(AVERAGE(F3:AO3), 0)</f>
         <v/>
       </c>
       <c r="D3" s="1">
-        <f>SUM(F3:AA3)</f>
+        <f>SUM(F3:AO3)</f>
         <v/>
       </c>
       <c r="E3" s="14" t="n">
-        <v>31350</v>
+        <v>22000</v>
       </c>
       <c r="F3" s="13" t="n"/>
-      <c r="G3" s="13" t="n"/>
-      <c r="H3" s="13" t="n"/>
-      <c r="I3" s="13" t="n"/>
+      <c r="G3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="13" t="n">
+        <v>6050</v>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>8300</v>
+      </c>
       <c r="J3" s="13" t="n">
-        <v>10000</v>
+        <v>5950</v>
       </c>
       <c r="K3" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="L3" s="13" t="n"/>
+      <c r="M3" s="13" t="n"/>
+      <c r="N3" s="13" t="n"/>
+      <c r="O3" s="13" t="n"/>
+      <c r="P3" s="13" t="n"/>
+      <c r="Q3" s="13" t="n"/>
+      <c r="R3" s="13" t="n"/>
+      <c r="S3" s="13" t="n"/>
+      <c r="T3" s="13" t="n"/>
+      <c r="U3" s="13" t="n"/>
+      <c r="V3" s="13" t="n"/>
     </row>
     <row r="4" ht="16.5" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
@@ -1027,28 +1035,30 @@
         </is>
       </c>
       <c r="C4" s="12">
-        <f>ROUND(AVERAGE(F4:AA4), 0)</f>
+        <f>ROUND(AVERAGE(F4:AO4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="1">
-        <f>SUM(F4:AA4)</f>
+        <f>SUM(F4:AO4)</f>
         <v/>
       </c>
       <c r="E4" s="14" t="n">
-        <v>22000</v>
-      </c>
-      <c r="F4" s="13" t="n"/>
+        <v>47650</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G4" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H4" s="13" t="n">
-        <v>6050</v>
+        <v>10000</v>
       </c>
       <c r="I4" s="13" t="n">
-        <v>8300</v>
+        <v>10000</v>
       </c>
       <c r="J4" s="13" t="n">
-        <v>5950</v>
+        <v>10000</v>
       </c>
       <c r="K4" s="13" t="n">
         <v>10000</v>
@@ -1068,7 +1078,7 @@
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
@@ -1077,19 +1087,17 @@
         </is>
       </c>
       <c r="C5" s="12">
-        <f>ROUND(AVERAGE(F5:AA5), 0)</f>
+        <f>ROUND(AVERAGE(F5:AO5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="1">
-        <f>SUM(F5:AA5)</f>
+        <f>SUM(F5:AO5)</f>
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>47650</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>4000</v>
-      </c>
+        <v>55400</v>
+      </c>
+      <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n">
         <v>4000</v>
       </c>
@@ -1120,38 +1128,30 @@
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C6" s="12">
-        <f>ROUND(AVERAGE(F6:AA6), 0)</f>
+        <f>ROUND(AVERAGE(F6:AO6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="1">
-        <f>SUM(F6:AA6)</f>
+        <f>SUM(F6:AO6)</f>
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>55400</v>
+        <v>5500</v>
       </c>
       <c r="F6" s="13" t="n"/>
-      <c r="G6" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H6" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J6" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="G6" s="13" t="n"/>
+      <c r="H6" s="13" t="n"/>
+      <c r="I6" s="13" t="n"/>
+      <c r="J6" s="13" t="n"/>
       <c r="K6" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1170,30 +1170,36 @@
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C7" s="12">
-        <f>ROUND(AVERAGE(F7:AA7), 0)</f>
+        <f>ROUND(AVERAGE(F7:AO7), 0)</f>
         <v/>
       </c>
       <c r="D7" s="1">
-        <f>SUM(F7:AA7)</f>
+        <f>SUM(F7:AO7)</f>
         <v/>
       </c>
       <c r="E7" s="14" t="n">
-        <v>5500</v>
+        <v>58700</v>
       </c>
       <c r="F7" s="13" t="n"/>
       <c r="G7" s="13" t="n"/>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="K7" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1212,7 +1218,7 @@
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
@@ -1221,15 +1227,15 @@
         </is>
       </c>
       <c r="C8" s="12">
-        <f>ROUND(AVERAGE(F8:AA8), 0)</f>
+        <f>ROUND(AVERAGE(F8:AO8), 0)</f>
         <v/>
       </c>
       <c r="D8" s="1">
-        <f>SUM(F8:AA8)</f>
+        <f>SUM(F8:AO8)</f>
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>58700</v>
+        <v>51200</v>
       </c>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
@@ -1260,30 +1266,28 @@
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C9" s="12">
-        <f>ROUND(AVERAGE(F9:AA9), 0)</f>
+        <f>ROUND(AVERAGE(F9:AO9), 0)</f>
         <v/>
       </c>
       <c r="D9" s="1">
-        <f>SUM(F9:AA9)</f>
+        <f>SUM(F9:AO9)</f>
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>51200</v>
+        <v>106725</v>
       </c>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H9" s="13" t="n"/>
       <c r="I9" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1296,8 +1300,16 @@
       <c r="L9" s="13" t="n"/>
       <c r="M9" s="13" t="n"/>
       <c r="N9" s="13" t="n"/>
-      <c r="O9" s="13" t="n"/>
-      <c r="P9" s="13" t="n"/>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +</t>
+        </is>
+      </c>
       <c r="Q9" s="13" t="n"/>
       <c r="R9" s="13" t="n"/>
       <c r="S9" s="13" t="n"/>
@@ -1308,50 +1320,44 @@
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C10" s="12">
-        <f>ROUND(AVERAGE(F10:AA10), 0)</f>
+        <f>ROUND(AVERAGE(F10:AO10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="1">
-        <f>SUM(F10:AA10)</f>
+        <f>SUM(F10:AO10)</f>
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>106725</v>
+        <v>109220</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
+      <c r="H10" s="13" t="n">
+        <v>3850</v>
+      </c>
       <c r="I10" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>10000</v>
+        <v>8800</v>
       </c>
       <c r="L10" s="13" t="n"/>
       <c r="M10" s="13" t="n"/>
       <c r="N10" s="13" t="n"/>
-      <c r="O10" s="13" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="P10" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> +</t>
-        </is>
-      </c>
+      <c r="O10" s="13" t="n"/>
+      <c r="P10" s="13" t="n"/>
       <c r="Q10" s="13" t="n"/>
       <c r="R10" s="13" t="n"/>
       <c r="S10" s="13" t="n"/>
@@ -1362,7 +1368,7 @@
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -1371,29 +1377,29 @@
         </is>
       </c>
       <c r="C11" s="12">
-        <f>ROUND(AVERAGE(F11:AA11), 0)</f>
+        <f>ROUND(AVERAGE(F11:AO11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="1">
-        <f>SUM(F11:AA11)</f>
+        <f>SUM(F11:AO11)</f>
         <v/>
       </c>
       <c r="E11" s="14" t="n">
-        <v>109220</v>
+        <v>56300</v>
       </c>
       <c r="F11" s="13" t="n"/>
       <c r="G11" s="13" t="n"/>
       <c r="H11" s="13" t="n">
-        <v>3850</v>
+        <v>10000</v>
       </c>
       <c r="I11" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>8800</v>
+        <v>8600</v>
       </c>
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="13" t="n"/>
@@ -1410,7 +1416,7 @@
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
@@ -1419,29 +1425,31 @@
         </is>
       </c>
       <c r="C12" s="12">
-        <f>ROUND(AVERAGE(F12:AA12), 0)</f>
+        <f>ROUND(AVERAGE(F12:AO12), 0)</f>
         <v/>
       </c>
       <c r="D12" s="1">
-        <f>SUM(F12:AA12)</f>
+        <f>SUM(F12:AO12)</f>
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>56300</v>
+        <v>27500</v>
       </c>
       <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
+      <c r="G12" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H12" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>10000</v>
+        <v>4300</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>8600</v>
+        <v>6300</v>
       </c>
       <c r="L12" s="13" t="n"/>
       <c r="M12" s="13" t="n"/>
@@ -1450,7 +1458,7 @@
       <c r="P12" s="13" t="n"/>
       <c r="Q12" s="13" t="n"/>
       <c r="R12" s="13" t="n"/>
-      <c r="S12" s="13" t="n"/>
+      <c r="S12" s="21" t="n"/>
       <c r="T12" s="13" t="n"/>
       <c r="U12" s="13" t="n"/>
       <c r="V12" s="13" t="n"/>
@@ -1458,32 +1466,34 @@
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C13" s="12">
-        <f>ROUND(AVERAGE(F13:AA13), 0)</f>
+        <f>ROUND(AVERAGE(F13:AO13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="1">
-        <f>SUM(F13:AA13)</f>
+        <f>SUM(F13:AO13)</f>
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>26050</v>
+        <v>76700</v>
       </c>
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n"/>
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="13" t="n"/>
-      <c r="J13" s="13" t="n"/>
+      <c r="J13" s="13" t="n">
+        <v>5000</v>
+      </c>
       <c r="K13" s="13" t="n">
-        <v>8200</v>
+        <v>6100</v>
       </c>
       <c r="L13" s="13" t="n"/>
       <c r="M13" s="13" t="n"/>
@@ -1494,31 +1504,13 @@
       <c r="R13" s="13" t="n"/>
       <c r="S13" s="21" t="n"/>
       <c r="T13" s="13" t="n"/>
-      <c r="U13" s="21" t="n"/>
-      <c r="V13" s="21" t="n"/>
-      <c r="W13" s="22" t="n"/>
-      <c r="X13" s="22" t="n"/>
-      <c r="Y13" s="22" t="n"/>
-      <c r="Z13" s="22" t="n"/>
-      <c r="AA13" s="22" t="n"/>
-      <c r="AB13" s="22" t="n"/>
-      <c r="AC13" s="22" t="n"/>
-      <c r="AD13" s="22" t="n"/>
-      <c r="AE13" s="22" t="n"/>
-      <c r="AF13" s="22" t="n"/>
-      <c r="AG13" s="22" t="n"/>
-      <c r="AH13" s="22" t="n"/>
-      <c r="AI13" s="22" t="n"/>
-      <c r="AJ13" s="22" t="n"/>
-      <c r="AK13" s="22" t="n"/>
-      <c r="AL13" s="22" t="n"/>
-      <c r="AM13" s="22" t="n"/>
-      <c r="AN13" s="22" t="n"/>
+      <c r="U13" s="13" t="n"/>
+      <c r="V13" s="13" t="n"/>
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
@@ -1527,31 +1519,31 @@
         </is>
       </c>
       <c r="C14" s="12">
-        <f>ROUND(AVERAGE(F14:AA14), 0)</f>
+        <f>ROUND(AVERAGE(F14:AO14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="1">
-        <f>SUM(F14:AA14)</f>
+        <f>SUM(F14:AO14)</f>
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>27500</v>
+        <v>12250</v>
       </c>
       <c r="F14" s="13" t="n"/>
       <c r="G14" s="13" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>4300</v>
+        <v>0</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>6300</v>
+        <v>6100</v>
       </c>
       <c r="L14" s="13" t="n"/>
       <c r="M14" s="13" t="n"/>
@@ -1568,34 +1560,36 @@
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C15" s="12">
-        <f>ROUND(AVERAGE(F15:AA15), 0)</f>
+        <f>ROUND(AVERAGE(F15:AO15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="1">
-        <f>SUM(F15:AA15)</f>
+        <f>SUM(F15:AO15)</f>
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>76700</v>
+        <v>28225</v>
       </c>
       <c r="F15" s="13" t="n"/>
       <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n"/>
-      <c r="I15" s="13" t="n"/>
+      <c r="I15" s="13" t="n">
+        <v>2000</v>
+      </c>
       <c r="J15" s="13" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="K15" s="13" t="n">
-        <v>6100</v>
+        <v>5100</v>
       </c>
       <c r="L15" s="13" t="n"/>
       <c r="M15" s="13" t="n"/>
@@ -1612,7 +1606,7 @@
     <row r="16" ht="16.5" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
@@ -1621,31 +1615,33 @@
         </is>
       </c>
       <c r="C16" s="12">
-        <f>ROUND(AVERAGE(F16:AA16), 0)</f>
+        <f>ROUND(AVERAGE(F16:AO16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="1">
-        <f>SUM(F16:AA16)</f>
+        <f>SUM(F16:AO16)</f>
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>12250</v>
-      </c>
-      <c r="F16" s="13" t="n"/>
+        <v>33025</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G16" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0</v>
+        <v>4850</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="K16" s="13" t="n">
-        <v>6100</v>
+        <v>5050</v>
       </c>
       <c r="L16" s="13" t="n"/>
       <c r="M16" s="13" t="n"/>
@@ -1662,36 +1658,42 @@
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C17" s="12">
-        <f>ROUND(AVERAGE(F17:AA17), 0)</f>
+        <f>ROUND(AVERAGE(F17:AO17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="1">
-        <f>SUM(F17:AA17)</f>
+        <f>SUM(F17:AO17)</f>
         <v/>
       </c>
       <c r="E17" s="14" t="n">
-        <v>28225</v>
-      </c>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
+        <v>33700</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="I17" s="13" t="n">
-        <v>2000</v>
+        <v>2450</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>8000</v>
+        <v>4050</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>5100</v>
+        <v>4650</v>
       </c>
       <c r="L17" s="13" t="n"/>
       <c r="M17" s="13" t="n"/>
@@ -1708,7 +1710,7 @@
     <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
@@ -1717,33 +1719,33 @@
         </is>
       </c>
       <c r="C18" s="12">
-        <f>ROUND(AVERAGE(F18:AA18), 0)</f>
+        <f>ROUND(AVERAGE(F18:AO18), 0)</f>
         <v/>
       </c>
       <c r="D18" s="1">
-        <f>SUM(F18:AA18)</f>
+        <f>SUM(F18:AO18)</f>
         <v/>
       </c>
       <c r="E18" s="14" t="n">
-        <v>33025</v>
+        <v>33050</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>4000</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>4000</v>
+        <v>2100</v>
       </c>
       <c r="H18" s="13" t="n">
+        <v>5800</v>
+      </c>
+      <c r="I18" s="13" t="n">
         <v>4050</v>
       </c>
-      <c r="I18" s="13" t="n">
-        <v>4850</v>
-      </c>
       <c r="J18" s="13" t="n">
-        <v>4000</v>
+        <v>4350</v>
       </c>
       <c r="K18" s="13" t="n">
-        <v>5050</v>
+        <v>4600</v>
       </c>
       <c r="L18" s="13" t="n"/>
       <c r="M18" s="13" t="n"/>
@@ -1760,42 +1762,34 @@
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C19" s="12">
-        <f>ROUND(AVERAGE(F19:AA19), 0)</f>
+        <f>ROUND(AVERAGE(F19:AO19), 0)</f>
         <v/>
       </c>
       <c r="D19" s="1">
-        <f>SUM(F19:AA19)</f>
+        <f>SUM(F19:AO19)</f>
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>33700</v>
-      </c>
-      <c r="F19" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G19" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H19" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I19" s="13" t="n">
-        <v>2450</v>
-      </c>
+        <v>23750</v>
+      </c>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
       <c r="J19" s="13" t="n">
-        <v>4050</v>
+        <v>4300</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>4650</v>
+        <v>4200</v>
       </c>
       <c r="L19" s="13" t="n"/>
       <c r="M19" s="13" t="n"/>
@@ -1812,42 +1806,36 @@
     <row r="20" ht="16.5" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C20" s="12">
-        <f>ROUND(AVERAGE(F20:AA20), 0)</f>
+        <f>ROUND(AVERAGE(F20:AO20), 0)</f>
         <v/>
       </c>
       <c r="D20" s="1">
-        <f>SUM(F20:AA20)</f>
+        <f>SUM(F20:AO20)</f>
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>33050</v>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G20" s="13" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H20" s="13" t="n">
-        <v>5800</v>
-      </c>
+        <v>44550</v>
+      </c>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
       <c r="I20" s="13" t="n">
-        <v>4050</v>
+        <v>4300</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>4350</v>
+        <v>4100</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>4600</v>
+        <v>4200</v>
       </c>
       <c r="L20" s="13" t="n"/>
       <c r="M20" s="13" t="n"/>
@@ -1864,34 +1852,42 @@
     <row r="21" ht="16.5" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C21" s="12">
-        <f>ROUND(AVERAGE(F21:AA21), 0)</f>
+        <f>ROUND(AVERAGE(F21:AO21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="1">
-        <f>SUM(F21:AA21)</f>
+        <f>SUM(F21:AO21)</f>
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>23750</v>
-      </c>
-      <c r="F21" s="13" t="n"/>
-      <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="13" t="n"/>
+        <v>32200</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H21" s="13" t="n">
+        <v>4100</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>4400</v>
+      </c>
       <c r="J21" s="13" t="n">
-        <v>4300</v>
+        <v>4700</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>4200</v>
+        <v>4150</v>
       </c>
       <c r="L21" s="13" t="n"/>
       <c r="M21" s="13" t="n"/>
@@ -1908,36 +1904,38 @@
     <row r="22" ht="16.5" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C22" s="12">
-        <f>ROUND(AVERAGE(F22:AA22), 0)</f>
+        <f>ROUND(AVERAGE(F22:AO22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="1">
-        <f>SUM(F22:AA22)</f>
+        <f>SUM(F22:AO22)</f>
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>44550</v>
+        <v>123800</v>
       </c>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="n"/>
-      <c r="H22" s="13" t="n"/>
+      <c r="H22" s="13" t="n">
+        <v>4050</v>
+      </c>
       <c r="I22" s="13" t="n">
-        <v>4300</v>
+        <v>4100</v>
       </c>
       <c r="J22" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K22" s="13" t="n">
         <v>4100</v>
-      </c>
-      <c r="K22" s="13" t="n">
-        <v>4200</v>
       </c>
       <c r="L22" s="13" t="n"/>
       <c r="M22" s="13" t="n"/>
@@ -1954,7 +1952,7 @@
     <row r="23" ht="16.5" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
@@ -1963,33 +1961,29 @@
         </is>
       </c>
       <c r="C23" s="12">
-        <f>ROUND(AVERAGE(F23:AA23), 0)</f>
+        <f>ROUND(AVERAGE(F23:AO23), 0)</f>
         <v/>
       </c>
       <c r="D23" s="1">
-        <f>SUM(F23:AA23)</f>
+        <f>SUM(F23:AO23)</f>
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>32200</v>
-      </c>
-      <c r="F23" s="13" t="n">
+        <v>41000</v>
+      </c>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I23" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H23" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I23" s="13" t="n">
-        <v>4400</v>
-      </c>
       <c r="J23" s="13" t="n">
-        <v>4700</v>
+        <v>150</v>
       </c>
       <c r="K23" s="13" t="n">
-        <v>4150</v>
+        <v>4050</v>
       </c>
       <c r="L23" s="13" t="n"/>
       <c r="M23" s="13" t="n"/>
@@ -2006,7 +2000,7 @@
     <row r="24" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
@@ -2015,31 +2009,29 @@
         </is>
       </c>
       <c r="C24" s="12">
-        <f>ROUND(AVERAGE(F24:AA24), 0)</f>
+        <f>ROUND(AVERAGE(F24:AO24), 0)</f>
         <v/>
       </c>
       <c r="D24" s="1">
-        <f>SUM(F24:AA24)</f>
+        <f>SUM(F24:AO24)</f>
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>33550</v>
+        <v>29350</v>
       </c>
       <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n">
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J24" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="K24" s="13" t="n">
         <v>4000</v>
-      </c>
-      <c r="H24" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I24" s="13" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J24" s="13" t="n">
-        <v>5050</v>
-      </c>
-      <c r="K24" s="13" t="n">
-        <v>4150</v>
       </c>
       <c r="L24" s="13" t="n"/>
       <c r="M24" s="13" t="n"/>
@@ -2056,38 +2048,42 @@
     <row r="25" ht="16.5" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C25" s="12">
-        <f>ROUND(AVERAGE(F25:AA25), 0)</f>
+        <f>ROUND(AVERAGE(F25:AO25), 0)</f>
         <v/>
       </c>
       <c r="D25" s="1">
-        <f>SUM(F25:AA25)</f>
+        <f>SUM(F25:AO25)</f>
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>123800</v>
-      </c>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="13" t="n"/>
+        <v>39900</v>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H25" s="13" t="n">
         <v>4050</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>4100</v>
+        <v>5600</v>
       </c>
       <c r="J25" s="13" t="n">
-        <v>4000</v>
+        <v>1300</v>
       </c>
       <c r="K25" s="13" t="n">
-        <v>4100</v>
+        <v>3100</v>
       </c>
       <c r="L25" s="13" t="n"/>
       <c r="M25" s="13" t="n"/>
@@ -2104,7 +2100,7 @@
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
@@ -2113,29 +2109,29 @@
         </is>
       </c>
       <c r="C26" s="12">
-        <f>ROUND(AVERAGE(F26:AA26), 0)</f>
+        <f>ROUND(AVERAGE(F26:AO26), 0)</f>
         <v/>
       </c>
       <c r="D26" s="1">
-        <f>SUM(F26:AA26)</f>
+        <f>SUM(F26:AO26)</f>
         <v/>
       </c>
       <c r="E26" s="14" t="n">
-        <v>41000</v>
+        <v>31825</v>
       </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
       <c r="H26" s="13" t="n">
-        <v>1200</v>
+        <v>3650</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>4000</v>
+        <v>7600</v>
       </c>
       <c r="J26" s="13" t="n">
-        <v>150</v>
+        <v>3150</v>
       </c>
       <c r="K26" s="13" t="n">
-        <v>4050</v>
+        <v>3000</v>
       </c>
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="n"/>
@@ -2152,34 +2148,36 @@
     <row r="27" ht="16.5" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C27" s="12">
-        <f>ROUND(AVERAGE(F27:AA27), 0)</f>
+        <f>ROUND(AVERAGE(F27:AO27), 0)</f>
         <v/>
       </c>
       <c r="D27" s="1">
-        <f>SUM(F27:AA27)</f>
+        <f>SUM(F27:AO27)</f>
         <v/>
       </c>
       <c r="E27" s="14" t="n">
-        <v>27155</v>
+        <v>75000</v>
       </c>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
       <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
+      <c r="I27" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="J27" s="13" t="n">
-        <v>4250</v>
+        <v>950</v>
       </c>
       <c r="K27" s="13" t="n">
-        <v>4050</v>
+        <v>1400</v>
       </c>
       <c r="L27" s="13" t="n"/>
       <c r="M27" s="13" t="n"/>
@@ -2196,38 +2194,36 @@
     <row r="28" ht="16.5" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C28" s="12">
-        <f>ROUND(AVERAGE(F28:AA28), 0)</f>
+        <f>ROUND(AVERAGE(F28:AO28), 0)</f>
         <v/>
       </c>
       <c r="D28" s="1">
-        <f>SUM(F28:AA28)</f>
+        <f>SUM(F28:AO28)</f>
         <v/>
       </c>
       <c r="E28" s="14" t="n">
-        <v>29350</v>
+        <v>6800</v>
       </c>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H28" s="13" t="n"/>
       <c r="I28" s="13" t="n">
-        <v>3500</v>
+        <v>4150</v>
       </c>
       <c r="J28" s="13" t="n">
-        <v>4050</v>
+        <v>2650</v>
       </c>
       <c r="K28" s="13" t="n">
-        <v>4000</v>
+        <v>1050</v>
       </c>
       <c r="L28" s="13" t="n"/>
       <c r="M28" s="13" t="n"/>
@@ -2236,7 +2232,7 @@
       <c r="P28" s="13" t="n"/>
       <c r="Q28" s="13" t="n"/>
       <c r="R28" s="13" t="n"/>
-      <c r="S28" s="21" t="n"/>
+      <c r="S28" s="13" t="n"/>
       <c r="T28" s="13" t="n"/>
       <c r="U28" s="13" t="n"/>
       <c r="V28" s="13" t="n"/>
@@ -2244,42 +2240,32 @@
     <row r="29" ht="16.5" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C29" s="12">
-        <f>ROUND(AVERAGE(F29:AA29), 0)</f>
+        <f>ROUND(AVERAGE(F29:AO29), 0)</f>
         <v/>
       </c>
       <c r="D29" s="1">
-        <f>SUM(F29:AA29)</f>
+        <f>SUM(F29:AO29)</f>
         <v/>
       </c>
       <c r="E29" s="14" t="n">
-        <v>39900</v>
-      </c>
-      <c r="F29" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G29" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H29" s="13" t="n">
-        <v>4050</v>
-      </c>
-      <c r="I29" s="13" t="n">
-        <v>5600</v>
-      </c>
-      <c r="J29" s="13" t="n">
-        <v>1300</v>
-      </c>
+        <v>18000</v>
+      </c>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
       <c r="K29" s="13" t="n">
-        <v>3100</v>
+        <v>600</v>
       </c>
       <c r="L29" s="13" t="n"/>
       <c r="M29" s="13" t="n"/>
@@ -2288,7 +2274,7 @@
       <c r="P29" s="13" t="n"/>
       <c r="Q29" s="13" t="n"/>
       <c r="R29" s="13" t="n"/>
-      <c r="S29" s="21" t="n"/>
+      <c r="S29" s="13" t="n"/>
       <c r="T29" s="13" t="n"/>
       <c r="U29" s="13" t="n"/>
       <c r="V29" s="13" t="n"/>
@@ -2296,7 +2282,7 @@
     <row r="30" ht="16.5" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B30" s="16" t="inlineStr">
@@ -2305,29 +2291,29 @@
         </is>
       </c>
       <c r="C30" s="12">
-        <f>ROUND(AVERAGE(F30:AA30), 0)</f>
+        <f>ROUND(AVERAGE(F30:AO30), 0)</f>
         <v/>
       </c>
       <c r="D30" s="1">
-        <f>SUM(F30:AA30)</f>
+        <f>SUM(F30:AO30)</f>
         <v/>
       </c>
       <c r="E30" s="14" t="n">
-        <v>31825</v>
+        <v>15150</v>
       </c>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
       <c r="H30" s="13" t="n">
-        <v>3650</v>
+        <v>500</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>7600</v>
+        <v>1500</v>
       </c>
       <c r="J30" s="13" t="n">
-        <v>3150</v>
+        <v>0</v>
       </c>
       <c r="K30" s="13" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="L30" s="13" t="n"/>
       <c r="M30" s="13" t="n"/>
@@ -2336,7 +2322,7 @@
       <c r="P30" s="13" t="n"/>
       <c r="Q30" s="13" t="n"/>
       <c r="R30" s="13" t="n"/>
-      <c r="S30" s="21" t="n"/>
+      <c r="S30" s="13" t="n"/>
       <c r="T30" s="13" t="n"/>
       <c r="U30" s="13" t="n"/>
       <c r="V30" s="13" t="n"/>
@@ -2344,34 +2330,36 @@
     <row r="31" ht="16.5" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C31" s="12">
-        <f>ROUND(AVERAGE(F31:AA31), 0)</f>
+        <f>ROUND(AVERAGE(F31:AO31), 0)</f>
         <v/>
       </c>
       <c r="D31" s="1">
-        <f>SUM(F31:AA31)</f>
+        <f>SUM(F31:AO31)</f>
         <v/>
       </c>
       <c r="E31" s="14" t="n">
-        <v>2150</v>
+        <v>69000</v>
       </c>
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="13" t="n"/>
       <c r="H31" s="13" t="n"/>
-      <c r="I31" s="13" t="n"/>
+      <c r="I31" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="J31" s="13" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K31" s="13" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="L31" s="13" t="n"/>
       <c r="M31" s="13" t="n"/>
@@ -2380,7 +2368,7 @@
       <c r="P31" s="13" t="n"/>
       <c r="Q31" s="13" t="n"/>
       <c r="R31" s="13" t="n"/>
-      <c r="S31" s="21" t="n"/>
+      <c r="S31" s="13" t="n"/>
       <c r="T31" s="13" t="n"/>
       <c r="U31" s="13" t="n"/>
       <c r="V31" s="13" t="n"/>
@@ -2388,37 +2376,31 @@
     <row r="32" ht="16.5" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C32" s="12">
-        <f>ROUND(AVERAGE(F32:AA32), 0)</f>
+        <f>ROUND(AVERAGE(F32:AO32), 0)</f>
         <v/>
       </c>
       <c r="D32" s="1">
-        <f>SUM(F32:AA32)</f>
+        <f>SUM(F32:AO32)</f>
         <v/>
       </c>
       <c r="E32" s="14" t="n">
-        <v>75000</v>
+        <v>43650</v>
       </c>
       <c r="F32" s="13" t="n"/>
       <c r="G32" s="13" t="n"/>
       <c r="H32" s="13" t="n"/>
-      <c r="I32" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="13" t="n">
-        <v>950</v>
-      </c>
-      <c r="K32" s="13" t="n">
-        <v>1400</v>
-      </c>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
       <c r="L32" s="13" t="n"/>
       <c r="M32" s="13" t="n"/>
       <c r="N32" s="13" t="n"/>
@@ -2426,7 +2408,7 @@
       <c r="P32" s="13" t="n"/>
       <c r="Q32" s="13" t="n"/>
       <c r="R32" s="13" t="n"/>
-      <c r="S32" s="21" t="n"/>
+      <c r="S32" s="13" t="n"/>
       <c r="T32" s="13" t="n"/>
       <c r="U32" s="13" t="n"/>
       <c r="V32" s="13" t="n"/>
@@ -2434,37 +2416,31 @@
     <row r="33" ht="16.5" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C33" s="12">
-        <f>ROUND(AVERAGE(F33:AA33), 0)</f>
+        <f>ROUND(AVERAGE(F33:AO33), 0)</f>
         <v/>
       </c>
       <c r="D33" s="1">
-        <f>SUM(F33:AA33)</f>
+        <f>SUM(F33:AO33)</f>
         <v/>
       </c>
       <c r="E33" s="14" t="n">
-        <v>6800</v>
+        <v>13125</v>
       </c>
       <c r="F33" s="13" t="n"/>
       <c r="G33" s="13" t="n"/>
       <c r="H33" s="13" t="n"/>
-      <c r="I33" s="13" t="n">
-        <v>4150</v>
-      </c>
-      <c r="J33" s="13" t="n">
-        <v>2650</v>
-      </c>
-      <c r="K33" s="13" t="n">
-        <v>1050</v>
-      </c>
+      <c r="I33" s="13" t="n"/>
+      <c r="J33" s="13" t="n"/>
+      <c r="K33" s="13" t="n"/>
       <c r="L33" s="13" t="n"/>
       <c r="M33" s="13" t="n"/>
       <c r="N33" s="13" t="n"/>
@@ -2480,33 +2456,31 @@
     <row r="34" ht="16.5" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C34" s="12">
-        <f>ROUND(AVERAGE(F34:AA34), 0)</f>
+        <f>ROUND(AVERAGE(F34:AO34), 0)</f>
         <v/>
       </c>
       <c r="D34" s="1">
-        <f>SUM(F34:AA34)</f>
+        <f>SUM(F34:AO34)</f>
         <v/>
       </c>
       <c r="E34" s="14" t="n">
-        <v>18000</v>
+        <v>11250</v>
       </c>
       <c r="F34" s="13" t="n"/>
       <c r="G34" s="13" t="n"/>
       <c r="H34" s="13" t="n"/>
       <c r="I34" s="13" t="n"/>
       <c r="J34" s="13" t="n"/>
-      <c r="K34" s="13" t="n">
-        <v>600</v>
-      </c>
+      <c r="K34" s="13" t="n"/>
       <c r="L34" s="13" t="n"/>
       <c r="M34" s="13" t="n"/>
       <c r="N34" s="13" t="n"/>
@@ -2522,39 +2496,31 @@
     <row r="35" ht="16.5" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C35" s="12">
-        <f>ROUND(AVERAGE(F35:AA35), 0)</f>
+        <f>ROUND(AVERAGE(F35:AO35), 0)</f>
         <v/>
       </c>
       <c r="D35" s="1">
-        <f>SUM(F35:AA35)</f>
+        <f>SUM(F35:AO35)</f>
         <v/>
       </c>
       <c r="E35" s="14" t="n">
-        <v>15150</v>
+        <v>40640</v>
       </c>
       <c r="F35" s="13" t="n"/>
       <c r="G35" s="13" t="n"/>
-      <c r="H35" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="I35" s="13" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J35" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
+      <c r="J35" s="13" t="n"/>
+      <c r="K35" s="13" t="n"/>
       <c r="L35" s="13" t="n"/>
       <c r="M35" s="13" t="n"/>
       <c r="N35" s="13" t="n"/>
@@ -2570,37 +2536,31 @@
     <row r="36" ht="16.5" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>nanni</t>
         </is>
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C36" s="12">
-        <f>ROUND(AVERAGE(F36:AA36), 0)</f>
+        <f>ROUND(AVERAGE(F36:AO36), 0)</f>
         <v/>
       </c>
       <c r="D36" s="1">
-        <f>SUM(F36:AA36)</f>
+        <f>SUM(F36:AO36)</f>
         <v/>
       </c>
       <c r="E36" s="14" t="n">
-        <v>69000</v>
+        <v>69525</v>
       </c>
       <c r="F36" s="13" t="n"/>
       <c r="G36" s="13" t="n"/>
       <c r="H36" s="13" t="n"/>
-      <c r="I36" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J36" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K36" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="I36" s="13" t="n"/>
+      <c r="J36" s="13" t="n"/>
+      <c r="K36" s="13" t="n"/>
       <c r="L36" s="13" t="n"/>
       <c r="M36" s="13" t="n"/>
       <c r="N36" s="13" t="n"/>
@@ -2616,24 +2576,24 @@
     <row r="37" ht="16.5" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>falcuns</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>27/03/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C37" s="12">
-        <f>ROUND(AVERAGE(F37:AA37), 0)</f>
+        <f>ROUND(AVERAGE(F37:AO37), 0)</f>
         <v/>
       </c>
       <c r="D37" s="1">
-        <f>SUM(F37:AA37)</f>
+        <f>SUM(F37:AO37)</f>
         <v/>
       </c>
       <c r="E37" s="14" t="n">
-        <v>250</v>
+        <v>56200</v>
       </c>
       <c r="F37" s="13" t="n"/>
       <c r="G37" s="13" t="n"/>
@@ -2656,24 +2616,24 @@
     <row r="38" ht="16.5" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>DJ Tony</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C38" s="12">
-        <f>ROUND(AVERAGE(F38:AA38), 0)</f>
+        <f>ROUND(AVERAGE(F38:AO38), 0)</f>
         <v/>
       </c>
       <c r="D38" s="1">
-        <f>SUM(F38:AA38)</f>
+        <f>SUM(F38:AO38)</f>
         <v/>
       </c>
       <c r="E38" s="14" t="n">
-        <v>43650</v>
+        <v>14060</v>
       </c>
       <c r="F38" s="13" t="n"/>
       <c r="G38" s="13" t="n"/>
@@ -2696,24 +2656,24 @@
     <row r="39" ht="16.5" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C39" s="12">
-        <f>ROUND(AVERAGE(F39:AA39), 0)</f>
+        <f>ROUND(AVERAGE(F39:AO39), 0)</f>
         <v/>
       </c>
       <c r="D39" s="1">
-        <f>SUM(F39:AA39)</f>
+        <f>SUM(F39:AO39)</f>
         <v/>
       </c>
       <c r="E39" s="14" t="n">
-        <v>13125</v>
+        <v>39650</v>
       </c>
       <c r="F39" s="13" t="n"/>
       <c r="G39" s="13" t="n"/>
@@ -2736,24 +2696,24 @@
     <row r="40" ht="16.5" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C40" s="12">
-        <f>ROUND(AVERAGE(F40:AA40), 0)</f>
+        <f>ROUND(AVERAGE(F40:AO40), 0)</f>
         <v/>
       </c>
       <c r="D40" s="1">
-        <f>SUM(F40:AA40)</f>
+        <f>SUM(F40:AO40)</f>
         <v/>
       </c>
       <c r="E40" s="14" t="n">
-        <v>250</v>
+        <v>42850</v>
       </c>
       <c r="F40" s="13" t="n"/>
       <c r="G40" s="13" t="n"/>
@@ -2776,24 +2736,24 @@
     <row r="41" ht="16.5" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C41" s="12">
-        <f>ROUND(AVERAGE(F41:AA41), 0)</f>
+        <f>ROUND(AVERAGE(F41:AO41), 0)</f>
         <v/>
       </c>
       <c r="D41" s="1">
-        <f>SUM(F41:AA41)</f>
+        <f>SUM(F41:AO41)</f>
         <v/>
       </c>
       <c r="E41" s="14" t="n">
-        <v>0</v>
+        <v>56865</v>
       </c>
       <c r="F41" s="13" t="n"/>
       <c r="G41" s="13" t="n"/>
@@ -2816,24 +2776,24 @@
     <row r="42" ht="16.5" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C42" s="12">
-        <f>ROUND(AVERAGE(F42:AA42), 0)</f>
+        <f>ROUND(AVERAGE(F42:AO42), 0)</f>
         <v/>
       </c>
       <c r="D42" s="1">
-        <f>SUM(F42:AA42)</f>
+        <f>SUM(F42:AO42)</f>
         <v/>
       </c>
       <c r="E42" s="14" t="n">
-        <v>11250</v>
+        <v>25810</v>
       </c>
       <c r="F42" s="13" t="n"/>
       <c r="G42" s="13" t="n"/>
@@ -2856,24 +2816,24 @@
     <row r="43" ht="16.5" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C43" s="12">
-        <f>ROUND(AVERAGE(F43:AA43), 0)</f>
+        <f>ROUND(AVERAGE(F43:AO43), 0)</f>
         <v/>
       </c>
       <c r="D43" s="1">
-        <f>SUM(F43:AA43)</f>
+        <f>SUM(F43:AO43)</f>
         <v/>
       </c>
       <c r="E43" s="14" t="n">
-        <v>40640</v>
+        <v>110325</v>
       </c>
       <c r="F43" s="13" t="n"/>
       <c r="G43" s="13" t="n"/>
@@ -2896,24 +2856,24 @@
     <row r="44" ht="16.5" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>re deo</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C44" s="12">
-        <f>ROUND(AVERAGE(F44:AA44), 0)</f>
+        <f>ROUND(AVERAGE(F44:AO44), 0)</f>
         <v/>
       </c>
       <c r="D44" s="1">
-        <f>SUM(F44:AA44)</f>
+        <f>SUM(F44:AO44)</f>
         <v/>
       </c>
       <c r="E44" s="14" t="n">
-        <v>12375</v>
+        <v>33210</v>
       </c>
       <c r="F44" s="13" t="n"/>
       <c r="G44" s="13" t="n"/>
@@ -2933,246 +2893,12 @@
       <c r="U44" s="13" t="n"/>
       <c r="V44" s="13" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
-        <is>
-          <t>Dade_Aca_03</t>
-        </is>
-      </c>
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="C45" s="12">
-        <f>ROUND(AVERAGE(F45:AA45), 0)</f>
-        <v/>
-      </c>
-      <c r="D45" s="1">
-        <f>SUM(F45:AA45)</f>
-        <v/>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>26325</v>
-      </c>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="13" t="n"/>
-      <c r="H45" s="13" t="n"/>
-      <c r="I45" s="13" t="n"/>
-      <c r="J45" s="13" t="n"/>
-      <c r="K45" s="13" t="n"/>
-      <c r="L45" s="13" t="n"/>
-      <c r="M45" s="13" t="n"/>
-      <c r="N45" s="13" t="n"/>
-      <c r="O45" s="13" t="n"/>
-      <c r="P45" s="13" t="n"/>
-      <c r="Q45" s="13" t="n"/>
-      <c r="R45" s="13" t="n"/>
-      <c r="S45" s="13" t="n"/>
-      <c r="T45" s="13" t="n"/>
-      <c r="U45" s="13" t="n"/>
-      <c r="V45" s="13" t="n"/>
-    </row>
-    <row r="46" ht="16.5" customHeight="1">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>-_HORROR_-</t>
-        </is>
-      </c>
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="12">
-        <f>ROUND(AVERAGE(F46:AA46), 0)</f>
-        <v/>
-      </c>
-      <c r="D46" s="1">
-        <f>SUM(F46:AA46)</f>
-        <v/>
-      </c>
-      <c r="E46" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="13" t="n"/>
-      <c r="G46" s="13" t="n"/>
-      <c r="H46" s="13" t="n"/>
-      <c r="I46" s="13" t="n"/>
-      <c r="J46" s="13" t="n"/>
-      <c r="K46" s="13" t="n"/>
-      <c r="L46" s="13" t="n"/>
-      <c r="M46" s="13" t="n"/>
-      <c r="N46" s="13" t="n"/>
-      <c r="O46" s="13" t="n"/>
-      <c r="P46" s="13" t="n"/>
-      <c r="Q46" s="13" t="n"/>
-      <c r="R46" s="13" t="n"/>
-      <c r="S46" s="13" t="n"/>
-      <c r="T46" s="13" t="n"/>
-      <c r="U46" s="13" t="n"/>
-      <c r="V46" s="13" t="n"/>
-    </row>
-    <row r="47" ht="16.5" customHeight="1">
-      <c r="A47" s="14" t="inlineStr">
-        <is>
-          <t>-WOLF-</t>
-        </is>
-      </c>
-      <c r="B47" s="16" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="12">
-        <f>ROUND(AVERAGE(F47:AA47), 0)</f>
-        <v/>
-      </c>
-      <c r="D47" s="1">
-        <f>SUM(F47:AA47)</f>
-        <v/>
-      </c>
-      <c r="E47" s="14" t="n">
-        <v>17500</v>
-      </c>
-      <c r="F47" s="13" t="n"/>
-      <c r="G47" s="13" t="n"/>
-      <c r="H47" s="13" t="n"/>
-      <c r="I47" s="13" t="n"/>
-      <c r="J47" s="13" t="n"/>
-      <c r="K47" s="13" t="n"/>
-      <c r="L47" s="13" t="n"/>
-      <c r="M47" s="13" t="n"/>
-      <c r="N47" s="13" t="n"/>
-      <c r="O47" s="13" t="n"/>
-      <c r="P47" s="13" t="n"/>
-      <c r="Q47" s="13" t="n"/>
-      <c r="R47" s="13" t="n"/>
-      <c r="S47" s="13" t="n"/>
-      <c r="T47" s="13" t="n"/>
-      <c r="U47" s="13" t="n"/>
-      <c r="V47" s="13" t="n"/>
-    </row>
-    <row r="48" ht="16.5" customHeight="1">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t>AnT0x</t>
-        </is>
-      </c>
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="12">
-        <f>ROUND(AVERAGE(F48:AA48), 0)</f>
-        <v/>
-      </c>
-      <c r="D48" s="1">
-        <f>SUM(F48:AA48)</f>
-        <v/>
-      </c>
-      <c r="E48" s="14" t="n">
-        <v>30095</v>
-      </c>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="13" t="n"/>
-      <c r="H48" s="13" t="n"/>
-      <c r="I48" s="13" t="n"/>
-      <c r="J48" s="13" t="n"/>
-      <c r="K48" s="13" t="n"/>
-      <c r="L48" s="13" t="n"/>
-      <c r="M48" s="13" t="n"/>
-      <c r="N48" s="13" t="n"/>
-      <c r="O48" s="13" t="n"/>
-      <c r="P48" s="13" t="n"/>
-      <c r="Q48" s="13" t="n"/>
-      <c r="R48" s="13" t="n"/>
-      <c r="S48" s="13" t="n"/>
-      <c r="T48" s="13" t="n"/>
-      <c r="U48" s="13" t="n"/>
-      <c r="V48" s="13" t="n"/>
-    </row>
-    <row r="49" ht="16.5" customHeight="1">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>Tropical</t>
-        </is>
-      </c>
-      <c r="B49" s="16" t="inlineStr">
-        <is>
-          <t>27/04/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="12">
-        <f>ROUND(AVERAGE(F49:AA49), 0)</f>
-        <v/>
-      </c>
-      <c r="D49" s="1">
-        <f>SUM(F49:AA49)</f>
-        <v/>
-      </c>
-      <c r="E49" s="14" t="n">
-        <v>8350</v>
-      </c>
-      <c r="F49" s="13" t="n"/>
-      <c r="G49" s="13" t="n"/>
-      <c r="H49" s="13" t="n"/>
-      <c r="I49" s="13" t="n"/>
-      <c r="J49" s="13" t="n"/>
-      <c r="K49" s="13" t="n"/>
-      <c r="L49" s="13" t="n"/>
-      <c r="M49" s="13" t="n"/>
-      <c r="N49" s="13" t="n"/>
-      <c r="O49" s="13" t="n"/>
-      <c r="P49" s="13" t="n"/>
-      <c r="Q49" s="13" t="n"/>
-      <c r="R49" s="13" t="n"/>
-      <c r="S49" s="13" t="n"/>
-      <c r="T49" s="13" t="n"/>
-      <c r="U49" s="13" t="n"/>
-      <c r="V49" s="13" t="n"/>
-    </row>
-    <row r="50" ht="16.5" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t>ldl</t>
-        </is>
-      </c>
-      <c r="B50" s="16" t="inlineStr">
-        <is>
-          <t>28/04/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="12">
-        <f>ROUND(AVERAGE(F50:AA50), 0)</f>
-        <v/>
-      </c>
-      <c r="D50" s="1">
-        <f>SUM(F50:AA50)</f>
-        <v/>
-      </c>
-      <c r="E50" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="13" t="n"/>
-      <c r="J50" s="13" t="n"/>
-      <c r="K50" s="13" t="n"/>
-      <c r="L50" s="13" t="n"/>
-      <c r="M50" s="13" t="n"/>
-      <c r="N50" s="13" t="n"/>
-      <c r="O50" s="13" t="n"/>
-      <c r="P50" s="13" t="n"/>
-      <c r="Q50" s="13" t="n"/>
-      <c r="R50" s="13" t="n"/>
-      <c r="S50" s="13" t="n"/>
-      <c r="T50" s="13" t="n"/>
-      <c r="U50" s="13" t="n"/>
-      <c r="V50" s="13" t="n"/>
-    </row>
+    <row r="45" ht="16.5" customHeight="1"/>
+    <row r="46" ht="16.5" customHeight="1"/>
+    <row r="47" ht="16.5" customHeight="1"/>
+    <row r="48" ht="16.5" customHeight="1"/>
+    <row r="49" ht="16.5" customHeight="1"/>
+    <row r="50" ht="16.5" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:AN1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-10
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -4319,7 +4319,7 @@
         <v>6</v>
       </c>
       <c r="AB17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -5000,7 +5000,7 @@
         <v>4</v>
       </c>
       <c r="AB26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -5253,7 +5253,7 @@
         <v>6</v>
       </c>
       <c r="AB29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -5534,7 +5534,7 @@
         <v>6</v>
       </c>
       <c r="AB34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-11
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3354,7 +3354,7 @@
         <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3445,7 +3445,7 @@
         <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -3536,7 +3536,7 @@
         <v>6</v>
       </c>
       <c r="AB7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -3679,7 +3679,7 @@
         <v>0</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -3810,7 +3810,7 @@
         <v>6</v>
       </c>
       <c r="AB11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -4228,7 +4228,7 @@
         <v>0</v>
       </c>
       <c r="AB16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -4456,7 +4456,7 @@
         <v>0</v>
       </c>
       <c r="AB19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -4690,7 +4690,7 @@
         <v>0</v>
       </c>
       <c r="AB22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -4772,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="AB23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -4839,7 +4839,7 @@
         <v>0</v>
       </c>
       <c r="AB24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -4909,7 +4909,7 @@
         <v>2</v>
       </c>
       <c r="AB25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -5000,7 +5000,7 @@
         <v>4</v>
       </c>
       <c r="AB26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -5091,7 +5091,7 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -5182,7 +5182,7 @@
         <v>0</v>
       </c>
       <c r="AB28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -5534,7 +5534,7 @@
         <v>6</v>
       </c>
       <c r="AB34" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-16
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2891,7 +2891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH44"/>
+  <dimension ref="A1:AH46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="9" min="1" max="1"/>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="AC1" s="3" t="inlineStr">
         <is>
-          <t>Colonna27</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="AD1" s="3" t="inlineStr">
@@ -3148,6 +3148,9 @@
       <c r="AB2" t="n">
         <v>0</v>
       </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -3213,6 +3216,9 @@
         <v>0</v>
       </c>
       <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3274,6 +3280,9 @@
       <c r="AB4" t="n">
         <v>6</v>
       </c>
+      <c r="AC4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -3356,6 +3365,9 @@
       <c r="AB5" t="n">
         <v>6</v>
       </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -3447,6 +3459,9 @@
       <c r="AB6" t="n">
         <v>6</v>
       </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -3537,6 +3552,9 @@
       </c>
       <c r="AB7" t="n">
         <v>6</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3599,6 +3617,9 @@
       <c r="AB8" t="n">
         <v>0</v>
       </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -3680,6 +3701,9 @@
       </c>
       <c r="AB9" t="n">
         <v>6</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3730,6 +3754,9 @@
       <c r="AB10" t="n">
         <v>0</v>
       </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -3812,6 +3839,9 @@
       <c r="AB11" t="n">
         <v>6</v>
       </c>
+      <c r="AC11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -3903,34 +3933,25 @@
       <c r="AB12" t="n">
         <v>6</v>
       </c>
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C13" s="9">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
-      <c r="D13" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="H13" s="5" t="n">
         <v>6</v>
       </c>
@@ -3977,39 +3998,54 @@
         <v>6</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB13" t="n">
         <v>0</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C14" s="9">
         <f>ROUND(AVERAGE(D14:AH14), 0)</f>
         <v/>
       </c>
+      <c r="D14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="H14" s="5" t="n">
         <v>6</v>
       </c>
@@ -4053,74 +4089,52 @@
         <v>6</v>
       </c>
       <c r="V14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA14" t="n">
         <v>6</v>
       </c>
       <c r="AB14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C15" s="9">
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
-      <c r="D15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
       <c r="M15" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N15" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O15" t="n">
         <v>6</v>
@@ -4141,52 +4155,80 @@
         <v>6</v>
       </c>
       <c r="U15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z15" t="n">
         <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC15" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="9">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="6" t="n"/>
+      <c r="D16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="M16" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N16" s="13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O16" t="n">
         <v>6</v>
@@ -4207,7 +4249,7 @@
         <v>6</v>
       </c>
       <c r="U16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V16" t="n">
         <v>6</v>
@@ -4219,77 +4261,44 @@
         <v>6</v>
       </c>
       <c r="Y16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z16" t="n">
         <v>0</v>
       </c>
       <c r="AA16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB16" t="n">
         <v>6</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C17" s="9">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="D17" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N17" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="O17" t="n">
-        <v>6</v>
-      </c>
-      <c r="P17" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>6</v>
-      </c>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="19" t="n"/>
+      <c r="P17" s="19" t="n"/>
+      <c r="Q17" s="19" t="n"/>
       <c r="R17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
         <v>6</v>
@@ -4307,44 +4316,74 @@
         <v>6</v>
       </c>
       <c r="X17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA17" t="n">
         <v>6</v>
       </c>
       <c r="AB17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC17" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C18" s="9">
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
-      <c r="K18" s="6" t="n"/>
-      <c r="L18" s="6" t="n"/>
-      <c r="N18" s="6" t="n"/>
-      <c r="O18" s="19" t="n"/>
-      <c r="P18" s="19" t="n"/>
-      <c r="Q18" s="19" t="n"/>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O18" t="n">
+        <v>6</v>
+      </c>
+      <c r="P18" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>6</v>
+      </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S18" t="n">
         <v>6</v>
@@ -4359,28 +4398,31 @@
         <v>6</v>
       </c>
       <c r="W18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AA18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB18" t="n">
         <v>6</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -4392,11 +4434,20 @@
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
+      <c r="D19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>6</v>
@@ -4405,16 +4456,16 @@
         <v>6</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
         <v>6</v>
@@ -4435,34 +4486,37 @@
         <v>6</v>
       </c>
       <c r="U19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X19" t="n">
         <v>6</v>
       </c>
       <c r="Y19" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z19" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB19" t="n">
         <v>6</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -4474,20 +4528,11 @@
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="D20" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G20" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>6</v>
@@ -4496,24 +4541,24 @@
         <v>6</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q20" t="n">
+        <v>6</v>
+      </c>
+      <c r="O20" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P20" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q20" s="20" t="n">
         <v>6</v>
       </c>
       <c r="R20" t="n">
@@ -4526,50 +4571,74 @@
         <v>6</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB20" t="n">
         <v>6</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C21" s="9">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="n"/>
-      <c r="N21" s="6" t="n"/>
+      <c r="G21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="O21" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P21" s="20" t="n">
         <v>6</v>
@@ -4590,57 +4659,45 @@
         <v>6</v>
       </c>
       <c r="V21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W21" t="n">
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA21" t="n">
         <v>0</v>
       </c>
       <c r="AB21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C22" s="9">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
-      <c r="G22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K22" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L22" s="6" t="n">
         <v>6</v>
       </c>
@@ -4659,7 +4716,7 @@
       <c r="Q22" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="R22" t="n">
+      <c r="R22" s="20" t="n">
         <v>6</v>
       </c>
       <c r="S22" t="n">
@@ -4681,45 +4738,36 @@
         <v>0</v>
       </c>
       <c r="Y22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
       </c>
       <c r="AB22" t="n">
         <v>6</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C23" s="9">
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
-      <c r="G23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J23" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="K23" s="6" t="n">
         <v>6</v>
       </c>
@@ -4741,7 +4789,7 @@
       <c r="Q23" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="R23" t="n">
+      <c r="R23" s="20" t="n">
         <v>6</v>
       </c>
       <c r="S23" t="n">
@@ -4757,39 +4805,66 @@
         <v>6</v>
       </c>
       <c r="W23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB23" t="n">
         <v>6</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C24" s="9">
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
+      <c r="D24" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="L24" s="6" t="n">
         <v>6</v>
       </c>
@@ -4815,48 +4890,72 @@
         <v>6</v>
       </c>
       <c r="T24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V24" t="n">
         <v>6</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AB24" t="n">
         <v>6</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C25" s="9">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
+      <c r="D25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="K25" s="6" t="n">
         <v>6</v>
       </c>
@@ -4881,7 +4980,7 @@
       <c r="R25" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S25" t="n">
+      <c r="S25" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T25" t="n">
@@ -4891,31 +4990,34 @@
         <v>6</v>
       </c>
       <c r="V25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB25" t="n">
         <v>6</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -4972,41 +5074,44 @@
       <c r="R26" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S26" t="n">
+      <c r="S26" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T26" t="n">
+        <v>6</v>
+      </c>
+      <c r="U26" t="n">
+        <v>6</v>
+      </c>
+      <c r="V26" t="n">
+        <v>6</v>
+      </c>
+      <c r="W26" t="n">
+        <v>6</v>
+      </c>
+      <c r="X26" t="n">
         <v>4</v>
       </c>
-      <c r="U26" t="n">
-        <v>0</v>
-      </c>
-      <c r="V26" t="n">
-        <v>6</v>
-      </c>
-      <c r="W26" t="n">
+      <c r="Y26" t="n">
         <v>3</v>
       </c>
-      <c r="X26" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>0</v>
-      </c>
       <c r="Z26" t="n">
         <v>0</v>
       </c>
       <c r="AA26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -5018,86 +5123,69 @@
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
-      <c r="D27" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J27" s="6" t="n">
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N27" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U27" t="n">
+        <v>6</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" t="n">
         <v>5</v>
       </c>
-      <c r="K27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T27" t="n">
-        <v>6</v>
-      </c>
-      <c r="U27" t="n">
-        <v>6</v>
-      </c>
-      <c r="V27" t="n">
-        <v>0</v>
-      </c>
-      <c r="W27" t="n">
-        <v>0</v>
-      </c>
       <c r="X27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB27" t="n">
         <v>6</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -5109,15 +5197,6 @@
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
-      <c r="D28" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F28" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G28" s="5" t="n">
         <v>6</v>
       </c>
@@ -5146,7 +5225,7 @@
         <v>6</v>
       </c>
       <c r="P28" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q28" s="20" t="n">
         <v>6</v>
@@ -5157,50 +5236,52 @@
       <c r="S28" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="T28" t="n">
-        <v>6</v>
-      </c>
-      <c r="U28" t="n">
+      <c r="T28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U28" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W28" t="n">
         <v>6</v>
       </c>
       <c r="X28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA28" t="n">
         <v>0</v>
       </c>
       <c r="AB28" t="n">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="C29" s="9">
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n">
         <v>6</v>
       </c>
@@ -5208,10 +5289,10 @@
         <v>6</v>
       </c>
       <c r="M29" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O29" s="20" t="n">
         <v>6</v>
@@ -5223,177 +5304,122 @@
         <v>6</v>
       </c>
       <c r="R29" s="20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S29" s="20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U29" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="U29" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="V29" t="n">
         <v>0</v>
       </c>
       <c r="W29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB29" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C30" s="9">
         <f>ROUND(AVERAGE(D30:AH30), 0)</f>
         <v/>
       </c>
-      <c r="G30" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J30" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K30" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L30" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M30" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N30" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P30" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T30" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U30" s="20" t="n">
-        <v>6</v>
-      </c>
+      <c r="K30" s="6" t="n"/>
+      <c r="L30" s="6" t="n"/>
+      <c r="N30" s="6" t="n"/>
+      <c r="O30" s="20" t="n"/>
+      <c r="P30" s="20" t="n"/>
+      <c r="Q30" s="20" t="n"/>
+      <c r="R30" s="20" t="n"/>
+      <c r="S30" s="20" t="n"/>
+      <c r="T30" s="20" t="n"/>
+      <c r="U30" s="20" t="n"/>
       <c r="V30" t="n">
         <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X30" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y30" t="n">
         <v>0</v>
       </c>
       <c r="Z30" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AA30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB30" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C31" s="9">
         <f>ROUND(AVERAGE(D31:AH31), 0)</f>
         <v/>
       </c>
-      <c r="K31" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L31" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q31" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="U31" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V31" t="n">
-        <v>0</v>
-      </c>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="n"/>
+      <c r="N31" s="6" t="n"/>
+      <c r="O31" s="20" t="n"/>
+      <c r="P31" s="20" t="n"/>
+      <c r="Q31" s="20" t="n"/>
+      <c r="R31" s="20" t="n"/>
+      <c r="S31" s="20" t="n"/>
+      <c r="T31" s="20" t="n"/>
+      <c r="U31" s="20" t="n"/>
       <c r="W31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y31" t="n">
         <v>0</v>
@@ -5402,21 +5428,24 @@
         <v>0</v>
       </c>
       <c r="AA31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C32" s="9">
@@ -5433,17 +5462,8 @@
       <c r="S32" s="20" t="n"/>
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X32" t="n">
-        <v>6</v>
-      </c>
       <c r="Y32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z32" t="n">
         <v>3</v>
@@ -5452,18 +5472,21 @@
         <v>6</v>
       </c>
       <c r="AB32" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C33" s="9">
@@ -5480,12 +5503,6 @@
       <c r="S33" s="20" t="n"/>
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
-      <c r="W33" t="n">
-        <v>6</v>
-      </c>
-      <c r="X33" t="n">
-        <v>6</v>
-      </c>
       <c r="Y33" t="n">
         <v>0</v>
       </c>
@@ -5493,21 +5510,24 @@
         <v>0</v>
       </c>
       <c r="AA33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB33" t="n">
         <v>0</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C34" s="9">
@@ -5524,28 +5544,28 @@
       <c r="S34" s="20" t="n"/>
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
-      <c r="Y34" t="n">
-        <v>6</v>
-      </c>
       <c r="Z34" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA34" t="n">
         <v>3</v>
       </c>
-      <c r="AA34" t="n">
-        <v>6</v>
-      </c>
       <c r="AB34" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC34" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C35" s="9">
@@ -5562,28 +5582,25 @@
       <c r="S35" s="20" t="n"/>
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
-      <c r="Y35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>0</v>
-      </c>
       <c r="AA35" t="n">
         <v>0</v>
       </c>
       <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C36" s="9">
@@ -5600,20 +5617,20 @@
       <c r="S36" s="20" t="n"/>
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
-      <c r="Z36" t="n">
-        <v>6</v>
-      </c>
       <c r="AA36" t="n">
         <v>3</v>
       </c>
       <c r="AB36" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
@@ -5641,16 +5658,19 @@
       <c r="AB37" t="n">
         <v>0</v>
       </c>
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C38" s="9">
@@ -5667,22 +5687,22 @@
       <c r="S38" s="20" t="n"/>
       <c r="T38" s="20" t="n"/>
       <c r="U38" s="20" t="n"/>
-      <c r="AA38" t="n">
-        <v>3</v>
-      </c>
       <c r="AB38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C39" s="9">
@@ -5699,17 +5719,17 @@
       <c r="S39" s="20" t="n"/>
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
-      <c r="AA39" t="n">
-        <v>0</v>
-      </c>
       <c r="AB39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -5732,13 +5752,16 @@
       <c r="T40" s="20" t="n"/>
       <c r="U40" s="20" t="n"/>
       <c r="AB40" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>DJ Tony</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
@@ -5761,18 +5784,21 @@
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
       <c r="AB41" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C42" s="9">
@@ -5789,19 +5815,19 @@
       <c r="S42" s="20" t="n"/>
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
-      <c r="AB42" t="n">
+      <c r="AC42" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>nanni</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C43" s="9">
@@ -5818,19 +5844,19 @@
       <c r="S43" s="20" t="n"/>
       <c r="T43" s="20" t="n"/>
       <c r="U43" s="20" t="n"/>
-      <c r="AB43" t="n">
+      <c r="AC43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>DJ Tony</t>
+          <t>Space_GG</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C44" s="9">
@@ -5847,8 +5873,66 @@
       <c r="S44" s="20" t="n"/>
       <c r="T44" s="20" t="n"/>
       <c r="U44" s="20" t="n"/>
-      <c r="AB44" t="n">
-        <v>0</v>
+      <c r="AC44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Matrox☆ita</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="9">
+        <f>ROUND(AVERAGE(D45:AH45), 0)</f>
+        <v/>
+      </c>
+      <c r="K45" s="6" t="n"/>
+      <c r="L45" s="6" t="n"/>
+      <c r="N45" s="6" t="n"/>
+      <c r="O45" s="20" t="n"/>
+      <c r="P45" s="20" t="n"/>
+      <c r="Q45" s="20" t="n"/>
+      <c r="R45" s="20" t="n"/>
+      <c r="S45" s="20" t="n"/>
+      <c r="T45" s="20" t="n"/>
+      <c r="U45" s="20" t="n"/>
+      <c r="AC45" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>roberto</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="9">
+        <f>ROUND(AVERAGE(D46:AH46), 0)</f>
+        <v/>
+      </c>
+      <c r="K46" s="6" t="n"/>
+      <c r="L46" s="6" t="n"/>
+      <c r="N46" s="6" t="n"/>
+      <c r="O46" s="20" t="n"/>
+      <c r="P46" s="20" t="n"/>
+      <c r="Q46" s="20" t="n"/>
+      <c r="R46" s="20" t="n"/>
+      <c r="S46" s="20" t="n"/>
+      <c r="T46" s="20" t="n"/>
+      <c r="U46" s="20" t="n"/>
+      <c r="AC46" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-17
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2891,7 +2891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH46"/>
+  <dimension ref="A1:AH45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="9" min="1" max="1"/>
@@ -3934,7 +3934,7 @@
         <v>6</v>
       </c>
       <c r="AC12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -4416,7 +4416,7 @@
         <v>6</v>
       </c>
       <c r="AC18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -4595,7 +4595,7 @@
         <v>6</v>
       </c>
       <c r="AC20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -4680,7 +4680,7 @@
         <v>6</v>
       </c>
       <c r="AC21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -5105,7 +5105,7 @@
         <v>2</v>
       </c>
       <c r="AC26" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -5270,51 +5270,28 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="C29" s="9">
         <f>ROUND(AVERAGE(D29:AH29), 0)</f>
         <v/>
       </c>
-      <c r="K29" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L29" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q29" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="U29" s="20" t="n">
-        <v>0</v>
-      </c>
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="6" t="n"/>
+      <c r="N29" s="6" t="n"/>
+      <c r="O29" s="20" t="n"/>
+      <c r="P29" s="20" t="n"/>
+      <c r="Q29" s="20" t="n"/>
+      <c r="R29" s="20" t="n"/>
+      <c r="S29" s="20" t="n"/>
+      <c r="T29" s="20" t="n"/>
+      <c r="U29" s="20" t="n"/>
       <c r="V29" t="n">
         <v>0</v>
       </c>
@@ -5322,16 +5299,16 @@
         <v>0</v>
       </c>
       <c r="X29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y29" t="n">
         <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -5343,12 +5320,12 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C30" s="9">
@@ -5365,11 +5342,8 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="V30" t="n">
-        <v>0</v>
-      </c>
       <c r="W30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X30" t="n">
         <v>6</v>
@@ -5378,27 +5352,27 @@
         <v>0</v>
       </c>
       <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
         <v>3</v>
-      </c>
-      <c r="AA30" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C31" s="9">
@@ -5415,23 +5389,17 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="W31" t="n">
-        <v>6</v>
-      </c>
-      <c r="X31" t="n">
-        <v>6</v>
-      </c>
       <c r="Y31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA31" t="n">
         <v>6</v>
       </c>
       <c r="AB31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC31" t="n">
         <v>0</v>
@@ -5440,7 +5408,7 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -5463,30 +5431,30 @@
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
       <c r="Y32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C33" s="9">
@@ -5503,17 +5471,14 @@
       <c r="S33" s="20" t="n"/>
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
-      <c r="Y33" t="n">
-        <v>0</v>
-      </c>
       <c r="Z33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC33" t="n">
         <v>6</v>
@@ -5522,12 +5487,12 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C34" s="9">
@@ -5544,23 +5509,20 @@
       <c r="S34" s="20" t="n"/>
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
-      <c r="Z34" t="n">
-        <v>6</v>
-      </c>
       <c r="AA34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
@@ -5583,19 +5545,19 @@
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
       <c r="AA35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB35" t="n">
         <v>0</v>
       </c>
       <c r="AC35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -5618,7 +5580,7 @@
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
       <c r="AA36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB36" t="n">
         <v>0</v>
@@ -5630,12 +5592,12 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C37" s="9">
@@ -5652,11 +5614,8 @@
       <c r="S37" s="20" t="n"/>
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
-      <c r="AA37" t="n">
-        <v>0</v>
-      </c>
       <c r="AB37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC37" t="n">
         <v>0</v>
@@ -5665,7 +5624,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -5697,7 +5656,7 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
@@ -5720,7 +5679,7 @@
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
       <c r="AB39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC39" t="n">
         <v>0</v>
@@ -5729,12 +5688,12 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C40" s="9">
@@ -5751,9 +5710,6 @@
       <c r="S40" s="20" t="n"/>
       <c r="T40" s="20" t="n"/>
       <c r="U40" s="20" t="n"/>
-      <c r="AB40" t="n">
-        <v>0</v>
-      </c>
       <c r="AC40" t="n">
         <v>0</v>
       </c>
@@ -5761,12 +5717,12 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>DJ Tony</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C41" s="9">
@@ -5783,9 +5739,6 @@
       <c r="S41" s="20" t="n"/>
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
-      <c r="AB41" t="n">
-        <v>0</v>
-      </c>
       <c r="AC41" t="n">
         <v>0</v>
       </c>
@@ -5793,7 +5746,7 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>Space_GG</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -5822,7 +5775,7 @@
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
@@ -5845,13 +5798,13 @@
       <c r="T43" s="20" t="n"/>
       <c r="U43" s="20" t="n"/>
       <c r="AC43" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>Space_GG</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -5874,18 +5827,18 @@
       <c r="T44" s="20" t="n"/>
       <c r="U44" s="20" t="n"/>
       <c r="AC44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C45" s="9">
@@ -5903,35 +5856,6 @@
       <c r="T45" s="20" t="n"/>
       <c r="U45" s="20" t="n"/>
       <c r="AC45" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>roberto</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>16/05/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="9">
-        <f>ROUND(AVERAGE(D46:AH46), 0)</f>
-        <v/>
-      </c>
-      <c r="K46" s="6" t="n"/>
-      <c r="L46" s="6" t="n"/>
-      <c r="N46" s="6" t="n"/>
-      <c r="O46" s="20" t="n"/>
-      <c r="P46" s="20" t="n"/>
-      <c r="Q46" s="20" t="n"/>
-      <c r="R46" s="20" t="n"/>
-      <c r="S46" s="20" t="n"/>
-      <c r="T46" s="20" t="n"/>
-      <c r="U46" s="20" t="n"/>
-      <c r="AC46" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-18
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2891,7 +2891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH45"/>
+  <dimension ref="A1:AH44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="9" min="1" max="1"/>
@@ -3366,7 +3366,7 @@
         <v>6</v>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3460,7 +3460,7 @@
         <v>6</v>
       </c>
       <c r="AC6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4110,7 +4110,7 @@
         <v>6</v>
       </c>
       <c r="AC14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -4273,7 +4273,7 @@
         <v>6</v>
       </c>
       <c r="AC16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -4510,7 +4510,7 @@
         <v>6</v>
       </c>
       <c r="AC19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -4750,7 +4750,7 @@
         <v>6</v>
       </c>
       <c r="AC22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -4823,7 +4823,7 @@
         <v>6</v>
       </c>
       <c r="AC23" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -4917,7 +4917,7 @@
         <v>6</v>
       </c>
       <c r="AC24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -5011,7 +5011,7 @@
         <v>6</v>
       </c>
       <c r="AC25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -5270,12 +5270,12 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C29" s="9">
@@ -5292,11 +5292,8 @@
       <c r="S29" s="20" t="n"/>
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
-      <c r="V29" t="n">
-        <v>0</v>
-      </c>
       <c r="W29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X29" t="n">
         <v>6</v>
@@ -5305,7 +5302,7 @@
         <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA29" t="n">
         <v>6</v>
@@ -5314,18 +5311,18 @@
         <v>0</v>
       </c>
       <c r="AC29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C30" s="9">
@@ -5342,32 +5339,26 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="W30" t="n">
-        <v>6</v>
-      </c>
-      <c r="X30" t="n">
-        <v>6</v>
-      </c>
       <c r="Y30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA30" t="n">
         <v>6</v>
       </c>
       <c r="AB30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC30" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
@@ -5390,30 +5381,30 @@
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
       <c r="Y31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C32" s="9">
@@ -5430,17 +5421,14 @@
       <c r="S32" s="20" t="n"/>
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
-      <c r="Y32" t="n">
-        <v>0</v>
-      </c>
       <c r="Z32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC32" t="n">
         <v>6</v>
@@ -5449,12 +5437,12 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C33" s="9">
@@ -5471,14 +5459,11 @@
       <c r="S33" s="20" t="n"/>
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
-      <c r="Z33" t="n">
-        <v>6</v>
-      </c>
       <c r="AA33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC33" t="n">
         <v>6</v>
@@ -5487,7 +5472,7 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -5510,19 +5495,19 @@
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
       <c r="AA34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB34" t="n">
         <v>0</v>
       </c>
       <c r="AC34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
@@ -5545,24 +5530,24 @@
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
       <c r="AA35" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB35" t="n">
         <v>0</v>
       </c>
       <c r="AC35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C36" s="9">
@@ -5579,20 +5564,17 @@
       <c r="S36" s="20" t="n"/>
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
-      <c r="AA36" t="n">
-        <v>0</v>
-      </c>
       <c r="AB36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
@@ -5624,7 +5606,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -5647,7 +5629,7 @@
       <c r="T38" s="20" t="n"/>
       <c r="U38" s="20" t="n"/>
       <c r="AB38" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC38" t="n">
         <v>0</v>
@@ -5656,12 +5638,12 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C39" s="9">
@@ -5678,9 +5660,6 @@
       <c r="S39" s="20" t="n"/>
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
-      <c r="AB39" t="n">
-        <v>0</v>
-      </c>
       <c r="AC39" t="n">
         <v>0</v>
       </c>
@@ -5688,7 +5667,7 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -5717,7 +5696,7 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>Space_GG</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
@@ -5746,7 +5725,7 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>Space_GG</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -5769,13 +5748,13 @@
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
       <c r="AC42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
@@ -5804,12 +5783,12 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C44" s="9">
@@ -5827,35 +5806,6 @@
       <c r="T44" s="20" t="n"/>
       <c r="U44" s="20" t="n"/>
       <c r="AC44" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>KAIZERS</t>
-        </is>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>17/05/2026</t>
-        </is>
-      </c>
-      <c r="C45" s="9">
-        <f>ROUND(AVERAGE(D45:AH45), 0)</f>
-        <v/>
-      </c>
-      <c r="K45" s="6" t="n"/>
-      <c r="L45" s="6" t="n"/>
-      <c r="N45" s="6" t="n"/>
-      <c r="O45" s="20" t="n"/>
-      <c r="P45" s="20" t="n"/>
-      <c r="Q45" s="20" t="n"/>
-      <c r="R45" s="20" t="n"/>
-      <c r="S45" s="20" t="n"/>
-      <c r="T45" s="20" t="n"/>
-      <c r="U45" s="20" t="n"/>
-      <c r="AC45" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH44"/>
+  <dimension ref="A1:AH47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -969,7 +969,7 @@
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B3" s="16" t="inlineStr">
@@ -986,20 +986,22 @@
         <v/>
       </c>
       <c r="E3" s="14" t="n">
-        <v>22000</v>
-      </c>
-      <c r="F3" s="13" t="n"/>
+        <v>47650</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G3" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H3" s="13" t="n">
-        <v>6050</v>
+        <v>10000</v>
       </c>
       <c r="I3" s="13" t="n">
-        <v>8300</v>
+        <v>10000</v>
       </c>
       <c r="J3" s="13" t="n">
-        <v>5950</v>
+        <v>10000</v>
       </c>
       <c r="K3" s="13" t="n">
         <v>10000</v>
@@ -1019,7 +1021,7 @@
     <row r="4" ht="16.5" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
@@ -1036,11 +1038,9 @@
         <v/>
       </c>
       <c r="E4" s="14" t="n">
-        <v>47650</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>4000</v>
-      </c>
+        <v>55400</v>
+      </c>
+      <c r="F4" s="13" t="n"/>
       <c r="G4" s="13" t="n">
         <v>4000</v>
       </c>
@@ -1071,12 +1071,12 @@
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C5" s="12">
@@ -1088,21 +1088,13 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>55400</v>
+        <v>5500</v>
       </c>
       <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H5" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I5" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="G5" s="13" t="n"/>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="13" t="n"/>
       <c r="K5" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1121,12 +1113,12 @@
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C6" s="12">
@@ -1138,13 +1130,19 @@
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>5500</v>
+        <v>58700</v>
       </c>
       <c r="F6" s="13" t="n"/>
       <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n"/>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="13" t="n"/>
+      <c r="H6" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="K6" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1163,7 +1161,7 @@
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
@@ -1180,7 +1178,7 @@
         <v/>
       </c>
       <c r="E7" s="14" t="n">
-        <v>58700</v>
+        <v>51200</v>
       </c>
       <c r="F7" s="13" t="n"/>
       <c r="G7" s="13" t="n"/>
@@ -1211,12 +1209,12 @@
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C8" s="12">
@@ -1228,13 +1226,11 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>51200</v>
+        <v>106725</v>
       </c>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H8" s="13" t="n"/>
       <c r="I8" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1247,7 +1243,7 @@
       <c r="L8" s="13" t="n"/>
       <c r="M8" s="13" t="n"/>
       <c r="N8" s="13" t="n"/>
-      <c r="O8" s="13" t="n"/>
+      <c r="O8" s="13" t="inlineStr"/>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="13" t="n"/>
       <c r="R8" s="13" t="n"/>
@@ -1259,12 +1255,12 @@
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C9" s="12">
@@ -1276,24 +1272,26 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>106725</v>
+        <v>109220</v>
       </c>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>3850</v>
+      </c>
       <c r="I9" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>10000</v>
+        <v>8800</v>
       </c>
       <c r="L9" s="13" t="n"/>
       <c r="M9" s="13" t="n"/>
       <c r="N9" s="13" t="n"/>
-      <c r="O9" s="13" t="inlineStr"/>
+      <c r="O9" s="13" t="n"/>
       <c r="P9" s="13" t="n"/>
       <c r="Q9" s="13" t="n"/>
       <c r="R9" s="13" t="n"/>
@@ -1305,7 +1303,7 @@
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
@@ -1322,21 +1320,21 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>109220</v>
+        <v>56300</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
       <c r="H10" s="13" t="n">
-        <v>3850</v>
+        <v>10000</v>
       </c>
       <c r="I10" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>8800</v>
+        <v>8600</v>
       </c>
       <c r="L10" s="13" t="n"/>
       <c r="M10" s="13" t="n"/>
@@ -1353,7 +1351,7 @@
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -1370,21 +1368,23 @@
         <v/>
       </c>
       <c r="E11" s="14" t="n">
-        <v>56300</v>
+        <v>27500</v>
       </c>
       <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
+      <c r="G11" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H11" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>10000</v>
+        <v>4300</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>8600</v>
+        <v>6300</v>
       </c>
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="13" t="n"/>
@@ -1393,7 +1393,7 @@
       <c r="P11" s="13" t="n"/>
       <c r="Q11" s="13" t="n"/>
       <c r="R11" s="13" t="n"/>
-      <c r="S11" s="13" t="n"/>
+      <c r="S11" s="21" t="n"/>
       <c r="T11" s="13" t="n"/>
       <c r="U11" s="13" t="n"/>
       <c r="V11" s="13" t="n"/>
@@ -1401,12 +1401,12 @@
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C12" s="12">
@@ -1418,23 +1418,17 @@
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>27500</v>
+        <v>76700</v>
       </c>
       <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H12" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4500</v>
-      </c>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
       <c r="J12" s="13" t="n">
-        <v>4300</v>
+        <v>5000</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>6300</v>
+        <v>6100</v>
       </c>
       <c r="L12" s="13" t="n"/>
       <c r="M12" s="13" t="n"/>
@@ -1451,12 +1445,12 @@
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C13" s="12">
@@ -1468,14 +1462,20 @@
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>76700</v>
+        <v>12250</v>
       </c>
       <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="13" t="n"/>
+      <c r="G13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="J13" s="13" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="K13" s="13" t="n">
         <v>6100</v>
@@ -1495,7 +1495,7 @@
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
@@ -1512,23 +1512,25 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>12250</v>
-      </c>
-      <c r="F14" s="13" t="n"/>
+        <v>33025</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G14" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>0</v>
+        <v>4850</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>6100</v>
+        <v>5050</v>
       </c>
       <c r="L14" s="13" t="n"/>
       <c r="M14" s="13" t="n"/>
@@ -1545,12 +1547,12 @@
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C15" s="12">
@@ -1562,19 +1564,25 @@
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>28225</v>
-      </c>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n"/>
+        <v>33700</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="I15" s="13" t="n">
-        <v>2000</v>
+        <v>2450</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>8000</v>
+        <v>4050</v>
       </c>
       <c r="K15" s="13" t="n">
-        <v>5100</v>
+        <v>4650</v>
       </c>
       <c r="L15" s="13" t="n"/>
       <c r="M15" s="13" t="n"/>
@@ -1591,7 +1599,7 @@
     <row r="16" ht="16.5" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
@@ -1608,25 +1616,25 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>33025</v>
+        <v>33050</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>4000</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>4000</v>
+        <v>2100</v>
       </c>
       <c r="H16" s="13" t="n">
+        <v>5800</v>
+      </c>
+      <c r="I16" s="13" t="n">
         <v>4050</v>
       </c>
-      <c r="I16" s="13" t="n">
-        <v>4850</v>
-      </c>
       <c r="J16" s="13" t="n">
-        <v>4000</v>
+        <v>4350</v>
       </c>
       <c r="K16" s="13" t="n">
-        <v>5050</v>
+        <v>4600</v>
       </c>
       <c r="L16" s="13" t="n"/>
       <c r="M16" s="13" t="n"/>
@@ -1643,12 +1651,12 @@
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C17" s="12">
@@ -1660,25 +1668,19 @@
         <v/>
       </c>
       <c r="E17" s="14" t="n">
-        <v>33700</v>
-      </c>
-      <c r="F17" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H17" s="13" t="n">
-        <v>10000</v>
-      </c>
+        <v>44550</v>
+      </c>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
       <c r="I17" s="13" t="n">
-        <v>2450</v>
+        <v>4300</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>4050</v>
+        <v>4100</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>4650</v>
+        <v>4200</v>
       </c>
       <c r="L17" s="13" t="n"/>
       <c r="M17" s="13" t="n"/>
@@ -1695,7 +1697,7 @@
     <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
@@ -1712,25 +1714,25 @@
         <v/>
       </c>
       <c r="E18" s="14" t="n">
-        <v>33050</v>
+        <v>32200</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>4000</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>2100</v>
+        <v>4000</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>5800</v>
+        <v>4100</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>4050</v>
+        <v>4400</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>4350</v>
+        <v>4700</v>
       </c>
       <c r="K18" s="13" t="n">
-        <v>4600</v>
+        <v>4150</v>
       </c>
       <c r="L18" s="13" t="n"/>
       <c r="M18" s="13" t="n"/>
@@ -1747,12 +1749,12 @@
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C19" s="12">
@@ -1764,17 +1766,21 @@
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>23750</v>
+        <v>123800</v>
       </c>
       <c r="F19" s="13" t="n"/>
       <c r="G19" s="13" t="n"/>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
+      <c r="H19" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>4100</v>
+      </c>
       <c r="J19" s="13" t="n">
-        <v>4300</v>
+        <v>4000</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>4200</v>
+        <v>4100</v>
       </c>
       <c r="L19" s="13" t="n"/>
       <c r="M19" s="13" t="n"/>
@@ -1791,12 +1797,12 @@
     <row r="20" ht="16.5" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C20" s="12">
@@ -1808,19 +1814,21 @@
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>44550</v>
+        <v>41000</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="H20" s="13" t="n">
+        <v>1200</v>
+      </c>
       <c r="I20" s="13" t="n">
-        <v>4300</v>
+        <v>4000</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>4100</v>
+        <v>150</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>4200</v>
+        <v>4050</v>
       </c>
       <c r="L20" s="13" t="n"/>
       <c r="M20" s="13" t="n"/>
@@ -1837,7 +1845,7 @@
     <row r="21" ht="16.5" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
@@ -1854,25 +1862,21 @@
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>32200</v>
-      </c>
-      <c r="F21" s="13" t="n">
+        <v>29350</v>
+      </c>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="K21" s="13" t="n">
         <v>4000</v>
-      </c>
-      <c r="G21" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H21" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>4400</v>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>4700</v>
-      </c>
-      <c r="K21" s="13" t="n">
-        <v>4150</v>
       </c>
       <c r="L21" s="13" t="n"/>
       <c r="M21" s="13" t="n"/>
@@ -1889,12 +1893,12 @@
     <row r="22" ht="16.5" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C22" s="12">
@@ -1906,21 +1910,25 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>123800</v>
-      </c>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="13" t="n"/>
+        <v>39900</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H22" s="13" t="n">
         <v>4050</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>4100</v>
+        <v>5600</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>4000</v>
+        <v>1300</v>
       </c>
       <c r="K22" s="13" t="n">
-        <v>4100</v>
+        <v>3100</v>
       </c>
       <c r="L22" s="13" t="n"/>
       <c r="M22" s="13" t="n"/>
@@ -1937,7 +1945,7 @@
     <row r="23" ht="16.5" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
@@ -1954,21 +1962,21 @@
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>41000</v>
+        <v>31825</v>
       </c>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
       <c r="H23" s="13" t="n">
-        <v>1200</v>
+        <v>3650</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>4000</v>
+        <v>7600</v>
       </c>
       <c r="J23" s="13" t="n">
-        <v>150</v>
+        <v>3150</v>
       </c>
       <c r="K23" s="13" t="n">
-        <v>4050</v>
+        <v>3000</v>
       </c>
       <c r="L23" s="13" t="n"/>
       <c r="M23" s="13" t="n"/>
@@ -1985,12 +1993,12 @@
     <row r="24" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C24" s="12">
@@ -2002,21 +2010,19 @@
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>29350</v>
+        <v>75000</v>
       </c>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H24" s="13" t="n"/>
       <c r="I24" s="13" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="J24" s="13" t="n">
-        <v>4050</v>
+        <v>950</v>
       </c>
       <c r="K24" s="13" t="n">
-        <v>4000</v>
+        <v>1400</v>
       </c>
       <c r="L24" s="13" t="n"/>
       <c r="M24" s="13" t="n"/>
@@ -2033,12 +2039,12 @@
     <row r="25" ht="16.5" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C25" s="12">
@@ -2050,25 +2056,19 @@
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>39900</v>
-      </c>
-      <c r="F25" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G25" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H25" s="13" t="n">
-        <v>4050</v>
-      </c>
+        <v>6800</v>
+      </c>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
       <c r="I25" s="13" t="n">
-        <v>5600</v>
+        <v>4150</v>
       </c>
       <c r="J25" s="13" t="n">
-        <v>1300</v>
+        <v>2650</v>
       </c>
       <c r="K25" s="13" t="n">
-        <v>3100</v>
+        <v>1050</v>
       </c>
       <c r="L25" s="13" t="n"/>
       <c r="M25" s="13" t="n"/>
@@ -2077,7 +2077,7 @@
       <c r="P25" s="13" t="n"/>
       <c r="Q25" s="13" t="n"/>
       <c r="R25" s="13" t="n"/>
-      <c r="S25" s="21" t="n"/>
+      <c r="S25" s="13" t="n"/>
       <c r="T25" s="13" t="n"/>
       <c r="U25" s="13" t="n"/>
       <c r="V25" s="13" t="n"/>
@@ -2085,12 +2085,12 @@
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C26" s="12">
@@ -2102,21 +2102,15 @@
         <v/>
       </c>
       <c r="E26" s="14" t="n">
-        <v>31825</v>
+        <v>18000</v>
       </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
-      <c r="H26" s="13" t="n">
-        <v>3650</v>
-      </c>
-      <c r="I26" s="13" t="n">
-        <v>7600</v>
-      </c>
-      <c r="J26" s="13" t="n">
-        <v>3150</v>
-      </c>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
       <c r="K26" s="13" t="n">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="n"/>
@@ -2125,7 +2119,7 @@
       <c r="P26" s="13" t="n"/>
       <c r="Q26" s="13" t="n"/>
       <c r="R26" s="13" t="n"/>
-      <c r="S26" s="21" t="n"/>
+      <c r="S26" s="13" t="n"/>
       <c r="T26" s="13" t="n"/>
       <c r="U26" s="13" t="n"/>
       <c r="V26" s="13" t="n"/>
@@ -2133,12 +2127,12 @@
     <row r="27" ht="16.5" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C27" s="12">
@@ -2150,19 +2144,21 @@
         <v/>
       </c>
       <c r="E27" s="14" t="n">
-        <v>75000</v>
+        <v>15150</v>
       </c>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
+      <c r="H27" s="13" t="n">
+        <v>500</v>
+      </c>
       <c r="I27" s="13" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="J27" s="13" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="K27" s="13" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="L27" s="13" t="n"/>
       <c r="M27" s="13" t="n"/>
@@ -2171,7 +2167,7 @@
       <c r="P27" s="13" t="n"/>
       <c r="Q27" s="13" t="n"/>
       <c r="R27" s="13" t="n"/>
-      <c r="S27" s="21" t="n"/>
+      <c r="S27" s="13" t="n"/>
       <c r="T27" s="13" t="n"/>
       <c r="U27" s="13" t="n"/>
       <c r="V27" s="13" t="n"/>
@@ -2179,12 +2175,12 @@
     <row r="28" ht="16.5" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C28" s="12">
@@ -2196,20 +2192,14 @@
         <v/>
       </c>
       <c r="E28" s="14" t="n">
-        <v>6800</v>
+        <v>13125</v>
       </c>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
       <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n">
-        <v>4150</v>
-      </c>
-      <c r="J28" s="13" t="n">
-        <v>2650</v>
-      </c>
-      <c r="K28" s="13" t="n">
-        <v>1050</v>
-      </c>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
       <c r="L28" s="13" t="n"/>
       <c r="M28" s="13" t="n"/>
       <c r="N28" s="13" t="n"/>
@@ -2225,12 +2215,12 @@
     <row r="29" ht="16.5" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C29" s="12">
@@ -2242,16 +2232,14 @@
         <v/>
       </c>
       <c r="E29" s="14" t="n">
-        <v>18000</v>
+        <v>11250</v>
       </c>
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="13" t="n"/>
       <c r="H29" s="13" t="n"/>
       <c r="I29" s="13" t="n"/>
       <c r="J29" s="13" t="n"/>
-      <c r="K29" s="13" t="n">
-        <v>600</v>
-      </c>
+      <c r="K29" s="13" t="n"/>
       <c r="L29" s="13" t="n"/>
       <c r="M29" s="13" t="n"/>
       <c r="N29" s="13" t="n"/>
@@ -2267,12 +2255,12 @@
     <row r="30" ht="16.5" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C30" s="12">
@@ -2284,22 +2272,14 @@
         <v/>
       </c>
       <c r="E30" s="14" t="n">
-        <v>15150</v>
+        <v>40640</v>
       </c>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="I30" s="13" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J30" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
+      <c r="J30" s="13" t="n"/>
+      <c r="K30" s="13" t="n"/>
       <c r="L30" s="13" t="n"/>
       <c r="M30" s="13" t="n"/>
       <c r="N30" s="13" t="n"/>
@@ -2315,12 +2295,12 @@
     <row r="31" ht="16.5" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C31" s="12">
@@ -2332,20 +2312,14 @@
         <v/>
       </c>
       <c r="E31" s="14" t="n">
-        <v>69000</v>
+        <v>56200</v>
       </c>
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="13" t="n"/>
       <c r="H31" s="13" t="n"/>
-      <c r="I31" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J31" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K31" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n"/>
+      <c r="K31" s="13" t="n"/>
       <c r="L31" s="13" t="n"/>
       <c r="M31" s="13" t="n"/>
       <c r="N31" s="13" t="n"/>
@@ -2361,12 +2335,12 @@
     <row r="32" ht="16.5" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C32" s="12">
@@ -2378,7 +2352,7 @@
         <v/>
       </c>
       <c r="E32" s="14" t="n">
-        <v>43650</v>
+        <v>39650</v>
       </c>
       <c r="F32" s="13" t="n"/>
       <c r="G32" s="13" t="n"/>
@@ -2401,12 +2375,12 @@
     <row r="33" ht="16.5" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C33" s="12">
@@ -2418,7 +2392,7 @@
         <v/>
       </c>
       <c r="E33" s="14" t="n">
-        <v>13125</v>
+        <v>42850</v>
       </c>
       <c r="F33" s="13" t="n"/>
       <c r="G33" s="13" t="n"/>
@@ -2441,12 +2415,12 @@
     <row r="34" ht="16.5" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C34" s="12">
@@ -2458,7 +2432,7 @@
         <v/>
       </c>
       <c r="E34" s="14" t="n">
-        <v>11250</v>
+        <v>56865</v>
       </c>
       <c r="F34" s="13" t="n"/>
       <c r="G34" s="13" t="n"/>
@@ -2481,12 +2455,12 @@
     <row r="35" ht="16.5" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C35" s="12">
@@ -2498,7 +2472,7 @@
         <v/>
       </c>
       <c r="E35" s="14" t="n">
-        <v>40640</v>
+        <v>25810</v>
       </c>
       <c r="F35" s="13" t="n"/>
       <c r="G35" s="13" t="n"/>
@@ -2521,7 +2495,7 @@
     <row r="36" ht="16.5" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>nanni</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B36" s="16" t="inlineStr">
@@ -2538,7 +2512,7 @@
         <v/>
       </c>
       <c r="E36" s="14" t="n">
-        <v>69525</v>
+        <v>110325</v>
       </c>
       <c r="F36" s="13" t="n"/>
       <c r="G36" s="13" t="n"/>
@@ -2561,7 +2535,7 @@
     <row r="37" ht="16.5" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
@@ -2578,7 +2552,7 @@
         <v/>
       </c>
       <c r="E37" s="14" t="n">
-        <v>56200</v>
+        <v>33210</v>
       </c>
       <c r="F37" s="13" t="n"/>
       <c r="G37" s="13" t="n"/>
@@ -2601,12 +2575,12 @@
     <row r="38" ht="16.5" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>DJ Tony</t>
+          <t>Space_GG</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C38" s="12">
@@ -2618,7 +2592,7 @@
         <v/>
       </c>
       <c r="E38" s="14" t="n">
-        <v>14060</v>
+        <v>45325</v>
       </c>
       <c r="F38" s="13" t="n"/>
       <c r="G38" s="13" t="n"/>
@@ -2641,12 +2615,12 @@
     <row r="39" ht="16.5" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C39" s="12">
@@ -2658,7 +2632,7 @@
         <v/>
       </c>
       <c r="E39" s="14" t="n">
-        <v>39650</v>
+        <v>113225</v>
       </c>
       <c r="F39" s="13" t="n"/>
       <c r="G39" s="13" t="n"/>
@@ -2681,12 +2655,12 @@
     <row r="40" ht="16.5" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C40" s="12">
@@ -2698,7 +2672,7 @@
         <v/>
       </c>
       <c r="E40" s="14" t="n">
-        <v>42850</v>
+        <v>0</v>
       </c>
       <c r="F40" s="13" t="n"/>
       <c r="G40" s="13" t="n"/>
@@ -2721,12 +2695,12 @@
     <row r="41" ht="16.5" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C41" s="12">
@@ -2738,7 +2712,7 @@
         <v/>
       </c>
       <c r="E41" s="14" t="n">
-        <v>56865</v>
+        <v>36875</v>
       </c>
       <c r="F41" s="13" t="n"/>
       <c r="G41" s="13" t="n"/>
@@ -2761,12 +2735,12 @@
     <row r="42" ht="16.5" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>Frost Walker</t>
         </is>
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C42" s="12">
@@ -2778,7 +2752,7 @@
         <v/>
       </c>
       <c r="E42" s="14" t="n">
-        <v>25810</v>
+        <v>30615</v>
       </c>
       <c r="F42" s="13" t="n"/>
       <c r="G42" s="13" t="n"/>
@@ -2801,12 +2775,12 @@
     <row r="43" ht="16.5" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C43" s="12">
@@ -2818,7 +2792,7 @@
         <v/>
       </c>
       <c r="E43" s="14" t="n">
-        <v>110325</v>
+        <v>6950</v>
       </c>
       <c r="F43" s="13" t="n"/>
       <c r="G43" s="13" t="n"/>
@@ -2841,12 +2815,12 @@
     <row r="44" ht="16.5" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C44" s="12">
@@ -2858,7 +2832,7 @@
         <v/>
       </c>
       <c r="E44" s="14" t="n">
-        <v>33210</v>
+        <v>29825</v>
       </c>
       <c r="F44" s="13" t="n"/>
       <c r="G44" s="13" t="n"/>
@@ -2877,6 +2851,126 @@
       <c r="T44" s="13" t="n"/>
       <c r="U44" s="13" t="n"/>
       <c r="V44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>roberto</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="12">
+        <f>ROUND(AVERAGE(F45:AI45), 0)</f>
+        <v/>
+      </c>
+      <c r="D45" s="1">
+        <f>SUM(F45:AI45)</f>
+        <v/>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>39900</v>
+      </c>
+      <c r="F45" s="13" t="n"/>
+      <c r="G45" s="13" t="n"/>
+      <c r="H45" s="13" t="n"/>
+      <c r="I45" s="13" t="n"/>
+      <c r="J45" s="13" t="n"/>
+      <c r="K45" s="13" t="n"/>
+      <c r="L45" s="13" t="n"/>
+      <c r="M45" s="13" t="n"/>
+      <c r="N45" s="13" t="n"/>
+      <c r="O45" s="13" t="n"/>
+      <c r="P45" s="13" t="n"/>
+      <c r="Q45" s="13" t="n"/>
+      <c r="R45" s="13" t="n"/>
+      <c r="S45" s="13" t="n"/>
+      <c r="T45" s="13" t="n"/>
+      <c r="U45" s="13" t="n"/>
+      <c r="V45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>escanor</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="12">
+        <f>ROUND(AVERAGE(F46:AI46), 0)</f>
+        <v/>
+      </c>
+      <c r="D46" s="1">
+        <f>SUM(F46:AI46)</f>
+        <v/>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>33800</v>
+      </c>
+      <c r="F46" s="13" t="n"/>
+      <c r="G46" s="13" t="n"/>
+      <c r="H46" s="13" t="n"/>
+      <c r="I46" s="13" t="n"/>
+      <c r="J46" s="13" t="n"/>
+      <c r="K46" s="13" t="n"/>
+      <c r="L46" s="13" t="n"/>
+      <c r="M46" s="13" t="n"/>
+      <c r="N46" s="13" t="n"/>
+      <c r="O46" s="13" t="n"/>
+      <c r="P46" s="13" t="n"/>
+      <c r="Q46" s="13" t="n"/>
+      <c r="R46" s="13" t="n"/>
+      <c r="S46" s="13" t="n"/>
+      <c r="T46" s="13" t="n"/>
+      <c r="U46" s="13" t="n"/>
+      <c r="V46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>fre 2000</t>
+        </is>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="12">
+        <f>ROUND(AVERAGE(F47:AI47), 0)</f>
+        <v/>
+      </c>
+      <c r="D47" s="1">
+        <f>SUM(F47:AI47)</f>
+        <v/>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F47" s="13" t="n"/>
+      <c r="G47" s="13" t="n"/>
+      <c r="H47" s="13" t="n"/>
+      <c r="I47" s="13" t="n"/>
+      <c r="J47" s="13" t="n"/>
+      <c r="K47" s="13" t="n"/>
+      <c r="L47" s="13" t="n"/>
+      <c r="M47" s="13" t="n"/>
+      <c r="N47" s="13" t="n"/>
+      <c r="O47" s="13" t="n"/>
+      <c r="P47" s="13" t="n"/>
+      <c r="Q47" s="13" t="n"/>
+      <c r="R47" s="13" t="n"/>
+      <c r="S47" s="13" t="n"/>
+      <c r="T47" s="13" t="n"/>
+      <c r="U47" s="13" t="n"/>
+      <c r="V47" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AN1"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -952,7 +952,7 @@
         <v/>
       </c>
       <c r="E2" s="14" t="n">
-        <v>31350</v>
+        <v>51700</v>
       </c>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
@@ -964,7 +964,9 @@
       <c r="K2" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L2" s="13" t="n"/>
+      <c r="L2" s="13" t="n">
+        <v>10000</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
@@ -986,7 +988,7 @@
         <v/>
       </c>
       <c r="E3" s="14" t="n">
-        <v>47650</v>
+        <v>68200</v>
       </c>
       <c r="F3" s="13" t="n">
         <v>4000</v>
@@ -1006,7 +1008,9 @@
       <c r="K3" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L3" s="13" t="n"/>
+      <c r="L3" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M3" s="13" t="n"/>
       <c r="N3" s="13" t="n"/>
       <c r="O3" s="13" t="n"/>
@@ -1038,7 +1042,7 @@
         <v/>
       </c>
       <c r="E4" s="14" t="n">
-        <v>55400</v>
+        <v>75500</v>
       </c>
       <c r="F4" s="13" t="n"/>
       <c r="G4" s="13" t="n">
@@ -1056,7 +1060,9 @@
       <c r="K4" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L4" s="13" t="n"/>
+      <c r="L4" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M4" s="13" t="n"/>
       <c r="N4" s="13" t="n"/>
       <c r="O4" s="13" t="n"/>
@@ -1088,7 +1094,7 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>5500</v>
+        <v>25650</v>
       </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
@@ -1098,7 +1104,9 @@
       <c r="K5" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L5" s="13" t="n"/>
+      <c r="L5" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M5" s="13" t="n"/>
       <c r="N5" s="13" t="n"/>
       <c r="O5" s="13" t="n"/>
@@ -1130,7 +1138,7 @@
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>58700</v>
+        <v>80450</v>
       </c>
       <c r="F6" s="13" t="n"/>
       <c r="G6" s="13" t="n"/>
@@ -1146,7 +1154,9 @@
       <c r="K6" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L6" s="13" t="n"/>
+      <c r="L6" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M6" s="13" t="n"/>
       <c r="N6" s="13" t="n"/>
       <c r="O6" s="13" t="n"/>
@@ -1178,7 +1188,7 @@
         <v/>
       </c>
       <c r="E7" s="14" t="n">
-        <v>51200</v>
+        <v>72050</v>
       </c>
       <c r="F7" s="13" t="n"/>
       <c r="G7" s="13" t="n"/>
@@ -1194,7 +1204,9 @@
       <c r="K7" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L7" s="13" t="n"/>
+      <c r="L7" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M7" s="13" t="n"/>
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="n"/>
@@ -1226,7 +1238,7 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>106725</v>
+        <v>127225</v>
       </c>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
@@ -1240,7 +1252,9 @@
       <c r="K8" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="L8" s="13" t="n"/>
+      <c r="L8" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M8" s="13" t="n"/>
       <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="inlineStr"/>
@@ -1272,7 +1286,7 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>109220</v>
+        <v>121370</v>
       </c>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n"/>
@@ -1288,7 +1302,9 @@
       <c r="K9" s="13" t="n">
         <v>8800</v>
       </c>
-      <c r="L9" s="13" t="n"/>
+      <c r="L9" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M9" s="13" t="n"/>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
@@ -1320,7 +1336,7 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>56300</v>
+        <v>70450</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
@@ -1336,7 +1352,9 @@
       <c r="K10" s="13" t="n">
         <v>8600</v>
       </c>
-      <c r="L10" s="13" t="n"/>
+      <c r="L10" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M10" s="13" t="n"/>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
@@ -1368,7 +1386,7 @@
         <v/>
       </c>
       <c r="E11" s="14" t="n">
-        <v>27500</v>
+        <v>38200</v>
       </c>
       <c r="F11" s="13" t="n"/>
       <c r="G11" s="13" t="n">
@@ -1386,7 +1404,9 @@
       <c r="K11" s="13" t="n">
         <v>6300</v>
       </c>
-      <c r="L11" s="13" t="n"/>
+      <c r="L11" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M11" s="13" t="n"/>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
@@ -1418,7 +1438,7 @@
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>76700</v>
+        <v>87650</v>
       </c>
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
@@ -1430,7 +1450,9 @@
       <c r="K12" s="13" t="n">
         <v>6100</v>
       </c>
-      <c r="L12" s="13" t="n"/>
+      <c r="L12" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M12" s="13" t="n"/>
       <c r="N12" s="13" t="n"/>
       <c r="O12" s="13" t="n"/>
@@ -1462,7 +1484,7 @@
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>12250</v>
+        <v>18350</v>
       </c>
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n">
@@ -1480,7 +1502,9 @@
       <c r="K13" s="13" t="n">
         <v>6100</v>
       </c>
-      <c r="L13" s="13" t="n"/>
+      <c r="L13" s="13" t="n">
+        <v>6100</v>
+      </c>
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
@@ -1512,7 +1536,7 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>33025</v>
+        <v>38075</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>4000</v>
@@ -1532,7 +1556,9 @@
       <c r="K14" s="13" t="n">
         <v>5050</v>
       </c>
-      <c r="L14" s="13" t="n"/>
+      <c r="L14" s="13" t="n">
+        <v>5050</v>
+      </c>
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="13" t="n"/>
       <c r="O14" s="13" t="n"/>
@@ -1564,7 +1590,7 @@
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>33700</v>
+        <v>46700</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>4000</v>
@@ -1584,7 +1610,9 @@
       <c r="K15" s="13" t="n">
         <v>4650</v>
       </c>
-      <c r="L15" s="13" t="n"/>
+      <c r="L15" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
@@ -1616,7 +1644,7 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>33050</v>
+        <v>41650</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>4000</v>
@@ -1636,7 +1664,9 @@
       <c r="K16" s="13" t="n">
         <v>4600</v>
       </c>
-      <c r="L16" s="13" t="n"/>
+      <c r="L16" s="13" t="n">
+        <v>8600</v>
+      </c>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="n"/>
@@ -1668,7 +1698,7 @@
         <v/>
       </c>
       <c r="E17" s="14" t="n">
-        <v>44550</v>
+        <v>52850</v>
       </c>
       <c r="F17" s="13" t="n"/>
       <c r="G17" s="13" t="n"/>
@@ -1682,7 +1712,9 @@
       <c r="K17" s="13" t="n">
         <v>4200</v>
       </c>
-      <c r="L17" s="13" t="n"/>
+      <c r="L17" s="13" t="n">
+        <v>8300</v>
+      </c>
       <c r="M17" s="13" t="n"/>
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="13" t="n"/>
@@ -1714,7 +1746,7 @@
         <v/>
       </c>
       <c r="E18" s="14" t="n">
-        <v>32200</v>
+        <v>40550</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>4000</v>
@@ -1734,7 +1766,9 @@
       <c r="K18" s="13" t="n">
         <v>4150</v>
       </c>
-      <c r="L18" s="13" t="n"/>
+      <c r="L18" s="13" t="n">
+        <v>8350</v>
+      </c>
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="13" t="n"/>
       <c r="O18" s="13" t="n"/>
@@ -1766,7 +1800,7 @@
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>123800</v>
+        <v>133100</v>
       </c>
       <c r="F19" s="13" t="n"/>
       <c r="G19" s="13" t="n"/>
@@ -1782,7 +1816,9 @@
       <c r="K19" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="L19" s="13" t="n"/>
+      <c r="L19" s="13" t="n">
+        <v>9300</v>
+      </c>
       <c r="M19" s="13" t="n"/>
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="13" t="n"/>
@@ -1814,7 +1850,7 @@
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>41000</v>
+        <v>47550</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
@@ -1830,7 +1866,9 @@
       <c r="K20" s="13" t="n">
         <v>4050</v>
       </c>
-      <c r="L20" s="13" t="n"/>
+      <c r="L20" s="13" t="n">
+        <v>6550</v>
+      </c>
       <c r="M20" s="13" t="n"/>
       <c r="N20" s="13" t="n"/>
       <c r="O20" s="13" t="n"/>
@@ -1862,7 +1900,7 @@
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>29350</v>
+        <v>37400</v>
       </c>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
@@ -1878,7 +1916,9 @@
       <c r="K21" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="L21" s="13" t="n"/>
+      <c r="L21" s="13" t="n">
+        <v>8050</v>
+      </c>
       <c r="M21" s="13" t="n"/>
       <c r="N21" s="13" t="n"/>
       <c r="O21" s="13" t="n"/>
@@ -1910,7 +1950,7 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>39900</v>
+        <v>43450</v>
       </c>
       <c r="F22" s="13" t="n">
         <v>4000</v>
@@ -1930,7 +1970,9 @@
       <c r="K22" s="13" t="n">
         <v>3100</v>
       </c>
-      <c r="L22" s="13" t="n"/>
+      <c r="L22" s="13" t="n">
+        <v>3550</v>
+      </c>
       <c r="M22" s="13" t="n"/>
       <c r="N22" s="13" t="n"/>
       <c r="O22" s="13" t="n"/>
@@ -1962,7 +2004,7 @@
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>31825</v>
+        <v>37125</v>
       </c>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
@@ -1978,7 +2020,9 @@
       <c r="K23" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="L23" s="13" t="n"/>
+      <c r="L23" s="13" t="n">
+        <v>5300</v>
+      </c>
       <c r="M23" s="13" t="n"/>
       <c r="N23" s="13" t="n"/>
       <c r="O23" s="13" t="n"/>
@@ -2010,7 +2054,7 @@
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>75000</v>
+        <v>76400</v>
       </c>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
@@ -2024,7 +2068,9 @@
       <c r="K24" s="13" t="n">
         <v>1400</v>
       </c>
-      <c r="L24" s="13" t="n"/>
+      <c r="L24" s="13" t="n">
+        <v>1400</v>
+      </c>
       <c r="M24" s="13" t="n"/>
       <c r="N24" s="13" t="n"/>
       <c r="O24" s="13" t="n"/>
@@ -2056,7 +2102,7 @@
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>6800</v>
+        <v>7850</v>
       </c>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
@@ -2070,7 +2116,9 @@
       <c r="K25" s="13" t="n">
         <v>1050</v>
       </c>
-      <c r="L25" s="13" t="n"/>
+      <c r="L25" s="13" t="n">
+        <v>1050</v>
+      </c>
       <c r="M25" s="13" t="n"/>
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="13" t="n"/>
@@ -2102,7 +2150,7 @@
         <v/>
       </c>
       <c r="E26" s="14" t="n">
-        <v>18000</v>
+        <v>18850</v>
       </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
@@ -2112,7 +2160,9 @@
       <c r="K26" s="13" t="n">
         <v>600</v>
       </c>
-      <c r="L26" s="13" t="n"/>
+      <c r="L26" s="13" t="n">
+        <v>850</v>
+      </c>
       <c r="M26" s="13" t="n"/>
       <c r="N26" s="13" t="n"/>
       <c r="O26" s="13" t="n"/>
@@ -2144,7 +2194,7 @@
         <v/>
       </c>
       <c r="E27" s="14" t="n">
-        <v>15150</v>
+        <v>17200</v>
       </c>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
@@ -2160,7 +2210,9 @@
       <c r="K27" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L27" s="13" t="n"/>
+      <c r="L27" s="13" t="n">
+        <v>2050</v>
+      </c>
       <c r="M27" s="13" t="n"/>
       <c r="N27" s="13" t="n"/>
       <c r="O27" s="13" t="n"/>
@@ -2192,7 +2244,7 @@
         <v/>
       </c>
       <c r="E28" s="14" t="n">
-        <v>13125</v>
+        <v>13725</v>
       </c>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
@@ -2200,7 +2252,9 @@
       <c r="I28" s="13" t="n"/>
       <c r="J28" s="13" t="n"/>
       <c r="K28" s="13" t="n"/>
-      <c r="L28" s="13" t="n"/>
+      <c r="L28" s="13" t="n">
+        <v>600</v>
+      </c>
       <c r="M28" s="13" t="n"/>
       <c r="N28" s="13" t="n"/>
       <c r="O28" s="13" t="n"/>
@@ -2232,7 +2286,7 @@
         <v/>
       </c>
       <c r="E29" s="14" t="n">
-        <v>11250</v>
+        <v>11400</v>
       </c>
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="13" t="n"/>
@@ -2240,7 +2294,9 @@
       <c r="I29" s="13" t="n"/>
       <c r="J29" s="13" t="n"/>
       <c r="K29" s="13" t="n"/>
-      <c r="L29" s="13" t="n"/>
+      <c r="L29" s="13" t="n">
+        <v>150</v>
+      </c>
       <c r="M29" s="13" t="n"/>
       <c r="N29" s="13" t="n"/>
       <c r="O29" s="13" t="n"/>
@@ -2272,7 +2328,7 @@
         <v/>
       </c>
       <c r="E30" s="14" t="n">
-        <v>40640</v>
+        <v>46540</v>
       </c>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
@@ -2280,7 +2336,9 @@
       <c r="I30" s="13" t="n"/>
       <c r="J30" s="13" t="n"/>
       <c r="K30" s="13" t="n"/>
-      <c r="L30" s="13" t="n"/>
+      <c r="L30" s="13" t="n">
+        <v>5900</v>
+      </c>
       <c r="M30" s="13" t="n"/>
       <c r="N30" s="13" t="n"/>
       <c r="O30" s="13" t="n"/>
@@ -2320,7 +2378,9 @@
       <c r="I31" s="13" t="n"/>
       <c r="J31" s="13" t="n"/>
       <c r="K31" s="13" t="n"/>
-      <c r="L31" s="13" t="n"/>
+      <c r="L31" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M31" s="13" t="n"/>
       <c r="N31" s="13" t="n"/>
       <c r="O31" s="13" t="n"/>
@@ -2360,7 +2420,9 @@
       <c r="I32" s="13" t="n"/>
       <c r="J32" s="13" t="n"/>
       <c r="K32" s="13" t="n"/>
-      <c r="L32" s="13" t="n"/>
+      <c r="L32" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M32" s="13" t="n"/>
       <c r="N32" s="13" t="n"/>
       <c r="O32" s="13" t="n"/>
@@ -2400,7 +2462,9 @@
       <c r="I33" s="13" t="n"/>
       <c r="J33" s="13" t="n"/>
       <c r="K33" s="13" t="n"/>
-      <c r="L33" s="13" t="n"/>
+      <c r="L33" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M33" s="13" t="n"/>
       <c r="N33" s="13" t="n"/>
       <c r="O33" s="13" t="n"/>
@@ -2440,7 +2504,9 @@
       <c r="I34" s="13" t="n"/>
       <c r="J34" s="13" t="n"/>
       <c r="K34" s="13" t="n"/>
-      <c r="L34" s="13" t="n"/>
+      <c r="L34" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M34" s="13" t="n"/>
       <c r="N34" s="13" t="n"/>
       <c r="O34" s="13" t="n"/>
@@ -2480,7 +2546,9 @@
       <c r="I35" s="13" t="n"/>
       <c r="J35" s="13" t="n"/>
       <c r="K35" s="13" t="n"/>
-      <c r="L35" s="13" t="n"/>
+      <c r="L35" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M35" s="13" t="n"/>
       <c r="N35" s="13" t="n"/>
       <c r="O35" s="13" t="n"/>
@@ -2520,7 +2588,9 @@
       <c r="I36" s="13" t="n"/>
       <c r="J36" s="13" t="n"/>
       <c r="K36" s="13" t="n"/>
-      <c r="L36" s="13" t="n"/>
+      <c r="L36" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M36" s="13" t="n"/>
       <c r="N36" s="13" t="n"/>
       <c r="O36" s="13" t="n"/>
@@ -2560,7 +2630,9 @@
       <c r="I37" s="13" t="n"/>
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
-      <c r="L37" s="13" t="n"/>
+      <c r="L37" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M37" s="13" t="n"/>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
@@ -2600,7 +2672,9 @@
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
+      <c r="L38" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M38" s="13" t="n"/>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
@@ -2640,7 +2714,9 @@
       <c r="I39" s="13" t="n"/>
       <c r="J39" s="13" t="n"/>
       <c r="K39" s="13" t="n"/>
-      <c r="L39" s="13" t="n"/>
+      <c r="L39" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M39" s="13" t="n"/>
       <c r="N39" s="13" t="n"/>
       <c r="O39" s="13" t="n"/>
@@ -2680,7 +2756,9 @@
       <c r="I40" s="13" t="n"/>
       <c r="J40" s="13" t="n"/>
       <c r="K40" s="13" t="n"/>
-      <c r="L40" s="13" t="n"/>
+      <c r="L40" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M40" s="13" t="n"/>
       <c r="N40" s="13" t="n"/>
       <c r="O40" s="13" t="n"/>
@@ -2720,7 +2798,9 @@
       <c r="I41" s="13" t="n"/>
       <c r="J41" s="13" t="n"/>
       <c r="K41" s="13" t="n"/>
-      <c r="L41" s="13" t="n"/>
+      <c r="L41" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M41" s="13" t="n"/>
       <c r="N41" s="13" t="n"/>
       <c r="O41" s="13" t="n"/>
@@ -2760,7 +2840,9 @@
       <c r="I42" s="13" t="n"/>
       <c r="J42" s="13" t="n"/>
       <c r="K42" s="13" t="n"/>
-      <c r="L42" s="13" t="n"/>
+      <c r="L42" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M42" s="13" t="n"/>
       <c r="N42" s="13" t="n"/>
       <c r="O42" s="13" t="n"/>
@@ -2800,7 +2882,9 @@
       <c r="I43" s="13" t="n"/>
       <c r="J43" s="13" t="n"/>
       <c r="K43" s="13" t="n"/>
-      <c r="L43" s="13" t="n"/>
+      <c r="L43" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M43" s="13" t="n"/>
       <c r="N43" s="13" t="n"/>
       <c r="O43" s="13" t="n"/>
@@ -2840,7 +2924,9 @@
       <c r="I44" s="13" t="n"/>
       <c r="J44" s="13" t="n"/>
       <c r="K44" s="13" t="n"/>
-      <c r="L44" s="13" t="n"/>
+      <c r="L44" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M44" s="13" t="n"/>
       <c r="N44" s="13" t="n"/>
       <c r="O44" s="13" t="n"/>
@@ -2880,7 +2966,9 @@
       <c r="I45" s="13" t="n"/>
       <c r="J45" s="13" t="n"/>
       <c r="K45" s="13" t="n"/>
-      <c r="L45" s="13" t="n"/>
+      <c r="L45" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M45" s="13" t="n"/>
       <c r="N45" s="13" t="n"/>
       <c r="O45" s="13" t="n"/>
@@ -2920,7 +3008,9 @@
       <c r="I46" s="13" t="n"/>
       <c r="J46" s="13" t="n"/>
       <c r="K46" s="13" t="n"/>
-      <c r="L46" s="13" t="n"/>
+      <c r="L46" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M46" s="13" t="n"/>
       <c r="N46" s="13" t="n"/>
       <c r="O46" s="13" t="n"/>
@@ -2960,7 +3050,9 @@
       <c r="I47" s="13" t="n"/>
       <c r="J47" s="13" t="n"/>
       <c r="K47" s="13" t="n"/>
-      <c r="L47" s="13" t="n"/>
+      <c r="L47" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M47" s="13" t="n"/>
       <c r="N47" s="13" t="n"/>
       <c r="O47" s="13" t="n"/>
@@ -3000,7 +3092,9 @@
       <c r="I48" s="13" t="n"/>
       <c r="J48" s="13" t="n"/>
       <c r="K48" s="13" t="n"/>
-      <c r="L48" s="13" t="n"/>
+      <c r="L48" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M48" s="13" t="n"/>
       <c r="N48" s="13" t="n"/>
       <c r="O48" s="13" t="n"/>
@@ -3040,7 +3134,9 @@
       <c r="I49" s="13" t="n"/>
       <c r="J49" s="13" t="n"/>
       <c r="K49" s="13" t="n"/>
-      <c r="L49" s="13" t="n"/>
+      <c r="L49" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="M49" s="13" t="n"/>
       <c r="N49" s="13" t="n"/>
       <c r="O49" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -3189,6 +3189,48 @@
       <c r="T50" s="13" t="n"/>
       <c r="U50" s="13" t="n"/>
       <c r="V50" s="13" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Mini Golem</t>
+        </is>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="12">
+        <f>ROUND(AVERAGE(F51:AI51), 0)</f>
+        <v/>
+      </c>
+      <c r="D51" s="1">
+        <f>SUM(F51:AI51)</f>
+        <v/>
+      </c>
+      <c r="E51" s="14" t="n">
+        <v>42975</v>
+      </c>
+      <c r="F51" s="13" t="n"/>
+      <c r="G51" s="13" t="n"/>
+      <c r="H51" s="13" t="n"/>
+      <c r="I51" s="13" t="n"/>
+      <c r="J51" s="13" t="n"/>
+      <c r="K51" s="13" t="n"/>
+      <c r="L51" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="13" t="n"/>
+      <c r="N51" s="13" t="n"/>
+      <c r="O51" s="13" t="n"/>
+      <c r="P51" s="13" t="n"/>
+      <c r="Q51" s="13" t="n"/>
+      <c r="R51" s="13" t="n"/>
+      <c r="S51" s="13" t="n"/>
+      <c r="T51" s="13" t="n"/>
+      <c r="U51" s="13" t="n"/>
+      <c r="V51" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AN1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3245,7 +3245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH44"/>
+  <dimension ref="A1:AH51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="9" min="1" max="1"/>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="AD1" s="3" t="inlineStr">
         <is>
-          <t>Colonna28</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="AE1" s="3" t="inlineStr">
@@ -3505,34 +3505,29 @@
       <c r="AC2" t="n">
         <v>0</v>
       </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>14/02/2026</t>
         </is>
       </c>
       <c r="C3" s="9">
         <f>ROUND(AVERAGE(D3:AH3), 0)</f>
         <v/>
       </c>
-      <c r="L3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="O3" t="n">
-        <v>6</v>
-      </c>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="n"/>
+      <c r="N3" s="13" t="n"/>
+      <c r="O3" s="19" t="n"/>
       <c r="P3" t="n">
         <v>6</v>
       </c>
@@ -3546,7 +3541,7 @@
         <v>6</v>
       </c>
       <c r="T3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U3" t="n">
         <v>6</v>
@@ -3558,43 +3553,69 @@
         <v>6</v>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C4" s="9">
         <f>ROUND(AVERAGE(D4:AH4), 0)</f>
         <v/>
       </c>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
-      <c r="N4" s="13" t="n"/>
-      <c r="O4" s="19" t="n"/>
+      <c r="G4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O4" t="n">
+        <v>6</v>
+      </c>
       <c r="P4" t="n">
         <v>6</v>
       </c>
@@ -3608,7 +3629,7 @@
         <v>6</v>
       </c>
       <c r="T4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
         <v>6</v>
@@ -3620,28 +3641,31 @@
         <v>6</v>
       </c>
       <c r="X4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
         <v>6</v>
       </c>
       <c r="Z4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
         <v>6</v>
       </c>
       <c r="AC4" t="n">
         <v>6</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -3653,11 +3677,20 @@
         <f>ROUND(AVERAGE(D5:AH5), 0)</f>
         <v/>
       </c>
+      <c r="D5" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G5" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>6</v>
@@ -3669,13 +3702,13 @@
         <v>6</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N5" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O5" t="n">
         <v>6</v>
@@ -3693,19 +3726,19 @@
         <v>6</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U5" t="n">
         <v>6</v>
       </c>
       <c r="V5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y5" t="n">
         <v>6</v>
@@ -3721,12 +3754,15 @@
       </c>
       <c r="AC5" t="n">
         <v>6</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -3754,34 +3790,34 @@
         <v>0</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N6" s="13" t="n">
         <v>6</v>
       </c>
       <c r="O6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>6</v>
@@ -3796,86 +3832,59 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="n">
         <v>6</v>
       </c>
       <c r="Z6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB6" t="n">
         <v>6</v>
       </c>
       <c r="AC6" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C7" s="9">
         <f>ROUND(AVERAGE(D7:AH7), 0)</f>
         <v/>
       </c>
-      <c r="D7" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="13" t="n">
-        <v>6</v>
-      </c>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
+      <c r="N7" s="13" t="n"/>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S7" t="n">
         <v>6</v>
@@ -3887,13 +3896,13 @@
         <v>6</v>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W7" t="n">
         <v>6</v>
       </c>
       <c r="X7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y7" t="n">
         <v>6</v>
@@ -3902,199 +3911,229 @@
         <v>6</v>
       </c>
       <c r="AA7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C8" s="9">
         <f>ROUND(AVERAGE(D8:AH8), 0)</f>
         <v/>
       </c>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="n"/>
-      <c r="N8" s="13" t="n"/>
+      <c r="G8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="13" t="n">
+        <v>6</v>
+      </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
         <v>6</v>
       </c>
       <c r="Y8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AA8" t="n">
         <v>0</v>
       </c>
       <c r="AB8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C9" s="9">
         <f>ROUND(AVERAGE(D9:AH9), 0)</f>
         <v/>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="N9" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="O9" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>4</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0</v>
-      </c>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
+      <c r="N9" s="13" t="n"/>
+      <c r="O9" s="19" t="n"/>
+      <c r="P9" s="19" t="n"/>
+      <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
+      <c r="T9" s="19" t="n"/>
       <c r="U9" t="n">
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Y9" t="n">
         <v>0</v>
       </c>
       <c r="Z9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C10" s="9">
         <f>ROUND(AVERAGE(D10:AH10), 0)</f>
         <v/>
       </c>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
-      <c r="N10" s="13" t="n"/>
-      <c r="O10" s="19" t="n"/>
-      <c r="P10" s="19" t="n"/>
-      <c r="Q10" s="19" t="n"/>
-      <c r="R10" s="19" t="n"/>
-      <c r="S10" s="19" t="n"/>
-      <c r="T10" s="19" t="n"/>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="O10" t="n">
+        <v>6</v>
+      </c>
+      <c r="P10" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>6</v>
+      </c>
+      <c r="R10" t="n">
+        <v>6</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>6</v>
+      </c>
       <c r="U10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="n">
         <v>0</v>
@@ -4103,19 +4142,22 @@
         <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AB10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC10" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -4127,8 +4169,17 @@
         <f>ROUND(AVERAGE(D11:AH11), 0)</f>
         <v/>
       </c>
+      <c r="D11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>6</v>
@@ -4137,7 +4188,7 @@
         <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>6</v>
@@ -4158,13 +4209,13 @@
         <v>6</v>
       </c>
       <c r="Q11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R11" t="n">
         <v>6</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T11" t="n">
         <v>6</v>
@@ -4176,16 +4227,16 @@
         <v>6</v>
       </c>
       <c r="W11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA11" t="n">
         <v>6</v>
@@ -4194,36 +4245,27 @@
         <v>6</v>
       </c>
       <c r="AC11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD11" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C12" s="9">
         <f>ROUND(AVERAGE(D12:AH12), 0)</f>
         <v/>
       </c>
-      <c r="D12" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>5</v>
-      </c>
       <c r="H12" s="5" t="n">
         <v>6</v>
       </c>
@@ -4252,7 +4294,7 @@
         <v>6</v>
       </c>
       <c r="Q12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R12" t="n">
         <v>6</v>
@@ -4285,27 +4327,42 @@
         <v>6</v>
       </c>
       <c r="AB12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC12" t="n">
         <v>6</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C13" s="9">
         <f>ROUND(AVERAGE(D13:AH13), 0)</f>
         <v/>
       </c>
+      <c r="D13" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="H13" s="5" t="n">
         <v>6</v>
       </c>
@@ -4349,77 +4406,55 @@
         <v>6</v>
       </c>
       <c r="V13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA13" t="n">
         <v>6</v>
       </c>
       <c r="AB13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC13" t="n">
         <v>6</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C14" s="9">
         <f>ROUND(AVERAGE(D14:AH14), 0)</f>
         <v/>
       </c>
-      <c r="D14" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J14" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K14" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L14" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
       <c r="M14" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N14" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
         <v>6</v>
@@ -4440,55 +4475,83 @@
         <v>6</v>
       </c>
       <c r="U14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
       </c>
       <c r="AA14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB14" t="n">
         <v>6</v>
       </c>
       <c r="AC14" t="n">
         <v>6</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C15" s="9">
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
+      <c r="D15" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="M15" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N15" s="13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O15" t="n">
         <v>6</v>
@@ -4509,7 +4572,7 @@
         <v>6</v>
       </c>
       <c r="U15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V15" t="n">
         <v>6</v>
@@ -4521,80 +4584,47 @@
         <v>6</v>
       </c>
       <c r="Y15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="n">
         <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB15" t="n">
         <v>6</v>
       </c>
       <c r="AC15" t="n">
         <v>6</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C16" s="9">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="D16" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N16" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="O16" t="n">
-        <v>6</v>
-      </c>
-      <c r="P16" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>6</v>
-      </c>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="N16" s="6" t="n"/>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
+      <c r="Q16" s="19" t="n"/>
       <c r="R16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>6</v>
@@ -4612,13 +4642,13 @@
         <v>6</v>
       </c>
       <c r="X16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA16" t="n">
         <v>6</v>
@@ -4628,31 +4658,61 @@
       </c>
       <c r="AC16" t="n">
         <v>6</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C17" s="9">
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="6" t="n"/>
-      <c r="N17" s="6" t="n"/>
-      <c r="O17" s="19" t="n"/>
-      <c r="P17" s="19" t="n"/>
-      <c r="Q17" s="19" t="n"/>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" t="n">
+        <v>6</v>
+      </c>
+      <c r="P17" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>6</v>
+      </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S17" t="n">
         <v>6</v>
@@ -4667,31 +4727,34 @@
         <v>6</v>
       </c>
       <c r="W17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AA17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB17" t="n">
         <v>6</v>
       </c>
       <c r="AC17" t="n">
         <v>6</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -4703,11 +4766,20 @@
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
+      <c r="D18" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>6</v>
@@ -4716,16 +4788,16 @@
         <v>6</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
         <v>6</v>
@@ -4746,37 +4818,40 @@
         <v>6</v>
       </c>
       <c r="U18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X18" t="n">
         <v>6</v>
       </c>
       <c r="Y18" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z18" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB18" t="n">
         <v>6</v>
       </c>
       <c r="AC18" t="n">
         <v>6</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -4788,20 +4863,11 @@
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
-      <c r="D19" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>6</v>
@@ -4810,24 +4876,24 @@
         <v>6</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
-        <v>6</v>
-      </c>
-      <c r="P19" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q19" t="n">
+        <v>6</v>
+      </c>
+      <c r="O19" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P19" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q19" s="20" t="n">
         <v>6</v>
       </c>
       <c r="R19" t="n">
@@ -4840,37 +4906,40 @@
         <v>6</v>
       </c>
       <c r="U19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB19" t="n">
         <v>6</v>
       </c>
       <c r="AC19" t="n">
         <v>6</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -4883,7 +4952,7 @@
         <v/>
       </c>
       <c r="G20" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H20" s="5" t="n">
         <v>6</v>
@@ -4934,7 +5003,7 @@
         <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -4950,38 +5019,26 @@
       </c>
       <c r="AC20" t="n">
         <v>6</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C21" s="9">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
-      <c r="G21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J21" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K21" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L21" s="6" t="n">
         <v>6</v>
       </c>
@@ -5000,7 +5057,7 @@
       <c r="Q21" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="R21" t="n">
+      <c r="R21" s="20" t="n">
         <v>6</v>
       </c>
       <c r="S21" t="n">
@@ -5019,13 +5076,13 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA21" t="n">
         <v>0</v>
@@ -5035,23 +5092,29 @@
       </c>
       <c r="AC21" t="n">
         <v>6</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C22" s="9">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
+      <c r="K22" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="L22" s="6" t="n">
         <v>6</v>
       </c>
@@ -5086,42 +5149,66 @@
         <v>6</v>
       </c>
       <c r="W22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y22" t="n">
         <v>6</v>
       </c>
       <c r="Z22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AA22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB22" t="n">
         <v>6</v>
       </c>
       <c r="AC22" t="n">
         <v>6</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C23" s="9">
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
+      <c r="D23" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K23" s="6" t="n">
         <v>6</v>
       </c>
@@ -5150,40 +5237,43 @@
         <v>6</v>
       </c>
       <c r="T23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
         <v>6</v>
       </c>
       <c r="W23" t="n">
+        <v>3</v>
+      </c>
+      <c r="X23" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="n">
         <v>4</v>
       </c>
-      <c r="X23" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>2</v>
-      </c>
       <c r="AB23" t="n">
         <v>6</v>
       </c>
       <c r="AC23" t="n">
         <v>6</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -5196,7 +5286,7 @@
         <v/>
       </c>
       <c r="D24" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>6</v>
@@ -5214,7 +5304,7 @@
         <v>6</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K24" s="6" t="n">
         <v>6</v>
@@ -5240,23 +5330,23 @@
       <c r="R24" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S24" t="n">
+      <c r="S24" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y24" t="n">
         <v>0</v>
@@ -5265,19 +5355,22 @@
         <v>0</v>
       </c>
       <c r="AA24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB24" t="n">
         <v>6</v>
       </c>
       <c r="AC24" t="n">
         <v>6</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -5290,7 +5383,7 @@
         <v/>
       </c>
       <c r="D25" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E25" s="5" t="n">
         <v>6</v>
@@ -5308,7 +5401,7 @@
         <v>6</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K25" s="6" t="n">
         <v>6</v>
@@ -5344,16 +5437,16 @@
         <v>6</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X25" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Y25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z25" t="n">
         <v>0</v>
@@ -5362,16 +5455,19 @@
         <v>0</v>
       </c>
       <c r="AB25" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AC25" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -5383,27 +5479,7 @@
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
-      <c r="D26" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J26" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n">
         <v>6</v>
       </c>
@@ -5431,41 +5507,44 @@
       <c r="S26" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="T26" t="n">
+      <c r="T26" s="20" t="n">
         <v>6</v>
       </c>
       <c r="U26" t="n">
         <v>6</v>
       </c>
       <c r="V26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Z26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB26" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AC26" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -5477,7 +5556,18 @@
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
-      <c r="J27" s="6" t="n"/>
+      <c r="G27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K27" s="6" t="n">
         <v>6</v>
       </c>
@@ -5494,7 +5584,7 @@
         <v>6</v>
       </c>
       <c r="P27" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q27" s="20" t="n">
         <v>6</v>
@@ -5508,128 +5598,96 @@
       <c r="T27" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="U27" t="n">
+      <c r="U27" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V27" t="n">
         <v>0</v>
       </c>
       <c r="W27" t="n">
+        <v>6</v>
+      </c>
+      <c r="X27" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" t="n">
         <v>5</v>
       </c>
-      <c r="X27" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>6</v>
-      </c>
       <c r="AA27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB27" t="n">
         <v>6</v>
       </c>
       <c r="AC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C28" s="9">
         <f>ROUND(AVERAGE(D28:AH28), 0)</f>
         <v/>
       </c>
-      <c r="G28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J28" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K28" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L28" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N28" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P28" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U28" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V28" t="n">
-        <v>0</v>
-      </c>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="n"/>
+      <c r="N28" s="6" t="n"/>
+      <c r="O28" s="20" t="n"/>
+      <c r="P28" s="20" t="n"/>
+      <c r="Q28" s="20" t="n"/>
+      <c r="R28" s="20" t="n"/>
+      <c r="S28" s="20" t="n"/>
+      <c r="T28" s="20" t="n"/>
+      <c r="U28" s="20" t="n"/>
       <c r="W28" t="n">
         <v>6</v>
       </c>
       <c r="X28" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y28" t="n">
         <v>0</v>
       </c>
       <c r="Z28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC28" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C29" s="9">
@@ -5646,32 +5704,29 @@
       <c r="S29" s="20" t="n"/>
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
-      <c r="W29" t="n">
-        <v>6</v>
-      </c>
-      <c r="X29" t="n">
-        <v>6</v>
-      </c>
       <c r="Y29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA29" t="n">
         <v>6</v>
       </c>
       <c r="AB29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC29" t="n">
         <v>6</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -5694,30 +5749,33 @@
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
       <c r="Y30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z30" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC30" t="n">
         <v>6</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C31" s="9">
@@ -5734,31 +5792,31 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="Y31" t="n">
-        <v>0</v>
-      </c>
       <c r="Z31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC31" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD31" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C32" s="9">
@@ -5775,23 +5833,23 @@
       <c r="S32" s="20" t="n"/>
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
-      <c r="Z32" t="n">
-        <v>6</v>
-      </c>
       <c r="AA32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC32" t="n">
         <v>6</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
@@ -5814,19 +5872,22 @@
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
       <c r="AA33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB33" t="n">
         <v>0</v>
       </c>
       <c r="AC33" t="n">
         <v>6</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -5849,24 +5910,27 @@
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
       <c r="AA34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB34" t="n">
         <v>0</v>
       </c>
       <c r="AC34" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C35" s="9">
@@ -5883,20 +5947,20 @@
       <c r="S35" s="20" t="n"/>
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
-      <c r="AA35" t="n">
-        <v>0</v>
-      </c>
       <c r="AB35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC35" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -5922,13 +5986,16 @@
         <v>6</v>
       </c>
       <c r="AC36" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
@@ -5951,21 +6018,24 @@
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
       <c r="AB37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C38" s="9">
@@ -5982,17 +6052,17 @@
       <c r="S38" s="20" t="n"/>
       <c r="T38" s="20" t="n"/>
       <c r="U38" s="20" t="n"/>
-      <c r="AB38" t="n">
-        <v>0</v>
-      </c>
       <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
@@ -6017,11 +6087,14 @@
       <c r="AC39" t="n">
         <v>0</v>
       </c>
+      <c r="AD39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>Space_GG</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -6046,11 +6119,14 @@
       <c r="AC40" t="n">
         <v>0</v>
       </c>
+      <c r="AD40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Space_GG</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
@@ -6073,13 +6149,16 @@
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
       <c r="AC41" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD41" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -6104,16 +6183,19 @@
       <c r="AC42" t="n">
         <v>6</v>
       </c>
+      <c r="AD42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C43" s="9">
@@ -6133,16 +6215,19 @@
       <c r="AC43" t="n">
         <v>6</v>
       </c>
+      <c r="AD43" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C44" s="9">
@@ -6159,11 +6244,213 @@
       <c r="S44" s="20" t="n"/>
       <c r="T44" s="20" t="n"/>
       <c r="U44" s="20" t="n"/>
-      <c r="AC44" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1"/>
+      <c r="AD44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>KingAleGolem03</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="9">
+        <f>ROUND(AVERAGE(D45:AH45), 0)</f>
+        <v/>
+      </c>
+      <c r="K45" s="6" t="n"/>
+      <c r="L45" s="6" t="n"/>
+      <c r="N45" s="6" t="n"/>
+      <c r="O45" s="20" t="n"/>
+      <c r="P45" s="20" t="n"/>
+      <c r="Q45" s="20" t="n"/>
+      <c r="R45" s="20" t="n"/>
+      <c r="S45" s="20" t="n"/>
+      <c r="T45" s="20" t="n"/>
+      <c r="U45" s="20" t="n"/>
+      <c r="AD45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Frost Walker</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="9">
+        <f>ROUND(AVERAGE(D46:AH46), 0)</f>
+        <v/>
+      </c>
+      <c r="K46" s="6" t="n"/>
+      <c r="L46" s="6" t="n"/>
+      <c r="N46" s="6" t="n"/>
+      <c r="O46" s="20" t="n"/>
+      <c r="P46" s="20" t="n"/>
+      <c r="Q46" s="20" t="n"/>
+      <c r="R46" s="20" t="n"/>
+      <c r="S46" s="20" t="n"/>
+      <c r="T46" s="20" t="n"/>
+      <c r="U46" s="20" t="n"/>
+      <c r="AD46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>Z☆PAINKILLER☆Z</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="9">
+        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
+        <v/>
+      </c>
+      <c r="K47" s="6" t="n"/>
+      <c r="L47" s="6" t="n"/>
+      <c r="N47" s="6" t="n"/>
+      <c r="O47" s="20" t="n"/>
+      <c r="P47" s="20" t="n"/>
+      <c r="Q47" s="20" t="n"/>
+      <c r="R47" s="20" t="n"/>
+      <c r="S47" s="20" t="n"/>
+      <c r="T47" s="20" t="n"/>
+      <c r="U47" s="20" t="n"/>
+      <c r="AD47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>zpercu</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="9">
+        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
+        <v/>
+      </c>
+      <c r="K48" s="6" t="n"/>
+      <c r="L48" s="6" t="n"/>
+      <c r="N48" s="6" t="n"/>
+      <c r="O48" s="20" t="n"/>
+      <c r="P48" s="20" t="n"/>
+      <c r="Q48" s="20" t="n"/>
+      <c r="R48" s="20" t="n"/>
+      <c r="S48" s="20" t="n"/>
+      <c r="T48" s="20" t="n"/>
+      <c r="U48" s="20" t="n"/>
+      <c r="AD48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>Mini Golem</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="9">
+        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
+        <v/>
+      </c>
+      <c r="K49" s="6" t="n"/>
+      <c r="L49" s="6" t="n"/>
+      <c r="N49" s="6" t="n"/>
+      <c r="O49" s="20" t="n"/>
+      <c r="P49" s="20" t="n"/>
+      <c r="Q49" s="20" t="n"/>
+      <c r="R49" s="20" t="n"/>
+      <c r="S49" s="20" t="n"/>
+      <c r="T49" s="20" t="n"/>
+      <c r="U49" s="20" t="n"/>
+      <c r="AD49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Breso</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="9">
+        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
+        <v/>
+      </c>
+      <c r="K50" s="6" t="n"/>
+      <c r="L50" s="6" t="n"/>
+      <c r="N50" s="6" t="n"/>
+      <c r="O50" s="20" t="n"/>
+      <c r="P50" s="20" t="n"/>
+      <c r="Q50" s="20" t="n"/>
+      <c r="R50" s="20" t="n"/>
+      <c r="S50" s="20" t="n"/>
+      <c r="T50" s="20" t="n"/>
+      <c r="U50" s="20" t="n"/>
+      <c r="AD50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>escanor</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="9">
+        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
+        <v/>
+      </c>
+      <c r="K51" s="6" t="n"/>
+      <c r="L51" s="6" t="n"/>
+      <c r="N51" s="6" t="n"/>
+      <c r="O51" s="20" t="n"/>
+      <c r="P51" s="20" t="n"/>
+      <c r="Q51" s="20" t="n"/>
+      <c r="R51" s="20" t="n"/>
+      <c r="S51" s="20" t="n"/>
+      <c r="T51" s="20" t="n"/>
+      <c r="U51" s="20" t="n"/>
+      <c r="AD51" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-24
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1286,7 +1286,7 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>124970</v>
+        <v>126020</v>
       </c>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n"/>
@@ -1303,7 +1303,7 @@
         <v>8800</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>13600</v>
+        <v>14650</v>
       </c>
       <c r="M9" s="13" t="n"/>
       <c r="N9" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-24
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -4660,7 +4660,7 @@
         <v>6</v>
       </c>
       <c r="AD16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -4845,7 +4845,7 @@
         <v>6</v>
       </c>
       <c r="AD18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -5626,7 +5626,7 @@
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
@@ -5720,7 +5720,7 @@
         <v>6</v>
       </c>
       <c r="AD29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -5954,13 +5954,13 @@
         <v>6</v>
       </c>
       <c r="AD35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -5983,7 +5983,7 @@
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
       <c r="AB36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC36" t="n">
         <v>0</v>
@@ -5995,12 +5995,12 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C37" s="9">
@@ -6017,9 +6017,6 @@
       <c r="S37" s="20" t="n"/>
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
-      <c r="AB37" t="n">
-        <v>0</v>
-      </c>
       <c r="AC37" t="n">
         <v>0</v>
       </c>
@@ -6030,7 +6027,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -6062,7 +6059,7 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
@@ -6085,7 +6082,7 @@
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
       <c r="AC39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD39" t="n">
         <v>0</v>
@@ -6094,7 +6091,7 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Space_GG</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -6117,21 +6114,21 @@
       <c r="T40" s="20" t="n"/>
       <c r="U40" s="20" t="n"/>
       <c r="AC40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C41" s="9">
@@ -6152,18 +6149,18 @@
         <v>6</v>
       </c>
       <c r="AD41" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C42" s="9">
@@ -6180,9 +6177,6 @@
       <c r="S42" s="20" t="n"/>
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
-      <c r="AC42" t="n">
-        <v>6</v>
-      </c>
       <c r="AD42" t="n">
         <v>0</v>
       </c>
@@ -6190,12 +6184,12 @@
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>KingAleGolem03</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C43" s="9">
@@ -6212,17 +6206,14 @@
       <c r="S43" s="20" t="n"/>
       <c r="T43" s="20" t="n"/>
       <c r="U43" s="20" t="n"/>
-      <c r="AC43" t="n">
-        <v>6</v>
-      </c>
       <c r="AD43" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>Frost Walker</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -6251,7 +6242,7 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>KingAleGolem03</t>
+          <t>Z☆PAINKILLER☆Z</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
@@ -6280,7 +6271,7 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Frost Walker</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -6303,13 +6294,13 @@
       <c r="T46" s="20" t="n"/>
       <c r="U46" s="20" t="n"/>
       <c r="AD46" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>Z☆PAINKILLER☆Z</t>
+          <t>Mini Golem</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
@@ -6332,13 +6323,13 @@
       <c r="T47" s="20" t="n"/>
       <c r="U47" s="20" t="n"/>
       <c r="AD47" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>Breso</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
@@ -6367,7 +6358,7 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>Mini Golem</t>
+          <t>escanor</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
@@ -6390,18 +6381,18 @@
       <c r="T49" s="20" t="n"/>
       <c r="U49" s="20" t="n"/>
       <c r="AD49" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>Breso</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="C50" s="9">
@@ -6425,12 +6416,12 @@
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>escanor</t>
+          <t>cioli03</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="C51" s="9">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3756,7 +3756,7 @@
         <v>6</v>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4008,7 +4008,7 @@
         <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -4063,7 +4063,7 @@
         <v>0</v>
       </c>
       <c r="AD9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -4151,7 +4151,7 @@
         <v>6</v>
       </c>
       <c r="AD10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4333,7 +4333,7 @@
         <v>6</v>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -4430,7 +4430,7 @@
         <v>6</v>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4599,7 +4599,7 @@
         <v>6</v>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -4748,7 +4748,7 @@
         <v>6</v>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4933,7 +4933,7 @@
         <v>6</v>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -5021,7 +5021,7 @@
         <v>6</v>
       </c>
       <c r="AD20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -5170,7 +5170,7 @@
         <v>6</v>
       </c>
       <c r="AD22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -5538,7 +5538,7 @@
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -5676,7 +5676,7 @@
         <v>6</v>
       </c>
       <c r="AD28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -5720,7 +5720,7 @@
         <v>6</v>
       </c>
       <c r="AD29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -5843,7 +5843,7 @@
         <v>6</v>
       </c>
       <c r="AD32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -6085,7 +6085,7 @@
         <v>6</v>
       </c>
       <c r="AD39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -6236,7 +6236,7 @@
       <c r="T44" s="20" t="n"/>
       <c r="U44" s="20" t="n"/>
       <c r="AD44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -6381,7 +6381,7 @@
       <c r="T49" s="20" t="n"/>
       <c r="U49" s="20" t="n"/>
       <c r="AD49" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -988,7 +988,7 @@
         <v/>
       </c>
       <c r="E3" s="14" t="n">
-        <v>70400</v>
+        <v>72800</v>
       </c>
       <c r="F3" s="13" t="n">
         <v>4000</v>
@@ -1009,7 +1009,7 @@
         <v>10000</v>
       </c>
       <c r="L3" s="13" t="n">
-        <v>12200</v>
+        <v>14600</v>
       </c>
       <c r="M3" s="13" t="n"/>
       <c r="N3" s="13" t="n"/>
@@ -1336,7 +1336,7 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>73600</v>
+        <v>74400</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
@@ -1353,7 +1353,7 @@
         <v>8600</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>13150</v>
+        <v>13950</v>
       </c>
       <c r="M10" s="13" t="n"/>
       <c r="N10" s="13" t="n"/>
@@ -1438,7 +1438,7 @@
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>90800</v>
+        <v>90900</v>
       </c>
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
@@ -1451,7 +1451,7 @@
         <v>6100</v>
       </c>
       <c r="L12" s="13" t="n">
-        <v>13150</v>
+        <v>13250</v>
       </c>
       <c r="M12" s="13" t="n"/>
       <c r="N12" s="13" t="n"/>
@@ -2004,7 +2004,7 @@
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>37125</v>
+        <v>37575</v>
       </c>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
@@ -2021,7 +2021,7 @@
         <v>3000</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>5300</v>
+        <v>5750</v>
       </c>
       <c r="M23" s="13" t="n"/>
       <c r="N23" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-26
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2706,7 +2706,7 @@
         <v/>
       </c>
       <c r="E39" s="14" t="n">
-        <v>46125</v>
+        <v>47025</v>
       </c>
       <c r="F39" s="13" t="n"/>
       <c r="G39" s="13" t="n"/>
@@ -2715,7 +2715,7 @@
       <c r="J39" s="13" t="n"/>
       <c r="K39" s="13" t="n"/>
       <c r="L39" s="13" t="n">
-        <v>9250</v>
+        <v>10150</v>
       </c>
       <c r="M39" s="13" t="n"/>
       <c r="N39" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2328,7 +2328,7 @@
         <v/>
       </c>
       <c r="E30" s="14" t="n">
-        <v>50690</v>
+        <v>51290</v>
       </c>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
@@ -2337,7 +2337,7 @@
       <c r="J30" s="13" t="n"/>
       <c r="K30" s="13" t="n"/>
       <c r="L30" s="13" t="n">
-        <v>10050</v>
+        <v>10650</v>
       </c>
       <c r="M30" s="13" t="n"/>
       <c r="N30" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-05-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1950,7 +1950,7 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>48800</v>
+        <v>49250</v>
       </c>
       <c r="F22" s="13" t="n">
         <v>4000</v>
@@ -1971,7 +1971,7 @@
         <v>3100</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>8900</v>
+        <v>9350</v>
       </c>
       <c r="M22" s="13" t="n"/>
       <c r="N22" s="13" t="n"/>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>76400</v>
+        <v>77200</v>
       </c>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
@@ -2069,7 +2069,7 @@
         <v>1400</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>1400</v>
+        <v>2200</v>
       </c>
       <c r="M24" s="13" t="n"/>
       <c r="N24" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-30
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3414,7 +3414,7 @@
       </c>
       <c r="AE1" s="3" t="inlineStr">
         <is>
-          <t>Colonna29</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="AF1" s="3" t="inlineStr">
@@ -3506,6 +3506,9 @@
         <v>0</v>
       </c>
       <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3573,6 +3576,9 @@
       <c r="AD3" t="n">
         <v>6</v>
       </c>
+      <c r="AE3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -3661,6 +3667,9 @@
       <c r="AD4" t="n">
         <v>0</v>
       </c>
+      <c r="AE4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -3758,6 +3767,9 @@
       <c r="AD5" t="n">
         <v>6</v>
       </c>
+      <c r="AE5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -3853,6 +3865,9 @@
         <v>0</v>
       </c>
       <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3922,6 +3937,9 @@
       <c r="AD7" t="n">
         <v>0</v>
       </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -4009,6 +4027,9 @@
       </c>
       <c r="AD8" t="n">
         <v>1</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4065,6 +4086,9 @@
       <c r="AD9" t="n">
         <v>4</v>
       </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -4153,6 +4177,9 @@
       <c r="AD10" t="n">
         <v>6</v>
       </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -4250,6 +4277,9 @@
       <c r="AD11" t="n">
         <v>6</v>
       </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -4335,6 +4365,9 @@
       <c r="AD12" t="n">
         <v>6</v>
       </c>
+      <c r="AE12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -4430,6 +4463,9 @@
         <v>6</v>
       </c>
       <c r="AD13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE13" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4504,6 +4540,9 @@
       <c r="AD14" t="n">
         <v>0</v>
       </c>
+      <c r="AE14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -4600,6 +4639,9 @@
       </c>
       <c r="AD15" t="n">
         <v>6</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -4662,6 +4704,9 @@
       <c r="AD16" t="n">
         <v>6</v>
       </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -4750,6 +4795,9 @@
       <c r="AD17" t="n">
         <v>6</v>
       </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -4847,6 +4895,9 @@
       <c r="AD18" t="n">
         <v>6</v>
       </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -4935,6 +4986,9 @@
       <c r="AD19" t="n">
         <v>6</v>
       </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -5023,6 +5077,9 @@
       <c r="AD20" t="n">
         <v>5</v>
       </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -5096,6 +5153,9 @@
       <c r="AD21" t="n">
         <v>0</v>
       </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -5172,6 +5232,9 @@
       <c r="AD22" t="n">
         <v>4</v>
       </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -5269,6 +5332,9 @@
       <c r="AD23" t="n">
         <v>0</v>
       </c>
+      <c r="AE23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -5366,6 +5432,9 @@
       <c r="AD24" t="n">
         <v>0</v>
       </c>
+      <c r="AE24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -5463,6 +5532,9 @@
       <c r="AD25" t="n">
         <v>5</v>
       </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -5540,6 +5612,9 @@
       <c r="AD26" t="n">
         <v>6</v>
       </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -5626,6 +5701,9 @@
         <v>0</v>
       </c>
       <c r="AD27" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE27" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5678,6 +5756,9 @@
       <c r="AD28" t="n">
         <v>5</v>
       </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -5722,6 +5803,9 @@
       <c r="AD29" t="n">
         <v>6</v>
       </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -5766,6 +5850,9 @@
       <c r="AD30" t="n">
         <v>0</v>
       </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
@@ -5807,6 +5894,9 @@
       <c r="AD31" t="n">
         <v>6</v>
       </c>
+      <c r="AE31" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -5844,6 +5934,9 @@
       </c>
       <c r="AD32" t="n">
         <v>6</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -5883,6 +5976,9 @@
       <c r="AD33" t="n">
         <v>0</v>
       </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -5921,6 +6017,9 @@
       <c r="AD34" t="n">
         <v>0</v>
       </c>
+      <c r="AE34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
@@ -5956,6 +6055,9 @@
       <c r="AD35" t="n">
         <v>6</v>
       </c>
+      <c r="AE35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
@@ -5991,6 +6093,9 @@
       <c r="AD36" t="n">
         <v>0</v>
       </c>
+      <c r="AE36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
@@ -6023,11 +6128,14 @@
       <c r="AD37" t="n">
         <v>0</v>
       </c>
+      <c r="AE37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -6050,16 +6158,19 @@
       <c r="T38" s="20" t="n"/>
       <c r="U38" s="20" t="n"/>
       <c r="AC38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
@@ -6087,16 +6198,19 @@
       <c r="AD39" t="n">
         <v>6</v>
       </c>
+      <c r="AE39" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C40" s="9">
@@ -6119,16 +6233,19 @@
       <c r="AD40" t="n">
         <v>6</v>
       </c>
+      <c r="AE40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>KingAleGolem03</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C41" s="9">
@@ -6145,17 +6262,17 @@
       <c r="S41" s="20" t="n"/>
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
-      <c r="AC41" t="n">
-        <v>6</v>
-      </c>
       <c r="AD41" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>Frost Walker</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -6178,13 +6295,16 @@
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
       <c r="AD42" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE42" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>KingAleGolem03</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
@@ -6207,13 +6327,16 @@
       <c r="T43" s="20" t="n"/>
       <c r="U43" s="20" t="n"/>
       <c r="AD43" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>Frost Walker</t>
+          <t>escanor</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -6238,16 +6361,19 @@
       <c r="AD44" t="n">
         <v>6</v>
       </c>
+      <c r="AE44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>Z☆PAINKILLER☆Z</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="C45" s="9">
@@ -6267,16 +6393,19 @@
       <c r="AD45" t="n">
         <v>0</v>
       </c>
+      <c r="AE45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C46" s="9">
@@ -6293,19 +6422,19 @@
       <c r="S46" s="20" t="n"/>
       <c r="T46" s="20" t="n"/>
       <c r="U46" s="20" t="n"/>
-      <c r="AD46" t="n">
-        <v>6</v>
+      <c r="AE46" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>Mini Golem</t>
+          <t>ale mugna</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C47" s="9">
@@ -6322,19 +6451,19 @@
       <c r="S47" s="20" t="n"/>
       <c r="T47" s="20" t="n"/>
       <c r="U47" s="20" t="n"/>
-      <c r="AD47" t="n">
-        <v>6</v>
+      <c r="AE47" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>Breso</t>
+          <t>ale 12</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C48" s="9">
@@ -6351,19 +6480,19 @@
       <c r="S48" s="20" t="n"/>
       <c r="T48" s="20" t="n"/>
       <c r="U48" s="20" t="n"/>
-      <c r="AD48" t="n">
+      <c r="AE48" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>escanor</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C49" s="9">
@@ -6380,19 +6509,19 @@
       <c r="S49" s="20" t="n"/>
       <c r="T49" s="20" t="n"/>
       <c r="U49" s="20" t="n"/>
-      <c r="AD49" t="n">
-        <v>6</v>
+      <c r="AE49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>SgherroMutante</t>
+          <t>marcobeltra._</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C50" s="9">
@@ -6409,19 +6538,19 @@
       <c r="S50" s="20" t="n"/>
       <c r="T50" s="20" t="n"/>
       <c r="U50" s="20" t="n"/>
-      <c r="AD50" t="n">
+      <c r="AE50" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>cioli03</t>
+          <t>vito</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C51" s="9">
@@ -6438,7 +6567,7 @@
       <c r="S51" s="20" t="n"/>
       <c r="T51" s="20" t="n"/>
       <c r="U51" s="20" t="n"/>
-      <c r="AD51" t="n">
+      <c r="AE51" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-05-31
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3245,7 +3245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="9" min="1" max="1"/>
@@ -4705,7 +4705,7 @@
         <v>6</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -4796,7 +4796,7 @@
         <v>6</v>
       </c>
       <c r="AE17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4896,7 +4896,7 @@
         <v>6</v>
       </c>
       <c r="AE18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -5804,7 +5804,7 @@
         <v>6</v>
       </c>
       <c r="AE29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -6164,7 +6164,7 @@
         <v>6</v>
       </c>
       <c r="AE38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -6272,7 +6272,7 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>Frost Walker</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -6298,18 +6298,18 @@
         <v>6</v>
       </c>
       <c r="AE42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="C43" s="9">
@@ -6327,7 +6327,7 @@
       <c r="T43" s="20" t="n"/>
       <c r="U43" s="20" t="n"/>
       <c r="AD43" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE43" t="n">
         <v>0</v>
@@ -6336,12 +6336,12 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>escanor</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C44" s="9">
@@ -6358,22 +6358,19 @@
       <c r="S44" s="20" t="n"/>
       <c r="T44" s="20" t="n"/>
       <c r="U44" s="20" t="n"/>
-      <c r="AD44" t="n">
-        <v>6</v>
-      </c>
       <c r="AE44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>SgherroMutante</t>
+          <t>ale mugna</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C45" s="9">
@@ -6390,9 +6387,6 @@
       <c r="S45" s="20" t="n"/>
       <c r="T45" s="20" t="n"/>
       <c r="U45" s="20" t="n"/>
-      <c r="AD45" t="n">
-        <v>0</v>
-      </c>
       <c r="AE45" t="n">
         <v>0</v>
       </c>
@@ -6400,7 +6394,7 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>ale 12</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -6429,7 +6423,7 @@
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>ale mugna</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
@@ -6458,7 +6452,7 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>ale 12</t>
+          <t>marcobeltra._</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
@@ -6487,7 +6481,7 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>vito</t>
         </is>
       </c>
       <c r="B49" s="11" t="inlineStr">
@@ -6516,12 +6510,12 @@
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>marcobeltra._</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C50" s="9">
@@ -6539,35 +6533,6 @@
       <c r="T50" s="20" t="n"/>
       <c r="U50" s="20" t="n"/>
       <c r="AE50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>vito</t>
-        </is>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="9">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="6" t="n"/>
-      <c r="L51" s="6" t="n"/>
-      <c r="N51" s="6" t="n"/>
-      <c r="O51" s="20" t="n"/>
-      <c r="P51" s="20" t="n"/>
-      <c r="Q51" s="20" t="n"/>
-      <c r="R51" s="20" t="n"/>
-      <c r="S51" s="20" t="n"/>
-      <c r="T51" s="20" t="n"/>
-      <c r="U51" s="20" t="n"/>
-      <c r="AE51" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-06
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3248,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="AF1" s="3" t="inlineStr">
         <is>
-          <t>Colonna30</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="AG1" s="3" t="inlineStr">
@@ -3512,6 +3512,9 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3582,6 +3585,9 @@
       <c r="AE3" t="n">
         <v>6</v>
       </c>
+      <c r="AF3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3673,6 +3679,9 @@
       <c r="AE4" t="n">
         <v>0</v>
       </c>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3773,6 +3782,9 @@
       <c r="AE5" t="n">
         <v>6</v>
       </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3871,6 +3883,9 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3943,6 +3958,9 @@
       <c r="AE7" t="n">
         <v>0</v>
       </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4032,6 +4050,9 @@
         <v>1</v>
       </c>
       <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4092,6 +4113,9 @@
       <c r="AE9" t="n">
         <v>6</v>
       </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4183,6 +4207,9 @@
       <c r="AE10" t="n">
         <v>3</v>
       </c>
+      <c r="AF10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4283,6 +4310,9 @@
       <c r="AE11" t="n">
         <v>6</v>
       </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4371,6 +4401,9 @@
       <c r="AE12" t="n">
         <v>0</v>
       </c>
+      <c r="AF12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4470,6 +4503,9 @@
       </c>
       <c r="AE13" t="n">
         <v>6</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4546,6 +4582,9 @@
       <c r="AE14" t="n">
         <v>6</v>
       </c>
+      <c r="AF14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4644,6 +4683,9 @@
         <v>6</v>
       </c>
       <c r="AE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4710,6 +4752,9 @@
       <c r="AE16" t="n">
         <v>4</v>
       </c>
+      <c r="AF16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4801,6 +4846,9 @@
       <c r="AE17" t="n">
         <v>6</v>
       </c>
+      <c r="AF17" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4901,6 +4949,9 @@
       <c r="AE18" t="n">
         <v>6</v>
       </c>
+      <c r="AF18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -4992,6 +5043,9 @@
       <c r="AE19" t="n">
         <v>6</v>
       </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5083,6 +5137,9 @@
       <c r="AE20" t="n">
         <v>6</v>
       </c>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5159,6 +5216,9 @@
       <c r="AE21" t="n">
         <v>0</v>
       </c>
+      <c r="AF21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5238,6 +5298,9 @@
       <c r="AE22" t="n">
         <v>0</v>
       </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5338,6 +5401,9 @@
       <c r="AE23" t="n">
         <v>0</v>
       </c>
+      <c r="AF23" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5438,6 +5504,9 @@
       <c r="AE24" t="n">
         <v>0</v>
       </c>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5538,6 +5607,9 @@
       <c r="AE25" t="n">
         <v>0</v>
       </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5618,6 +5690,9 @@
       <c r="AE26" t="n">
         <v>6</v>
       </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5707,6 +5782,9 @@
         <v>6</v>
       </c>
       <c r="AE27" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF27" t="n">
         <v>6</v>
       </c>
     </row>
@@ -5762,6 +5840,9 @@
       <c r="AE28" t="n">
         <v>6</v>
       </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -5809,6 +5890,9 @@
       <c r="AE29" t="n">
         <v>6</v>
       </c>
+      <c r="AF29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -5856,6 +5940,9 @@
       <c r="AE30" t="n">
         <v>0</v>
       </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -5900,6 +5987,9 @@
       <c r="AE31" t="n">
         <v>6</v>
       </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -5940,6 +6030,9 @@
       </c>
       <c r="AE32" t="n">
         <v>6</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -5982,16 +6075,19 @@
       <c r="AE33" t="n">
         <v>0</v>
       </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C34" s="28">
@@ -6008,31 +6104,31 @@
       <c r="S34" s="20" t="n"/>
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
-      <c r="AA34" t="n">
-        <v>0</v>
-      </c>
       <c r="AB34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE34" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF34" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C35" s="28">
@@ -6049,9 +6145,6 @@
       <c r="S35" s="20" t="n"/>
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
-      <c r="AB35" t="n">
-        <v>6</v>
-      </c>
       <c r="AC35" t="n">
         <v>6</v>
       </c>
@@ -6060,17 +6153,20 @@
       </c>
       <c r="AE35" t="n">
         <v>6</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C36" s="28">
@@ -6087,28 +6183,28 @@
       <c r="S36" s="20" t="n"/>
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
-      <c r="AB36" t="n">
-        <v>0</v>
-      </c>
       <c r="AC36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE36" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C37" s="28">
@@ -6126,24 +6222,27 @@
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
       <c r="AC37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF37" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C38" s="28">
@@ -6160,25 +6259,25 @@
       <c r="S38" s="20" t="n"/>
       <c r="T38" s="20" t="n"/>
       <c r="U38" s="20" t="n"/>
-      <c r="AC38" t="n">
-        <v>6</v>
-      </c>
       <c r="AD38" t="n">
         <v>6</v>
       </c>
       <c r="AE38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF38" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="28" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C39" s="28">
@@ -6195,25 +6294,22 @@
       <c r="S39" s="20" t="n"/>
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
-      <c r="AC39" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD39" t="n">
-        <v>6</v>
-      </c>
       <c r="AE39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF39" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C40" s="28">
@@ -6230,25 +6326,22 @@
       <c r="S40" s="20" t="n"/>
       <c r="T40" s="20" t="n"/>
       <c r="U40" s="20" t="n"/>
-      <c r="AC40" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD40" t="n">
-        <v>6</v>
-      </c>
       <c r="AE40" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF40" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="28" t="inlineStr">
         <is>
-          <t>KingAleGolem03</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C41" s="28">
@@ -6265,22 +6358,22 @@
       <c r="S41" s="20" t="n"/>
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
-      <c r="AD41" t="n">
-        <v>0</v>
-      </c>
       <c r="AE41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF41" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C42" s="28">
@@ -6297,22 +6390,22 @@
       <c r="S42" s="20" t="n"/>
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
-      <c r="AD42" t="n">
-        <v>6</v>
-      </c>
       <c r="AE42" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="AF42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="28" t="inlineStr">
         <is>
-          <t>SgherroMutante</t>
+          <t>favretto</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="C43" s="28">
@@ -6329,245 +6422,11 @@
       <c r="S43" s="20" t="n"/>
       <c r="T43" s="20" t="n"/>
       <c r="U43" s="20" t="n"/>
-      <c r="AD43" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="28" t="inlineStr">
-        <is>
-          <t>rasim01</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C44" s="28">
-        <f>ROUND(AVERAGE(D44:AH44), 0)</f>
-        <v/>
-      </c>
-      <c r="K44" s="6" t="n"/>
-      <c r="L44" s="6" t="n"/>
-      <c r="N44" s="6" t="n"/>
-      <c r="O44" s="20" t="n"/>
-      <c r="P44" s="20" t="n"/>
-      <c r="Q44" s="20" t="n"/>
-      <c r="R44" s="20" t="n"/>
-      <c r="S44" s="20" t="n"/>
-      <c r="T44" s="20" t="n"/>
-      <c r="U44" s="20" t="n"/>
-      <c r="AE44" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="28" t="inlineStr">
-        <is>
-          <t>ale mugna</t>
-        </is>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C45" s="28">
-        <f>ROUND(AVERAGE(D45:AH45), 0)</f>
-        <v/>
-      </c>
-      <c r="K45" s="6" t="n"/>
-      <c r="L45" s="6" t="n"/>
-      <c r="N45" s="6" t="n"/>
-      <c r="O45" s="20" t="n"/>
-      <c r="P45" s="20" t="n"/>
-      <c r="Q45" s="20" t="n"/>
-      <c r="R45" s="20" t="n"/>
-      <c r="S45" s="20" t="n"/>
-      <c r="T45" s="20" t="n"/>
-      <c r="U45" s="20" t="n"/>
-      <c r="AE45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="28" t="inlineStr">
-        <is>
-          <t>ale 12</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="28">
-        <f>ROUND(AVERAGE(D46:AH46), 0)</f>
-        <v/>
-      </c>
-      <c r="K46" s="6" t="n"/>
-      <c r="L46" s="6" t="n"/>
-      <c r="N46" s="6" t="n"/>
-      <c r="O46" s="20" t="n"/>
-      <c r="P46" s="20" t="n"/>
-      <c r="Q46" s="20" t="n"/>
-      <c r="R46" s="20" t="n"/>
-      <c r="S46" s="20" t="n"/>
-      <c r="T46" s="20" t="n"/>
-      <c r="U46" s="20" t="n"/>
-      <c r="AE46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="28" t="inlineStr">
-        <is>
-          <t>maragno</t>
-        </is>
-      </c>
-      <c r="B47" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="28">
-        <f>ROUND(AVERAGE(D47:AH47), 0)</f>
-        <v/>
-      </c>
-      <c r="K47" s="6" t="n"/>
-      <c r="L47" s="6" t="n"/>
-      <c r="N47" s="6" t="n"/>
-      <c r="O47" s="20" t="n"/>
-      <c r="P47" s="20" t="n"/>
-      <c r="Q47" s="20" t="n"/>
-      <c r="R47" s="20" t="n"/>
-      <c r="S47" s="20" t="n"/>
-      <c r="T47" s="20" t="n"/>
-      <c r="U47" s="20" t="n"/>
-      <c r="AE47" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="28" t="inlineStr">
-        <is>
-          <t>marcobeltra._</t>
-        </is>
-      </c>
-      <c r="B48" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="28">
-        <f>ROUND(AVERAGE(D48:AH48), 0)</f>
-        <v/>
-      </c>
-      <c r="K48" s="6" t="n"/>
-      <c r="L48" s="6" t="n"/>
-      <c r="N48" s="6" t="n"/>
-      <c r="O48" s="20" t="n"/>
-      <c r="P48" s="20" t="n"/>
-      <c r="Q48" s="20" t="n"/>
-      <c r="R48" s="20" t="n"/>
-      <c r="S48" s="20" t="n"/>
-      <c r="T48" s="20" t="n"/>
-      <c r="U48" s="20" t="n"/>
-      <c r="AE48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="28" t="inlineStr">
-        <is>
-          <t>vito</t>
-        </is>
-      </c>
-      <c r="B49" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="28">
-        <f>ROUND(AVERAGE(D49:AH49), 0)</f>
-        <v/>
-      </c>
-      <c r="K49" s="6" t="n"/>
-      <c r="L49" s="6" t="n"/>
-      <c r="N49" s="6" t="n"/>
-      <c r="O49" s="20" t="n"/>
-      <c r="P49" s="20" t="n"/>
-      <c r="Q49" s="20" t="n"/>
-      <c r="R49" s="20" t="n"/>
-      <c r="S49" s="20" t="n"/>
-      <c r="T49" s="20" t="n"/>
-      <c r="U49" s="20" t="n"/>
-      <c r="AE49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="28" t="inlineStr">
-        <is>
-          <t>Akemi</t>
-        </is>
-      </c>
-      <c r="B50" s="11" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="28">
-        <f>ROUND(AVERAGE(D50:AH50), 0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="6" t="n"/>
-      <c r="L50" s="6" t="n"/>
-      <c r="N50" s="6" t="n"/>
-      <c r="O50" s="20" t="n"/>
-      <c r="P50" s="20" t="n"/>
-      <c r="Q50" s="20" t="n"/>
-      <c r="R50" s="20" t="n"/>
-      <c r="S50" s="20" t="n"/>
-      <c r="T50" s="20" t="n"/>
-      <c r="U50" s="20" t="n"/>
-      <c r="AE50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="28" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="28">
-        <f>ROUND(AVERAGE(D51:AH51), 0)</f>
-        <v/>
-      </c>
-      <c r="K51" s="6" t="n"/>
-      <c r="L51" s="6" t="n"/>
-      <c r="N51" s="6" t="n"/>
-      <c r="O51" s="20" t="n"/>
-      <c r="P51" s="20" t="n"/>
-      <c r="Q51" s="20" t="n"/>
-      <c r="R51" s="20" t="n"/>
-      <c r="S51" s="20" t="n"/>
-      <c r="T51" s="20" t="n"/>
-      <c r="U51" s="20" t="n"/>
-      <c r="AE51" t="n">
-        <v>6</v>
-      </c>
-    </row>
+      <c r="AF43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:AT1">
     <sortState ref="A2:AT50">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-07
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3248,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH43"/>
+  <dimension ref="A1:AH42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3680,7 +3680,7 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -4311,7 +4311,7 @@
         <v>6</v>
       </c>
       <c r="AF11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -5044,7 +5044,7 @@
         <v>6</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -5891,7 +5891,7 @@
         <v>6</v>
       </c>
       <c r="AF29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -6117,13 +6117,13 @@
         <v>6</v>
       </c>
       <c r="AF34" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
@@ -6155,18 +6155,18 @@
         <v>6</v>
       </c>
       <c r="AF35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C36" s="28">
@@ -6190,21 +6190,21 @@
         <v>6</v>
       </c>
       <c r="AE36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C37" s="28">
@@ -6221,28 +6221,25 @@
       <c r="S37" s="20" t="n"/>
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
-      <c r="AC37" t="n">
-        <v>6</v>
-      </c>
       <c r="AD37" t="n">
         <v>6</v>
       </c>
       <c r="AE37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF37" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C38" s="28">
@@ -6259,11 +6256,8 @@
       <c r="S38" s="20" t="n"/>
       <c r="T38" s="20" t="n"/>
       <c r="U38" s="20" t="n"/>
-      <c r="AD38" t="n">
-        <v>6</v>
-      </c>
       <c r="AE38" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF38" t="n">
         <v>6</v>
@@ -6272,7 +6266,7 @@
     <row r="39">
       <c r="A39" s="28" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
@@ -6298,18 +6292,18 @@
         <v>6</v>
       </c>
       <c r="AF39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C40" s="28">
@@ -6327,21 +6321,21 @@
       <c r="T40" s="20" t="n"/>
       <c r="U40" s="20" t="n"/>
       <c r="AE40" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF40" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C41" s="28">
@@ -6359,7 +6353,7 @@
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
       <c r="AE41" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF41" t="n">
         <v>0</v>
@@ -6368,12 +6362,12 @@
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>favretto</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="C42" s="28">
@@ -6390,39 +6384,7 @@
       <c r="S42" s="20" t="n"/>
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
-      <c r="AE42" t="n">
-        <v>6</v>
-      </c>
       <c r="AF42" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="28" t="inlineStr">
-        <is>
-          <t>favretto</t>
-        </is>
-      </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>06/06/2026</t>
-        </is>
-      </c>
-      <c r="C43" s="28">
-        <f>ROUND(AVERAGE(D43:AH43), 0)</f>
-        <v/>
-      </c>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="6" t="n"/>
-      <c r="N43" s="6" t="n"/>
-      <c r="O43" s="20" t="n"/>
-      <c r="P43" s="20" t="n"/>
-      <c r="Q43" s="20" t="n"/>
-      <c r="R43" s="20" t="n"/>
-      <c r="S43" s="20" t="n"/>
-      <c r="T43" s="20" t="n"/>
-      <c r="U43" s="20" t="n"/>
-      <c r="AF43" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-08
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3783,7 +3783,7 @@
         <v>6</v>
       </c>
       <c r="AF5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4114,7 +4114,7 @@
         <v>6</v>
       </c>
       <c r="AF9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -4505,7 +4505,7 @@
         <v>6</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4847,7 +4847,7 @@
         <v>6</v>
       </c>
       <c r="AF17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -5138,7 +5138,7 @@
         <v>6</v>
       </c>
       <c r="AF20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -5505,7 +5505,7 @@
         <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -5841,7 +5841,7 @@
         <v>6</v>
       </c>
       <c r="AF28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -5988,7 +5988,7 @@
         <v>6</v>
       </c>
       <c r="AF31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -6292,7 +6292,7 @@
         <v>6</v>
       </c>
       <c r="AF39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -6324,7 +6324,7 @@
         <v>0</v>
       </c>
       <c r="AF40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
@@ -6356,7 +6356,7 @@
         <v>6</v>
       </c>
       <c r="AF41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -6385,7 +6385,7 @@
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
       <c r="AF42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-13
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3427,7 +3427,7 @@
       </c>
       <c r="AG1" s="3" t="inlineStr">
         <is>
-          <t>Colonna31</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="AH1" s="3" t="inlineStr">
@@ -3515,6 +3515,9 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3588,6 +3591,9 @@
       <c r="AF3" t="n">
         <v>6</v>
       </c>
+      <c r="AG3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3682,6 +3688,9 @@
       <c r="AF4" t="n">
         <v>6</v>
       </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3785,6 +3794,9 @@
       <c r="AF5" t="n">
         <v>6</v>
       </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3886,6 +3898,9 @@
         <v>0</v>
       </c>
       <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3961,6 +3976,9 @@
       <c r="AF7" t="n">
         <v>0</v>
       </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4053,6 +4071,9 @@
         <v>0</v>
       </c>
       <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4116,6 +4137,9 @@
       <c r="AF9" t="n">
         <v>3</v>
       </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4210,6 +4234,9 @@
       <c r="AF10" t="n">
         <v>6</v>
       </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4313,6 +4340,9 @@
       <c r="AF11" t="n">
         <v>6</v>
       </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4404,6 +4434,9 @@
       <c r="AF12" t="n">
         <v>0</v>
       </c>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4506,6 +4539,9 @@
       </c>
       <c r="AF13" t="n">
         <v>6</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4585,66 +4621,33 @@
       <c r="AF14" t="n">
         <v>0</v>
       </c>
+      <c r="AG14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C15" s="28">
         <f>ROUND(AVERAGE(D15:AH15), 0)</f>
         <v/>
       </c>
-      <c r="D15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N15" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="O15" t="n">
-        <v>6</v>
-      </c>
-      <c r="P15" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>6</v>
-      </c>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="19" t="n"/>
+      <c r="P15" s="19" t="n"/>
+      <c r="Q15" s="19" t="n"/>
       <c r="R15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>6</v>
@@ -4662,13 +4665,13 @@
         <v>6</v>
       </c>
       <c r="X15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA15" t="n">
         <v>6</v>
@@ -4683,35 +4686,65 @@
         <v>6</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF15" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C16" s="28">
         <f>ROUND(AVERAGE(D16:AH16), 0)</f>
         <v/>
       </c>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="6" t="n"/>
-      <c r="N16" s="6" t="n"/>
-      <c r="O16" s="19" t="n"/>
-      <c r="P16" s="19" t="n"/>
-      <c r="Q16" s="19" t="n"/>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O16" t="n">
+        <v>6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>6</v>
+      </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S16" t="n">
         <v>6</v>
@@ -4726,19 +4759,19 @@
         <v>6</v>
       </c>
       <c r="W16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AA16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB16" t="n">
         <v>6</v>
@@ -4750,16 +4783,19 @@
         <v>6</v>
       </c>
       <c r="AE16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AF16" t="n">
         <v>6</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -4771,11 +4807,20 @@
         <f>ROUND(AVERAGE(D17:AH17), 0)</f>
         <v/>
       </c>
+      <c r="D17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>6</v>
@@ -4784,16 +4829,16 @@
         <v>6</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
         <v>6</v>
@@ -4814,25 +4859,25 @@
         <v>6</v>
       </c>
       <c r="U17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X17" t="n">
         <v>6</v>
       </c>
       <c r="Y17" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z17" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB17" t="n">
         <v>6</v>
@@ -4848,12 +4893,15 @@
       </c>
       <c r="AF17" t="n">
         <v>6</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -4865,20 +4913,11 @@
         <f>ROUND(AVERAGE(D18:AH18), 0)</f>
         <v/>
       </c>
-      <c r="D18" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G18" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>6</v>
@@ -4887,24 +4926,24 @@
         <v>6</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="n">
-        <v>6</v>
-      </c>
-      <c r="P18" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q18" t="n">
+        <v>6</v>
+      </c>
+      <c r="O18" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P18" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q18" s="20" t="n">
         <v>6</v>
       </c>
       <c r="R18" t="n">
@@ -4917,25 +4956,25 @@
         <v>6</v>
       </c>
       <c r="U18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB18" t="n">
         <v>6</v>
@@ -4951,12 +4990,15 @@
       </c>
       <c r="AF18" t="n">
         <v>6</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -4969,7 +5011,7 @@
         <v/>
       </c>
       <c r="G19" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>6</v>
@@ -5020,7 +5062,7 @@
         <v>0</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y19" t="n">
         <v>0</v>
@@ -5038,45 +5080,33 @@
         <v>6</v>
       </c>
       <c r="AD19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AE19" t="n">
         <v>6</v>
       </c>
       <c r="AF19" t="n">
         <v>6</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
-      <c r="G20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J20" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L20" s="6" t="n">
         <v>6</v>
       </c>
@@ -5095,7 +5125,7 @@
       <c r="Q20" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="R20" t="n">
+      <c r="R20" s="20" t="n">
         <v>6</v>
       </c>
       <c r="S20" t="n">
@@ -5114,13 +5144,13 @@
         <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA20" t="n">
         <v>0</v>
@@ -5132,30 +5162,36 @@
         <v>6</v>
       </c>
       <c r="AD20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AE20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C21" s="28">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
+      <c r="K21" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="L21" s="6" t="n">
         <v>6</v>
       </c>
@@ -5190,19 +5226,19 @@
         <v>6</v>
       </c>
       <c r="W21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y21" t="n">
         <v>6</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AA21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB21" t="n">
         <v>6</v>
@@ -5211,30 +5247,54 @@
         <v>6</v>
       </c>
       <c r="AD21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE21" t="n">
         <v>0</v>
       </c>
       <c r="AF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C22" s="28">
         <f>ROUND(AVERAGE(D22:AH22), 0)</f>
         <v/>
       </c>
+      <c r="D22" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K22" s="6" t="n">
         <v>6</v>
       </c>
@@ -5263,29 +5323,29 @@
         <v>6</v>
       </c>
       <c r="T22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V22" t="n">
         <v>6</v>
       </c>
       <c r="W22" t="n">
+        <v>3</v>
+      </c>
+      <c r="X22" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
         <v>4</v>
       </c>
-      <c r="X22" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>2</v>
-      </c>
       <c r="AB22" t="n">
         <v>6</v>
       </c>
@@ -5293,19 +5353,22 @@
         <v>6</v>
       </c>
       <c r="AD22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE22" t="n">
         <v>0</v>
       </c>
       <c r="AF22" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -5318,7 +5381,7 @@
         <v/>
       </c>
       <c r="D23" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E23" s="5" t="n">
         <v>6</v>
@@ -5336,7 +5399,7 @@
         <v>6</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K23" s="6" t="n">
         <v>6</v>
@@ -5362,23 +5425,23 @@
       <c r="R23" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S23" t="n">
+      <c r="S23" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -5387,7 +5450,7 @@
         <v>0</v>
       </c>
       <c r="AA23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB23" t="n">
         <v>6</v>
@@ -5402,13 +5465,16 @@
         <v>0</v>
       </c>
       <c r="AF23" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -5421,7 +5487,7 @@
         <v/>
       </c>
       <c r="D24" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>6</v>
@@ -5439,79 +5505,82 @@
         <v>6</v>
       </c>
       <c r="J24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T24" t="n">
+        <v>6</v>
+      </c>
+      <c r="U24" t="n">
+        <v>6</v>
+      </c>
+      <c r="V24" t="n">
+        <v>6</v>
+      </c>
+      <c r="W24" t="n">
+        <v>6</v>
+      </c>
+      <c r="X24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD24" t="n">
         <v>5</v>
       </c>
-      <c r="K24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T24" t="n">
-        <v>6</v>
-      </c>
-      <c r="U24" t="n">
-        <v>6</v>
-      </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>0</v>
-      </c>
       <c r="AE24" t="n">
         <v>0</v>
       </c>
       <c r="AF24" t="n">
         <v>6</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -5523,27 +5592,7 @@
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
-      <c r="D25" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J25" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n">
         <v>6</v>
       </c>
@@ -5571,50 +5620,53 @@
       <c r="S25" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="T25" t="n">
+      <c r="T25" s="20" t="n">
         <v>6</v>
       </c>
       <c r="U25" t="n">
         <v>6</v>
       </c>
       <c r="V25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X25" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y25" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Z25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB25" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AC25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF25" t="n">
         <v>6</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -5626,7 +5678,18 @@
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
-      <c r="J26" s="6" t="n"/>
+      <c r="G26" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K26" s="6" t="n">
         <v>6</v>
       </c>
@@ -5643,7 +5706,7 @@
         <v>6</v>
       </c>
       <c r="P26" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q26" s="20" t="n">
         <v>6</v>
@@ -5657,26 +5720,26 @@
       <c r="T26" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="U26" t="n">
+      <c r="U26" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V26" t="n">
         <v>0</v>
       </c>
       <c r="W26" t="n">
+        <v>6</v>
+      </c>
+      <c r="X26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="n">
         <v>5</v>
       </c>
-      <c r="X26" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>6</v>
-      </c>
       <c r="AA26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB26" t="n">
         <v>6</v>
@@ -5692,111 +5755,79 @@
       </c>
       <c r="AF26" t="n">
         <v>6</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
         <f>ROUND(AVERAGE(D27:AH27), 0)</f>
         <v/>
       </c>
-      <c r="G27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M27" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N27" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P27" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U27" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V27" t="n">
-        <v>0</v>
-      </c>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="N27" s="6" t="n"/>
+      <c r="O27" s="20" t="n"/>
+      <c r="P27" s="20" t="n"/>
+      <c r="Q27" s="20" t="n"/>
+      <c r="R27" s="20" t="n"/>
+      <c r="S27" s="20" t="n"/>
+      <c r="T27" s="20" t="n"/>
+      <c r="U27" s="20" t="n"/>
       <c r="W27" t="n">
         <v>6</v>
       </c>
       <c r="X27" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y27" t="n">
         <v>0</v>
       </c>
       <c r="Z27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD27" t="n">
         <v>5</v>
       </c>
-      <c r="AA27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>6</v>
-      </c>
       <c r="AE27" t="n">
         <v>6</v>
       </c>
       <c r="AF27" t="n">
         <v>6</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C28" s="28">
@@ -5813,41 +5844,38 @@
       <c r="S28" s="20" t="n"/>
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
-      <c r="W28" t="n">
-        <v>6</v>
-      </c>
-      <c r="X28" t="n">
-        <v>6</v>
-      </c>
       <c r="Y28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA28" t="n">
         <v>6</v>
       </c>
       <c r="AB28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC28" t="n">
         <v>6</v>
       </c>
       <c r="AD28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE28" t="n">
         <v>6</v>
       </c>
       <c r="AF28" t="n">
         <v>6</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
@@ -5870,39 +5898,42 @@
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
       <c r="Y29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC29" t="n">
         <v>6</v>
       </c>
       <c r="AD29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C30" s="28">
@@ -5919,40 +5950,40 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="Y30" t="n">
-        <v>0</v>
-      </c>
       <c r="Z30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC30" t="n">
         <v>6</v>
       </c>
       <c r="AD30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF30" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C31" s="28">
@@ -5969,14 +6000,11 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="Z31" t="n">
-        <v>6</v>
-      </c>
       <c r="AA31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC31" t="n">
         <v>6</v>
@@ -5988,13 +6016,16 @@
         <v>6</v>
       </c>
       <c r="AF31" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -6017,7 +6048,7 @@
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
       <c r="AA32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB32" t="n">
         <v>0</v>
@@ -6026,24 +6057,27 @@
         <v>6</v>
       </c>
       <c r="AD32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C33" s="28">
@@ -6060,34 +6094,34 @@
       <c r="S33" s="20" t="n"/>
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
-      <c r="AA33" t="n">
-        <v>3</v>
-      </c>
       <c r="AB33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC33" t="n">
         <v>6</v>
       </c>
       <c r="AD33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF33" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C34" s="28">
@@ -6104,9 +6138,6 @@
       <c r="S34" s="20" t="n"/>
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
-      <c r="AB34" t="n">
-        <v>6</v>
-      </c>
       <c r="AC34" t="n">
         <v>6</v>
       </c>
@@ -6118,17 +6149,20 @@
       </c>
       <c r="AF34" t="n">
         <v>6</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C35" s="28">
@@ -6152,21 +6186,24 @@
         <v>6</v>
       </c>
       <c r="AE35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C36" s="28">
@@ -6183,28 +6220,28 @@
       <c r="S36" s="20" t="n"/>
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
-      <c r="AC36" t="n">
-        <v>6</v>
-      </c>
       <c r="AD36" t="n">
         <v>6</v>
       </c>
       <c r="AE36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF36" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG36" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C37" s="28">
@@ -6221,20 +6258,20 @@
       <c r="S37" s="20" t="n"/>
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
-      <c r="AD37" t="n">
-        <v>6</v>
-      </c>
       <c r="AE37" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF37" t="n">
         <v>6</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -6262,16 +6299,19 @@
       <c r="AF38" t="n">
         <v>6</v>
       </c>
+      <c r="AG38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C39" s="28">
@@ -6289,21 +6329,24 @@
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
       <c r="AE39" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF39" t="n">
         <v>6</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C40" s="28">
@@ -6321,21 +6364,24 @@
       <c r="T40" s="20" t="n"/>
       <c r="U40" s="20" t="n"/>
       <c r="AE40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF40" t="n">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="AG40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>favretto</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="C41" s="28">
@@ -6352,22 +6398,22 @@
       <c r="S41" s="20" t="n"/>
       <c r="T41" s="20" t="n"/>
       <c r="U41" s="20" t="n"/>
-      <c r="AE41" t="n">
-        <v>6</v>
-      </c>
       <c r="AF41" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="AG41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
         <is>
-          <t>favretto</t>
+          <t>vTrxzys</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>06/06/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="C42" s="28">
@@ -6384,8 +6430,8 @@
       <c r="S42" s="20" t="n"/>
       <c r="T42" s="20" t="n"/>
       <c r="U42" s="20" t="n"/>
-      <c r="AF42" t="n">
-        <v>6</v>
+      <c r="AG42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-14
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3248,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH42"/>
+  <dimension ref="A1:AH39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -4341,7 +4341,7 @@
         <v>6</v>
       </c>
       <c r="AG11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -4435,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -4895,7 +4895,7 @@
         <v>6</v>
       </c>
       <c r="AG17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -4998,33 +4998,18 @@
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C19" s="28">
         <f>ROUND(AVERAGE(D19:AH19), 0)</f>
         <v/>
       </c>
-      <c r="G19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="L19" s="6" t="n">
         <v>6</v>
       </c>
@@ -5043,7 +5028,7 @@
       <c r="Q19" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="R19" t="n">
+      <c r="R19" s="20" t="n">
         <v>6</v>
       </c>
       <c r="S19" t="n">
@@ -5062,13 +5047,13 @@
         <v>0</v>
       </c>
       <c r="X19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA19" t="n">
         <v>0</v>
@@ -5080,13 +5065,13 @@
         <v>6</v>
       </c>
       <c r="AD19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AE19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG19" t="n">
         <v>0</v>
@@ -5095,18 +5080,21 @@
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
         <f>ROUND(AVERAGE(D20:AH20), 0)</f>
         <v/>
       </c>
+      <c r="K20" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="L20" s="6" t="n">
         <v>6</v>
       </c>
@@ -5141,19 +5129,19 @@
         <v>6</v>
       </c>
       <c r="W20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y20" t="n">
         <v>6</v>
       </c>
       <c r="Z20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AA20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB20" t="n">
         <v>6</v>
@@ -5162,7 +5150,7 @@
         <v>6</v>
       </c>
       <c r="AD20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE20" t="n">
         <v>0</v>
@@ -5177,18 +5165,39 @@
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C21" s="28">
         <f>ROUND(AVERAGE(D21:AH21), 0)</f>
         <v/>
       </c>
+      <c r="D21" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K21" s="6" t="n">
         <v>6</v>
       </c>
@@ -5217,29 +5226,29 @@
         <v>6</v>
       </c>
       <c r="T21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V21" t="n">
         <v>6</v>
       </c>
       <c r="W21" t="n">
+        <v>3</v>
+      </c>
+      <c r="X21" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" t="n">
         <v>4</v>
       </c>
-      <c r="X21" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>2</v>
-      </c>
       <c r="AB21" t="n">
         <v>6</v>
       </c>
@@ -5247,22 +5256,22 @@
         <v>6</v>
       </c>
       <c r="AD21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE21" t="n">
         <v>0</v>
       </c>
       <c r="AF21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -5275,7 +5284,7 @@
         <v/>
       </c>
       <c r="D22" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>6</v>
@@ -5293,7 +5302,7 @@
         <v>6</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K22" s="6" t="n">
         <v>6</v>
@@ -5319,56 +5328,56 @@
       <c r="R22" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S22" t="n">
+      <c r="S22" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W22" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG22" t="n">
         <v>3</v>
-      </c>
-      <c r="X22" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>4</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG22" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -5380,89 +5389,69 @@
         <f>ROUND(AVERAGE(D23:AH23), 0)</f>
         <v/>
       </c>
-      <c r="D23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J23" s="6" t="n">
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N23" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T23" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U23" t="n">
+        <v>6</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" t="n">
         <v>5</v>
       </c>
-      <c r="K23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T23" t="n">
-        <v>6</v>
-      </c>
-      <c r="U23" t="n">
-        <v>6</v>
-      </c>
-      <c r="V23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W23" t="n">
-        <v>0</v>
-      </c>
       <c r="X23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB23" t="n">
         <v>6</v>
       </c>
       <c r="AC23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF23" t="n">
         <v>6</v>
@@ -5474,7 +5463,7 @@
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -5486,15 +5475,6 @@
         <f>ROUND(AVERAGE(D24:AH24), 0)</f>
         <v/>
       </c>
-      <c r="D24" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G24" s="5" t="n">
         <v>6</v>
       </c>
@@ -5523,7 +5503,7 @@
         <v>6</v>
       </c>
       <c r="P24" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q24" s="20" t="n">
         <v>6</v>
@@ -5534,41 +5514,41 @@
       <c r="S24" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="T24" t="n">
-        <v>6</v>
-      </c>
-      <c r="U24" t="n">
+      <c r="T24" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U24" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
         <v>6</v>
       </c>
       <c r="X24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA24" t="n">
         <v>0</v>
       </c>
       <c r="AB24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AC24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AD24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF24" t="n">
         <v>6</v>
@@ -5580,78 +5560,51 @@
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
         <f>ROUND(AVERAGE(D25:AH25), 0)</f>
         <v/>
       </c>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L25" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M25" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N25" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T25" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U25" t="n">
-        <v>6</v>
-      </c>
-      <c r="V25" t="n">
-        <v>0</v>
-      </c>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+      <c r="N25" s="6" t="n"/>
+      <c r="O25" s="20" t="n"/>
+      <c r="P25" s="20" t="n"/>
+      <c r="Q25" s="20" t="n"/>
+      <c r="R25" s="20" t="n"/>
+      <c r="S25" s="20" t="n"/>
+      <c r="T25" s="20" t="n"/>
+      <c r="U25" s="20" t="n"/>
       <c r="W25" t="n">
+        <v>6</v>
+      </c>
+      <c r="X25" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD25" t="n">
         <v>5</v>
-      </c>
-      <c r="X25" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>6</v>
       </c>
       <c r="AE25" t="n">
         <v>6</v>
@@ -5666,86 +5619,42 @@
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
         <f>ROUND(AVERAGE(D26:AH26), 0)</f>
         <v/>
       </c>
-      <c r="G26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J26" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K26" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L26" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M26" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N26" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P26" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U26" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V26" t="n">
-        <v>0</v>
-      </c>
-      <c r="W26" t="n">
-        <v>6</v>
-      </c>
-      <c r="X26" t="n">
-        <v>2</v>
-      </c>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="20" t="n"/>
+      <c r="P26" s="20" t="n"/>
+      <c r="Q26" s="20" t="n"/>
+      <c r="R26" s="20" t="n"/>
+      <c r="S26" s="20" t="n"/>
+      <c r="T26" s="20" t="n"/>
+      <c r="U26" s="20" t="n"/>
       <c r="Y26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AA26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB26" t="n">
         <v>6</v>
       </c>
       <c r="AC26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD26" t="n">
         <v>6</v>
@@ -5757,18 +5666,18 @@
         <v>6</v>
       </c>
       <c r="AG26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
@@ -5785,12 +5694,6 @@
       <c r="S27" s="20" t="n"/>
       <c r="T27" s="20" t="n"/>
       <c r="U27" s="20" t="n"/>
-      <c r="W27" t="n">
-        <v>6</v>
-      </c>
-      <c r="X27" t="n">
-        <v>6</v>
-      </c>
       <c r="Y27" t="n">
         <v>0</v>
       </c>
@@ -5798,7 +5701,7 @@
         <v>0</v>
       </c>
       <c r="AA27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB27" t="n">
         <v>0</v>
@@ -5807,27 +5710,27 @@
         <v>6</v>
       </c>
       <c r="AD27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AE27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C28" s="28">
@@ -5844,15 +5747,12 @@
       <c r="S28" s="20" t="n"/>
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
-      <c r="Y28" t="n">
-        <v>6</v>
-      </c>
       <c r="Z28" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA28" t="n">
         <v>3</v>
       </c>
-      <c r="AA28" t="n">
-        <v>6</v>
-      </c>
       <c r="AB28" t="n">
         <v>6</v>
       </c>
@@ -5869,18 +5769,18 @@
         <v>6</v>
       </c>
       <c r="AG28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C29" s="28">
@@ -5897,12 +5797,6 @@
       <c r="S29" s="20" t="n"/>
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
-      <c r="Y29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>0</v>
-      </c>
       <c r="AA29" t="n">
         <v>0</v>
       </c>
@@ -5913,10 +5807,10 @@
         <v>6</v>
       </c>
       <c r="AD29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF29" t="n">
         <v>0</v>
@@ -5928,12 +5822,12 @@
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C30" s="28">
@@ -5950,26 +5844,23 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="Z30" t="n">
-        <v>6</v>
-      </c>
       <c r="AA30" t="n">
         <v>3</v>
       </c>
       <c r="AB30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC30" t="n">
         <v>6</v>
       </c>
       <c r="AD30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG30" t="n">
         <v>0</v>
@@ -5978,12 +5869,12 @@
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C31" s="28">
@@ -6000,11 +5891,8 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="AA31" t="n">
-        <v>0</v>
-      </c>
       <c r="AB31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC31" t="n">
         <v>6</v>
@@ -6016,7 +5904,7 @@
         <v>6</v>
       </c>
       <c r="AF31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG31" t="n">
         <v>0</v>
@@ -6025,12 +5913,12 @@
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C32" s="28">
@@ -6047,37 +5935,31 @@
       <c r="S32" s="20" t="n"/>
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
-      <c r="AA32" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB32" t="n">
-        <v>0</v>
-      </c>
       <c r="AC32" t="n">
         <v>6</v>
       </c>
       <c r="AD32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C33" s="28">
@@ -6094,9 +5976,6 @@
       <c r="S33" s="20" t="n"/>
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
-      <c r="AB33" t="n">
-        <v>6</v>
-      </c>
       <c r="AC33" t="n">
         <v>6</v>
       </c>
@@ -6104,10 +5983,10 @@
         <v>6</v>
       </c>
       <c r="AE33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG33" t="n">
         <v>0</v>
@@ -6116,12 +5995,12 @@
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C34" s="28">
@@ -6138,31 +6017,28 @@
       <c r="S34" s="20" t="n"/>
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
-      <c r="AC34" t="n">
-        <v>6</v>
-      </c>
       <c r="AD34" t="n">
         <v>6</v>
       </c>
       <c r="AE34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AF34" t="n">
         <v>6</v>
       </c>
       <c r="AG34" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C35" s="28">
@@ -6179,17 +6055,11 @@
       <c r="S35" s="20" t="n"/>
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
-      <c r="AC35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>6</v>
-      </c>
       <c r="AE35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -6198,12 +6068,12 @@
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C36" s="28">
@@ -6220,11 +6090,8 @@
       <c r="S36" s="20" t="n"/>
       <c r="T36" s="20" t="n"/>
       <c r="U36" s="20" t="n"/>
-      <c r="AD36" t="n">
-        <v>6</v>
-      </c>
       <c r="AE36" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF36" t="n">
         <v>6</v>
@@ -6236,12 +6103,12 @@
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C37" s="28">
@@ -6259,7 +6126,7 @@
       <c r="T37" s="20" t="n"/>
       <c r="U37" s="20" t="n"/>
       <c r="AE37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF37" t="n">
         <v>6</v>
@@ -6271,12 +6138,12 @@
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C38" s="28">
@@ -6297,7 +6164,7 @@
         <v>6</v>
       </c>
       <c r="AF38" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG38" t="n">
         <v>0</v>
@@ -6306,12 +6173,12 @@
     <row r="39">
       <c r="A39" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>vTrxzys</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="C39" s="28">
@@ -6328,109 +6195,7 @@
       <c r="S39" s="20" t="n"/>
       <c r="T39" s="20" t="n"/>
       <c r="U39" s="20" t="n"/>
-      <c r="AE39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF39" t="n">
-        <v>6</v>
-      </c>
       <c r="AG39" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="28" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
-      <c r="C40" s="28">
-        <f>ROUND(AVERAGE(D40:AH40), 0)</f>
-        <v/>
-      </c>
-      <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
-      <c r="N40" s="6" t="n"/>
-      <c r="O40" s="20" t="n"/>
-      <c r="P40" s="20" t="n"/>
-      <c r="Q40" s="20" t="n"/>
-      <c r="R40" s="20" t="n"/>
-      <c r="S40" s="20" t="n"/>
-      <c r="T40" s="20" t="n"/>
-      <c r="U40" s="20" t="n"/>
-      <c r="AE40" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="28" t="inlineStr">
-        <is>
-          <t>favretto</t>
-        </is>
-      </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>06/06/2026</t>
-        </is>
-      </c>
-      <c r="C41" s="28">
-        <f>ROUND(AVERAGE(D41:AH41), 0)</f>
-        <v/>
-      </c>
-      <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
-      <c r="N41" s="6" t="n"/>
-      <c r="O41" s="20" t="n"/>
-      <c r="P41" s="20" t="n"/>
-      <c r="Q41" s="20" t="n"/>
-      <c r="R41" s="20" t="n"/>
-      <c r="S41" s="20" t="n"/>
-      <c r="T41" s="20" t="n"/>
-      <c r="U41" s="20" t="n"/>
-      <c r="AF41" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="28" t="inlineStr">
-        <is>
-          <t>vTrxzys</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="inlineStr">
-        <is>
-          <t>13/06/2026</t>
-        </is>
-      </c>
-      <c r="C42" s="28">
-        <f>ROUND(AVERAGE(D42:AH42), 0)</f>
-        <v/>
-      </c>
-      <c r="K42" s="6" t="n"/>
-      <c r="L42" s="6" t="n"/>
-      <c r="N42" s="6" t="n"/>
-      <c r="O42" s="20" t="n"/>
-      <c r="P42" s="20" t="n"/>
-      <c r="Q42" s="20" t="n"/>
-      <c r="R42" s="20" t="n"/>
-      <c r="S42" s="20" t="n"/>
-      <c r="T42" s="20" t="n"/>
-      <c r="U42" s="20" t="n"/>
-      <c r="AG42" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-15
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3795,7 +3795,7 @@
         <v>6</v>
       </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4541,7 +4541,7 @@
         <v>6</v>
       </c>
       <c r="AG13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -5371,7 +5371,7 @@
         <v>6</v>
       </c>
       <c r="AG22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -5457,7 +5457,7 @@
         <v>6</v>
       </c>
       <c r="AG23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -5769,7 +5769,7 @@
         <v>6</v>
       </c>
       <c r="AG28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29">
@@ -5907,7 +5907,7 @@
         <v>6</v>
       </c>
       <c r="AG31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -6027,7 +6027,7 @@
         <v>6</v>
       </c>
       <c r="AG34" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-20
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -3248,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH39"/>
+  <dimension ref="A1:AH38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="AH1" s="3" t="inlineStr">
         <is>
-          <t>Colonna32</t>
+          <t>19/06/2026</t>
         </is>
       </c>
     </row>
@@ -3518,6 +3518,9 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3594,6 +3597,9 @@
       <c r="AG3" t="n">
         <v>6</v>
       </c>
+      <c r="AH3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3691,6 +3697,9 @@
       <c r="AG4" t="n">
         <v>0</v>
       </c>
+      <c r="AH4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3797,6 +3806,9 @@
       <c r="AG5" t="n">
         <v>6</v>
       </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3901,6 +3913,9 @@
         <v>0</v>
       </c>
       <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3979,6 +3994,9 @@
       <c r="AG7" t="n">
         <v>0</v>
       </c>
+      <c r="AH7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4075,6 +4093,9 @@
       </c>
       <c r="AG8" t="n">
         <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -4140,6 +4161,9 @@
       <c r="AG9" t="n">
         <v>0</v>
       </c>
+      <c r="AH9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4237,6 +4261,9 @@
       <c r="AG10" t="n">
         <v>0</v>
       </c>
+      <c r="AH10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4343,6 +4370,9 @@
       <c r="AG11" t="n">
         <v>6</v>
       </c>
+      <c r="AH11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4437,6 +4467,9 @@
       <c r="AG12" t="n">
         <v>6</v>
       </c>
+      <c r="AH12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4542,6 +4575,9 @@
       </c>
       <c r="AG13" t="n">
         <v>6</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4623,6 +4659,9 @@
       </c>
       <c r="AG14" t="n">
         <v>0</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -4694,6 +4733,9 @@
       <c r="AG15" t="n">
         <v>6</v>
       </c>
+      <c r="AH15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4791,6 +4833,9 @@
       <c r="AG16" t="n">
         <v>6</v>
       </c>
+      <c r="AH16" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4897,6 +4942,9 @@
       <c r="AG17" t="n">
         <v>6</v>
       </c>
+      <c r="AH17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4994,6 +5042,9 @@
       <c r="AG18" t="n">
         <v>0</v>
       </c>
+      <c r="AH18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5076,6 +5127,9 @@
       <c r="AG19" t="n">
         <v>0</v>
       </c>
+      <c r="AH19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5161,6 +5215,9 @@
       <c r="AG20" t="n">
         <v>0</v>
       </c>
+      <c r="AH20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5267,6 +5324,9 @@
       <c r="AG21" t="n">
         <v>6</v>
       </c>
+      <c r="AH21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5373,6 +5433,9 @@
       <c r="AG22" t="n">
         <v>6</v>
       </c>
+      <c r="AH22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5459,6 +5522,9 @@
       <c r="AG23" t="n">
         <v>6</v>
       </c>
+      <c r="AH23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5555,6 +5621,9 @@
       </c>
       <c r="AG24" t="n">
         <v>0</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -5615,6 +5684,9 @@
       <c r="AG25" t="n">
         <v>0</v>
       </c>
+      <c r="AH25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5668,6 +5740,9 @@
       <c r="AG26" t="n">
         <v>6</v>
       </c>
+      <c r="AH26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5721,6 +5796,9 @@
       <c r="AG27" t="n">
         <v>6</v>
       </c>
+      <c r="AH27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -5771,6 +5849,9 @@
       <c r="AG28" t="n">
         <v>6</v>
       </c>
+      <c r="AH28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -5817,6 +5898,9 @@
       </c>
       <c r="AG29" t="n">
         <v>6</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -5865,6 +5949,9 @@
       <c r="AG30" t="n">
         <v>0</v>
       </c>
+      <c r="AH30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -5909,6 +5996,9 @@
       <c r="AG31" t="n">
         <v>6</v>
       </c>
+      <c r="AH31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -5950,6 +6040,9 @@
       <c r="AG32" t="n">
         <v>6</v>
       </c>
+      <c r="AH32" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -5991,6 +6084,9 @@
       <c r="AG33" t="n">
         <v>0</v>
       </c>
+      <c r="AH33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -6029,6 +6125,9 @@
       <c r="AG34" t="n">
         <v>6</v>
       </c>
+      <c r="AH34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -6064,6 +6163,9 @@
       <c r="AG35" t="n">
         <v>0</v>
       </c>
+      <c r="AH35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -6099,6 +6201,9 @@
       <c r="AG36" t="n">
         <v>0</v>
       </c>
+      <c r="AH36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
@@ -6134,6 +6239,9 @@
       <c r="AG37" t="n">
         <v>0</v>
       </c>
+      <c r="AH37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
@@ -6169,33 +6277,7 @@
       <c r="AG38" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="28" t="inlineStr">
-        <is>
-          <t>vTrxzys</t>
-        </is>
-      </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>13/06/2026</t>
-        </is>
-      </c>
-      <c r="C39" s="28">
-        <f>ROUND(AVERAGE(D39:AH39), 0)</f>
-        <v/>
-      </c>
-      <c r="K39" s="6" t="n"/>
-      <c r="L39" s="6" t="n"/>
-      <c r="N39" s="6" t="n"/>
-      <c r="O39" s="20" t="n"/>
-      <c r="P39" s="20" t="n"/>
-      <c r="Q39" s="20" t="n"/>
-      <c r="R39" s="20" t="n"/>
-      <c r="S39" s="20" t="n"/>
-      <c r="T39" s="20" t="n"/>
-      <c r="U39" s="20" t="n"/>
-      <c r="AG39" t="n">
+      <c r="AH38" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH51"/>
+  <dimension ref="A1:AH38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -1028,12 +1028,12 @@
     <row r="4" ht="16.5" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/03/2026</t>
         </is>
       </c>
       <c r="C4" s="12">
@@ -1045,21 +1045,13 @@
         <v/>
       </c>
       <c r="E4" s="14" t="n">
-        <v>82800</v>
+        <v>35700</v>
       </c>
       <c r="F4" s="13" t="n"/>
-      <c r="G4" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H4" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I4" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="G4" s="13" t="n"/>
+      <c r="H4" s="13" t="n"/>
+      <c r="I4" s="13" t="n"/>
+      <c r="J4" s="13" t="n"/>
       <c r="K4" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1080,12 +1072,12 @@
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C5" s="12">
@@ -1097,13 +1089,19 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>35700</v>
+        <v>90500</v>
       </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
-      <c r="I5" s="13" t="n"/>
-      <c r="J5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="K5" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1124,12 +1122,12 @@
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C6" s="12">
@@ -1141,13 +1139,11 @@
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>90500</v>
+        <v>135225</v>
       </c>
       <c r="F6" s="13" t="n"/>
       <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H6" s="13" t="n"/>
       <c r="I6" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1174,7 +1170,7 @@
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
@@ -1191,21 +1187,21 @@
         <v/>
       </c>
       <c r="E7" s="14" t="n">
-        <v>82100</v>
+        <v>126020</v>
       </c>
       <c r="F7" s="13" t="n"/>
       <c r="G7" s="13" t="n"/>
       <c r="H7" s="13" t="n">
-        <v>10000</v>
+        <v>3850</v>
       </c>
       <c r="I7" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>10000</v>
+        <v>8800</v>
       </c>
       <c r="L7" s="13" t="n">
         <v>10000</v>
@@ -1224,12 +1220,12 @@
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C8" s="12">
@@ -1241,11 +1237,13 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>135225</v>
+        <v>78550</v>
       </c>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n"/>
+      <c r="H8" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="I8" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1253,7 +1251,7 @@
         <v>10000</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>10000</v>
+        <v>8600</v>
       </c>
       <c r="L8" s="13" t="n">
         <v>10000</v>
@@ -1272,7 +1270,7 @@
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
@@ -1289,21 +1287,23 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>126020</v>
+        <v>42250</v>
       </c>
       <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
+      <c r="G9" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H9" s="13" t="n">
-        <v>3850</v>
+        <v>10000</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0</v>
+        <v>4300</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>8800</v>
+        <v>6300</v>
       </c>
       <c r="L9" s="13" t="n">
         <v>10000</v>
@@ -1314,7 +1314,7 @@
       <c r="P9" s="13" t="n"/>
       <c r="Q9" s="13" t="n"/>
       <c r="R9" s="13" t="n"/>
-      <c r="S9" s="13" t="n"/>
+      <c r="S9" s="21" t="n"/>
       <c r="T9" s="13" t="n"/>
       <c r="U9" s="13" t="n"/>
       <c r="V9" s="13" t="n"/>
@@ -1322,12 +1322,12 @@
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C10" s="12">
@@ -1339,21 +1339,17 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>78550</v>
+        <v>93950</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I10" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
       <c r="J10" s="13" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>8600</v>
+        <v>6100</v>
       </c>
       <c r="L10" s="13" t="n">
         <v>10000</v>
@@ -1364,7 +1360,7 @@
       <c r="P10" s="13" t="n"/>
       <c r="Q10" s="13" t="n"/>
       <c r="R10" s="13" t="n"/>
-      <c r="S10" s="13" t="n"/>
+      <c r="S10" s="21" t="n"/>
       <c r="T10" s="13" t="n"/>
       <c r="U10" s="13" t="n"/>
       <c r="V10" s="13" t="n"/>
@@ -1372,7 +1368,7 @@
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -1389,26 +1385,26 @@
         <v/>
       </c>
       <c r="E11" s="14" t="n">
-        <v>42250</v>
+        <v>18350</v>
       </c>
       <c r="F11" s="13" t="n"/>
       <c r="G11" s="13" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>4300</v>
+        <v>0</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>6300</v>
+        <v>6100</v>
       </c>
       <c r="L11" s="13" t="n">
-        <v>10000</v>
+        <v>6100</v>
       </c>
       <c r="M11" s="13" t="n"/>
       <c r="N11" s="13" t="n"/>
@@ -1424,12 +1420,12 @@
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C12" s="12">
@@ -1441,17 +1437,25 @@
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>93950</v>
-      </c>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="13" t="n"/>
+        <v>50600</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>2450</v>
+      </c>
       <c r="J12" s="13" t="n">
-        <v>5000</v>
+        <v>4050</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>6100</v>
+        <v>4650</v>
       </c>
       <c r="L12" s="13" t="n">
         <v>10000</v>
@@ -1470,7 +1474,7 @@
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
@@ -1487,26 +1491,28 @@
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>18350</v>
-      </c>
-      <c r="F13" s="13" t="n"/>
+        <v>45700</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G13" s="13" t="n">
-        <v>0</v>
+        <v>2100</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>0</v>
+        <v>5800</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>0</v>
+        <v>4350</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>6100</v>
+        <v>4600</v>
       </c>
       <c r="L13" s="13" t="n">
-        <v>6100</v>
+        <v>10000</v>
       </c>
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="13" t="n"/>
@@ -1522,12 +1528,12 @@
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C14" s="12">
@@ -1539,28 +1545,22 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>42675</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G14" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H14" s="13" t="n">
-        <v>4050</v>
-      </c>
+        <v>53000</v>
+      </c>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
       <c r="I14" s="13" t="n">
-        <v>4850</v>
+        <v>4300</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>4000</v>
+        <v>4100</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>5050</v>
+        <v>4200</v>
       </c>
       <c r="L14" s="13" t="n">
-        <v>9650</v>
+        <v>8450</v>
       </c>
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="13" t="n"/>
@@ -1576,7 +1576,7 @@
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
@@ -1593,7 +1593,7 @@
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>50600</v>
+        <v>41500</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>4000</v>
@@ -1602,19 +1602,19 @@
         <v>4000</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>10000</v>
+        <v>4100</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>2450</v>
+        <v>4400</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>4050</v>
+        <v>4700</v>
       </c>
       <c r="K15" s="13" t="n">
-        <v>4650</v>
+        <v>4150</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>10000</v>
+        <v>9300</v>
       </c>
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="13" t="n"/>
@@ -1630,12 +1630,12 @@
     <row r="16" ht="16.5" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C16" s="12">
@@ -1647,28 +1647,24 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>45700</v>
-      </c>
-      <c r="F16" s="13" t="n">
+        <v>137200</v>
+      </c>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J16" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H16" s="13" t="n">
-        <v>5800</v>
-      </c>
-      <c r="I16" s="13" t="n">
-        <v>4050</v>
-      </c>
-      <c r="J16" s="13" t="n">
-        <v>4350</v>
-      </c>
       <c r="K16" s="13" t="n">
-        <v>4600</v>
+        <v>4100</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>10000</v>
+        <v>13400</v>
       </c>
       <c r="M16" s="13" t="n"/>
       <c r="N16" s="13" t="n"/>
@@ -1684,12 +1680,12 @@
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C17" s="12">
@@ -1701,22 +1697,24 @@
         <v/>
       </c>
       <c r="E17" s="14" t="n">
-        <v>53000</v>
+        <v>47650</v>
       </c>
       <c r="F17" s="13" t="n"/>
       <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
+      <c r="H17" s="13" t="n">
+        <v>1200</v>
+      </c>
       <c r="I17" s="13" t="n">
-        <v>4300</v>
+        <v>4000</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>4100</v>
+        <v>150</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>4200</v>
+        <v>4050</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>8450</v>
+        <v>6650</v>
       </c>
       <c r="M17" s="13" t="n"/>
       <c r="N17" s="13" t="n"/>
@@ -1732,7 +1730,7 @@
     <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
@@ -1749,28 +1747,24 @@
         <v/>
       </c>
       <c r="E18" s="14" t="n">
-        <v>41500</v>
-      </c>
-      <c r="F18" s="13" t="n">
+        <v>41400</v>
+      </c>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="K18" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H18" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I18" s="13" t="n">
-        <v>4400</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>4700</v>
-      </c>
-      <c r="K18" s="13" t="n">
-        <v>4150</v>
-      </c>
       <c r="L18" s="13" t="n">
-        <v>9300</v>
+        <v>10000</v>
       </c>
       <c r="M18" s="13" t="n"/>
       <c r="N18" s="13" t="n"/>
@@ -1786,12 +1780,12 @@
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C19" s="12">
@@ -1803,24 +1797,28 @@
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>137200</v>
-      </c>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="13" t="n"/>
+        <v>49250</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H19" s="13" t="n">
         <v>4050</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>4100</v>
+        <v>5600</v>
       </c>
       <c r="J19" s="13" t="n">
-        <v>4000</v>
+        <v>1300</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>4100</v>
+        <v>3100</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>13400</v>
+        <v>9350</v>
       </c>
       <c r="M19" s="13" t="n"/>
       <c r="N19" s="13" t="n"/>
@@ -1836,7 +1834,7 @@
     <row r="20" ht="16.5" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
@@ -1853,24 +1851,24 @@
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>47650</v>
+        <v>44225</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n">
-        <v>1200</v>
+        <v>3650</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>4000</v>
+        <v>7600</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>150</v>
+        <v>3150</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>4050</v>
+        <v>3000</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>6650</v>
+        <v>10000</v>
       </c>
       <c r="M20" s="13" t="n"/>
       <c r="N20" s="13" t="n"/>
@@ -1886,12 +1884,12 @@
     <row r="21" ht="16.5" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C21" s="12">
@@ -1903,24 +1901,22 @@
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>41400</v>
+        <v>77200</v>
       </c>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H21" s="13" t="n"/>
       <c r="I21" s="13" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="J21" s="13" t="n">
-        <v>4050</v>
+        <v>950</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>4000</v>
+        <v>1400</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>10000</v>
+        <v>2200</v>
       </c>
       <c r="M21" s="13" t="n"/>
       <c r="N21" s="13" t="n"/>
@@ -1936,12 +1932,12 @@
     <row r="22" ht="16.5" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C22" s="12">
@@ -1953,28 +1949,22 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>49250</v>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G22" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H22" s="13" t="n">
-        <v>4050</v>
-      </c>
+        <v>7850</v>
+      </c>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
       <c r="I22" s="13" t="n">
-        <v>5600</v>
+        <v>4150</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>1300</v>
+        <v>2650</v>
       </c>
       <c r="K22" s="13" t="n">
-        <v>3100</v>
+        <v>1050</v>
       </c>
       <c r="L22" s="13" t="n">
-        <v>9350</v>
+        <v>1050</v>
       </c>
       <c r="M22" s="13" t="n"/>
       <c r="N22" s="13" t="n"/>
@@ -1982,7 +1972,7 @@
       <c r="P22" s="13" t="n"/>
       <c r="Q22" s="13" t="n"/>
       <c r="R22" s="13" t="n"/>
-      <c r="S22" s="21" t="n"/>
+      <c r="S22" s="13" t="n"/>
       <c r="T22" s="13" t="n"/>
       <c r="U22" s="13" t="n"/>
       <c r="V22" s="13" t="n"/>
@@ -1990,12 +1980,12 @@
     <row r="23" ht="16.5" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C23" s="12">
@@ -2007,24 +1997,18 @@
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>44225</v>
+        <v>19100</v>
       </c>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n">
-        <v>3650</v>
-      </c>
-      <c r="I23" s="13" t="n">
-        <v>7600</v>
-      </c>
-      <c r="J23" s="13" t="n">
-        <v>3150</v>
-      </c>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
       <c r="K23" s="13" t="n">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>10000</v>
+        <v>1100</v>
       </c>
       <c r="M23" s="13" t="n"/>
       <c r="N23" s="13" t="n"/>
@@ -2032,7 +2016,7 @@
       <c r="P23" s="13" t="n"/>
       <c r="Q23" s="13" t="n"/>
       <c r="R23" s="13" t="n"/>
-      <c r="S23" s="21" t="n"/>
+      <c r="S23" s="13" t="n"/>
       <c r="T23" s="13" t="n"/>
       <c r="U23" s="13" t="n"/>
       <c r="V23" s="13" t="n"/>
@@ -2040,12 +2024,12 @@
     <row r="24" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C24" s="12">
@@ -2057,22 +2041,24 @@
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>77200</v>
+        <v>17200</v>
       </c>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
+      <c r="H24" s="13" t="n">
+        <v>500</v>
+      </c>
       <c r="I24" s="13" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="J24" s="13" t="n">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="K24" s="13" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="L24" s="13" t="n">
-        <v>2200</v>
+        <v>2050</v>
       </c>
       <c r="M24" s="13" t="n"/>
       <c r="N24" s="13" t="n"/>
@@ -2080,7 +2066,7 @@
       <c r="P24" s="13" t="n"/>
       <c r="Q24" s="13" t="n"/>
       <c r="R24" s="13" t="n"/>
-      <c r="S24" s="21" t="n"/>
+      <c r="S24" s="13" t="n"/>
       <c r="T24" s="13" t="n"/>
       <c r="U24" s="13" t="n"/>
       <c r="V24" s="13" t="n"/>
@@ -2088,12 +2074,12 @@
     <row r="25" ht="16.5" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C25" s="12">
@@ -2105,22 +2091,16 @@
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>7850</v>
+        <v>13725</v>
       </c>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n"/>
-      <c r="I25" s="13" t="n">
-        <v>4150</v>
-      </c>
-      <c r="J25" s="13" t="n">
-        <v>2650</v>
-      </c>
-      <c r="K25" s="13" t="n">
-        <v>1050</v>
-      </c>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
       <c r="L25" s="13" t="n">
-        <v>1050</v>
+        <v>600</v>
       </c>
       <c r="M25" s="13" t="n"/>
       <c r="N25" s="13" t="n"/>
@@ -2136,12 +2116,12 @@
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C26" s="12">
@@ -2153,18 +2133,16 @@
         <v/>
       </c>
       <c r="E26" s="14" t="n">
-        <v>19100</v>
+        <v>11550</v>
       </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
       <c r="H26" s="13" t="n"/>
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="13" t="n"/>
-      <c r="K26" s="13" t="n">
-        <v>600</v>
-      </c>
+      <c r="K26" s="13" t="n"/>
       <c r="L26" s="13" t="n">
-        <v>1100</v>
+        <v>300</v>
       </c>
       <c r="M26" s="13" t="n"/>
       <c r="N26" s="13" t="n"/>
@@ -2180,12 +2158,12 @@
     <row r="27" ht="16.5" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C27" s="12">
@@ -2197,24 +2175,16 @@
         <v/>
       </c>
       <c r="E27" s="14" t="n">
-        <v>17200</v>
+        <v>51290</v>
       </c>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="I27" s="13" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
       <c r="L27" s="13" t="n">
-        <v>2050</v>
+        <v>10650</v>
       </c>
       <c r="M27" s="13" t="n"/>
       <c r="N27" s="13" t="n"/>
@@ -2230,12 +2200,12 @@
     <row r="28" ht="16.5" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C28" s="12">
@@ -2247,7 +2217,7 @@
         <v/>
       </c>
       <c r="E28" s="14" t="n">
-        <v>13725</v>
+        <v>60600</v>
       </c>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
@@ -2256,7 +2226,7 @@
       <c r="J28" s="13" t="n"/>
       <c r="K28" s="13" t="n"/>
       <c r="L28" s="13" t="n">
-        <v>600</v>
+        <v>4400</v>
       </c>
       <c r="M28" s="13" t="n"/>
       <c r="N28" s="13" t="n"/>
@@ -2272,12 +2242,12 @@
     <row r="29" ht="16.5" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C29" s="12">
@@ -2289,7 +2259,7 @@
         <v/>
       </c>
       <c r="E29" s="14" t="n">
-        <v>11550</v>
+        <v>44150</v>
       </c>
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="13" t="n"/>
@@ -2298,7 +2268,7 @@
       <c r="J29" s="13" t="n"/>
       <c r="K29" s="13" t="n"/>
       <c r="L29" s="13" t="n">
-        <v>300</v>
+        <v>4500</v>
       </c>
       <c r="M29" s="13" t="n"/>
       <c r="N29" s="13" t="n"/>
@@ -2314,12 +2284,12 @@
     <row r="30" ht="16.5" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C30" s="12">
@@ -2331,7 +2301,7 @@
         <v/>
       </c>
       <c r="E30" s="14" t="n">
-        <v>51290</v>
+        <v>114425</v>
       </c>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
@@ -2340,7 +2310,7 @@
       <c r="J30" s="13" t="n"/>
       <c r="K30" s="13" t="n"/>
       <c r="L30" s="13" t="n">
-        <v>10650</v>
+        <v>4100</v>
       </c>
       <c r="M30" s="13" t="n"/>
       <c r="N30" s="13" t="n"/>
@@ -2356,7 +2326,7 @@
     <row r="31" ht="16.5" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
@@ -2373,7 +2343,7 @@
         <v/>
       </c>
       <c r="E31" s="14" t="n">
-        <v>60600</v>
+        <v>43210</v>
       </c>
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="13" t="n"/>
@@ -2382,7 +2352,7 @@
       <c r="J31" s="13" t="n"/>
       <c r="K31" s="13" t="n"/>
       <c r="L31" s="13" t="n">
-        <v>4400</v>
+        <v>10000</v>
       </c>
       <c r="M31" s="13" t="n"/>
       <c r="N31" s="13" t="n"/>
@@ -2398,12 +2368,12 @@
     <row r="32" ht="16.5" customHeight="1">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C32" s="12">
@@ -2415,7 +2385,7 @@
         <v/>
       </c>
       <c r="E32" s="14" t="n">
-        <v>44150</v>
+        <v>0</v>
       </c>
       <c r="F32" s="13" t="n"/>
       <c r="G32" s="13" t="n"/>
@@ -2424,7 +2394,7 @@
       <c r="J32" s="13" t="n"/>
       <c r="K32" s="13" t="n"/>
       <c r="L32" s="13" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="M32" s="13" t="n"/>
       <c r="N32" s="13" t="n"/>
@@ -2440,12 +2410,12 @@
     <row r="33" ht="16.5" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C33" s="12">
@@ -2457,7 +2427,7 @@
         <v/>
       </c>
       <c r="E33" s="14" t="n">
-        <v>42850</v>
+        <v>47025</v>
       </c>
       <c r="F33" s="13" t="n"/>
       <c r="G33" s="13" t="n"/>
@@ -2466,7 +2436,7 @@
       <c r="J33" s="13" t="n"/>
       <c r="K33" s="13" t="n"/>
       <c r="L33" s="13" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="M33" s="13" t="n"/>
       <c r="N33" s="13" t="n"/>
@@ -2482,12 +2452,12 @@
     <row r="34" ht="16.5" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C34" s="12">
@@ -2499,7 +2469,7 @@
         <v/>
       </c>
       <c r="E34" s="14" t="n">
-        <v>29860</v>
+        <v>44100</v>
       </c>
       <c r="F34" s="13" t="n"/>
       <c r="G34" s="13" t="n"/>
@@ -2508,7 +2478,7 @@
       <c r="J34" s="13" t="n"/>
       <c r="K34" s="13" t="n"/>
       <c r="L34" s="13" t="n">
-        <v>4050</v>
+        <v>4200</v>
       </c>
       <c r="M34" s="13" t="n"/>
       <c r="N34" s="13" t="n"/>
@@ -2524,12 +2494,12 @@
     <row r="35" ht="16.5" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="C35" s="12">
@@ -2541,7 +2511,7 @@
         <v/>
       </c>
       <c r="E35" s="14" t="n">
-        <v>114425</v>
+        <v>99900</v>
       </c>
       <c r="F35" s="13" t="n"/>
       <c r="G35" s="13" t="n"/>
@@ -2550,7 +2520,7 @@
       <c r="J35" s="13" t="n"/>
       <c r="K35" s="13" t="n"/>
       <c r="L35" s="13" t="n">
-        <v>4100</v>
+        <v>9500</v>
       </c>
       <c r="M35" s="13" t="n"/>
       <c r="N35" s="13" t="n"/>
@@ -2566,12 +2536,12 @@
     <row r="36" ht="16.5" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="C36" s="12">
@@ -2583,7 +2553,7 @@
         <v/>
       </c>
       <c r="E36" s="14" t="n">
-        <v>43210</v>
+        <v>28450</v>
       </c>
       <c r="F36" s="13" t="n"/>
       <c r="G36" s="13" t="n"/>
@@ -2592,7 +2562,7 @@
       <c r="J36" s="13" t="n"/>
       <c r="K36" s="13" t="n"/>
       <c r="L36" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="M36" s="13" t="n"/>
       <c r="N36" s="13" t="n"/>
@@ -2608,12 +2578,12 @@
     <row r="37" ht="16.5" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C37" s="12">
@@ -2625,7 +2595,7 @@
         <v/>
       </c>
       <c r="E37" s="14" t="n">
-        <v>123225</v>
+        <v>13250</v>
       </c>
       <c r="F37" s="13" t="n"/>
       <c r="G37" s="13" t="n"/>
@@ -2633,9 +2603,7 @@
       <c r="I37" s="13" t="n"/>
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
-      <c r="L37" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="L37" s="13" t="n"/>
       <c r="M37" s="13" t="n"/>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
@@ -2650,12 +2618,12 @@
     <row r="38" ht="16.5" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C38" s="12">
@@ -2667,7 +2635,7 @@
         <v/>
       </c>
       <c r="E38" s="14" t="n">
-        <v>0</v>
+        <v>150440</v>
       </c>
       <c r="F38" s="13" t="n"/>
       <c r="G38" s="13" t="n"/>
@@ -2675,9 +2643,7 @@
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="L38" s="13" t="n"/>
       <c r="M38" s="13" t="n"/>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
@@ -2689,552 +2655,19 @@
       <c r="U38" s="13" t="n"/>
       <c r="V38" s="13" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>KAIZERS</t>
-        </is>
-      </c>
-      <c r="B39" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C39" s="12">
-        <f>ROUND(AVERAGE(F39:AI39), 0)</f>
-        <v/>
-      </c>
-      <c r="D39" s="1">
-        <f>SUM(F39:AI39)</f>
-        <v/>
-      </c>
-      <c r="E39" s="14" t="n">
-        <v>47025</v>
-      </c>
-      <c r="F39" s="13" t="n"/>
-      <c r="G39" s="13" t="n"/>
-      <c r="H39" s="13" t="n"/>
-      <c r="I39" s="13" t="n"/>
-      <c r="J39" s="13" t="n"/>
-      <c r="K39" s="13" t="n"/>
-      <c r="L39" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="M39" s="13" t="n"/>
-      <c r="N39" s="13" t="n"/>
-      <c r="O39" s="13" t="n"/>
-      <c r="P39" s="13" t="n"/>
-      <c r="Q39" s="13" t="n"/>
-      <c r="R39" s="13" t="n"/>
-      <c r="S39" s="13" t="n"/>
-      <c r="T39" s="13" t="n"/>
-      <c r="U39" s="13" t="n"/>
-      <c r="V39" s="13" t="n"/>
-    </row>
-    <row r="40" ht="16.5" customHeight="1">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>Frost Walker</t>
-        </is>
-      </c>
-      <c r="B40" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C40" s="12">
-        <f>ROUND(AVERAGE(F40:AI40), 0)</f>
-        <v/>
-      </c>
-      <c r="D40" s="1">
-        <f>SUM(F40:AI40)</f>
-        <v/>
-      </c>
-      <c r="E40" s="14" t="n">
-        <v>30615</v>
-      </c>
-      <c r="F40" s="13" t="n"/>
-      <c r="G40" s="13" t="n"/>
-      <c r="H40" s="13" t="n"/>
-      <c r="I40" s="13" t="n"/>
-      <c r="J40" s="13" t="n"/>
-      <c r="K40" s="13" t="n"/>
-      <c r="L40" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" s="13" t="n"/>
-      <c r="N40" s="13" t="n"/>
-      <c r="O40" s="13" t="n"/>
-      <c r="P40" s="13" t="n"/>
-      <c r="Q40" s="13" t="n"/>
-      <c r="R40" s="13" t="n"/>
-      <c r="S40" s="13" t="n"/>
-      <c r="T40" s="13" t="n"/>
-      <c r="U40" s="13" t="n"/>
-      <c r="V40" s="13" t="n"/>
-    </row>
-    <row r="41" ht="16.5" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>roberto</t>
-        </is>
-      </c>
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C41" s="12">
-        <f>ROUND(AVERAGE(F41:AI41), 0)</f>
-        <v/>
-      </c>
-      <c r="D41" s="1">
-        <f>SUM(F41:AI41)</f>
-        <v/>
-      </c>
-      <c r="E41" s="14" t="n">
-        <v>44100</v>
-      </c>
-      <c r="F41" s="13" t="n"/>
-      <c r="G41" s="13" t="n"/>
-      <c r="H41" s="13" t="n"/>
-      <c r="I41" s="13" t="n"/>
-      <c r="J41" s="13" t="n"/>
-      <c r="K41" s="13" t="n"/>
-      <c r="L41" s="13" t="n">
-        <v>4200</v>
-      </c>
-      <c r="M41" s="13" t="n"/>
-      <c r="N41" s="13" t="n"/>
-      <c r="O41" s="13" t="n"/>
-      <c r="P41" s="13" t="n"/>
-      <c r="Q41" s="13" t="n"/>
-      <c r="R41" s="13" t="n"/>
-      <c r="S41" s="13" t="n"/>
-      <c r="T41" s="13" t="n"/>
-      <c r="U41" s="13" t="n"/>
-      <c r="V41" s="13" t="n"/>
-    </row>
-    <row r="42" ht="16.5" customHeight="1">
-      <c r="A42" s="14" t="inlineStr">
-        <is>
-          <t>escanor</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C42" s="12">
-        <f>ROUND(AVERAGE(F42:AI42), 0)</f>
-        <v/>
-      </c>
-      <c r="D42" s="1">
-        <f>SUM(F42:AI42)</f>
-        <v/>
-      </c>
-      <c r="E42" s="14" t="n">
-        <v>33800</v>
-      </c>
-      <c r="F42" s="13" t="n"/>
-      <c r="G42" s="13" t="n"/>
-      <c r="H42" s="13" t="n"/>
-      <c r="I42" s="13" t="n"/>
-      <c r="J42" s="13" t="n"/>
-      <c r="K42" s="13" t="n"/>
-      <c r="L42" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" s="13" t="n"/>
-      <c r="N42" s="13" t="n"/>
-      <c r="O42" s="13" t="n"/>
-      <c r="P42" s="13" t="n"/>
-      <c r="Q42" s="13" t="n"/>
-      <c r="R42" s="13" t="n"/>
-      <c r="S42" s="13" t="n"/>
-      <c r="T42" s="13" t="n"/>
-      <c r="U42" s="13" t="n"/>
-      <c r="V42" s="13" t="n"/>
-    </row>
-    <row r="43" ht="16.5" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
-        <is>
-          <t>fre 2000</t>
-        </is>
-      </c>
-      <c r="B43" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C43" s="12">
-        <f>ROUND(AVERAGE(F43:AI43), 0)</f>
-        <v/>
-      </c>
-      <c r="D43" s="1">
-        <f>SUM(F43:AI43)</f>
-        <v/>
-      </c>
-      <c r="E43" s="14" t="n">
-        <v>1050</v>
-      </c>
-      <c r="F43" s="13" t="n"/>
-      <c r="G43" s="13" t="n"/>
-      <c r="H43" s="13" t="n"/>
-      <c r="I43" s="13" t="n"/>
-      <c r="J43" s="13" t="n"/>
-      <c r="K43" s="13" t="n"/>
-      <c r="L43" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M43" s="13" t="n"/>
-      <c r="N43" s="13" t="n"/>
-      <c r="O43" s="13" t="n"/>
-      <c r="P43" s="13" t="n"/>
-      <c r="Q43" s="13" t="n"/>
-      <c r="R43" s="13" t="n"/>
-      <c r="S43" s="13" t="n"/>
-      <c r="T43" s="13" t="n"/>
-      <c r="U43" s="13" t="n"/>
-      <c r="V43" s="13" t="n"/>
-    </row>
-    <row r="44" ht="16.5" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
-        <is>
-          <t>KingAleGolem03</t>
-        </is>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>22/05/2026</t>
-        </is>
-      </c>
-      <c r="C44" s="12">
-        <f>ROUND(AVERAGE(F44:AI44), 0)</f>
-        <v/>
-      </c>
-      <c r="D44" s="1">
-        <f>SUM(F44:AI44)</f>
-        <v/>
-      </c>
-      <c r="E44" s="14" t="n">
-        <v>19475</v>
-      </c>
-      <c r="F44" s="13" t="n"/>
-      <c r="G44" s="13" t="n"/>
-      <c r="H44" s="13" t="n"/>
-      <c r="I44" s="13" t="n"/>
-      <c r="J44" s="13" t="n"/>
-      <c r="K44" s="13" t="n"/>
-      <c r="L44" s="13" t="n">
-        <v>1100</v>
-      </c>
-      <c r="M44" s="13" t="n"/>
-      <c r="N44" s="13" t="n"/>
-      <c r="O44" s="13" t="n"/>
-      <c r="P44" s="13" t="n"/>
-      <c r="Q44" s="13" t="n"/>
-      <c r="R44" s="13" t="n"/>
-      <c r="S44" s="13" t="n"/>
-      <c r="T44" s="13" t="n"/>
-      <c r="U44" s="13" t="n"/>
-      <c r="V44" s="13" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
-        <is>
-          <t>SgherroMutante</t>
-        </is>
-      </c>
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>23/05/2026</t>
-        </is>
-      </c>
-      <c r="C45" s="12">
-        <f>ROUND(AVERAGE(F45:AI45), 0)</f>
-        <v/>
-      </c>
-      <c r="D45" s="1">
-        <f>SUM(F45:AI45)</f>
-        <v/>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="13" t="n"/>
-      <c r="H45" s="13" t="n"/>
-      <c r="I45" s="13" t="n"/>
-      <c r="J45" s="13" t="n"/>
-      <c r="K45" s="13" t="n"/>
-      <c r="L45" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" s="13" t="n"/>
-      <c r="N45" s="13" t="n"/>
-      <c r="O45" s="13" t="n"/>
-      <c r="P45" s="13" t="n"/>
-      <c r="Q45" s="13" t="n"/>
-      <c r="R45" s="13" t="n"/>
-      <c r="S45" s="13" t="n"/>
-      <c r="T45" s="13" t="n"/>
-      <c r="U45" s="13" t="n"/>
-      <c r="V45" s="13" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>marcobeltra._</t>
-        </is>
-      </c>
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
-      <c r="C46" s="12">
-        <f>ROUND(AVERAGE(F46:AI46), 0)</f>
-        <v/>
-      </c>
-      <c r="D46" s="1">
-        <f>SUM(F46:AI46)</f>
-        <v/>
-      </c>
-      <c r="E46" s="14" t="n">
-        <v>15885</v>
-      </c>
-      <c r="F46" s="13" t="n"/>
-      <c r="G46" s="13" t="n"/>
-      <c r="H46" s="13" t="n"/>
-      <c r="I46" s="13" t="n"/>
-      <c r="J46" s="13" t="n"/>
-      <c r="K46" s="13" t="n"/>
-      <c r="L46" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M46" s="13" t="n"/>
-      <c r="N46" s="13" t="n"/>
-      <c r="O46" s="13" t="n"/>
-      <c r="P46" s="13" t="n"/>
-      <c r="Q46" s="13" t="n"/>
-      <c r="R46" s="13" t="n"/>
-      <c r="S46" s="13" t="n"/>
-      <c r="T46" s="13" t="n"/>
-      <c r="U46" s="13" t="n"/>
-      <c r="V46" s="13" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="14" t="inlineStr">
-        <is>
-          <t>maragno</t>
-        </is>
-      </c>
-      <c r="B47" s="16" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
-      <c r="C47" s="12">
-        <f>ROUND(AVERAGE(F47:AI47), 0)</f>
-        <v/>
-      </c>
-      <c r="D47" s="1">
-        <f>SUM(F47:AI47)</f>
-        <v/>
-      </c>
-      <c r="E47" s="14" t="n">
-        <v>99900</v>
-      </c>
-      <c r="F47" s="13" t="n"/>
-      <c r="G47" s="13" t="n"/>
-      <c r="H47" s="13" t="n"/>
-      <c r="I47" s="13" t="n"/>
-      <c r="J47" s="13" t="n"/>
-      <c r="K47" s="13" t="n"/>
-      <c r="L47" s="13" t="n">
-        <v>9500</v>
-      </c>
-      <c r="M47" s="13" t="n"/>
-      <c r="N47" s="13" t="n"/>
-      <c r="O47" s="13" t="n"/>
-      <c r="P47" s="13" t="n"/>
-      <c r="Q47" s="13" t="n"/>
-      <c r="R47" s="13" t="n"/>
-      <c r="S47" s="13" t="n"/>
-      <c r="T47" s="13" t="n"/>
-      <c r="U47" s="13" t="n"/>
-      <c r="V47" s="13" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t>vito</t>
-        </is>
-      </c>
-      <c r="B48" s="16" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
-      <c r="C48" s="12">
-        <f>ROUND(AVERAGE(F48:AI48), 0)</f>
-        <v/>
-      </c>
-      <c r="D48" s="1">
-        <f>SUM(F48:AI48)</f>
-        <v/>
-      </c>
-      <c r="E48" s="14" t="n">
-        <v>36860</v>
-      </c>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="13" t="n"/>
-      <c r="H48" s="13" t="n"/>
-      <c r="I48" s="13" t="n"/>
-      <c r="J48" s="13" t="n"/>
-      <c r="K48" s="13" t="n"/>
-      <c r="L48" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" s="13" t="n"/>
-      <c r="N48" s="13" t="n"/>
-      <c r="O48" s="13" t="n"/>
-      <c r="P48" s="13" t="n"/>
-      <c r="Q48" s="13" t="n"/>
-      <c r="R48" s="13" t="n"/>
-      <c r="S48" s="13" t="n"/>
-      <c r="T48" s="13" t="n"/>
-      <c r="U48" s="13" t="n"/>
-      <c r="V48" s="13" t="n"/>
-    </row>
-    <row r="49" ht="15" customHeight="1">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>ale mugna</t>
-        </is>
-      </c>
-      <c r="B49" s="16" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
-      <c r="C49" s="12">
-        <f>ROUND(AVERAGE(F49:AI49), 0)</f>
-        <v/>
-      </c>
-      <c r="D49" s="1">
-        <f>SUM(F49:AI49)</f>
-        <v/>
-      </c>
-      <c r="E49" s="14" t="n">
-        <v>37635</v>
-      </c>
-      <c r="F49" s="13" t="n"/>
-      <c r="G49" s="13" t="n"/>
-      <c r="H49" s="13" t="n"/>
-      <c r="I49" s="13" t="n"/>
-      <c r="J49" s="13" t="n"/>
-      <c r="K49" s="13" t="n"/>
-      <c r="L49" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" s="13" t="n"/>
-      <c r="N49" s="13" t="n"/>
-      <c r="O49" s="13" t="n"/>
-      <c r="P49" s="13" t="n"/>
-      <c r="Q49" s="13" t="n"/>
-      <c r="R49" s="13" t="n"/>
-      <c r="S49" s="13" t="n"/>
-      <c r="T49" s="13" t="n"/>
-      <c r="U49" s="13" t="n"/>
-      <c r="V49" s="13" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t>ale 12</t>
-        </is>
-      </c>
-      <c r="B50" s="16" t="inlineStr">
-        <is>
-          <t>28/05/2026</t>
-        </is>
-      </c>
-      <c r="C50" s="12">
-        <f>ROUND(AVERAGE(F50:AI50), 0)</f>
-        <v/>
-      </c>
-      <c r="D50" s="1">
-        <f>SUM(F50:AI50)</f>
-        <v/>
-      </c>
-      <c r="E50" s="14" t="n">
-        <v>66760</v>
-      </c>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="13" t="n"/>
-      <c r="J50" s="13" t="n"/>
-      <c r="K50" s="13" t="n"/>
-      <c r="L50" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M50" s="13" t="n"/>
-      <c r="N50" s="13" t="n"/>
-      <c r="O50" s="13" t="n"/>
-      <c r="P50" s="13" t="n"/>
-      <c r="Q50" s="13" t="n"/>
-      <c r="R50" s="13" t="n"/>
-      <c r="S50" s="13" t="n"/>
-      <c r="T50" s="13" t="n"/>
-      <c r="U50" s="13" t="n"/>
-      <c r="V50" s="13" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="14" t="inlineStr">
-        <is>
-          <t>rasim01</t>
-        </is>
-      </c>
-      <c r="B51" s="16" t="inlineStr">
-        <is>
-          <t>28/05/2026</t>
-        </is>
-      </c>
-      <c r="C51" s="12">
-        <f>ROUND(AVERAGE(F51:AI51), 0)</f>
-        <v/>
-      </c>
-      <c r="D51" s="1">
-        <f>SUM(F51:AI51)</f>
-        <v/>
-      </c>
-      <c r="E51" s="14" t="n">
-        <v>28450</v>
-      </c>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="13" t="n"/>
-      <c r="H51" s="13" t="n"/>
-      <c r="I51" s="13" t="n"/>
-      <c r="J51" s="13" t="n"/>
-      <c r="K51" s="13" t="n"/>
-      <c r="L51" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M51" s="13" t="n"/>
-      <c r="N51" s="13" t="n"/>
-      <c r="O51" s="13" t="n"/>
-      <c r="P51" s="13" t="n"/>
-      <c r="Q51" s="13" t="n"/>
-      <c r="R51" s="13" t="n"/>
-      <c r="S51" s="13" t="n"/>
-      <c r="T51" s="13" t="n"/>
-      <c r="U51" s="13" t="n"/>
-      <c r="V51" s="13" t="n"/>
-    </row>
+    <row r="39" ht="16.5" customHeight="1"/>
+    <row r="40" ht="16.5" customHeight="1"/>
+    <row r="41" ht="16.5" customHeight="1"/>
+    <row r="42" ht="16.5" customHeight="1"/>
+    <row r="43" ht="16.5" customHeight="1"/>
+    <row r="44" ht="16.5" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:AN1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2681,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI38"/>
+  <dimension ref="A1:AJ38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2873,6 +2873,11 @@
           <t>19/06/2026</t>
         </is>
       </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>19/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2886,7 +2891,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AI2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AJ2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2962,6 +2967,9 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2977,7 +2985,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AI3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AJ3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3044,6 +3052,9 @@
       <c r="AI3" t="n">
         <v>2</v>
       </c>
+      <c r="AJ3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3057,7 +3068,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AI4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AJ4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3147,6 +3158,9 @@
       <c r="AI4" t="n">
         <v>0</v>
       </c>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3160,7 +3174,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AI5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AJ5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3257,6 +3271,9 @@
         <v>0</v>
       </c>
       <c r="AI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3272,7 +3289,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AI6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AJ6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3371,6 +3388,9 @@
       <c r="AI6" t="n">
         <v>0</v>
       </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3384,7 +3404,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AI7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AJ7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3453,6 +3473,9 @@
       <c r="AI7" t="n">
         <v>0</v>
       </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3466,7 +3489,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AI8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AJ8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3556,6 +3579,9 @@
       <c r="AI8" t="n">
         <v>2</v>
       </c>
+      <c r="AJ8" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3569,7 +3595,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AI9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AJ9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3626,6 +3652,9 @@
       <c r="AI9" t="n">
         <v>0</v>
       </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -3639,7 +3668,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AI10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AJ10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -3729,6 +3758,9 @@
       <c r="AI10" t="n">
         <v>6</v>
       </c>
+      <c r="AJ10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -3742,7 +3774,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AI11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AJ11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -3841,6 +3873,9 @@
       <c r="AI11" t="n">
         <v>6</v>
       </c>
+      <c r="AJ11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -3854,7 +3889,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AI12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AJ12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -3939,6 +3974,9 @@
         <v>0</v>
       </c>
       <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3954,7 +3992,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AI13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AJ13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4052,6 +4090,9 @@
       </c>
       <c r="AI13" t="n">
         <v>0</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4066,7 +4107,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AI14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AJ14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4140,6 +4181,9 @@
       <c r="AI14" t="n">
         <v>6</v>
       </c>
+      <c r="AJ14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4153,7 +4197,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AI15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AJ15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4216,6 +4260,9 @@
       <c r="AI15" t="n">
         <v>0</v>
       </c>
+      <c r="AJ15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4229,7 +4276,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AI16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AJ16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4319,6 +4366,9 @@
       <c r="AI16" t="n">
         <v>6</v>
       </c>
+      <c r="AJ16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4332,7 +4382,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AI17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AJ17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -4431,6 +4481,9 @@
       <c r="AI17" t="n">
         <v>6</v>
       </c>
+      <c r="AJ17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4444,7 +4497,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AI18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AJ18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -4532,6 +4585,9 @@
         <v>0</v>
       </c>
       <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4547,7 +4603,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AI19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AJ19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -4622,6 +4678,9 @@
       <c r="AI19" t="n">
         <v>0</v>
       </c>
+      <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -4635,7 +4694,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AI20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AJ20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -4713,6 +4772,9 @@
       <c r="AI20" t="n">
         <v>0</v>
       </c>
+      <c r="AJ20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -4726,7 +4788,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AI21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AJ21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -4825,6 +4887,9 @@
       <c r="AI21" t="n">
         <v>0</v>
       </c>
+      <c r="AJ21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -4838,7 +4903,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AI22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AJ22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -4937,6 +5002,9 @@
       <c r="AI22" t="n">
         <v>0</v>
       </c>
+      <c r="AJ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -4950,7 +5018,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AI23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AJ23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5029,6 +5097,9 @@
       <c r="AI23" t="n">
         <v>0</v>
       </c>
+      <c r="AJ23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5042,7 +5113,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AI24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AJ24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5132,6 +5203,9 @@
       <c r="AI24" t="n">
         <v>5</v>
       </c>
+      <c r="AJ24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5145,7 +5219,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AI25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AJ25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -5197,6 +5271,9 @@
       <c r="AI25" t="n">
         <v>0</v>
       </c>
+      <c r="AJ25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5210,7 +5287,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AI26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AJ26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -5256,6 +5333,9 @@
       <c r="AI26" t="n">
         <v>0</v>
       </c>
+      <c r="AJ26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5269,7 +5349,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AI27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AJ27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -5315,6 +5395,9 @@
       <c r="AI27" t="n">
         <v>0</v>
       </c>
+      <c r="AJ27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -5328,7 +5411,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AI28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AJ28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -5371,6 +5454,9 @@
       <c r="AI28" t="n">
         <v>0</v>
       </c>
+      <c r="AJ28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -5384,7 +5470,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AI29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AJ29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -5424,6 +5510,9 @@
       <c r="AI29" t="n">
         <v>0</v>
       </c>
+      <c r="AJ29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -5437,7 +5526,7 @@
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AI30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AJ30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -5477,6 +5566,9 @@
       <c r="AI30" t="n">
         <v>0</v>
       </c>
+      <c r="AJ30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -5490,7 +5582,7 @@
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AI31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AJ31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -5527,6 +5619,9 @@
       <c r="AI31" t="n">
         <v>5</v>
       </c>
+      <c r="AJ31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -5540,7 +5635,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AI32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AJ32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -5574,6 +5669,9 @@
       <c r="AI32" t="n">
         <v>5</v>
       </c>
+      <c r="AJ32" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -5587,7 +5685,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AI33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AJ33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -5621,6 +5719,9 @@
       <c r="AI33" t="n">
         <v>0</v>
       </c>
+      <c r="AJ33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -5634,7 +5735,7 @@
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AI34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AJ34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -5665,6 +5766,9 @@
       <c r="AI34" t="n">
         <v>0</v>
       </c>
+      <c r="AJ34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -5678,7 +5782,7 @@
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AI35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AJ35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -5706,6 +5810,9 @@
       <c r="AI35" t="n">
         <v>0</v>
       </c>
+      <c r="AJ35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -5719,7 +5826,7 @@
         </is>
       </c>
       <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AI36), 0)</f>
+        <f>ROUND(AVERAGE(D36:AJ36), 0)</f>
         <v/>
       </c>
       <c r="K36" s="6" t="n"/>
@@ -5747,6 +5854,9 @@
       <c r="AI36" t="n">
         <v>0</v>
       </c>
+      <c r="AJ36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
@@ -5760,7 +5870,7 @@
         </is>
       </c>
       <c r="C37" s="28">
-        <f>ROUND(AVERAGE(D37:AI37), 0)</f>
+        <f>ROUND(AVERAGE(D37:AJ37), 0)</f>
         <v/>
       </c>
       <c r="K37" s="6" t="n"/>
@@ -5788,6 +5898,9 @@
       <c r="AI37" t="n">
         <v>0</v>
       </c>
+      <c r="AJ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
@@ -5801,7 +5914,7 @@
         </is>
       </c>
       <c r="C38" s="28">
-        <f>ROUND(AVERAGE(D38:AI38), 0)</f>
+        <f>ROUND(AVERAGE(D38:AJ38), 0)</f>
         <v/>
       </c>
       <c r="K38" s="6" t="n"/>
@@ -5827,6 +5940,9 @@
         <v>0</v>
       </c>
       <c r="AI38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ38" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -970,6 +970,9 @@
       <c r="L2" s="13" t="n">
         <v>10000</v>
       </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
@@ -1014,7 +1017,9 @@
       <c r="L3" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M3" s="13" t="n"/>
+      <c r="M3" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N3" s="13" t="n"/>
       <c r="O3" s="13" t="n"/>
       <c r="P3" s="13" t="n"/>
@@ -1058,7 +1063,9 @@
       <c r="L4" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M4" s="13" t="n"/>
+      <c r="M4" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N4" s="13" t="n"/>
       <c r="O4" s="13" t="n"/>
       <c r="P4" s="13" t="n"/>
@@ -1108,7 +1115,9 @@
       <c r="L5" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M5" s="13" t="n"/>
+      <c r="M5" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N5" s="13" t="n"/>
       <c r="O5" s="13" t="n"/>
       <c r="P5" s="13" t="n"/>
@@ -1156,7 +1165,9 @@
       <c r="L6" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M6" s="13" t="n"/>
+      <c r="M6" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N6" s="13" t="n"/>
       <c r="O6" s="13" t="n"/>
       <c r="P6" s="13" t="n"/>
@@ -1206,7 +1217,9 @@
       <c r="L7" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M7" s="13" t="n"/>
+      <c r="M7" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="n"/>
       <c r="P7" s="13" t="n"/>
@@ -1256,7 +1269,9 @@
       <c r="L8" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M8" s="13" t="n"/>
+      <c r="M8" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="n"/>
@@ -1308,7 +1323,9 @@
       <c r="L9" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M9" s="13" t="n"/>
+      <c r="M9" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
       <c r="P9" s="13" t="n"/>
@@ -1354,7 +1371,9 @@
       <c r="L10" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M10" s="13" t="n"/>
+      <c r="M10" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
       <c r="P10" s="13" t="n"/>
@@ -1406,7 +1425,9 @@
       <c r="L11" s="13" t="n">
         <v>6100</v>
       </c>
-      <c r="M11" s="13" t="n"/>
+      <c r="M11" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
       <c r="P11" s="13" t="n"/>
@@ -1460,7 +1481,9 @@
       <c r="L12" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M12" s="13" t="n"/>
+      <c r="M12" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N12" s="13" t="n"/>
       <c r="O12" s="13" t="n"/>
       <c r="P12" s="13" t="n"/>
@@ -1514,7 +1537,9 @@
       <c r="L13" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M13" s="13" t="n"/>
+      <c r="M13" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
       <c r="P13" s="13" t="n"/>
@@ -1562,7 +1587,9 @@
       <c r="L14" s="13" t="n">
         <v>8450</v>
       </c>
-      <c r="M14" s="13" t="n"/>
+      <c r="M14" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N14" s="13" t="n"/>
       <c r="O14" s="13" t="n"/>
       <c r="P14" s="13" t="n"/>
@@ -1616,7 +1643,9 @@
       <c r="L15" s="13" t="n">
         <v>9300</v>
       </c>
-      <c r="M15" s="13" t="n"/>
+      <c r="M15" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
       <c r="P15" s="13" t="n"/>
@@ -1666,7 +1695,9 @@
       <c r="L16" s="13" t="n">
         <v>13400</v>
       </c>
-      <c r="M16" s="13" t="n"/>
+      <c r="M16" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="13" t="n"/>
@@ -1716,7 +1747,9 @@
       <c r="L17" s="13" t="n">
         <v>6650</v>
       </c>
-      <c r="M17" s="13" t="n"/>
+      <c r="M17" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="13" t="n"/>
@@ -1766,7 +1799,9 @@
       <c r="L18" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M18" s="13" t="n"/>
+      <c r="M18" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N18" s="13" t="n"/>
       <c r="O18" s="13" t="n"/>
       <c r="P18" s="13" t="n"/>
@@ -1820,7 +1855,9 @@
       <c r="L19" s="13" t="n">
         <v>9350</v>
       </c>
-      <c r="M19" s="13" t="n"/>
+      <c r="M19" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="13" t="n"/>
       <c r="P19" s="13" t="n"/>
@@ -1870,7 +1907,9 @@
       <c r="L20" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M20" s="13" t="n"/>
+      <c r="M20" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N20" s="13" t="n"/>
       <c r="O20" s="13" t="n"/>
       <c r="P20" s="13" t="n"/>
@@ -1918,7 +1957,9 @@
       <c r="L21" s="13" t="n">
         <v>2200</v>
       </c>
-      <c r="M21" s="13" t="n"/>
+      <c r="M21" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N21" s="13" t="n"/>
       <c r="O21" s="13" t="n"/>
       <c r="P21" s="13" t="n"/>
@@ -1966,7 +2007,9 @@
       <c r="L22" s="13" t="n">
         <v>1050</v>
       </c>
-      <c r="M22" s="13" t="n"/>
+      <c r="M22" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N22" s="13" t="n"/>
       <c r="O22" s="13" t="n"/>
       <c r="P22" s="13" t="n"/>
@@ -2010,7 +2053,9 @@
       <c r="L23" s="13" t="n">
         <v>1100</v>
       </c>
-      <c r="M23" s="13" t="n"/>
+      <c r="M23" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N23" s="13" t="n"/>
       <c r="O23" s="13" t="n"/>
       <c r="P23" s="13" t="n"/>
@@ -2060,7 +2105,9 @@
       <c r="L24" s="13" t="n">
         <v>2050</v>
       </c>
-      <c r="M24" s="13" t="n"/>
+      <c r="M24" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N24" s="13" t="n"/>
       <c r="O24" s="13" t="n"/>
       <c r="P24" s="13" t="n"/>
@@ -2102,7 +2149,9 @@
       <c r="L25" s="13" t="n">
         <v>600</v>
       </c>
-      <c r="M25" s="13" t="n"/>
+      <c r="M25" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="13" t="n"/>
       <c r="P25" s="13" t="n"/>
@@ -2144,7 +2193,9 @@
       <c r="L26" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="M26" s="13" t="n"/>
+      <c r="M26" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N26" s="13" t="n"/>
       <c r="O26" s="13" t="n"/>
       <c r="P26" s="13" t="n"/>
@@ -2186,7 +2237,9 @@
       <c r="L27" s="13" t="n">
         <v>10650</v>
       </c>
-      <c r="M27" s="13" t="n"/>
+      <c r="M27" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N27" s="13" t="n"/>
       <c r="O27" s="13" t="n"/>
       <c r="P27" s="13" t="n"/>
@@ -2228,7 +2281,9 @@
       <c r="L28" s="13" t="n">
         <v>4400</v>
       </c>
-      <c r="M28" s="13" t="n"/>
+      <c r="M28" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N28" s="13" t="n"/>
       <c r="O28" s="13" t="n"/>
       <c r="P28" s="13" t="n"/>
@@ -2270,7 +2325,9 @@
       <c r="L29" s="13" t="n">
         <v>4500</v>
       </c>
-      <c r="M29" s="13" t="n"/>
+      <c r="M29" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N29" s="13" t="n"/>
       <c r="O29" s="13" t="n"/>
       <c r="P29" s="13" t="n"/>
@@ -2312,7 +2369,9 @@
       <c r="L30" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="M30" s="13" t="n"/>
+      <c r="M30" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N30" s="13" t="n"/>
       <c r="O30" s="13" t="n"/>
       <c r="P30" s="13" t="n"/>
@@ -2354,7 +2413,9 @@
       <c r="L31" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M31" s="13" t="n"/>
+      <c r="M31" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N31" s="13" t="n"/>
       <c r="O31" s="13" t="n"/>
       <c r="P31" s="13" t="n"/>
@@ -2396,7 +2457,9 @@
       <c r="L32" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="M32" s="13" t="n"/>
+      <c r="M32" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N32" s="13" t="n"/>
       <c r="O32" s="13" t="n"/>
       <c r="P32" s="13" t="n"/>
@@ -2438,7 +2501,9 @@
       <c r="L33" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="M33" s="13" t="n"/>
+      <c r="M33" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N33" s="13" t="n"/>
       <c r="O33" s="13" t="n"/>
       <c r="P33" s="13" t="n"/>
@@ -2480,7 +2545,9 @@
       <c r="L34" s="13" t="n">
         <v>4200</v>
       </c>
-      <c r="M34" s="13" t="n"/>
+      <c r="M34" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N34" s="13" t="n"/>
       <c r="O34" s="13" t="n"/>
       <c r="P34" s="13" t="n"/>
@@ -2522,7 +2589,9 @@
       <c r="L35" s="13" t="n">
         <v>9500</v>
       </c>
-      <c r="M35" s="13" t="n"/>
+      <c r="M35" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N35" s="13" t="n"/>
       <c r="O35" s="13" t="n"/>
       <c r="P35" s="13" t="n"/>
@@ -2564,7 +2633,9 @@
       <c r="L36" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="M36" s="13" t="n"/>
+      <c r="M36" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N36" s="13" t="n"/>
       <c r="O36" s="13" t="n"/>
       <c r="P36" s="13" t="n"/>
@@ -2604,7 +2675,9 @@
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
       <c r="L37" s="13" t="n"/>
-      <c r="M37" s="13" t="n"/>
+      <c r="M37" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
       <c r="P37" s="13" t="n"/>
@@ -2644,7 +2717,9 @@
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
       <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n"/>
+      <c r="M38" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
       <c r="P38" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK38"/>
+  <dimension ref="A1:AL38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2958,6 +2958,11 @@
           <t>19/06/2026</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>19/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2971,7 +2976,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AK2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AL2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3053,6 +3058,9 @@
         <v>0</v>
       </c>
       <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3068,7 +3076,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AK3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AL3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3141,6 +3149,9 @@
       <c r="AK3" t="n">
         <v>6</v>
       </c>
+      <c r="AL3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3154,7 +3165,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AK4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AL4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3250,6 +3261,9 @@
       <c r="AK4" t="n">
         <v>0</v>
       </c>
+      <c r="AL4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3263,7 +3277,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AK5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AL5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3367,6 +3381,9 @@
       </c>
       <c r="AK5" t="n">
         <v>0</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3381,7 +3398,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AK6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AL6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3486,6 +3503,9 @@
       <c r="AK6" t="n">
         <v>0</v>
       </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3499,7 +3519,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AK7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AL7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3574,6 +3594,9 @@
       <c r="AK7" t="n">
         <v>0</v>
       </c>
+      <c r="AL7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3587,7 +3610,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AK8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AL8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3683,6 +3706,9 @@
       <c r="AK8" t="n">
         <v>2</v>
       </c>
+      <c r="AL8" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3696,7 +3722,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AK9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AL9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3759,6 +3785,9 @@
       <c r="AK9" t="n">
         <v>0</v>
       </c>
+      <c r="AL9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -3772,7 +3801,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AK10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AL10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -3868,6 +3897,9 @@
       <c r="AK10" t="n">
         <v>6</v>
       </c>
+      <c r="AL10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -3881,7 +3913,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AK11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AL11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -3986,6 +4018,9 @@
       <c r="AK11" t="n">
         <v>6</v>
       </c>
+      <c r="AL11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -3999,7 +4034,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AK12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AL12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4091,6 +4126,9 @@
       </c>
       <c r="AK12" t="n">
         <v>0</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -4105,7 +4143,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AK13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AL13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4208,6 +4246,9 @@
         <v>6</v>
       </c>
       <c r="AK13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL13" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4223,7 +4264,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AK14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AL14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4303,6 +4344,9 @@
       <c r="AK14" t="n">
         <v>6</v>
       </c>
+      <c r="AL14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4316,7 +4360,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AK15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AL15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4385,6 +4429,9 @@
       <c r="AK15" t="n">
         <v>6</v>
       </c>
+      <c r="AL15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4398,7 +4445,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AK16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AL16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4494,6 +4541,9 @@
       <c r="AK16" t="n">
         <v>6</v>
       </c>
+      <c r="AL16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4507,7 +4557,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AK17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AL17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -4612,6 +4662,9 @@
       <c r="AK17" t="n">
         <v>6</v>
       </c>
+      <c r="AL17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4625,7 +4678,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AK18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AL18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -4719,6 +4772,9 @@
         <v>0</v>
       </c>
       <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4734,7 +4790,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AK19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AL19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -4815,6 +4871,9 @@
       <c r="AK19" t="n">
         <v>0</v>
       </c>
+      <c r="AL19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -4828,7 +4887,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AK20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AL20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -4912,6 +4971,9 @@
       <c r="AK20" t="n">
         <v>0</v>
       </c>
+      <c r="AL20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -4925,7 +4987,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AK21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AL21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5030,6 +5092,9 @@
       <c r="AK21" t="n">
         <v>0</v>
       </c>
+      <c r="AL21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5043,7 +5108,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AK22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AL22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5148,6 +5213,9 @@
       <c r="AK22" t="n">
         <v>0</v>
       </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5161,7 +5229,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AK23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AL23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5246,6 +5314,9 @@
       <c r="AK23" t="n">
         <v>0</v>
       </c>
+      <c r="AL23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5259,7 +5330,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AK24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AL24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5355,6 +5426,9 @@
       <c r="AK24" t="n">
         <v>5</v>
       </c>
+      <c r="AL24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5368,7 +5442,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AK25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AL25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -5426,6 +5500,9 @@
       <c r="AK25" t="n">
         <v>0</v>
       </c>
+      <c r="AL25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5439,7 +5516,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AK26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AL26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -5491,6 +5568,9 @@
       <c r="AK26" t="n">
         <v>6</v>
       </c>
+      <c r="AL26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5504,7 +5584,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AK27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AL27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -5556,6 +5636,9 @@
       <c r="AK27" t="n">
         <v>0</v>
       </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -5569,7 +5652,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AK28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AL28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -5618,6 +5701,9 @@
       <c r="AK28" t="n">
         <v>0</v>
       </c>
+      <c r="AL28" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -5631,7 +5717,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AK29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AL29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -5677,6 +5763,9 @@
       <c r="AK29" t="n">
         <v>0</v>
       </c>
+      <c r="AL29" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -5690,7 +5779,7 @@
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AK30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AL30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -5736,6 +5825,9 @@
       <c r="AK30" t="n">
         <v>0</v>
       </c>
+      <c r="AL30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -5749,7 +5841,7 @@
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AK31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AL31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -5792,6 +5884,9 @@
       <c r="AK31" t="n">
         <v>5</v>
       </c>
+      <c r="AL31" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -5805,7 +5900,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AK32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AL32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -5845,6 +5940,9 @@
       <c r="AK32" t="n">
         <v>6</v>
       </c>
+      <c r="AL32" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -5858,7 +5956,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AK33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AL33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -5898,6 +5996,9 @@
       <c r="AK33" t="n">
         <v>0</v>
       </c>
+      <c r="AL33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -5911,7 +6012,7 @@
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AK34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AL34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -5948,6 +6049,9 @@
       <c r="AK34" t="n">
         <v>0</v>
       </c>
+      <c r="AL34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -5961,7 +6065,7 @@
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AK35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AL35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -5995,6 +6099,9 @@
       <c r="AK35" t="n">
         <v>0</v>
       </c>
+      <c r="AL35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -6008,7 +6115,7 @@
         </is>
       </c>
       <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AK36), 0)</f>
+        <f>ROUND(AVERAGE(D36:AL36), 0)</f>
         <v/>
       </c>
       <c r="K36" s="6" t="n"/>
@@ -6042,6 +6149,9 @@
       <c r="AK36" t="n">
         <v>6</v>
       </c>
+      <c r="AL36" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
@@ -6055,7 +6165,7 @@
         </is>
       </c>
       <c r="C37" s="28">
-        <f>ROUND(AVERAGE(D37:AK37), 0)</f>
+        <f>ROUND(AVERAGE(D37:AL37), 0)</f>
         <v/>
       </c>
       <c r="K37" s="6" t="n"/>
@@ -6089,6 +6199,9 @@
       <c r="AK37" t="n">
         <v>0</v>
       </c>
+      <c r="AL37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
@@ -6102,7 +6215,7 @@
         </is>
       </c>
       <c r="C38" s="28">
-        <f>ROUND(AVERAGE(D38:AK38), 0)</f>
+        <f>ROUND(AVERAGE(D38:AL38), 0)</f>
         <v/>
       </c>
       <c r="K38" s="6" t="n"/>
@@ -6134,6 +6247,9 @@
         <v>0</v>
       </c>
       <c r="AK38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL38" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -955,7 +955,7 @@
         <v/>
       </c>
       <c r="E2" s="14" t="n">
-        <v>60000</v>
+        <v>60300</v>
       </c>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
@@ -971,7 +971,7 @@
         <v>10000</v>
       </c>
       <c r="M2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
@@ -2270,7 +2270,7 @@
         <v/>
       </c>
       <c r="E28" s="14" t="n">
-        <v>60600</v>
+        <v>64300</v>
       </c>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
@@ -2282,7 +2282,7 @@
         <v>4400</v>
       </c>
       <c r="M28" s="13" t="n">
-        <v>0</v>
+        <v>3700</v>
       </c>
       <c r="N28" s="13" t="n"/>
       <c r="O28" s="13" t="n"/>
@@ -2666,7 +2666,7 @@
         <v/>
       </c>
       <c r="E37" s="14" t="n">
-        <v>13250</v>
+        <v>14150</v>
       </c>
       <c r="F37" s="13" t="n"/>
       <c r="G37" s="13" t="n"/>
@@ -2676,7 +2676,7 @@
       <c r="K37" s="13" t="n"/>
       <c r="L37" s="13" t="n"/>
       <c r="M37" s="13" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-24
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2226,7 +2226,7 @@
         <v/>
       </c>
       <c r="E27" s="14" t="n">
-        <v>53090</v>
+        <v>53990</v>
       </c>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
@@ -2238,7 +2238,7 @@
         <v>10650</v>
       </c>
       <c r="M27" s="13" t="n">
-        <v>1800</v>
+        <v>2700</v>
       </c>
       <c r="N27" s="13" t="n"/>
       <c r="O27" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1356,7 +1356,7 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>96650</v>
+        <v>97100</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
@@ -1372,7 +1372,7 @@
         <v>10000</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>2700</v>
+        <v>3150</v>
       </c>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-26
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1356,7 +1356,7 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>97800</v>
+        <v>97950</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
@@ -1372,7 +1372,7 @@
         <v>10000</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>3850</v>
+        <v>4000</v>
       </c>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
@@ -1990,7 +1990,7 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>8600</v>
+        <v>8750</v>
       </c>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="n"/>
@@ -2008,7 +2008,7 @@
         <v>1050</v>
       </c>
       <c r="M22" s="13" t="n">
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="N22" s="13" t="n"/>
       <c r="O22" s="13" t="n"/>
@@ -2358,7 +2358,7 @@
         <v/>
       </c>
       <c r="E30" s="14" t="n">
-        <v>117725</v>
+        <v>118325</v>
       </c>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
@@ -2370,7 +2370,7 @@
         <v>4100</v>
       </c>
       <c r="M30" s="13" t="n">
-        <v>3300</v>
+        <v>3900</v>
       </c>
       <c r="N30" s="13" t="n"/>
       <c r="O30" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL38"/>
+  <dimension ref="A1:AM38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2963,6 +2963,11 @@
           <t>19/06/2026</t>
         </is>
       </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2976,7 +2981,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AL2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AM2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3061,6 +3066,9 @@
         <v>0</v>
       </c>
       <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3076,7 +3084,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AL3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AM3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3152,6 +3160,9 @@
       <c r="AL3" t="n">
         <v>6</v>
       </c>
+      <c r="AM3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3165,7 +3176,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AL4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AM4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3264,6 +3275,9 @@
       <c r="AL4" t="n">
         <v>0</v>
       </c>
+      <c r="AM4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3277,7 +3291,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AL5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AM5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3384,6 +3398,9 @@
       </c>
       <c r="AL5" t="n">
         <v>6</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3398,7 +3415,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AL6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AM6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3506,6 +3523,9 @@
       <c r="AL6" t="n">
         <v>0</v>
       </c>
+      <c r="AM6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3519,7 +3539,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AL7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AM7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3597,6 +3617,9 @@
       <c r="AL7" t="n">
         <v>0</v>
       </c>
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3610,7 +3633,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AL8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AM8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3709,6 +3732,9 @@
       <c r="AL8" t="n">
         <v>2</v>
       </c>
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3722,7 +3748,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AL9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AM9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3788,6 +3814,9 @@
       <c r="AL9" t="n">
         <v>0</v>
       </c>
+      <c r="AM9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -3801,7 +3830,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AL10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AM10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -3900,6 +3929,9 @@
       <c r="AL10" t="n">
         <v>6</v>
       </c>
+      <c r="AM10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -3913,7 +3945,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AL11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AM11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4021,6 +4053,9 @@
       <c r="AL11" t="n">
         <v>6</v>
       </c>
+      <c r="AM11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4034,7 +4069,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AL12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AM12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4128,6 +4163,9 @@
         <v>0</v>
       </c>
       <c r="AL12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4143,7 +4181,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AL13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AM13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4250,6 +4288,9 @@
       </c>
       <c r="AL13" t="n">
         <v>6</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4264,7 +4305,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AL14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AM14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4347,6 +4388,9 @@
       <c r="AL14" t="n">
         <v>6</v>
       </c>
+      <c r="AM14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4360,7 +4404,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AL15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AM15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4432,6 +4476,9 @@
       <c r="AL15" t="n">
         <v>6</v>
       </c>
+      <c r="AM15" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4445,7 +4492,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AL16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AM16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4544,6 +4591,9 @@
       <c r="AL16" t="n">
         <v>6</v>
       </c>
+      <c r="AM16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4557,7 +4607,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AL17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AM17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -4665,6 +4715,9 @@
       <c r="AL17" t="n">
         <v>6</v>
       </c>
+      <c r="AM17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4678,7 +4731,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AL18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AM18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -4775,6 +4828,9 @@
         <v>0</v>
       </c>
       <c r="AL18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4790,7 +4846,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AL19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AM19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -4874,6 +4930,9 @@
       <c r="AL19" t="n">
         <v>0</v>
       </c>
+      <c r="AM19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -4887,7 +4946,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AL20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AM20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -4974,6 +5033,9 @@
       <c r="AL20" t="n">
         <v>0</v>
       </c>
+      <c r="AM20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -4987,7 +5049,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AL21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AM21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5095,6 +5157,9 @@
       <c r="AL21" t="n">
         <v>0</v>
       </c>
+      <c r="AM21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5108,7 +5173,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AL22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AM22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5216,6 +5281,9 @@
       <c r="AL22" t="n">
         <v>0</v>
       </c>
+      <c r="AM22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5229,7 +5297,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AL23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AM23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5317,6 +5385,9 @@
       <c r="AL23" t="n">
         <v>0</v>
       </c>
+      <c r="AM23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5330,7 +5401,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AL24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AM24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5429,6 +5500,9 @@
       <c r="AL24" t="n">
         <v>5</v>
       </c>
+      <c r="AM24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5442,7 +5516,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AL25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AM25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -5503,6 +5577,9 @@
       <c r="AL25" t="n">
         <v>6</v>
       </c>
+      <c r="AM25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5516,7 +5593,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AL26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AM26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -5571,6 +5648,9 @@
       <c r="AL26" t="n">
         <v>6</v>
       </c>
+      <c r="AM26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5584,7 +5664,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AL27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AM27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -5639,6 +5719,9 @@
       <c r="AL27" t="n">
         <v>0</v>
       </c>
+      <c r="AM27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -5652,7 +5735,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AL28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AM28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -5704,6 +5787,9 @@
       <c r="AL28" t="n">
         <v>6</v>
       </c>
+      <c r="AM28" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -5717,7 +5803,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AL29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AM29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -5766,6 +5852,9 @@
       <c r="AL29" t="n">
         <v>6</v>
       </c>
+      <c r="AM29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -5779,7 +5868,7 @@
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AL30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AM30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -5828,6 +5917,9 @@
       <c r="AL30" t="n">
         <v>0</v>
       </c>
+      <c r="AM30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -5841,7 +5933,7 @@
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AL31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AM31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -5887,6 +5979,9 @@
       <c r="AL31" t="n">
         <v>6</v>
       </c>
+      <c r="AM31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -5900,7 +5995,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AL32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AM32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -5943,6 +6038,9 @@
       <c r="AL32" t="n">
         <v>6</v>
       </c>
+      <c r="AM32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -5956,7 +6054,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AL33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AM33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -5999,6 +6097,9 @@
       <c r="AL33" t="n">
         <v>0</v>
       </c>
+      <c r="AM33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -6012,7 +6113,7 @@
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AL34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AM34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -6052,6 +6153,9 @@
       <c r="AL34" t="n">
         <v>0</v>
       </c>
+      <c r="AM34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -6065,7 +6169,7 @@
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AL35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AM35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -6102,6 +6206,9 @@
       <c r="AL35" t="n">
         <v>0</v>
       </c>
+      <c r="AM35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -6115,7 +6222,7 @@
         </is>
       </c>
       <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AL36), 0)</f>
+        <f>ROUND(AVERAGE(D36:AM36), 0)</f>
         <v/>
       </c>
       <c r="K36" s="6" t="n"/>
@@ -6152,6 +6259,9 @@
       <c r="AL36" t="n">
         <v>6</v>
       </c>
+      <c r="AM36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
@@ -6165,7 +6275,7 @@
         </is>
       </c>
       <c r="C37" s="28">
-        <f>ROUND(AVERAGE(D37:AL37), 0)</f>
+        <f>ROUND(AVERAGE(D37:AM37), 0)</f>
         <v/>
       </c>
       <c r="K37" s="6" t="n"/>
@@ -6202,6 +6312,9 @@
       <c r="AL37" t="n">
         <v>0</v>
       </c>
+      <c r="AM37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
@@ -6215,7 +6328,7 @@
         </is>
       </c>
       <c r="C38" s="28">
-        <f>ROUND(AVERAGE(D38:AL38), 0)</f>
+        <f>ROUND(AVERAGE(D38:AM38), 0)</f>
         <v/>
       </c>
       <c r="K38" s="6" t="n"/>
@@ -6250,6 +6363,9 @@
         <v>0</v>
       </c>
       <c r="AL38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM38" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1302,7 +1302,7 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>47750</v>
+        <v>48250</v>
       </c>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n">
@@ -1324,7 +1324,7 @@
         <v>10000</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>5500</v>
+        <v>6000</v>
       </c>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
@@ -1356,7 +1356,7 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>98400</v>
+        <v>98550</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
@@ -1372,7 +1372,7 @@
         <v>10000</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>4450</v>
+        <v>4600</v>
       </c>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-06-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -994,7 +994,7 @@
         <v/>
       </c>
       <c r="E3" s="14" t="n">
-        <v>84250</v>
+        <v>88250</v>
       </c>
       <c r="F3" s="13" t="n">
         <v>4000</v>
@@ -1018,7 +1018,7 @@
         <v>10000</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>6000</v>
+        <v>10000</v>
       </c>
       <c r="N3" s="13" t="n"/>
       <c r="O3" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN38"/>
+  <dimension ref="A1:AO38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2973,6 +2973,11 @@
           <t>26/06/2026</t>
         </is>
       </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2986,7 +2991,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AN2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AO2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3077,6 +3082,9 @@
         <v>0</v>
       </c>
       <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3092,7 +3100,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AN3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AO3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3174,6 +3182,9 @@
       <c r="AN3" t="n">
         <v>3</v>
       </c>
+      <c r="AO3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3187,7 +3198,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AN4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AO4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3292,6 +3303,9 @@
       <c r="AN4" t="n">
         <v>0</v>
       </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3305,7 +3319,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AN5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AO5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3417,6 +3431,9 @@
         <v>0</v>
       </c>
       <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3432,7 +3449,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AN6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AO6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3546,6 +3563,9 @@
       <c r="AN6" t="n">
         <v>0</v>
       </c>
+      <c r="AO6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3559,7 +3579,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AN7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AO7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3643,6 +3663,9 @@
       <c r="AN7" t="n">
         <v>0</v>
       </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3656,7 +3679,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AN8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AO8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3761,6 +3784,9 @@
       <c r="AN8" t="n">
         <v>0</v>
       </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3774,7 +3800,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AN9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AO9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3846,6 +3872,9 @@
       <c r="AN9" t="n">
         <v>1</v>
       </c>
+      <c r="AO9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -3859,7 +3888,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AN10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AO10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -3964,6 +3993,9 @@
       <c r="AN10" t="n">
         <v>6</v>
       </c>
+      <c r="AO10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -3977,7 +4009,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AN11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AO11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4091,6 +4123,9 @@
       <c r="AN11" t="n">
         <v>0</v>
       </c>
+      <c r="AO11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4104,7 +4139,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AN12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AO12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4204,6 +4239,9 @@
         <v>6</v>
       </c>
       <c r="AN12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4219,7 +4257,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AN13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AO13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4331,6 +4369,9 @@
         <v>0</v>
       </c>
       <c r="AN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4346,7 +4387,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AN14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AO14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4435,6 +4476,9 @@
       <c r="AN14" t="n">
         <v>0</v>
       </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4448,7 +4492,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AN15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AO15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4526,6 +4570,9 @@
       <c r="AN15" t="n">
         <v>3</v>
       </c>
+      <c r="AO15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4539,7 +4586,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AN16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AO16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4644,6 +4691,9 @@
       <c r="AN16" t="n">
         <v>1</v>
       </c>
+      <c r="AO16" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4657,7 +4707,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AN17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AO17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -4771,6 +4821,9 @@
       <c r="AN17" t="n">
         <v>6</v>
       </c>
+      <c r="AO17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4784,7 +4837,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AN18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AO18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -4887,6 +4940,9 @@
         <v>0</v>
       </c>
       <c r="AN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4902,7 +4958,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AN19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AO19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -4992,6 +5048,9 @@
       <c r="AN19" t="n">
         <v>0</v>
       </c>
+      <c r="AO19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5005,7 +5064,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AN20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AO20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -5098,6 +5157,9 @@
       <c r="AN20" t="n">
         <v>0</v>
       </c>
+      <c r="AO20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5111,7 +5173,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AN21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AO21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5225,6 +5287,9 @@
       <c r="AN21" t="n">
         <v>1</v>
       </c>
+      <c r="AO21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5238,7 +5303,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AN22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AO22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5352,6 +5417,9 @@
       <c r="AN22" t="n">
         <v>0</v>
       </c>
+      <c r="AO22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5365,7 +5433,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AN23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AO23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5459,6 +5527,9 @@
       <c r="AN23" t="n">
         <v>0</v>
       </c>
+      <c r="AO23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5472,7 +5543,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AN24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AO24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5577,6 +5648,9 @@
       <c r="AN24" t="n">
         <v>0</v>
       </c>
+      <c r="AO24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5590,7 +5664,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AN25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AO25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -5657,6 +5731,9 @@
       <c r="AN25" t="n">
         <v>6</v>
       </c>
+      <c r="AO25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5670,7 +5747,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AN26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AO26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -5731,6 +5808,9 @@
       <c r="AN26" t="n">
         <v>4</v>
       </c>
+      <c r="AO26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5744,7 +5824,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AN27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AO27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -5805,6 +5885,9 @@
       <c r="AN27" t="n">
         <v>0</v>
       </c>
+      <c r="AO27" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -5818,7 +5901,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AN28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AO28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -5876,6 +5959,9 @@
       <c r="AN28" t="n">
         <v>6</v>
       </c>
+      <c r="AO28" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -5889,7 +5975,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AN29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AO29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -5944,6 +6030,9 @@
       <c r="AN29" t="n">
         <v>0</v>
       </c>
+      <c r="AO29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -5957,7 +6046,7 @@
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AN30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AO30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -6012,6 +6101,9 @@
       <c r="AN30" t="n">
         <v>0</v>
       </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -6025,7 +6117,7 @@
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AN31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AO31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -6077,6 +6169,9 @@
       <c r="AN31" t="n">
         <v>5</v>
       </c>
+      <c r="AO31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -6090,7 +6185,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AN32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AO32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -6139,6 +6234,9 @@
       <c r="AN32" t="n">
         <v>0</v>
       </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -6152,7 +6250,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AN33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AO33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -6201,6 +6299,9 @@
       <c r="AN33" t="n">
         <v>0</v>
       </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -6214,7 +6315,7 @@
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AN34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AO34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -6260,6 +6361,9 @@
       <c r="AN34" t="n">
         <v>0</v>
       </c>
+      <c r="AO34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -6273,7 +6377,7 @@
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AN35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AO35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -6316,6 +6420,9 @@
       <c r="AN35" t="n">
         <v>0</v>
       </c>
+      <c r="AO35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -6329,7 +6436,7 @@
         </is>
       </c>
       <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AN36), 0)</f>
+        <f>ROUND(AVERAGE(D36:AO36), 0)</f>
         <v/>
       </c>
       <c r="K36" s="6" t="n"/>
@@ -6372,6 +6479,9 @@
       <c r="AN36" t="n">
         <v>0</v>
       </c>
+      <c r="AO36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
@@ -6385,7 +6495,7 @@
         </is>
       </c>
       <c r="C37" s="28">
-        <f>ROUND(AVERAGE(D37:AN37), 0)</f>
+        <f>ROUND(AVERAGE(D37:AO37), 0)</f>
         <v/>
       </c>
       <c r="K37" s="6" t="n"/>
@@ -6428,6 +6538,9 @@
       <c r="AN37" t="n">
         <v>0</v>
       </c>
+      <c r="AO37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
@@ -6441,7 +6554,7 @@
         </is>
       </c>
       <c r="C38" s="28">
-        <f>ROUND(AVERAGE(D38:AN38), 0)</f>
+        <f>ROUND(AVERAGE(D38:AO38), 0)</f>
         <v/>
       </c>
       <c r="K38" s="6" t="n"/>
@@ -6483,6 +6596,9 @@
       </c>
       <c r="AN38" t="n">
         <v>0</v>
+      </c>
+      <c r="AO38" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-06-29
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP38"/>
+  <dimension ref="A1:AQ38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2983,6 +2983,11 @@
           <t>26/06/2026</t>
         </is>
       </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2996,7 +3001,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AP2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AQ2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3093,6 +3098,9 @@
         <v>0</v>
       </c>
       <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3108,7 +3116,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AP3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AQ3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3196,6 +3204,9 @@
       <c r="AP3" t="n">
         <v>6</v>
       </c>
+      <c r="AQ3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3209,7 +3220,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AP4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AQ4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3320,6 +3331,9 @@
       <c r="AP4" t="n">
         <v>0</v>
       </c>
+      <c r="AQ4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3333,7 +3347,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AP5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AQ5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3452,6 +3466,9 @@
       </c>
       <c r="AP5" t="n">
         <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3466,7 +3483,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AP6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AQ6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3586,6 +3603,9 @@
       <c r="AP6" t="n">
         <v>0</v>
       </c>
+      <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3599,7 +3619,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AP7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AQ7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3689,6 +3709,9 @@
       <c r="AP7" t="n">
         <v>0</v>
       </c>
+      <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3702,7 +3725,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AP8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AQ8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3813,6 +3836,9 @@
       <c r="AP8" t="n">
         <v>0</v>
       </c>
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3826,7 +3852,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AP9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AQ9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3904,6 +3930,9 @@
       <c r="AP9" t="n">
         <v>3</v>
       </c>
+      <c r="AQ9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -3917,7 +3946,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AP10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AQ10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -4028,6 +4057,9 @@
       <c r="AP10" t="n">
         <v>6</v>
       </c>
+      <c r="AQ10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4041,7 +4073,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AP11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AQ11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4161,6 +4193,9 @@
       <c r="AP11" t="n">
         <v>6</v>
       </c>
+      <c r="AQ11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4174,7 +4209,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AP12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AQ12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4280,6 +4315,9 @@
         <v>6</v>
       </c>
       <c r="AP12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AQ12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4295,7 +4333,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AP13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AQ13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4414,6 +4452,9 @@
       </c>
       <c r="AP13" t="n">
         <v>0</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4428,7 +4469,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AP14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AQ14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4523,6 +4564,9 @@
       <c r="AP14" t="n">
         <v>0</v>
       </c>
+      <c r="AQ14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4536,7 +4580,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AP15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AQ15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4620,6 +4664,9 @@
       <c r="AP15" t="n">
         <v>6</v>
       </c>
+      <c r="AQ15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4633,7 +4680,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AP16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AQ16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4744,6 +4791,9 @@
       <c r="AP16" t="n">
         <v>2</v>
       </c>
+      <c r="AQ16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4757,7 +4807,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AP17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AQ17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -4877,6 +4927,9 @@
       <c r="AP17" t="n">
         <v>6</v>
       </c>
+      <c r="AQ17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4890,7 +4943,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AP18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AQ18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -4999,6 +5052,9 @@
         <v>0</v>
       </c>
       <c r="AP18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5014,7 +5070,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AP19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AQ19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -5110,6 +5166,9 @@
       <c r="AP19" t="n">
         <v>0</v>
       </c>
+      <c r="AQ19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5123,7 +5182,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AP20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AQ20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -5222,6 +5281,9 @@
       <c r="AP20" t="n">
         <v>0</v>
       </c>
+      <c r="AQ20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5235,7 +5297,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AP21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AQ21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5355,6 +5417,9 @@
       <c r="AP21" t="n">
         <v>1</v>
       </c>
+      <c r="AQ21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5368,7 +5433,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AP22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AQ22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5488,6 +5553,9 @@
       <c r="AP22" t="n">
         <v>6</v>
       </c>
+      <c r="AQ22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5501,7 +5569,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AP23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AQ23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5601,6 +5669,9 @@
       <c r="AP23" t="n">
         <v>0</v>
       </c>
+      <c r="AQ23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5614,7 +5685,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AP24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AQ24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5725,6 +5796,9 @@
       <c r="AP24" t="n">
         <v>0</v>
       </c>
+      <c r="AQ24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5738,7 +5812,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AP25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AQ25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -5811,6 +5885,9 @@
       <c r="AP25" t="n">
         <v>6</v>
       </c>
+      <c r="AQ25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5824,7 +5901,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AP26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AQ26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -5891,6 +5968,9 @@
       <c r="AP26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -5904,7 +5984,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AP27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AQ27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -5971,6 +6051,9 @@
       <c r="AP27" t="n">
         <v>6</v>
       </c>
+      <c r="AQ27" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -5984,7 +6067,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AP28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AQ28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6048,6 +6131,9 @@
       <c r="AP28" t="n">
         <v>6</v>
       </c>
+      <c r="AQ28" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -6061,7 +6147,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AP29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AQ29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6122,6 +6208,9 @@
       <c r="AP29" t="n">
         <v>0</v>
       </c>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -6135,7 +6224,7 @@
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AP30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AQ30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -6196,6 +6285,9 @@
       <c r="AP30" t="n">
         <v>0</v>
       </c>
+      <c r="AQ30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -6209,7 +6301,7 @@
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AP31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AQ31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -6267,6 +6359,9 @@
       <c r="AP31" t="n">
         <v>5</v>
       </c>
+      <c r="AQ31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -6280,7 +6375,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AP32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AQ32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -6335,6 +6430,9 @@
       <c r="AP32" t="n">
         <v>0</v>
       </c>
+      <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -6348,7 +6446,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AP33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AQ33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -6403,6 +6501,9 @@
       <c r="AP33" t="n">
         <v>0</v>
       </c>
+      <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -6416,7 +6517,7 @@
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AP34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AQ34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -6468,6 +6569,9 @@
       <c r="AP34" t="n">
         <v>0</v>
       </c>
+      <c r="AQ34" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -6481,7 +6585,7 @@
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AP35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AQ35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -6530,6 +6634,9 @@
       <c r="AP35" t="n">
         <v>0</v>
       </c>
+      <c r="AQ35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
@@ -6543,7 +6650,7 @@
         </is>
       </c>
       <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AP36), 0)</f>
+        <f>ROUND(AVERAGE(D36:AQ36), 0)</f>
         <v/>
       </c>
       <c r="K36" s="6" t="n"/>
@@ -6592,6 +6699,9 @@
       <c r="AP36" t="n">
         <v>0</v>
       </c>
+      <c r="AQ36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
@@ -6605,7 +6715,7 @@
         </is>
       </c>
       <c r="C37" s="28">
-        <f>ROUND(AVERAGE(D37:AP37), 0)</f>
+        <f>ROUND(AVERAGE(D37:AQ37), 0)</f>
         <v/>
       </c>
       <c r="K37" s="6" t="n"/>
@@ -6654,6 +6764,9 @@
       <c r="AP37" t="n">
         <v>0</v>
       </c>
+      <c r="AQ37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
@@ -6667,7 +6780,7 @@
         </is>
       </c>
       <c r="C38" s="28">
-        <f>ROUND(AVERAGE(D38:AP38), 0)</f>
+        <f>ROUND(AVERAGE(D38:AQ38), 0)</f>
         <v/>
       </c>
       <c r="K38" s="6" t="n"/>
@@ -6714,6 +6827,9 @@
         <v>6</v>
       </c>
       <c r="AP38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AQ38" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-04
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ38"/>
+  <dimension ref="A1:AR36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2988,6 +2988,11 @@
           <t>26/06/2026</t>
         </is>
       </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3001,7 +3006,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AQ2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AR2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3101,6 +3106,9 @@
         <v>0</v>
       </c>
       <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3116,7 +3124,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AQ3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AR3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3207,6 +3215,9 @@
       <c r="AQ3" t="n">
         <v>6</v>
       </c>
+      <c r="AR3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3220,7 +3231,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AQ4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AR4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3334,6 +3345,9 @@
       <c r="AQ4" t="n">
         <v>6</v>
       </c>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3347,7 +3361,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AQ5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AR5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3469,6 +3483,9 @@
       </c>
       <c r="AQ5" t="n">
         <v>6</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3483,7 +3500,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AQ6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AR6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3606,6 +3623,9 @@
       <c r="AQ6" t="n">
         <v>0</v>
       </c>
+      <c r="AR6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3619,7 +3639,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AQ7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AR7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3712,6 +3732,9 @@
       <c r="AQ7" t="n">
         <v>0</v>
       </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3725,7 +3748,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AQ8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AR8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3839,6 +3862,9 @@
       <c r="AQ8" t="n">
         <v>0</v>
       </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3852,7 +3878,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AQ9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AR9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3933,6 +3959,9 @@
       <c r="AQ9" t="n">
         <v>3</v>
       </c>
+      <c r="AR9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -3946,7 +3975,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AQ10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AR10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -4060,6 +4089,9 @@
       <c r="AQ10" t="n">
         <v>6</v>
       </c>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4073,7 +4105,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AQ11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AR11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4196,6 +4228,9 @@
       <c r="AQ11" t="n">
         <v>6</v>
       </c>
+      <c r="AR11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4209,7 +4244,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AQ12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AR12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4318,6 +4353,9 @@
         <v>6</v>
       </c>
       <c r="AQ12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4333,7 +4371,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AQ13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AR13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4455,6 +4493,9 @@
       </c>
       <c r="AQ13" t="n">
         <v>6</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4469,7 +4510,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AQ14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AR14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4567,6 +4608,9 @@
       <c r="AQ14" t="n">
         <v>0</v>
       </c>
+      <c r="AR14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4580,7 +4624,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AQ15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AR15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4667,6 +4711,9 @@
       <c r="AQ15" t="n">
         <v>6</v>
       </c>
+      <c r="AR15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4680,7 +4727,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AQ16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AR16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4794,6 +4841,9 @@
       <c r="AQ16" t="n">
         <v>6</v>
       </c>
+      <c r="AR16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4807,7 +4857,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AQ17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AR17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -4930,6 +4980,9 @@
       <c r="AQ17" t="n">
         <v>6</v>
       </c>
+      <c r="AR17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -4943,7 +4996,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AQ18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AR18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5055,6 +5108,9 @@
         <v>0</v>
       </c>
       <c r="AQ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5070,7 +5126,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AQ19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AR19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -5169,6 +5225,9 @@
       <c r="AQ19" t="n">
         <v>0</v>
       </c>
+      <c r="AR19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5182,7 +5241,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AQ20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AR20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -5284,6 +5343,9 @@
       <c r="AQ20" t="n">
         <v>0</v>
       </c>
+      <c r="AR20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5297,7 +5359,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AQ21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AR21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5420,6 +5482,9 @@
       <c r="AQ21" t="n">
         <v>1</v>
       </c>
+      <c r="AR21" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5433,7 +5498,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AQ22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AR22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5556,6 +5621,9 @@
       <c r="AQ22" t="n">
         <v>6</v>
       </c>
+      <c r="AR22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5569,7 +5637,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AQ23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AR23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5672,6 +5740,9 @@
       <c r="AQ23" t="n">
         <v>6</v>
       </c>
+      <c r="AR23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5685,7 +5756,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AQ24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AR24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5799,6 +5870,9 @@
       <c r="AQ24" t="n">
         <v>0</v>
       </c>
+      <c r="AR24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5812,7 +5886,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AQ25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AR25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -5888,6 +5962,9 @@
       <c r="AQ25" t="n">
         <v>6</v>
       </c>
+      <c r="AR25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -5901,7 +5978,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AQ26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AR26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -5971,20 +6048,23 @@
       <c r="AQ26" t="n">
         <v>6</v>
       </c>
+      <c r="AR26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AQ27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AR27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -5997,29 +6077,26 @@
       <c r="S27" s="20" t="n"/>
       <c r="T27" s="20" t="n"/>
       <c r="U27" s="20" t="n"/>
-      <c r="Y27" t="n">
-        <v>0</v>
-      </c>
       <c r="Z27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA27" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC27" t="n">
         <v>6</v>
       </c>
       <c r="AD27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG27" t="n">
         <v>6</v>
@@ -6037,13 +6114,13 @@
         <v>0</v>
       </c>
       <c r="AL27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO27" t="n">
         <v>6</v>
@@ -6053,21 +6130,24 @@
       </c>
       <c r="AQ27" t="n">
         <v>6</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AQ28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AR28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6080,14 +6160,11 @@
       <c r="S28" s="20" t="n"/>
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
-      <c r="Z28" t="n">
-        <v>6</v>
-      </c>
       <c r="AA28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC28" t="n">
         <v>6</v>
@@ -6099,7 +6176,7 @@
         <v>6</v>
       </c>
       <c r="AF28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG28" t="n">
         <v>6</v>
@@ -6120,25 +6197,28 @@
         <v>6</v>
       </c>
       <c r="AM28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR28" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
@@ -6147,7 +6227,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AQ29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AR29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6161,7 +6241,7 @@
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
       <c r="AA29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -6170,16 +6250,16 @@
         <v>6</v>
       </c>
       <c r="AD29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF29" t="n">
         <v>0</v>
       </c>
       <c r="AG29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH29" t="n">
         <v>0</v>
@@ -6194,7 +6274,7 @@
         <v>0</v>
       </c>
       <c r="AL29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM29" t="n">
         <v>0</v>
@@ -6209,22 +6289,25 @@
         <v>0</v>
       </c>
       <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AQ30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AR30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -6237,71 +6320,71 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="AA30" t="n">
-        <v>3</v>
-      </c>
       <c r="AB30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC30" t="n">
         <v>6</v>
       </c>
       <c r="AD30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AN30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AO30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AP30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AQ30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AQ31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AR31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -6314,9 +6397,6 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="AB31" t="n">
-        <v>6</v>
-      </c>
       <c r="AC31" t="n">
         <v>6</v>
       </c>
@@ -6324,58 +6404,61 @@
         <v>6</v>
       </c>
       <c r="AE31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AK31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ31" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AQ32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AR32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -6388,14 +6471,11 @@
       <c r="S32" s="20" t="n"/>
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
-      <c r="AC32" t="n">
-        <v>6</v>
-      </c>
       <c r="AD32" t="n">
         <v>6</v>
       </c>
       <c r="AE32" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AF32" t="n">
         <v>6</v>
@@ -6404,19 +6484,19 @@
         <v>6</v>
       </c>
       <c r="AH32" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -6431,22 +6511,25 @@
         <v>0</v>
       </c>
       <c r="AQ32" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AQ33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AR33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -6459,17 +6542,11 @@
       <c r="S33" s="20" t="n"/>
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
-      <c r="AC33" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>6</v>
-      </c>
       <c r="AE33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG33" t="n">
         <v>0</v>
@@ -6502,22 +6579,25 @@
         <v>0</v>
       </c>
       <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AQ34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AR34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -6530,17 +6610,14 @@
       <c r="S34" s="20" t="n"/>
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
-      <c r="AD34" t="n">
-        <v>6</v>
-      </c>
       <c r="AE34" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF34" t="n">
         <v>6</v>
       </c>
       <c r="AG34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH34" t="n">
         <v>0</v>
@@ -6549,13 +6626,13 @@
         <v>0</v>
       </c>
       <c r="AJ34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM34" t="n">
         <v>0</v>
@@ -6570,22 +6647,25 @@
         <v>0</v>
       </c>
       <c r="AQ34" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AQ35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AR35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -6599,7 +6679,7 @@
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
       <c r="AE35" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF35" t="n">
         <v>6</v>
@@ -6635,22 +6715,25 @@
         <v>0</v>
       </c>
       <c r="AQ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AQ36), 0)</f>
+        <f>ROUND(AVERAGE(D36:AR36), 0)</f>
         <v/>
       </c>
       <c r="K36" s="6" t="n"/>
@@ -6667,7 +6750,7 @@
         <v>6</v>
       </c>
       <c r="AF36" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG36" t="n">
         <v>0</v>
@@ -6679,13 +6762,13 @@
         <v>0</v>
       </c>
       <c r="AJ36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -6694,142 +6777,15 @@
         <v>0</v>
       </c>
       <c r="AO36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP36" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="28" t="inlineStr">
-        <is>
-          <t>Akemi</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="C37" s="28">
-        <f>ROUND(AVERAGE(D37:AQ37), 0)</f>
-        <v/>
-      </c>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
-      <c r="N37" s="6" t="n"/>
-      <c r="O37" s="20" t="n"/>
-      <c r="P37" s="20" t="n"/>
-      <c r="Q37" s="20" t="n"/>
-      <c r="R37" s="20" t="n"/>
-      <c r="S37" s="20" t="n"/>
-      <c r="T37" s="20" t="n"/>
-      <c r="U37" s="20" t="n"/>
-      <c r="AE37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF37" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP37" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ37" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="28" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
-      <c r="C38" s="28">
-        <f>ROUND(AVERAGE(D38:AQ38), 0)</f>
-        <v/>
-      </c>
-      <c r="K38" s="6" t="n"/>
-      <c r="L38" s="6" t="n"/>
-      <c r="N38" s="6" t="n"/>
-      <c r="O38" s="20" t="n"/>
-      <c r="P38" s="20" t="n"/>
-      <c r="Q38" s="20" t="n"/>
-      <c r="R38" s="20" t="n"/>
-      <c r="S38" s="20" t="n"/>
-      <c r="T38" s="20" t="n"/>
-      <c r="U38" s="20" t="n"/>
-      <c r="AE38" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN38" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO38" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP38" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR36" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-05
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS36"/>
+  <dimension ref="A1:AT35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2998,6 +2998,11 @@
           <t>03/07/2026</t>
         </is>
       </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3011,7 +3016,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AS2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AT2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3117,6 +3122,9 @@
         <v>0</v>
       </c>
       <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3132,7 +3140,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AS3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AT3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3229,6 +3237,9 @@
       <c r="AS3" t="n">
         <v>6</v>
       </c>
+      <c r="AT3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3242,7 +3253,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AS4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AT4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3362,6 +3373,9 @@
       <c r="AS4" t="n">
         <v>0</v>
       </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3375,7 +3389,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AS5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AT5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3503,6 +3517,9 @@
       </c>
       <c r="AS5" t="n">
         <v>0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3517,7 +3534,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AS6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AT6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3646,6 +3663,9 @@
       <c r="AS6" t="n">
         <v>0</v>
       </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3659,7 +3679,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AS7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AT7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3758,6 +3778,9 @@
       <c r="AS7" t="n">
         <v>0</v>
       </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3771,7 +3794,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AS8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AT8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3891,6 +3914,9 @@
       <c r="AS8" t="n">
         <v>0</v>
       </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3904,7 +3930,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AS9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AT9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -3991,6 +4017,9 @@
       <c r="AS9" t="n">
         <v>0</v>
       </c>
+      <c r="AT9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4004,7 +4033,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AS10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AT10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -4124,6 +4153,9 @@
       <c r="AS10" t="n">
         <v>0</v>
       </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4137,7 +4169,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AS11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AT11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4266,6 +4298,9 @@
       <c r="AS11" t="n">
         <v>6</v>
       </c>
+      <c r="AT11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4279,7 +4314,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AS12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AT12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4394,6 +4429,9 @@
         <v>6</v>
       </c>
       <c r="AS12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4409,7 +4447,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AS13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AT13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4537,6 +4575,9 @@
       </c>
       <c r="AS13" t="n">
         <v>0</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4551,7 +4592,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AS14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AT14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4655,6 +4696,9 @@
       <c r="AS14" t="n">
         <v>6</v>
       </c>
+      <c r="AT14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4668,7 +4712,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AS15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AT15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4761,6 +4805,9 @@
       <c r="AS15" t="n">
         <v>6</v>
       </c>
+      <c r="AT15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4774,7 +4821,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AS16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AT16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4894,6 +4941,9 @@
       <c r="AS16" t="n">
         <v>1</v>
       </c>
+      <c r="AT16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -4907,7 +4957,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AS17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AT17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5036,6 +5086,9 @@
       <c r="AS17" t="n">
         <v>0</v>
       </c>
+      <c r="AT17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5049,7 +5102,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AS18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AT18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5167,6 +5220,9 @@
         <v>0</v>
       </c>
       <c r="AS18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5182,7 +5238,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AS19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AT19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -5287,6 +5343,9 @@
       <c r="AS19" t="n">
         <v>0</v>
       </c>
+      <c r="AT19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5300,7 +5359,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AS20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AT20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -5408,6 +5467,9 @@
       <c r="AS20" t="n">
         <v>0</v>
       </c>
+      <c r="AT20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5421,7 +5483,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AS21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AT21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5550,6 +5612,9 @@
       <c r="AS21" t="n">
         <v>3</v>
       </c>
+      <c r="AT21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5563,7 +5628,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AS22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AT22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5692,6 +5757,9 @@
       <c r="AS22" t="n">
         <v>0</v>
       </c>
+      <c r="AT22" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5705,7 +5773,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AS23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AT23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5814,6 +5882,9 @@
       <c r="AS23" t="n">
         <v>0</v>
       </c>
+      <c r="AT23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5827,7 +5898,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AS24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AT24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -5947,6 +6018,9 @@
       <c r="AS24" t="n">
         <v>6</v>
       </c>
+      <c r="AT24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -5960,7 +6034,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AS25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AT25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6042,6 +6116,9 @@
       <c r="AS25" t="n">
         <v>5</v>
       </c>
+      <c r="AT25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6055,7 +6132,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AS26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AT26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6131,6 +6208,9 @@
       <c r="AS26" t="n">
         <v>5</v>
       </c>
+      <c r="AT26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6144,7 +6224,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AS27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AT27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6217,11 +6297,14 @@
       <c r="AS27" t="n">
         <v>0</v>
       </c>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -6230,7 +6313,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AS28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AT28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6244,7 +6327,7 @@
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
       <c r="AA28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB28" t="n">
         <v>0</v>
@@ -6253,16 +6336,16 @@
         <v>6</v>
       </c>
       <c r="AD28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
       </c>
       <c r="AG28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH28" t="n">
         <v>0</v>
@@ -6277,7 +6360,7 @@
         <v>0</v>
       </c>
       <c r="AL28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM28" t="n">
         <v>0</v>
@@ -6295,25 +6378,28 @@
         <v>0</v>
       </c>
       <c r="AR28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS28" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AS29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AT29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6326,77 +6412,77 @@
       <c r="S29" s="20" t="n"/>
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
-      <c r="AA29" t="n">
-        <v>3</v>
-      </c>
       <c r="AB29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC29" t="n">
         <v>6</v>
       </c>
       <c r="AD29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AN29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AO29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AP29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AQ29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AR29" t="n">
         <v>0</v>
       </c>
       <c r="AS29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AS30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AT30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -6409,9 +6495,6 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="AB30" t="n">
-        <v>6</v>
-      </c>
       <c r="AC30" t="n">
         <v>6</v>
       </c>
@@ -6419,64 +6502,67 @@
         <v>6</v>
       </c>
       <c r="AE30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AK30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ30" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AR30" t="n">
         <v>0</v>
       </c>
       <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AS31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AT31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -6489,20 +6575,17 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="AC31" t="n">
-        <v>6</v>
-      </c>
       <c r="AD31" t="n">
         <v>6</v>
       </c>
       <c r="AE31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH31" t="n">
         <v>0</v>
@@ -6532,28 +6615,31 @@
         <v>0</v>
       </c>
       <c r="AQ31" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS31" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AS32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AT32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -6566,17 +6652,14 @@
       <c r="S32" s="20" t="n"/>
       <c r="T32" s="20" t="n"/>
       <c r="U32" s="20" t="n"/>
-      <c r="AD32" t="n">
-        <v>6</v>
-      </c>
       <c r="AE32" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF32" t="n">
         <v>6</v>
       </c>
       <c r="AG32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH32" t="n">
         <v>0</v>
@@ -6606,19 +6689,22 @@
         <v>0</v>
       </c>
       <c r="AQ32" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AR32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS32" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
@@ -6627,7 +6713,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AS33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AT33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -6656,13 +6742,13 @@
         <v>0</v>
       </c>
       <c r="AJ33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM33" t="n">
         <v>0</v>
@@ -6683,22 +6769,25 @@
         <v>0</v>
       </c>
       <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AS34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AT34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -6712,7 +6801,7 @@
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
       <c r="AE34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF34" t="n">
         <v>6</v>
@@ -6727,13 +6816,13 @@
         <v>0</v>
       </c>
       <c r="AJ34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM34" t="n">
         <v>0</v>
@@ -6754,22 +6843,25 @@
         <v>0</v>
       </c>
       <c r="AS34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT34" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AS35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AT35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -6783,10 +6875,10 @@
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
       <c r="AE35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF35" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -6813,89 +6905,21 @@
         <v>0</v>
       </c>
       <c r="AO35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS35" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="28" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
-      <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AS36), 0)</f>
-        <v/>
-      </c>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-      <c r="N36" s="6" t="n"/>
-      <c r="O36" s="20" t="n"/>
-      <c r="P36" s="20" t="n"/>
-      <c r="Q36" s="20" t="n"/>
-      <c r="R36" s="20" t="n"/>
-      <c r="S36" s="20" t="n"/>
-      <c r="T36" s="20" t="n"/>
-      <c r="U36" s="20" t="n"/>
-      <c r="AE36" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF36" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN36" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO36" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP36" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ36" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR36" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS36" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT35" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-06
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU35"/>
+  <dimension ref="A1:AV36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3008,6 +3008,11 @@
           <t>03/07/2026</t>
         </is>
       </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3021,7 +3026,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AU2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AV2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3133,6 +3138,9 @@
         <v>0</v>
       </c>
       <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3148,7 +3156,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AU3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AV3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3251,6 +3259,9 @@
       <c r="AU3" t="n">
         <v>6</v>
       </c>
+      <c r="AV3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3264,7 +3275,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AU4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AV4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3390,6 +3401,9 @@
       <c r="AU4" t="n">
         <v>0</v>
       </c>
+      <c r="AV4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3403,7 +3417,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AU5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AV5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3536,6 +3550,9 @@
         <v>6</v>
       </c>
       <c r="AU5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV5" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3551,7 +3568,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AU6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AV6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3686,6 +3703,9 @@
       <c r="AU6" t="n">
         <v>0</v>
       </c>
+      <c r="AV6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3699,7 +3719,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AU7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AV7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3804,6 +3824,9 @@
       <c r="AU7" t="n">
         <v>0</v>
       </c>
+      <c r="AV7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3817,7 +3840,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AU8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AV8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3943,6 +3966,9 @@
       <c r="AU8" t="n">
         <v>0</v>
       </c>
+      <c r="AV8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3956,7 +3982,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AU9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AV9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -4049,6 +4075,9 @@
       <c r="AU9" t="n">
         <v>0</v>
       </c>
+      <c r="AV9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4062,7 +4091,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AU10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AV10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -4188,6 +4217,9 @@
       <c r="AU10" t="n">
         <v>0</v>
       </c>
+      <c r="AV10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4201,7 +4233,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AU11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AV11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4336,6 +4368,9 @@
       <c r="AU11" t="n">
         <v>6</v>
       </c>
+      <c r="AV11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4349,7 +4384,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AU12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AV12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4470,6 +4505,9 @@
         <v>6</v>
       </c>
       <c r="AU12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4485,7 +4523,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AU13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AV13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4618,6 +4656,9 @@
         <v>6</v>
       </c>
       <c r="AU13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV13" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4633,7 +4674,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AU14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AV14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4743,6 +4784,9 @@
       <c r="AU14" t="n">
         <v>6</v>
       </c>
+      <c r="AV14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4756,7 +4800,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AU15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AV15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4855,6 +4899,9 @@
       <c r="AU15" t="n">
         <v>6</v>
       </c>
+      <c r="AV15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4868,7 +4915,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AU16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AV16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -4994,6 +5041,9 @@
       <c r="AU16" t="n">
         <v>1</v>
       </c>
+      <c r="AV16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5007,7 +5057,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AU17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AV17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5142,6 +5192,9 @@
       <c r="AU17" t="n">
         <v>6</v>
       </c>
+      <c r="AV17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5155,7 +5208,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AU18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AV18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5279,6 +5332,9 @@
         <v>0</v>
       </c>
       <c r="AU18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5294,7 +5350,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AU19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AV19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -5405,6 +5461,9 @@
       <c r="AU19" t="n">
         <v>0</v>
       </c>
+      <c r="AV19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5418,7 +5477,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AU20), 0)</f>
+        <f>ROUND(AVERAGE(D20:AV20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n">
@@ -5532,6 +5591,9 @@
       <c r="AU20" t="n">
         <v>0</v>
       </c>
+      <c r="AV20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5545,7 +5607,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AU21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AV21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
@@ -5680,6 +5742,9 @@
       <c r="AU21" t="n">
         <v>6</v>
       </c>
+      <c r="AV21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5693,7 +5758,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AU22), 0)</f>
+        <f>ROUND(AVERAGE(D22:AV22), 0)</f>
         <v/>
       </c>
       <c r="D22" s="10" t="n">
@@ -5828,6 +5893,9 @@
       <c r="AU22" t="n">
         <v>2</v>
       </c>
+      <c r="AV22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -5841,7 +5909,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AU23), 0)</f>
+        <f>ROUND(AVERAGE(D23:AV23), 0)</f>
         <v/>
       </c>
       <c r="J23" s="6" t="n"/>
@@ -5956,6 +6024,9 @@
       <c r="AU23" t="n">
         <v>0</v>
       </c>
+      <c r="AV23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -5969,7 +6040,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AU24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AV24), 0)</f>
         <v/>
       </c>
       <c r="G24" s="5" t="n">
@@ -6095,6 +6166,9 @@
       <c r="AU24" t="n">
         <v>6</v>
       </c>
+      <c r="AV24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6108,7 +6182,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AU25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AV25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6196,6 +6270,9 @@
       <c r="AU25" t="n">
         <v>5</v>
       </c>
+      <c r="AV25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6209,7 +6286,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AU26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AV26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6291,6 +6368,9 @@
       <c r="AU26" t="n">
         <v>5</v>
       </c>
+      <c r="AV26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6304,7 +6384,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AU27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AV27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6383,6 +6463,9 @@
       <c r="AU27" t="n">
         <v>0</v>
       </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -6396,7 +6479,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AU28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AV28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6472,6 +6555,9 @@
       <c r="AU28" t="n">
         <v>0</v>
       </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -6485,7 +6571,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AU29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AV29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6558,6 +6644,9 @@
       <c r="AU29" t="n">
         <v>0</v>
       </c>
+      <c r="AV29" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
@@ -6571,7 +6660,7 @@
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AU30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AV30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -6641,6 +6730,9 @@
       <c r="AU30" t="n">
         <v>0</v>
       </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -6654,7 +6746,7 @@
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AU31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AV31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -6721,6 +6813,9 @@
       <c r="AU31" t="n">
         <v>3</v>
       </c>
+      <c r="AV31" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
@@ -6734,7 +6829,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AU32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AV32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -6798,6 +6893,9 @@
       <c r="AU32" t="n">
         <v>0</v>
       </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
@@ -6811,7 +6909,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AU33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AV33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -6875,6 +6973,9 @@
       <c r="AU33" t="n">
         <v>0</v>
       </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
@@ -6888,7 +6989,7 @@
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AU34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AV34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -6952,6 +7053,9 @@
       <c r="AU34" t="n">
         <v>0</v>
       </c>
+      <c r="AV34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
@@ -6965,7 +7069,7 @@
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AU35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AV35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -7027,6 +7131,38 @@
         <v>6</v>
       </c>
       <c r="AU35" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>xNullx</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C36" s="28">
+        <f>ROUND(AVERAGE(D36:AV36), 0)</f>
+        <v/>
+      </c>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="6" t="n"/>
+      <c r="N36" s="6" t="n"/>
+      <c r="O36" s="20" t="n"/>
+      <c r="P36" s="20" t="n"/>
+      <c r="Q36" s="20" t="n"/>
+      <c r="R36" s="20" t="n"/>
+      <c r="S36" s="20" t="n"/>
+      <c r="T36" s="20" t="n"/>
+      <c r="U36" s="20" t="n"/>
+      <c r="AV36" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-11
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV36"/>
+  <dimension ref="A1:AW35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3013,6 +3013,11 @@
           <t>03/07/2026</t>
         </is>
       </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3026,7 +3031,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AV2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AW2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3141,6 +3146,9 @@
         <v>0</v>
       </c>
       <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3156,7 +3164,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AV3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AW3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3262,6 +3270,9 @@
       <c r="AV3" t="n">
         <v>6</v>
       </c>
+      <c r="AW3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3275,7 +3286,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AV4), 0)</f>
+        <f>ROUND(AVERAGE(D4:AW4), 0)</f>
         <v/>
       </c>
       <c r="G4" s="5" t="n">
@@ -3404,6 +3415,9 @@
       <c r="AV4" t="n">
         <v>6</v>
       </c>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3417,7 +3431,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AV5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AW5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3554,6 +3568,9 @@
       </c>
       <c r="AV5" t="n">
         <v>6</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3568,7 +3585,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AV6), 0)</f>
+        <f>ROUND(AVERAGE(D6:AW6), 0)</f>
         <v/>
       </c>
       <c r="D6" s="10" t="n">
@@ -3706,6 +3723,9 @@
       <c r="AV6" t="n">
         <v>0</v>
       </c>
+      <c r="AW6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3719,7 +3739,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AV7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AW7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3827,6 +3847,9 @@
       <c r="AV7" t="n">
         <v>0</v>
       </c>
+      <c r="AW7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3840,7 +3863,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AV8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AW8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3969,6 +3992,9 @@
       <c r="AV8" t="n">
         <v>0</v>
       </c>
+      <c r="AW8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3982,7 +4008,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AV9), 0)</f>
+        <f>ROUND(AVERAGE(D9:AW9), 0)</f>
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
@@ -4078,6 +4104,9 @@
       <c r="AV9" t="n">
         <v>0</v>
       </c>
+      <c r="AW9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4091,7 +4120,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AV10), 0)</f>
+        <f>ROUND(AVERAGE(D10:AW10), 0)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
@@ -4220,6 +4249,9 @@
       <c r="AV10" t="n">
         <v>0</v>
       </c>
+      <c r="AW10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4233,7 +4265,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AV11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AW11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4371,6 +4403,9 @@
       <c r="AV11" t="n">
         <v>6</v>
       </c>
+      <c r="AW11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4384,7 +4419,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AV12), 0)</f>
+        <f>ROUND(AVERAGE(D12:AW12), 0)</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
@@ -4509,6 +4544,9 @@
       </c>
       <c r="AV12" t="n">
         <v>6</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -4523,7 +4561,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AV13), 0)</f>
+        <f>ROUND(AVERAGE(D13:AW13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -4660,6 +4698,9 @@
       </c>
       <c r="AV13" t="n">
         <v>6</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4674,7 +4715,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AV14), 0)</f>
+        <f>ROUND(AVERAGE(D14:AW14), 0)</f>
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
@@ -4787,6 +4828,9 @@
       <c r="AV14" t="n">
         <v>6</v>
       </c>
+      <c r="AW14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4800,7 +4844,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AV15), 0)</f>
+        <f>ROUND(AVERAGE(D15:AW15), 0)</f>
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
@@ -4902,6 +4946,9 @@
       <c r="AV15" t="n">
         <v>6</v>
       </c>
+      <c r="AW15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -4915,7 +4962,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AV16), 0)</f>
+        <f>ROUND(AVERAGE(D16:AW16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -5044,6 +5091,9 @@
       <c r="AV16" t="n">
         <v>6</v>
       </c>
+      <c r="AW16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5057,7 +5107,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AV17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AW17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5195,6 +5245,9 @@
       <c r="AV17" t="n">
         <v>6</v>
       </c>
+      <c r="AW17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5208,7 +5261,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AV18), 0)</f>
+        <f>ROUND(AVERAGE(D18:AW18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5335,6 +5388,9 @@
         <v>0</v>
       </c>
       <c r="AV18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5350,7 +5406,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AV19), 0)</f>
+        <f>ROUND(AVERAGE(D19:AW19), 0)</f>
         <v/>
       </c>
       <c r="L19" s="6" t="n">
@@ -5464,21 +5520,45 @@
       <c r="AV19" t="n">
         <v>0</v>
       </c>
+      <c r="AW19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AV20), 0)</f>
-        <v/>
+        <f>ROUND(AVERAGE(D20:AW20), 0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>6</v>
@@ -5508,29 +5588,29 @@
         <v>6</v>
       </c>
       <c r="T20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V20" t="n">
         <v>6</v>
       </c>
       <c r="W20" t="n">
+        <v>3</v>
+      </c>
+      <c r="X20" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="n">
         <v>4</v>
       </c>
-      <c r="X20" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>2</v>
-      </c>
       <c r="AB20" t="n">
         <v>6</v>
       </c>
@@ -5538,16 +5618,16 @@
         <v>6</v>
       </c>
       <c r="AD20" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE20" t="n">
         <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH20" t="n">
         <v>0</v>
@@ -5565,40 +5645,43 @@
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
@@ -5607,11 +5690,11 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AV21), 0)</f>
+        <f>ROUND(AVERAGE(D21:AW21), 0)</f>
         <v/>
       </c>
       <c r="D21" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>6</v>
@@ -5629,7 +5712,7 @@
         <v>6</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>6</v>
@@ -5655,23 +5738,23 @@
       <c r="R21" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S21" t="n">
+      <c r="S21" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
@@ -5680,7 +5763,7 @@
         <v>0</v>
       </c>
       <c r="AA21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB21" t="n">
         <v>6</v>
@@ -5695,7 +5778,7 @@
         <v>0</v>
       </c>
       <c r="AF21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG21" t="n">
         <v>6</v>
@@ -5716,40 +5799,43 @@
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AP21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AQ21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AR21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT21" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AU21" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AV21" t="n">
         <v>6</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -5758,92 +5844,72 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AV22), 0)</f>
-        <v/>
-      </c>
-      <c r="D22" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J22" s="6" t="n">
+        <f>ROUND(AVERAGE(D22:AW22), 0)</f>
+        <v/>
+      </c>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N22" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O22" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P22" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q22" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R22" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S22" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T22" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U22" t="n">
+        <v>6</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
         <v>5</v>
       </c>
-      <c r="K22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T22" t="n">
-        <v>6</v>
-      </c>
-      <c r="U22" t="n">
-        <v>6</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" t="n">
-        <v>0</v>
-      </c>
       <c r="X22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB22" t="n">
         <v>6</v>
       </c>
       <c r="AC22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF22" t="n">
         <v>6</v>
@@ -5873,10 +5939,10 @@
         <v>0</v>
       </c>
       <c r="AO22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ22" t="n">
         <v>6</v>
@@ -5888,19 +5954,22 @@
         <v>0</v>
       </c>
       <c r="AT22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV22" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -5909,10 +5978,21 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AV23), 0)</f>
-        <v/>
-      </c>
-      <c r="J23" s="6" t="n"/>
+        <f>ROUND(AVERAGE(D23:AW23), 0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K23" s="6" t="n">
         <v>6</v>
       </c>
@@ -5929,7 +6009,7 @@
         <v>6</v>
       </c>
       <c r="P23" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q23" s="20" t="n">
         <v>6</v>
@@ -5943,26 +6023,26 @@
       <c r="T23" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="U23" t="n">
+      <c r="U23" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
       </c>
       <c r="W23" t="n">
+        <v>6</v>
+      </c>
+      <c r="X23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" t="n">
         <v>5</v>
       </c>
-      <c r="X23" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>6</v>
-      </c>
       <c r="AA23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB23" t="n">
         <v>6</v>
@@ -5980,22 +6060,22 @@
         <v>6</v>
       </c>
       <c r="AG23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AM23" t="n">
         <v>0</v>
@@ -6010,111 +6090,76 @@
         <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV23" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AV24), 0)</f>
-        <v/>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M24" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N24" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P24" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U24" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
+        <f>ROUND(AVERAGE(D24:AW24), 0)</f>
+        <v/>
+      </c>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="n"/>
+      <c r="N24" s="6" t="n"/>
+      <c r="O24" s="20" t="n"/>
+      <c r="P24" s="20" t="n"/>
+      <c r="Q24" s="20" t="n"/>
+      <c r="R24" s="20" t="n"/>
+      <c r="S24" s="20" t="n"/>
+      <c r="T24" s="20" t="n"/>
+      <c r="U24" s="20" t="n"/>
       <c r="W24" t="n">
         <v>6</v>
       </c>
       <c r="X24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y24" t="n">
         <v>0</v>
       </c>
       <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD24" t="n">
         <v>5</v>
       </c>
-      <c r="AA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>6</v>
-      </c>
       <c r="AE24" t="n">
         <v>6</v>
       </c>
@@ -6125,64 +6170,67 @@
         <v>0</v>
       </c>
       <c r="AH24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR24" t="n">
         <v>5</v>
       </c>
-      <c r="AI24" t="n">
+      <c r="AS24" t="n">
         <v>5</v>
       </c>
-      <c r="AJ24" t="n">
+      <c r="AT24" t="n">
         <v>5</v>
       </c>
-      <c r="AK24" t="n">
+      <c r="AU24" t="n">
         <v>5</v>
       </c>
-      <c r="AL24" t="n">
+      <c r="AV24" t="n">
         <v>5</v>
       </c>
-      <c r="AM24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AV24" t="n">
-        <v>6</v>
+      <c r="AW24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AV25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AW25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6195,65 +6243,59 @@
       <c r="S25" s="20" t="n"/>
       <c r="T25" s="20" t="n"/>
       <c r="U25" s="20" t="n"/>
-      <c r="W25" t="n">
-        <v>6</v>
-      </c>
-      <c r="X25" t="n">
-        <v>6</v>
-      </c>
       <c r="Y25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA25" t="n">
         <v>6</v>
       </c>
       <c r="AB25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC25" t="n">
         <v>6</v>
       </c>
       <c r="AD25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO25" t="n">
         <v>5</v>
       </c>
-      <c r="AE25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AO25" t="n">
-        <v>6</v>
-      </c>
       <c r="AP25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ25" t="n">
         <v>6</v>
@@ -6271,22 +6313,25 @@
         <v>5</v>
       </c>
       <c r="AV25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW25" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AV26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AW26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6299,15 +6344,12 @@
       <c r="S26" s="20" t="n"/>
       <c r="T26" s="20" t="n"/>
       <c r="U26" s="20" t="n"/>
-      <c r="Y26" t="n">
-        <v>6</v>
-      </c>
       <c r="Z26" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA26" t="n">
         <v>3</v>
       </c>
-      <c r="AA26" t="n">
-        <v>6</v>
-      </c>
       <c r="AB26" t="n">
         <v>6</v>
       </c>
@@ -6333,58 +6375,61 @@
         <v>0</v>
       </c>
       <c r="AJ26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL26" t="n">
         <v>6</v>
       </c>
       <c r="AM26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ26" t="n">
         <v>6</v>
       </c>
       <c r="AR26" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT26" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AU26" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV26" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AV27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AW27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6397,29 +6442,26 @@
       <c r="S27" s="20" t="n"/>
       <c r="T27" s="20" t="n"/>
       <c r="U27" s="20" t="n"/>
-      <c r="Z27" t="n">
-        <v>6</v>
-      </c>
       <c r="AA27" t="n">
         <v>3</v>
       </c>
       <c r="AB27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC27" t="n">
         <v>6</v>
       </c>
       <c r="AD27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH27" t="n">
         <v>0</v>
@@ -6434,22 +6476,22 @@
         <v>0</v>
       </c>
       <c r="AL27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ27" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR27" t="n">
         <v>0</v>
@@ -6464,22 +6506,25 @@
         <v>0</v>
       </c>
       <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AV28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AW28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6492,56 +6537,53 @@
       <c r="S28" s="20" t="n"/>
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
-      <c r="AA28" t="n">
-        <v>3</v>
-      </c>
       <c r="AB28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC28" t="n">
         <v>6</v>
       </c>
       <c r="AD28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AN28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AO28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AP28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AQ28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AR28" t="n">
         <v>0</v>
@@ -6556,22 +6598,25 @@
         <v>0</v>
       </c>
       <c r="AV28" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AV29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AW29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6584,9 +6629,6 @@
       <c r="S29" s="20" t="n"/>
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
-      <c r="AB29" t="n">
-        <v>6</v>
-      </c>
       <c r="AC29" t="n">
         <v>6</v>
       </c>
@@ -6594,43 +6636,43 @@
         <v>6</v>
       </c>
       <c r="AE29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AK29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AL29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AR29" t="n">
         <v>0</v>
@@ -6645,22 +6687,25 @@
         <v>0</v>
       </c>
       <c r="AV29" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AV30), 0)</f>
+        <f>ROUND(AVERAGE(D30:AW30), 0)</f>
         <v/>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -6673,20 +6718,17 @@
       <c r="S30" s="20" t="n"/>
       <c r="T30" s="20" t="n"/>
       <c r="U30" s="20" t="n"/>
-      <c r="AC30" t="n">
-        <v>6</v>
-      </c>
       <c r="AD30" t="n">
         <v>6</v>
       </c>
       <c r="AE30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH30" t="n">
         <v>0</v>
@@ -6716,37 +6758,40 @@
         <v>0</v>
       </c>
       <c r="AQ30" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AV31), 0)</f>
+        <f>ROUND(AVERAGE(D31:AW31), 0)</f>
         <v/>
       </c>
       <c r="K31" s="6" t="n"/>
@@ -6759,17 +6804,14 @@
       <c r="S31" s="20" t="n"/>
       <c r="T31" s="20" t="n"/>
       <c r="U31" s="20" t="n"/>
-      <c r="AD31" t="n">
-        <v>6</v>
-      </c>
       <c r="AE31" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF31" t="n">
         <v>6</v>
       </c>
       <c r="AG31" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH31" t="n">
         <v>0</v>
@@ -6799,28 +6841,31 @@
         <v>0</v>
       </c>
       <c r="AQ31" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AR31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV31" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -6829,7 +6874,7 @@
         </is>
       </c>
       <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AV32), 0)</f>
+        <f>ROUND(AVERAGE(D32:AW32), 0)</f>
         <v/>
       </c>
       <c r="K32" s="6" t="n"/>
@@ -6858,13 +6903,13 @@
         <v>0</v>
       </c>
       <c r="AJ32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -6895,21 +6940,24 @@
       </c>
       <c r="AV32" t="n">
         <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AV33), 0)</f>
+        <f>ROUND(AVERAGE(D33:AW33), 0)</f>
         <v/>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -6923,7 +6971,7 @@
       <c r="T33" s="20" t="n"/>
       <c r="U33" s="20" t="n"/>
       <c r="AE33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF33" t="n">
         <v>6</v>
@@ -6938,13 +6986,13 @@
         <v>0</v>
       </c>
       <c r="AJ33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL33" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM33" t="n">
         <v>0</v>
@@ -6974,22 +7022,25 @@
         <v>0</v>
       </c>
       <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AV34), 0)</f>
+        <f>ROUND(AVERAGE(D34:AW34), 0)</f>
         <v/>
       </c>
       <c r="K34" s="6" t="n"/>
@@ -7003,10 +7054,10 @@
       <c r="T34" s="20" t="n"/>
       <c r="U34" s="20" t="n"/>
       <c r="AE34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG34" t="n">
         <v>0</v>
@@ -7033,43 +7084,46 @@
         <v>0</v>
       </c>
       <c r="AO34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV34" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW34" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AV35), 0)</f>
+        <f>ROUND(AVERAGE(D35:AW35), 0)</f>
         <v/>
       </c>
       <c r="K35" s="6" t="n"/>
@@ -7082,88 +7136,11 @@
       <c r="S35" s="20" t="n"/>
       <c r="T35" s="20" t="n"/>
       <c r="U35" s="20" t="n"/>
-      <c r="AE35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU35" t="n">
-        <v>6</v>
-      </c>
       <c r="AV35" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="28" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C36" s="28">
-        <f>ROUND(AVERAGE(D36:AV36), 0)</f>
-        <v/>
-      </c>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-      <c r="N36" s="6" t="n"/>
-      <c r="O36" s="20" t="n"/>
-      <c r="P36" s="20" t="n"/>
-      <c r="Q36" s="20" t="n"/>
-      <c r="R36" s="20" t="n"/>
-      <c r="S36" s="20" t="n"/>
-      <c r="T36" s="20" t="n"/>
-      <c r="U36" s="20" t="n"/>
-      <c r="AV36" t="n">
-        <v>6</v>
+      <c r="AW35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-12
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX35"/>
+  <dimension ref="A1:AY29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3023,6 +3023,11 @@
           <t>10/07/2026</t>
         </is>
       </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3036,7 +3041,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AX2), 0)</f>
+        <f>ROUND(AVERAGE(D2:AY2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3157,6 +3162,9 @@
         <v>0</v>
       </c>
       <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3172,7 +3180,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AX3), 0)</f>
+        <f>ROUND(AVERAGE(D3:AY3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3284,11 +3292,14 @@
       <c r="AX3" t="n">
         <v>6</v>
       </c>
+      <c r="AY3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -3297,14 +3308,23 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AX4), 0)</f>
-        <v/>
+        <f>ROUND(AVERAGE(D4:AY4), 0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>6</v>
@@ -3316,13 +3336,13 @@
         <v>6</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N4" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O4" t="n">
         <v>6</v>
@@ -3340,19 +3360,19 @@
         <v>6</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U4" t="n">
         <v>6</v>
       </c>
       <c r="V4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y4" t="n">
         <v>6</v>
@@ -3370,16 +3390,16 @@
         <v>6</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF4" t="n">
         <v>6</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH4" t="n">
         <v>0</v>
@@ -3394,7 +3414,7 @@
         <v>0</v>
       </c>
       <c r="AL4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM4" t="n">
         <v>0</v>
@@ -3418,10 +3438,10 @@
         <v>0</v>
       </c>
       <c r="AT4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV4" t="n">
         <v>6</v>
@@ -3430,13 +3450,16 @@
         <v>0</v>
       </c>
       <c r="AX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -3445,7 +3468,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AX5), 0)</f>
+        <f>ROUND(AVERAGE(D5:AY5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3464,34 +3487,34 @@
         <v>0</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N5" s="13" t="n">
         <v>6</v>
       </c>
       <c r="O5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>6</v>
@@ -3506,37 +3529,37 @@
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y5" t="n">
         <v>6</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB5" t="n">
         <v>6</v>
       </c>
       <c r="AC5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="n">
         <v>0</v>
@@ -3551,7 +3574,7 @@
         <v>0</v>
       </c>
       <c r="AL5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM5" t="n">
         <v>0</v>
@@ -3566,7 +3589,7 @@
         <v>0</v>
       </c>
       <c r="AQ5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR5" t="n">
         <v>0</v>
@@ -3575,80 +3598,53 @@
         <v>0</v>
       </c>
       <c r="AT5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AU5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AV5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
       </c>
       <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AX6), 0)</f>
-        <v/>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="13" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D6:AY6), 0)</f>
+        <v/>
+      </c>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+      <c r="N6" s="13" t="n"/>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S6" t="n">
         <v>6</v>
@@ -3660,13 +3656,13 @@
         <v>6</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W6" t="n">
         <v>6</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y6" t="n">
         <v>6</v>
@@ -3675,10 +3671,10 @@
         <v>6</v>
       </c>
       <c r="AA6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -3744,65 +3740,56 @@
         <v>0</v>
       </c>
       <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AX7), 0)</f>
+        <f>ROUND(AVERAGE(D7:AY7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="6" t="n"/>
       <c r="N7" s="13" t="n"/>
-      <c r="O7" t="n">
-        <v>6</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>6</v>
-      </c>
-      <c r="S7" t="n">
-        <v>6</v>
-      </c>
-      <c r="T7" t="n">
-        <v>6</v>
-      </c>
+      <c r="O7" s="19" t="n"/>
+      <c r="P7" s="19" t="n"/>
+      <c r="Q7" s="19" t="n"/>
+      <c r="R7" s="19" t="n"/>
+      <c r="S7" s="19" t="n"/>
+      <c r="T7" s="19" t="n"/>
       <c r="U7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Y7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB7" t="n">
         <v>0</v>
@@ -3811,13 +3798,13 @@
         <v>0</v>
       </c>
       <c r="AD7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG7" t="n">
         <v>0</v>
@@ -3838,19 +3825,19 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR7" t="n">
         <v>0</v>
@@ -3871,13 +3858,16 @@
         <v>0</v>
       </c>
       <c r="AX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -3886,20 +3876,20 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AX8), 0)</f>
+        <f>ROUND(AVERAGE(D8:AY8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>6</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K8" s="6" t="n">
         <v>6</v>
@@ -3908,31 +3898,31 @@
         <v>6</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N8" s="13" t="n">
         <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="P8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V8" t="n">
         <v>6</v>
@@ -3941,64 +3931,64 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="n">
         <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB8" t="n">
         <v>6</v>
       </c>
       <c r="AC8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG8" t="n">
         <v>0</v>
       </c>
       <c r="AH8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AI8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AJ8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AK8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AL8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AM8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR8" t="n">
         <v>0</v>
@@ -4016,144 +4006,189 @@
         <v>0</v>
       </c>
       <c r="AW8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AX8" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AX9), 0)</f>
-        <v/>
-      </c>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="n"/>
-      <c r="N9" s="13" t="n"/>
-      <c r="O9" s="19" t="n"/>
-      <c r="P9" s="19" t="n"/>
-      <c r="Q9" s="19" t="n"/>
-      <c r="R9" s="19" t="n"/>
-      <c r="S9" s="19" t="n"/>
-      <c r="T9" s="19" t="n"/>
+        <f>ROUND(AVERAGE(D9:AY9), 0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N9" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" t="n">
+        <v>6</v>
+      </c>
+      <c r="P9" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>5</v>
+      </c>
+      <c r="R9" t="n">
+        <v>6</v>
+      </c>
+      <c r="S9" t="n">
+        <v>6</v>
+      </c>
+      <c r="T9" t="n">
+        <v>6</v>
+      </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE9" t="n">
         <v>6</v>
       </c>
       <c r="AF9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AI9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AP9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AQ9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AR9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
       </c>
       <c r="AX9" t="n">
         <v>0</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AX10), 0)</f>
-        <v/>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>0</v>
+        <f>ROUND(AVERAGE(D10:AY10), 0)</f>
+        <v/>
       </c>
       <c r="H10" s="5" t="n">
         <v>6</v>
@@ -4162,7 +4197,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>6</v>
@@ -4189,7 +4224,7 @@
         <v>6</v>
       </c>
       <c r="S10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T10" t="n">
         <v>6</v>
@@ -4201,22 +4236,22 @@
         <v>6</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA10" t="n">
         <v>6</v>
       </c>
       <c r="AB10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC10" t="n">
         <v>6</v>
@@ -4225,25 +4260,25 @@
         <v>6</v>
       </c>
       <c r="AE10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL10" t="n">
         <v>6</v>
@@ -4264,31 +4299,34 @@
         <v>6</v>
       </c>
       <c r="AR10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -4297,7 +4335,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AX11), 0)</f>
+        <f>ROUND(AVERAGE(D11:AY11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4310,7 +4348,7 @@
         <v>6</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>6</v>
@@ -4340,7 +4378,7 @@
         <v>6</v>
       </c>
       <c r="Q11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R11" t="n">
         <v>6</v>
@@ -4355,19 +4393,19 @@
         <v>6</v>
       </c>
       <c r="V11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
         <v>6</v>
@@ -4391,10 +4429,10 @@
         <v>6</v>
       </c>
       <c r="AH11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ11" t="n">
         <v>6</v>
@@ -4412,19 +4450,19 @@
         <v>0</v>
       </c>
       <c r="AO11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ11" t="n">
         <v>6</v>
       </c>
       <c r="AR11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT11" t="n">
         <v>6</v>
@@ -4439,44 +4477,34 @@
         <v>0</v>
       </c>
       <c r="AX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AX12), 0)</f>
-        <v/>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L12" s="6" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D12:AY12), 0)</f>
+        <v/>
+      </c>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
       <c r="M12" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N12" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
         <v>6</v>
@@ -4497,7 +4525,7 @@
         <v>6</v>
       </c>
       <c r="U12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V12" t="n">
         <v>6</v>
@@ -4512,58 +4540,58 @@
         <v>6</v>
       </c>
       <c r="Z12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC12" t="n">
         <v>6</v>
       </c>
       <c r="AD12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AI12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL12" t="n">
         <v>6</v>
       </c>
       <c r="AM12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR12" t="n">
         <v>6</v>
@@ -4584,68 +4612,35 @@
         <v>0</v>
       </c>
       <c r="AX12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AX13), 0)</f>
-        <v/>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N13" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="O13" t="n">
-        <v>6</v>
-      </c>
-      <c r="P13" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D13:AY13), 0)</f>
+        <v/>
+      </c>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="19" t="n"/>
+      <c r="P13" s="19" t="n"/>
+      <c r="Q13" s="19" t="n"/>
       <c r="R13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>6</v>
@@ -4657,19 +4652,19 @@
         <v>6</v>
       </c>
       <c r="V13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA13" t="n">
         <v>6</v>
@@ -4684,7 +4679,7 @@
         <v>6</v>
       </c>
       <c r="AE13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AF13" t="n">
         <v>6</v>
@@ -4708,25 +4703,25 @@
         <v>6</v>
       </c>
       <c r="AM13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AN13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ13" t="n">
         <v>6</v>
       </c>
       <c r="AR13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT13" t="n">
         <v>6</v>
@@ -4741,130 +4736,149 @@
         <v>0</v>
       </c>
       <c r="AX13" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AX14), 0)</f>
-        <v/>
-      </c>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
+        <f>ROUND(AVERAGE(D14:AY14), 0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="M14" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="N14" s="13" t="n">
+      <c r="N14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O14" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>6</v>
+      </c>
+      <c r="R14" t="n">
+        <v>6</v>
+      </c>
+      <c r="S14" t="n">
+        <v>6</v>
+      </c>
+      <c r="T14" t="n">
+        <v>6</v>
+      </c>
+      <c r="U14" t="n">
+        <v>6</v>
+      </c>
+      <c r="V14" t="n">
+        <v>6</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM14" t="n">
         <v>1</v>
       </c>
-      <c r="O14" t="n">
-        <v>6</v>
-      </c>
-      <c r="P14" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>6</v>
-      </c>
-      <c r="R14" t="n">
-        <v>6</v>
-      </c>
-      <c r="S14" t="n">
-        <v>6</v>
-      </c>
-      <c r="T14" t="n">
-        <v>6</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="n">
-        <v>6</v>
-      </c>
-      <c r="W14" t="n">
-        <v>6</v>
-      </c>
-      <c r="X14" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>0</v>
-      </c>
       <c r="AN14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AS14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AT14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AV14" t="n">
         <v>6</v>
@@ -4874,31 +4888,70 @@
       </c>
       <c r="AX14" t="n">
         <v>0</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AX15), 0)</f>
-        <v/>
-      </c>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
-      <c r="N15" s="6" t="n"/>
-      <c r="O15" s="19" t="n"/>
-      <c r="P15" s="19" t="n"/>
-      <c r="Q15" s="19" t="n"/>
+        <f>ROUND(AVERAGE(D15:AY15), 0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>6</v>
+      </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S15" t="n">
         <v>6</v>
@@ -4907,16 +4960,16 @@
         <v>6</v>
       </c>
       <c r="U15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W15" t="n">
         <v>6</v>
       </c>
       <c r="X15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y15" t="n">
         <v>6</v>
@@ -4937,7 +4990,7 @@
         <v>6</v>
       </c>
       <c r="AE15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AF15" t="n">
         <v>6</v>
@@ -4946,10 +4999,10 @@
         <v>6</v>
       </c>
       <c r="AH15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AI15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ15" t="n">
         <v>6</v>
@@ -4961,10 +5014,10 @@
         <v>6</v>
       </c>
       <c r="AM15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AN15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AO15" t="n">
         <v>6</v>
@@ -4976,10 +5029,10 @@
         <v>6</v>
       </c>
       <c r="AR15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
         <v>6</v>
@@ -4994,13 +5047,16 @@
         <v>0</v>
       </c>
       <c r="AX15" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -5009,11 +5065,20 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AX16), 0)</f>
-        <v/>
+        <f>ROUND(AVERAGE(D16:AY16), 0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H16" s="5" t="n">
         <v>6</v>
@@ -5036,44 +5101,44 @@
       <c r="N16" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="O16" t="n">
-        <v>6</v>
-      </c>
-      <c r="P16" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>6</v>
-      </c>
-      <c r="R16" t="n">
+      <c r="O16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R16" s="20" t="n">
         <v>6</v>
       </c>
       <c r="S16" t="n">
         <v>6</v>
       </c>
       <c r="T16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V16" t="n">
         <v>6</v>
       </c>
       <c r="W16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AB16" t="n">
         <v>6</v>
@@ -5082,31 +5147,31 @@
         <v>6</v>
       </c>
       <c r="AD16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG16" t="n">
         <v>6</v>
       </c>
       <c r="AH16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AI16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM16" t="n">
         <v>1</v>
@@ -5115,25 +5180,25 @@
         <v>1</v>
       </c>
       <c r="AO16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AP16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AQ16" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AR16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AU16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AV16" t="n">
         <v>6</v>
@@ -5143,12 +5208,15 @@
       </c>
       <c r="AX16" t="n">
         <v>0</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -5157,80 +5225,80 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AX17), 0)</f>
+        <f>ROUND(AVERAGE(D17:AY17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>6</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="I17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="K17" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="n">
-        <v>6</v>
-      </c>
-      <c r="P17" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>6</v>
-      </c>
-      <c r="R17" t="n">
-        <v>6</v>
-      </c>
-      <c r="S17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S17" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T17" t="n">
         <v>6</v>
       </c>
       <c r="U17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V17" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB17" t="n">
         <v>6</v>
@@ -5239,10 +5307,10 @@
         <v>6</v>
       </c>
       <c r="AD17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF17" t="n">
         <v>6</v>
@@ -5251,25 +5319,25 @@
         <v>6</v>
       </c>
       <c r="AH17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO17" t="n">
         <v>6</v>
@@ -5287,10 +5355,10 @@
         <v>0</v>
       </c>
       <c r="AT17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AU17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AV17" t="n">
         <v>6</v>
@@ -5299,13 +5367,16 @@
         <v>0</v>
       </c>
       <c r="AX17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -5314,21 +5385,10 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AX18), 0)</f>
-        <v/>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J18" s="6" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D18:AY18), 0)</f>
+        <v/>
+      </c>
+      <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n">
         <v>6</v>
       </c>
@@ -5350,41 +5410,41 @@
       <c r="Q18" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="R18" t="n">
-        <v>6</v>
-      </c>
-      <c r="S18" t="n">
-        <v>6</v>
-      </c>
-      <c r="T18" t="n">
+      <c r="R18" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S18" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T18" s="20" t="n">
         <v>6</v>
       </c>
       <c r="U18" t="n">
         <v>6</v>
       </c>
       <c r="V18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB18" t="n">
         <v>6</v>
       </c>
       <c r="AC18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD18" t="n">
         <v>6</v>
@@ -5396,7 +5456,7 @@
         <v>6</v>
       </c>
       <c r="AG18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH18" t="n">
         <v>0</v>
@@ -5426,7 +5486,7 @@
         <v>0</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR18" t="n">
         <v>0</v>
@@ -5447,23 +5507,41 @@
         <v>0</v>
       </c>
       <c r="AX18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AX19), 0)</f>
-        <v/>
+        <f>ROUND(AVERAGE(D19:AY19), 0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>6</v>
@@ -5478,7 +5556,7 @@
         <v>6</v>
       </c>
       <c r="P19" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="20" t="n">
         <v>6</v>
@@ -5486,29 +5564,29 @@
       <c r="R19" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S19" t="n">
-        <v>6</v>
-      </c>
-      <c r="T19" t="n">
-        <v>6</v>
-      </c>
-      <c r="U19" t="n">
+      <c r="S19" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T19" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U19" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AA19" t="n">
         <v>0</v>
@@ -5517,34 +5595,34 @@
         <v>6</v>
       </c>
       <c r="AC19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG19" t="n">
         <v>0</v>
       </c>
       <c r="AH19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AM19" t="n">
         <v>0</v>
@@ -5562,131 +5640,87 @@
         <v>0</v>
       </c>
       <c r="AR19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
       </c>
       <c r="AX19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AX20), 0)</f>
-        <v/>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J20" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L20" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N20" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O20" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P20" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q20" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R20" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T20" t="n">
-        <v>4</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D20:AY20), 0)</f>
+        <v/>
+      </c>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+      <c r="N20" s="6" t="n"/>
+      <c r="O20" s="20" t="n"/>
+      <c r="P20" s="20" t="n"/>
+      <c r="Q20" s="20" t="n"/>
+      <c r="R20" s="20" t="n"/>
+      <c r="S20" s="20" t="n"/>
+      <c r="T20" s="20" t="n"/>
+      <c r="U20" s="20" t="n"/>
       <c r="W20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="X20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD20" t="n">
         <v>5</v>
       </c>
-      <c r="Y20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>4</v>
-      </c>
-      <c r="AB20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD20" t="n">
-        <v>0</v>
-      </c>
       <c r="AE20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH20" t="n">
         <v>0</v>
@@ -5701,274 +5735,191 @@
         <v>0</v>
       </c>
       <c r="AL20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AN20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AO20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AP20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AQ20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AR20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AS20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AT20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AU20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AV20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
       </c>
       <c r="AX20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AX21), 0)</f>
-        <v/>
-      </c>
-      <c r="D21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J21" s="6" t="n">
+        <f>ROUND(AVERAGE(D21:AY21), 0)</f>
+        <v/>
+      </c>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+      <c r="N21" s="6" t="n"/>
+      <c r="O21" s="20" t="n"/>
+      <c r="P21" s="20" t="n"/>
+      <c r="Q21" s="20" t="n"/>
+      <c r="R21" s="20" t="n"/>
+      <c r="S21" s="20" t="n"/>
+      <c r="T21" s="20" t="n"/>
+      <c r="U21" s="20" t="n"/>
+      <c r="Y21" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO21" t="n">
         <v>5</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L21" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M21" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N21" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O21" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P21" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q21" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R21" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S21" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T21" t="n">
-        <v>6</v>
-      </c>
-      <c r="U21" t="n">
-        <v>6</v>
-      </c>
-      <c r="V21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W21" t="n">
-        <v>0</v>
-      </c>
-      <c r="X21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AH21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>6</v>
-      </c>
       <c r="AP21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ21" t="n">
         <v>6</v>
       </c>
       <c r="AR21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AS21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AT21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AU21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AV21" t="n">
         <v>6</v>
       </c>
       <c r="AW21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AX21" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="AY21" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AX22), 0)</f>
-        <v/>
-      </c>
-      <c r="J22" s="6" t="n"/>
-      <c r="K22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M22" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N22" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T22" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U22" t="n">
-        <v>6</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" t="n">
-        <v>5</v>
-      </c>
-      <c r="X22" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D22:AY22), 0)</f>
+        <v/>
+      </c>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+      <c r="N22" s="6" t="n"/>
+      <c r="O22" s="20" t="n"/>
+      <c r="P22" s="20" t="n"/>
+      <c r="Q22" s="20" t="n"/>
+      <c r="R22" s="20" t="n"/>
+      <c r="S22" s="20" t="n"/>
+      <c r="T22" s="20" t="n"/>
+      <c r="U22" s="20" t="n"/>
       <c r="Z22" t="n">
         <v>6</v>
       </c>
       <c r="AA22" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AB22" t="n">
         <v>6</v>
       </c>
       <c r="AC22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD22" t="n">
         <v>6</v>
@@ -5995,19 +5946,19 @@
         <v>0</v>
       </c>
       <c r="AL22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ22" t="n">
         <v>6</v>
@@ -6028,95 +5979,45 @@
         <v>0</v>
       </c>
       <c r="AW22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AX22" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AX23), 0)</f>
-        <v/>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M23" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N23" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P23" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U23" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V23" t="n">
-        <v>0</v>
-      </c>
-      <c r="W23" t="n">
-        <v>6</v>
-      </c>
-      <c r="X23" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>0</v>
-      </c>
+        <f>ROUND(AVERAGE(D23:AY23), 0)</f>
+        <v/>
+      </c>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+      <c r="N23" s="6" t="n"/>
+      <c r="O23" s="20" t="n"/>
+      <c r="P23" s="20" t="n"/>
+      <c r="Q23" s="20" t="n"/>
+      <c r="R23" s="20" t="n"/>
+      <c r="S23" s="20" t="n"/>
+      <c r="T23" s="20" t="n"/>
+      <c r="U23" s="20" t="n"/>
       <c r="AB23" t="n">
         <v>6</v>
       </c>
       <c r="AC23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD23" t="n">
         <v>6</v>
@@ -6128,7 +6029,7 @@
         <v>6</v>
       </c>
       <c r="AG23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH23" t="n">
         <v>5</v>
@@ -6143,58 +6044,61 @@
         <v>5</v>
       </c>
       <c r="AL23" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM23" t="n">
         <v>5</v>
       </c>
-      <c r="AM23" t="n">
-        <v>0</v>
-      </c>
       <c r="AN23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AO23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AP23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AR23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AU23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AV23" t="n">
         <v>6</v>
       </c>
       <c r="AW23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AX23" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AY23" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AX24), 0)</f>
+        <f>ROUND(AVERAGE(D24:AY24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6207,35 +6111,17 @@
       <c r="S24" s="20" t="n"/>
       <c r="T24" s="20" t="n"/>
       <c r="U24" s="20" t="n"/>
-      <c r="W24" t="n">
-        <v>6</v>
-      </c>
-      <c r="X24" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>0</v>
-      </c>
       <c r="AC24" t="n">
         <v>6</v>
       </c>
       <c r="AD24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG24" t="n">
         <v>0</v>
@@ -6253,58 +6139,61 @@
         <v>0</v>
       </c>
       <c r="AL24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AW24" t="n">
         <v>0</v>
       </c>
       <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AX25), 0)</f>
+        <f>ROUND(AVERAGE(D25:AY25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6317,98 +6206,86 @@
       <c r="S25" s="20" t="n"/>
       <c r="T25" s="20" t="n"/>
       <c r="U25" s="20" t="n"/>
-      <c r="Y25" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z25" t="n">
+      <c r="AD25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR25" t="n">
         <v>3</v>
       </c>
-      <c r="AA25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>4</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>4</v>
-      </c>
-      <c r="AO25" t="n">
-        <v>5</v>
-      </c>
-      <c r="AP25" t="n">
-        <v>5</v>
-      </c>
-      <c r="AQ25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR25" t="n">
-        <v>5</v>
-      </c>
       <c r="AS25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AT25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AU25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AV25" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AW25" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AX25" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AX26), 0)</f>
+        <f>ROUND(AVERAGE(D26:AY26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6421,21 +6298,6 @@
       <c r="S26" s="20" t="n"/>
       <c r="T26" s="20" t="n"/>
       <c r="U26" s="20" t="n"/>
-      <c r="Z26" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB26" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>6</v>
-      </c>
       <c r="AE26" t="n">
         <v>6</v>
       </c>
@@ -6443,7 +6305,7 @@
         <v>6</v>
       </c>
       <c r="AG26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH26" t="n">
         <v>0</v>
@@ -6452,28 +6314,28 @@
         <v>0</v>
       </c>
       <c r="AJ26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL26" t="n">
         <v>6</v>
       </c>
       <c r="AM26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR26" t="n">
         <v>0</v>
@@ -6491,25 +6353,28 @@
         <v>0</v>
       </c>
       <c r="AW26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AX26" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AX27), 0)</f>
+        <f>ROUND(AVERAGE(D27:AY27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6522,23 +6387,11 @@
       <c r="S27" s="20" t="n"/>
       <c r="T27" s="20" t="n"/>
       <c r="U27" s="20" t="n"/>
-      <c r="AA27" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>0</v>
-      </c>
       <c r="AE27" t="n">
         <v>0</v>
       </c>
       <c r="AF27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG27" t="n">
         <v>0</v>
@@ -6592,22 +6445,25 @@
         <v>0</v>
       </c>
       <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AX28), 0)</f>
+        <f>ROUND(AVERAGE(D28:AY28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6620,89 +6476,83 @@
       <c r="S28" s="20" t="n"/>
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
-      <c r="AB28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>6</v>
-      </c>
       <c r="AE28" t="n">
         <v>6</v>
       </c>
       <c r="AF28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AK28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AL28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN28" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AR28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU28" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV28" t="n">
         <v>6</v>
       </c>
       <c r="AW28" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX28" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AX29), 0)</f>
+        <f>ROUND(AVERAGE(D29:AY29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6715,65 +6565,8 @@
       <c r="S29" s="20" t="n"/>
       <c r="T29" s="20" t="n"/>
       <c r="U29" s="20" t="n"/>
-      <c r="AC29" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU29" t="n">
-        <v>0</v>
-      </c>
       <c r="AV29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW29" t="n">
         <v>0</v>
@@ -6781,472 +6574,7 @@
       <c r="AX29" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="28" t="inlineStr">
-        <is>
-          <t>zpercu</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>23/05/2026</t>
-        </is>
-      </c>
-      <c r="C30" s="28">
-        <f>ROUND(AVERAGE(D30:AX30), 0)</f>
-        <v/>
-      </c>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="20" t="n"/>
-      <c r="P30" s="20" t="n"/>
-      <c r="Q30" s="20" t="n"/>
-      <c r="R30" s="20" t="n"/>
-      <c r="S30" s="20" t="n"/>
-      <c r="T30" s="20" t="n"/>
-      <c r="U30" s="20" t="n"/>
-      <c r="AD30" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF30" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG30" t="n">
-        <v>6</v>
-      </c>
-      <c r="AH30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ30" t="n">
-        <v>4</v>
-      </c>
-      <c r="AR30" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS30" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT30" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU30" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV30" t="n">
-        <v>3</v>
-      </c>
-      <c r="AW30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX30" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="28" t="inlineStr">
-        <is>
-          <t>rasim01</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C31" s="28">
-        <f>ROUND(AVERAGE(D31:AX31), 0)</f>
-        <v/>
-      </c>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
-      <c r="N31" s="6" t="n"/>
-      <c r="O31" s="20" t="n"/>
-      <c r="P31" s="20" t="n"/>
-      <c r="Q31" s="20" t="n"/>
-      <c r="R31" s="20" t="n"/>
-      <c r="S31" s="20" t="n"/>
-      <c r="T31" s="20" t="n"/>
-      <c r="U31" s="20" t="n"/>
-      <c r="AE31" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX31" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="28" t="inlineStr">
-        <is>
-          <t>maragno</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>30/05/2026</t>
-        </is>
-      </c>
-      <c r="C32" s="28">
-        <f>ROUND(AVERAGE(D32:AX32), 0)</f>
-        <v/>
-      </c>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
-      <c r="N32" s="6" t="n"/>
-      <c r="O32" s="20" t="n"/>
-      <c r="P32" s="20" t="n"/>
-      <c r="Q32" s="20" t="n"/>
-      <c r="R32" s="20" t="n"/>
-      <c r="S32" s="20" t="n"/>
-      <c r="T32" s="20" t="n"/>
-      <c r="U32" s="20" t="n"/>
-      <c r="AE32" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ32" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK32" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL32" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW32" t="n">
-        <v>6</v>
-      </c>
-      <c r="AX32" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="28" t="inlineStr">
-        <is>
-          <t>Akemi</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>31/05/2026</t>
-        </is>
-      </c>
-      <c r="C33" s="28">
-        <f>ROUND(AVERAGE(D33:AX33), 0)</f>
-        <v/>
-      </c>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
-      <c r="N33" s="6" t="n"/>
-      <c r="O33" s="20" t="n"/>
-      <c r="P33" s="20" t="n"/>
-      <c r="Q33" s="20" t="n"/>
-      <c r="R33" s="20" t="n"/>
-      <c r="S33" s="20" t="n"/>
-      <c r="T33" s="20" t="n"/>
-      <c r="U33" s="20" t="n"/>
-      <c r="AE33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="28" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
-      <c r="C34" s="28">
-        <f>ROUND(AVERAGE(D34:AX34), 0)</f>
-        <v/>
-      </c>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
-      <c r="N34" s="6" t="n"/>
-      <c r="O34" s="20" t="n"/>
-      <c r="P34" s="20" t="n"/>
-      <c r="Q34" s="20" t="n"/>
-      <c r="R34" s="20" t="n"/>
-      <c r="S34" s="20" t="n"/>
-      <c r="T34" s="20" t="n"/>
-      <c r="U34" s="20" t="n"/>
-      <c r="AE34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AV34" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="28" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C35" s="28">
-        <f>ROUND(AVERAGE(D35:AX35), 0)</f>
-        <v/>
-      </c>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
-      <c r="N35" s="6" t="n"/>
-      <c r="O35" s="20" t="n"/>
-      <c r="P35" s="20" t="n"/>
-      <c r="Q35" s="20" t="n"/>
-      <c r="R35" s="20" t="n"/>
-      <c r="S35" s="20" t="n"/>
-      <c r="T35" s="20" t="n"/>
-      <c r="U35" s="20" t="n"/>
-      <c r="AV35" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX35" t="n">
+      <c r="AY29" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-13
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ29"/>
+  <dimension ref="A1:BA29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3033,6 +3033,11 @@
           <t>10/07/2026</t>
         </is>
       </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3046,7 +3051,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:AZ2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BA2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3173,6 +3178,9 @@
         <v>0</v>
       </c>
       <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3188,7 +3196,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:AZ3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BA3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3306,6 +3314,9 @@
       <c r="AZ3" t="n">
         <v>6</v>
       </c>
+      <c r="BA3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3319,7 +3330,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:AZ4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BA4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3468,6 +3479,9 @@
       </c>
       <c r="AZ4" t="n">
         <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -3482,7 +3496,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:AZ5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BA5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3632,6 +3646,9 @@
       <c r="AZ5" t="n">
         <v>0</v>
       </c>
+      <c r="BA5" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3645,7 +3662,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:AZ6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BA6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3765,6 +3782,9 @@
       <c r="AZ6" t="n">
         <v>0</v>
       </c>
+      <c r="BA6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3778,7 +3798,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:AZ7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BA7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3886,6 +3906,9 @@
       <c r="AZ7" t="n">
         <v>0</v>
       </c>
+      <c r="BA7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3899,7 +3922,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:AZ8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BA8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4040,6 +4063,9 @@
       <c r="AZ8" t="n">
         <v>6</v>
       </c>
+      <c r="BA8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4053,7 +4079,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:AZ9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BA9), 0)</f>
         <v/>
       </c>
       <c r="D9" s="10" t="n">
@@ -4203,6 +4229,9 @@
       <c r="AZ9" t="n">
         <v>6</v>
       </c>
+      <c r="BA9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4216,7 +4245,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:AZ10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BA10), 0)</f>
         <v/>
       </c>
       <c r="H10" s="5" t="n">
@@ -4352,6 +4381,9 @@
         <v>6</v>
       </c>
       <c r="AZ10" t="n">
+        <v>6</v>
+      </c>
+      <c r="BA10" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4367,7 +4399,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:AZ11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BA11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4516,6 +4548,9 @@
       </c>
       <c r="AZ11" t="n">
         <v>0</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -4530,7 +4565,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:AZ12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BA12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4655,6 +4690,9 @@
       <c r="AZ12" t="n">
         <v>0</v>
       </c>
+      <c r="BA12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4668,7 +4706,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:AZ13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BA13), 0)</f>
         <v/>
       </c>
       <c r="K13" s="6" t="n"/>
@@ -4782,6 +4820,9 @@
       <c r="AZ13" t="n">
         <v>6</v>
       </c>
+      <c r="BA13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4795,7 +4836,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:AZ14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BA14), 0)</f>
         <v/>
       </c>
       <c r="G14" s="5" t="n">
@@ -4936,6 +4977,9 @@
       <c r="AZ14" t="n">
         <v>6</v>
       </c>
+      <c r="BA14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4949,7 +4993,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:AZ15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BA15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5099,6 +5143,9 @@
       <c r="AZ15" t="n">
         <v>0</v>
       </c>
+      <c r="BA15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5112,7 +5159,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:AZ16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BA16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5262,6 +5309,9 @@
       <c r="AZ16" t="n">
         <v>4</v>
       </c>
+      <c r="BA16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5275,7 +5325,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:AZ17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BA17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5425,6 +5475,9 @@
       <c r="AZ17" t="n">
         <v>0</v>
       </c>
+      <c r="BA17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5438,7 +5491,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:AZ18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BA18), 0)</f>
         <v/>
       </c>
       <c r="J18" s="6" t="n"/>
@@ -5568,6 +5621,9 @@
       <c r="AZ18" t="n">
         <v>0</v>
       </c>
+      <c r="BA18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5581,7 +5637,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:AZ19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BA19), 0)</f>
         <v/>
       </c>
       <c r="G19" s="5" t="n">
@@ -5722,6 +5778,9 @@
       <c r="AZ19" t="n">
         <v>0</v>
       </c>
+      <c r="BA19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5735,7 +5794,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:AZ20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BA20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -5838,6 +5897,9 @@
       <c r="AZ20" t="n">
         <v>0</v>
       </c>
+      <c r="BA20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5851,7 +5913,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:AZ21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BA21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -5948,6 +6010,9 @@
       <c r="AZ21" t="n">
         <v>5</v>
       </c>
+      <c r="BA21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5961,7 +6026,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:AZ22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BA22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6055,6 +6120,9 @@
       <c r="AZ22" t="n">
         <v>3</v>
       </c>
+      <c r="BA22" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6068,7 +6136,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:AZ23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BA23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6156,6 +6224,9 @@
       <c r="AZ23" t="n">
         <v>6</v>
       </c>
+      <c r="BA23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6169,7 +6240,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:AZ24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BA24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6254,6 +6325,9 @@
       <c r="AZ24" t="n">
         <v>0</v>
       </c>
+      <c r="BA24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6267,7 +6341,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:AZ25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BA25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6349,6 +6423,9 @@
       <c r="AZ25" t="n">
         <v>0</v>
       </c>
+      <c r="BA25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6362,7 +6439,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:AZ26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BA26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6441,6 +6518,9 @@
       <c r="AZ26" t="n">
         <v>6</v>
       </c>
+      <c r="BA26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6454,7 +6534,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:AZ27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BA27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6533,6 +6613,9 @@
       <c r="AZ27" t="n">
         <v>0</v>
       </c>
+      <c r="BA27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -6546,7 +6629,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:AZ28), 0)</f>
+        <f>ROUND(AVERAGE(D28:BA28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6625,6 +6708,9 @@
       <c r="AZ28" t="n">
         <v>0</v>
       </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -6638,7 +6724,7 @@
         </is>
       </c>
       <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:AZ29), 0)</f>
+        <f>ROUND(AVERAGE(D29:BA29), 0)</f>
         <v/>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -6665,6 +6751,9 @@
       </c>
       <c r="AZ29" t="n">
         <v>0</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-18
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA29"/>
+  <dimension ref="A1:BB28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3038,6 +3038,11 @@
           <t>10/07/2026</t>
         </is>
       </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3051,7 +3056,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BA2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BB2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3181,6 +3186,9 @@
         <v>0</v>
       </c>
       <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3196,7 +3204,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BA3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BB3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3317,6 +3325,9 @@
       <c r="BA3" t="n">
         <v>6</v>
       </c>
+      <c r="BB3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3330,7 +3341,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BA4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BB4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3482,6 +3493,9 @@
       </c>
       <c r="BA4" t="n">
         <v>6</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3496,7 +3510,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BA5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BB5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3649,6 +3663,9 @@
       <c r="BA5" t="n">
         <v>6</v>
       </c>
+      <c r="BB5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3662,7 +3679,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BA6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BB6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3785,6 +3802,9 @@
       <c r="BA6" t="n">
         <v>0</v>
       </c>
+      <c r="BB6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3798,7 +3818,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BA7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BB7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3909,6 +3929,9 @@
       <c r="BA7" t="n">
         <v>0</v>
       </c>
+      <c r="BB7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3922,7 +3945,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BA8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BB8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4066,6 +4089,9 @@
       <c r="BA8" t="n">
         <v>6</v>
       </c>
+      <c r="BB8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4079,7 +4105,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BA9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BB9), 0)</f>
         <v/>
       </c>
       <c r="D9" s="10" t="n">
@@ -4232,6 +4258,9 @@
       <c r="BA9" t="n">
         <v>6</v>
       </c>
+      <c r="BB9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4245,7 +4274,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BA10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BB10), 0)</f>
         <v/>
       </c>
       <c r="H10" s="5" t="n">
@@ -4385,6 +4414,9 @@
       </c>
       <c r="BA10" t="n">
         <v>6</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4399,7 +4431,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BA11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BB11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4551,6 +4583,9 @@
       </c>
       <c r="BA11" t="n">
         <v>6</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -4565,7 +4600,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BA12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BB12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4693,6 +4728,9 @@
       <c r="BA12" t="n">
         <v>0</v>
       </c>
+      <c r="BB12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4706,7 +4744,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BA13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BB13), 0)</f>
         <v/>
       </c>
       <c r="K13" s="6" t="n"/>
@@ -4823,6 +4861,9 @@
       <c r="BA13" t="n">
         <v>6</v>
       </c>
+      <c r="BB13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4836,7 +4877,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BA14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BB14), 0)</f>
         <v/>
       </c>
       <c r="G14" s="5" t="n">
@@ -4980,6 +5021,9 @@
       <c r="BA14" t="n">
         <v>6</v>
       </c>
+      <c r="BB14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4993,7 +5037,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BA15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BB15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5146,6 +5190,9 @@
       <c r="BA15" t="n">
         <v>6</v>
       </c>
+      <c r="BB15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5159,7 +5206,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BA16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BB16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5312,6 +5359,9 @@
       <c r="BA16" t="n">
         <v>6</v>
       </c>
+      <c r="BB16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5325,7 +5375,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BA17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BB17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5478,6 +5528,9 @@
       <c r="BA17" t="n">
         <v>6</v>
       </c>
+      <c r="BB17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5491,7 +5544,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BA18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BB18), 0)</f>
         <v/>
       </c>
       <c r="J18" s="6" t="n"/>
@@ -5624,6 +5677,9 @@
       <c r="BA18" t="n">
         <v>0</v>
       </c>
+      <c r="BB18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5637,7 +5693,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BA19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BB19), 0)</f>
         <v/>
       </c>
       <c r="G19" s="5" t="n">
@@ -5781,6 +5837,9 @@
       <c r="BA19" t="n">
         <v>0</v>
       </c>
+      <c r="BB19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5794,7 +5853,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BA20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BB20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -5900,6 +5959,9 @@
       <c r="BA20" t="n">
         <v>0</v>
       </c>
+      <c r="BB20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5913,7 +5975,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BA21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BB21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6013,6 +6075,9 @@
       <c r="BA21" t="n">
         <v>6</v>
       </c>
+      <c r="BB21" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6026,7 +6091,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BA22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BB22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6123,6 +6188,9 @@
       <c r="BA22" t="n">
         <v>3</v>
       </c>
+      <c r="BB22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6136,7 +6204,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BA23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BB23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6227,20 +6295,23 @@
       <c r="BA23" t="n">
         <v>6</v>
       </c>
+      <c r="BB23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BA24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BB24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6253,20 +6324,17 @@
       <c r="S24" s="20" t="n"/>
       <c r="T24" s="20" t="n"/>
       <c r="U24" s="20" t="n"/>
-      <c r="AC24" t="n">
-        <v>6</v>
-      </c>
       <c r="AD24" t="n">
         <v>6</v>
       </c>
       <c r="AE24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH24" t="n">
         <v>0</v>
@@ -6296,22 +6364,22 @@
         <v>0</v>
       </c>
       <c r="AQ24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW24" t="n">
         <v>0</v>
@@ -6326,22 +6394,25 @@
         <v>0</v>
       </c>
       <c r="BA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BA25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BB25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6354,17 +6425,14 @@
       <c r="S25" s="20" t="n"/>
       <c r="T25" s="20" t="n"/>
       <c r="U25" s="20" t="n"/>
-      <c r="AD25" t="n">
-        <v>6</v>
-      </c>
       <c r="AE25" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AF25" t="n">
         <v>6</v>
       </c>
       <c r="AG25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH25" t="n">
         <v>0</v>
@@ -6373,13 +6441,13 @@
         <v>0</v>
       </c>
       <c r="AJ25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM25" t="n">
         <v>0</v>
@@ -6394,52 +6462,55 @@
         <v>0</v>
       </c>
       <c r="AQ25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AR25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AW25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AX25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AY25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AZ25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BA25" t="n">
+        <v>6</v>
+      </c>
+      <c r="BB25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BA26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BB26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6453,7 +6524,7 @@
       <c r="T26" s="20" t="n"/>
       <c r="U26" s="20" t="n"/>
       <c r="AE26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF26" t="n">
         <v>6</v>
@@ -6468,13 +6539,13 @@
         <v>0</v>
       </c>
       <c r="AJ26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM26" t="n">
         <v>0</v>
@@ -6507,34 +6578,37 @@
         <v>0</v>
       </c>
       <c r="AW26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ26" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA26" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BA27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BB27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6548,10 +6622,10 @@
       <c r="T27" s="20" t="n"/>
       <c r="U27" s="20" t="n"/>
       <c r="AE27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG27" t="n">
         <v>0</v>
@@ -6578,28 +6652,28 @@
         <v>0</v>
       </c>
       <c r="AO27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV27" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW27" t="n">
         <v>0</v>
@@ -6614,22 +6688,25 @@
         <v>0</v>
       </c>
       <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:BA28), 0)</f>
+        <f>ROUND(AVERAGE(D28:BB28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6642,57 +6719,6 @@
       <c r="S28" s="20" t="n"/>
       <c r="T28" s="20" t="n"/>
       <c r="U28" s="20" t="n"/>
-      <c r="AE28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU28" t="n">
-        <v>6</v>
-      </c>
       <c r="AV28" t="n">
         <v>6</v>
       </c>
@@ -6709,51 +6735,10 @@
         <v>0</v>
       </c>
       <c r="BA28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="28" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C29" s="28">
-        <f>ROUND(AVERAGE(D29:BA29), 0)</f>
-        <v/>
-      </c>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-      <c r="N29" s="6" t="n"/>
-      <c r="O29" s="20" t="n"/>
-      <c r="P29" s="20" t="n"/>
-      <c r="Q29" s="20" t="n"/>
-      <c r="R29" s="20" t="n"/>
-      <c r="S29" s="20" t="n"/>
-      <c r="T29" s="20" t="n"/>
-      <c r="U29" s="20" t="n"/>
-      <c r="AV29" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ29" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA29" t="n">
-        <v>6</v>
+        <v>6</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-19
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC28"/>
+  <dimension ref="A1:BD28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3048,6 +3048,11 @@
           <t>17/07/2026</t>
         </is>
       </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3061,7 +3066,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BC2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BD2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3197,6 +3202,9 @@
         <v>0</v>
       </c>
       <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3212,7 +3220,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BC3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BD3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3339,6 +3347,9 @@
       <c r="BC3" t="n">
         <v>6</v>
       </c>
+      <c r="BD3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3352,7 +3363,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BC4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BD4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3509,6 +3520,9 @@
         <v>0</v>
       </c>
       <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3524,7 +3538,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BC5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BD5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3683,6 +3697,9 @@
       <c r="BC5" t="n">
         <v>0</v>
       </c>
+      <c r="BD5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3696,7 +3713,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BC6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BD6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3825,6 +3842,9 @@
       <c r="BC6" t="n">
         <v>0</v>
       </c>
+      <c r="BD6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3838,7 +3858,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BC7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BD7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3955,6 +3975,9 @@
       <c r="BC7" t="n">
         <v>0</v>
       </c>
+      <c r="BD7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3968,7 +3991,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BC8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BD8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4118,6 +4141,9 @@
       <c r="BC8" t="n">
         <v>0</v>
       </c>
+      <c r="BD8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4131,7 +4157,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BC9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BD9), 0)</f>
         <v/>
       </c>
       <c r="D9" s="10" t="n">
@@ -4290,6 +4316,9 @@
       <c r="BC9" t="n">
         <v>0</v>
       </c>
+      <c r="BD9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4303,7 +4332,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BC10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BD10), 0)</f>
         <v/>
       </c>
       <c r="H10" s="5" t="n">
@@ -4448,6 +4477,9 @@
         <v>0</v>
       </c>
       <c r="BC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4463,7 +4495,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BC11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BD11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4620,6 +4652,9 @@
         <v>0</v>
       </c>
       <c r="BC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4635,7 +4670,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BC12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BD12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4769,6 +4804,9 @@
       <c r="BC12" t="n">
         <v>0</v>
       </c>
+      <c r="BD12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4782,7 +4820,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BC13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BD13), 0)</f>
         <v/>
       </c>
       <c r="K13" s="6" t="n"/>
@@ -4905,6 +4943,9 @@
       <c r="BC13" t="n">
         <v>0</v>
       </c>
+      <c r="BD13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4918,7 +4959,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BC14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BD14), 0)</f>
         <v/>
       </c>
       <c r="G14" s="5" t="n">
@@ -5068,6 +5109,9 @@
       <c r="BC14" t="n">
         <v>0</v>
       </c>
+      <c r="BD14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5081,7 +5125,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BC15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BD15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5240,6 +5284,9 @@
       <c r="BC15" t="n">
         <v>0</v>
       </c>
+      <c r="BD15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5253,7 +5300,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BC16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BD16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5412,6 +5459,9 @@
       <c r="BC16" t="n">
         <v>1</v>
       </c>
+      <c r="BD16" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5425,7 +5475,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BC17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BD17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5584,6 +5634,9 @@
       <c r="BC17" t="n">
         <v>0</v>
       </c>
+      <c r="BD17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5597,7 +5650,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BC18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BD18), 0)</f>
         <v/>
       </c>
       <c r="J18" s="6" t="n"/>
@@ -5736,6 +5789,9 @@
       <c r="BC18" t="n">
         <v>0</v>
       </c>
+      <c r="BD18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5749,7 +5805,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BC19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BD19), 0)</f>
         <v/>
       </c>
       <c r="G19" s="5" t="n">
@@ -5899,6 +5955,9 @@
       <c r="BC19" t="n">
         <v>0</v>
       </c>
+      <c r="BD19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5912,7 +5971,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BC20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BD20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6024,6 +6083,9 @@
       <c r="BC20" t="n">
         <v>0</v>
       </c>
+      <c r="BD20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6037,7 +6099,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BC21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BD21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6143,6 +6205,9 @@
       <c r="BC21" t="n">
         <v>3</v>
       </c>
+      <c r="BD21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6156,7 +6221,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BC22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BD22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6259,6 +6324,9 @@
       <c r="BC22" t="n">
         <v>6</v>
       </c>
+      <c r="BD22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6272,7 +6340,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BC23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BD23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6369,6 +6437,9 @@
       <c r="BC23" t="n">
         <v>0</v>
       </c>
+      <c r="BD23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6382,7 +6453,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BC24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BD24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6473,6 +6544,9 @@
       <c r="BC24" t="n">
         <v>0</v>
       </c>
+      <c r="BD24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6486,7 +6560,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BC25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BD25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6574,6 +6648,9 @@
       <c r="BC25" t="n">
         <v>0</v>
       </c>
+      <c r="BD25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6587,7 +6664,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BC26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BD26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6675,6 +6752,9 @@
       <c r="BC26" t="n">
         <v>0</v>
       </c>
+      <c r="BD26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6688,7 +6768,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BC27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BD27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6776,6 +6856,9 @@
       <c r="BC27" t="n">
         <v>0</v>
       </c>
+      <c r="BD27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -6789,7 +6872,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:BC28), 0)</f>
+        <f>ROUND(AVERAGE(D28:BD28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6825,6 +6908,9 @@
       </c>
       <c r="BC28" t="n">
         <v>0</v>
+      </c>
+      <c r="BD28" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-20
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2756,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE28"/>
+  <dimension ref="A1:BF28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3058,6 +3058,11 @@
           <t>17/07/2026</t>
         </is>
       </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -3071,7 +3076,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BE2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BF2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -3213,6 +3218,9 @@
         <v>0</v>
       </c>
       <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3228,7 +3236,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BE3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BF3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3361,6 +3369,9 @@
       <c r="BE3" t="n">
         <v>6</v>
       </c>
+      <c r="BF3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3374,7 +3385,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BE4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BF4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3538,6 +3549,9 @@
       </c>
       <c r="BE4" t="n">
         <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -3552,7 +3566,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BE5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BF5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3717,6 +3731,9 @@
       <c r="BE5" t="n">
         <v>0</v>
       </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3730,7 +3747,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BE6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BF6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3865,6 +3882,9 @@
       <c r="BE6" t="n">
         <v>0</v>
       </c>
+      <c r="BF6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3878,7 +3898,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BE7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BF7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -4001,6 +4021,9 @@
       <c r="BE7" t="n">
         <v>0</v>
       </c>
+      <c r="BF7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4014,7 +4037,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BE8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BF8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4170,6 +4193,9 @@
       <c r="BE8" t="n">
         <v>0</v>
       </c>
+      <c r="BF8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4183,7 +4209,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BE9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BF9), 0)</f>
         <v/>
       </c>
       <c r="D9" s="10" t="n">
@@ -4348,6 +4374,9 @@
       <c r="BE9" t="n">
         <v>0</v>
       </c>
+      <c r="BF9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4361,7 +4390,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BE10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BF10), 0)</f>
         <v/>
       </c>
       <c r="H10" s="5" t="n">
@@ -4513,6 +4542,9 @@
       </c>
       <c r="BE10" t="n">
         <v>0</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4527,7 +4559,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BE11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BF11), 0)</f>
         <v/>
       </c>
       <c r="D11" s="10" t="n">
@@ -4691,6 +4723,9 @@
       </c>
       <c r="BE11" t="n">
         <v>0</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -4705,7 +4740,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BE12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BF12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4845,6 +4880,9 @@
       <c r="BE12" t="n">
         <v>0</v>
       </c>
+      <c r="BF12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4858,7 +4896,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BE13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BF13), 0)</f>
         <v/>
       </c>
       <c r="K13" s="6" t="n"/>
@@ -4987,6 +5025,9 @@
       <c r="BE13" t="n">
         <v>6</v>
       </c>
+      <c r="BF13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5000,7 +5041,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BE14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BF14), 0)</f>
         <v/>
       </c>
       <c r="G14" s="5" t="n">
@@ -5156,6 +5197,9 @@
       <c r="BE14" t="n">
         <v>0</v>
       </c>
+      <c r="BF14" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5169,7 +5213,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BE15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BF15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5334,6 +5378,9 @@
       <c r="BE15" t="n">
         <v>6</v>
       </c>
+      <c r="BF15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5347,7 +5394,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BE16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BF16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5512,6 +5559,9 @@
       <c r="BE16" t="n">
         <v>4</v>
       </c>
+      <c r="BF16" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5525,7 +5575,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BE17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BF17), 0)</f>
         <v/>
       </c>
       <c r="D17" s="10" t="n">
@@ -5690,6 +5740,9 @@
       <c r="BE17" t="n">
         <v>0</v>
       </c>
+      <c r="BF17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5703,7 +5756,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BE18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BF18), 0)</f>
         <v/>
       </c>
       <c r="J18" s="6" t="n"/>
@@ -5848,6 +5901,9 @@
       <c r="BE18" t="n">
         <v>6</v>
       </c>
+      <c r="BF18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5861,7 +5917,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BE19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BF19), 0)</f>
         <v/>
       </c>
       <c r="G19" s="5" t="n">
@@ -6017,6 +6073,9 @@
       <c r="BE19" t="n">
         <v>6</v>
       </c>
+      <c r="BF19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6030,7 +6089,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BE20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BF20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6148,6 +6207,9 @@
       <c r="BE20" t="n">
         <v>6</v>
       </c>
+      <c r="BF20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6161,7 +6223,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BE21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BF21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6273,6 +6335,9 @@
       <c r="BE21" t="n">
         <v>6</v>
       </c>
+      <c r="BF21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6286,7 +6351,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BE22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BF22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6395,6 +6460,9 @@
       <c r="BE22" t="n">
         <v>6</v>
       </c>
+      <c r="BF22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6408,7 +6476,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BE23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BF23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6511,6 +6579,9 @@
       <c r="BE23" t="n">
         <v>4</v>
       </c>
+      <c r="BF23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6524,7 +6595,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BE24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BF24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6621,6 +6692,9 @@
       <c r="BE24" t="n">
         <v>0</v>
       </c>
+      <c r="BF24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6634,7 +6708,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BE25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BF25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6728,6 +6802,9 @@
       <c r="BE25" t="n">
         <v>0</v>
       </c>
+      <c r="BF25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6741,7 +6818,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BE26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BF26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6835,6 +6912,9 @@
       <c r="BE26" t="n">
         <v>0</v>
       </c>
+      <c r="BF26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6848,7 +6928,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BE27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BF27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6942,6 +7022,9 @@
       <c r="BE27" t="n">
         <v>0</v>
       </c>
+      <c r="BF27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -6955,7 +7038,7 @@
         </is>
       </c>
       <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:BE28), 0)</f>
+        <f>ROUND(AVERAGE(D28:BF28), 0)</f>
         <v/>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -6996,6 +7079,9 @@
         <v>6</v>
       </c>
       <c r="BE28" t="n">
+        <v>6</v>
+      </c>
+      <c r="BF28" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH38"/>
+  <dimension ref="A1:AH26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -1079,7 +1079,7 @@
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
@@ -1096,21 +1096,21 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>90500</v>
+        <v>126020</v>
       </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
       <c r="H5" s="13" t="n">
-        <v>10000</v>
+        <v>3850</v>
       </c>
       <c r="I5" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J5" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>10000</v>
+        <v>8800</v>
       </c>
       <c r="L5" s="13" t="n">
         <v>10000</v>
@@ -1131,12 +1131,12 @@
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C6" s="12">
@@ -1148,11 +1148,13 @@
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>135225</v>
+        <v>83900</v>
       </c>
       <c r="F6" s="13" t="n"/>
       <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n"/>
+      <c r="H6" s="13" t="n">
+        <v>10000</v>
+      </c>
       <c r="I6" s="13" t="n">
         <v>10000</v>
       </c>
@@ -1160,13 +1162,13 @@
         <v>10000</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>10000</v>
+        <v>8600</v>
       </c>
       <c r="L6" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0</v>
+        <v>5350</v>
       </c>
       <c r="N6" s="13" t="n"/>
       <c r="O6" s="13" t="n"/>
@@ -1181,7 +1183,7 @@
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
@@ -1198,34 +1200,36 @@
         <v/>
       </c>
       <c r="E7" s="14" t="n">
-        <v>126020</v>
+        <v>48250</v>
       </c>
       <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
+      <c r="G7" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H7" s="13" t="n">
-        <v>3850</v>
+        <v>10000</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>0</v>
+        <v>4300</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>8800</v>
+        <v>6300</v>
       </c>
       <c r="L7" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="n"/>
       <c r="P7" s="13" t="n"/>
       <c r="Q7" s="13" t="n"/>
       <c r="R7" s="13" t="n"/>
-      <c r="S7" s="13" t="n"/>
+      <c r="S7" s="21" t="n"/>
       <c r="T7" s="13" t="n"/>
       <c r="U7" s="13" t="n"/>
       <c r="V7" s="13" t="n"/>
@@ -1233,12 +1237,12 @@
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C8" s="12">
@@ -1250,34 +1254,30 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>83900</v>
+        <v>99500</v>
       </c>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>10000</v>
-      </c>
+      <c r="H8" s="13" t="n"/>
+      <c r="I8" s="13" t="n"/>
       <c r="J8" s="13" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>8600</v>
+        <v>6100</v>
       </c>
       <c r="L8" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>5350</v>
+        <v>5550</v>
       </c>
       <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="13" t="n"/>
       <c r="R8" s="13" t="n"/>
-      <c r="S8" s="13" t="n"/>
+      <c r="S8" s="21" t="n"/>
       <c r="T8" s="13" t="n"/>
       <c r="U8" s="13" t="n"/>
       <c r="V8" s="13" t="n"/>
@@ -1285,7 +1285,7 @@
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
@@ -1302,29 +1302,29 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>48250</v>
+        <v>18350</v>
       </c>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>4300</v>
+        <v>0</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>6300</v>
+        <v>6100</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>10000</v>
+        <v>6100</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
@@ -1339,12 +1339,12 @@
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C10" s="12">
@@ -1356,23 +1356,31 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>99500</v>
-      </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
+        <v>49800</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>5800</v>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>4050</v>
+      </c>
       <c r="J10" s="13" t="n">
-        <v>5000</v>
+        <v>4350</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>6100</v>
+        <v>4600</v>
       </c>
       <c r="L10" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M10" s="13" t="n">
-        <v>5550</v>
+        <v>4100</v>
       </c>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
@@ -1387,7 +1395,7 @@
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -1404,29 +1412,31 @@
         <v/>
       </c>
       <c r="E11" s="14" t="n">
-        <v>18350</v>
-      </c>
-      <c r="F11" s="13" t="n"/>
+        <v>45850</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G11" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>0</v>
+        <v>4100</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>0</v>
+        <v>4400</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>0</v>
+        <v>4700</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>6100</v>
+        <v>4150</v>
       </c>
       <c r="L11" s="13" t="n">
-        <v>6100</v>
+        <v>9300</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>0</v>
+        <v>4350</v>
       </c>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
@@ -1441,12 +1451,12 @@
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C12" s="12">
@@ -1458,28 +1468,24 @@
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>54800</v>
-      </c>
-      <c r="F12" s="13" t="n">
+        <v>141400</v>
+      </c>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J12" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H12" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>2450</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>4050</v>
-      </c>
       <c r="K12" s="13" t="n">
-        <v>4650</v>
+        <v>4100</v>
       </c>
       <c r="L12" s="13" t="n">
-        <v>10000</v>
+        <v>13400</v>
       </c>
       <c r="M12" s="13" t="n">
         <v>4200</v>
@@ -1497,7 +1503,7 @@
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
@@ -1514,31 +1520,27 @@
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>49800</v>
-      </c>
-      <c r="F13" s="13" t="n">
+        <v>45700</v>
+      </c>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="13" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J13" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="K13" s="13" t="n">
         <v>4000</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H13" s="13" t="n">
-        <v>5800</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>4050</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>4350</v>
-      </c>
-      <c r="K13" s="13" t="n">
-        <v>4600</v>
       </c>
       <c r="L13" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>4100</v>
+        <v>4300</v>
       </c>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
@@ -1553,12 +1555,12 @@
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C14" s="12">
@@ -1570,22 +1572,28 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>53000</v>
-      </c>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
+        <v>49250</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>4050</v>
+      </c>
       <c r="I14" s="13" t="n">
-        <v>4300</v>
+        <v>5600</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>4100</v>
+        <v>1300</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>4200</v>
+        <v>3100</v>
       </c>
       <c r="L14" s="13" t="n">
-        <v>8450</v>
+        <v>9350</v>
       </c>
       <c r="M14" s="13" t="n">
         <v>0</v>
@@ -1603,7 +1611,7 @@
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
@@ -1620,31 +1628,27 @@
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>45850</v>
-      </c>
-      <c r="F15" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G15" s="13" t="n">
-        <v>4000</v>
-      </c>
+        <v>46775</v>
+      </c>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n">
-        <v>4100</v>
+        <v>3650</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>4400</v>
+        <v>7600</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>4700</v>
+        <v>3150</v>
       </c>
       <c r="K15" s="13" t="n">
-        <v>4150</v>
+        <v>3000</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>9300</v>
+        <v>10000</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>4350</v>
+        <v>2550</v>
       </c>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
@@ -1659,12 +1663,12 @@
     <row r="16" ht="16.5" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C16" s="12">
@@ -1676,27 +1680,25 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>141400</v>
+        <v>77200</v>
       </c>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
-      <c r="H16" s="13" t="n">
-        <v>4050</v>
-      </c>
+      <c r="H16" s="13" t="n"/>
       <c r="I16" s="13" t="n">
-        <v>4100</v>
+        <v>0</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>4000</v>
+        <v>950</v>
       </c>
       <c r="K16" s="13" t="n">
-        <v>4100</v>
+        <v>1400</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>13400</v>
+        <v>2200</v>
       </c>
       <c r="M16" s="13" t="n">
-        <v>4200</v>
+        <v>0</v>
       </c>
       <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="n"/>
@@ -1711,12 +1713,12 @@
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C17" s="12">
@@ -1728,34 +1730,32 @@
         <v/>
       </c>
       <c r="E17" s="14" t="n">
-        <v>47650</v>
+        <v>8750</v>
       </c>
       <c r="F17" s="13" t="n"/>
       <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n">
-        <v>1200</v>
-      </c>
+      <c r="H17" s="13" t="n"/>
       <c r="I17" s="13" t="n">
-        <v>4000</v>
+        <v>4150</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>150</v>
+        <v>2650</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>4050</v>
+        <v>1050</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>6650</v>
+        <v>1050</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="13" t="n"/>
       <c r="Q17" s="13" t="n"/>
       <c r="R17" s="13" t="n"/>
-      <c r="S17" s="21" t="n"/>
+      <c r="S17" s="13" t="n"/>
       <c r="T17" s="13" t="n"/>
       <c r="U17" s="13" t="n"/>
       <c r="V17" s="13" t="n"/>
@@ -1763,12 +1763,12 @@
     <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C18" s="12">
@@ -1780,34 +1780,28 @@
         <v/>
       </c>
       <c r="E18" s="14" t="n">
-        <v>45700</v>
+        <v>21150</v>
       </c>
       <c r="F18" s="13" t="n"/>
       <c r="G18" s="13" t="n"/>
-      <c r="H18" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="13" t="n">
-        <v>3500</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>4050</v>
-      </c>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
       <c r="K18" s="13" t="n">
-        <v>4000</v>
+        <v>600</v>
       </c>
       <c r="L18" s="13" t="n">
-        <v>10000</v>
+        <v>1100</v>
       </c>
       <c r="M18" s="13" t="n">
-        <v>4300</v>
+        <v>2050</v>
       </c>
       <c r="N18" s="13" t="n"/>
       <c r="O18" s="13" t="n"/>
       <c r="P18" s="13" t="n"/>
       <c r="Q18" s="13" t="n"/>
       <c r="R18" s="13" t="n"/>
-      <c r="S18" s="21" t="n"/>
+      <c r="S18" s="13" t="n"/>
       <c r="T18" s="13" t="n"/>
       <c r="U18" s="13" t="n"/>
       <c r="V18" s="13" t="n"/>
@@ -1815,12 +1809,12 @@
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C19" s="12">
@@ -1832,28 +1826,16 @@
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>49250</v>
-      </c>
-      <c r="F19" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G19" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H19" s="13" t="n">
-        <v>4050</v>
-      </c>
-      <c r="I19" s="13" t="n">
-        <v>5600</v>
-      </c>
-      <c r="J19" s="13" t="n">
-        <v>1300</v>
-      </c>
-      <c r="K19" s="13" t="n">
-        <v>3100</v>
-      </c>
+        <v>11550</v>
+      </c>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
       <c r="L19" s="13" t="n">
-        <v>9350</v>
+        <v>300</v>
       </c>
       <c r="M19" s="13" t="n">
         <v>0</v>
@@ -1863,7 +1845,7 @@
       <c r="P19" s="13" t="n"/>
       <c r="Q19" s="13" t="n"/>
       <c r="R19" s="13" t="n"/>
-      <c r="S19" s="21" t="n"/>
+      <c r="S19" s="13" t="n"/>
       <c r="T19" s="13" t="n"/>
       <c r="U19" s="13" t="n"/>
       <c r="V19" s="13" t="n"/>
@@ -1871,12 +1853,12 @@
     <row r="20" ht="16.5" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C20" s="12">
@@ -1888,34 +1870,26 @@
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>46775</v>
+        <v>55390</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n">
-        <v>3650</v>
-      </c>
-      <c r="I20" s="13" t="n">
-        <v>7600</v>
-      </c>
-      <c r="J20" s="13" t="n">
-        <v>3150</v>
-      </c>
-      <c r="K20" s="13" t="n">
-        <v>3000</v>
-      </c>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="13" t="n"/>
       <c r="L20" s="13" t="n">
-        <v>10000</v>
+        <v>10650</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>2550</v>
+        <v>4100</v>
       </c>
       <c r="N20" s="13" t="n"/>
       <c r="O20" s="13" t="n"/>
       <c r="P20" s="13" t="n"/>
       <c r="Q20" s="13" t="n"/>
       <c r="R20" s="13" t="n"/>
-      <c r="S20" s="21" t="n"/>
+      <c r="S20" s="13" t="n"/>
       <c r="T20" s="13" t="n"/>
       <c r="U20" s="13" t="n"/>
       <c r="V20" s="13" t="n"/>
@@ -1923,12 +1897,12 @@
     <row r="21" ht="16.5" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C21" s="12">
@@ -1940,32 +1914,26 @@
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>77200</v>
+        <v>64600</v>
       </c>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
       <c r="H21" s="13" t="n"/>
-      <c r="I21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>950</v>
-      </c>
-      <c r="K21" s="13" t="n">
-        <v>1400</v>
-      </c>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="13" t="n"/>
       <c r="L21" s="13" t="n">
-        <v>2200</v>
+        <v>4400</v>
       </c>
       <c r="M21" s="13" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="N21" s="13" t="n"/>
       <c r="O21" s="13" t="n"/>
       <c r="P21" s="13" t="n"/>
       <c r="Q21" s="13" t="n"/>
       <c r="R21" s="13" t="n"/>
-      <c r="S21" s="21" t="n"/>
+      <c r="S21" s="13" t="n"/>
       <c r="T21" s="13" t="n"/>
       <c r="U21" s="13" t="n"/>
       <c r="V21" s="13" t="n"/>
@@ -1973,12 +1941,12 @@
     <row r="22" ht="16.5" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C22" s="12">
@@ -1990,25 +1958,19 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>8750</v>
+        <v>48250</v>
       </c>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="n"/>
       <c r="H22" s="13" t="n"/>
-      <c r="I22" s="13" t="n">
-        <v>4150</v>
-      </c>
-      <c r="J22" s="13" t="n">
-        <v>2650</v>
-      </c>
-      <c r="K22" s="13" t="n">
-        <v>1050</v>
-      </c>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
+      <c r="K22" s="13" t="n"/>
       <c r="L22" s="13" t="n">
-        <v>1050</v>
+        <v>4500</v>
       </c>
       <c r="M22" s="13" t="n">
-        <v>900</v>
+        <v>4100</v>
       </c>
       <c r="N22" s="13" t="n"/>
       <c r="O22" s="13" t="n"/>
@@ -2023,12 +1985,12 @@
     <row r="23" ht="16.5" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C23" s="12">
@@ -2040,21 +2002,19 @@
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>21150</v>
+        <v>118475</v>
       </c>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
       <c r="H23" s="13" t="n"/>
       <c r="I23" s="13" t="n"/>
       <c r="J23" s="13" t="n"/>
-      <c r="K23" s="13" t="n">
-        <v>600</v>
-      </c>
+      <c r="K23" s="13" t="n"/>
       <c r="L23" s="13" t="n">
-        <v>1100</v>
+        <v>4100</v>
       </c>
       <c r="M23" s="13" t="n">
-        <v>2050</v>
+        <v>4050</v>
       </c>
       <c r="N23" s="13" t="n"/>
       <c r="O23" s="13" t="n"/>
@@ -2069,12 +2029,12 @@
     <row r="24" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="C24" s="12">
@@ -2086,27 +2046,19 @@
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>17200</v>
+        <v>110000</v>
       </c>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="I24" s="13" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J24" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="13" t="n"/>
       <c r="L24" s="13" t="n">
-        <v>2050</v>
+        <v>9500</v>
       </c>
       <c r="M24" s="13" t="n">
-        <v>0</v>
+        <v>10100</v>
       </c>
       <c r="N24" s="13" t="n"/>
       <c r="O24" s="13" t="n"/>
@@ -2121,12 +2073,12 @@
     <row r="25" ht="16.5" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C25" s="12">
@@ -2138,7 +2090,7 @@
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>13875</v>
+        <v>14750</v>
       </c>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
@@ -2146,11 +2098,9 @@
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="13" t="n"/>
       <c r="K25" s="13" t="n"/>
-      <c r="L25" s="13" t="n">
-        <v>600</v>
-      </c>
+      <c r="L25" s="13" t="n"/>
       <c r="M25" s="13" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="13" t="n"/>
@@ -2165,12 +2115,12 @@
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C26" s="12">
@@ -2182,7 +2132,7 @@
         <v/>
       </c>
       <c r="E26" s="14" t="n">
-        <v>11550</v>
+        <v>156740</v>
       </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
@@ -2190,11 +2140,9 @@
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="13" t="n"/>
       <c r="K26" s="13" t="n"/>
-      <c r="L26" s="13" t="n">
-        <v>300</v>
-      </c>
+      <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="n">
-        <v>0</v>
+        <v>6300</v>
       </c>
       <c r="N26" s="13" t="n"/>
       <c r="O26" s="13" t="n"/>
@@ -2206,530 +2154,18 @@
       <c r="U26" s="13" t="n"/>
       <c r="V26" s="13" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>Anonymous</t>
-        </is>
-      </c>
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>21/04/2026</t>
-        </is>
-      </c>
-      <c r="C27" s="12">
-        <f>ROUND(AVERAGE(F27:AI27), 0)</f>
-        <v/>
-      </c>
-      <c r="D27" s="1">
-        <f>SUM(F27:AI27)</f>
-        <v/>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>55390</v>
-      </c>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="n"/>
-      <c r="L27" s="13" t="n">
-        <v>10650</v>
-      </c>
-      <c r="M27" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="N27" s="13" t="n"/>
-      <c r="O27" s="13" t="n"/>
-      <c r="P27" s="13" t="n"/>
-      <c r="Q27" s="13" t="n"/>
-      <c r="R27" s="13" t="n"/>
-      <c r="S27" s="13" t="n"/>
-      <c r="T27" s="13" t="n"/>
-      <c r="U27" s="13" t="n"/>
-      <c r="V27" s="13" t="n"/>
-    </row>
-    <row r="28" ht="16.5" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C28" s="12">
-        <f>ROUND(AVERAGE(F28:AI28), 0)</f>
-        <v/>
-      </c>
-      <c r="D28" s="1">
-        <f>SUM(F28:AI28)</f>
-        <v/>
-      </c>
-      <c r="E28" s="14" t="n">
-        <v>64600</v>
-      </c>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="13" t="n"/>
-      <c r="L28" s="13" t="n">
-        <v>4400</v>
-      </c>
-      <c r="M28" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="N28" s="13" t="n"/>
-      <c r="O28" s="13" t="n"/>
-      <c r="P28" s="13" t="n"/>
-      <c r="Q28" s="13" t="n"/>
-      <c r="R28" s="13" t="n"/>
-      <c r="S28" s="13" t="n"/>
-      <c r="T28" s="13" t="n"/>
-      <c r="U28" s="13" t="n"/>
-      <c r="V28" s="13" t="n"/>
-    </row>
-    <row r="29" ht="16.5" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>TinoGiusa</t>
-        </is>
-      </c>
-      <c r="B29" s="16" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C29" s="12">
-        <f>ROUND(AVERAGE(F29:AI29), 0)</f>
-        <v/>
-      </c>
-      <c r="D29" s="1">
-        <f>SUM(F29:AI29)</f>
-        <v/>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>48250</v>
-      </c>
-      <c r="F29" s="13" t="n"/>
-      <c r="G29" s="13" t="n"/>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="13" t="n"/>
-      <c r="K29" s="13" t="n"/>
-      <c r="L29" s="13" t="n">
-        <v>4500</v>
-      </c>
-      <c r="M29" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="N29" s="13" t="n"/>
-      <c r="O29" s="13" t="n"/>
-      <c r="P29" s="13" t="n"/>
-      <c r="Q29" s="13" t="n"/>
-      <c r="R29" s="13" t="n"/>
-      <c r="S29" s="13" t="n"/>
-      <c r="T29" s="13" t="n"/>
-      <c r="U29" s="13" t="n"/>
-      <c r="V29" s="13" t="n"/>
-    </row>
-    <row r="30" ht="16.5" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>fhhgggf</t>
-        </is>
-      </c>
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C30" s="12">
-        <f>ROUND(AVERAGE(F30:AI30), 0)</f>
-        <v/>
-      </c>
-      <c r="D30" s="1">
-        <f>SUM(F30:AI30)</f>
-        <v/>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>118475</v>
-      </c>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="13" t="n"/>
-      <c r="J30" s="13" t="n"/>
-      <c r="K30" s="13" t="n"/>
-      <c r="L30" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="M30" s="13" t="n">
-        <v>4050</v>
-      </c>
-      <c r="N30" s="13" t="n"/>
-      <c r="O30" s="13" t="n"/>
-      <c r="P30" s="13" t="n"/>
-      <c r="Q30" s="13" t="n"/>
-      <c r="R30" s="13" t="n"/>
-      <c r="S30" s="13" t="n"/>
-      <c r="T30" s="13" t="n"/>
-      <c r="U30" s="13" t="n"/>
-      <c r="V30" s="13" t="n"/>
-    </row>
-    <row r="31" ht="16.5" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>Francesco10</t>
-        </is>
-      </c>
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C31" s="12">
-        <f>ROUND(AVERAGE(F31:AI31), 0)</f>
-        <v/>
-      </c>
-      <c r="D31" s="1">
-        <f>SUM(F31:AI31)</f>
-        <v/>
-      </c>
-      <c r="E31" s="14" t="n">
-        <v>43210</v>
-      </c>
-      <c r="F31" s="13" t="n"/>
-      <c r="G31" s="13" t="n"/>
-      <c r="H31" s="13" t="n"/>
-      <c r="I31" s="13" t="n"/>
-      <c r="J31" s="13" t="n"/>
-      <c r="K31" s="13" t="n"/>
-      <c r="L31" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="M31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="13" t="n"/>
-      <c r="O31" s="13" t="n"/>
-      <c r="P31" s="13" t="n"/>
-      <c r="Q31" s="13" t="n"/>
-      <c r="R31" s="13" t="n"/>
-      <c r="S31" s="13" t="n"/>
-      <c r="T31" s="13" t="n"/>
-      <c r="U31" s="13" t="n"/>
-      <c r="V31" s="13" t="n"/>
-    </row>
-    <row r="32" ht="16.5" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
-        <is>
-          <t>zpercu</t>
-        </is>
-      </c>
-      <c r="B32" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C32" s="12">
-        <f>ROUND(AVERAGE(F32:AI32), 0)</f>
-        <v/>
-      </c>
-      <c r="D32" s="1">
-        <f>SUM(F32:AI32)</f>
-        <v/>
-      </c>
-      <c r="E32" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="13" t="n"/>
-      <c r="J32" s="13" t="n"/>
-      <c r="K32" s="13" t="n"/>
-      <c r="L32" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="13" t="n"/>
-      <c r="O32" s="13" t="n"/>
-      <c r="P32" s="13" t="n"/>
-      <c r="Q32" s="13" t="n"/>
-      <c r="R32" s="13" t="n"/>
-      <c r="S32" s="13" t="n"/>
-      <c r="T32" s="13" t="n"/>
-      <c r="U32" s="13" t="n"/>
-      <c r="V32" s="13" t="n"/>
-    </row>
-    <row r="33" ht="16.5" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>KAIZERS</t>
-        </is>
-      </c>
-      <c r="B33" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C33" s="12">
-        <f>ROUND(AVERAGE(F33:AI33), 0)</f>
-        <v/>
-      </c>
-      <c r="D33" s="1">
-        <f>SUM(F33:AI33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="14" t="n">
-        <v>47025</v>
-      </c>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
-      <c r="H33" s="13" t="n"/>
-      <c r="I33" s="13" t="n"/>
-      <c r="J33" s="13" t="n"/>
-      <c r="K33" s="13" t="n"/>
-      <c r="L33" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="M33" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="13" t="n"/>
-      <c r="O33" s="13" t="n"/>
-      <c r="P33" s="13" t="n"/>
-      <c r="Q33" s="13" t="n"/>
-      <c r="R33" s="13" t="n"/>
-      <c r="S33" s="13" t="n"/>
-      <c r="T33" s="13" t="n"/>
-      <c r="U33" s="13" t="n"/>
-      <c r="V33" s="13" t="n"/>
-    </row>
-    <row r="34" ht="16.5" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t>roberto</t>
-        </is>
-      </c>
-      <c r="B34" s="16" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-      <c r="C34" s="12">
-        <f>ROUND(AVERAGE(F34:AI34), 0)</f>
-        <v/>
-      </c>
-      <c r="D34" s="1">
-        <f>SUM(F34:AI34)</f>
-        <v/>
-      </c>
-      <c r="E34" s="14" t="n">
-        <v>48200</v>
-      </c>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
-      <c r="I34" s="13" t="n"/>
-      <c r="J34" s="13" t="n"/>
-      <c r="K34" s="13" t="n"/>
-      <c r="L34" s="13" t="n">
-        <v>4200</v>
-      </c>
-      <c r="M34" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="N34" s="13" t="n"/>
-      <c r="O34" s="13" t="n"/>
-      <c r="P34" s="13" t="n"/>
-      <c r="Q34" s="13" t="n"/>
-      <c r="R34" s="13" t="n"/>
-      <c r="S34" s="13" t="n"/>
-      <c r="T34" s="13" t="n"/>
-      <c r="U34" s="13" t="n"/>
-      <c r="V34" s="13" t="n"/>
-    </row>
-    <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>maragno</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
-      <c r="C35" s="12">
-        <f>ROUND(AVERAGE(F35:AI35), 0)</f>
-        <v/>
-      </c>
-      <c r="D35" s="1">
-        <f>SUM(F35:AI35)</f>
-        <v/>
-      </c>
-      <c r="E35" s="14" t="n">
-        <v>110000</v>
-      </c>
-      <c r="F35" s="13" t="n"/>
-      <c r="G35" s="13" t="n"/>
-      <c r="H35" s="13" t="n"/>
-      <c r="I35" s="13" t="n"/>
-      <c r="J35" s="13" t="n"/>
-      <c r="K35" s="13" t="n"/>
-      <c r="L35" s="13" t="n">
-        <v>9500</v>
-      </c>
-      <c r="M35" s="13" t="n">
-        <v>10100</v>
-      </c>
-      <c r="N35" s="13" t="n"/>
-      <c r="O35" s="13" t="n"/>
-      <c r="P35" s="13" t="n"/>
-      <c r="Q35" s="13" t="n"/>
-      <c r="R35" s="13" t="n"/>
-      <c r="S35" s="13" t="n"/>
-      <c r="T35" s="13" t="n"/>
-      <c r="U35" s="13" t="n"/>
-      <c r="V35" s="13" t="n"/>
-    </row>
-    <row r="36" ht="16.5" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>rasim01</t>
-        </is>
-      </c>
-      <c r="B36" s="16" t="inlineStr">
-        <is>
-          <t>28/05/2026</t>
-        </is>
-      </c>
-      <c r="C36" s="12">
-        <f>ROUND(AVERAGE(F36:AI36), 0)</f>
-        <v/>
-      </c>
-      <c r="D36" s="1">
-        <f>SUM(F36:AI36)</f>
-        <v/>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>28450</v>
-      </c>
-      <c r="F36" s="13" t="n"/>
-      <c r="G36" s="13" t="n"/>
-      <c r="H36" s="13" t="n"/>
-      <c r="I36" s="13" t="n"/>
-      <c r="J36" s="13" t="n"/>
-      <c r="K36" s="13" t="n"/>
-      <c r="L36" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="13" t="n"/>
-      <c r="O36" s="13" t="n"/>
-      <c r="P36" s="13" t="n"/>
-      <c r="Q36" s="13" t="n"/>
-      <c r="R36" s="13" t="n"/>
-      <c r="S36" s="13" t="n"/>
-      <c r="T36" s="13" t="n"/>
-      <c r="U36" s="13" t="n"/>
-      <c r="V36" s="13" t="n"/>
-    </row>
-    <row r="37" ht="16.5" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B37" s="16" t="inlineStr">
-        <is>
-          <t>21/06/2026</t>
-        </is>
-      </c>
-      <c r="C37" s="12">
-        <f>ROUND(AVERAGE(F37:AI37), 0)</f>
-        <v/>
-      </c>
-      <c r="D37" s="1">
-        <f>SUM(F37:AI37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="14" t="n">
-        <v>14750</v>
-      </c>
-      <c r="F37" s="13" t="n"/>
-      <c r="G37" s="13" t="n"/>
-      <c r="H37" s="13" t="n"/>
-      <c r="I37" s="13" t="n"/>
-      <c r="J37" s="13" t="n"/>
-      <c r="K37" s="13" t="n"/>
-      <c r="L37" s="13" t="n"/>
-      <c r="M37" s="13" t="n">
-        <v>1500</v>
-      </c>
-      <c r="N37" s="13" t="n"/>
-      <c r="O37" s="13" t="n"/>
-      <c r="P37" s="13" t="n"/>
-      <c r="Q37" s="13" t="n"/>
-      <c r="R37" s="13" t="n"/>
-      <c r="S37" s="13" t="n"/>
-      <c r="T37" s="13" t="n"/>
-      <c r="U37" s="13" t="n"/>
-      <c r="V37" s="13" t="n"/>
-    </row>
-    <row r="38" ht="16.5" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>Akemi</t>
-        </is>
-      </c>
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>21/06/2026</t>
-        </is>
-      </c>
-      <c r="C38" s="12">
-        <f>ROUND(AVERAGE(F38:AI38), 0)</f>
-        <v/>
-      </c>
-      <c r="D38" s="1">
-        <f>SUM(F38:AI38)</f>
-        <v/>
-      </c>
-      <c r="E38" s="14" t="n">
-        <v>156740</v>
-      </c>
-      <c r="F38" s="13" t="n"/>
-      <c r="G38" s="13" t="n"/>
-      <c r="H38" s="13" t="n"/>
-      <c r="I38" s="13" t="n"/>
-      <c r="J38" s="13" t="n"/>
-      <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n">
-        <v>6300</v>
-      </c>
-      <c r="N38" s="13" t="n"/>
-      <c r="O38" s="13" t="n"/>
-      <c r="P38" s="13" t="n"/>
-      <c r="Q38" s="13" t="n"/>
-      <c r="R38" s="13" t="n"/>
-      <c r="S38" s="13" t="n"/>
-      <c r="T38" s="13" t="n"/>
-      <c r="U38" s="13" t="n"/>
-      <c r="V38" s="13" t="n"/>
-    </row>
+    <row r="27" ht="16.5" customHeight="1"/>
+    <row r="28" ht="16.5" customHeight="1"/>
+    <row r="29" ht="16.5" customHeight="1"/>
+    <row r="30" ht="16.5" customHeight="1"/>
+    <row r="31" ht="16.5" customHeight="1"/>
+    <row r="32" ht="16.5" customHeight="1"/>
+    <row r="33" ht="16.5" customHeight="1"/>
+    <row r="34" ht="16.5" customHeight="1"/>
+    <row r="35" ht="16.5" customHeight="1"/>
+    <row r="36" ht="16.5" customHeight="1"/>
+    <row r="37" ht="16.5" customHeight="1"/>
+    <row r="38" ht="16.5" customHeight="1"/>
     <row r="39" ht="16.5" customHeight="1"/>
     <row r="40" ht="16.5" customHeight="1"/>
     <row r="41" ht="16.5" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -973,6 +973,9 @@
       <c r="M2" t="n">
         <v>2450</v>
       </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
@@ -1020,7 +1023,9 @@
       <c r="M3" s="13" t="n">
         <v>10000</v>
       </c>
-      <c r="N3" s="13" t="n"/>
+      <c r="N3" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O3" s="13" t="n"/>
       <c r="P3" s="13" t="n"/>
       <c r="Q3" s="13" t="n"/>
@@ -1066,7 +1071,9 @@
       <c r="M4" s="13" t="n">
         <v>10050</v>
       </c>
-      <c r="N4" s="13" t="n"/>
+      <c r="N4" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O4" s="13" t="n"/>
       <c r="P4" s="13" t="n"/>
       <c r="Q4" s="13" t="n"/>
@@ -1118,7 +1125,9 @@
       <c r="M5" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="13" t="n"/>
+      <c r="N5" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O5" s="13" t="n"/>
       <c r="P5" s="13" t="n"/>
       <c r="Q5" s="13" t="n"/>
@@ -1170,7 +1179,9 @@
       <c r="M6" s="13" t="n">
         <v>5350</v>
       </c>
-      <c r="N6" s="13" t="n"/>
+      <c r="N6" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O6" s="13" t="n"/>
       <c r="P6" s="13" t="n"/>
       <c r="Q6" s="13" t="n"/>
@@ -1224,7 +1235,9 @@
       <c r="M7" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="N7" s="13" t="n"/>
+      <c r="N7" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O7" s="13" t="n"/>
       <c r="P7" s="13" t="n"/>
       <c r="Q7" s="13" t="n"/>
@@ -1272,7 +1285,9 @@
       <c r="M8" s="13" t="n">
         <v>5550</v>
       </c>
-      <c r="N8" s="13" t="n"/>
+      <c r="N8" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="13" t="n"/>
@@ -1326,7 +1341,9 @@
       <c r="M9" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="13" t="n"/>
+      <c r="N9" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O9" s="13" t="n"/>
       <c r="P9" s="13" t="n"/>
       <c r="Q9" s="13" t="n"/>
@@ -1382,7 +1399,9 @@
       <c r="M10" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="N10" s="13" t="n"/>
+      <c r="N10" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O10" s="13" t="n"/>
       <c r="P10" s="13" t="n"/>
       <c r="Q10" s="13" t="n"/>
@@ -1438,7 +1457,9 @@
       <c r="M11" s="13" t="n">
         <v>4350</v>
       </c>
-      <c r="N11" s="13" t="n"/>
+      <c r="N11" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O11" s="13" t="n"/>
       <c r="P11" s="13" t="n"/>
       <c r="Q11" s="13" t="n"/>
@@ -1490,7 +1511,9 @@
       <c r="M12" s="13" t="n">
         <v>4200</v>
       </c>
-      <c r="N12" s="13" t="n"/>
+      <c r="N12" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O12" s="13" t="n"/>
       <c r="P12" s="13" t="n"/>
       <c r="Q12" s="13" t="n"/>
@@ -1542,7 +1565,9 @@
       <c r="M13" s="13" t="n">
         <v>4300</v>
       </c>
-      <c r="N13" s="13" t="n"/>
+      <c r="N13" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O13" s="13" t="n"/>
       <c r="P13" s="13" t="n"/>
       <c r="Q13" s="13" t="n"/>
@@ -1598,7 +1623,9 @@
       <c r="M14" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="13" t="n"/>
+      <c r="N14" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O14" s="13" t="n"/>
       <c r="P14" s="13" t="n"/>
       <c r="Q14" s="13" t="n"/>
@@ -1650,7 +1677,9 @@
       <c r="M15" s="13" t="n">
         <v>2550</v>
       </c>
-      <c r="N15" s="13" t="n"/>
+      <c r="N15" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O15" s="13" t="n"/>
       <c r="P15" s="13" t="n"/>
       <c r="Q15" s="13" t="n"/>
@@ -1700,7 +1729,9 @@
       <c r="M16" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="13" t="n"/>
+      <c r="N16" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="13" t="n"/>
       <c r="Q16" s="13" t="n"/>
@@ -1750,7 +1781,9 @@
       <c r="M17" s="13" t="n">
         <v>900</v>
       </c>
-      <c r="N17" s="13" t="n"/>
+      <c r="N17" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="13" t="n"/>
       <c r="Q17" s="13" t="n"/>
@@ -1796,7 +1829,9 @@
       <c r="M18" s="13" t="n">
         <v>2050</v>
       </c>
-      <c r="N18" s="13" t="n"/>
+      <c r="N18" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O18" s="13" t="n"/>
       <c r="P18" s="13" t="n"/>
       <c r="Q18" s="13" t="n"/>
@@ -1840,7 +1875,9 @@
       <c r="M19" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="N19" s="13" t="n"/>
+      <c r="N19" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O19" s="13" t="n"/>
       <c r="P19" s="13" t="n"/>
       <c r="Q19" s="13" t="n"/>
@@ -1884,7 +1921,9 @@
       <c r="M20" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="N20" s="13" t="n"/>
+      <c r="N20" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O20" s="13" t="n"/>
       <c r="P20" s="13" t="n"/>
       <c r="Q20" s="13" t="n"/>
@@ -1928,7 +1967,9 @@
       <c r="M21" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="N21" s="13" t="n"/>
+      <c r="N21" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O21" s="13" t="n"/>
       <c r="P21" s="13" t="n"/>
       <c r="Q21" s="13" t="n"/>
@@ -1972,7 +2013,9 @@
       <c r="M22" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="N22" s="13" t="n"/>
+      <c r="N22" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O22" s="13" t="n"/>
       <c r="P22" s="13" t="n"/>
       <c r="Q22" s="13" t="n"/>
@@ -2016,7 +2059,9 @@
       <c r="M23" s="13" t="n">
         <v>4050</v>
       </c>
-      <c r="N23" s="13" t="n"/>
+      <c r="N23" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O23" s="13" t="n"/>
       <c r="P23" s="13" t="n"/>
       <c r="Q23" s="13" t="n"/>
@@ -2060,7 +2105,9 @@
       <c r="M24" s="13" t="n">
         <v>10100</v>
       </c>
-      <c r="N24" s="13" t="n"/>
+      <c r="N24" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O24" s="13" t="n"/>
       <c r="P24" s="13" t="n"/>
       <c r="Q24" s="13" t="n"/>
@@ -2102,7 +2149,9 @@
       <c r="M25" s="13" t="n">
         <v>1500</v>
       </c>
-      <c r="N25" s="13" t="n"/>
+      <c r="N25" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O25" s="13" t="n"/>
       <c r="P25" s="13" t="n"/>
       <c r="Q25" s="13" t="n"/>
@@ -2144,7 +2193,9 @@
       <c r="M26" s="13" t="n">
         <v>6300</v>
       </c>
-      <c r="N26" s="13" t="n"/>
+      <c r="N26" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="O26" s="13" t="n"/>
       <c r="P26" s="13" t="n"/>
       <c r="Q26" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1709,7 +1709,7 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>78300</v>
+        <v>79400</v>
       </c>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
@@ -1730,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="13" t="n">
-        <v>1100</v>
+        <v>2200</v>
       </c>
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-24
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1709,7 +1709,7 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>80800</v>
+        <v>82000</v>
       </c>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
@@ -1730,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="13" t="n">
-        <v>3600</v>
+        <v>4800</v>
       </c>
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1103,7 +1103,7 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>133420</v>
+        <v>134020</v>
       </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
@@ -1126,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="13" t="n">
-        <v>7400</v>
+        <v>8000</v>
       </c>
       <c r="O5" s="13" t="n"/>
       <c r="P5" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF28"/>
+  <dimension ref="A1:BG27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2591,6 +2591,11 @@
           <t>17/07/2026</t>
         </is>
       </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2604,7 +2609,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BF2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BG2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2749,6 +2754,9 @@
         <v>0</v>
       </c>
       <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2764,7 +2772,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BF3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BG3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -2900,6 +2908,9 @@
       <c r="BF3" t="n">
         <v>6</v>
       </c>
+      <c r="BG3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -2913,7 +2924,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BF4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BG4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3080,6 +3091,9 @@
       </c>
       <c r="BF4" t="n">
         <v>6</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3094,7 +3108,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BF5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BG5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3262,6 +3276,9 @@
       <c r="BF5" t="n">
         <v>0</v>
       </c>
+      <c r="BG5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3275,7 +3292,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BF6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BG6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3413,6 +3430,9 @@
       <c r="BF6" t="n">
         <v>0</v>
       </c>
+      <c r="BG6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3426,7 +3446,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BF7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BG7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3552,6 +3572,9 @@
       <c r="BF7" t="n">
         <v>0</v>
       </c>
+      <c r="BG7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3565,7 +3588,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BF8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BG8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3724,33 +3747,24 @@
       <c r="BF8" t="n">
         <v>0</v>
       </c>
+      <c r="BG8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BF9), 0)</f>
-        <v/>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>5</v>
+        <f>ROUND(AVERAGE(D9:BG9), 0)</f>
+        <v/>
       </c>
       <c r="H9" s="5" t="n">
         <v>6</v>
@@ -3780,7 +3794,7 @@
         <v>6</v>
       </c>
       <c r="Q9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R9" t="n">
         <v>6</v>
@@ -3813,7 +3827,7 @@
         <v>6</v>
       </c>
       <c r="AB9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC9" t="n">
         <v>6</v>
@@ -3822,34 +3836,34 @@
         <v>6</v>
       </c>
       <c r="AE9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG9" t="n">
         <v>6</v>
       </c>
       <c r="AH9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL9" t="n">
         <v>6</v>
       </c>
       <c r="AM9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AN9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AO9" t="n">
         <v>6</v>
@@ -3903,23 +3917,38 @@
         <v>0</v>
       </c>
       <c r="BF9" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BF10), 0)</f>
-        <v/>
+        <f>ROUND(AVERAGE(D10:BG10), 0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>6</v>
@@ -3964,25 +3993,25 @@
         <v>6</v>
       </c>
       <c r="V10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
         <v>6</v>
       </c>
       <c r="AB10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC10" t="n">
         <v>6</v>
@@ -3991,10 +4020,10 @@
         <v>6</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG10" t="n">
         <v>6</v>
@@ -4006,34 +4035,34 @@
         <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL10" t="n">
         <v>6</v>
       </c>
       <c r="AM10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ10" t="n">
         <v>6</v>
       </c>
       <c r="AR10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT10" t="n">
         <v>6</v>
@@ -4051,10 +4080,10 @@
         <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA10" t="n">
         <v>6</v>
@@ -4073,55 +4102,33 @@
       </c>
       <c r="BF10" t="n">
         <v>6</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BF11), 0)</f>
-        <v/>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>6</v>
-      </c>
+        <f>ROUND(AVERAGE(D11:BG11), 0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
       <c r="M11" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N11" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
         <v>6</v>
@@ -4142,25 +4149,25 @@
         <v>6</v>
       </c>
       <c r="U11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z11" t="n">
         <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB11" t="n">
         <v>6</v>
@@ -4169,22 +4176,22 @@
         <v>6</v>
       </c>
       <c r="AD11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE11" t="n">
         <v>6</v>
       </c>
       <c r="AF11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AI11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ11" t="n">
         <v>6</v>
@@ -4208,13 +4215,13 @@
         <v>0</v>
       </c>
       <c r="AQ11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT11" t="n">
         <v>6</v>
@@ -4238,7 +4245,7 @@
         <v>0</v>
       </c>
       <c r="BA11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB11" t="n">
         <v>0</v>
@@ -4253,43 +4260,35 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BF12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BG12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="n"/>
-      <c r="M12" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N12" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
-        <v>6</v>
-      </c>
-      <c r="P12" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>6</v>
-      </c>
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="19" t="n"/>
+      <c r="P12" s="19" t="n"/>
+      <c r="Q12" s="19" t="n"/>
       <c r="R12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>6</v>
@@ -4298,7 +4297,7 @@
         <v>6</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V12" t="n">
         <v>6</v>
@@ -4307,16 +4306,16 @@
         <v>6</v>
       </c>
       <c r="X12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y12" t="n">
         <v>6</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB12" t="n">
         <v>6</v>
@@ -4325,22 +4324,22 @@
         <v>6</v>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AF12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ12" t="n">
         <v>6</v>
@@ -4352,19 +4351,19 @@
         <v>6</v>
       </c>
       <c r="AM12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AN12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR12" t="n">
         <v>6</v>
@@ -4385,16 +4384,16 @@
         <v>0</v>
       </c>
       <c r="AX12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AY12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BA12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB12" t="n">
         <v>0</v>
@@ -4403,38 +4402,68 @@
         <v>0</v>
       </c>
       <c r="BD12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF12" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BF13), 0)</f>
-        <v/>
-      </c>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
-      <c r="N13" s="6" t="n"/>
-      <c r="O13" s="19" t="n"/>
-      <c r="P13" s="19" t="n"/>
-      <c r="Q13" s="19" t="n"/>
+        <f>ROUND(AVERAGE(D13:BG13), 0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O13" t="n">
+        <v>6</v>
+      </c>
+      <c r="P13" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>6</v>
+      </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S13" t="n">
         <v>6</v>
@@ -4449,19 +4478,19 @@
         <v>6</v>
       </c>
       <c r="W13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AA13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB13" t="n">
         <v>6</v>
@@ -4473,19 +4502,19 @@
         <v>6</v>
       </c>
       <c r="AE13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH13" t="n">
         <v>4</v>
       </c>
-      <c r="AF13" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>6</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>0</v>
-      </c>
       <c r="AI13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ13" t="n">
         <v>6</v>
@@ -4497,31 +4526,31 @@
         <v>6</v>
       </c>
       <c r="AM13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AP13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AQ13" t="n">
         <v>6</v>
       </c>
       <c r="AR13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AT13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AV13" t="n">
         <v>6</v>
@@ -4530,7 +4559,7 @@
         <v>0</v>
       </c>
       <c r="AX13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY13" t="n">
         <v>6</v>
@@ -4548,19 +4577,22 @@
         <v>0</v>
       </c>
       <c r="BD13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BE13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BF13" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -4569,14 +4601,23 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BF14), 0)</f>
-        <v/>
+        <f>ROUND(AVERAGE(D14:BG14), 0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>6</v>
@@ -4585,16 +4626,16 @@
         <v>6</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O14" t="n">
         <v>6</v>
@@ -4615,25 +4656,25 @@
         <v>6</v>
       </c>
       <c r="U14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X14" t="n">
         <v>6</v>
       </c>
       <c r="Y14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB14" t="n">
         <v>6</v>
@@ -4654,7 +4695,7 @@
         <v>6</v>
       </c>
       <c r="AH14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AI14" t="n">
         <v>6</v>
@@ -4669,31 +4710,31 @@
         <v>6</v>
       </c>
       <c r="AM14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AN14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AO14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AP14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AQ14" t="n">
         <v>6</v>
       </c>
       <c r="AR14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AU14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AV14" t="n">
         <v>6</v>
@@ -4705,10 +4746,10 @@
         <v>0</v>
       </c>
       <c r="AY14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA14" t="n">
         <v>6</v>
@@ -4720,19 +4761,22 @@
         <v>0</v>
       </c>
       <c r="BD14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF14" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -4741,80 +4785,80 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BF15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BG15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
         <v>6</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>6</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S15" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" t="n">
+        <v>4</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="n">
+        <v>6</v>
+      </c>
+      <c r="W15" t="n">
+        <v>3</v>
+      </c>
+      <c r="X15" t="n">
         <v>5</v>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>6</v>
-      </c>
-      <c r="P15" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>6</v>
-      </c>
-      <c r="R15" t="n">
-        <v>6</v>
-      </c>
-      <c r="S15" t="n">
-        <v>6</v>
-      </c>
-      <c r="T15" t="n">
-        <v>6</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="n">
-        <v>5</v>
-      </c>
-      <c r="W15" t="n">
-        <v>6</v>
-      </c>
-      <c r="X15" t="n">
-        <v>6</v>
-      </c>
       <c r="Y15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AB15" t="n">
         <v>6</v>
@@ -4823,52 +4867,52 @@
         <v>6</v>
       </c>
       <c r="AD15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG15" t="n">
         <v>6</v>
       </c>
       <c r="AH15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AO15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AP15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AQ15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AR15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT15" t="n">
         <v>6</v>
@@ -4886,34 +4930,37 @@
         <v>0</v>
       </c>
       <c r="AY15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BA15" t="n">
         <v>6</v>
       </c>
       <c r="BB15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF15" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -4922,11 +4969,11 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BF16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BG16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>6</v>
@@ -4944,7 +4991,7 @@
         <v>6</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>6</v>
@@ -4970,23 +5017,23 @@
       <c r="R16" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S16" t="n">
+      <c r="S16" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -4995,7 +5042,7 @@
         <v>0</v>
       </c>
       <c r="AA16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB16" t="n">
         <v>6</v>
@@ -5010,7 +5057,7 @@
         <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG16" t="n">
         <v>6</v>
@@ -5031,31 +5078,31 @@
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AP16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AQ16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AR16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AU16" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AV16" t="n">
         <v>6</v>
@@ -5067,34 +5114,37 @@
         <v>0</v>
       </c>
       <c r="AY16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AZ16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BA16" t="n">
         <v>6</v>
       </c>
       <c r="BB16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BE16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF16" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -5103,92 +5153,72 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BF17), 0)</f>
-        <v/>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="6" t="n">
+        <f>ROUND(AVERAGE(D17:BG17), 0)</f>
+        <v/>
+      </c>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T17" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U17" t="n">
+        <v>6</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
         <v>5</v>
       </c>
-      <c r="K17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T17" t="n">
-        <v>6</v>
-      </c>
-      <c r="U17" t="n">
-        <v>6</v>
-      </c>
-      <c r="V17" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" t="n">
-        <v>0</v>
-      </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB17" t="n">
         <v>6</v>
       </c>
       <c r="AC17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF17" t="n">
         <v>6</v>
@@ -5218,10 +5248,10 @@
         <v>0</v>
       </c>
       <c r="AO17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ17" t="n">
         <v>6</v>
@@ -5233,13 +5263,13 @@
         <v>0</v>
       </c>
       <c r="AT17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -5254,7 +5284,7 @@
         <v>0</v>
       </c>
       <c r="BA17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB17" t="n">
         <v>0</v>
@@ -5263,19 +5293,22 @@
         <v>0</v>
       </c>
       <c r="BD17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF17" t="n">
         <v>6</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -5284,10 +5317,21 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BF18), 0)</f>
-        <v/>
-      </c>
-      <c r="J18" s="6" t="n"/>
+        <f>ROUND(AVERAGE(D18:BG18), 0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K18" s="6" t="n">
         <v>6</v>
       </c>
@@ -5304,7 +5348,7 @@
         <v>6</v>
       </c>
       <c r="P18" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q18" s="20" t="n">
         <v>6</v>
@@ -5318,26 +5362,26 @@
       <c r="T18" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="U18" t="n">
+      <c r="U18" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V18" t="n">
         <v>0</v>
       </c>
       <c r="W18" t="n">
+        <v>6</v>
+      </c>
+      <c r="X18" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="n">
         <v>5</v>
       </c>
-      <c r="X18" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>6</v>
-      </c>
       <c r="AA18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB18" t="n">
         <v>6</v>
@@ -5355,22 +5399,22 @@
         <v>6</v>
       </c>
       <c r="AG18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AM18" t="n">
         <v>0</v>
@@ -5385,22 +5429,22 @@
         <v>0</v>
       </c>
       <c r="AQ18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -5430,96 +5474,61 @@
         <v>6</v>
       </c>
       <c r="BF18" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG18" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BF19), 0)</f>
-        <v/>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P19" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U19" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V19" t="n">
-        <v>0</v>
-      </c>
+        <f>ROUND(AVERAGE(D19:BG19), 0)</f>
+        <v/>
+      </c>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="N19" s="6" t="n"/>
+      <c r="O19" s="20" t="n"/>
+      <c r="P19" s="20" t="n"/>
+      <c r="Q19" s="20" t="n"/>
+      <c r="R19" s="20" t="n"/>
+      <c r="S19" s="20" t="n"/>
+      <c r="T19" s="20" t="n"/>
+      <c r="U19" s="20" t="n"/>
       <c r="W19" t="n">
         <v>6</v>
       </c>
       <c r="X19" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y19" t="n">
         <v>0</v>
       </c>
       <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD19" t="n">
         <v>5</v>
       </c>
-      <c r="AA19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD19" t="n">
-        <v>6</v>
-      </c>
       <c r="AE19" t="n">
         <v>6</v>
       </c>
@@ -5530,50 +5539,50 @@
         <v>0</v>
       </c>
       <c r="AH19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR19" t="n">
         <v>5</v>
       </c>
-      <c r="AI19" t="n">
+      <c r="AS19" t="n">
         <v>5</v>
       </c>
-      <c r="AJ19" t="n">
+      <c r="AT19" t="n">
         <v>5</v>
       </c>
-      <c r="AK19" t="n">
+      <c r="AU19" t="n">
         <v>5</v>
       </c>
-      <c r="AL19" t="n">
+      <c r="AV19" t="n">
         <v>5</v>
       </c>
-      <c r="AM19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>6</v>
-      </c>
       <c r="AW19" t="n">
         <v>0</v>
       </c>
@@ -5603,21 +5612,24 @@
       </c>
       <c r="BF19" t="n">
         <v>6</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BF20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BG20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -5630,65 +5642,59 @@
       <c r="S20" s="20" t="n"/>
       <c r="T20" s="20" t="n"/>
       <c r="U20" s="20" t="n"/>
-      <c r="W20" t="n">
-        <v>6</v>
-      </c>
-      <c r="X20" t="n">
-        <v>6</v>
-      </c>
       <c r="Y20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA20" t="n">
         <v>6</v>
       </c>
       <c r="AB20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC20" t="n">
         <v>6</v>
       </c>
       <c r="AD20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO20" t="n">
         <v>5</v>
       </c>
-      <c r="AE20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>6</v>
-      </c>
       <c r="AP20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ20" t="n">
         <v>6</v>
@@ -5706,28 +5712,28 @@
         <v>5</v>
       </c>
       <c r="AV20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW20" t="n">
         <v>5</v>
       </c>
-      <c r="AW20" t="n">
-        <v>0</v>
-      </c>
       <c r="AX20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AY20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AZ20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BA20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BC20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BD20" t="n">
         <v>6</v>
@@ -5737,21 +5743,24 @@
       </c>
       <c r="BF20" t="n">
         <v>6</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BF21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BG21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -5764,15 +5773,12 @@
       <c r="S21" s="20" t="n"/>
       <c r="T21" s="20" t="n"/>
       <c r="U21" s="20" t="n"/>
-      <c r="Y21" t="n">
-        <v>6</v>
-      </c>
       <c r="Z21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA21" t="n">
         <v>3</v>
       </c>
-      <c r="AA21" t="n">
-        <v>6</v>
-      </c>
       <c r="AB21" t="n">
         <v>6</v>
       </c>
@@ -5798,64 +5804,64 @@
         <v>0</v>
       </c>
       <c r="AJ21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL21" t="n">
         <v>6</v>
       </c>
       <c r="AM21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ21" t="n">
         <v>6</v>
       </c>
       <c r="AR21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AZ21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BA21" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BB21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BC21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BD21" t="n">
         <v>6</v>
@@ -5865,21 +5871,24 @@
       </c>
       <c r="BF21" t="n">
         <v>6</v>
+      </c>
+      <c r="BG21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BF22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BG22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -5892,12 +5901,6 @@
       <c r="S22" s="20" t="n"/>
       <c r="T22" s="20" t="n"/>
       <c r="U22" s="20" t="n"/>
-      <c r="Z22" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>3</v>
-      </c>
       <c r="AB22" t="n">
         <v>6</v>
       </c>
@@ -5917,34 +5920,34 @@
         <v>6</v>
       </c>
       <c r="AH22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL22" t="n">
         <v>6</v>
       </c>
       <c r="AM22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AO22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR22" t="n">
         <v>0</v>
@@ -5959,52 +5962,55 @@
         <v>0</v>
       </c>
       <c r="AV22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AX22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AY22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AZ22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BA22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BB22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BC22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BD22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF22" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BF23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BG23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6017,15 +6023,6 @@
       <c r="S23" s="20" t="n"/>
       <c r="T23" s="20" t="n"/>
       <c r="U23" s="20" t="n"/>
-      <c r="AB23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD23" t="n">
-        <v>6</v>
-      </c>
       <c r="AE23" t="n">
         <v>6</v>
       </c>
@@ -6033,37 +6030,37 @@
         <v>6</v>
       </c>
       <c r="AG23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL23" t="n">
         <v>6</v>
       </c>
       <c r="AM23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AR23" t="n">
         <v>0</v>
@@ -6078,7 +6075,7 @@
         <v>0</v>
       </c>
       <c r="AV23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW23" t="n">
         <v>6</v>
@@ -6102,28 +6099,31 @@
         <v>0</v>
       </c>
       <c r="BD23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BE23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF23" t="n">
         <v>6</v>
+      </c>
+      <c r="BG23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BF24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BG24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6136,17 +6136,14 @@
       <c r="S24" s="20" t="n"/>
       <c r="T24" s="20" t="n"/>
       <c r="U24" s="20" t="n"/>
-      <c r="AD24" t="n">
-        <v>6</v>
-      </c>
       <c r="AE24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF24" t="n">
         <v>6</v>
       </c>
       <c r="AG24" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH24" t="n">
         <v>0</v>
@@ -6176,22 +6173,22 @@
         <v>0</v>
       </c>
       <c r="AQ24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AR24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AW24" t="n">
         <v>0</v>
@@ -6221,22 +6218,25 @@
         <v>0</v>
       </c>
       <c r="BF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BF25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BG25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6253,7 +6253,7 @@
         <v>6</v>
       </c>
       <c r="AF25" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG25" t="n">
         <v>0</v>
@@ -6265,13 +6265,13 @@
         <v>0</v>
       </c>
       <c r="AJ25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM25" t="n">
         <v>0</v>
@@ -6280,43 +6280,43 @@
         <v>0</v>
       </c>
       <c r="AO25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB25" t="n">
         <v>0</v>
@@ -6331,22 +6331,25 @@
         <v>0</v>
       </c>
       <c r="BF25" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BF26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BG26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6359,59 +6362,8 @@
       <c r="S26" s="20" t="n"/>
       <c r="T26" s="20" t="n"/>
       <c r="U26" s="20" t="n"/>
-      <c r="AE26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF26" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU26" t="n">
-        <v>0</v>
-      </c>
       <c r="AV26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW26" t="n">
         <v>0</v>
@@ -6426,7 +6378,7 @@
         <v>0</v>
       </c>
       <c r="BA26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB26" t="n">
         <v>0</v>
@@ -6435,28 +6387,31 @@
         <v>0</v>
       </c>
       <c r="BD26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF26" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BF27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BG27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6469,148 +6424,8 @@
       <c r="S27" s="20" t="n"/>
       <c r="T27" s="20" t="n"/>
       <c r="U27" s="20" t="n"/>
-      <c r="AE27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AV27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="28" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C28" s="28">
-        <f>ROUND(AVERAGE(D28:BF28), 0)</f>
-        <v/>
-      </c>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-      <c r="N28" s="6" t="n"/>
-      <c r="O28" s="20" t="n"/>
-      <c r="P28" s="20" t="n"/>
-      <c r="Q28" s="20" t="n"/>
-      <c r="R28" s="20" t="n"/>
-      <c r="S28" s="20" t="n"/>
-      <c r="T28" s="20" t="n"/>
-      <c r="U28" s="20" t="n"/>
-      <c r="AV28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ28" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA28" t="n">
-        <v>6</v>
-      </c>
-      <c r="BB28" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC28" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD28" t="n">
-        <v>6</v>
-      </c>
-      <c r="BE28" t="n">
-        <v>6</v>
-      </c>
-      <c r="BF28" t="n">
-        <v>6</v>
+      <c r="BG27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-26
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1103,7 +1103,7 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>134570</v>
+        <v>134870</v>
       </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
@@ -1126,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="13" t="n">
-        <v>8550</v>
+        <v>8850</v>
       </c>
       <c r="O5" s="13" t="n"/>
       <c r="P5" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-26
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH27"/>
+  <dimension ref="A1:BI27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2601,6 +2601,11 @@
           <t>24/07/2026</t>
         </is>
       </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2614,7 +2619,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BH2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BI2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2765,6 +2770,9 @@
         <v>0</v>
       </c>
       <c r="BH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2780,7 +2788,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BH3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BI3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -2922,6 +2930,9 @@
       <c r="BH3" t="n">
         <v>4</v>
       </c>
+      <c r="BI3" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -2935,7 +2946,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BH4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BI4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3107,6 +3118,9 @@
         <v>0</v>
       </c>
       <c r="BH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3122,7 +3136,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BH5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BI5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3296,6 +3310,9 @@
       <c r="BH5" t="n">
         <v>0</v>
       </c>
+      <c r="BI5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3309,7 +3326,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BH6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BI6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3453,6 +3470,9 @@
       <c r="BH6" t="n">
         <v>0</v>
       </c>
+      <c r="BI6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3466,7 +3486,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BH7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BI7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3598,6 +3618,9 @@
       <c r="BH7" t="n">
         <v>0</v>
       </c>
+      <c r="BI7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3611,7 +3634,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BH8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BI8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3776,6 +3799,9 @@
       <c r="BH8" t="n">
         <v>6</v>
       </c>
+      <c r="BI8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3789,7 +3815,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BH9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BI9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -3949,6 +3975,9 @@
         <v>6</v>
       </c>
       <c r="BH9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BI9" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3964,7 +3993,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BH10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BI10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4136,6 +4165,9 @@
         <v>0</v>
       </c>
       <c r="BH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4151,7 +4183,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BH11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BI11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4300,6 +4332,9 @@
       <c r="BH11" t="n">
         <v>6</v>
       </c>
+      <c r="BI11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4313,7 +4348,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BH12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BI12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4451,6 +4486,9 @@
       <c r="BH12" t="n">
         <v>0</v>
       </c>
+      <c r="BI12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4464,7 +4502,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BH13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BI13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -4629,6 +4667,9 @@
       <c r="BH13" t="n">
         <v>0</v>
       </c>
+      <c r="BI13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4642,7 +4683,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BH14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BI14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -4816,6 +4857,9 @@
       <c r="BH14" t="n">
         <v>0</v>
       </c>
+      <c r="BI14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4829,7 +4873,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BH15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BI15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5003,6 +5047,9 @@
       <c r="BH15" t="n">
         <v>0</v>
       </c>
+      <c r="BI15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5016,7 +5063,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BH16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BI16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5190,6 +5237,9 @@
       <c r="BH16" t="n">
         <v>6</v>
       </c>
+      <c r="BI16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5203,7 +5253,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BH17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BI17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5357,6 +5407,9 @@
       <c r="BH17" t="n">
         <v>0</v>
       </c>
+      <c r="BI17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5370,7 +5423,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BH18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BI18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5535,6 +5588,9 @@
       <c r="BH18" t="n">
         <v>6</v>
       </c>
+      <c r="BI18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5548,7 +5604,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BH19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BI19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -5675,6 +5731,9 @@
       <c r="BH19" t="n">
         <v>0</v>
       </c>
+      <c r="BI19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5688,7 +5747,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BH20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BI20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -5809,6 +5868,9 @@
       <c r="BH20" t="n">
         <v>3</v>
       </c>
+      <c r="BI20" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5822,7 +5884,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BH21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BI21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -5940,6 +6002,9 @@
       <c r="BH21" t="n">
         <v>0</v>
       </c>
+      <c r="BI21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -5953,7 +6018,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BH22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BI22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6065,6 +6130,9 @@
       <c r="BH22" t="n">
         <v>6</v>
       </c>
+      <c r="BI22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6078,7 +6146,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BH23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BI23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6181,6 +6249,9 @@
       <c r="BH23" t="n">
         <v>0</v>
       </c>
+      <c r="BI23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6194,7 +6265,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BH24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BI24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6297,6 +6368,9 @@
       <c r="BH24" t="n">
         <v>0</v>
       </c>
+      <c r="BI24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6310,7 +6384,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BH25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BI25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6413,6 +6487,9 @@
       <c r="BH25" t="n">
         <v>0</v>
       </c>
+      <c r="BI25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6426,7 +6503,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BH26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BI26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6478,6 +6555,9 @@
       <c r="BH26" t="n">
         <v>0</v>
       </c>
+      <c r="BI26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6491,7 +6571,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BH27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BI27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6508,6 +6588,9 @@
         <v>0</v>
       </c>
       <c r="BH27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-07-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ27"/>
+  <dimension ref="A1:BK27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2611,6 +2611,11 @@
           <t>24/07/2026</t>
         </is>
       </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2624,7 +2629,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BJ2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BK2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2781,6 +2786,9 @@
         <v>0</v>
       </c>
       <c r="BJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2796,7 +2804,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BJ3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BK3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -2944,6 +2952,9 @@
       <c r="BJ3" t="n">
         <v>4</v>
       </c>
+      <c r="BK3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -2957,7 +2968,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BJ4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BK4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3136,6 +3147,9 @@
       </c>
       <c r="BJ4" t="n">
         <v>0</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -3150,7 +3164,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BJ5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BK5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3330,6 +3344,9 @@
       <c r="BJ5" t="n">
         <v>0</v>
       </c>
+      <c r="BK5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3343,7 +3360,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BJ6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BK6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3493,6 +3510,9 @@
       <c r="BJ6" t="n">
         <v>0</v>
       </c>
+      <c r="BK6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3506,7 +3526,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BJ7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BK7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3644,6 +3664,9 @@
       <c r="BJ7" t="n">
         <v>0</v>
       </c>
+      <c r="BK7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3657,7 +3680,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BJ8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BK8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3828,6 +3851,9 @@
       <c r="BJ8" t="n">
         <v>6</v>
       </c>
+      <c r="BK8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3841,7 +3867,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BJ9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BK9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4007,6 +4033,9 @@
         <v>6</v>
       </c>
       <c r="BJ9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BK9" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4022,7 +4051,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BJ10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BK10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4201,6 +4230,9 @@
       </c>
       <c r="BJ10" t="n">
         <v>0</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4215,7 +4247,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BJ11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BK11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4370,6 +4402,9 @@
       <c r="BJ11" t="n">
         <v>6</v>
       </c>
+      <c r="BK11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4383,7 +4418,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BJ12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BK12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4527,6 +4562,9 @@
       <c r="BJ12" t="n">
         <v>0</v>
       </c>
+      <c r="BK12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4540,7 +4578,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BJ13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BK13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -4711,6 +4749,9 @@
       <c r="BJ13" t="n">
         <v>0</v>
       </c>
+      <c r="BK13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4724,7 +4765,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BJ14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BK14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -4904,6 +4945,9 @@
       <c r="BJ14" t="n">
         <v>0</v>
       </c>
+      <c r="BK14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4917,7 +4961,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BJ15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BK15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5097,6 +5141,9 @@
       <c r="BJ15" t="n">
         <v>0</v>
       </c>
+      <c r="BK15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5110,7 +5157,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BJ16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BK16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5290,6 +5337,9 @@
       <c r="BJ16" t="n">
         <v>6</v>
       </c>
+      <c r="BK16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5303,7 +5353,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BJ17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BK17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5463,6 +5513,9 @@
       <c r="BJ17" t="n">
         <v>0</v>
       </c>
+      <c r="BK17" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5476,7 +5529,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BJ18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BK18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5647,6 +5700,9 @@
       <c r="BJ18" t="n">
         <v>6</v>
       </c>
+      <c r="BK18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5660,7 +5716,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BJ19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BK19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -5793,6 +5849,9 @@
       <c r="BJ19" t="n">
         <v>0</v>
       </c>
+      <c r="BK19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5806,7 +5865,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BJ20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BK20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -5933,6 +5992,9 @@
       <c r="BJ20" t="n">
         <v>3</v>
       </c>
+      <c r="BK20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -5946,7 +6008,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BJ21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BK21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6070,6 +6132,9 @@
       <c r="BJ21" t="n">
         <v>0</v>
       </c>
+      <c r="BK21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6083,7 +6148,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BJ22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BK22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6201,6 +6266,9 @@
       <c r="BJ22" t="n">
         <v>6</v>
       </c>
+      <c r="BK22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6214,7 +6282,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BJ23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BK23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6323,6 +6391,9 @@
       <c r="BJ23" t="n">
         <v>0</v>
       </c>
+      <c r="BK23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6336,7 +6407,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BJ24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BK24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6445,6 +6516,9 @@
       <c r="BJ24" t="n">
         <v>0</v>
       </c>
+      <c r="BK24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6458,7 +6532,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BJ25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BK25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6567,6 +6641,9 @@
       <c r="BJ25" t="n">
         <v>0</v>
       </c>
+      <c r="BK25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6580,7 +6657,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BJ26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BK26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6638,6 +6715,9 @@
       <c r="BJ26" t="n">
         <v>0</v>
       </c>
+      <c r="BK26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6651,7 +6731,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BJ27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BK27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6674,6 +6754,9 @@
         <v>0</v>
       </c>
       <c r="BJ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-27
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -997,7 +997,7 @@
         <v/>
       </c>
       <c r="E3" s="14" t="n">
-        <v>94050</v>
+        <v>94200</v>
       </c>
       <c r="F3" s="13" t="n">
         <v>4000</v>
@@ -1024,7 +1024,7 @@
         <v>10000</v>
       </c>
       <c r="N3" s="13" t="n">
-        <v>5800</v>
+        <v>5950</v>
       </c>
       <c r="O3" s="13" t="n"/>
       <c r="P3" s="13" t="n"/>
@@ -1267,7 +1267,7 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>104050</v>
+        <v>104850</v>
       </c>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
@@ -1286,7 +1286,7 @@
         <v>5550</v>
       </c>
       <c r="N8" s="13" t="n">
-        <v>4550</v>
+        <v>5350</v>
       </c>
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="n"/>
@@ -1543,7 +1543,7 @@
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>48100</v>
+        <v>49900</v>
       </c>
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n"/>
@@ -1566,7 +1566,7 @@
         <v>4300</v>
       </c>
       <c r="N13" s="13" t="n">
-        <v>2400</v>
+        <v>4200</v>
       </c>
       <c r="O13" s="13" t="n"/>
       <c r="P13" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-07-28
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>50400</v>
+        <v>50600</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>4000</v>
@@ -1624,7 +1624,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="13" t="n">
-        <v>1150</v>
+        <v>1350</v>
       </c>
       <c r="O14" s="13" t="n"/>
       <c r="P14" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-01
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK27"/>
+  <dimension ref="A1:BL27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2616,6 +2616,11 @@
           <t>24/07/2026</t>
         </is>
       </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2629,7 +2634,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BK2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BL2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2789,6 +2794,9 @@
         <v>0</v>
       </c>
       <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2804,7 +2812,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BK3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BL3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -2955,6 +2963,9 @@
       <c r="BK3" t="n">
         <v>6</v>
       </c>
+      <c r="BL3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -2968,7 +2979,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BK4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BL4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3150,6 +3161,9 @@
       </c>
       <c r="BK4" t="n">
         <v>6</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3164,7 +3178,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BK5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BL5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3347,6 +3361,9 @@
       <c r="BK5" t="n">
         <v>0</v>
       </c>
+      <c r="BL5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3360,7 +3377,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BK6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BL6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3513,6 +3530,9 @@
       <c r="BK6" t="n">
         <v>0</v>
       </c>
+      <c r="BL6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3526,7 +3546,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BK7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BL7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3667,6 +3687,9 @@
       <c r="BK7" t="n">
         <v>0</v>
       </c>
+      <c r="BL7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3680,7 +3703,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BK8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BL8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3854,6 +3877,9 @@
       <c r="BK8" t="n">
         <v>6</v>
       </c>
+      <c r="BL8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3867,7 +3893,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BK9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BL9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4036,6 +4062,9 @@
         <v>6</v>
       </c>
       <c r="BK9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BL9" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4051,7 +4080,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BK10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BL10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4233,6 +4262,9 @@
       </c>
       <c r="BK10" t="n">
         <v>6</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4247,7 +4279,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BK11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BL11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4405,6 +4437,9 @@
       <c r="BK11" t="n">
         <v>6</v>
       </c>
+      <c r="BL11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4418,7 +4453,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BK12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BL12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4565,6 +4600,9 @@
       <c r="BK12" t="n">
         <v>6</v>
       </c>
+      <c r="BL12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4578,7 +4616,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BK13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BL13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -4752,6 +4790,9 @@
       <c r="BK13" t="n">
         <v>0</v>
       </c>
+      <c r="BL13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4765,7 +4806,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BK14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BL14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -4948,6 +4989,9 @@
       <c r="BK14" t="n">
         <v>0</v>
       </c>
+      <c r="BL14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -4961,7 +5005,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BK15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BL15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5144,6 +5188,9 @@
       <c r="BK15" t="n">
         <v>0</v>
       </c>
+      <c r="BL15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5157,7 +5204,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BK16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BL16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5340,6 +5387,9 @@
       <c r="BK16" t="n">
         <v>6</v>
       </c>
+      <c r="BL16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5353,7 +5403,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BK17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BL17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5516,6 +5566,9 @@
       <c r="BK17" t="n">
         <v>3</v>
       </c>
+      <c r="BL17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5529,7 +5582,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BK18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BL18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5703,6 +5756,9 @@
       <c r="BK18" t="n">
         <v>6</v>
       </c>
+      <c r="BL18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5716,7 +5772,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BK19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BL19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -5852,6 +5908,9 @@
       <c r="BK19" t="n">
         <v>0</v>
       </c>
+      <c r="BL19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5865,7 +5924,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BK20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BL20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -5995,6 +6054,9 @@
       <c r="BK20" t="n">
         <v>6</v>
       </c>
+      <c r="BL20" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6008,7 +6070,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BK21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BL21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6135,6 +6197,9 @@
       <c r="BK21" t="n">
         <v>6</v>
       </c>
+      <c r="BL21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6148,7 +6213,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BK22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BL22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6269,6 +6334,9 @@
       <c r="BK22" t="n">
         <v>6</v>
       </c>
+      <c r="BL22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6282,7 +6350,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BK23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BL23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6394,6 +6462,9 @@
       <c r="BK23" t="n">
         <v>6</v>
       </c>
+      <c r="BL23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6407,7 +6478,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BK24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BL24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6519,6 +6590,9 @@
       <c r="BK24" t="n">
         <v>0</v>
       </c>
+      <c r="BL24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6532,7 +6606,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BK25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BL25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6644,6 +6718,9 @@
       <c r="BK25" t="n">
         <v>0</v>
       </c>
+      <c r="BL25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6657,7 +6734,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BK26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BL26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6718,6 +6795,9 @@
       <c r="BK26" t="n">
         <v>0</v>
       </c>
+      <c r="BL26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6731,7 +6811,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BK27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BL27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6757,6 +6837,9 @@
         <v>0</v>
       </c>
       <c r="BK27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-02
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM27"/>
+  <dimension ref="A1:BN27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2626,6 +2626,11 @@
           <t>31/07/2026</t>
         </is>
       </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2639,7 +2644,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BM2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BN2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2805,6 +2810,9 @@
         <v>0</v>
       </c>
       <c r="BM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2820,7 +2828,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BM3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BN3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -2977,6 +2985,9 @@
       <c r="BM3" t="n">
         <v>0</v>
       </c>
+      <c r="BN3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -2990,7 +3001,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BM4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BN4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3177,6 +3188,9 @@
         <v>0</v>
       </c>
       <c r="BM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3192,7 +3206,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BM5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BN5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3381,6 +3395,9 @@
       <c r="BM5" t="n">
         <v>0</v>
       </c>
+      <c r="BN5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3394,7 +3411,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BM6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BN6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3553,6 +3570,9 @@
       <c r="BM6" t="n">
         <v>0</v>
       </c>
+      <c r="BN6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3566,7 +3586,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BM7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BN7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3713,6 +3733,9 @@
       <c r="BM7" t="n">
         <v>0</v>
       </c>
+      <c r="BN7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3726,7 +3749,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BM8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BN8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3906,6 +3929,9 @@
       <c r="BM8" t="n">
         <v>6</v>
       </c>
+      <c r="BN8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3919,7 +3945,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BM9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BN9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4094,6 +4120,9 @@
         <v>6</v>
       </c>
       <c r="BM9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BN9" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4109,7 +4138,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BM10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BN10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4296,6 +4325,9 @@
         <v>0</v>
       </c>
       <c r="BM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4311,7 +4343,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BM11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BN11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4475,6 +4507,9 @@
       <c r="BM11" t="n">
         <v>0</v>
       </c>
+      <c r="BN11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4488,7 +4523,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BM12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BN12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4641,6 +4676,9 @@
       <c r="BM12" t="n">
         <v>6</v>
       </c>
+      <c r="BN12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4654,7 +4692,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BM13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BN13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -4834,6 +4872,9 @@
       <c r="BM13" t="n">
         <v>0</v>
       </c>
+      <c r="BN13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4847,7 +4888,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BM14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BN14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5036,6 +5077,9 @@
       <c r="BM14" t="n">
         <v>0</v>
       </c>
+      <c r="BN14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5049,7 +5093,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BM15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BN15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5238,6 +5282,9 @@
       <c r="BM15" t="n">
         <v>0</v>
       </c>
+      <c r="BN15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5251,7 +5298,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BM16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BN16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5440,6 +5487,9 @@
       <c r="BM16" t="n">
         <v>0</v>
       </c>
+      <c r="BN16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5453,7 +5503,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BM17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BN17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5622,6 +5672,9 @@
       <c r="BM17" t="n">
         <v>0</v>
       </c>
+      <c r="BN17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5635,7 +5688,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BM18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BN18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5815,6 +5868,9 @@
       <c r="BM18" t="n">
         <v>6</v>
       </c>
+      <c r="BN18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5828,7 +5884,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BM19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BN19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -5970,6 +6026,9 @@
       <c r="BM19" t="n">
         <v>0</v>
       </c>
+      <c r="BN19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -5983,7 +6042,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BM20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BN20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6119,6 +6178,9 @@
       <c r="BM20" t="n">
         <v>4</v>
       </c>
+      <c r="BN20" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6132,7 +6194,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BM21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BN21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6265,6 +6327,9 @@
       <c r="BM21" t="n">
         <v>6</v>
       </c>
+      <c r="BN21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6278,7 +6343,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BM22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BN22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6405,6 +6470,9 @@
       <c r="BM22" t="n">
         <v>4</v>
       </c>
+      <c r="BN22" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6418,7 +6486,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BM23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BN23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6536,6 +6604,9 @@
       <c r="BM23" t="n">
         <v>0</v>
       </c>
+      <c r="BN23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6549,7 +6620,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BM24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BN24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6667,6 +6738,9 @@
       <c r="BM24" t="n">
         <v>0</v>
       </c>
+      <c r="BN24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6680,7 +6754,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BM25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BN25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6798,6 +6872,9 @@
       <c r="BM25" t="n">
         <v>0</v>
       </c>
+      <c r="BN25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6811,7 +6888,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BM26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BN26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -6878,6 +6955,9 @@
       <c r="BM26" t="n">
         <v>0</v>
       </c>
+      <c r="BN26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -6891,7 +6971,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BM27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BN27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -6923,6 +7003,9 @@
         <v>0</v>
       </c>
       <c r="BM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-03
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO27"/>
+  <dimension ref="A1:BP27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2636,6 +2636,11 @@
           <t>31/07/2026</t>
         </is>
       </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2649,7 +2654,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BO2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BP2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2821,6 +2826,9 @@
         <v>0</v>
       </c>
       <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2836,7 +2844,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BO3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BP3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -2999,6 +3007,9 @@
       <c r="BO3" t="n">
         <v>3</v>
       </c>
+      <c r="BP3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3012,7 +3023,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BO4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BP4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3206,6 +3217,9 @@
       </c>
       <c r="BO4" t="n">
         <v>0</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -3220,7 +3234,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BO5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BP5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3415,6 +3429,9 @@
       <c r="BO5" t="n">
         <v>0</v>
       </c>
+      <c r="BP5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3428,7 +3445,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BO6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BP6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3593,6 +3610,9 @@
       <c r="BO6" t="n">
         <v>0</v>
       </c>
+      <c r="BP6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3606,7 +3626,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BO7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BP7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3759,6 +3779,9 @@
       <c r="BO7" t="n">
         <v>0</v>
       </c>
+      <c r="BP7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3772,7 +3795,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BO8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BP8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3958,6 +3981,9 @@
       <c r="BO8" t="n">
         <v>6</v>
       </c>
+      <c r="BP8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3971,7 +3997,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BO9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BP9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4152,6 +4178,9 @@
         <v>6</v>
       </c>
       <c r="BO9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BP9" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4167,7 +4196,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BO10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BP10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4361,6 +4390,9 @@
       </c>
       <c r="BO10" t="n">
         <v>0</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4375,7 +4407,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BO11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BP11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4545,6 +4577,9 @@
       <c r="BO11" t="n">
         <v>0</v>
       </c>
+      <c r="BP11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4558,7 +4593,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BO12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BP12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4717,6 +4752,9 @@
       <c r="BO12" t="n">
         <v>6</v>
       </c>
+      <c r="BP12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4730,7 +4768,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BO13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BP13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -4916,6 +4954,9 @@
       <c r="BO13" t="n">
         <v>0</v>
       </c>
+      <c r="BP13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4929,7 +4970,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BO14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BP14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5124,6 +5165,9 @@
       <c r="BO14" t="n">
         <v>3</v>
       </c>
+      <c r="BP14" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5137,7 +5181,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BO15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BP15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5332,6 +5376,9 @@
       <c r="BO15" t="n">
         <v>6</v>
       </c>
+      <c r="BP15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5345,7 +5392,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BO16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BP16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5540,6 +5587,9 @@
       <c r="BO16" t="n">
         <v>0</v>
       </c>
+      <c r="BP16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5553,7 +5603,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BO17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BP17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5728,6 +5778,9 @@
       <c r="BO17" t="n">
         <v>0</v>
       </c>
+      <c r="BP17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5741,7 +5794,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BO18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BP18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5927,6 +5980,9 @@
       <c r="BO18" t="n">
         <v>6</v>
       </c>
+      <c r="BP18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -5940,7 +5996,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BO19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BP19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6088,6 +6144,9 @@
       <c r="BO19" t="n">
         <v>0</v>
       </c>
+      <c r="BP19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6101,7 +6160,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BO20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BP20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6243,6 +6302,9 @@
       <c r="BO20" t="n">
         <v>4</v>
       </c>
+      <c r="BP20" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6256,7 +6318,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BO21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BP21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6395,6 +6457,9 @@
       <c r="BO21" t="n">
         <v>6</v>
       </c>
+      <c r="BP21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6408,7 +6473,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BO22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BP22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6541,6 +6606,9 @@
       <c r="BO22" t="n">
         <v>5</v>
       </c>
+      <c r="BP22" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6554,7 +6622,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BO23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BP23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6678,6 +6746,9 @@
       <c r="BO23" t="n">
         <v>6</v>
       </c>
+      <c r="BP23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6691,7 +6762,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BO24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BP24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6815,6 +6886,9 @@
       <c r="BO24" t="n">
         <v>0</v>
       </c>
+      <c r="BP24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -6828,7 +6902,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BO25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BP25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6952,6 +7026,9 @@
       <c r="BO25" t="n">
         <v>0</v>
       </c>
+      <c r="BP25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -6965,7 +7042,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BO26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BP26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -7038,6 +7115,9 @@
       <c r="BO26" t="n">
         <v>0</v>
       </c>
+      <c r="BP26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
@@ -7051,7 +7131,7 @@
         </is>
       </c>
       <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BO27), 0)</f>
+        <f>ROUND(AVERAGE(D27:BP27), 0)</f>
         <v/>
       </c>
       <c r="K27" s="6" t="n"/>
@@ -7089,6 +7169,9 @@
         <v>0</v>
       </c>
       <c r="BO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-08
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP27"/>
+  <dimension ref="A1:BQ26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2641,6 +2641,11 @@
           <t>31/07/2026</t>
         </is>
       </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2654,7 +2659,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BP2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BQ2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2829,6 +2834,9 @@
         <v>0</v>
       </c>
       <c r="BP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2844,7 +2852,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BP3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BQ3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3010,6 +3018,9 @@
       <c r="BP3" t="n">
         <v>6</v>
       </c>
+      <c r="BQ3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3023,7 +3034,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BP4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BQ4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3220,6 +3231,9 @@
       </c>
       <c r="BP4" t="n">
         <v>6</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3234,7 +3248,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BP5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BQ5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3432,6 +3446,9 @@
       <c r="BP5" t="n">
         <v>0</v>
       </c>
+      <c r="BQ5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3445,7 +3462,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BP6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BQ6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3613,6 +3630,9 @@
       <c r="BP6" t="n">
         <v>0</v>
       </c>
+      <c r="BQ6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3626,7 +3646,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BP7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BQ7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3782,6 +3802,9 @@
       <c r="BP7" t="n">
         <v>0</v>
       </c>
+      <c r="BQ7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3795,7 +3818,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BP8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BQ8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -3984,6 +4007,9 @@
       <c r="BP8" t="n">
         <v>6</v>
       </c>
+      <c r="BQ8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -3997,7 +4023,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BP9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BQ9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4182,6 +4208,9 @@
       </c>
       <c r="BP9" t="n">
         <v>6</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -4196,7 +4225,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BP10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BQ10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4393,6 +4422,9 @@
       </c>
       <c r="BP10" t="n">
         <v>6</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4407,7 +4439,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BP11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BQ11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4580,6 +4612,9 @@
       <c r="BP11" t="n">
         <v>0</v>
       </c>
+      <c r="BQ11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4593,7 +4628,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BP12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BQ12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4755,6 +4790,9 @@
       <c r="BP12" t="n">
         <v>6</v>
       </c>
+      <c r="BQ12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4768,7 +4806,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BP13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BQ13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -4957,6 +4995,9 @@
       <c r="BP13" t="n">
         <v>0</v>
       </c>
+      <c r="BQ13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -4970,7 +5011,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BP14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BQ14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5168,6 +5209,9 @@
       <c r="BP14" t="n">
         <v>3</v>
       </c>
+      <c r="BQ14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5181,7 +5225,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BP15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BQ15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5379,6 +5423,9 @@
       <c r="BP15" t="n">
         <v>6</v>
       </c>
+      <c r="BQ15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5392,7 +5439,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BP16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BQ16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5590,6 +5637,9 @@
       <c r="BP16" t="n">
         <v>0</v>
       </c>
+      <c r="BQ16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5603,7 +5653,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BP17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BQ17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5781,6 +5831,9 @@
       <c r="BP17" t="n">
         <v>0</v>
       </c>
+      <c r="BQ17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5794,7 +5847,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BP18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BQ18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -5983,20 +6036,23 @@
       <c r="BP18" t="n">
         <v>6</v>
       </c>
+      <c r="BQ18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BP19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BQ19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6009,65 +6065,59 @@
       <c r="S19" s="20" t="n"/>
       <c r="T19" s="20" t="n"/>
       <c r="U19" s="20" t="n"/>
-      <c r="W19" t="n">
-        <v>6</v>
-      </c>
-      <c r="X19" t="n">
-        <v>6</v>
-      </c>
       <c r="Y19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA19" t="n">
         <v>6</v>
       </c>
       <c r="AB19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC19" t="n">
         <v>6</v>
       </c>
       <c r="AD19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO19" t="n">
         <v>5</v>
       </c>
-      <c r="AE19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>6</v>
-      </c>
       <c r="AP19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ19" t="n">
         <v>6</v>
@@ -6085,28 +6135,28 @@
         <v>5</v>
       </c>
       <c r="AV19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW19" t="n">
         <v>5</v>
       </c>
-      <c r="AW19" t="n">
-        <v>0</v>
-      </c>
       <c r="AX19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AY19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AZ19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BA19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BC19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BD19" t="n">
         <v>6</v>
@@ -6118,49 +6168,52 @@
         <v>6</v>
       </c>
       <c r="BG19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BH19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BI19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BJ19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BK19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BL19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BM19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BN19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BO19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BP19" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BP20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BQ20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6173,15 +6226,12 @@
       <c r="S20" s="20" t="n"/>
       <c r="T20" s="20" t="n"/>
       <c r="U20" s="20" t="n"/>
-      <c r="Y20" t="n">
-        <v>6</v>
-      </c>
       <c r="Z20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA20" t="n">
         <v>3</v>
       </c>
-      <c r="AA20" t="n">
-        <v>6</v>
-      </c>
       <c r="AB20" t="n">
         <v>6</v>
       </c>
@@ -6207,64 +6257,64 @@
         <v>0</v>
       </c>
       <c r="AJ20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL20" t="n">
         <v>6</v>
       </c>
       <c r="AM20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ20" t="n">
         <v>6</v>
       </c>
       <c r="AR20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AZ20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BA20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BB20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BC20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BD20" t="n">
         <v>6</v>
@@ -6276,49 +6326,52 @@
         <v>6</v>
       </c>
       <c r="BG20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BH20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BI20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BJ20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BK20" t="n">
         <v>6</v>
       </c>
       <c r="BL20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BM20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BN20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BO20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BP20" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BP21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BQ21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6331,12 +6384,6 @@
       <c r="S21" s="20" t="n"/>
       <c r="T21" s="20" t="n"/>
       <c r="U21" s="20" t="n"/>
-      <c r="Z21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>3</v>
-      </c>
       <c r="AB21" t="n">
         <v>6</v>
       </c>
@@ -6356,34 +6403,34 @@
         <v>6</v>
       </c>
       <c r="AH21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL21" t="n">
         <v>6</v>
       </c>
       <c r="AM21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AO21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR21" t="n">
         <v>0</v>
@@ -6398,82 +6445,85 @@
         <v>0</v>
       </c>
       <c r="AV21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AX21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AY21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AZ21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BA21" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BB21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BC21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BD21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF21" t="n">
         <v>6</v>
       </c>
       <c r="BG21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK21" t="n">
         <v>6</v>
       </c>
       <c r="BL21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BM21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BN21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BO21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BP21" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="BQ21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BP22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BQ22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6486,15 +6536,6 @@
       <c r="S22" s="20" t="n"/>
       <c r="T22" s="20" t="n"/>
       <c r="U22" s="20" t="n"/>
-      <c r="AB22" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD22" t="n">
-        <v>6</v>
-      </c>
       <c r="AE22" t="n">
         <v>6</v>
       </c>
@@ -6502,37 +6543,37 @@
         <v>6</v>
       </c>
       <c r="AG22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL22" t="n">
         <v>6</v>
       </c>
       <c r="AM22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AR22" t="n">
         <v>0</v>
@@ -6547,7 +6588,7 @@
         <v>0</v>
       </c>
       <c r="AV22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW22" t="n">
         <v>6</v>
@@ -6571,58 +6612,61 @@
         <v>0</v>
       </c>
       <c r="BD22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BE22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF22" t="n">
         <v>6</v>
       </c>
       <c r="BG22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BH22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BI22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BJ22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BK22" t="n">
         <v>6</v>
       </c>
       <c r="BL22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BM22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BN22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="BO22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BP22" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="BQ22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BP23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BQ23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6636,7 +6680,7 @@
       <c r="T23" s="20" t="n"/>
       <c r="U23" s="20" t="n"/>
       <c r="AE23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF23" t="n">
         <v>6</v>
@@ -6651,13 +6695,13 @@
         <v>0</v>
       </c>
       <c r="AJ23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM23" t="n">
         <v>0</v>
@@ -6690,19 +6734,19 @@
         <v>0</v>
       </c>
       <c r="AW23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB23" t="n">
         <v>0</v>
@@ -6717,7 +6761,7 @@
         <v>0</v>
       </c>
       <c r="BF23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BG23" t="n">
         <v>0</v>
@@ -6732,7 +6776,7 @@
         <v>0</v>
       </c>
       <c r="BK23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BL23" t="n">
         <v>0</v>
@@ -6744,25 +6788,28 @@
         <v>0</v>
       </c>
       <c r="BO23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP23" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="BQ23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BP24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BQ24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -6776,10 +6823,10 @@
       <c r="T24" s="20" t="n"/>
       <c r="U24" s="20" t="n"/>
       <c r="AE24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF24" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG24" t="n">
         <v>0</v>
@@ -6806,28 +6853,28 @@
         <v>0</v>
       </c>
       <c r="AO24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW24" t="n">
         <v>0</v>
@@ -6887,22 +6934,25 @@
         <v>0</v>
       </c>
       <c r="BP24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BP25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BQ25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -6915,57 +6965,6 @@
       <c r="S25" s="20" t="n"/>
       <c r="T25" s="20" t="n"/>
       <c r="U25" s="20" t="n"/>
-      <c r="AE25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU25" t="n">
-        <v>6</v>
-      </c>
       <c r="AV25" t="n">
         <v>6</v>
       </c>
@@ -6982,7 +6981,7 @@
         <v>0</v>
       </c>
       <c r="BA25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB25" t="n">
         <v>0</v>
@@ -6991,13 +6990,13 @@
         <v>0</v>
       </c>
       <c r="BD25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BG25" t="n">
         <v>0</v>
@@ -7027,22 +7026,25 @@
         <v>0</v>
       </c>
       <c r="BP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>25/07/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BP26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BQ26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -7055,39 +7057,6 @@
       <c r="S26" s="20" t="n"/>
       <c r="T26" s="20" t="n"/>
       <c r="U26" s="20" t="n"/>
-      <c r="AV26" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA26" t="n">
-        <v>6</v>
-      </c>
-      <c r="BB26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD26" t="n">
-        <v>6</v>
-      </c>
-      <c r="BE26" t="n">
-        <v>6</v>
-      </c>
-      <c r="BF26" t="n">
-        <v>6</v>
-      </c>
       <c r="BG26" t="n">
         <v>0</v>
       </c>
@@ -7118,60 +7087,7 @@
       <c r="BP26" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>dado</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-      <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BP27), 0)</f>
-        <v/>
-      </c>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="20" t="n"/>
-      <c r="P27" s="20" t="n"/>
-      <c r="Q27" s="20" t="n"/>
-      <c r="R27" s="20" t="n"/>
-      <c r="S27" s="20" t="n"/>
-      <c r="T27" s="20" t="n"/>
-      <c r="U27" s="20" t="n"/>
-      <c r="BG27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP27" t="n">
+      <c r="BQ26" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-09
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR26"/>
+  <dimension ref="A1:BS27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2651,6 +2651,11 @@
           <t>07/08/2026</t>
         </is>
       </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2664,7 +2669,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BR2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BS2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2845,6 +2850,9 @@
         <v>0</v>
       </c>
       <c r="BR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2860,7 +2868,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BR3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BS3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3032,6 +3040,9 @@
       <c r="BR3" t="n">
         <v>6</v>
       </c>
+      <c r="BS3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3045,7 +3056,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BR4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BS4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3247,6 +3258,9 @@
         <v>0</v>
       </c>
       <c r="BR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3262,7 +3276,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BR5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BS5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3466,6 +3480,9 @@
       <c r="BR5" t="n">
         <v>0</v>
       </c>
+      <c r="BS5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3479,7 +3496,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BR6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BS6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3653,6 +3670,9 @@
       <c r="BR6" t="n">
         <v>0</v>
       </c>
+      <c r="BS6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3666,7 +3686,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BR7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BS7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3828,6 +3848,9 @@
       <c r="BR7" t="n">
         <v>0</v>
       </c>
+      <c r="BS7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3841,7 +3864,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BR8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BS8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4036,6 +4059,9 @@
       <c r="BR8" t="n">
         <v>0</v>
       </c>
+      <c r="BS8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4049,7 +4075,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BR9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BS9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4241,6 +4267,9 @@
       <c r="BR9" t="n">
         <v>1</v>
       </c>
+      <c r="BS9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4254,7 +4283,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BR10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BS10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4456,6 +4485,9 @@
         <v>0</v>
       </c>
       <c r="BR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4471,7 +4503,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BR11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BS11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4650,6 +4682,9 @@
       <c r="BR11" t="n">
         <v>6</v>
       </c>
+      <c r="BS11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4663,7 +4698,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BR12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BS12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4831,6 +4866,9 @@
       <c r="BR12" t="n">
         <v>0</v>
       </c>
+      <c r="BS12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4844,7 +4882,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BR13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BS13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -5039,6 +5077,9 @@
       <c r="BR13" t="n">
         <v>0</v>
       </c>
+      <c r="BS13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5052,7 +5093,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BR14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BS14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5256,6 +5297,9 @@
       <c r="BR14" t="n">
         <v>0</v>
       </c>
+      <c r="BS14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5269,7 +5313,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BR15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BS15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5473,6 +5517,9 @@
       <c r="BR15" t="n">
         <v>0</v>
       </c>
+      <c r="BS15" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5486,7 +5533,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BR16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BS16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5690,6 +5737,9 @@
       <c r="BR16" t="n">
         <v>0</v>
       </c>
+      <c r="BS16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5703,7 +5753,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BR17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BS17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5887,6 +5937,9 @@
       <c r="BR17" t="n">
         <v>0</v>
       </c>
+      <c r="BS17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -5900,7 +5953,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BR18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BS18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -6095,6 +6148,9 @@
       <c r="BR18" t="n">
         <v>0</v>
       </c>
+      <c r="BS18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -6108,7 +6164,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BR19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BS19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6259,6 +6315,9 @@
       <c r="BR19" t="n">
         <v>0</v>
       </c>
+      <c r="BS19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6272,7 +6331,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BR20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BS20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6420,6 +6479,9 @@
       <c r="BR20" t="n">
         <v>6</v>
       </c>
+      <c r="BS20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6433,7 +6495,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BR21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BS21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6575,6 +6637,9 @@
       <c r="BR21" t="n">
         <v>0</v>
       </c>
+      <c r="BS21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6588,7 +6653,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BR22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BS22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6721,6 +6786,9 @@
       <c r="BR22" t="n">
         <v>0</v>
       </c>
+      <c r="BS22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6734,7 +6802,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BR23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BS23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -6867,6 +6935,9 @@
       <c r="BR23" t="n">
         <v>0</v>
       </c>
+      <c r="BS23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -6880,7 +6951,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BR24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BS24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7013,6 +7084,9 @@
       <c r="BR24" t="n">
         <v>0</v>
       </c>
+      <c r="BS24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -7026,7 +7100,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BR25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BS25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -7108,6 +7182,9 @@
       <c r="BR25" t="n">
         <v>0</v>
       </c>
+      <c r="BS25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
@@ -7121,7 +7198,7 @@
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BR26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BS26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -7168,6 +7245,38 @@
         <v>0</v>
       </c>
       <c r="BR26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>TinoGiusa</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
+      <c r="C27" s="28">
+        <f>ROUND(AVERAGE(D27:BS27), 0)</f>
+        <v/>
+      </c>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="N27" s="6" t="n"/>
+      <c r="O27" s="20" t="n"/>
+      <c r="P27" s="20" t="n"/>
+      <c r="Q27" s="20" t="n"/>
+      <c r="R27" s="20" t="n"/>
+      <c r="S27" s="20" t="n"/>
+      <c r="T27" s="20" t="n"/>
+      <c r="U27" s="20" t="n"/>
+      <c r="BS27" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-10
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT27"/>
+  <dimension ref="A1:BU26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2661,6 +2661,11 @@
           <t>07/08/2026</t>
         </is>
       </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2674,7 +2679,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BT2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BU2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2861,6 +2866,9 @@
         <v>0</v>
       </c>
       <c r="BT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2876,7 +2884,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BT3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BU3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3054,6 +3062,9 @@
       <c r="BT3" t="n">
         <v>6</v>
       </c>
+      <c r="BU3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3067,7 +3078,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BT4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BU4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3276,6 +3287,9 @@
       </c>
       <c r="BT4" t="n">
         <v>0</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -3290,7 +3304,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BT5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BU5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3500,6 +3514,9 @@
       <c r="BT5" t="n">
         <v>0</v>
       </c>
+      <c r="BU5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3513,7 +3530,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BT6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BU6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3693,6 +3710,9 @@
       <c r="BT6" t="n">
         <v>0</v>
       </c>
+      <c r="BU6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3706,7 +3726,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BT7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BU7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3874,6 +3894,9 @@
       <c r="BT7" t="n">
         <v>0</v>
       </c>
+      <c r="BU7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3887,7 +3910,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BT8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BU8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4088,6 +4111,9 @@
       <c r="BT8" t="n">
         <v>0</v>
       </c>
+      <c r="BU8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4101,7 +4127,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BT9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BU9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4299,6 +4325,9 @@
       <c r="BT9" t="n">
         <v>1</v>
       </c>
+      <c r="BU9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4312,7 +4341,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BT10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BU10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4521,6 +4550,9 @@
       </c>
       <c r="BT10" t="n">
         <v>0</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4535,7 +4567,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BT11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BU11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4720,6 +4752,9 @@
       <c r="BT11" t="n">
         <v>6</v>
       </c>
+      <c r="BU11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4733,7 +4768,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BT12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BU12), 0)</f>
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
@@ -4907,6 +4942,9 @@
       <c r="BT12" t="n">
         <v>1</v>
       </c>
+      <c r="BU12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -4920,7 +4958,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BT13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BU13), 0)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
@@ -5121,6 +5159,9 @@
       <c r="BT13" t="n">
         <v>0</v>
       </c>
+      <c r="BU13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5134,7 +5175,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BT14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BU14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5344,6 +5385,9 @@
       <c r="BT14" t="n">
         <v>0</v>
       </c>
+      <c r="BU14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5357,7 +5401,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BT15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BU15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5567,6 +5611,9 @@
       <c r="BT15" t="n">
         <v>2</v>
       </c>
+      <c r="BU15" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5580,7 +5627,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BT16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BU16), 0)</f>
         <v/>
       </c>
       <c r="D16" s="10" t="n">
@@ -5790,6 +5837,9 @@
       <c r="BT16" t="n">
         <v>0</v>
       </c>
+      <c r="BU16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -5803,7 +5853,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BT17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BU17), 0)</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
@@ -5993,6 +6043,9 @@
       <c r="BT17" t="n">
         <v>0</v>
       </c>
+      <c r="BU17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -6006,7 +6059,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BT18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BU18), 0)</f>
         <v/>
       </c>
       <c r="G18" s="5" t="n">
@@ -6207,6 +6260,9 @@
       <c r="BT18" t="n">
         <v>0</v>
       </c>
+      <c r="BU18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -6220,7 +6276,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BT19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BU19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6377,6 +6433,9 @@
       <c r="BT19" t="n">
         <v>0</v>
       </c>
+      <c r="BU19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6390,7 +6449,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BT20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BU20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6544,6 +6603,9 @@
       <c r="BT20" t="n">
         <v>6</v>
       </c>
+      <c r="BU20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6557,7 +6619,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BT21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BU21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6705,6 +6767,9 @@
       <c r="BT21" t="n">
         <v>0</v>
       </c>
+      <c r="BU21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6718,7 +6783,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BT22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BU22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6857,6 +6922,9 @@
       <c r="BT22" t="n">
         <v>0</v>
       </c>
+      <c r="BU22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -6870,7 +6938,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BT23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BU23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7009,6 +7077,9 @@
       <c r="BT23" t="n">
         <v>0</v>
       </c>
+      <c r="BU23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -7022,7 +7093,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BT24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BU24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7161,6 +7232,9 @@
       <c r="BT24" t="n">
         <v>0</v>
       </c>
+      <c r="BU24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -7174,7 +7248,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BT25), 0)</f>
+        <f>ROUND(AVERAGE(D25:BU25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -7262,20 +7336,23 @@
       <c r="BT25" t="n">
         <v>0</v>
       </c>
+      <c r="BU25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>25/07/2026</t>
+          <t>09/08/2026</t>
         </is>
       </c>
       <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BT26), 0)</f>
+        <f>ROUND(AVERAGE(D26:BU26), 0)</f>
         <v/>
       </c>
       <c r="K26" s="6" t="n"/>
@@ -7288,78 +7365,13 @@
       <c r="S26" s="20" t="n"/>
       <c r="T26" s="20" t="n"/>
       <c r="U26" s="20" t="n"/>
-      <c r="BG26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR26" t="n">
-        <v>0</v>
-      </c>
       <c r="BS26" t="n">
         <v>0</v>
       </c>
       <c r="BT26" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>TinoGiusa</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>09/08/2026</t>
-        </is>
-      </c>
-      <c r="C27" s="28">
-        <f>ROUND(AVERAGE(D27:BT27), 0)</f>
-        <v/>
-      </c>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="20" t="n"/>
-      <c r="P27" s="20" t="n"/>
-      <c r="Q27" s="20" t="n"/>
-      <c r="R27" s="20" t="n"/>
-      <c r="S27" s="20" t="n"/>
-      <c r="T27" s="20" t="n"/>
-      <c r="U27" s="20" t="n"/>
-      <c r="BS27" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT27" t="n">
+      <c r="BU26" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-15
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV26"/>
+  <dimension ref="A1:BW24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2671,6 +2671,11 @@
           <t>07/08/2026</t>
         </is>
       </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2684,7 +2689,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BV2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BW2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2877,6 +2882,9 @@
         <v>0</v>
       </c>
       <c r="BV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2892,7 +2900,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BV3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BW3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3076,6 +3084,9 @@
       <c r="BV3" t="n">
         <v>6</v>
       </c>
+      <c r="BW3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3089,7 +3100,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BV4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BW4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3304,6 +3315,9 @@
       </c>
       <c r="BV4" t="n">
         <v>6</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3318,7 +3332,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BV5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BW5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3534,6 +3548,9 @@
       <c r="BV5" t="n">
         <v>0</v>
       </c>
+      <c r="BW5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3547,7 +3564,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BV6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BW6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3733,6 +3750,9 @@
       <c r="BV6" t="n">
         <v>0</v>
       </c>
+      <c r="BW6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3746,7 +3766,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BV7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BW7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3920,6 +3940,9 @@
       <c r="BV7" t="n">
         <v>0</v>
       </c>
+      <c r="BW7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3933,7 +3956,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BV8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BW8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4140,6 +4163,9 @@
       <c r="BV8" t="n">
         <v>0</v>
       </c>
+      <c r="BW8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4153,7 +4179,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BV9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BW9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4357,6 +4383,9 @@
       <c r="BV9" t="n">
         <v>6</v>
       </c>
+      <c r="BW9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4370,7 +4399,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BV10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BW10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4585,6 +4614,9 @@
       </c>
       <c r="BV10" t="n">
         <v>6</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4599,7 +4631,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BV11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BW11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4790,30 +4822,60 @@
       <c r="BV11" t="n">
         <v>6</v>
       </c>
+      <c r="BW11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BV12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BW12), 0)</f>
         <v/>
       </c>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
-      <c r="N12" s="6" t="n"/>
-      <c r="O12" s="19" t="n"/>
-      <c r="P12" s="19" t="n"/>
-      <c r="Q12" s="19" t="n"/>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O12" t="n">
+        <v>6</v>
+      </c>
+      <c r="P12" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>6</v>
+      </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S12" t="n">
         <v>6</v>
@@ -4828,19 +4890,19 @@
         <v>6</v>
       </c>
       <c r="W12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AA12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB12" t="n">
         <v>6</v>
@@ -4852,19 +4914,19 @@
         <v>6</v>
       </c>
       <c r="AE12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH12" t="n">
         <v>4</v>
       </c>
-      <c r="AF12" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>6</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>0</v>
-      </c>
       <c r="AI12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ12" t="n">
         <v>6</v>
@@ -4876,31 +4938,31 @@
         <v>6</v>
       </c>
       <c r="AM12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AP12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AQ12" t="n">
         <v>6</v>
       </c>
       <c r="AR12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AS12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AT12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AV12" t="n">
         <v>6</v>
@@ -4909,7 +4971,7 @@
         <v>0</v>
       </c>
       <c r="AX12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY12" t="n">
         <v>6</v>
@@ -4927,13 +4989,13 @@
         <v>0</v>
       </c>
       <c r="BD12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BE12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -4948,22 +5010,22 @@
         <v>0</v>
       </c>
       <c r="BK12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BL12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BM12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BN12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BO12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ12" t="n">
         <v>0</v>
@@ -4972,22 +5034,25 @@
         <v>0</v>
       </c>
       <c r="BS12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BT12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BU12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BV12" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -4996,14 +5061,23 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BV13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BW13), 0)</f>
         <v/>
       </c>
+      <c r="D13" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>6</v>
@@ -5012,16 +5086,16 @@
         <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
         <v>6</v>
@@ -5042,25 +5116,25 @@
         <v>6</v>
       </c>
       <c r="U13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X13" t="n">
         <v>6</v>
       </c>
       <c r="Y13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB13" t="n">
         <v>6</v>
@@ -5081,7 +5155,7 @@
         <v>6</v>
       </c>
       <c r="AH13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AI13" t="n">
         <v>6</v>
@@ -5096,31 +5170,31 @@
         <v>6</v>
       </c>
       <c r="AM13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AN13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AO13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AP13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AQ13" t="n">
         <v>6</v>
       </c>
       <c r="AR13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AU13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AV13" t="n">
         <v>6</v>
@@ -5132,10 +5206,10 @@
         <v>0</v>
       </c>
       <c r="AY13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA13" t="n">
         <v>6</v>
@@ -5147,13 +5221,13 @@
         <v>0</v>
       </c>
       <c r="BD13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BG13" t="n">
         <v>0</v>
@@ -5180,10 +5254,10 @@
         <v>0</v>
       </c>
       <c r="BO13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BP13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BQ13" t="n">
         <v>0</v>
@@ -5198,16 +5272,19 @@
         <v>0</v>
       </c>
       <c r="BU13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BV13" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -5216,80 +5293,80 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BV14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BW14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
         <v>6</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>6</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O14" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R14" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S14" t="n">
+        <v>6</v>
+      </c>
+      <c r="T14" t="n">
+        <v>4</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>6</v>
+      </c>
+      <c r="W14" t="n">
+        <v>3</v>
+      </c>
+      <c r="X14" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J14" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>6</v>
-      </c>
-      <c r="P14" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>6</v>
-      </c>
-      <c r="R14" t="n">
-        <v>6</v>
-      </c>
-      <c r="S14" t="n">
-        <v>6</v>
-      </c>
-      <c r="T14" t="n">
-        <v>6</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="n">
-        <v>5</v>
-      </c>
-      <c r="W14" t="n">
-        <v>6</v>
-      </c>
-      <c r="X14" t="n">
-        <v>6</v>
-      </c>
       <c r="Y14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AB14" t="n">
         <v>6</v>
@@ -5298,52 +5375,52 @@
         <v>6</v>
       </c>
       <c r="AD14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG14" t="n">
         <v>6</v>
       </c>
       <c r="AH14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AO14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AP14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AQ14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AR14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT14" t="n">
         <v>6</v>
@@ -5361,28 +5438,28 @@
         <v>0</v>
       </c>
       <c r="AY14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BA14" t="n">
         <v>6</v>
       </c>
       <c r="BB14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BG14" t="n">
         <v>0</v>
@@ -5406,13 +5483,13 @@
         <v>0</v>
       </c>
       <c r="BN14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BO14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BP14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BQ14" t="n">
         <v>0</v>
@@ -5421,22 +5498,25 @@
         <v>0</v>
       </c>
       <c r="BS14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BT14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BU14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="BV14" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -5445,11 +5525,11 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BV15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BW15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>6</v>
@@ -5467,7 +5547,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>6</v>
@@ -5493,23 +5573,23 @@
       <c r="R15" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S15" t="n">
+      <c r="S15" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -5518,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="n">
         <v>6</v>
@@ -5533,7 +5613,7 @@
         <v>0</v>
       </c>
       <c r="AF15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG15" t="n">
         <v>6</v>
@@ -5554,31 +5634,31 @@
         <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO15" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AP15" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AQ15" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AR15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AU15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AV15" t="n">
         <v>6</v>
@@ -5590,43 +5670,43 @@
         <v>0</v>
       </c>
       <c r="AY15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AZ15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BA15" t="n">
         <v>6</v>
       </c>
       <c r="BB15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BE15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BG15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BL15" t="n">
         <v>0</v>
@@ -5635,13 +5715,13 @@
         <v>0</v>
       </c>
       <c r="BN15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BO15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ15" t="n">
         <v>0</v>
@@ -5650,22 +5730,25 @@
         <v>0</v>
       </c>
       <c r="BS15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BT15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BU15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BV15" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -5674,92 +5757,72 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BV16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BW16), 0)</f>
         <v/>
       </c>
-      <c r="D16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J16" s="6" t="n">
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T16" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U16" t="n">
+        <v>6</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
         <v>5</v>
       </c>
-      <c r="K16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N16" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O16" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P16" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q16" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R16" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S16" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T16" t="n">
-        <v>6</v>
-      </c>
-      <c r="U16" t="n">
-        <v>6</v>
-      </c>
-      <c r="V16" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" t="n">
-        <v>0</v>
-      </c>
       <c r="X16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB16" t="n">
         <v>6</v>
       </c>
       <c r="AC16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF16" t="n">
         <v>6</v>
@@ -5789,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="AO16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ16" t="n">
         <v>6</v>
@@ -5804,13 +5867,13 @@
         <v>0</v>
       </c>
       <c r="AT16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -5825,7 +5888,7 @@
         <v>0</v>
       </c>
       <c r="BA16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB16" t="n">
         <v>0</v>
@@ -5834,28 +5897,28 @@
         <v>0</v>
       </c>
       <c r="BD16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF16" t="n">
         <v>6</v>
       </c>
       <c r="BG16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BH16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BI16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BJ16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BK16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BL16" t="n">
         <v>0</v>
@@ -5888,13 +5951,16 @@
         <v>0</v>
       </c>
       <c r="BV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -5903,10 +5969,21 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BV17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BW17), 0)</f>
         <v/>
       </c>
-      <c r="J17" s="6" t="n"/>
+      <c r="G17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K17" s="6" t="n">
         <v>6</v>
       </c>
@@ -5923,7 +6000,7 @@
         <v>6</v>
       </c>
       <c r="P17" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q17" s="20" t="n">
         <v>6</v>
@@ -5937,26 +6014,26 @@
       <c r="T17" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U17" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
       </c>
       <c r="W17" t="n">
+        <v>6</v>
+      </c>
+      <c r="X17" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
         <v>5</v>
       </c>
-      <c r="X17" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>6</v>
-      </c>
       <c r="AA17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB17" t="n">
         <v>6</v>
@@ -5974,22 +6051,22 @@
         <v>6</v>
       </c>
       <c r="AG17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AM17" t="n">
         <v>0</v>
@@ -6004,22 +6081,22 @@
         <v>0</v>
       </c>
       <c r="AQ17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -6052,34 +6129,34 @@
         <v>6</v>
       </c>
       <c r="BG17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BL17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BM17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BN17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BO17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BP17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BQ17" t="n">
         <v>0</v>
@@ -6094,173 +6171,132 @@
         <v>0</v>
       </c>
       <c r="BU17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BV17" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="BW17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BV18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BW18), 0)</f>
         <v/>
       </c>
-      <c r="G18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J18" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K18" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L18" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N18" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P18" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U18" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V18" t="n">
-        <v>0</v>
-      </c>
-      <c r="W18" t="n">
-        <v>6</v>
-      </c>
-      <c r="X18" t="n">
-        <v>2</v>
-      </c>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="N18" s="6" t="n"/>
+      <c r="O18" s="20" t="n"/>
+      <c r="P18" s="20" t="n"/>
+      <c r="Q18" s="20" t="n"/>
+      <c r="R18" s="20" t="n"/>
+      <c r="S18" s="20" t="n"/>
+      <c r="T18" s="20" t="n"/>
+      <c r="U18" s="20" t="n"/>
       <c r="Y18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO18" t="n">
         <v>5</v>
       </c>
-      <c r="AA18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH18" t="n">
+      <c r="AP18" t="n">
         <v>5</v>
       </c>
-      <c r="AI18" t="n">
+      <c r="AQ18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR18" t="n">
         <v>5</v>
       </c>
-      <c r="AJ18" t="n">
+      <c r="AS18" t="n">
         <v>5</v>
       </c>
-      <c r="AK18" t="n">
+      <c r="AT18" t="n">
         <v>5</v>
       </c>
-      <c r="AL18" t="n">
+      <c r="AU18" t="n">
         <v>5</v>
       </c>
-      <c r="AM18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>6</v>
-      </c>
       <c r="AV18" t="n">
         <v>6</v>
       </c>
       <c r="AW18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AX18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AY18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BA18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BC18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BD18" t="n">
         <v>6</v>
@@ -6272,34 +6308,34 @@
         <v>6</v>
       </c>
       <c r="BG18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BH18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BI18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BJ18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BK18" t="n">
         <v>6</v>
       </c>
       <c r="BL18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BM18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BN18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BO18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BP18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BQ18" t="n">
         <v>0</v>
@@ -6318,21 +6354,24 @@
       </c>
       <c r="BV18" t="n">
         <v>6</v>
+      </c>
+      <c r="BW18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BV19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BW19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6345,15 +6384,12 @@
       <c r="S19" s="20" t="n"/>
       <c r="T19" s="20" t="n"/>
       <c r="U19" s="20" t="n"/>
-      <c r="Y19" t="n">
-        <v>6</v>
-      </c>
       <c r="Z19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA19" t="n">
         <v>3</v>
       </c>
-      <c r="AA19" t="n">
-        <v>6</v>
-      </c>
       <c r="AB19" t="n">
         <v>6</v>
       </c>
@@ -6379,64 +6415,64 @@
         <v>0</v>
       </c>
       <c r="AJ19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL19" t="n">
         <v>6</v>
       </c>
       <c r="AM19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ19" t="n">
         <v>6</v>
       </c>
       <c r="AR19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AZ19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BA19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BB19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BC19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BD19" t="n">
         <v>6</v>
@@ -6448,67 +6484,70 @@
         <v>6</v>
       </c>
       <c r="BG19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BH19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BI19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BJ19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BK19" t="n">
         <v>6</v>
       </c>
       <c r="BL19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BM19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BN19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BO19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BP19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BQ19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BR19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BS19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BT19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BU19" t="n">
         <v>6</v>
       </c>
       <c r="BV19" t="n">
         <v>6</v>
+      </c>
+      <c r="BW19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BV20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BW20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6521,12 +6560,6 @@
       <c r="S20" s="20" t="n"/>
       <c r="T20" s="20" t="n"/>
       <c r="U20" s="20" t="n"/>
-      <c r="Z20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>3</v>
-      </c>
       <c r="AB20" t="n">
         <v>6</v>
       </c>
@@ -6546,34 +6579,34 @@
         <v>6</v>
       </c>
       <c r="AH20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL20" t="n">
         <v>6</v>
       </c>
       <c r="AM20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AO20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR20" t="n">
         <v>0</v>
@@ -6588,100 +6621,103 @@
         <v>0</v>
       </c>
       <c r="AV20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AX20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AY20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AZ20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BA20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BB20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BC20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BD20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF20" t="n">
         <v>6</v>
       </c>
       <c r="BG20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK20" t="n">
         <v>6</v>
       </c>
       <c r="BL20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BM20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BN20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BO20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BP20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BQ20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BR20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BS20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BT20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BU20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BV20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW20" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BV21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BW21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6694,15 +6730,6 @@
       <c r="S21" s="20" t="n"/>
       <c r="T21" s="20" t="n"/>
       <c r="U21" s="20" t="n"/>
-      <c r="AB21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>6</v>
-      </c>
       <c r="AE21" t="n">
         <v>6</v>
       </c>
@@ -6710,37 +6737,37 @@
         <v>6</v>
       </c>
       <c r="AG21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AI21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL21" t="n">
         <v>6</v>
       </c>
       <c r="AM21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AN21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AO21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AP21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AR21" t="n">
         <v>0</v>
@@ -6755,7 +6782,7 @@
         <v>0</v>
       </c>
       <c r="AV21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW21" t="n">
         <v>6</v>
@@ -6779,43 +6806,43 @@
         <v>0</v>
       </c>
       <c r="BD21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BE21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF21" t="n">
         <v>6</v>
       </c>
       <c r="BG21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BH21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BI21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BJ21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BK21" t="n">
         <v>6</v>
       </c>
       <c r="BL21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BM21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BN21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="BO21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BP21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BQ21" t="n">
         <v>0</v>
@@ -6833,22 +6860,25 @@
         <v>0</v>
       </c>
       <c r="BV21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BV22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BW22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -6862,7 +6892,7 @@
       <c r="T22" s="20" t="n"/>
       <c r="U22" s="20" t="n"/>
       <c r="AE22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF22" t="n">
         <v>6</v>
@@ -6877,13 +6907,13 @@
         <v>0</v>
       </c>
       <c r="AJ22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM22" t="n">
         <v>0</v>
@@ -6916,19 +6946,19 @@
         <v>0</v>
       </c>
       <c r="AW22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB22" t="n">
         <v>0</v>
@@ -6943,7 +6973,7 @@
         <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BG22" t="n">
         <v>0</v>
@@ -6958,7 +6988,7 @@
         <v>0</v>
       </c>
       <c r="BK22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BL22" t="n">
         <v>0</v>
@@ -6970,10 +7000,10 @@
         <v>0</v>
       </c>
       <c r="BO22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ22" t="n">
         <v>0</v>
@@ -6991,22 +7021,25 @@
         <v>0</v>
       </c>
       <c r="BV22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BV23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BW23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7020,10 +7053,10 @@
       <c r="T23" s="20" t="n"/>
       <c r="U23" s="20" t="n"/>
       <c r="AE23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF23" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG23" t="n">
         <v>0</v>
@@ -7050,28 +7083,28 @@
         <v>0</v>
       </c>
       <c r="AO23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW23" t="n">
         <v>0</v>
@@ -7149,22 +7182,25 @@
         <v>0</v>
       </c>
       <c r="BV23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BV24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BW24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7177,57 +7213,6 @@
       <c r="S24" s="20" t="n"/>
       <c r="T24" s="20" t="n"/>
       <c r="U24" s="20" t="n"/>
-      <c r="AE24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>6</v>
-      </c>
       <c r="AV24" t="n">
         <v>6</v>
       </c>
@@ -7244,7 +7229,7 @@
         <v>0</v>
       </c>
       <c r="BA24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB24" t="n">
         <v>0</v>
@@ -7253,13 +7238,13 @@
         <v>0</v>
       </c>
       <c r="BD24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BG24" t="n">
         <v>0</v>
@@ -7309,149 +7294,7 @@
       <c r="BV24" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="28" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:BV25), 0)</f>
-        <v/>
-      </c>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-      <c r="N25" s="6" t="n"/>
-      <c r="O25" s="20" t="n"/>
-      <c r="P25" s="20" t="n"/>
-      <c r="Q25" s="20" t="n"/>
-      <c r="R25" s="20" t="n"/>
-      <c r="S25" s="20" t="n"/>
-      <c r="T25" s="20" t="n"/>
-      <c r="U25" s="20" t="n"/>
-      <c r="AV25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA25" t="n">
-        <v>6</v>
-      </c>
-      <c r="BB25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD25" t="n">
-        <v>6</v>
-      </c>
-      <c r="BE25" t="n">
-        <v>6</v>
-      </c>
-      <c r="BF25" t="n">
-        <v>6</v>
-      </c>
-      <c r="BG25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV25" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="28" t="inlineStr">
-        <is>
-          <t>TinoGiusa</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>09/08/2026</t>
-        </is>
-      </c>
-      <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:BV26), 0)</f>
-        <v/>
-      </c>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
-      <c r="N26" s="6" t="n"/>
-      <c r="O26" s="20" t="n"/>
-      <c r="P26" s="20" t="n"/>
-      <c r="Q26" s="20" t="n"/>
-      <c r="R26" s="20" t="n"/>
-      <c r="S26" s="20" t="n"/>
-      <c r="T26" s="20" t="n"/>
-      <c r="U26" s="20" t="n"/>
-      <c r="BS26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV26" t="n">
+      <c r="BW24" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-16
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX24"/>
+  <dimension ref="A1:BY24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2681,6 +2681,11 @@
           <t>14/08/2026</t>
         </is>
       </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2694,7 +2699,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BX2), 0)</f>
+        <f>ROUND(AVERAGE(D2:BY2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2893,6 +2898,9 @@
         <v>0</v>
       </c>
       <c r="BX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2908,7 +2916,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BX3), 0)</f>
+        <f>ROUND(AVERAGE(D3:BY3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3098,6 +3106,9 @@
       <c r="BX3" t="n">
         <v>0</v>
       </c>
+      <c r="BY3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3111,7 +3122,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BX4), 0)</f>
+        <f>ROUND(AVERAGE(D4:BY4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3332,6 +3343,9 @@
       </c>
       <c r="BX4" t="n">
         <v>0</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -3346,7 +3360,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BX5), 0)</f>
+        <f>ROUND(AVERAGE(D5:BY5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3568,6 +3582,9 @@
       <c r="BX5" t="n">
         <v>0</v>
       </c>
+      <c r="BY5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3581,7 +3598,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BX6), 0)</f>
+        <f>ROUND(AVERAGE(D6:BY6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3773,6 +3790,9 @@
       <c r="BX6" t="n">
         <v>0</v>
       </c>
+      <c r="BY6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3786,7 +3806,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BX7), 0)</f>
+        <f>ROUND(AVERAGE(D7:BY7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -3966,6 +3986,9 @@
       <c r="BX7" t="n">
         <v>0</v>
       </c>
+      <c r="BY7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -3979,7 +4002,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BX8), 0)</f>
+        <f>ROUND(AVERAGE(D8:BY8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4192,6 +4215,9 @@
       <c r="BX8" t="n">
         <v>0</v>
       </c>
+      <c r="BY8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4205,7 +4231,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BX9), 0)</f>
+        <f>ROUND(AVERAGE(D9:BY9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4415,6 +4441,9 @@
       <c r="BX9" t="n">
         <v>6</v>
       </c>
+      <c r="BY9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4428,7 +4457,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BX10), 0)</f>
+        <f>ROUND(AVERAGE(D10:BY10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4648,6 +4677,9 @@
         <v>0</v>
       </c>
       <c r="BX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4663,7 +4695,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BX11), 0)</f>
+        <f>ROUND(AVERAGE(D11:BY11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4860,6 +4892,9 @@
       <c r="BX11" t="n">
         <v>0</v>
       </c>
+      <c r="BY11" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4873,7 +4908,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BX12), 0)</f>
+        <f>ROUND(AVERAGE(D12:BY12), 0)</f>
         <v/>
       </c>
       <c r="G12" s="5" t="n">
@@ -5086,6 +5121,9 @@
       <c r="BX12" t="n">
         <v>0</v>
       </c>
+      <c r="BY12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -5099,7 +5137,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BX13), 0)</f>
+        <f>ROUND(AVERAGE(D13:BY13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -5321,6 +5359,9 @@
       <c r="BX13" t="n">
         <v>6</v>
       </c>
+      <c r="BY13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5334,7 +5375,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BX14), 0)</f>
+        <f>ROUND(AVERAGE(D14:BY14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5556,6 +5597,9 @@
       <c r="BX14" t="n">
         <v>0</v>
       </c>
+      <c r="BY14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5569,7 +5613,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BX15), 0)</f>
+        <f>ROUND(AVERAGE(D15:BY15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5791,6 +5835,9 @@
       <c r="BX15" t="n">
         <v>0</v>
       </c>
+      <c r="BY15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5804,7 +5851,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BX16), 0)</f>
+        <f>ROUND(AVERAGE(D16:BY16), 0)</f>
         <v/>
       </c>
       <c r="J16" s="6" t="n"/>
@@ -6006,6 +6053,9 @@
       <c r="BX16" t="n">
         <v>0</v>
       </c>
+      <c r="BY16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -6019,7 +6069,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BX17), 0)</f>
+        <f>ROUND(AVERAGE(D17:BY17), 0)</f>
         <v/>
       </c>
       <c r="G17" s="5" t="n">
@@ -6232,6 +6282,9 @@
       <c r="BX17" t="n">
         <v>2</v>
       </c>
+      <c r="BY17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -6245,7 +6298,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BX18), 0)</f>
+        <f>ROUND(AVERAGE(D18:BY18), 0)</f>
         <v/>
       </c>
       <c r="K18" s="6" t="n"/>
@@ -6414,6 +6467,9 @@
       <c r="BX18" t="n">
         <v>3</v>
       </c>
+      <c r="BY18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -6427,7 +6483,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BX19), 0)</f>
+        <f>ROUND(AVERAGE(D19:BY19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6593,6 +6649,9 @@
       <c r="BX19" t="n">
         <v>0</v>
       </c>
+      <c r="BY19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6606,7 +6665,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BX20), 0)</f>
+        <f>ROUND(AVERAGE(D20:BY20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6766,6 +6825,9 @@
       <c r="BX20" t="n">
         <v>6</v>
       </c>
+      <c r="BY20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6779,7 +6841,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BX21), 0)</f>
+        <f>ROUND(AVERAGE(D21:BY21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -6930,6 +6992,9 @@
       <c r="BX21" t="n">
         <v>0</v>
       </c>
+      <c r="BY21" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -6943,7 +7008,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BX22), 0)</f>
+        <f>ROUND(AVERAGE(D22:BY22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -7094,6 +7159,9 @@
       <c r="BX22" t="n">
         <v>0</v>
       </c>
+      <c r="BY22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -7107,7 +7175,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BX23), 0)</f>
+        <f>ROUND(AVERAGE(D23:BY23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7258,6 +7326,9 @@
       <c r="BX23" t="n">
         <v>0</v>
       </c>
+      <c r="BY23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -7271,7 +7342,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BX24), 0)</f>
+        <f>ROUND(AVERAGE(D24:BY24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7369,6 +7440,9 @@
         <v>0</v>
       </c>
       <c r="BX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY24" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-17
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BZ24"/>
+  <dimension ref="A1:CA25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2691,6 +2691,11 @@
           <t>14/08/2026</t>
         </is>
       </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2704,7 +2709,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:BZ2), 0)</f>
+        <f>ROUND(AVERAGE(D2:CA2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2909,6 +2914,9 @@
         <v>0</v>
       </c>
       <c r="BZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2924,7 +2932,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:BZ3), 0)</f>
+        <f>ROUND(AVERAGE(D3:CA3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3120,6 +3128,9 @@
       <c r="BZ3" t="n">
         <v>6</v>
       </c>
+      <c r="CA3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3133,7 +3144,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:BZ4), 0)</f>
+        <f>ROUND(AVERAGE(D4:CA4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3359,6 +3370,9 @@
         <v>6</v>
       </c>
       <c r="BZ4" t="n">
+        <v>6</v>
+      </c>
+      <c r="CA4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3374,7 +3388,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:BZ5), 0)</f>
+        <f>ROUND(AVERAGE(D5:CA5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3602,6 +3616,9 @@
       <c r="BZ5" t="n">
         <v>0</v>
       </c>
+      <c r="CA5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3615,7 +3632,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:BZ6), 0)</f>
+        <f>ROUND(AVERAGE(D6:CA6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3813,6 +3830,9 @@
       <c r="BZ6" t="n">
         <v>0</v>
       </c>
+      <c r="CA6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3826,7 +3846,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:BZ7), 0)</f>
+        <f>ROUND(AVERAGE(D7:CA7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -4012,6 +4032,9 @@
       <c r="BZ7" t="n">
         <v>3</v>
       </c>
+      <c r="CA7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4025,7 +4048,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:BZ8), 0)</f>
+        <f>ROUND(AVERAGE(D8:CA8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4244,6 +4267,9 @@
       <c r="BZ8" t="n">
         <v>0</v>
       </c>
+      <c r="CA8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4257,7 +4283,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:BZ9), 0)</f>
+        <f>ROUND(AVERAGE(D9:CA9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4473,6 +4499,9 @@
       <c r="BZ9" t="n">
         <v>6</v>
       </c>
+      <c r="CA9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4486,7 +4515,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:BZ10), 0)</f>
+        <f>ROUND(AVERAGE(D10:CA10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4713,6 +4742,9 @@
       </c>
       <c r="BZ10" t="n">
         <v>0</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -4727,7 +4759,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:BZ11), 0)</f>
+        <f>ROUND(AVERAGE(D11:CA11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -4930,6 +4962,9 @@
       <c r="BZ11" t="n">
         <v>5</v>
       </c>
+      <c r="CA11" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -4943,7 +4978,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:BZ12), 0)</f>
+        <f>ROUND(AVERAGE(D12:CA12), 0)</f>
         <v/>
       </c>
       <c r="G12" s="5" t="n">
@@ -5162,6 +5197,9 @@
       <c r="BZ12" t="n">
         <v>0</v>
       </c>
+      <c r="CA12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -5175,7 +5213,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:BZ13), 0)</f>
+        <f>ROUND(AVERAGE(D13:CA13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -5403,6 +5441,9 @@
       <c r="BZ13" t="n">
         <v>6</v>
       </c>
+      <c r="CA13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5416,7 +5457,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:BZ14), 0)</f>
+        <f>ROUND(AVERAGE(D14:CA14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5644,6 +5685,9 @@
       <c r="BZ14" t="n">
         <v>0</v>
       </c>
+      <c r="CA14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5657,7 +5701,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:BZ15), 0)</f>
+        <f>ROUND(AVERAGE(D15:CA15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5885,6 +5929,9 @@
       <c r="BZ15" t="n">
         <v>0</v>
       </c>
+      <c r="CA15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5898,7 +5945,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:BZ16), 0)</f>
+        <f>ROUND(AVERAGE(D16:CA16), 0)</f>
         <v/>
       </c>
       <c r="J16" s="6" t="n"/>
@@ -6106,6 +6153,9 @@
       <c r="BZ16" t="n">
         <v>0</v>
       </c>
+      <c r="CA16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -6119,7 +6169,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:BZ17), 0)</f>
+        <f>ROUND(AVERAGE(D17:CA17), 0)</f>
         <v/>
       </c>
       <c r="G17" s="5" t="n">
@@ -6338,6 +6388,9 @@
       <c r="BZ17" t="n">
         <v>6</v>
       </c>
+      <c r="CA17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -6351,7 +6404,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:BZ18), 0)</f>
+        <f>ROUND(AVERAGE(D18:CA18), 0)</f>
         <v/>
       </c>
       <c r="K18" s="6" t="n"/>
@@ -6526,6 +6579,9 @@
       <c r="BZ18" t="n">
         <v>6</v>
       </c>
+      <c r="CA18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -6539,7 +6595,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:BZ19), 0)</f>
+        <f>ROUND(AVERAGE(D19:CA19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6711,6 +6767,9 @@
       <c r="BZ19" t="n">
         <v>0</v>
       </c>
+      <c r="CA19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6724,7 +6783,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:BZ20), 0)</f>
+        <f>ROUND(AVERAGE(D20:CA20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6890,6 +6949,9 @@
       <c r="BZ20" t="n">
         <v>6</v>
       </c>
+      <c r="CA20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -6903,7 +6965,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:BZ21), 0)</f>
+        <f>ROUND(AVERAGE(D21:CA21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -7060,6 +7122,9 @@
       <c r="BZ21" t="n">
         <v>5</v>
       </c>
+      <c r="CA21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -7073,7 +7138,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:BZ22), 0)</f>
+        <f>ROUND(AVERAGE(D22:CA22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -7230,6 +7295,9 @@
       <c r="BZ22" t="n">
         <v>0</v>
       </c>
+      <c r="CA22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -7243,7 +7311,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:BZ23), 0)</f>
+        <f>ROUND(AVERAGE(D23:CA23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7400,6 +7468,9 @@
       <c r="BZ23" t="n">
         <v>0</v>
       </c>
+      <c r="CA23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -7413,7 +7484,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:BZ24), 0)</f>
+        <f>ROUND(AVERAGE(D24:CA24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7517,6 +7588,38 @@
         <v>0</v>
       </c>
       <c r="BZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Floky23</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="28">
+        <f>ROUND(AVERAGE(D25:CA25), 0)</f>
+        <v/>
+      </c>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+      <c r="N25" s="6" t="n"/>
+      <c r="O25" s="20" t="n"/>
+      <c r="P25" s="20" t="n"/>
+      <c r="Q25" s="20" t="n"/>
+      <c r="R25" s="20" t="n"/>
+      <c r="S25" s="20" t="n"/>
+      <c r="T25" s="20" t="n"/>
+      <c r="U25" s="20" t="n"/>
+      <c r="CA25" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-08-21
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH27"/>
+  <dimension ref="A1:AH26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="14.28515625" customWidth="1" style="15" min="1" max="1"/>
@@ -1038,12 +1038,12 @@
     <row r="4" ht="16.5" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C4" s="12">
@@ -1055,24 +1055,30 @@
         <v/>
       </c>
       <c r="E4" s="14" t="n">
-        <v>55850</v>
+        <v>136220</v>
       </c>
       <c r="F4" s="13" t="n"/>
       <c r="G4" s="13" t="n"/>
-      <c r="H4" s="13" t="n"/>
-      <c r="I4" s="13" t="n"/>
-      <c r="J4" s="13" t="n"/>
+      <c r="H4" s="13" t="n">
+        <v>3850</v>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="K4" s="13" t="n">
-        <v>10000</v>
+        <v>8800</v>
       </c>
       <c r="L4" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M4" s="13" t="n">
-        <v>10050</v>
+        <v>0</v>
       </c>
       <c r="N4" s="13" t="n">
-        <v>10100</v>
+        <v>10200</v>
       </c>
       <c r="O4" s="13" t="n"/>
       <c r="P4" s="13" t="n"/>
@@ -1086,7 +1092,7 @@
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
@@ -1103,30 +1109,30 @@
         <v/>
       </c>
       <c r="E5" s="14" t="n">
-        <v>136220</v>
+        <v>84700</v>
       </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
       <c r="H5" s="13" t="n">
-        <v>3850</v>
+        <v>10000</v>
       </c>
       <c r="I5" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="J5" s="13" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>8800</v>
+        <v>8600</v>
       </c>
       <c r="L5" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>0</v>
+        <v>5350</v>
       </c>
       <c r="N5" s="13" t="n">
-        <v>10200</v>
+        <v>800</v>
       </c>
       <c r="O5" s="13" t="n"/>
       <c r="P5" s="13" t="n"/>
@@ -1140,7 +1146,7 @@
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -1157,36 +1163,38 @@
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>84700</v>
+        <v>58450</v>
       </c>
       <c r="F6" s="13" t="n"/>
-      <c r="G6" s="13" t="n"/>
+      <c r="G6" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H6" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>10000</v>
+        <v>4500</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>10000</v>
+        <v>4300</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>8600</v>
+        <v>6300</v>
       </c>
       <c r="L6" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>5350</v>
+        <v>6000</v>
       </c>
       <c r="N6" s="13" t="n">
-        <v>800</v>
+        <v>10200</v>
       </c>
       <c r="O6" s="13" t="n"/>
       <c r="P6" s="13" t="n"/>
       <c r="Q6" s="13" t="n"/>
       <c r="R6" s="13" t="n"/>
-      <c r="S6" s="13" t="n"/>
+      <c r="S6" s="21" t="n"/>
       <c r="T6" s="13" t="n"/>
       <c r="U6" s="13" t="n"/>
       <c r="V6" s="13" t="n"/>
@@ -1194,12 +1202,12 @@
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="C7" s="12">
@@ -1211,32 +1219,26 @@
         <v/>
       </c>
       <c r="E7" s="14" t="n">
-        <v>58450</v>
+        <v>105600</v>
       </c>
       <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H7" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>4500</v>
-      </c>
+      <c r="G7" s="13" t="n"/>
+      <c r="H7" s="13" t="n"/>
+      <c r="I7" s="13" t="n"/>
       <c r="J7" s="13" t="n">
-        <v>4300</v>
+        <v>5000</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>6300</v>
+        <v>6100</v>
       </c>
       <c r="L7" s="13" t="n">
         <v>10000</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>6000</v>
+        <v>5550</v>
       </c>
       <c r="N7" s="13" t="n">
-        <v>10200</v>
+        <v>6100</v>
       </c>
       <c r="O7" s="13" t="n"/>
       <c r="P7" s="13" t="n"/>
@@ -1250,12 +1252,12 @@
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C8" s="12">
@@ -1267,26 +1269,32 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>105600</v>
+        <v>18350</v>
       </c>
       <c r="F8" s="13" t="n"/>
-      <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n"/>
-      <c r="I8" s="13" t="n"/>
+      <c r="G8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="J8" s="13" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="K8" s="13" t="n">
         <v>6100</v>
       </c>
       <c r="L8" s="13" t="n">
-        <v>10000</v>
+        <v>6100</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>5550</v>
+        <v>0</v>
       </c>
       <c r="N8" s="13" t="n">
-        <v>6100</v>
+        <v>0</v>
       </c>
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="n"/>
@@ -1300,7 +1308,7 @@
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
@@ -1317,32 +1325,34 @@
         <v/>
       </c>
       <c r="E9" s="14" t="n">
-        <v>18350</v>
-      </c>
-      <c r="F9" s="13" t="n"/>
+        <v>54050</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>2100</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>0</v>
+        <v>5800</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0</v>
+        <v>4350</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>6100</v>
+        <v>4600</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>6100</v>
+        <v>10000</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>0</v>
+        <v>4100</v>
       </c>
       <c r="N9" s="13" t="n">
-        <v>0</v>
+        <v>4250</v>
       </c>
       <c r="O9" s="13" t="n"/>
       <c r="P9" s="13" t="n"/>
@@ -1356,7 +1366,7 @@
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
@@ -1373,34 +1383,34 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>54050</v>
+        <v>45850</v>
       </c>
       <c r="F10" s="13" t="n">
         <v>4000</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>2100</v>
+        <v>4000</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>5800</v>
+        <v>4100</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>4050</v>
+        <v>4400</v>
       </c>
       <c r="J10" s="13" t="n">
+        <v>4700</v>
+      </c>
+      <c r="K10" s="13" t="n">
+        <v>4150</v>
+      </c>
+      <c r="L10" s="13" t="n">
+        <v>9300</v>
+      </c>
+      <c r="M10" s="13" t="n">
         <v>4350</v>
       </c>
-      <c r="K10" s="13" t="n">
-        <v>4600</v>
-      </c>
-      <c r="L10" s="13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="M10" s="13" t="n">
-        <v>4100</v>
-      </c>
       <c r="N10" s="13" t="n">
-        <v>4250</v>
+        <v>0</v>
       </c>
       <c r="O10" s="13" t="n"/>
       <c r="P10" s="13" t="n"/>
@@ -1414,12 +1424,12 @@
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C11" s="12">
@@ -1431,34 +1441,30 @@
         <v/>
       </c>
       <c r="E11" s="14" t="n">
-        <v>45850</v>
-      </c>
-      <c r="F11" s="13" t="n">
+        <v>145400</v>
+      </c>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>4050</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J11" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="K11" s="13" t="n">
+        <v>4100</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>13400</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>4200</v>
+      </c>
+      <c r="N11" s="13" t="n">
         <v>4000</v>
-      </c>
-      <c r="H11" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I11" s="13" t="n">
-        <v>4400</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>4700</v>
-      </c>
-      <c r="K11" s="13" t="n">
-        <v>4150</v>
-      </c>
-      <c r="L11" s="13" t="n">
-        <v>9300</v>
-      </c>
-      <c r="M11" s="13" t="n">
-        <v>4350</v>
-      </c>
-      <c r="N11" s="13" t="n">
-        <v>0</v>
       </c>
       <c r="O11" s="13" t="n"/>
       <c r="P11" s="13" t="n"/>
@@ -1472,12 +1478,12 @@
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C12" s="12">
@@ -1489,30 +1495,30 @@
         <v/>
       </c>
       <c r="E12" s="14" t="n">
-        <v>145400</v>
+        <v>49900</v>
       </c>
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
       <c r="H12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J12" s="13" t="n">
         <v>4050</v>
       </c>
-      <c r="I12" s="13" t="n">
-        <v>4100</v>
-      </c>
-      <c r="J12" s="13" t="n">
+      <c r="K12" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="K12" s="13" t="n">
-        <v>4100</v>
-      </c>
       <c r="L12" s="13" t="n">
-        <v>13400</v>
+        <v>10000</v>
       </c>
       <c r="M12" s="13" t="n">
+        <v>4300</v>
+      </c>
+      <c r="N12" s="13" t="n">
         <v>4200</v>
-      </c>
-      <c r="N12" s="13" t="n">
-        <v>4000</v>
       </c>
       <c r="O12" s="13" t="n"/>
       <c r="P12" s="13" t="n"/>
@@ -1526,7 +1532,7 @@
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
@@ -1543,30 +1549,34 @@
         <v/>
       </c>
       <c r="E13" s="14" t="n">
-        <v>49900</v>
-      </c>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
+        <v>50600</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>4000</v>
+      </c>
       <c r="H13" s="13" t="n">
-        <v>0</v>
+        <v>4050</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>3500</v>
+        <v>5600</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>4050</v>
+        <v>1300</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>4000</v>
+        <v>3100</v>
       </c>
       <c r="L13" s="13" t="n">
-        <v>10000</v>
+        <v>9350</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>4300</v>
+        <v>0</v>
       </c>
       <c r="N13" s="13" t="n">
-        <v>4200</v>
+        <v>1350</v>
       </c>
       <c r="O13" s="13" t="n"/>
       <c r="P13" s="13" t="n"/>
@@ -1580,7 +1590,7 @@
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
@@ -1597,34 +1607,30 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>50600</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G14" s="13" t="n">
-        <v>4000</v>
-      </c>
+        <v>50875</v>
+      </c>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
       <c r="H14" s="13" t="n">
-        <v>4050</v>
+        <v>3650</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>5600</v>
+        <v>7600</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>1300</v>
+        <v>3150</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>3100</v>
+        <v>3000</v>
       </c>
       <c r="L14" s="13" t="n">
-        <v>9350</v>
+        <v>10000</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>0</v>
+        <v>2550</v>
       </c>
       <c r="N14" s="13" t="n">
-        <v>1350</v>
+        <v>4100</v>
       </c>
       <c r="O14" s="13" t="n"/>
       <c r="P14" s="13" t="n"/>
@@ -1638,12 +1644,12 @@
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C15" s="12">
@@ -1655,30 +1661,28 @@
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>50875</v>
+        <v>82800</v>
       </c>
       <c r="F15" s="13" t="n"/>
       <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n">
-        <v>3650</v>
-      </c>
+      <c r="H15" s="13" t="n"/>
       <c r="I15" s="13" t="n">
-        <v>7600</v>
+        <v>0</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>3150</v>
+        <v>950</v>
       </c>
       <c r="K15" s="13" t="n">
-        <v>3000</v>
+        <v>1400</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>10000</v>
+        <v>2200</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>2550</v>
+        <v>0</v>
       </c>
       <c r="N15" s="13" t="n">
-        <v>4100</v>
+        <v>5600</v>
       </c>
       <c r="O15" s="13" t="n"/>
       <c r="P15" s="13" t="n"/>
@@ -1692,12 +1696,12 @@
     <row r="16" ht="16.5" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>655321</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>16/01/2026</t>
         </is>
       </c>
       <c r="C16" s="12">
@@ -1709,34 +1713,34 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>82800</v>
+        <v>8750</v>
       </c>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="13" t="n">
-        <v>0</v>
+        <v>4150</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>950</v>
+        <v>2650</v>
       </c>
       <c r="K16" s="13" t="n">
-        <v>1400</v>
+        <v>1050</v>
       </c>
       <c r="L16" s="13" t="n">
-        <v>2200</v>
+        <v>1050</v>
       </c>
       <c r="M16" s="13" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="N16" s="13" t="n">
-        <v>5600</v>
+        <v>0</v>
       </c>
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="13" t="n"/>
       <c r="Q16" s="13" t="n"/>
       <c r="R16" s="13" t="n"/>
-      <c r="S16" s="21" t="n"/>
+      <c r="S16" s="13" t="n"/>
       <c r="T16" s="13" t="n"/>
       <c r="U16" s="13" t="n"/>
       <c r="V16" s="13" t="n"/>
@@ -1744,12 +1748,12 @@
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="C17" s="12">
@@ -1761,28 +1765,24 @@
         <v/>
       </c>
       <c r="E17" s="14" t="n">
-        <v>8750</v>
+        <v>23300</v>
       </c>
       <c r="F17" s="13" t="n"/>
       <c r="G17" s="13" t="n"/>
       <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n">
-        <v>4150</v>
-      </c>
-      <c r="J17" s="13" t="n">
-        <v>2650</v>
-      </c>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
       <c r="K17" s="13" t="n">
-        <v>1050</v>
+        <v>600</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>900</v>
+        <v>2050</v>
       </c>
       <c r="N17" s="13" t="n">
-        <v>0</v>
+        <v>2150</v>
       </c>
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="13" t="n"/>
@@ -1796,12 +1796,12 @@
     <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C18" s="12">
@@ -1813,24 +1813,22 @@
         <v/>
       </c>
       <c r="E18" s="14" t="n">
-        <v>23300</v>
+        <v>11750</v>
       </c>
       <c r="F18" s="13" t="n"/>
       <c r="G18" s="13" t="n"/>
       <c r="H18" s="13" t="n"/>
       <c r="I18" s="13" t="n"/>
       <c r="J18" s="13" t="n"/>
-      <c r="K18" s="13" t="n">
-        <v>600</v>
-      </c>
+      <c r="K18" s="13" t="n"/>
       <c r="L18" s="13" t="n">
-        <v>1100</v>
+        <v>300</v>
       </c>
       <c r="M18" s="13" t="n">
-        <v>2050</v>
+        <v>0</v>
       </c>
       <c r="N18" s="13" t="n">
-        <v>2150</v>
+        <v>200</v>
       </c>
       <c r="O18" s="13" t="n"/>
       <c r="P18" s="13" t="n"/>
@@ -1844,7 +1842,7 @@
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
@@ -1861,7 +1859,7 @@
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>11750</v>
+        <v>61390</v>
       </c>
       <c r="F19" s="13" t="n"/>
       <c r="G19" s="13" t="n"/>
@@ -1870,13 +1868,13 @@
       <c r="J19" s="13" t="n"/>
       <c r="K19" s="13" t="n"/>
       <c r="L19" s="13" t="n">
-        <v>300</v>
+        <v>10650</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>0</v>
+        <v>4100</v>
       </c>
       <c r="N19" s="13" t="n">
-        <v>200</v>
+        <v>6000</v>
       </c>
       <c r="O19" s="13" t="n"/>
       <c r="P19" s="13" t="n"/>
@@ -1890,12 +1888,12 @@
     <row r="20" ht="16.5" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C20" s="12">
@@ -1907,7 +1905,7 @@
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>61390</v>
+        <v>68700</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
@@ -1916,13 +1914,13 @@
       <c r="J20" s="13" t="n"/>
       <c r="K20" s="13" t="n"/>
       <c r="L20" s="13" t="n">
-        <v>10650</v>
+        <v>4400</v>
       </c>
       <c r="M20" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="N20" s="13" t="n">
         <v>4100</v>
-      </c>
-      <c r="N20" s="13" t="n">
-        <v>6000</v>
       </c>
       <c r="O20" s="13" t="n"/>
       <c r="P20" s="13" t="n"/>
@@ -1936,7 +1934,7 @@
     <row r="21" ht="16.5" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
@@ -1953,7 +1951,7 @@
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>68700</v>
+        <v>50800</v>
       </c>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
@@ -1962,13 +1960,13 @@
       <c r="J21" s="13" t="n"/>
       <c r="K21" s="13" t="n"/>
       <c r="L21" s="13" t="n">
-        <v>4400</v>
+        <v>4500</v>
       </c>
       <c r="M21" s="13" t="n">
-        <v>4000</v>
+        <v>4100</v>
       </c>
       <c r="N21" s="13" t="n">
-        <v>4100</v>
+        <v>2550</v>
       </c>
       <c r="O21" s="13" t="n"/>
       <c r="P21" s="13" t="n"/>
@@ -1982,7 +1980,7 @@
     <row r="22" ht="16.5" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B22" s="16" t="inlineStr">
@@ -1999,7 +1997,7 @@
         <v/>
       </c>
       <c r="E22" s="14" t="n">
-        <v>50800</v>
+        <v>122475</v>
       </c>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="n"/>
@@ -2008,13 +2006,13 @@
       <c r="J22" s="13" t="n"/>
       <c r="K22" s="13" t="n"/>
       <c r="L22" s="13" t="n">
-        <v>4500</v>
+        <v>4100</v>
       </c>
       <c r="M22" s="13" t="n">
-        <v>4100</v>
+        <v>4050</v>
       </c>
       <c r="N22" s="13" t="n">
-        <v>2550</v>
+        <v>4000</v>
       </c>
       <c r="O22" s="13" t="n"/>
       <c r="P22" s="13" t="n"/>
@@ -2028,12 +2026,12 @@
     <row r="23" ht="16.5" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="C23" s="12">
@@ -2045,7 +2043,7 @@
         <v/>
       </c>
       <c r="E23" s="14" t="n">
-        <v>122475</v>
+        <v>120100</v>
       </c>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
@@ -2054,13 +2052,13 @@
       <c r="J23" s="13" t="n"/>
       <c r="K23" s="13" t="n"/>
       <c r="L23" s="13" t="n">
-        <v>4100</v>
+        <v>9500</v>
       </c>
       <c r="M23" s="13" t="n">
-        <v>4050</v>
+        <v>10100</v>
       </c>
       <c r="N23" s="13" t="n">
-        <v>4000</v>
+        <v>10100</v>
       </c>
       <c r="O23" s="13" t="n"/>
       <c r="P23" s="13" t="n"/>
@@ -2074,12 +2072,12 @@
     <row r="24" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C24" s="12">
@@ -2091,7 +2089,7 @@
         <v/>
       </c>
       <c r="E24" s="14" t="n">
-        <v>120100</v>
+        <v>14750</v>
       </c>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
@@ -2099,14 +2097,12 @@
       <c r="I24" s="13" t="n"/>
       <c r="J24" s="13" t="n"/>
       <c r="K24" s="13" t="n"/>
-      <c r="L24" s="13" t="n">
-        <v>9500</v>
-      </c>
+      <c r="L24" s="13" t="n"/>
       <c r="M24" s="13" t="n">
-        <v>10100</v>
+        <v>1500</v>
       </c>
       <c r="N24" s="13" t="n">
-        <v>10100</v>
+        <v>0</v>
       </c>
       <c r="O24" s="13" t="n"/>
       <c r="P24" s="13" t="n"/>
@@ -2120,7 +2116,7 @@
     <row r="25" ht="16.5" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
@@ -2137,7 +2133,7 @@
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>14750</v>
+        <v>156740</v>
       </c>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
@@ -2147,7 +2143,7 @@
       <c r="K25" s="13" t="n"/>
       <c r="L25" s="13" t="n"/>
       <c r="M25" s="13" t="n">
-        <v>1500</v>
+        <v>6300</v>
       </c>
       <c r="N25" s="13" t="n">
         <v>0</v>
@@ -2164,12 +2160,12 @@
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>21/06/2026</t>
+          <t>21/08/2026</t>
         </is>
       </c>
       <c r="C26" s="12">
@@ -2181,7 +2177,7 @@
         <v/>
       </c>
       <c r="E26" s="14" t="n">
-        <v>156740</v>
+        <v>54800</v>
       </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
@@ -2190,12 +2186,8 @@
       <c r="J26" s="13" t="n"/>
       <c r="K26" s="13" t="n"/>
       <c r="L26" s="13" t="n"/>
-      <c r="M26" s="13" t="n">
-        <v>6300</v>
-      </c>
-      <c r="N26" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="M26" s="13" t="n"/>
+      <c r="N26" s="13" t="n"/>
       <c r="O26" s="13" t="n"/>
       <c r="P26" s="13" t="n"/>
       <c r="Q26" s="13" t="n"/>
@@ -2205,48 +2197,7 @@
       <c r="U26" s="13" t="n"/>
       <c r="V26" s="13" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>dado</t>
-        </is>
-      </c>
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>22/07/2026</t>
-        </is>
-      </c>
-      <c r="C27" s="12">
-        <f>ROUND(AVERAGE(F27:AI27), 0)</f>
-        <v/>
-      </c>
-      <c r="D27" s="1">
-        <f>SUM(F27:AI27)</f>
-        <v/>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>47650</v>
-      </c>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="n"/>
-      <c r="L27" s="13" t="n"/>
-      <c r="M27" s="13" t="n"/>
-      <c r="N27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="13" t="n"/>
-      <c r="P27" s="13" t="n"/>
-      <c r="Q27" s="13" t="n"/>
-      <c r="R27" s="13" t="n"/>
-      <c r="S27" s="13" t="n"/>
-      <c r="T27" s="13" t="n"/>
-      <c r="U27" s="13" t="n"/>
-      <c r="V27" s="13" t="n"/>
-    </row>
+    <row r="27" ht="16.5" customHeight="1"/>
     <row r="28" ht="16.5" customHeight="1"/>
     <row r="29" ht="16.5" customHeight="1"/>
     <row r="30" ht="16.5" customHeight="1"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-08-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -976,6 +976,9 @@
       <c r="N2" t="n">
         <v>3550</v>
       </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
@@ -1026,7 +1029,9 @@
       <c r="N3" s="13" t="n">
         <v>10200</v>
       </c>
-      <c r="O3" s="13" t="n"/>
+      <c r="O3" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P3" s="13" t="n"/>
       <c r="Q3" s="13" t="n"/>
       <c r="R3" s="13" t="n"/>
@@ -1080,7 +1085,9 @@
       <c r="N4" s="13" t="n">
         <v>10200</v>
       </c>
-      <c r="O4" s="13" t="n"/>
+      <c r="O4" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P4" s="13" t="n"/>
       <c r="Q4" s="13" t="n"/>
       <c r="R4" s="13" t="n"/>
@@ -1134,7 +1141,9 @@
       <c r="N5" s="13" t="n">
         <v>800</v>
       </c>
-      <c r="O5" s="13" t="n"/>
+      <c r="O5" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P5" s="13" t="n"/>
       <c r="Q5" s="13" t="n"/>
       <c r="R5" s="13" t="n"/>
@@ -1190,7 +1199,9 @@
       <c r="N6" s="13" t="n">
         <v>10200</v>
       </c>
-      <c r="O6" s="13" t="n"/>
+      <c r="O6" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P6" s="13" t="n"/>
       <c r="Q6" s="13" t="n"/>
       <c r="R6" s="13" t="n"/>
@@ -1240,7 +1251,9 @@
       <c r="N7" s="13" t="n">
         <v>6100</v>
       </c>
-      <c r="O7" s="13" t="n"/>
+      <c r="O7" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P7" s="13" t="n"/>
       <c r="Q7" s="13" t="n"/>
       <c r="R7" s="13" t="n"/>
@@ -1296,7 +1309,9 @@
       <c r="N8" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="13" t="n"/>
+      <c r="O8" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="13" t="n"/>
       <c r="R8" s="13" t="n"/>
@@ -1354,7 +1369,9 @@
       <c r="N9" s="13" t="n">
         <v>4250</v>
       </c>
-      <c r="O9" s="13" t="n"/>
+      <c r="O9" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P9" s="13" t="n"/>
       <c r="Q9" s="13" t="n"/>
       <c r="R9" s="13" t="n"/>
@@ -1412,7 +1429,9 @@
       <c r="N10" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="13" t="n"/>
+      <c r="O10" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P10" s="13" t="n"/>
       <c r="Q10" s="13" t="n"/>
       <c r="R10" s="13" t="n"/>
@@ -1466,7 +1485,9 @@
       <c r="N11" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="O11" s="13" t="n"/>
+      <c r="O11" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P11" s="13" t="n"/>
       <c r="Q11" s="13" t="n"/>
       <c r="R11" s="13" t="n"/>
@@ -1520,7 +1541,9 @@
       <c r="N12" s="13" t="n">
         <v>4200</v>
       </c>
-      <c r="O12" s="13" t="n"/>
+      <c r="O12" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P12" s="13" t="n"/>
       <c r="Q12" s="13" t="n"/>
       <c r="R12" s="13" t="n"/>
@@ -1578,7 +1601,9 @@
       <c r="N13" s="13" t="n">
         <v>1350</v>
       </c>
-      <c r="O13" s="13" t="n"/>
+      <c r="O13" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P13" s="13" t="n"/>
       <c r="Q13" s="13" t="n"/>
       <c r="R13" s="13" t="n"/>
@@ -1632,7 +1657,9 @@
       <c r="N14" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="O14" s="13" t="n"/>
+      <c r="O14" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P14" s="13" t="n"/>
       <c r="Q14" s="13" t="n"/>
       <c r="R14" s="13" t="n"/>
@@ -1684,7 +1711,9 @@
       <c r="N15" s="13" t="n">
         <v>5600</v>
       </c>
-      <c r="O15" s="13" t="n"/>
+      <c r="O15" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P15" s="13" t="n"/>
       <c r="Q15" s="13" t="n"/>
       <c r="R15" s="13" t="n"/>
@@ -1736,7 +1765,9 @@
       <c r="N16" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O16" s="13" t="n"/>
+      <c r="O16" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P16" s="13" t="n"/>
       <c r="Q16" s="13" t="n"/>
       <c r="R16" s="13" t="n"/>
@@ -1784,7 +1815,9 @@
       <c r="N17" s="13" t="n">
         <v>2150</v>
       </c>
-      <c r="O17" s="13" t="n"/>
+      <c r="O17" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P17" s="13" t="n"/>
       <c r="Q17" s="13" t="n"/>
       <c r="R17" s="13" t="n"/>
@@ -1830,7 +1863,9 @@
       <c r="N18" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="O18" s="13" t="n"/>
+      <c r="O18" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P18" s="13" t="n"/>
       <c r="Q18" s="13" t="n"/>
       <c r="R18" s="13" t="n"/>
@@ -1876,7 +1911,9 @@
       <c r="N19" s="13" t="n">
         <v>6000</v>
       </c>
-      <c r="O19" s="13" t="n"/>
+      <c r="O19" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P19" s="13" t="n"/>
       <c r="Q19" s="13" t="n"/>
       <c r="R19" s="13" t="n"/>
@@ -1922,7 +1959,9 @@
       <c r="N20" s="13" t="n">
         <v>4100</v>
       </c>
-      <c r="O20" s="13" t="n"/>
+      <c r="O20" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P20" s="13" t="n"/>
       <c r="Q20" s="13" t="n"/>
       <c r="R20" s="13" t="n"/>
@@ -1968,7 +2007,9 @@
       <c r="N21" s="13" t="n">
         <v>2550</v>
       </c>
-      <c r="O21" s="13" t="n"/>
+      <c r="O21" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P21" s="13" t="n"/>
       <c r="Q21" s="13" t="n"/>
       <c r="R21" s="13" t="n"/>
@@ -2014,7 +2055,9 @@
       <c r="N22" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="O22" s="13" t="n"/>
+      <c r="O22" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P22" s="13" t="n"/>
       <c r="Q22" s="13" t="n"/>
       <c r="R22" s="13" t="n"/>
@@ -2060,7 +2103,9 @@
       <c r="N23" s="13" t="n">
         <v>10100</v>
       </c>
-      <c r="O23" s="13" t="n"/>
+      <c r="O23" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P23" s="13" t="n"/>
       <c r="Q23" s="13" t="n"/>
       <c r="R23" s="13" t="n"/>
@@ -2104,7 +2149,9 @@
       <c r="N24" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O24" s="13" t="n"/>
+      <c r="O24" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P24" s="13" t="n"/>
       <c r="Q24" s="13" t="n"/>
       <c r="R24" s="13" t="n"/>
@@ -2148,7 +2195,9 @@
       <c r="N25" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="O25" s="13" t="n"/>
+      <c r="O25" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P25" s="13" t="n"/>
       <c r="Q25" s="13" t="n"/>
       <c r="R25" s="13" t="n"/>
@@ -2188,7 +2237,9 @@
       <c r="L26" s="13" t="n"/>
       <c r="M26" s="13" t="n"/>
       <c r="N26" s="13" t="n"/>
-      <c r="O26" s="13" t="n"/>
+      <c r="O26" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="P26" s="13" t="n"/>
       <c r="Q26" s="13" t="n"/>
       <c r="R26" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-22
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2286,7 +2286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CB25"/>
+  <dimension ref="A1:CC26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2703,6 +2703,11 @@
           <t>14/08/2026</t>
         </is>
       </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2716,7 +2721,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:CB2), 0)</f>
+        <f>ROUND(AVERAGE(D2:CC2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2927,6 +2932,9 @@
         <v>0</v>
       </c>
       <c r="CB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2942,7 +2950,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:CB3), 0)</f>
+        <f>ROUND(AVERAGE(D3:CC3), 0)</f>
         <v/>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -3144,6 +3152,9 @@
       <c r="CB3" t="n">
         <v>6</v>
       </c>
+      <c r="CC3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -3157,7 +3168,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:CB4), 0)</f>
+        <f>ROUND(AVERAGE(D4:CC4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3390,6 +3401,9 @@
       </c>
       <c r="CB4" t="n">
         <v>6</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3404,7 +3418,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:CB5), 0)</f>
+        <f>ROUND(AVERAGE(D5:CC5), 0)</f>
         <v/>
       </c>
       <c r="D5" s="10" t="n">
@@ -3638,6 +3652,9 @@
       <c r="CB5" t="n">
         <v>0</v>
       </c>
+      <c r="CC5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3651,7 +3668,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:CB6), 0)</f>
+        <f>ROUND(AVERAGE(D6:CC6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3855,6 +3872,9 @@
       <c r="CB6" t="n">
         <v>0</v>
       </c>
+      <c r="CC6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3868,7 +3888,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:CB7), 0)</f>
+        <f>ROUND(AVERAGE(D7:CC7), 0)</f>
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
@@ -4060,6 +4080,9 @@
       <c r="CB7" t="n">
         <v>3</v>
       </c>
+      <c r="CC7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4073,7 +4096,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:CB8), 0)</f>
+        <f>ROUND(AVERAGE(D8:CC8), 0)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
@@ -4298,6 +4321,9 @@
       <c r="CB8" t="n">
         <v>6</v>
       </c>
+      <c r="CC8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4311,7 +4337,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:CB9), 0)</f>
+        <f>ROUND(AVERAGE(D9:CC9), 0)</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
@@ -4533,6 +4559,9 @@
       <c r="CB9" t="n">
         <v>6</v>
       </c>
+      <c r="CC9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
@@ -4546,7 +4575,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:CB10), 0)</f>
+        <f>ROUND(AVERAGE(D10:CC10), 0)</f>
         <v/>
       </c>
       <c r="D10" s="10" t="n">
@@ -4779,6 +4808,9 @@
       </c>
       <c r="CB10" t="n">
         <v>6</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4793,7 +4825,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:CB11), 0)</f>
+        <f>ROUND(AVERAGE(D11:CC11), 0)</f>
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
@@ -5002,6 +5034,9 @@
       <c r="CB11" t="n">
         <v>6</v>
       </c>
+      <c r="CC11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -5015,7 +5050,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:CB12), 0)</f>
+        <f>ROUND(AVERAGE(D12:CC12), 0)</f>
         <v/>
       </c>
       <c r="G12" s="5" t="n">
@@ -5240,6 +5275,9 @@
       <c r="CB12" t="n">
         <v>0</v>
       </c>
+      <c r="CC12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -5253,7 +5291,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:CB13), 0)</f>
+        <f>ROUND(AVERAGE(D13:CC13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -5487,6 +5525,9 @@
       <c r="CB13" t="n">
         <v>6</v>
       </c>
+      <c r="CC13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5500,7 +5541,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:CB14), 0)</f>
+        <f>ROUND(AVERAGE(D14:CC14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5734,6 +5775,9 @@
       <c r="CB14" t="n">
         <v>0</v>
       </c>
+      <c r="CC14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5747,7 +5791,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:CB15), 0)</f>
+        <f>ROUND(AVERAGE(D15:CC15), 0)</f>
         <v/>
       </c>
       <c r="D15" s="10" t="n">
@@ -5981,6 +6025,9 @@
       <c r="CB15" t="n">
         <v>0</v>
       </c>
+      <c r="CC15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -5994,7 +6041,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:CB16), 0)</f>
+        <f>ROUND(AVERAGE(D16:CC16), 0)</f>
         <v/>
       </c>
       <c r="J16" s="6" t="n"/>
@@ -6208,6 +6255,9 @@
       <c r="CB16" t="n">
         <v>6</v>
       </c>
+      <c r="CC16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -6221,7 +6271,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:CB17), 0)</f>
+        <f>ROUND(AVERAGE(D17:CC17), 0)</f>
         <v/>
       </c>
       <c r="G17" s="5" t="n">
@@ -6446,6 +6496,9 @@
       <c r="CB17" t="n">
         <v>6</v>
       </c>
+      <c r="CC17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -6459,7 +6512,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:CB18), 0)</f>
+        <f>ROUND(AVERAGE(D18:CC18), 0)</f>
         <v/>
       </c>
       <c r="K18" s="6" t="n"/>
@@ -6640,6 +6693,9 @@
       <c r="CB18" t="n">
         <v>6</v>
       </c>
+      <c r="CC18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -6653,7 +6709,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:CB19), 0)</f>
+        <f>ROUND(AVERAGE(D19:CC19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6831,6 +6887,9 @@
       <c r="CB19" t="n">
         <v>6</v>
       </c>
+      <c r="CC19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6844,7 +6903,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:CB20), 0)</f>
+        <f>ROUND(AVERAGE(D20:CC20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -7016,6 +7075,9 @@
       <c r="CB20" t="n">
         <v>6</v>
       </c>
+      <c r="CC20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -7029,7 +7091,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:CB21), 0)</f>
+        <f>ROUND(AVERAGE(D21:CC21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -7192,6 +7254,9 @@
       <c r="CB21" t="n">
         <v>6</v>
       </c>
+      <c r="CC21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -7205,7 +7270,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:CB22), 0)</f>
+        <f>ROUND(AVERAGE(D22:CC22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -7368,6 +7433,9 @@
       <c r="CB22" t="n">
         <v>0</v>
       </c>
+      <c r="CC22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -7381,7 +7449,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:CB23), 0)</f>
+        <f>ROUND(AVERAGE(D23:CC23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7544,6 +7612,9 @@
       <c r="CB23" t="n">
         <v>0</v>
       </c>
+      <c r="CC23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -7557,7 +7628,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:CB24), 0)</f>
+        <f>ROUND(AVERAGE(D24:CC24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7669,6 +7740,9 @@
       <c r="CB24" t="n">
         <v>0</v>
       </c>
+      <c r="CC24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -7682,7 +7756,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:CB25), 0)</f>
+        <f>ROUND(AVERAGE(D25:CC25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -7699,6 +7773,38 @@
         <v>0</v>
       </c>
       <c r="CB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>TinoGiusa</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
+        </is>
+      </c>
+      <c r="C26" s="28">
+        <f>ROUND(AVERAGE(D26:CC26), 0)</f>
+        <v/>
+      </c>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="20" t="n"/>
+      <c r="P26" s="20" t="n"/>
+      <c r="Q26" s="20" t="n"/>
+      <c r="R26" s="20" t="n"/>
+      <c r="S26" s="20" t="n"/>
+      <c r="T26" s="20" t="n"/>
+      <c r="U26" s="20" t="n"/>
+      <c r="CC26" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2235,7 +2235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CD26"/>
+  <dimension ref="A1:CE25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2662,6 +2662,11 @@
           <t>21/08/2026</t>
         </is>
       </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2675,7 +2680,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:CD2), 0)</f>
+        <f>ROUND(AVERAGE(D2:CE2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2892,28 +2897,63 @@
         <v>0</v>
       </c>
       <c r="CD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>14/02/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:CD3), 0)</f>
+        <f>ROUND(AVERAGE(D3:CE3), 0)</f>
         <v/>
       </c>
-      <c r="K3" s="6" t="n"/>
-      <c r="L3" s="6" t="n"/>
-      <c r="N3" s="13" t="n"/>
-      <c r="O3" s="19" t="n"/>
+      <c r="D3" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N3" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="O3" t="n">
+        <v>6</v>
+      </c>
       <c r="P3" t="n">
         <v>6</v>
       </c>
@@ -2933,10 +2973,10 @@
         <v>6</v>
       </c>
       <c r="V3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
         <v>6</v>
@@ -2945,10 +2985,10 @@
         <v>6</v>
       </c>
       <c r="Z3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="n">
         <v>6</v>
@@ -2969,40 +3009,40 @@
         <v>6</v>
       </c>
       <c r="AH3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL3" t="n">
         <v>6</v>
       </c>
       <c r="AM3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AN3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AO3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ3" t="n">
         <v>6</v>
       </c>
       <c r="AR3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT3" t="n">
         <v>6</v>
@@ -3014,31 +3054,31 @@
         <v>6</v>
       </c>
       <c r="AW3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA3" t="n">
         <v>6</v>
       </c>
       <c r="BB3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BC3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BD3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BE3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BF3" t="n">
         <v>6</v>
@@ -3047,13 +3087,13 @@
         <v>0</v>
       </c>
       <c r="BH3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BI3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BJ3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BK3" t="n">
         <v>6</v>
@@ -3065,25 +3105,25 @@
         <v>0</v>
       </c>
       <c r="BN3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BO3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BP3" t="n">
         <v>6</v>
       </c>
       <c r="BQ3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BR3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BS3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BT3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BU3" t="n">
         <v>6</v>
@@ -3113,13 +3153,16 @@
         <v>0</v>
       </c>
       <c r="CD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -3128,7 +3171,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:CD4), 0)</f>
+        <f>ROUND(AVERAGE(D4:CE4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3147,34 +3190,34 @@
         <v>0</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N4" s="13" t="n">
         <v>6</v>
       </c>
       <c r="O4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
         <v>6</v>
@@ -3189,37 +3232,37 @@
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
         <v>6</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB4" t="n">
         <v>6</v>
       </c>
       <c r="AC4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH4" t="n">
         <v>0</v>
@@ -3234,7 +3277,7 @@
         <v>0</v>
       </c>
       <c r="AL4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM4" t="n">
         <v>0</v>
@@ -3249,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="AQ4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR4" t="n">
         <v>0</v>
@@ -3258,13 +3301,13 @@
         <v>0</v>
       </c>
       <c r="AT4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AU4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AV4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -3294,7 +3337,7 @@
         <v>0</v>
       </c>
       <c r="BF4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BG4" t="n">
         <v>0</v>
@@ -3309,7 +3352,7 @@
         <v>0</v>
       </c>
       <c r="BK4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BL4" t="n">
         <v>0</v>
@@ -3324,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="BP4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ4" t="n">
         <v>0</v>
@@ -3339,10 +3382,10 @@
         <v>0</v>
       </c>
       <c r="BU4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BV4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BW4" t="n">
         <v>0</v>
@@ -3351,83 +3394,56 @@
         <v>0</v>
       </c>
       <c r="BY4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BZ4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CA4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CB4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CC4" t="n">
         <v>0</v>
       </c>
       <c r="CD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:CD5), 0)</f>
+        <f>ROUND(AVERAGE(D5:CE5), 0)</f>
         <v/>
       </c>
-      <c r="D5" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>6</v>
-      </c>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="n"/>
+      <c r="N5" s="13" t="n"/>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
         <v>6</v>
@@ -3439,13 +3455,13 @@
         <v>6</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W5" t="n">
         <v>6</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y5" t="n">
         <v>6</v>
@@ -3454,10 +3470,10 @@
         <v>6</v>
       </c>
       <c r="AA5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -3532,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="BA5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB5" t="n">
         <v>0</v>
@@ -3619,65 +3635,56 @@
         <v>0</v>
       </c>
       <c r="CD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:CD6), 0)</f>
+        <f>ROUND(AVERAGE(D6:CE6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6" t="n"/>
       <c r="N6" s="13" t="n"/>
-      <c r="O6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T6" t="n">
-        <v>6</v>
-      </c>
+      <c r="O6" s="19" t="n"/>
+      <c r="P6" s="19" t="n"/>
+      <c r="Q6" s="19" t="n"/>
+      <c r="R6" s="19" t="n"/>
+      <c r="S6" s="19" t="n"/>
+      <c r="T6" s="19" t="n"/>
       <c r="U6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Y6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB6" t="n">
         <v>0</v>
@@ -3686,13 +3693,13 @@
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG6" t="n">
         <v>0</v>
@@ -3713,19 +3720,19 @@
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR6" t="n">
         <v>0</v>
@@ -3827,116 +3834,152 @@
         <v>0</v>
       </c>
       <c r="BY6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BZ6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="CA6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="CB6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="CC6" t="n">
         <v>0</v>
       </c>
       <c r="CD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:CD7), 0)</f>
+        <f>ROUND(AVERAGE(D7:CE7), 0)</f>
         <v/>
       </c>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
-      <c r="N7" s="13" t="n"/>
-      <c r="O7" s="19" t="n"/>
-      <c r="P7" s="19" t="n"/>
-      <c r="Q7" s="19" t="n"/>
-      <c r="R7" s="19" t="n"/>
-      <c r="S7" s="19" t="n"/>
-      <c r="T7" s="19" t="n"/>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="O7" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>6</v>
+      </c>
+      <c r="R7" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>6</v>
+      </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE7" t="n">
         <v>3</v>
       </c>
-      <c r="Y7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>6</v>
-      </c>
       <c r="AF7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG7" t="n">
         <v>0</v>
       </c>
       <c r="AH7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AI7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AM7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AN7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AO7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AP7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AQ7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AR7" t="n">
         <v>0</v>
@@ -3954,19 +3997,19 @@
         <v>0</v>
       </c>
       <c r="AW7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AX7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AY7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AZ7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BA7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB7" t="n">
         <v>0</v>
@@ -3984,34 +4027,34 @@
         <v>0</v>
       </c>
       <c r="BG7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BL7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BM7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BN7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BO7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BP7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BQ7" t="n">
         <v>0</v>
@@ -4038,42 +4081,42 @@
         <v>0</v>
       </c>
       <c r="BY7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BZ7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="CA7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="CB7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="CC7" t="n">
         <v>0</v>
       </c>
       <c r="CD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:CD8), 0)</f>
+        <f>ROUND(AVERAGE(D8:CE8), 0)</f>
         <v/>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>0</v>
-      </c>
       <c r="H8" s="5" t="n">
         <v>6</v>
       </c>
@@ -4081,7 +4124,7 @@
         <v>6</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K8" s="6" t="n">
         <v>6</v>
@@ -4108,7 +4151,7 @@
         <v>6</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="T8" t="n">
         <v>6</v>
@@ -4120,22 +4163,22 @@
         <v>6</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA8" t="n">
         <v>6</v>
       </c>
       <c r="AB8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AC8" t="n">
         <v>6</v>
@@ -4144,25 +4187,25 @@
         <v>6</v>
       </c>
       <c r="AE8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AH8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL8" t="n">
         <v>6</v>
@@ -4183,25 +4226,25 @@
         <v>6</v>
       </c>
       <c r="AR8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY8" t="n">
         <v>6</v>
@@ -4225,7 +4268,7 @@
         <v>0</v>
       </c>
       <c r="BF8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BG8" t="n">
         <v>6</v>
@@ -4258,34 +4301,34 @@
         <v>6</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BS8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BT8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BU8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BV8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BW8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BX8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BY8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BZ8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CA8" t="n">
         <v>6</v>
@@ -4298,23 +4341,38 @@
       </c>
       <c r="CD8" t="n">
         <v>0</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:CD9), 0)</f>
+        <f>ROUND(AVERAGE(D9:CE9), 0)</f>
         <v/>
       </c>
+      <c r="D9" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="H9" s="5" t="n">
         <v>6</v>
       </c>
@@ -4358,25 +4416,25 @@
         <v>6</v>
       </c>
       <c r="V9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA9" t="n">
         <v>6</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AC9" t="n">
         <v>6</v>
@@ -4385,10 +4443,10 @@
         <v>6</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AG9" t="n">
         <v>6</v>
@@ -4400,34 +4458,34 @@
         <v>0</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AK9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AL9" t="n">
         <v>6</v>
       </c>
       <c r="AM9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AN9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AO9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ9" t="n">
         <v>6</v>
       </c>
       <c r="AR9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AS9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AT9" t="n">
         <v>6</v>
@@ -4445,10 +4503,10 @@
         <v>0</v>
       </c>
       <c r="AY9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA9" t="n">
         <v>6</v>
@@ -4469,46 +4527,46 @@
         <v>6</v>
       </c>
       <c r="BG9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BH9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BI9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BJ9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BK9" t="n">
         <v>6</v>
       </c>
       <c r="BL9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BM9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BN9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BO9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP9" t="n">
         <v>6</v>
       </c>
       <c r="BQ9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BR9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BS9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BT9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BU9" t="n">
         <v>6</v>
@@ -4517,16 +4575,16 @@
         <v>6</v>
       </c>
       <c r="BW9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BX9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BY9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BZ9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CA9" t="n">
         <v>6</v>
@@ -4538,56 +4596,34 @@
         <v>0</v>
       </c>
       <c r="CD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>25/01/2026</t>
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:CD10), 0)</f>
+        <f>ROUND(AVERAGE(D10:CE10), 0)</f>
         <v/>
       </c>
-      <c r="D10" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
       <c r="M10" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N10" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O10" t="n">
         <v>6</v>
@@ -4608,25 +4644,25 @@
         <v>6</v>
       </c>
       <c r="U10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z10" t="n">
         <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="n">
         <v>6</v>
@@ -4635,22 +4671,22 @@
         <v>6</v>
       </c>
       <c r="AD10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE10" t="n">
         <v>6</v>
       </c>
       <c r="AF10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AI10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AJ10" t="n">
         <v>6</v>
@@ -4674,13 +4710,13 @@
         <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT10" t="n">
         <v>6</v>
@@ -4704,7 +4740,7 @@
         <v>0</v>
       </c>
       <c r="BA10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB10" t="n">
         <v>0</v>
@@ -4719,19 +4755,19 @@
         <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BG10" t="n">
         <v>0</v>
       </c>
       <c r="BH10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK10" t="n">
         <v>6</v>
@@ -4749,19 +4785,19 @@
         <v>0</v>
       </c>
       <c r="BP10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BR10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BS10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BT10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BU10" t="n">
         <v>6</v>
@@ -4776,10 +4812,10 @@
         <v>0</v>
       </c>
       <c r="BY10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BZ10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CA10" t="n">
         <v>6</v>
@@ -4792,129 +4828,148 @@
       </c>
       <c r="CD10" t="n">
         <v>0</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>15/12/2025</t>
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:CD11), 0)</f>
+        <f>ROUND(AVERAGE(D11:CE11), 0)</f>
         <v/>
       </c>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="M11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="N11" s="13" t="n">
+      <c r="N11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" t="n">
+        <v>6</v>
+      </c>
+      <c r="P11" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>6</v>
+      </c>
+      <c r="R11" t="n">
+        <v>6</v>
+      </c>
+      <c r="S11" t="n">
+        <v>6</v>
+      </c>
+      <c r="T11" t="n">
+        <v>6</v>
+      </c>
+      <c r="U11" t="n">
+        <v>6</v>
+      </c>
+      <c r="V11" t="n">
+        <v>6</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM11" t="n">
         <v>1</v>
       </c>
-      <c r="O11" t="n">
-        <v>6</v>
-      </c>
-      <c r="P11" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>6</v>
-      </c>
-      <c r="R11" t="n">
-        <v>6</v>
-      </c>
-      <c r="S11" t="n">
-        <v>6</v>
-      </c>
-      <c r="T11" t="n">
-        <v>6</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" t="n">
-        <v>6</v>
-      </c>
-      <c r="W11" t="n">
-        <v>6</v>
-      </c>
-      <c r="X11" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>0</v>
-      </c>
       <c r="AN11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AS11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AT11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AV11" t="n">
         <v>6</v>
@@ -4926,13 +4981,13 @@
         <v>0</v>
       </c>
       <c r="AY11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BA11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB11" t="n">
         <v>0</v>
@@ -4947,22 +5002,22 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BG11" t="n">
         <v>0</v>
       </c>
       <c r="BH11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BI11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BJ11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BK11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BL11" t="n">
         <v>0</v>
@@ -4980,22 +5035,22 @@
         <v>0</v>
       </c>
       <c r="BQ11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BR11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BS11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BT11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BU11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BV11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BW11" t="n">
         <v>0</v>
@@ -5004,28 +5059,31 @@
         <v>0</v>
       </c>
       <c r="BY11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="BZ11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="CA11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CB11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CC11" t="n">
         <v>0</v>
       </c>
       <c r="CD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -5034,14 +5092,23 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:CD12), 0)</f>
+        <f>ROUND(AVERAGE(D12:CE12), 0)</f>
         <v/>
       </c>
+      <c r="D12" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>6</v>
+      </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>6</v>
@@ -5050,16 +5117,16 @@
         <v>6</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
         <v>6</v>
@@ -5080,25 +5147,25 @@
         <v>6</v>
       </c>
       <c r="U12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X12" t="n">
         <v>6</v>
       </c>
       <c r="Y12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Z12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AA12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB12" t="n">
         <v>6</v>
@@ -5119,7 +5186,7 @@
         <v>6</v>
       </c>
       <c r="AH12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AI12" t="n">
         <v>6</v>
@@ -5134,31 +5201,31 @@
         <v>6</v>
       </c>
       <c r="AM12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AN12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AO12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AP12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AQ12" t="n">
         <v>6</v>
       </c>
       <c r="AR12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AU12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AV12" t="n">
         <v>6</v>
@@ -5170,10 +5237,10 @@
         <v>0</v>
       </c>
       <c r="AY12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ12" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA12" t="n">
         <v>6</v>
@@ -5185,13 +5252,13 @@
         <v>0</v>
       </c>
       <c r="BD12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -5218,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="BO12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BP12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BQ12" t="n">
         <v>0</v>
@@ -5236,40 +5303,43 @@
         <v>0</v>
       </c>
       <c r="BU12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BV12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BW12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BX12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BY12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BZ12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CA12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CB12" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CC12" t="n">
         <v>0</v>
       </c>
       <c r="CD12" t="n">
         <v>0</v>
+      </c>
+      <c r="CE12" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -5278,80 +5348,80 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:CD13), 0)</f>
+        <f>ROUND(AVERAGE(D13:CE13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
         <v>6</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>6</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O13" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P13" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q13" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R13" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S13" t="n">
+        <v>6</v>
+      </c>
+      <c r="T13" t="n">
+        <v>4</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>6</v>
+      </c>
+      <c r="W13" t="n">
+        <v>3</v>
+      </c>
+      <c r="X13" t="n">
         <v>5</v>
       </c>
-      <c r="I13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
-        <v>6</v>
-      </c>
-      <c r="P13" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>6</v>
-      </c>
-      <c r="R13" t="n">
-        <v>6</v>
-      </c>
-      <c r="S13" t="n">
-        <v>6</v>
-      </c>
-      <c r="T13" t="n">
-        <v>6</v>
-      </c>
-      <c r="U13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" t="n">
-        <v>5</v>
-      </c>
-      <c r="W13" t="n">
-        <v>6</v>
-      </c>
-      <c r="X13" t="n">
-        <v>6</v>
-      </c>
       <c r="Y13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AA13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AB13" t="n">
         <v>6</v>
@@ -5360,52 +5430,52 @@
         <v>6</v>
       </c>
       <c r="AD13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG13" t="n">
         <v>6</v>
       </c>
       <c r="AH13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AI13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AN13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AO13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AP13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AQ13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AR13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT13" t="n">
         <v>6</v>
@@ -5423,28 +5493,28 @@
         <v>0</v>
       </c>
       <c r="AY13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BA13" t="n">
         <v>6</v>
       </c>
       <c r="BB13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BD13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BG13" t="n">
         <v>0</v>
@@ -5468,13 +5538,13 @@
         <v>0</v>
       </c>
       <c r="BN13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BO13" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BP13" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BQ13" t="n">
         <v>0</v>
@@ -5483,46 +5553,49 @@
         <v>0</v>
       </c>
       <c r="BS13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BT13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BU13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="BV13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="BW13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BX13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BY13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BZ13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CA13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CB13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CC13" t="n">
         <v>0</v>
       </c>
       <c r="CD13" t="n">
         <v>0</v>
+      </c>
+      <c r="CE13" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -5531,11 +5604,11 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:CD14), 0)</f>
+        <f>ROUND(AVERAGE(D14:CE14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>6</v>
@@ -5553,7 +5626,7 @@
         <v>6</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K14" s="6" t="n">
         <v>6</v>
@@ -5579,23 +5652,23 @@
       <c r="R14" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="S14" t="n">
+      <c r="S14" s="20" t="n">
         <v>6</v>
       </c>
       <c r="T14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y14" t="n">
         <v>0</v>
@@ -5604,7 +5677,7 @@
         <v>0</v>
       </c>
       <c r="AA14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AB14" t="n">
         <v>6</v>
@@ -5619,7 +5692,7 @@
         <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG14" t="n">
         <v>6</v>
@@ -5640,31 +5713,31 @@
         <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AP14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AQ14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AR14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AU14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AV14" t="n">
         <v>6</v>
@@ -5676,43 +5749,43 @@
         <v>0</v>
       </c>
       <c r="AY14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AZ14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BA14" t="n">
         <v>6</v>
       </c>
       <c r="BB14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BE14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BG14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BL14" t="n">
         <v>0</v>
@@ -5721,13 +5794,13 @@
         <v>0</v>
       </c>
       <c r="BN14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BO14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ14" t="n">
         <v>0</v>
@@ -5736,16 +5809,16 @@
         <v>0</v>
       </c>
       <c r="BS14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BT14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BU14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BV14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BW14" t="n">
         <v>0</v>
@@ -5769,13 +5842,16 @@
         <v>0</v>
       </c>
       <c r="CD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -5784,92 +5860,72 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:CD15), 0)</f>
+        <f>ROUND(AVERAGE(D15:CE15), 0)</f>
         <v/>
       </c>
-      <c r="D15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="S15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" t="n">
+        <v>6</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="n">
         <v>5</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O15" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P15" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q15" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R15" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S15" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T15" t="n">
-        <v>6</v>
-      </c>
-      <c r="U15" t="n">
-        <v>6</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
       <c r="X15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AA15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AB15" t="n">
         <v>6</v>
       </c>
       <c r="AC15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF15" t="n">
         <v>6</v>
@@ -5899,10 +5955,10 @@
         <v>0</v>
       </c>
       <c r="AO15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AQ15" t="n">
         <v>6</v>
@@ -5914,13 +5970,13 @@
         <v>0</v>
       </c>
       <c r="AT15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
@@ -5935,7 +5991,7 @@
         <v>0</v>
       </c>
       <c r="BA15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB15" t="n">
         <v>0</v>
@@ -5944,28 +6000,28 @@
         <v>0</v>
       </c>
       <c r="BD15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF15" t="n">
         <v>6</v>
       </c>
       <c r="BG15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BH15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BI15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BK15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BL15" t="n">
         <v>0</v>
@@ -6013,22 +6069,25 @@
         <v>0</v>
       </c>
       <c r="CA15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CB15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CC15" t="n">
         <v>0</v>
       </c>
       <c r="CD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -6037,10 +6096,21 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:CD16), 0)</f>
+        <f>ROUND(AVERAGE(D16:CE16), 0)</f>
         <v/>
       </c>
-      <c r="J16" s="6" t="n"/>
+      <c r="G16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="K16" s="6" t="n">
         <v>6</v>
       </c>
@@ -6057,7 +6127,7 @@
         <v>6</v>
       </c>
       <c r="P16" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="20" t="n">
         <v>6</v>
@@ -6071,26 +6141,26 @@
       <c r="T16" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="U16" t="n">
+      <c r="U16" s="20" t="n">
         <v>6</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
       </c>
       <c r="W16" t="n">
+        <v>6</v>
+      </c>
+      <c r="X16" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="n">
         <v>5</v>
       </c>
-      <c r="X16" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>6</v>
-      </c>
       <c r="AA16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AB16" t="n">
         <v>6</v>
@@ -6108,22 +6178,22 @@
         <v>6</v>
       </c>
       <c r="AG16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AM16" t="n">
         <v>0</v>
@@ -6138,22 +6208,22 @@
         <v>0</v>
       </c>
       <c r="AQ16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AR16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -6186,34 +6256,34 @@
         <v>6</v>
       </c>
       <c r="BG16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BL16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BM16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BN16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BO16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BP16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BQ16" t="n">
         <v>0</v>
@@ -6228,22 +6298,22 @@
         <v>0</v>
       </c>
       <c r="BU16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BV16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BW16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BX16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BY16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BZ16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CA16" t="n">
         <v>6</v>
@@ -6255,170 +6325,129 @@
         <v>0</v>
       </c>
       <c r="CD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>15/12/2025</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:CD17), 0)</f>
+        <f>ROUND(AVERAGE(D17:CE17), 0)</f>
         <v/>
       </c>
-      <c r="G17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="P17" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="R17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="S17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="T17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="U17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="V17" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" t="n">
-        <v>6</v>
-      </c>
-      <c r="X17" t="n">
-        <v>2</v>
-      </c>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="20" t="n"/>
+      <c r="P17" s="20" t="n"/>
+      <c r="Q17" s="20" t="n"/>
+      <c r="R17" s="20" t="n"/>
+      <c r="S17" s="20" t="n"/>
+      <c r="T17" s="20" t="n"/>
+      <c r="U17" s="20" t="n"/>
       <c r="Y17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Z17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO17" t="n">
         <v>5</v>
       </c>
-      <c r="AA17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH17" t="n">
+      <c r="AP17" t="n">
         <v>5</v>
       </c>
-      <c r="AI17" t="n">
+      <c r="AQ17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AR17" t="n">
         <v>5</v>
       </c>
-      <c r="AJ17" t="n">
+      <c r="AS17" t="n">
         <v>5</v>
       </c>
-      <c r="AK17" t="n">
+      <c r="AT17" t="n">
         <v>5</v>
       </c>
-      <c r="AL17" t="n">
+      <c r="AU17" t="n">
         <v>5</v>
       </c>
-      <c r="AM17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU17" t="n">
-        <v>6</v>
-      </c>
       <c r="AV17" t="n">
         <v>6</v>
       </c>
       <c r="AW17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AX17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AY17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AZ17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BA17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BC17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BD17" t="n">
         <v>6</v>
@@ -6430,34 +6459,34 @@
         <v>6</v>
       </c>
       <c r="BG17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BH17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BI17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BJ17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BK17" t="n">
         <v>6</v>
       </c>
       <c r="BL17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BM17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BN17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BO17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BP17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BQ17" t="n">
         <v>0</v>
@@ -6478,10 +6507,10 @@
         <v>6</v>
       </c>
       <c r="BW17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BX17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BY17" t="n">
         <v>6</v>
@@ -6500,21 +6529,24 @@
       </c>
       <c r="CD17" t="n">
         <v>0</v>
+      </c>
+      <c r="CE17" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:CD18), 0)</f>
+        <f>ROUND(AVERAGE(D18:CE18), 0)</f>
         <v/>
       </c>
       <c r="K18" s="6" t="n"/>
@@ -6527,15 +6559,12 @@
       <c r="S18" s="20" t="n"/>
       <c r="T18" s="20" t="n"/>
       <c r="U18" s="20" t="n"/>
-      <c r="Y18" t="n">
-        <v>6</v>
-      </c>
       <c r="Z18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA18" t="n">
         <v>3</v>
       </c>
-      <c r="AA18" t="n">
-        <v>6</v>
-      </c>
       <c r="AB18" t="n">
         <v>6</v>
       </c>
@@ -6561,64 +6590,64 @@
         <v>0</v>
       </c>
       <c r="AJ18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL18" t="n">
         <v>6</v>
       </c>
       <c r="AM18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ18" t="n">
         <v>6</v>
       </c>
       <c r="AR18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AS18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AT18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AW18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AZ18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BA18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="BB18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BC18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BD18" t="n">
         <v>6</v>
@@ -6630,46 +6659,46 @@
         <v>6</v>
       </c>
       <c r="BG18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BH18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BI18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BK18" t="n">
         <v>6</v>
       </c>
       <c r="BL18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BM18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BN18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BO18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BP18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BQ18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BR18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BS18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BT18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BU18" t="n">
         <v>6</v>
@@ -6678,16 +6707,16 @@
         <v>6</v>
       </c>
       <c r="BW18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BX18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BY18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BZ18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CA18" t="n">
         <v>6</v>
@@ -6699,22 +6728,25 @@
         <v>0</v>
       </c>
       <c r="CD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:CD19), 0)</f>
+        <f>ROUND(AVERAGE(D19:CE19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6727,12 +6759,6 @@
       <c r="S19" s="20" t="n"/>
       <c r="T19" s="20" t="n"/>
       <c r="U19" s="20" t="n"/>
-      <c r="Z19" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>3</v>
-      </c>
       <c r="AB19" t="n">
         <v>6</v>
       </c>
@@ -6752,34 +6778,34 @@
         <v>6</v>
       </c>
       <c r="AH19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AI19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AK19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AL19" t="n">
         <v>6</v>
       </c>
       <c r="AM19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AO19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR19" t="n">
         <v>0</v>
@@ -6794,97 +6820,97 @@
         <v>0</v>
       </c>
       <c r="AV19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AX19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AY19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AZ19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BA19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BB19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BC19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BD19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BE19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BF19" t="n">
         <v>6</v>
       </c>
       <c r="BG19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BH19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BI19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BJ19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BK19" t="n">
         <v>6</v>
       </c>
       <c r="BL19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BM19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BN19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BO19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BP19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BQ19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BR19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BS19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BT19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BU19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BV19" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BW19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BX19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BY19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BZ19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CA19" t="n">
         <v>6</v>
@@ -6896,22 +6922,25 @@
         <v>0</v>
       </c>
       <c r="CD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:CD20), 0)</f>
+        <f>ROUND(AVERAGE(D20:CE20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -6924,15 +6953,6 @@
       <c r="S20" s="20" t="n"/>
       <c r="T20" s="20" t="n"/>
       <c r="U20" s="20" t="n"/>
-      <c r="AB20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD20" t="n">
-        <v>6</v>
-      </c>
       <c r="AE20" t="n">
         <v>6</v>
       </c>
@@ -6940,143 +6960,143 @@
         <v>6</v>
       </c>
       <c r="AG20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AH20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AZ20" t="n">
+        <v>6</v>
+      </c>
+      <c r="BA20" t="n">
+        <v>6</v>
+      </c>
+      <c r="BB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK20" t="n">
+        <v>6</v>
+      </c>
+      <c r="BL20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>6</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>6</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY20" t="n">
         <v>5</v>
       </c>
-      <c r="AI20" t="n">
+      <c r="BZ20" t="n">
         <v>5</v>
       </c>
-      <c r="AJ20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AR20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AX20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AY20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AZ20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BA20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BB20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD20" t="n">
-        <v>4</v>
-      </c>
-      <c r="BE20" t="n">
-        <v>4</v>
-      </c>
-      <c r="BF20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BG20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BH20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BI20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BJ20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BK20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BL20" t="n">
-        <v>4</v>
-      </c>
-      <c r="BM20" t="n">
-        <v>4</v>
-      </c>
-      <c r="BN20" t="n">
-        <v>5</v>
-      </c>
-      <c r="BO20" t="n">
-        <v>5</v>
-      </c>
-      <c r="BP20" t="n">
-        <v>5</v>
-      </c>
-      <c r="BQ20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV20" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BX20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BY20" t="n">
-        <v>6</v>
-      </c>
-      <c r="BZ20" t="n">
-        <v>6</v>
-      </c>
       <c r="CA20" t="n">
         <v>6</v>
       </c>
@@ -7088,21 +7108,24 @@
       </c>
       <c r="CD20" t="n">
         <v>0</v>
+      </c>
+      <c r="CE20" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:CD21), 0)</f>
+        <f>ROUND(AVERAGE(D21:CE21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -7116,7 +7139,7 @@
       <c r="T21" s="20" t="n"/>
       <c r="U21" s="20" t="n"/>
       <c r="AE21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF21" t="n">
         <v>6</v>
@@ -7131,13 +7154,13 @@
         <v>0</v>
       </c>
       <c r="AJ21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AK21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AL21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AM21" t="n">
         <v>0</v>
@@ -7170,19 +7193,19 @@
         <v>0</v>
       </c>
       <c r="AW21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AX21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AZ21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BA21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BB21" t="n">
         <v>0</v>
@@ -7197,7 +7220,7 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BG21" t="n">
         <v>0</v>
@@ -7212,7 +7235,7 @@
         <v>0</v>
       </c>
       <c r="BK21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BL21" t="n">
         <v>0</v>
@@ -7224,10 +7247,10 @@
         <v>0</v>
       </c>
       <c r="BO21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BP21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="BQ21" t="n">
         <v>0</v>
@@ -7254,37 +7277,40 @@
         <v>0</v>
       </c>
       <c r="BY21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="BZ21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="CA21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CB21" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CC21" t="n">
         <v>0</v>
       </c>
       <c r="CD21" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:CD22), 0)</f>
+        <f>ROUND(AVERAGE(D22:CE22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -7298,10 +7324,10 @@
       <c r="T22" s="20" t="n"/>
       <c r="U22" s="20" t="n"/>
       <c r="AE22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AF22" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AG22" t="n">
         <v>0</v>
@@ -7328,28 +7354,28 @@
         <v>0</v>
       </c>
       <c r="AO22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AP22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AR22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AT22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW22" t="n">
         <v>0</v>
@@ -7451,22 +7477,25 @@
         <v>0</v>
       </c>
       <c r="CD22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:CD23), 0)</f>
+        <f>ROUND(AVERAGE(D23:CE23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7479,57 +7508,6 @@
       <c r="S23" s="20" t="n"/>
       <c r="T23" s="20" t="n"/>
       <c r="U23" s="20" t="n"/>
-      <c r="AE23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AS23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AT23" t="n">
-        <v>6</v>
-      </c>
-      <c r="AU23" t="n">
-        <v>6</v>
-      </c>
       <c r="AV23" t="n">
         <v>6</v>
       </c>
@@ -7546,7 +7524,7 @@
         <v>0</v>
       </c>
       <c r="BA23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BB23" t="n">
         <v>0</v>
@@ -7555,13 +7533,13 @@
         <v>0</v>
       </c>
       <c r="BD23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BE23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BG23" t="n">
         <v>0</v>
@@ -7634,21 +7612,24 @@
       </c>
       <c r="CD23" t="n">
         <v>0</v>
+      </c>
+      <c r="CE23" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:CD24), 0)</f>
+        <f>ROUND(AVERAGE(D24:CE24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7661,99 +7642,6 @@
       <c r="S24" s="20" t="n"/>
       <c r="T24" s="20" t="n"/>
       <c r="U24" s="20" t="n"/>
-      <c r="AV24" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>6</v>
-      </c>
-      <c r="BB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD24" t="n">
-        <v>6</v>
-      </c>
-      <c r="BE24" t="n">
-        <v>6</v>
-      </c>
-      <c r="BF24" t="n">
-        <v>6</v>
-      </c>
-      <c r="BG24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BY24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BZ24" t="n">
-        <v>0</v>
-      </c>
       <c r="CA24" t="n">
         <v>0</v>
       </c>
@@ -7764,22 +7652,25 @@
         <v>0</v>
       </c>
       <c r="CD24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:CD25), 0)</f>
+        <f>ROUND(AVERAGE(D25:CE25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -7792,48 +7683,13 @@
       <c r="S25" s="20" t="n"/>
       <c r="T25" s="20" t="n"/>
       <c r="U25" s="20" t="n"/>
-      <c r="CA25" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB25" t="n">
-        <v>0</v>
-      </c>
       <c r="CC25" t="n">
         <v>0</v>
       </c>
       <c r="CD25" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="28" t="inlineStr">
-        <is>
-          <t>TinoGiusa</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="C26" s="28">
-        <f>ROUND(AVERAGE(D26:CD26), 0)</f>
-        <v/>
-      </c>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
-      <c r="N26" s="6" t="n"/>
-      <c r="O26" s="20" t="n"/>
-      <c r="P26" s="20" t="n"/>
-      <c r="Q26" s="20" t="n"/>
-      <c r="R26" s="20" t="n"/>
-      <c r="S26" s="20" t="n"/>
-      <c r="T26" s="20" t="n"/>
-      <c r="U26" s="20" t="n"/>
-      <c r="CC26" t="n">
-        <v>0</v>
-      </c>
-      <c r="CD26" t="n">
+      <c r="CE25" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-08-23
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -955,7 +955,7 @@
         <v/>
       </c>
       <c r="E2" s="14" t="n">
-        <v>65400</v>
+        <v>65550</v>
       </c>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
@@ -977,7 +977,7 @@
         <v>3550</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
@@ -1288,7 +1288,7 @@
         <v/>
       </c>
       <c r="E8" s="14" t="n">
-        <v>54650</v>
+        <v>54800</v>
       </c>
       <c r="F8" s="13" t="n">
         <v>4000</v>
@@ -1318,7 +1318,7 @@
         <v>4250</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="13" t="n"/>
@@ -1636,7 +1636,7 @@
         <v/>
       </c>
       <c r="E14" s="14" t="n">
-        <v>85300</v>
+        <v>85900</v>
       </c>
       <c r="F14" s="13" t="n"/>
       <c r="G14" s="13" t="n"/>
@@ -1660,7 +1660,7 @@
         <v>5600</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>2500</v>
+        <v>3100</v>
       </c>
       <c r="P14" s="13" t="n"/>
       <c r="Q14" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Capital data - 2026-08-24
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -2235,7 +2235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CF25"/>
+  <dimension ref="A1:CG25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2672,6 +2672,11 @@
           <t>21/08/2026</t>
         </is>
       </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
@@ -2685,7 +2690,7 @@
         </is>
       </c>
       <c r="C2" s="28">
-        <f>ROUND(AVERAGE(D2:CF2), 0)</f>
+        <f>ROUND(AVERAGE(D2:CG2), 0)</f>
         <v/>
       </c>
       <c r="K2" s="6" t="n">
@@ -2908,6 +2913,9 @@
         <v>0</v>
       </c>
       <c r="CF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2923,7 +2931,7 @@
         </is>
       </c>
       <c r="C3" s="28">
-        <f>ROUND(AVERAGE(D3:CF3), 0)</f>
+        <f>ROUND(AVERAGE(D3:CG3), 0)</f>
         <v/>
       </c>
       <c r="D3" s="10" t="n">
@@ -3168,6 +3176,9 @@
       </c>
       <c r="CF3" t="n">
         <v>0</v>
+      </c>
+      <c r="CG3" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -3182,7 +3193,7 @@
         </is>
       </c>
       <c r="C4" s="28">
-        <f>ROUND(AVERAGE(D4:CF4), 0)</f>
+        <f>ROUND(AVERAGE(D4:CG4), 0)</f>
         <v/>
       </c>
       <c r="D4" s="10" t="n">
@@ -3428,6 +3439,9 @@
       <c r="CF4" t="n">
         <v>0</v>
       </c>
+      <c r="CG4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3441,7 +3455,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>ROUND(AVERAGE(D5:CF5), 0)</f>
+        <f>ROUND(AVERAGE(D5:CG5), 0)</f>
         <v/>
       </c>
       <c r="K5" s="6" t="n"/>
@@ -3657,6 +3671,9 @@
       <c r="CF5" t="n">
         <v>0</v>
       </c>
+      <c r="CG5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
@@ -3670,7 +3687,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>ROUND(AVERAGE(D6:CF6), 0)</f>
+        <f>ROUND(AVERAGE(D6:CG6), 0)</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -3874,6 +3891,9 @@
       <c r="CF6" t="n">
         <v>0</v>
       </c>
+      <c r="CG6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
@@ -3887,7 +3907,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>ROUND(AVERAGE(D7:CF7), 0)</f>
+        <f>ROUND(AVERAGE(D7:CG7), 0)</f>
         <v/>
       </c>
       <c r="G7" s="5" t="n">
@@ -4124,6 +4144,9 @@
       <c r="CF7" t="n">
         <v>0</v>
       </c>
+      <c r="CG7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
@@ -4137,7 +4160,7 @@
         </is>
       </c>
       <c r="C8" s="28">
-        <f>ROUND(AVERAGE(D8:CF8), 0)</f>
+        <f>ROUND(AVERAGE(D8:CG8), 0)</f>
         <v/>
       </c>
       <c r="H8" s="5" t="n">
@@ -4371,6 +4394,9 @@
       <c r="CF8" t="n">
         <v>6</v>
       </c>
+      <c r="CG8" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="28" t="inlineStr">
@@ -4384,7 +4410,7 @@
         </is>
       </c>
       <c r="C9" s="28">
-        <f>ROUND(AVERAGE(D9:CF9), 0)</f>
+        <f>ROUND(AVERAGE(D9:CG9), 0)</f>
         <v/>
       </c>
       <c r="D9" s="10" t="n">
@@ -4629,6 +4655,9 @@
       </c>
       <c r="CF9" t="n">
         <v>0</v>
+      </c>
+      <c r="CG9" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -4643,7 +4672,7 @@
         </is>
       </c>
       <c r="C10" s="28">
-        <f>ROUND(AVERAGE(D10:CF10), 0)</f>
+        <f>ROUND(AVERAGE(D10:CG10), 0)</f>
         <v/>
       </c>
       <c r="K10" s="6" t="n"/>
@@ -4864,6 +4893,9 @@
       <c r="CF10" t="n">
         <v>6</v>
       </c>
+      <c r="CG10" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="28" t="inlineStr">
@@ -4877,7 +4909,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>ROUND(AVERAGE(D11:CF11), 0)</f>
+        <f>ROUND(AVERAGE(D11:CG11), 0)</f>
         <v/>
       </c>
       <c r="G11" s="5" t="n">
@@ -5114,6 +5146,9 @@
       <c r="CF11" t="n">
         <v>0</v>
       </c>
+      <c r="CG11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="inlineStr">
@@ -5127,7 +5162,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>ROUND(AVERAGE(D12:CF12), 0)</f>
+        <f>ROUND(AVERAGE(D12:CG12), 0)</f>
         <v/>
       </c>
       <c r="D12" s="10" t="n">
@@ -5373,6 +5408,9 @@
       <c r="CF12" t="n">
         <v>6</v>
       </c>
+      <c r="CG12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -5386,7 +5424,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>ROUND(AVERAGE(D13:CF13), 0)</f>
+        <f>ROUND(AVERAGE(D13:CG13), 0)</f>
         <v/>
       </c>
       <c r="D13" s="10" t="n">
@@ -5632,6 +5670,9 @@
       <c r="CF13" t="n">
         <v>4</v>
       </c>
+      <c r="CG13" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -5645,7 +5686,7 @@
         </is>
       </c>
       <c r="C14" s="28">
-        <f>ROUND(AVERAGE(D14:CF14), 0)</f>
+        <f>ROUND(AVERAGE(D14:CG14), 0)</f>
         <v/>
       </c>
       <c r="D14" s="10" t="n">
@@ -5891,6 +5932,9 @@
       <c r="CF14" t="n">
         <v>0</v>
       </c>
+      <c r="CG14" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
@@ -5904,7 +5948,7 @@
         </is>
       </c>
       <c r="C15" s="28">
-        <f>ROUND(AVERAGE(D15:CF15), 0)</f>
+        <f>ROUND(AVERAGE(D15:CG15), 0)</f>
         <v/>
       </c>
       <c r="J15" s="6" t="n"/>
@@ -6130,6 +6174,9 @@
       <c r="CF15" t="n">
         <v>0</v>
       </c>
+      <c r="CG15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -6143,7 +6190,7 @@
         </is>
       </c>
       <c r="C16" s="28">
-        <f>ROUND(AVERAGE(D16:CF16), 0)</f>
+        <f>ROUND(AVERAGE(D16:CG16), 0)</f>
         <v/>
       </c>
       <c r="G16" s="5" t="n">
@@ -6380,6 +6427,9 @@
       <c r="CF16" t="n">
         <v>0</v>
       </c>
+      <c r="CG16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -6393,7 +6443,7 @@
         </is>
       </c>
       <c r="C17" s="28">
-        <f>ROUND(AVERAGE(D17:CF17), 0)</f>
+        <f>ROUND(AVERAGE(D17:CG17), 0)</f>
         <v/>
       </c>
       <c r="K17" s="6" t="n"/>
@@ -6586,6 +6636,9 @@
       <c r="CF17" t="n">
         <v>3</v>
       </c>
+      <c r="CG17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -6599,7 +6652,7 @@
         </is>
       </c>
       <c r="C18" s="28">
-        <f>ROUND(AVERAGE(D18:CF18), 0)</f>
+        <f>ROUND(AVERAGE(D18:CG18), 0)</f>
         <v/>
       </c>
       <c r="K18" s="6" t="n"/>
@@ -6789,6 +6842,9 @@
       <c r="CF18" t="n">
         <v>0</v>
       </c>
+      <c r="CG18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -6802,7 +6858,7 @@
         </is>
       </c>
       <c r="C19" s="28">
-        <f>ROUND(AVERAGE(D19:CF19), 0)</f>
+        <f>ROUND(AVERAGE(D19:CG19), 0)</f>
         <v/>
       </c>
       <c r="K19" s="6" t="n"/>
@@ -6986,6 +7042,9 @@
       <c r="CF19" t="n">
         <v>0</v>
       </c>
+      <c r="CG19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="inlineStr">
@@ -6999,7 +7058,7 @@
         </is>
       </c>
       <c r="C20" s="28">
-        <f>ROUND(AVERAGE(D20:CF20), 0)</f>
+        <f>ROUND(AVERAGE(D20:CG20), 0)</f>
         <v/>
       </c>
       <c r="K20" s="6" t="n"/>
@@ -7174,6 +7233,9 @@
       <c r="CF20" t="n">
         <v>6</v>
       </c>
+      <c r="CG20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -7187,7 +7249,7 @@
         </is>
       </c>
       <c r="C21" s="28">
-        <f>ROUND(AVERAGE(D21:CF21), 0)</f>
+        <f>ROUND(AVERAGE(D21:CG21), 0)</f>
         <v/>
       </c>
       <c r="K21" s="6" t="n"/>
@@ -7362,6 +7424,9 @@
       <c r="CF21" t="n">
         <v>0</v>
       </c>
+      <c r="CG21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="28" t="inlineStr">
@@ -7375,7 +7440,7 @@
         </is>
       </c>
       <c r="C22" s="28">
-        <f>ROUND(AVERAGE(D22:CF22), 0)</f>
+        <f>ROUND(AVERAGE(D22:CG22), 0)</f>
         <v/>
       </c>
       <c r="K22" s="6" t="n"/>
@@ -7550,6 +7615,9 @@
       <c r="CF22" t="n">
         <v>0</v>
       </c>
+      <c r="CG22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="inlineStr">
@@ -7563,7 +7631,7 @@
         </is>
       </c>
       <c r="C23" s="28">
-        <f>ROUND(AVERAGE(D23:CF23), 0)</f>
+        <f>ROUND(AVERAGE(D23:CG23), 0)</f>
         <v/>
       </c>
       <c r="K23" s="6" t="n"/>
@@ -7687,6 +7755,9 @@
       <c r="CF23" t="n">
         <v>6</v>
       </c>
+      <c r="CG23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="28" t="inlineStr">
@@ -7700,7 +7771,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>ROUND(AVERAGE(D24:CF24), 0)</f>
+        <f>ROUND(AVERAGE(D24:CG24), 0)</f>
         <v/>
       </c>
       <c r="K24" s="6" t="n"/>
@@ -7731,6 +7802,9 @@
       <c r="CF24" t="n">
         <v>0</v>
       </c>
+      <c r="CG24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
@@ -7744,7 +7818,7 @@
         </is>
       </c>
       <c r="C25" s="28">
-        <f>ROUND(AVERAGE(D25:CF25), 0)</f>
+        <f>ROUND(AVERAGE(D25:CG25), 0)</f>
         <v/>
       </c>
       <c r="K25" s="6" t="n"/>
@@ -7767,6 +7841,9 @@
         <v>0</v>
       </c>
       <c r="CF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG25" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-08-24
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1172,7 +1172,7 @@
         <v/>
       </c>
       <c r="E6" s="14" t="n">
-        <v>59850</v>
+        <v>60050</v>
       </c>
       <c r="F6" s="13" t="n"/>
       <c r="G6" s="13" t="n">
@@ -1200,7 +1200,7 @@
         <v>10200</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="P6" s="13" t="n"/>
       <c r="Q6" s="13" t="n"/>
@@ -1408,7 +1408,7 @@
         <v/>
       </c>
       <c r="E10" s="14" t="n">
-        <v>155050</v>
+        <v>155450</v>
       </c>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
@@ -1434,7 +1434,7 @@
         <v>4000</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>9650</v>
+        <v>10050</v>
       </c>
       <c r="P10" s="13" t="n"/>
       <c r="Q10" s="13" t="n"/>

</xml_diff>

<commit_message>
Update Clan Games data - 2026-08-25
</commit_message>
<xml_diff>
--- a/cc_cg_events.xlsx
+++ b/cc_cg_events.xlsx
@@ -1938,7 +1938,7 @@
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>50800</v>
+        <v>50950</v>
       </c>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
@@ -1956,7 +1956,7 @@
         <v>2550</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="P20" s="13" t="n"/>
       <c r="Q20" s="13" t="n"/>

</xml_diff>